<commit_message>
Extend BMW repair-first review to 300 issues
</commit_message>
<xml_diff>
--- a/outputs/bmw-repair-first-review/BMW-repair-first-fitment-review.xlsx
+++ b/outputs/bmw-repair-first-review/BMW-repair-first-fitment-review.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rc5f8764a0ac34ac3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BMW Review" sheetId="2" r:id="Rab8651bc2dd1446b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remaining Queue" sheetId="3" r:id="Rfad3f01fdffd4e87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="4" r:id="R1d804c16cf87438d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2a2783990d0d40c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BMW Review" sheetId="2" r:id="R14520d05eee340ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remaining Queue" sheetId="3" r:id="R5abd430bd65d4c88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="4" r:id="Rad630376318b466d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -484,7 +484,7 @@
         <x:v>Reviewed in this batch</x:v>
       </x:c>
       <x:c r="B5" s="13" t="n">
-        <x:v>275</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="C5" s="11"/>
       <x:c r="D5" s="11"/>
@@ -498,7 +498,7 @@
         <x:v>Remaining queue</x:v>
       </x:c>
       <x:c r="B6" s="13" t="n">
-        <x:v>110</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="C6" s="11"/>
       <x:c r="D6" s="11"/>
@@ -512,7 +512,7 @@
         <x:v>Issues with destinations</x:v>
       </x:c>
       <x:c r="B7" s="13" t="n">
-        <x:v>272</x:v>
+        <x:v>297</x:v>
       </x:c>
       <x:c r="C7" s="11"/>
       <x:c r="D7" s="11"/>
@@ -526,7 +526,7 @@
         <x:v>Destination entries</x:v>
       </x:c>
       <x:c r="B8" s="13" t="n">
-        <x:v>392</x:v>
+        <x:v>430</x:v>
       </x:c>
       <x:c r="C8" s="11"/>
       <x:c r="D8" s="11"/>
@@ -540,7 +540,7 @@
         <x:v>Distinct URLs</x:v>
       </x:c>
       <x:c r="B9" s="13" t="n">
-        <x:v>132</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="C9" s="11"/>
       <x:c r="D9" s="11"/>
@@ -15192,28 +15192,1390 @@
       </x:c>
     </x:row>
     <x:row r="396" ht="66" hidden="0" customHeight="1">
-      <x:c r="A396" s="42" t="str"/>
-      <x:c r="B396" s="43" t="str"/>
-      <x:c r="C396" s="43" t="str"/>
-      <x:c r="D396" s="43" t="str"/>
-      <x:c r="E396" s="43" t="str"/>
-      <x:c r="F396" s="43" t="str"/>
-      <x:c r="G396" s="43" t="str"/>
-      <x:c r="H396" s="43" t="str">
+      <x:c r="A396" s="40" t="str"/>
+      <x:c r="B396" s="9" t="str"/>
+      <x:c r="C396" s="9" t="str"/>
+      <x:c r="D396" s="9" t="str"/>
+      <x:c r="E396" s="9" t="str"/>
+      <x:c r="F396" s="9" t="str"/>
+      <x:c r="G396" s="9" t="str"/>
+      <x:c r="H396" s="9" t="str">
         <x:v>BMW specialist locator</x:v>
       </x:c>
-      <x:c r="I396" s="43" t="str">
+      <x:c r="I396" s="9" t="str">
         <x:v>https://www.bimmershops.com/</x:v>
       </x:c>
-      <x:c r="J396" s="43" t="str">
+      <x:c r="J396" s="9" t="str">
         <x:v>actuator versus internal AWD diagnosis</x:v>
       </x:c>
-      <x:c r="K396" s="43" t="str">
+      <x:c r="K396" s="9" t="str">
         <x:v>drivetrain service</x:v>
       </x:c>
-      <x:c r="L396" s="43" t="str"/>
-      <x:c r="M396" s="43" t="str"/>
-      <x:c r="N396" s="44" t="str"/>
+      <x:c r="L396" s="9" t="str"/>
+      <x:c r="M396" s="9" t="str"/>
+      <x:c r="N396" s="41" t="str"/>
+    </x:row>
+    <x:row r="397" ht="448.79998779296875" hidden="0" customHeight="1">
+      <x:c r="A397" s="40" t="n">
+        <x:v>276</x:v>
+      </x:c>
+      <x:c r="B397" s="9" t="str">
+        <x:v>bmw-x1-transfer-case-actuator-2013</x:v>
+      </x:c>
+      <x:c r="C397" s="9" t="str">
+        <x:v>2013-2022 | BMW | X1</x:v>
+      </x:c>
+      <x:c r="D397" s="9" t="str">
+        <x:v>Transfer Case Actuator Motor Failure</x:v>
+      </x:c>
+      <x:c r="E397" s="9" t="str">
+        <x:v>Replace the transfer case actuator motor (also called the servo motor). The transfer case itself usually does not need replacement. Ensure the transfer case fluid is changed at the same time. Some owners report success with rebuilt actuators at lower cost.</x:v>
+      </x:c>
+      <x:c r="F397" s="9" t="str">
+        <x:v>xDrive-only diagnosis; split E84/F48 generations; exact actuator/servo if separately serviceable; internal transfer case check; unit-specific fluid</x:v>
+      </x:c>
+      <x:c r="G397" s="9" t="str">
+        <x:v>GENERATION / AWD-SYSTEM SPLIT</x:v>
+      </x:c>
+      <x:c r="H397" s="9" t="str">
+        <x:v>BMW X1 transfer-case catalog</x:v>
+      </x:c>
+      <x:c r="I397" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x1-transfer_case.html</x:v>
+      </x:c>
+      <x:c r="J397" s="9" t="str">
+        <x:v>2013-2022 xDrive X1; VIN and E84/F48 generation required</x:v>
+      </x:c>
+      <x:c r="K397" s="9" t="str">
+        <x:v>OEM actuator/transfer-case catalog</x:v>
+      </x:c>
+      <x:c r="L397" s="9" t="str"/>
+      <x:c r="M397" s="9" t="str">
+        <x:v>The row crosses longitudinal E84 and transverse F48 AWD systems, so one actuator cannot be approved for the full range.</x:v>
+      </x:c>
+      <x:c r="N397" s="41" t="str">
+        <x:v>Split generations and confirm the exact unit/fluid; the transfer case is not always healthy when an actuator fault is present.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="398" ht="66" hidden="0" customHeight="1">
+      <x:c r="A398" s="40" t="str"/>
+      <x:c r="B398" s="9" t="str"/>
+      <x:c r="C398" s="9" t="str"/>
+      <x:c r="D398" s="9" t="str"/>
+      <x:c r="E398" s="9" t="str"/>
+      <x:c r="F398" s="9" t="str"/>
+      <x:c r="G398" s="9" t="str"/>
+      <x:c r="H398" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I398" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J398" s="9" t="str">
+        <x:v>actuator versus internal AWD diagnosis</x:v>
+      </x:c>
+      <x:c r="K398" s="9" t="str">
+        <x:v>drivetrain service</x:v>
+      </x:c>
+      <x:c r="L398" s="9" t="str"/>
+      <x:c r="M398" s="9" t="str"/>
+      <x:c r="N398" s="41" t="str"/>
+    </x:row>
+    <x:row r="399" ht="382.79998779296875" hidden="0" customHeight="1">
+      <x:c r="A399" s="40" t="n">
+        <x:v>277</x:v>
+      </x:c>
+      <x:c r="B399" s="9" t="str">
+        <x:v>bmw-x2-b48-timing-chain-tensioner-2018</x:v>
+      </x:c>
+      <x:c r="C399" s="9" t="str">
+        <x:v>2018-2023 | BMW | X2 | B48</x:v>
+      </x:c>
+      <x:c r="D399" s="9" t="str">
+        <x:v>B48 Timing Chain Tensioner Weakness</x:v>
+      </x:c>
+      <x:c r="E399" s="9" t="str">
+        <x:v>Replace the timing chain tensioner and inspect the chain and guides. If the chain has stretched beyond specification, replace the full timing chain kit. Updated tensioner design from BMW addresses the oil pressure retention issue.</x:v>
+      </x:c>
+      <x:c r="F399" s="9" t="str">
+        <x:v>Cold-start noise and timing diagnosis; VIN/engine tensioner identification; chain stretch/guide inspection; full timing kit only if out of specification</x:v>
+      </x:c>
+      <x:c r="G399" s="9" t="str">
+        <x:v>DIAGNOSIS / VIN GATE; UPDATE CLAIM UNVERIFIED</x:v>
+      </x:c>
+      <x:c r="H399" s="9" t="str">
+        <x:v>Genuine BMW X2 timing catalog</x:v>
+      </x:c>
+      <x:c r="I399" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x2-timing_chain.html</x:v>
+      </x:c>
+      <x:c r="J399" s="9" t="str">
+        <x:v>2018-2023 X2; VIN, B46/B48 variant, and production date required</x:v>
+      </x:c>
+      <x:c r="K399" s="9" t="str">
+        <x:v>OEM timing-component catalog</x:v>
+      </x:c>
+      <x:c r="L399" s="9" t="str"/>
+      <x:c r="M399" s="9" t="str">
+        <x:v>A specific updated tensioner design and blanket B48 weakness were not substantiated by an exact bulletin or part supersession.</x:v>
+      </x:c>
+      <x:c r="N399" s="41" t="str">
+        <x:v>Do not order a tensioner from noise alone or promise that an 'updated design' cures the condition without VIN/part evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="400" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A400" s="40" t="str"/>
+      <x:c r="B400" s="9" t="str"/>
+      <x:c r="C400" s="9" t="str"/>
+      <x:c r="D400" s="9" t="str"/>
+      <x:c r="E400" s="9" t="str"/>
+      <x:c r="F400" s="9" t="str"/>
+      <x:c r="G400" s="9" t="str"/>
+      <x:c r="H400" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I400" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J400" s="9" t="str">
+        <x:v>B-series timing diagnosis</x:v>
+      </x:c>
+      <x:c r="K400" s="9" t="str">
+        <x:v>specialist service</x:v>
+      </x:c>
+      <x:c r="L400" s="9" t="str"/>
+      <x:c r="M400" s="9" t="str"/>
+      <x:c r="N400" s="41" t="str"/>
+    </x:row>
+    <x:row r="401" ht="580.7999877929688" hidden="0" customHeight="1">
+      <x:c r="A401" s="40" t="n">
+        <x:v>278</x:v>
+      </x:c>
+      <x:c r="B401" s="9" t="str">
+        <x:v>bmw-x2-crankshaft-sensor-recall-2018</x:v>
+      </x:c>
+      <x:c r="C401" s="9" t="str">
+        <x:v>2018-2018 | BMW | X2</x:v>
+      </x:c>
+      <x:c r="D401" s="9" t="str">
+        <x:v>2018 X2 Crankshaft Sensor Safety Recall 18V-465</x:v>
+      </x:c>
+      <x:c r="E401" s="9" t="str">
+        <x:v>Check the VIN for an open 18V-465 campaign. If open, an authorized BMW dealer replaces the crankshaft sensor free of charge. A stall or sudden loss of power requires moving to a safe location and arranging BMW assistance; do not order a sensor from this card. ShowMeTheParts resolved exact X2 category fitment only, so no commerce link is approved.</x:v>
+      </x:c>
+      <x:c r="F401" s="9" t="str">
+        <x:v>VIN recall 18V-465 check; free dealer sensor replacement if open; roadside assistance for stall/loss of power</x:v>
+      </x:c>
+      <x:c r="G401" s="9" t="str">
+        <x:v>RECALL ROUTES ONLY</x:v>
+      </x:c>
+      <x:c r="H401" s="9" t="str">
+        <x:v>BMW recall lookup</x:v>
+      </x:c>
+      <x:c r="I401" s="9" t="str">
+        <x:v>https://www.bmwusa.com/safety-and-emission-recalls.html</x:v>
+      </x:c>
+      <x:c r="J401" s="9" t="str">
+        <x:v>VIN check for 18V-465</x:v>
+      </x:c>
+      <x:c r="K401" s="9" t="str">
+        <x:v>manufacturer recall remedy</x:v>
+      </x:c>
+      <x:c r="L401" s="9" t="str"/>
+      <x:c r="M401" s="9" t="str">
+        <x:v>The corrected How to Fix explicitly says not to order a sensor from the card.</x:v>
+      </x:c>
+      <x:c r="N401" s="41" t="str">
+        <x:v>Keep model-year fitment separate from actual VIN recall eligibility.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="402" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A402" s="40" t="str"/>
+      <x:c r="B402" s="9" t="str"/>
+      <x:c r="C402" s="9" t="str"/>
+      <x:c r="D402" s="9" t="str"/>
+      <x:c r="E402" s="9" t="str"/>
+      <x:c r="F402" s="9" t="str"/>
+      <x:c r="G402" s="9" t="str"/>
+      <x:c r="H402" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I402" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J402" s="9" t="str">
+        <x:v>independent VIN recall-status check</x:v>
+      </x:c>
+      <x:c r="K402" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L402" s="9" t="str"/>
+      <x:c r="M402" s="9" t="str"/>
+      <x:c r="N402" s="41" t="str"/>
+    </x:row>
+    <x:row r="403" ht="382.79998779296875" hidden="0" customHeight="1">
+      <x:c r="A403" s="40" t="n">
+        <x:v>279</x:v>
+      </x:c>
+      <x:c r="B403" s="9" t="str">
+        <x:v>bmw-x2-front-control-arm-bushings-2018</x:v>
+      </x:c>
+      <x:c r="C403" s="9" t="str">
+        <x:v>2018-2023 | BMW | X2</x:v>
+      </x:c>
+      <x:c r="D403" s="9" t="str">
+        <x:v>Front Control Arm Bushing Premature Wear</x:v>
+      </x:c>
+      <x:c r="E403" s="9" t="str">
+        <x:v>Replace front control arms with new bushings (sold as complete assemblies by BMW). Aftermarket options with upgraded polyurethane bushings are available for longer life. Perform a four-wheel alignment after replacement.</x:v>
+      </x:c>
+      <x:c r="F403" s="9" t="str">
+        <x:v>Front suspension inspection; side/position-specific complete arm or serviceable bushing; alignment; polyurethane only after NVH/use review</x:v>
+      </x:c>
+      <x:c r="G403" s="9" t="str">
+        <x:v>SIDE-SPECIFIC SUSPENSION CATALOG</x:v>
+      </x:c>
+      <x:c r="H403" s="9" t="str">
+        <x:v>BMW X2 control-arm catalog</x:v>
+      </x:c>
+      <x:c r="I403" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/X2/Control-Arm/</x:v>
+      </x:c>
+      <x:c r="J403" s="9" t="str">
+        <x:v>2018-2023 F39 X2; select side, position, drivetrain, and VIN</x:v>
+      </x:c>
+      <x:c r="K403" s="9" t="str">
+        <x:v>vehicle-specific arm catalog</x:v>
+      </x:c>
+      <x:c r="L403" s="9" t="str"/>
+      <x:c r="M403" s="9" t="str">
+        <x:v>Control arms are side/position specific and polyurethane changes noise/harshness rather than being a universal longevity upgrade.</x:v>
+      </x:c>
+      <x:c r="N403" s="41" t="str">
+        <x:v>Approve the exact failed arm after inspection; do not default every owner to polyurethane.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="404" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A404" s="40" t="str"/>
+      <x:c r="B404" s="9" t="str"/>
+      <x:c r="C404" s="9" t="str"/>
+      <x:c r="D404" s="9" t="str"/>
+      <x:c r="E404" s="9" t="str"/>
+      <x:c r="F404" s="9" t="str"/>
+      <x:c r="G404" s="9" t="str"/>
+      <x:c r="H404" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I404" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J404" s="9" t="str">
+        <x:v>suspension inspection and four-wheel alignment</x:v>
+      </x:c>
+      <x:c r="K404" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L404" s="9" t="str"/>
+      <x:c r="M404" s="9" t="str"/>
+      <x:c r="N404" s="41" t="str"/>
+    </x:row>
+    <x:row r="405" ht="831.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A405" s="40" t="n">
+        <x:v>280</x:v>
+      </x:c>
+      <x:c r="B405" s="9" t="str">
+        <x:v>bmw-x2-oil-filter-housing-2018</x:v>
+      </x:c>
+      <x:c r="C405" s="9" t="str">
+        <x:v>2018-2023 | BMW | X2 | sDrive28i, xDrive28i | B48</x:v>
+      </x:c>
+      <x:c r="D405" s="9" t="str">
+        <x:v>B48 Oil Filter Housing Gasket Leak/Cracking</x:v>
+      </x:c>
+      <x:c r="E405" s="9" t="str">
+        <x:v>Replace the cracked oil filter housing. OEM plastic housing replacement (BMW 11428596283, $412 dealer) will eventually crack again. RECOMMENDED: Install aftermarket aluminum upgrade housing ($250-350) which permanently eliminates the heat-cycling crack issue. FCP Euro kit 11428596283KT ($450) includes all gaskets and seals. If coolant and oil have mixed, perform complete oil flush and coolant system flush before installing new housing. Check for engine damage if contamination was prolonged.</x:v>
+      </x:c>
+      <x:c r="F405" s="9" t="str">
+        <x:v>Leak/crack and contamination diagnosis; VIN-correct complete oil-filter housing and seals; oil/coolant service if mixed; engine-damage check if prolonged</x:v>
+      </x:c>
+      <x:c r="G405" s="9" t="str">
+        <x:v>EXACT OEM NUMBER CONDITIONAL; ALUMINUM CLAIM HELD</x:v>
+      </x:c>
+      <x:c r="H405" s="9" t="str">
+        <x:v>Genuine BMW X2 oil-filter-housing catalog</x:v>
+      </x:c>
+      <x:c r="I405" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x2-oil_filter_housing.html</x:v>
+      </x:c>
+      <x:c r="J405" s="9" t="str">
+        <x:v>2018-2023 F39 X2; VIN and engine required; verify 11428596283/supersession</x:v>
+      </x:c>
+      <x:c r="K405" s="9" t="str">
+        <x:v>OEM housing catalog</x:v>
+      </x:c>
+      <x:c r="L405" s="9" t="str"/>
+      <x:c r="M405" s="9" t="str">
+        <x:v>The OEM housing must be selected by VIN; no live aluminum-upgrade page with exact X2 fitment and complete oil/coolant interfaces was verified.</x:v>
+      </x:c>
+      <x:c r="N405" s="41" t="str">
+        <x:v>Reject 'permanently eliminates' and the unverified FCP kit claim until an exact live product page proves X2 fitment and completeness.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="406" ht="330" hidden="0" customHeight="1">
+      <x:c r="A406" s="40" t="n">
+        <x:v>281</x:v>
+      </x:c>
+      <x:c r="B406" s="9" t="str">
+        <x:v>bmw-x2-oil-filter-housing-gasket-2018</x:v>
+      </x:c>
+      <x:c r="C406" s="9" t="str">
+        <x:v>2018-2023 | BMW | X2 | B48</x:v>
+      </x:c>
+      <x:c r="D406" s="9" t="str">
+        <x:v>Oil Filter Housing Gasket Leak</x:v>
+      </x:c>
+      <x:c r="E406" s="9" t="str">
+        <x:v>Replace the oil filter housing gasket. Clean all oil-contaminated surfaces and inspect the serpentine belt for oil damage. Replace belt if oil-soaked. Use OEM-quality gasket material for longevity.</x:v>
+      </x:c>
+      <x:c r="F406" s="9" t="str">
+        <x:v>Confirm gasket-only versus cracked housing; exact gasket/seals; clean contamination; inspect and replace oil-soaked belt if needed</x:v>
+      </x:c>
+      <x:c r="G406" s="9" t="str">
+        <x:v>LEAK-SOURCE / HOUSING-CONDITION GATE</x:v>
+      </x:c>
+      <x:c r="H406" s="9" t="str">
+        <x:v>BMW X2 oil-filter-housing catalog</x:v>
+      </x:c>
+      <x:c r="I406" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x2-oil_filter_housing.html</x:v>
+      </x:c>
+      <x:c r="J406" s="9" t="str">
+        <x:v>2018-2023 F39 X2; VIN and gasket-versus-housing branch required</x:v>
+      </x:c>
+      <x:c r="K406" s="9" t="str">
+        <x:v>OEM housing/seal catalog</x:v>
+      </x:c>
+      <x:c r="L406" s="9" t="str"/>
+      <x:c r="M406" s="9" t="str">
+        <x:v>This row overlaps the cracked-housing row, and a gasket cannot repair a cracked plastic housing.</x:v>
+      </x:c>
+      <x:c r="N406" s="41" t="str">
+        <x:v>Consolidate duplicate rows and diagnose gasket versus housing before purchase.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="407" ht="448.79998779296875" hidden="0" customHeight="1">
+      <x:c r="A407" s="40" t="n">
+        <x:v>282</x:v>
+      </x:c>
+      <x:c r="B407" s="9" t="str">
+        <x:v>bmw-x2-tie-rod-recall-2019</x:v>
+      </x:c>
+      <x:c r="C407" s="9" t="str">
+        <x:v>2019-2019 | BMW | X2</x:v>
+      </x:c>
+      <x:c r="D407" s="9" t="str">
+        <x:v>2019 X2 Steering Tie-Rod Safety Recall 19V-601</x:v>
+      </x:c>
+      <x:c r="E407" s="9" t="str">
+        <x:v>Check the VIN in BMW AIR or NHTSA for an open 19V-601 campaign. If open, an authorized BMW dealer checks both tie rods and replaces the tie rods and ball joints as necessary free of charge. Do not infer recall eligibility from model year alone or order steering parts from this card.</x:v>
+      </x:c>
+      <x:c r="F407" s="9" t="str">
+        <x:v>VIN recall 19V-601 check; dealer inspection of both tie rods; free tie-rod/ball-joint replacement only as campaign requires</x:v>
+      </x:c>
+      <x:c r="G407" s="9" t="str">
+        <x:v>RECALL ROUTES ONLY</x:v>
+      </x:c>
+      <x:c r="H407" s="9" t="str">
+        <x:v>BMW recall lookup</x:v>
+      </x:c>
+      <x:c r="I407" s="9" t="str">
+        <x:v>https://www.bmwusa.com/safety-and-emission-recalls.html</x:v>
+      </x:c>
+      <x:c r="J407" s="9" t="str">
+        <x:v>VIN check for 19V-601</x:v>
+      </x:c>
+      <x:c r="K407" s="9" t="str">
+        <x:v>manufacturer recall remedy</x:v>
+      </x:c>
+      <x:c r="L407" s="9" t="str"/>
+      <x:c r="M407" s="9" t="str">
+        <x:v>Recall eligibility and replacement scope are VIN/campaign decisions, not retail fitment.</x:v>
+      </x:c>
+      <x:c r="N407" s="41" t="str">
+        <x:v>Do not order steering parts from model year alone.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="408" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A408" s="40" t="str"/>
+      <x:c r="B408" s="9" t="str"/>
+      <x:c r="C408" s="9" t="str"/>
+      <x:c r="D408" s="9" t="str"/>
+      <x:c r="E408" s="9" t="str"/>
+      <x:c r="F408" s="9" t="str"/>
+      <x:c r="G408" s="9" t="str"/>
+      <x:c r="H408" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I408" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J408" s="9" t="str">
+        <x:v>independent VIN recall-status check</x:v>
+      </x:c>
+      <x:c r="K408" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L408" s="9" t="str"/>
+      <x:c r="M408" s="9" t="str"/>
+      <x:c r="N408" s="41" t="str"/>
+    </x:row>
+    <x:row r="409" ht="646.7999877929688" hidden="0" customHeight="1">
+      <x:c r="A409" s="40" t="n">
+        <x:v>283</x:v>
+      </x:c>
+      <x:c r="B409" s="9" t="str">
+        <x:v>bmw-x2-transmission-jerking-2018</x:v>
+      </x:c>
+      <x:c r="C409" s="9" t="str">
+        <x:v>2018-2020 | BMW | X2</x:v>
+      </x:c>
+      <x:c r="D409" s="9" t="str">
+        <x:v>Aisin 8-Speed Transmission Jerking</x:v>
+      </x:c>
+      <x:c r="E409" s="9" t="str">
+        <x:v>Start with transmission software recalibration at BMW dealer ($200-500) which may resolve calibration-related shifting issues. If software update does not resolve, transmission may require oil pump replacement or internal repair ($2,000-5,000). In severe cases with extensive oil pump neck wear, complete transmission replacement required ($5,000-7,000). Reference TSB GBSEL-SELP24 when visiting dealer.</x:v>
+      </x:c>
+      <x:c r="F409" s="9" t="str">
+        <x:v>VIN/transmission identification; TSB and software level check; adaptation/road test; oil-pump/internal repair only after diagnosis</x:v>
+      </x:c>
+      <x:c r="G409" s="9" t="str">
+        <x:v>TSB / SOFTWARE / SPECIALIST ROUTE</x:v>
+      </x:c>
+      <x:c r="H409" s="9" t="str">
+        <x:v>BMW dealer locator</x:v>
+      </x:c>
+      <x:c r="I409" s="9" t="str">
+        <x:v>https://www.bmwusa.com/dealer-locator.html</x:v>
+      </x:c>
+      <x:c r="J409" s="9" t="str">
+        <x:v>2018-2020 X2 Aisin transmission software and TSB GBSEL-SELP24 check</x:v>
+      </x:c>
+      <x:c r="K409" s="9" t="str">
+        <x:v>manufacturer-capable diagnosis</x:v>
+      </x:c>
+      <x:c r="L409" s="9" t="str"/>
+      <x:c r="M409" s="9" t="str">
+        <x:v>Software, pump-neck wear, internal repair, and complete transmission are distinct branches; no retail part is justified before the TSB workflow.</x:v>
+      </x:c>
+      <x:c r="N409" s="41" t="str">
+        <x:v>Do not promise recalibration will fix mechanical wear or quote a universal repair price.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="410" ht="580.7999877929688" hidden="0" customHeight="1">
+      <x:c r="A410" s="40" t="n">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="B410" s="9" t="str">
+        <x:v>bmw-x2-valve-cover-gasket-2018</x:v>
+      </x:c>
+      <x:c r="C410" s="9" t="str">
+        <x:v>2018-2023 | BMW | X2</x:v>
+      </x:c>
+      <x:c r="D410" s="9" t="str">
+        <x:v>Valve Cover Gasket Oil Leak</x:v>
+      </x:c>
+      <x:c r="E410" s="9" t="str">
+        <x:v>Replace valve cover gasket. Genuine BMW valve cover assembly 11127611278 ($200-350) includes integrated gasket. Labor typically 2-3 hours ($300-500). Total cost $700-1,000 at shop. DIY possible with basic tools to save $300-500 in labor. Replace spark plug tube seals at same time if applicable - labor overlap saves money. Monitor oil level between repairs.</x:v>
+      </x:c>
+      <x:c r="F410" s="9" t="str">
+        <x:v>Leak/PCV diagnosis; complete cover 11127611278 where VIN-matched and cover/PCV failed; gasket/tube seals by condition; cleanup</x:v>
+      </x:c>
+      <x:c r="G410" s="9" t="str">
+        <x:v>EXACT OEM COVER CONDITIONAL</x:v>
+      </x:c>
+      <x:c r="H410" s="9" t="str">
+        <x:v>Genuine BMW valve cover 11127611278</x:v>
+      </x:c>
+      <x:c r="I410" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/products/bmw-cylinder-head-cover-11127611278</x:v>
+      </x:c>
+      <x:c r="J410" s="9" t="str">
+        <x:v>F39 X2 B46/B48 where validated; confirm VIN/current fitment</x:v>
+      </x:c>
+      <x:c r="K410" s="9" t="str">
+        <x:v>conditional complete valve-cover assembly</x:v>
+      </x:c>
+      <x:c r="L410" s="9" t="str"/>
+      <x:c r="M410" s="9" t="str">
+        <x:v>The live page identifies the genuine cover and includes X2 fitment, while the complete assembly remains conditional on cover/PCV condition.</x:v>
+      </x:c>
+      <x:c r="N410" s="41" t="str">
+        <x:v>Do not call a complete cover a gasket repair or automatically add tube seals without checking kit contents.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="411" ht="990" hidden="0" customHeight="1">
+      <x:c r="A411" s="40" t="n">
+        <x:v>285</x:v>
+      </x:c>
+      <x:c r="B411" s="9" t="str">
+        <x:v>bmw-x3-coolant-expansion-tank-2004</x:v>
+      </x:c>
+      <x:c r="C411" s="9" t="str">
+        <x:v>2004-2023 | BMW | X3</x:v>
+      </x:c>
+      <x:c r="D411" s="9" t="str">
+        <x:v>Coolant Expansion Tank Cracking</x:v>
+      </x:c>
+      <x:c r="E411" s="9" t="str">
+        <x:v>Replace expansion tank and coolant ($50-100 DIY parts, $200-400 independent shop, $400-580 dealer). Very simple DIY repair taking 30 minutes - drain coolant, unbolt old tank, install new tank, refill with BMW-spec coolant (blue or pink/orange premix). Use Behr or OEM BMW expansion tank - Dorman aftermarket tanks may fail prematurely. YouTube and Pelicanparts have detailed DIY guides. PREVENTIVE: Replace every 5-7 years or 80-100k miles before cracks develop. Check tank regularly for hairline cracks. Don't ignore coolant leaks - can lead to catastrophic overheating and head gasket failure.</x:v>
+      </x:c>
+      <x:c r="F411" s="9" t="str">
+        <x:v>Pressure-test leak source; generation/engine/VIN-specific expansion tank; correct current coolant specification; bleed/test; preventive replacement only by condition</x:v>
+      </x:c>
+      <x:c r="G411" s="9" t="str">
+        <x:v>MULTI-GENERATION VIN CATALOG</x:v>
+      </x:c>
+      <x:c r="H411" s="9" t="str">
+        <x:v>BMW X3 expansion-tank catalog</x:v>
+      </x:c>
+      <x:c r="I411" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/X3/Expansion-Tank/</x:v>
+      </x:c>
+      <x:c r="J411" s="9" t="str">
+        <x:v>2004-2023 E83/F25/G01 X3; select exact engine, generation, and VIN</x:v>
+      </x:c>
+      <x:c r="K411" s="9" t="str">
+        <x:v>vehicle-specific tank catalog</x:v>
+      </x:c>
+      <x:c r="L411" s="9" t="str"/>
+      <x:c r="M411" s="9" t="str">
+        <x:v>The 20-year range spans multiple tanks and coolant specifications; one Behr/OEM part cannot fit all.</x:v>
+      </x:c>
+      <x:c r="N411" s="41" t="str">
+        <x:v>Remove universal 30-minute labor, color-only coolant advice, fixed preventive interval, and blanket brand-failure claims.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="412" ht="435.6000061035156" hidden="0" customHeight="1">
+      <x:c r="A412" s="40" t="n">
+        <x:v>286</x:v>
+      </x:c>
+      <x:c r="B412" s="9" t="str">
+        <x:v>bmw-x3-electric-water-pump-2011</x:v>
+      </x:c>
+      <x:c r="C412" s="9" t="str">
+        <x:v>2011-2026 | BMW | X3</x:v>
+      </x:c>
+      <x:c r="D412" s="9" t="str">
+        <x:v>Electric Water Pump Failure</x:v>
+      </x:c>
+      <x:c r="E412" s="9" t="str">
+        <x:v>Replace the electric water pump and thermostat together, as they are part of the same cooling circuit and the thermostat often fails concurrently. Bleed the cooling system thoroughly after replacement. Some owners carry a spare pump due to the sudden failure nature.</x:v>
+      </x:c>
+      <x:c r="F412" s="9" t="str">
+        <x:v>Generation/engine/VIN diagnosis; identify mechanical main pump versus electric pump/auxiliary circuit; thermostat only if applicable/failed; exact bleed procedure</x:v>
+      </x:c>
+      <x:c r="G412" s="9" t="str">
+        <x:v>MAJOR ENGINE / PUMP-TYPE SPLIT</x:v>
+      </x:c>
+      <x:c r="H412" s="9" t="str">
+        <x:v>Genuine BMW X3 water-pump catalog</x:v>
+      </x:c>
+      <x:c r="I412" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x3-water_pump.html</x:v>
+      </x:c>
+      <x:c r="J412" s="9" t="str">
+        <x:v>2011-2026 X3; VIN, engine, pump circuit, and generation required</x:v>
+      </x:c>
+      <x:c r="K412" s="9" t="str">
+        <x:v>OEM pump catalog</x:v>
+      </x:c>
+      <x:c r="L412" s="9" t="str"/>
+      <x:c r="M412" s="9" t="str">
+        <x:v>Not every X3 engine in 2011-2026 uses the same electric main pump, and thermostat replacement is not universally paired.</x:v>
+      </x:c>
+      <x:c r="N412" s="41" t="str">
+        <x:v>Split by engine/pump type; remove the advice to carry a spare pump.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="413" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A413" s="40" t="str"/>
+      <x:c r="B413" s="9" t="str"/>
+      <x:c r="C413" s="9" t="str"/>
+      <x:c r="D413" s="9" t="str"/>
+      <x:c r="E413" s="9" t="str"/>
+      <x:c r="F413" s="9" t="str"/>
+      <x:c r="G413" s="9" t="str"/>
+      <x:c r="H413" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I413" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J413" s="9" t="str">
+        <x:v>cooling-system diagnosis and bleed</x:v>
+      </x:c>
+      <x:c r="K413" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L413" s="9" t="str"/>
+      <x:c r="M413" s="9" t="str"/>
+      <x:c r="N413" s="41" t="str"/>
+    </x:row>
+    <x:row r="414" ht="541.2000122070312" hidden="0" customHeight="1">
+      <x:c r="A414" s="40" t="n">
+        <x:v>287</x:v>
+      </x:c>
+      <x:c r="B414" s="9" t="str">
+        <x:v>bmw-x3-m-electric-wastegate-actuator-adaptation-fault-boost-cutout-ea</x:v>
+      </x:c>
+      <x:c r="C414" s="9" t="str">
+        <x:v>2020-2020 | BMW | X3 M | S58</x:v>
+      </x:c>
+      <x:c r="D414" s="9" t="str">
+        <x:v>2020 X3 M Wastegate Adaptation Faults Require Software Diagnosis</x:v>
+      </x:c>
+      <x:c r="E414" s="9" t="str">
+        <x:v>Confirm the production date, fault codes and current vehicle integration level. If the I-level is below S15A-20-03-510, a BMW-qualified repairer follows the bulletin and programs the vehicle with the specified or newer approved ISTA level. Diagnose unrelated mechanical noise separately; do not replace an actuator or turbocharger from this card.</x:v>
+      </x:c>
+      <x:c r="F414" s="9" t="str">
+        <x:v>Production date, fault-code, and integration-level confirmation; BMW ISTA programming to specified/newer approved level; mechanical diagnosis separately</x:v>
+      </x:c>
+      <x:c r="G414" s="9" t="str">
+        <x:v>SOFTWARE SERVICE ROUTE ONLY</x:v>
+      </x:c>
+      <x:c r="H414" s="9" t="str">
+        <x:v>BMW dealer locator</x:v>
+      </x:c>
+      <x:c r="I414" s="9" t="str">
+        <x:v>https://www.bmwusa.com/dealer-locator.html</x:v>
+      </x:c>
+      <x:c r="J414" s="9" t="str">
+        <x:v>2020 F97 X3 M ISTA integration-level check and programming</x:v>
+      </x:c>
+      <x:c r="K414" s="9" t="str">
+        <x:v>bulletin software remedy</x:v>
+      </x:c>
+      <x:c r="L414" s="9" t="str"/>
+      <x:c r="M414" s="9" t="str">
+        <x:v>The corrected How to Fix explicitly rejects actuator/turbo replacement from this card.</x:v>
+      </x:c>
+      <x:c r="N414" s="41" t="str">
+        <x:v>Do not attach wastegate hardware or a generic OBD scanner to a programming bulletin.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="415" ht="462" hidden="0" customHeight="1">
+      <x:c r="A415" s="40" t="n">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="B415" s="9" t="str">
+        <x:v>bmw-x3-m-fuel-tank-inlet-check-valve-weld-failure-2021-x3-m</x:v>
+      </x:c>
+      <x:c r="C415" s="9" t="str">
+        <x:v>2021-2021 | BMW | X3 M</x:v>
+      </x:c>
+      <x:c r="D415" s="9" t="str">
+        <x:v>2021 X3 M Fuel-Tank Safety Recall 21V-199</x:v>
+      </x:c>
+      <x:c r="E415" s="9" t="str">
+        <x:v>Check the VIN for an open 21V-199 campaign. If open, an authorized BMW dealer replaces the fuel tank free of charge. If fuel odor or leakage appears, move safely away from traffic, stop, have occupants exit and contact BMW roadside assistance; do not continue driving or order a tank from this card.</x:v>
+      </x:c>
+      <x:c r="F415" s="9" t="str">
+        <x:v>VIN recall 21V-199 check; free dealer fuel-tank replacement if open; roadside safety response for odor/leak</x:v>
+      </x:c>
+      <x:c r="G415" s="9" t="str">
+        <x:v>RECALL ROUTES ONLY</x:v>
+      </x:c>
+      <x:c r="H415" s="9" t="str">
+        <x:v>BMW recall lookup</x:v>
+      </x:c>
+      <x:c r="I415" s="9" t="str">
+        <x:v>https://www.bmwusa.com/safety-and-emission-recalls.html</x:v>
+      </x:c>
+      <x:c r="J415" s="9" t="str">
+        <x:v>VIN check for 21V-199</x:v>
+      </x:c>
+      <x:c r="K415" s="9" t="str">
+        <x:v>manufacturer recall remedy</x:v>
+      </x:c>
+      <x:c r="L415" s="9" t="str"/>
+      <x:c r="M415" s="9" t="str">
+        <x:v>The safety remedy is an authorized recall repair, not a retail tank sale.</x:v>
+      </x:c>
+      <x:c r="N415" s="41" t="str">
+        <x:v>Preserve the stop/evacuate/tow warning for active fuel leakage.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="416" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A416" s="40" t="str"/>
+      <x:c r="B416" s="9" t="str"/>
+      <x:c r="C416" s="9" t="str"/>
+      <x:c r="D416" s="9" t="str"/>
+      <x:c r="E416" s="9" t="str"/>
+      <x:c r="F416" s="9" t="str"/>
+      <x:c r="G416" s="9" t="str"/>
+      <x:c r="H416" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I416" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J416" s="9" t="str">
+        <x:v>independent VIN recall-status check</x:v>
+      </x:c>
+      <x:c r="K416" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L416" s="9" t="str"/>
+      <x:c r="M416" s="9" t="str"/>
+      <x:c r="N416" s="41" t="str"/>
+    </x:row>
+    <x:row r="417" ht="580.7999877929688" hidden="0" customHeight="1">
+      <x:c r="A417" s="40" t="n">
+        <x:v>289</x:v>
+      </x:c>
+      <x:c r="B417" s="9" t="str">
+        <x:v>bmw-x3-m-idrive-control-display-blank-screen-infotainment-glitches-f9</x:v>
+      </x:c>
+      <x:c r="C417" s="9" t="str">
+        <x:v>2020-2021 | BMW | X3 M | X3 M, X3 M Competition | S58, S58B30</x:v>
+      </x:c>
+      <x:c r="D417" s="9" t="str">
+        <x:v>iDrive Control Display Blank Screen and Infotainment Glitches - F97 X3 M (2019-2021)</x:v>
+      </x:c>
+      <x:c r="E417" s="9" t="str">
+        <x:v>First try the latest iDrive/head-unit software update at the dealer, which resolves many of the early glitches, reboots, and camera issues. If the display panel hardware has failed (lines, persistent blank screen with backlight off), the control display/screen assembly is replaced. A soft reset (press-and-hold volume/power) can temporarily clear a frozen screen.</x:v>
+      </x:c>
+      <x:c r="F417" s="9" t="str">
+        <x:v>Soft reset; current iDrive/head-unit software; 12-volt health check; screen assembly only after hardware diagnosis</x:v>
+      </x:c>
+      <x:c r="G417" s="9" t="str">
+        <x:v>SOFTWARE FIRST / CONDITIONAL HARDWARE</x:v>
+      </x:c>
+      <x:c r="H417" s="9" t="str">
+        <x:v>BMW Remote Software Upgrade</x:v>
+      </x:c>
+      <x:c r="I417" s="9" t="str">
+        <x:v>https://www.bmwusa.com/explore/connecteddrive/remote-software-upgrade.html</x:v>
+      </x:c>
+      <x:c r="J417" s="9" t="str">
+        <x:v>F97 X3 M only when update is offered to VIN</x:v>
+      </x:c>
+      <x:c r="K417" s="9" t="str">
+        <x:v>official update information</x:v>
+      </x:c>
+      <x:c r="L417" s="9" t="str"/>
+      <x:c r="M417" s="9" t="str">
+        <x:v>The source requires software first and reserves display replacement for confirmed hardware failure.</x:v>
+      </x:c>
+      <x:c r="N417" s="41" t="str">
+        <x:v>Do not sell a screen for a frozen head unit or low-voltage condition.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="418" ht="66" hidden="0" customHeight="1">
+      <x:c r="A418" s="40" t="str"/>
+      <x:c r="B418" s="9" t="str"/>
+      <x:c r="C418" s="9" t="str"/>
+      <x:c r="D418" s="9" t="str"/>
+      <x:c r="E418" s="9" t="str"/>
+      <x:c r="F418" s="9" t="str"/>
+      <x:c r="G418" s="9" t="str"/>
+      <x:c r="H418" s="9" t="str">
+        <x:v>BMW dealer locator</x:v>
+      </x:c>
+      <x:c r="I418" s="9" t="str">
+        <x:v>https://www.bmwusa.com/dealer-locator.html</x:v>
+      </x:c>
+      <x:c r="J418" s="9" t="str">
+        <x:v>recurring fault and display hardware diagnosis</x:v>
+      </x:c>
+      <x:c r="K418" s="9" t="str">
+        <x:v>software/hardware service</x:v>
+      </x:c>
+      <x:c r="L418" s="9" t="str"/>
+      <x:c r="M418" s="9" t="str"/>
+      <x:c r="N418" s="41" t="str"/>
+    </x:row>
+    <x:row r="419" ht="462" hidden="0" customHeight="1">
+      <x:c r="A419" s="40" t="n">
+        <x:v>290</x:v>
+      </x:c>
+      <x:c r="B419" s="9" t="str">
+        <x:v>bmw-x3-m-improperly-welded-front-seat-frame-2019-2021-x3-m</x:v>
+      </x:c>
+      <x:c r="C419" s="9" t="str">
+        <x:v>2021-2021 | BMW | X3 M</x:v>
+      </x:c>
+      <x:c r="D419" s="9" t="str">
+        <x:v>2021 X3 M Front Seat-Frame Safety Recall 23V-211</x:v>
+      </x:c>
+      <x:c r="E419" s="9" t="str">
+        <x:v>Check the VIN for an open 23V-211 campaign. If open, an authorized BMW dealer replaces the affected front seat frame and backrest free of charge using VIN-selected parts. Contact BMW promptly if a front seat vibrates or makes abnormal noise; do not order seat components from this card.</x:v>
+      </x:c>
+      <x:c r="F419" s="9" t="str">
+        <x:v>VIN recall 23V-211 check; free dealer seat-frame/backrest replacement using campaign-selected parts</x:v>
+      </x:c>
+      <x:c r="G419" s="9" t="str">
+        <x:v>RECALL ROUTES ONLY</x:v>
+      </x:c>
+      <x:c r="H419" s="9" t="str">
+        <x:v>BMW recall lookup</x:v>
+      </x:c>
+      <x:c r="I419" s="9" t="str">
+        <x:v>https://www.bmwusa.com/safety-and-emission-recalls.html</x:v>
+      </x:c>
+      <x:c r="J419" s="9" t="str">
+        <x:v>VIN check for 23V-211</x:v>
+      </x:c>
+      <x:c r="K419" s="9" t="str">
+        <x:v>manufacturer recall remedy</x:v>
+      </x:c>
+      <x:c r="L419" s="9" t="str"/>
+      <x:c r="M419" s="9" t="str">
+        <x:v>VIN-selected recall parts belong with the authorized campaign.</x:v>
+      </x:c>
+      <x:c r="N419" s="41" t="str">
+        <x:v>Do not order seat components from model year alone.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="420" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A420" s="40" t="str"/>
+      <x:c r="B420" s="9" t="str"/>
+      <x:c r="C420" s="9" t="str"/>
+      <x:c r="D420" s="9" t="str"/>
+      <x:c r="E420" s="9" t="str"/>
+      <x:c r="F420" s="9" t="str"/>
+      <x:c r="G420" s="9" t="str"/>
+      <x:c r="H420" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I420" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J420" s="9" t="str">
+        <x:v>independent VIN recall-status check</x:v>
+      </x:c>
+      <x:c r="K420" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L420" s="9" t="str"/>
+      <x:c r="M420" s="9" t="str"/>
+      <x:c r="N420" s="41" t="str"/>
+    </x:row>
+    <x:row r="421" ht="541.2000122070312" hidden="0" customHeight="1">
+      <x:c r="A421" s="40" t="n">
+        <x:v>291</x:v>
+      </x:c>
+      <x:c r="B421" s="9" t="str">
+        <x:v>bmw-x3-m-low-mounted-engine-oil-cooler-vulnerable-to-road-debris-punc</x:v>
+      </x:c>
+      <x:c r="C421" s="9" t="str">
+        <x:v>2020-2023 | BMW | X3 M | X3 M, X3 M Competition | S58, S58B30</x:v>
+      </x:c>
+      <x:c r="D421" s="9" t="str">
+        <x:v>Low-Mounted Engine Oil Cooler Vulnerable to Road-Debris Puncture - F97 X3 M (S58)</x:v>
+      </x:c>
+      <x:c r="E421" s="9" t="str">
+        <x:v>Inspect the oil cooler periodically for stone damage and weeping; fit a protective mesh/guard in front of the cooler as preventive insurance (popular among track and spirited-use owners). If punctured, stop driving immediately and replace the oil cooler and refill with the correct oil; verify no bearing damage occurred from any oil starvation.</x:v>
+      </x:c>
+      <x:c r="F421" s="9" t="str">
+        <x:v>Oil-cooler inspection; exact protective guard; punctured cooler replacement and correct oil; oil-pressure/bearing-damage assessment after starvation</x:v>
+      </x:c>
+      <x:c r="G421" s="9" t="str">
+        <x:v>EXACT F97/F98 GUARD APPROVAL</x:v>
+      </x:c>
+      <x:c r="H421" s="9" t="str">
+        <x:v>RW Carbon F97 X3M oil-cooler guard bmwf97022</x:v>
+      </x:c>
+      <x:c r="I421" s="9" t="str">
+        <x:v>https://www.rwcarbon.com/bmw-f97-x3m-f98-x4m-aluminum-oil-cooler-guard.html</x:v>
+      </x:c>
+      <x:c r="J421" s="9" t="str">
+        <x:v>2019+ F97 X3 M/F98 X4 M as explicitly listed; verify model year/current stock</x:v>
+      </x:c>
+      <x:c r="K421" s="9" t="str">
+        <x:v>preventive underbody oil-cooler guard</x:v>
+      </x:c>
+      <x:c r="L421" s="9" t="str"/>
+      <x:c r="M421" s="9" t="str">
+        <x:v>The guard manufacturer explicitly lists F97 X3 M fitment and factory mounting points.</x:v>
+      </x:c>
+      <x:c r="N421" s="41" t="str">
+        <x:v>A guard reduces road-debris exposure but cannot guarantee prevention; stop driving immediately after oil loss.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="422" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A422" s="40" t="str"/>
+      <x:c r="B422" s="9" t="str"/>
+      <x:c r="C422" s="9" t="str"/>
+      <x:c r="D422" s="9" t="str"/>
+      <x:c r="E422" s="9" t="str"/>
+      <x:c r="F422" s="9" t="str"/>
+      <x:c r="G422" s="9" t="str"/>
+      <x:c r="H422" s="9" t="str">
+        <x:v>Genuine BMW X3 M oil-cooler catalog</x:v>
+      </x:c>
+      <x:c r="I422" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x3_m-oil_cooler.html</x:v>
+      </x:c>
+      <x:c r="J422" s="9" t="str">
+        <x:v>VIN-specific replacement only after puncture/diagnosis</x:v>
+      </x:c>
+      <x:c r="K422" s="9" t="str">
+        <x:v>conditional OEM cooler</x:v>
+      </x:c>
+      <x:c r="L422" s="9" t="str"/>
+      <x:c r="M422" s="9" t="str"/>
+      <x:c r="N422" s="41" t="str"/>
+    </x:row>
+    <x:row r="423" ht="594" hidden="0" customHeight="1">
+      <x:c r="A423" s="40" t="n">
+        <x:v>292</x:v>
+      </x:c>
+      <x:c r="B423" s="9" t="str">
+        <x:v>bmw-x3-m-oem-plastic-charge-pipe-cracking-blow-off-under-boost-f97-x3</x:v>
+      </x:c>
+      <x:c r="C423" s="9" t="str">
+        <x:v>2020-2023 | BMW | X3 M | X3 M, X3 M Competition | S58, S58B30</x:v>
+      </x:c>
+      <x:c r="D423" s="9" t="str">
+        <x:v>OEM Plastic Charge Pipe Cracking / Blow-Off Under Boost - F97 X3 M (S58)</x:v>
+      </x:c>
+      <x:c r="E423" s="9" t="str">
+        <x:v>Replace the OEM plastic charge pipe with an aluminum (or reinforced) aftermarket charge pipe from suppliers such as FTP, Racing Dynamics, or Kies; this is the standard durable fix and is strongly recommended before or alongside any tune. A failed OEM pipe can be re-fitted with a new OEM unit but the same failure mode tends to recur, especially on modified cars.</x:v>
+      </x:c>
+      <x:c r="F423" s="9" t="str">
+        <x:v>Smoke/boost-leak diagnosis; F97 S58 charge-pipe kit; verify whether larger 2-to-1 pipe is included/needed; seals/clips</x:v>
+      </x:c>
+      <x:c r="G423" s="9" t="str">
+        <x:v>EXACT F97 S58 KIT WITH COMPLETENESS NOTE</x:v>
+      </x:c>
+      <x:c r="H423" s="9" t="str">
+        <x:v>FTP S58 charge-pipe kit sg71466</x:v>
+      </x:c>
+      <x:c r="I423" s="9" t="str">
+        <x:v>https://www.turnermotorsport.com/p-46444158-s58-charge-pipe-kit/</x:v>
+      </x:c>
+      <x:c r="J423" s="9" t="str">
+        <x:v>F97 X3 M S58 explicitly listed; special order; excludes larger 2-to-1 charge pipe</x:v>
+      </x:c>
+      <x:c r="K423" s="9" t="str">
+        <x:v>charge-pipe replacement kit</x:v>
+      </x:c>
+      <x:c r="L423" s="9" t="str"/>
+      <x:c r="M423" s="9" t="str">
+        <x:v>The live product page explicitly lists F97 X3 M S58 and discloses that the larger 2-to-1 pipe is not included.</x:v>
+      </x:c>
+      <x:c r="N423" s="41" t="str">
+        <x:v>The factory S58 pipes are mixed rubber/aluminum, not simply all plastic; do not call replacement mandatory for every tune.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="424" ht="382.79998779296875" hidden="0" customHeight="1">
+      <x:c r="A424" s="40" t="n">
+        <x:v>293</x:v>
+      </x:c>
+      <x:c r="B424" s="9" t="str">
+        <x:v>bmw-x3-n20-timing-chain-2011</x:v>
+      </x:c>
+      <x:c r="C424" s="9" t="str">
+        <x:v>2011-2017 | BMW | X3 | N20</x:v>
+      </x:c>
+      <x:c r="D424" s="9" t="str">
+        <x:v>N20 Timing Chain Guide Failure</x:v>
+      </x:c>
+      <x:c r="E424" s="9" t="str">
+        <x:v>Replace the complete timing chain kit including chain, guides, tensioner, and sprockets. Preventive replacement is strongly recommended at 80,000 miles before failure occurs. The updated guide design uses more durable materials.</x:v>
+      </x:c>
+      <x:c r="F424" s="9" t="str">
+        <x:v>Confirm N20 engine/production date and timing diagnosis; complete chain/guide/tensioner/oil-pump-chain service kit when failure confirmed</x:v>
+      </x:c>
+      <x:c r="G424" s="9" t="str">
+        <x:v>EXACT N20 KIT AFTER DIAGNOSIS</x:v>
+      </x:c>
+      <x:c r="H424" s="9" t="str">
+        <x:v>FCP Euro N20/N26 timing kit 11318648732KT</x:v>
+      </x:c>
+      <x:c r="I424" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/products/bmw-n20-n26-timing-chain-kit-11318648732kt</x:v>
+      </x:c>
+      <x:c r="J424" s="9" t="str">
+        <x:v>F25 X3 N20 where cataloged; verify VIN/production date and installer-required access parts</x:v>
+      </x:c>
+      <x:c r="K424" s="9" t="str">
+        <x:v>engine-specific timing kit</x:v>
+      </x:c>
+      <x:c r="L424" s="9" t="str"/>
+      <x:c r="M424" s="9" t="str">
+        <x:v>The live kit identifies N20/N26 applications including X3, but the broad 2011-2017 row still requires engine confirmation.</x:v>
+      </x:c>
+      <x:c r="N424" s="41" t="str">
+        <x:v>Remove the universal 80,000-mile preventive recommendation and diagnose before purchase.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="425" ht="673.2000122070312" hidden="0" customHeight="1">
+      <x:c r="A425" s="40" t="n">
+        <x:v>294</x:v>
+      </x:c>
+      <x:c r="B425" s="9" t="str">
+        <x:v>bmw-x3-n20-timing-chain-2012</x:v>
+      </x:c>
+      <x:c r="C425" s="9" t="str">
+        <x:v>2013-2015 | BMW | X3 | N20</x:v>
+      </x:c>
+      <x:c r="D425" s="9" t="str">
+        <x:v>Lower-Engine Whine Requires X3 N20 Timing-Chain Diagnosis</x:v>
+      </x:c>
+      <x:c r="E425" s="9" t="str">
+        <x:v>Confirm the exact X3 variant, N20 engine, production date and VIN eligibility, then have a BMW-qualified technician reproduce the noise and follow current BMW diagnosis before replacing anything. The historical seven-year/70,000-mile coverage was a limited warranty extension, not a recall, and is not a current coverage promise. ShowMeTheParts established category-level fitment only, so no commerce link is approved.</x:v>
+      </x:c>
+      <x:c r="F425" s="9" t="str">
+        <x:v>N20/production-date/VIN confirmation; noise reproduction and BMW diagnosis; historical extension disclosed as expired</x:v>
+      </x:c>
+      <x:c r="G425" s="9" t="str">
+        <x:v>DIAGNOSIS / WARRANTY-HISTORY ROUTE</x:v>
+      </x:c>
+      <x:c r="H425" s="9" t="str">
+        <x:v>BMW dealer locator</x:v>
+      </x:c>
+      <x:c r="I425" s="9" t="str">
+        <x:v>https://www.bmwusa.com/dealer-locator.html</x:v>
+      </x:c>
+      <x:c r="J425" s="9" t="str">
+        <x:v>2013-2015 F25 X3 N20 timing diagnosis and VIN history</x:v>
+      </x:c>
+      <x:c r="K425" s="9" t="str">
+        <x:v>BMW-qualified service</x:v>
+      </x:c>
+      <x:c r="L425" s="9" t="str"/>
+      <x:c r="M425" s="9" t="str">
+        <x:v>The corrected source rejects category fitment as proof and distinguishes an expired extension from a recall.</x:v>
+      </x:c>
+      <x:c r="N425" s="41" t="str">
+        <x:v>Do not attach a kit to lower-engine whine alone.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="426" ht="752.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A426" s="40" t="n">
+        <x:v>295</x:v>
+      </x:c>
+      <x:c r="B426" s="9" t="str">
+        <x:v>bmw-x3-oil-filter-housing-gasket-2007</x:v>
+      </x:c>
+      <x:c r="C426" s="9" t="str">
+        <x:v>2007-2017 | BMW | X3 | sDrive30i, xDrive28i, xDrive30i | N52, N20</x:v>
+      </x:c>
+      <x:c r="D426" s="9" t="str">
+        <x:v>Oil Filter Housing Gasket Leak (N52, N20 Engines)</x:v>
+      </x:c>
+      <x:c r="E426" s="9" t="str">
+        <x:v>Replace oil filter housing gasket and oil cooler gasket ($40-80 DIY repair kit, $300-500 independent shop, $500-800 dealer). Requires draining some coolant and oil, removing housing, replacing gaskets, reassembling. Moderate DIY difficulty - Pelicanparts and YouTube have detailed model-specific guides. Use Victor Reinz or OEM BMW gasket kit for long-lasting seal - cheap gaskets leak within 20k miles. Address leak early before oil damages serpentine belt or alternator.</x:v>
+      </x:c>
+      <x:c r="F426" s="9" t="str">
+        <x:v>Split N52 and N20 engines; leak-source diagnosis; housing and oil-cooler gaskets only as equipped; coolant/oil service; belt/alternator inspection</x:v>
+      </x:c>
+      <x:c r="G426" s="9" t="str">
+        <x:v>ENGINE / HOUSING CONFIGURATION SPLIT</x:v>
+      </x:c>
+      <x:c r="H426" s="9" t="str">
+        <x:v>BMW X3 oil-filter-housing gasket catalog</x:v>
+      </x:c>
+      <x:c r="I426" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/X3/Oil-Filter-Housing-Gasket/</x:v>
+      </x:c>
+      <x:c r="J426" s="9" t="str">
+        <x:v>2007-2017 X3; select exact engine, generation, VIN, and oil-cooler configuration</x:v>
+      </x:c>
+      <x:c r="K426" s="9" t="str">
+        <x:v>vehicle-specific gasket catalog</x:v>
+      </x:c>
+      <x:c r="L426" s="9" t="str"/>
+      <x:c r="M426" s="9" t="str">
+        <x:v>N52 and N20 housings and seals are not interchangeable, and not every configuration uses the same cooler gasket.</x:v>
+      </x:c>
+      <x:c r="N426" s="41" t="str">
+        <x:v>Split engines; remove universal labor/cost and blanket cheap-gasket lifespan claims.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="427" ht="950.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A427" s="40" t="n">
+        <x:v>296</x:v>
+      </x:c>
+      <x:c r="B427" s="9" t="str">
+        <x:v>bmw-x3-transfer-case-actuator-2004</x:v>
+      </x:c>
+      <x:c r="C427" s="9" t="str">
+        <x:v>2004-2023 | BMW | X3</x:v>
+      </x:c>
+      <x:c r="D427" s="9" t="str">
+        <x:v>Transfer Case Actuator Motor Failure (xDrive AWD System)</x:v>
+      </x:c>
+      <x:c r="E427" s="9" t="str">
+        <x:v>Replace the actuator motor assembly or rebuild using an aftermarket repair kit. DIY repair kits cost $100-150 and include replacement plastic gears, clips, and seals - straightforward installation saves $1,200+. Complete actuator motor replacement costs $540 for the assembly if DIY, or $1,500-2,200 at dealer. If transfer case itself is damaged from prolonged actuator failure, complete transfer case replacement costs $1,400-3,300. PREVENTIVE: If buying used X3 over 80k miles, budget for this repair - it's "when not if" on xDrive models. Check for clicking noise when shutting off ignition.</x:v>
+      </x:c>
+      <x:c r="F427" s="9" t="str">
+        <x:v>xDrive fault diagnosis; generation/unit identification; motor versus gear versus internal transfer-case failure; exact repair kit/actuator; unit-specific fluid</x:v>
+      </x:c>
+      <x:c r="G427" s="9" t="str">
+        <x:v>MULTI-GENERATION DRIVETRAIN SPLIT</x:v>
+      </x:c>
+      <x:c r="H427" s="9" t="str">
+        <x:v>BMW X3 transfer-case catalog</x:v>
+      </x:c>
+      <x:c r="I427" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x3-transfer_case.html</x:v>
+      </x:c>
+      <x:c r="J427" s="9" t="str">
+        <x:v>2004-2023 E83/F25/G01 xDrive; VIN and exact transfer-case unit required</x:v>
+      </x:c>
+      <x:c r="K427" s="9" t="str">
+        <x:v>OEM actuator/transfer-case catalog</x:v>
+      </x:c>
+      <x:c r="L427" s="9" t="str"/>
+      <x:c r="M427" s="9" t="str">
+        <x:v>The 20-year range spans multiple transfer cases; a plastic-gear kit cannot be approved across all units.</x:v>
+      </x:c>
+      <x:c r="N427" s="41" t="str">
+        <x:v>Remove 'when not if,' fixed prices, and generic clicking diagnosis; verify the fault and unit before parts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="428" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A428" s="40" t="str"/>
+      <x:c r="B428" s="9" t="str"/>
+      <x:c r="C428" s="9" t="str"/>
+      <x:c r="D428" s="9" t="str"/>
+      <x:c r="E428" s="9" t="str"/>
+      <x:c r="F428" s="9" t="str"/>
+      <x:c r="G428" s="9" t="str"/>
+      <x:c r="H428" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I428" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J428" s="9" t="str">
+        <x:v>actuator/motor/gear/internal diagnosis</x:v>
+      </x:c>
+      <x:c r="K428" s="9" t="str">
+        <x:v>drivetrain service</x:v>
+      </x:c>
+      <x:c r="L428" s="9" t="str"/>
+      <x:c r="M428" s="9" t="str"/>
+      <x:c r="N428" s="41" t="str"/>
+    </x:row>
+    <x:row r="429" ht="396" hidden="0" customHeight="1">
+      <x:c r="A429" s="40" t="n">
+        <x:v>297</x:v>
+      </x:c>
+      <x:c r="B429" s="9" t="str">
+        <x:v>bmw-x3-transfer-case-actuator-2011</x:v>
+      </x:c>
+      <x:c r="C429" s="9" t="str">
+        <x:v>2011-2026 | BMW | X3</x:v>
+      </x:c>
+      <x:c r="D429" s="9" t="str">
+        <x:v>Transfer Case Actuator Motor Failure</x:v>
+      </x:c>
+      <x:c r="E429" s="9" t="str">
+        <x:v>Replace the transfer case actuator motor. Change the transfer case fluid at the same time. The actuator can be replaced without removing the entire transfer case. Rebuilt units are available at lower cost but OEM is recommended for reliability.</x:v>
+      </x:c>
+      <x:c r="F429" s="9" t="str">
+        <x:v>Generation/unit-specific xDrive diagnosis; exact actuator only if confirmed; internal transfer-case inspection; correct fluid service</x:v>
+      </x:c>
+      <x:c r="G429" s="9" t="str">
+        <x:v>GENERATION / UNIT GATE</x:v>
+      </x:c>
+      <x:c r="H429" s="9" t="str">
+        <x:v>BMW X3 transfer-case catalog</x:v>
+      </x:c>
+      <x:c r="I429" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x3-transfer_case.html</x:v>
+      </x:c>
+      <x:c r="J429" s="9" t="str">
+        <x:v>2011-2026 F25/G01/G45 xDrive; VIN and transfer-case unit required</x:v>
+      </x:c>
+      <x:c r="K429" s="9" t="str">
+        <x:v>OEM drivetrain catalog</x:v>
+      </x:c>
+      <x:c r="L429" s="9" t="str"/>
+      <x:c r="M429" s="9" t="str">
+        <x:v>The row crosses at least three generations and cannot support one actuator or fluid.</x:v>
+      </x:c>
+      <x:c r="N429" s="41" t="str">
+        <x:v>Do not claim the actuator always replaces without transfer-case removal or that rebuilt units are universally inferior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="430" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A430" s="40" t="str"/>
+      <x:c r="B430" s="9" t="str"/>
+      <x:c r="C430" s="9" t="str"/>
+      <x:c r="D430" s="9" t="str"/>
+      <x:c r="E430" s="9" t="str"/>
+      <x:c r="F430" s="9" t="str"/>
+      <x:c r="G430" s="9" t="str"/>
+      <x:c r="H430" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I430" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J430" s="9" t="str">
+        <x:v>xDrive diagnosis and fluid/service functions</x:v>
+      </x:c>
+      <x:c r="K430" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L430" s="9" t="str"/>
+      <x:c r="M430" s="9" t="str"/>
+      <x:c r="N430" s="41" t="str"/>
+    </x:row>
+    <x:row r="431" ht="871.2000122070312" hidden="0" customHeight="1">
+      <x:c r="A431" s="40" t="n">
+        <x:v>298</x:v>
+      </x:c>
+      <x:c r="B431" s="9" t="str">
+        <x:v>bmw-x3-valve-cover-gasket-2004</x:v>
+      </x:c>
+      <x:c r="C431" s="9" t="str">
+        <x:v>2004-2017 | BMW | X3 | 2.5i, 3.0i, 3.0si | M54, N52</x:v>
+      </x:c>
+      <x:c r="D431" s="9" t="str">
+        <x:v>Valve Cover Gasket Oil Leaks (M54, N52 Engines)</x:v>
+      </x:c>
+      <x:c r="E431" s="9" t="str">
+        <x:v>Replace valve cover gasket and VANOS solenoid o-rings ($300-500 independent shop, $700-1,000 dealer, $80-150 DIY parts). On M54 engines, also replace ignition coil boots if contaminated by oil ($50 additional). Use OEM BMW gasket or Victor Reinz brand - aftermarket quality matters for long-term seal. Relatively straightforward DIY repair - saves $200-400 in labor. YouTube and Bimmerfest have detailed model-specific guides. Monitor oil level weekly and top off as needed (1 quart low is OK, 2+ quarts low risks engine damage).</x:v>
+      </x:c>
+      <x:c r="F431" s="9" t="str">
+        <x:v>Split M54 and N52 engines/model years; valve-cover gasket; cover/PCV by condition; coil boots only if oil-damaged; VANOS O-rings only if leaking</x:v>
+      </x:c>
+      <x:c r="G431" s="9" t="str">
+        <x:v>SOURCE RANGE / ENGINE CORRECTION</x:v>
+      </x:c>
+      <x:c r="H431" s="9" t="str">
+        <x:v>BMW X3 valve-cover gasket catalog</x:v>
+      </x:c>
+      <x:c r="I431" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/X3/Valve-Cover-Gasket/</x:v>
+      </x:c>
+      <x:c r="J431" s="9" t="str">
+        <x:v>E83/F25 X3; select exact M54 or N52 engine and VIN</x:v>
+      </x:c>
+      <x:c r="K431" s="9" t="str">
+        <x:v>engine-specific gasket catalog</x:v>
+      </x:c>
+      <x:c r="L431" s="9" t="str"/>
+      <x:c r="M431" s="9" t="str">
+        <x:v>The title names M54/N52 but the 2004-2017 range reaches other engines; VANOS O-rings and coil boots are conditional.</x:v>
+      </x:c>
+      <x:c r="N431" s="41" t="str">
+        <x:v>Narrow/split the years by engine, do not bundle unrelated VANOS seals, and remove unsafe 'one quart low is OK' guidance.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="432" ht="409.20001220703125" hidden="0" customHeight="1">
+      <x:c r="A432" s="40" t="n">
+        <x:v>299</x:v>
+      </x:c>
+      <x:c r="B432" s="9" t="str">
+        <x:v>bmw-x3-valve-cover-gasket-2011</x:v>
+      </x:c>
+      <x:c r="C432" s="9" t="str">
+        <x:v>2011-2022 | BMW | X3 | N20, B48</x:v>
+      </x:c>
+      <x:c r="D432" s="9" t="str">
+        <x:v>Valve Cover Gasket Oil Leak</x:v>
+      </x:c>
+      <x:c r="E432" s="9" t="str">
+        <x:v>Replace the valve cover gasket. Inspect the valve cover for warping or cracks — if damaged, replace the entire cover assembly. Clean all oil residue from surrounding components. Use a torque wrench to prevent over-tightening which causes cover warping.</x:v>
+      </x:c>
+      <x:c r="F432" s="9" t="str">
+        <x:v>Engine/VIN-specific leak diagnosis; gasket if cover serviceable; complete warped/cracked cover; PCV branch; cleanup and correct torque procedure</x:v>
+      </x:c>
+      <x:c r="G432" s="9" t="str">
+        <x:v>ENGINE / COVER-CONDITION GATE</x:v>
+      </x:c>
+      <x:c r="H432" s="9" t="str">
+        <x:v>BMW X3 valve-cover catalog</x:v>
+      </x:c>
+      <x:c r="I432" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/X3/Valve-Cover/</x:v>
+      </x:c>
+      <x:c r="J432" s="9" t="str">
+        <x:v>2011-2022 F25/G01 X3; select exact engine, VIN, gasket/cover branch</x:v>
+      </x:c>
+      <x:c r="K432" s="9" t="str">
+        <x:v>vehicle-specific cover catalog</x:v>
+      </x:c>
+      <x:c r="L432" s="9" t="str"/>
+      <x:c r="M432" s="9" t="str">
+        <x:v>The range spans multiple engines/covers; the source correctly makes the complete cover conditional on damage.</x:v>
+      </x:c>
+      <x:c r="N432" s="41" t="str">
+        <x:v>Do not attach one cover or gasket across N20/N52/N55/B-series engines.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="433" ht="858" hidden="0" customHeight="1">
+      <x:c r="A433" s="40" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="B433" s="9" t="str">
+        <x:v>bmw-x3-vanos-solenoid-2007</x:v>
+      </x:c>
+      <x:c r="C433" s="9" t="str">
+        <x:v>2007-2017 | BMW | X3 | M40i, M50, xDrive35i | N52, N55</x:v>
+      </x:c>
+      <x:c r="D433" s="9" t="str">
+        <x:v>VANOS Solenoid Failure (N52, N55 Engines)</x:v>
+      </x:c>
+      <x:c r="E433" s="9" t="str">
+        <x:v>Replace VANOS solenoids and seals ($250-400 European shops, $729-882 US average). Use high-quality oil (5W-30 or 0W-40 BMW LL-01 spec) and change every 5,000-7,000 miles to prevent future failures - cheap oil or extended intervals kill VANOS solenoids. Some cases may require complete VANOS unit rebuild ($1,500-2,500). PREVENTIVE: Replace VANOS solenoids and seals every 50k miles as maintenance - much cheaper than waiting for failure. On F25 X3 with N52/N55, check TSB SI B12 14 10 for VANOS gear assembly bolt issue.</x:v>
+      </x:c>
+      <x:c r="F433" s="9" t="str">
+        <x:v>Split N52 and N55 VANOS systems; BMW-capable diagnosis; affected intake/exhaust solenoid/seals; VIN campaign check where applicable; full VANOS only after confirmation</x:v>
+      </x:c>
+      <x:c r="G433" s="9" t="str">
+        <x:v>ENGINE / POSITION / CAMPAIGN SPLIT</x:v>
+      </x:c>
+      <x:c r="H433" s="9" t="str">
+        <x:v>BMW recall lookup</x:v>
+      </x:c>
+      <x:c r="I433" s="9" t="str">
+        <x:v>https://www.bmwusa.com/safety-and-emission-recalls.html</x:v>
+      </x:c>
+      <x:c r="J433" s="9" t="str">
+        <x:v>VIN check for applicable VANOS gear-bolt campaign</x:v>
+      </x:c>
+      <x:c r="K433" s="9" t="str">
+        <x:v>manufacturer campaign route</x:v>
+      </x:c>
+      <x:c r="L433" s="9" t="str"/>
+      <x:c r="M433" s="9" t="str">
+        <x:v>N52/N55 and campaign repairs cannot be combined into one solenoid replacement rule.</x:v>
+      </x:c>
+      <x:c r="N433" s="41" t="str">
+        <x:v>Remove fixed preventive replacement and oil-interval claims; no generic scanner link without BMW VANOS coverage.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="434" ht="132" hidden="0" customHeight="1">
+      <x:c r="A434" s="42" t="str"/>
+      <x:c r="B434" s="43" t="str"/>
+      <x:c r="C434" s="43" t="str"/>
+      <x:c r="D434" s="43" t="str"/>
+      <x:c r="E434" s="43" t="str"/>
+      <x:c r="F434" s="43" t="str"/>
+      <x:c r="G434" s="43" t="str"/>
+      <x:c r="H434" s="43" t="str">
+        <x:v>BMW X3 VANOS catalog</x:v>
+      </x:c>
+      <x:c r="I434" s="43" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/X3/VANOS-Solenoid/</x:v>
+      </x:c>
+      <x:c r="J434" s="43" t="str">
+        <x:v>2007-2017 X3; select N52/N55, intake/exhaust, VIN, and diagnosed component</x:v>
+      </x:c>
+      <x:c r="K434" s="43" t="str">
+        <x:v>engine-specific VANOS catalog</x:v>
+      </x:c>
+      <x:c r="L434" s="43" t="str"/>
+      <x:c r="M434" s="43" t="str"/>
+      <x:c r="N434" s="44" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -15256,21 +16618,21 @@
         <x:v>Queue status</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="448.79998779296875" hidden="0" customHeight="1">
+    <x:row r="2" ht="1016.4000244140625" hidden="0" customHeight="1">
       <x:c r="A2" s="40" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>bmw-x1-transfer-case-actuator-2013</x:v>
+        <x:v>bmw-x3-wastegate-rattle-2011</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>2013-2022 | BMW | X1</x:v>
+        <x:v>2011-2023 | BMW | X3 | M40i, M50, sDrive30i, xDrive28i, xDrive30i, xDrive35i</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
-        <x:v>Transfer Case Actuator Motor Failure</x:v>
+        <x:v>Turbocharger Wastegate Rattle (N55, N20, B58 Engines)</x:v>
       </x:c>
       <x:c r="E2" s="9" t="str">
-        <x:v>Replace the transfer case actuator motor (also called the servo motor). The transfer case itself usually does not need replacement. Ensure the transfer case fluid is changed at the same time. Some owners report success with rebuilt actuators at lower cost.</x:v>
+        <x:v>Replace wastegate actuator ($400-800) or use aftermarket wastegate repair kit with upgraded stainless steel bushings ($150-300). Some cases require complete turbocharger replacement ($2,000-$4,000). VTT (Vargas Turbo Technologies) repair kits popular on forums - upgraded materials prevent future rattle. MONITORING: Early wastegate rattle may be harmless (annoying but no performance loss). If car boosts normally and no underboost codes, can monitor rattle without urgent repair. However, if check engine light appears with code 30FF or boost pressure drops, repair immediately to prevent turbo damage.</x:v>
       </x:c>
       <x:c r="F2" s="9" t="n">
         <x:v>0</x:v>
@@ -15279,21 +16641,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="382.79998779296875" hidden="0" customHeight="1">
+    <x:row r="3" ht="778.7999877929688" hidden="0" customHeight="1">
       <x:c r="A3" s="40" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>bmw-x2-b48-timing-chain-tensioner-2018</x:v>
+        <x:v>bmw-x3-water-pump-2007</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
-        <x:v>2018-2023 | BMW | X2 | B48</x:v>
+        <x:v>2007-2017 | BMW | X3 | sDrive30i, xDrive28i, xDrive30i | N52, N20</x:v>
       </x:c>
       <x:c r="D3" s="9" t="str">
-        <x:v>B48 Timing Chain Tensioner Weakness</x:v>
+        <x:v>Electric Water Pump Failure (N52, N20 Engines)</x:v>
       </x:c>
       <x:c r="E3" s="9" t="str">
-        <x:v>Replace the timing chain tensioner and inspect the chain and guides. If the chain has stretched beyond specification, replace the full timing chain kit. Updated tensioner design from BMW addresses the oil pressure retention issue.</x:v>
+        <x:v>Replace electric water pump at first sign of failure ($800 parts + labor). Consider preventative replacement at 70-80k miles to avoid being stranded ($400 parts, DIY-able). CRITICAL: If you own 2013-2017 X3 28i, verify recall repair (protective shield installation) has been completed to prevent fire risk - check with BMW dealer using VIN. If engine overheats, PULL OVER IMMEDIATELY and shut off - driving with overheating warps cylinder heads ($4,000+ repair). Call tow truck.</x:v>
       </x:c>
       <x:c r="F3" s="9" t="n">
         <x:v>0</x:v>
@@ -15302,21 +16664,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="580.7999877929688" hidden="0" customHeight="1">
+    <x:row r="4" ht="1240.800048828125" hidden="0" customHeight="1">
       <x:c r="A4" s="40" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>bmw-x2-crankshaft-sensor-recall-2018</x:v>
+        <x:v>bmw-x3m-brake-wear-2020</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>2018-2018 | BMW | X2</x:v>
+        <x:v>2020-2023 | BMW | X3 M | S58</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
-        <x:v>2018 X2 Crankshaft Sensor Safety Recall 18V-465</x:v>
+        <x:v>Accelerated Brake Pad &amp; Rotor Wear from Vehicle Weight - F97 X3 M / F98 X4 M</x:v>
       </x:c>
       <x:c r="E4" s="9" t="str">
-        <x:v>Check the VIN for an open 18V-465 campaign. If open, an authorized BMW dealer replaces the crankshaft sensor free of charge. A stall or sudden loss of power requires moving to a safe location and arranging BMW assistance; do not order a sensor from this card. ShowMeTheParts resolved exact X2 category fitment only, so no commerce link is approved.</x:v>
+        <x:v>Front brake replacement: OEM front rotor (34118054825 left, matching right) with OEM M compound pads. Complete OEM front brake kit available from BimmerWorld (34108064561K1, ~$800-$1,000). Rear brake kit similarly priced. For track use: Upgrade to Brembo GT brake pad set (BM8 compound) for improved heat resistance and longer pad life. EBC Yellowstuff or Hawk HPS 5.0 pads are popular street/track compromise choices ($150-$250 per axle). StopTech slotted rotors offer improved heat dissipation. For dedicated track cars: Brembo GT big brake kit with 412x38mm discs available ($4,000-$6,000 installed). Budget $2,000-$3,000 per year for brake maintenance if driving spiritedly. Use high-temperature brake fluid (Motul RBF 660 or ATE Typ 200) and flush every 12 months.</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
         <x:v>0</x:v>
@@ -15325,21 +16687,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="382.79998779296875" hidden="0" customHeight="1">
+    <x:row r="5" ht="1188" hidden="0" customHeight="1">
       <x:c r="A5" s="40" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>bmw-x2-front-control-arm-bushings-2018</x:v>
+        <x:v>bmw-x3m-cooling-track-use-2020</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>2018-2023 | BMW | X2</x:v>
+        <x:v>2020-2023 | BMW | X3 M | S58</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Front Control Arm Bushing Premature Wear</x:v>
+        <x:v>Cooling System Heat Soak During Track/Spirited Driving - F97 X3 M / F98 X4 M</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>Replace front control arms with new bushings (sold as complete assemblies by BMW). Aftermarket options with upgraded polyurethane bushings are available for longer life. Perform a four-wheel alignment after replacement.</x:v>
+        <x:v>For track use: Upgrade intercooler to do88 front-mount intercooler ($1,200-$1,800) - the community standard for S58 heat management. Add CSF high-performance radiator ($600-$900) for sustained track work. Dinan or VRSF also offer intercooler upgrades in the $1,000-$1,500 range. For street/canyon driving: Stock cooling is adequate but ensure coolant flush every 2 years/30,000 miles and inspect expansion tank for cracks. Replace coolant expansion tank preemptively at 60,000 miles if car is driven hard. For all X3 M/X4 M: Use BMW coolant only (mixed 50/50 with distilled water), replace thermostat at 80,000 miles preventatively, inspect all coolant hoses for bulging or softening at every oil change.</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
         <x:v>0</x:v>
@@ -15348,21 +16710,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="831.5999755859375" hidden="0" customHeight="1">
+    <x:row r="6" ht="1214.4000244140625" hidden="0" customHeight="1">
       <x:c r="A6" s="40" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>bmw-x2-oil-filter-housing-2018</x:v>
+        <x:v>bmw-x3m-differential-bolt-2020</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
-        <x:v>2018-2023 | BMW | X2 | sDrive28i, xDrive28i | B48</x:v>
+        <x:v>2020-2023 | BMW | X3 M | S58</x:v>
       </x:c>
       <x:c r="D6" s="9" t="str">
-        <x:v>B48 Oil Filter Housing Gasket Leak/Cracking</x:v>
+        <x:v>Rear Differential Mounting Bolt &amp; Bush Failure - F97 X3 M / F98 X4 M</x:v>
       </x:c>
       <x:c r="E6" s="9" t="str">
-        <x:v>Replace the cracked oil filter housing. OEM plastic housing replacement (BMW 11428596283, $412 dealer) will eventually crack again. RECOMMENDED: Install aftermarket aluminum upgrade housing ($250-350) which permanently eliminates the heat-cycling crack issue. FCP Euro kit 11428596283KT ($450) includes all gaskets and seals. If coolant and oil have mixed, perform complete oil flush and coolant system flush before installing new housing. Check for engine damage if contamination was prolonged.</x:v>
+        <x:v>Replace factory differential bolt, bush, and collar with FJ Motorwerkes uprated diff bolt and collar upgrade kit. The FJ kit uses premium CNC-machined stainless steel components that can handle 170,000 PSI (39% stronger than BMW's revised bolt). Kit price approximately $255 (GBP). Available from FJ Motorwerkes directly, BMG Performance, AM Tuning, and H4ck Performance. Installation is straightforward - rear differential does not need to be fully removed. Budget $400-$600 total including labor. This upgrade is considered MANDATORY by the X3 M/X4 M community for any car making stock or above power. JXB Performance also offers a driveshaft carrier bearing upgrade for cars experiencing propshaft vibration as a companion fix.</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
         <x:v>0</x:v>
@@ -15371,21 +16733,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="330" hidden="0" customHeight="1">
+    <x:row r="7" ht="1293.5999755859375" hidden="0" customHeight="1">
       <x:c r="A7" s="40" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>bmw-x2-oil-filter-housing-gasket-2018</x:v>
+        <x:v>bmw-x3m-s58-bearing-recall-2020</x:v>
       </x:c>
       <x:c r="C7" s="9" t="str">
-        <x:v>2018-2023 | BMW | X2 | B48</x:v>
+        <x:v>2020-2021 | BMW | X3 M</x:v>
       </x:c>
       <x:c r="D7" s="9" t="str">
-        <x:v>Oil Filter Housing Gasket Leak</x:v>
+        <x:v>S58 Engine Main Bearing Shell Recall / Stop Sale - F97 X3 M / F98 X4 M</x:v>
       </x:c>
       <x:c r="E7" s="9" t="str">
-        <x:v>Replace the oil filter housing gasket. Clean all oil-contaminated surfaces and inspect the serpentine belt for oil damage. Replace belt if oil-soaked. Use OEM-quality gasket material for longevity.</x:v>
+        <x:v>Check VIN immediately against BMW recall database at bmwusa.com or contact your BMW dealer. If your vehicle is within the affected production date range, BMW will inspect and replace main bearing shells at no cost under the Tech Campaign. The repair requires removing the cylinder head and oil pan to access and replace all main bearing shells - this is a major repair (8-12 hours labor) but fully covered by BMW. Do NOT drive the vehicle if knocking is present. For S58 vehicles outside the recall range: Proactive rod bearing inspection is recommended at 60,000 miles for track-driven vehicles. ACL Race Series rod bearings 6B1510H-STD are the aftermarket upgrade choice on Bimmerpost for preventive replacement ($150-$250 for bearing set, $3,000-$5,000 total with labor).</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
         <x:v>0</x:v>
@@ -15394,21 +16756,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="448.79998779296875" hidden="0" customHeight="1">
+    <x:row r="8" ht="1227.5999755859375" hidden="0" customHeight="1">
       <x:c r="A8" s="40" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>bmw-x2-tie-rod-recall-2019</x:v>
+        <x:v>bmw-x3m-transfer-case-2020</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
-        <x:v>2019-2019 | BMW | X2</x:v>
+        <x:v>2020-2023 | BMW | X3 M | S58</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
-        <x:v>2019 X2 Steering Tie-Rod Safety Recall 19V-601</x:v>
+        <x:v>xDrive Transfer Case Stress &amp; Fluid Degradation - F97 X3 M / F98 X4 M</x:v>
       </x:c>
       <x:c r="E8" s="9" t="str">
-        <x:v>Check the VIN in BMW AIR or NHTSA for an open 19V-601 campaign. If open, an authorized BMW dealer checks both tie rods and replaces the tie rods and ball joints as necessary free of charge. Do not infer recall eligibility from model year alone or order steering parts from this card.</x:v>
+        <x:v>Change transfer case fluid every 30,000 miles (BMW says "lifetime fill" - this is NOT correct for M vehicles driven hard). Use BMW DTF-1 transfer case fluid or equivalent high-quality synthetic. Check tire tread depth at every service - all 4 tires must be within 2/32" of each other to prevent transfer case stress. Rotate tires every 5,000-7,000 miles. If transfer case actuator motor fails: FCP Euro guide for BMW transfer case actuator repair (part number varies by production date, ~$300-$600). For tuned cars: Consider transfer case brace/reinforcement and shortened fluid change intervals (every 15,000 miles). Complete transfer case replacement if internals are damaged: $3,000-$5,500 at independent specialist, $5,000-$8,000+ at dealer.</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
         <x:v>0</x:v>
@@ -15417,21 +16779,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="646.7999877929688" hidden="0" customHeight="1">
+    <x:row r="9" ht="673.2000122070312" hidden="0" customHeight="1">
       <x:c r="A9" s="40" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>bmw-x2-transmission-jerking-2018</x:v>
+        <x:v>bmw-x4-n20-timing-chain-2015</x:v>
       </x:c>
       <x:c r="C9" s="9" t="str">
-        <x:v>2018-2020 | BMW | X2</x:v>
+        <x:v>2015-2016 | BMW | X4 | xDrive28i, xDrive30i</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str">
-        <x:v>Aisin 8-Speed Transmission Jerking</x:v>
+        <x:v>N20 Timing Chain Premature Failure - F26 X4 xDrive28i</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
-        <x:v>Start with transmission software recalibration at BMW dealer ($200-500) which may resolve calibration-related shifting issues. If software update does not resolve, transmission may require oil pump replacement or internal repair ($2,000-5,000). In severe cases with extensive oil pump neck wear, complete transmission replacement required ($5,000-7,000). Reference TSB GBSEL-SELP24 when visiting dealer.</x:v>
+        <x:v>Complete timing chain kit replacement including chain, guides, tensioner, and sprockets. Must be performed by experienced BMW technician. Preventive replacement recommended at 60,000-80,000 miles. BMW extended warranty to 8 years/100,000 miles under class action settlement. Upgraded reinforced chain kit available from aftermarket. Labor is 10-14 hours for X4 due to AWD and tight engine bay.</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
         <x:v>0</x:v>
@@ -15440,21 +16802,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="580.7999877929688" hidden="0" customHeight="1">
+    <x:row r="10" ht="686.4000244140625" hidden="0" customHeight="1">
       <x:c r="A10" s="40" t="n">
         <x:v>9</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>bmw-x2-valve-cover-gasket-2018</x:v>
+        <x:v>bmw-x4-n20-timing-chain-guide-2015</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
-        <x:v>2018-2023 | BMW | X2</x:v>
+        <x:v>2015-2015 | BMW | X4 | N20</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
-        <x:v>Valve Cover Gasket Oil Leak</x:v>
+        <x:v>2015 X4 N20 Lower-Engine Whine Requires Timing-Chain Diagnosis</x:v>
       </x:c>
       <x:c r="E10" s="9" t="str">
-        <x:v>Replace valve cover gasket. Genuine BMW valve cover assembly 11127611278 ($200-350) includes integrated gasket. Labor typically 2-3 hours ($300-500). Total cost $700-1,000 at shop. DIY possible with basic tools to save $300-500 in labor. Replace spark plug tube seals at same time if applicable - labor overlap saves money. Monitor oil level between repairs.</x:v>
+        <x:v>Confirm the exact xDrive28i variant, N20 engine, production date and VIN eligibility, then have a BMW-qualified technician reproduce the noise and follow current BMW diagnosis before replacing anything. The historical seven-year/70,000-mile coverage was a limited warranty extension, not a recall, and is not a current coverage promise. ShowMeTheParts established category-level fitment only, so no commerce link is approved.</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
         <x:v>0</x:v>
@@ -15463,21 +16825,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="990" hidden="0" customHeight="1">
+    <x:row r="11" ht="554.4000244140625" hidden="0" customHeight="1">
       <x:c r="A11" s="40" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>bmw-x3-coolant-expansion-tank-2004</x:v>
+        <x:v>bmw-x4-oil-leak-2015</x:v>
       </x:c>
       <x:c r="C11" s="9" t="str">
-        <x:v>2004-2023 | BMW | X3</x:v>
+        <x:v>2015-2023 | BMW | X4</x:v>
       </x:c>
       <x:c r="D11" s="9" t="str">
-        <x:v>Coolant Expansion Tank Cracking</x:v>
+        <x:v>Oil Leaks - Valve Cover &amp; Oil Filter Housing - All Models</x:v>
       </x:c>
       <x:c r="E11" s="9" t="str">
-        <x:v>Replace expansion tank and coolant ($50-100 DIY parts, $200-400 independent shop, $400-580 dealer). Very simple DIY repair taking 30 minutes - drain coolant, unbolt old tank, install new tank, refill with BMW-spec coolant (blue or pink/orange premix). Use Behr or OEM BMW expansion tank - Dorman aftermarket tanks may fail prematurely. YouTube and Pelicanparts have detailed DIY guides. PREVENTIVE: Replace every 5-7 years or 80-100k miles before cracks develop. Check tank regularly for hairline cracks. Don't ignore coolant leaks - can lead to catastrophic overheating and head gasket failure.</x:v>
+        <x:v>Replace valve cover gasket and/or oil filter housing gasket. Valve cover replacement is 3-4 hours labor on X4. Oil filter housing gasket is 1-2 hours. Both are routine maintenance items on BMW turbo engines. Use OEM gaskets for best longevity. Clean oil residue from engine bay after repair. Monitor oil level regularly to catch leaks early.</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
         <x:v>0</x:v>
@@ -15486,44 +16848,44 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="435.6000061035156" hidden="0" customHeight="1">
+    <x:row r="12" ht="356.3999938964844" hidden="0" customHeight="1">
       <x:c r="A12" s="40" t="n">
         <x:v>11</x:v>
       </x:c>
       <x:c r="B12" s="9" t="str">
-        <x:v>bmw-x3-electric-water-pump-2011</x:v>
+        <x:v>bmw-x4-rear-differential-mount-2015</x:v>
       </x:c>
       <x:c r="C12" s="9" t="str">
-        <x:v>2011-2026 | BMW | X3</x:v>
+        <x:v>2015-2023 | BMW | X4</x:v>
       </x:c>
       <x:c r="D12" s="9" t="str">
-        <x:v>Electric Water Pump Failure</x:v>
+        <x:v>Rear Differential Mount Bushing Failure</x:v>
       </x:c>
       <x:c r="E12" s="9" t="str">
-        <x:v>Replace the electric water pump and thermostat together, as they are part of the same cooling circuit and the thermostat often fails concurrently. Bleed the cooling system thoroughly after replacement. Some owners carry a spare pump due to the sudden failure nature.</x:v>
+        <x:v>Replace rear differential mount bushings. Both front and rear differential bushings should be inspected and replaced as a set. Upgraded aftermarket bushings with stiffer rubber or polyurethane are available for longer service life.</x:v>
       </x:c>
       <x:c r="F12" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G12" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="541.2000122070312" hidden="0" customHeight="1">
+    <x:row r="13" ht="620.4000244140625" hidden="0" customHeight="1">
       <x:c r="A13" s="40" t="n">
         <x:v>12</x:v>
       </x:c>
       <x:c r="B13" s="9" t="str">
-        <x:v>bmw-x3-m-electric-wastegate-actuator-adaptation-fault-boost-cutout-ea</x:v>
+        <x:v>bmw-x4-transfer-case-2015</x:v>
       </x:c>
       <x:c r="C13" s="9" t="str">
-        <x:v>2020-2020 | BMW | X3 M | S58</x:v>
+        <x:v>2015-2023 | BMW | X4</x:v>
       </x:c>
       <x:c r="D13" s="9" t="str">
-        <x:v>2020 X3 M Wastegate Adaptation Faults Require Software Diagnosis</x:v>
+        <x:v>Transfer Case Actuator Motor Failure - All xDrive X4</x:v>
       </x:c>
       <x:c r="E13" s="9" t="str">
-        <x:v>Confirm the production date, fault codes and current vehicle integration level. If the I-level is below S15A-20-03-510, a BMW-qualified repairer follows the bulletin and programs the vehicle with the specified or newer approved ISTA level. Diagnose unrelated mechanical noise separately; do not replace an actuator or turbocharger from this card.</x:v>
+        <x:v>Diagnose specific failure. Transfer case actuator motor replacement ($800-1,200) is most common. Complete transfer case replacement required for internal failures ($2,500-4,000). Regular transfer case fluid changes every 50,000 miles may extend life. Some owners install aftermarket upgraded actuator motors. Common wear item on high-mileage xDrive BMW models.</x:v>
       </x:c>
       <x:c r="F13" s="9" t="n">
         <x:v>0</x:v>
@@ -15532,21 +16894,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="462" hidden="0" customHeight="1">
+    <x:row r="14" ht="1240.800048828125" hidden="0" customHeight="1">
       <x:c r="A14" s="40" t="n">
         <x:v>13</x:v>
       </x:c>
       <x:c r="B14" s="9" t="str">
-        <x:v>bmw-x3-m-fuel-tank-inlet-check-valve-weld-failure-2021-x3-m</x:v>
+        <x:v>bmw-x4m-brake-wear-2020</x:v>
       </x:c>
       <x:c r="C14" s="9" t="str">
-        <x:v>2021-2021 | BMW | X3 M</x:v>
+        <x:v>2020-2023 | BMW | X4 M | S58</x:v>
       </x:c>
       <x:c r="D14" s="9" t="str">
-        <x:v>2021 X3 M Fuel-Tank Safety Recall 21V-199</x:v>
+        <x:v>Accelerated Brake Pad &amp; Rotor Wear from Vehicle Weight - F98 X4 M / F98 X4 M</x:v>
       </x:c>
       <x:c r="E14" s="9" t="str">
-        <x:v>Check the VIN for an open 21V-199 campaign. If open, an authorized BMW dealer replaces the fuel tank free of charge. If fuel odor or leakage appears, move safely away from traffic, stop, have occupants exit and contact BMW roadside assistance; do not continue driving or order a tank from this card.</x:v>
+        <x:v>Front brake replacement: OEM front rotor (34118054825 left, matching right) with OEM M compound pads. Complete OEM front brake kit available from BimmerWorld (34108064561K1, ~$800-$1,000). Rear brake kit similarly priced. For track use: Upgrade to Brembo GT brake pad set (BM8 compound) for improved heat resistance and longer pad life. EBC Yellowstuff or Hawk HPS 5.0 pads are popular street/track compromise choices ($150-$250 per axle). StopTech slotted rotors offer improved heat dissipation. For dedicated track cars: Brembo GT big brake kit with 412x38mm discs available ($4,000-$6,000 installed). Budget $2,000-$3,000 per year for brake maintenance if driving spiritedly. Use high-temperature brake fluid (Motul RBF 660 or ATE Typ 200) and flush every 12 months.</x:v>
       </x:c>
       <x:c r="F14" s="9" t="n">
         <x:v>0</x:v>
@@ -15555,21 +16917,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="580.7999877929688" hidden="0" customHeight="1">
+    <x:row r="15" ht="1188" hidden="0" customHeight="1">
       <x:c r="A15" s="40" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="B15" s="9" t="str">
-        <x:v>bmw-x3-m-idrive-control-display-blank-screen-infotainment-glitches-f9</x:v>
+        <x:v>bmw-x4m-cooling-track-use-2020</x:v>
       </x:c>
       <x:c r="C15" s="9" t="str">
-        <x:v>2020-2021 | BMW | X3 M | X3 M, X3 M Competition | S58, S58B30</x:v>
+        <x:v>2020-2023 | BMW | X4 M</x:v>
       </x:c>
       <x:c r="D15" s="9" t="str">
-        <x:v>iDrive Control Display Blank Screen and Infotainment Glitches - F97 X3 M (2019-2021)</x:v>
+        <x:v>Cooling System Heat Soak During Track/Spirited Driving - F98 X4 M / F98 X4 M</x:v>
       </x:c>
       <x:c r="E15" s="9" t="str">
-        <x:v>First try the latest iDrive/head-unit software update at the dealer, which resolves many of the early glitches, reboots, and camera issues. If the display panel hardware has failed (lines, persistent blank screen with backlight off), the control display/screen assembly is replaced. A soft reset (press-and-hold volume/power) can temporarily clear a frozen screen.</x:v>
+        <x:v>For track use: Upgrade intercooler to do88 front-mount intercooler ($1,200-$1,800) - the community standard for S58 heat management. Add CSF high-performance radiator ($600-$900) for sustained track work. Dinan or VRSF also offer intercooler upgrades in the $1,000-$1,500 range. For street/canyon driving: Stock cooling is adequate but ensure coolant flush every 2 years/30,000 miles and inspect expansion tank for cracks. Replace coolant expansion tank preemptively at 60,000 miles if car is driven hard. For all X3 M/X4 M: Use BMW coolant only (mixed 50/50 with distilled water), replace thermostat at 80,000 miles preventatively, inspect all coolant hoses for bulging or softening at every oil change.</x:v>
       </x:c>
       <x:c r="F15" s="9" t="n">
         <x:v>0</x:v>
@@ -15578,21 +16940,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="462" hidden="0" customHeight="1">
+    <x:row r="16" ht="1214.4000244140625" hidden="0" customHeight="1">
       <x:c r="A16" s="40" t="n">
         <x:v>15</x:v>
       </x:c>
       <x:c r="B16" s="9" t="str">
-        <x:v>bmw-x3-m-improperly-welded-front-seat-frame-2019-2021-x3-m</x:v>
+        <x:v>bmw-x4m-differential-bolt-2020</x:v>
       </x:c>
       <x:c r="C16" s="9" t="str">
-        <x:v>2021-2021 | BMW | X3 M</x:v>
+        <x:v>2020-2023 | BMW | X4 M</x:v>
       </x:c>
       <x:c r="D16" s="9" t="str">
-        <x:v>2021 X3 M Front Seat-Frame Safety Recall 23V-211</x:v>
+        <x:v>Rear Differential Mounting Bolt &amp; Bush Failure - F98 X4 M / F98 X4 M</x:v>
       </x:c>
       <x:c r="E16" s="9" t="str">
-        <x:v>Check the VIN for an open 23V-211 campaign. If open, an authorized BMW dealer replaces the affected front seat frame and backrest free of charge using VIN-selected parts. Contact BMW promptly if a front seat vibrates or makes abnormal noise; do not order seat components from this card.</x:v>
+        <x:v>Replace factory differential bolt, bush, and collar with FJ Motorwerkes uprated diff bolt and collar upgrade kit. The FJ kit uses premium CNC-machined stainless steel components that can handle 170,000 PSI (39% stronger than BMW's revised bolt). Kit price approximately $255 (GBP). Available from FJ Motorwerkes directly, BMG Performance, AM Tuning, and H4ck Performance. Installation is straightforward - rear differential does not need to be fully removed. Budget $400-$600 total including labor. This upgrade is considered MANDATORY by the X3 M/X4 M community for any car making stock or above power. JXB Performance also offers a driveshaft carrier bearing upgrade for cars experiencing propshaft vibration as a companion fix.</x:v>
       </x:c>
       <x:c r="F16" s="9" t="n">
         <x:v>0</x:v>
@@ -15601,21 +16963,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="541.2000122070312" hidden="0" customHeight="1">
+    <x:row r="17" ht="1293.5999755859375" hidden="0" customHeight="1">
       <x:c r="A17" s="40" t="n">
         <x:v>16</x:v>
       </x:c>
       <x:c r="B17" s="9" t="str">
-        <x:v>bmw-x3-m-low-mounted-engine-oil-cooler-vulnerable-to-road-debris-punc</x:v>
+        <x:v>bmw-x4m-s58-bearing-recall-2020</x:v>
       </x:c>
       <x:c r="C17" s="9" t="str">
-        <x:v>2020-2023 | BMW | X3 M | X3 M, X3 M Competition | S58, S58B30</x:v>
+        <x:v>2020-2021 | BMW | X4 M | M40i, xDrive35i | S58</x:v>
       </x:c>
       <x:c r="D17" s="9" t="str">
-        <x:v>Low-Mounted Engine Oil Cooler Vulnerable to Road-Debris Puncture - F97 X3 M (S58)</x:v>
+        <x:v>S58 Engine Main Bearing Shell Recall / Stop Sale - F98 X4 M / F98 X4 M</x:v>
       </x:c>
       <x:c r="E17" s="9" t="str">
-        <x:v>Inspect the oil cooler periodically for stone damage and weeping; fit a protective mesh/guard in front of the cooler as preventive insurance (popular among track and spirited-use owners). If punctured, stop driving immediately and replace the oil cooler and refill with the correct oil; verify no bearing damage occurred from any oil starvation.</x:v>
+        <x:v>Check VIN immediately against BMW recall database at bmwusa.com or contact your BMW dealer. If your vehicle is within the affected production date range, BMW will inspect and replace main bearing shells at no cost under the Tech Campaign. The repair requires removing the cylinder head and oil pan to access and replace all main bearing shells - this is a major repair (8-12 hours labor) but fully covered by BMW. Do NOT drive the vehicle if knocking is present. For S58 vehicles outside the recall range: Proactive rod bearing inspection is recommended at 60,000 miles for track-driven vehicles. ACL Race Series rod bearings 6B1510H-STD are the aftermarket upgrade choice on Bimmerpost for preventive replacement ($150-$250 for bearing set, $3,000-$5,000 total with labor).</x:v>
       </x:c>
       <x:c r="F17" s="9" t="n">
         <x:v>0</x:v>
@@ -15624,21 +16986,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="594" hidden="0" customHeight="1">
+    <x:row r="18" ht="1227.5999755859375" hidden="0" customHeight="1">
       <x:c r="A18" s="40" t="n">
         <x:v>17</x:v>
       </x:c>
       <x:c r="B18" s="9" t="str">
-        <x:v>bmw-x3-m-oem-plastic-charge-pipe-cracking-blow-off-under-boost-f97-x3</x:v>
+        <x:v>bmw-x4m-transfer-case-2020</x:v>
       </x:c>
       <x:c r="C18" s="9" t="str">
-        <x:v>2020-2023 | BMW | X3 M | X3 M, X3 M Competition | S58, S58B30</x:v>
+        <x:v>2020-2023 | BMW | X4 M | S58</x:v>
       </x:c>
       <x:c r="D18" s="9" t="str">
-        <x:v>OEM Plastic Charge Pipe Cracking / Blow-Off Under Boost - F97 X3 M (S58)</x:v>
+        <x:v>xDrive Transfer Case Stress &amp; Fluid Degradation - F98 X4 M / F98 X4 M</x:v>
       </x:c>
       <x:c r="E18" s="9" t="str">
-        <x:v>Replace the OEM plastic charge pipe with an aluminum (or reinforced) aftermarket charge pipe from suppliers such as FTP, Racing Dynamics, or Kies; this is the standard durable fix and is strongly recommended before or alongside any tune. A failed OEM pipe can be re-fitted with a new OEM unit but the same failure mode tends to recur, especially on modified cars.</x:v>
+        <x:v>Change transfer case fluid every 30,000 miles (BMW says "lifetime fill" - this is NOT correct for M vehicles driven hard). Use BMW DTF-1 transfer case fluid or equivalent high-quality synthetic. Check tire tread depth at every service - all 4 tires must be within 2/32" of each other to prevent transfer case stress. Rotate tires every 5,000-7,000 miles. If transfer case actuator motor fails: FCP Euro guide for BMW transfer case actuator repair (part number varies by production date, ~$300-$600). For tuned cars: Consider transfer case brace/reinforcement and shortened fluid change intervals (every 15,000 miles). Complete transfer case replacement if internals are damaged: $3,000-$5,500 at independent specialist, $5,000-$8,000+ at dealer.</x:v>
       </x:c>
       <x:c r="F18" s="9" t="n">
         <x:v>0</x:v>
@@ -15647,21 +17009,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="382.79998779296875" hidden="0" customHeight="1">
+    <x:row r="19" ht="1042.800048828125" hidden="0" customHeight="1">
       <x:c r="A19" s="40" t="n">
         <x:v>18</x:v>
       </x:c>
       <x:c r="B19" s="9" t="str">
-        <x:v>bmw-x3-n20-timing-chain-2011</x:v>
+        <x:v>bmw-x5-air-suspension-2007</x:v>
       </x:c>
       <x:c r="C19" s="9" t="str">
-        <x:v>2011-2017 | BMW | X3 | N20</x:v>
+        <x:v>2019-2026 | BMW | X5</x:v>
       </x:c>
       <x:c r="D19" s="9" t="str">
-        <x:v>N20 Timing Chain Guide Failure</x:v>
+        <x:v>G05 Suspension Warning: Check Faults and Campaigns Before Parts</x:v>
       </x:c>
       <x:c r="E19" s="9" t="str">
-        <x:v>Replace the complete timing chain kit including chain, guides, tensioner, and sprockets. Preventive replacement is strongly recommended at 80,000 miles before failure occurs. The updated guide design uses more durable materials.</x:v>
+        <x:v>Start with the VIN build/options, open-campaign status, exact warning, complete fault memory, and BMW ISTA test plan. If the VIN and production date match a BMW action, follow that bulletin: inspect the specified sensor-link holders, apply the specified software correction, or inspect the affected air line as directed. For other vehicles, test the particular system shown by the VIN and fault path before selecting any component. Do not buy a compressor, strut, spring, or conversion kit until the failed part and its VIN-specific number are established. This article intentionally has no retail link because no single part repairs all of these conditions.</x:v>
       </x:c>
       <x:c r="F19" s="9" t="n">
         <x:v>0</x:v>
@@ -15670,44 +17032,44 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="673.2000122070312" hidden="0" customHeight="1">
+    <x:row r="20" ht="1148.4000244140625" hidden="0" customHeight="1">
       <x:c r="A20" s="40" t="n">
         <x:v>19</x:v>
       </x:c>
       <x:c r="B20" s="9" t="str">
-        <x:v>bmw-x3-n20-timing-chain-2012</x:v>
+        <x:v>bmw-x5-air-suspension-compressor-2007</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>2013-2015 | BMW | X3 | N20</x:v>
+        <x:v>2007-2013 | BMW | X5 | 3.0si, 4.8i, xDrive30i, xDrive35d, xDrive35i, xDrive48i, xDrive50i, X5 M | N52, N62, M57, N55, N63, S63</x:v>
       </x:c>
       <x:c r="D20" s="9" t="str">
-        <x:v>Lower-Engine Whine Requires X3 N20 Timing-Chain Diagnosis</x:v>
+        <x:v>E70 Rear Air-Supply Unit: Diagnose the Self-Leveling System First</x:v>
       </x:c>
       <x:c r="E20" s="9" t="str">
-        <x:v>Confirm the exact X3 variant, N20 engine, production date and VIN eligibility, then have a BMW-qualified technician reproduce the noise and follow current BMW diagnosis before replacing anything. The historical seven-year/70,000-mile coverage was a limited warranty extension, not a recall, and is not a current coverage promise. ShowMeTheParts established category-level fitment only, so no commerce link is approved.</x:v>
+        <x:v>Read the EHC fault memory and run the applicable BMW ISTA test plan before ordering a compressor. Confirm the vehicle is equipped with rear self-leveling suspension, compare left/right ride height, check system power and wiring, inspect the height-sensor links, and leak-test the air springs, lines, and valve system. Test the air supply only after those checks isolate it. If BMW ETK/AIR selects the E70 air-supply system for the VIN and diagnosis confirms that assembly, replace it with current part 37-20-6-859-714, follow the BMW repair procedure, clear faults, and perform the required ride-height calibration. Do not install a generic compressor or a coil-conversion kit from symptoms alone.</x:v>
       </x:c>
       <x:c r="F20" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G20" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="752.4000244140625" hidden="0" customHeight="1">
+    <x:row r="21" ht="1227.5999755859375" hidden="0" customHeight="1">
       <x:c r="A21" s="40" t="n">
         <x:v>20</x:v>
       </x:c>
       <x:c r="B21" s="9" t="str">
-        <x:v>bmw-x3-oil-filter-housing-gasket-2007</x:v>
+        <x:v>bmw-x5-carbon-buildup-2007</x:v>
       </x:c>
       <x:c r="C21" s="9" t="str">
-        <x:v>2007-2017 | BMW | X3 | sDrive30i, xDrive28i, xDrive30i | N52, N20</x:v>
+        <x:v>2011-2018 | BMW | X5 | xDrive35i, xDrive50i | N55, N63, N63TU1</x:v>
       </x:c>
       <x:c r="D21" s="9" t="str">
-        <x:v>Oil Filter Housing Gasket Leak (N52, N20 Engines)</x:v>
+        <x:v>Possible Intake-Valve Deposits on Direct-Injected Gasoline Engines</x:v>
       </x:c>
       <x:c r="E21" s="9" t="str">
-        <x:v>Replace oil filter housing gasket and oil cooler gasket ($40-80 DIY repair kit, $300-500 independent shop, $500-800 dealer). Requires draining some coolant and oil, removing housing, replacing gaskets, reassembling. Moderate DIY difficulty - Pelicanparts and YouTube have detailed model-specific guides. Use Victor Reinz or OEM BMW gasket kit for long-lasting seal - cheap gaskets leak within 20k miles. Address leak early before oil damages serpentine belt or alternator.</x:v>
+        <x:v>Diagnose the actual symptom before authorizing cleaning: read BMW-specific faults and misfire counters, check ignition and fueling, smoke-test the intake where indicated, verify crankcase ventilation operation, and inspect the intake valves with a borescope or by removing the intake manifold when the test plan supports it. If substantial deposits are confirmed and match the complaint, use an engine-specific professional mechanical-cleaning procedure that protects closed valves and removes all blasting media before reassembly. Do not present a universal catch can, chemical spray, fuel brand, short oil interval, or high-RPM driving as a proven repair. Any crankcase-ventilation modification also requires engine-specific fitment and emissions-law review.</x:v>
       </x:c>
       <x:c r="F21" s="9" t="n">
         <x:v>0</x:v>
@@ -15716,90 +17078,90 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="950.4000244140625" hidden="0" customHeight="1">
+    <x:row r="22" ht="884.4000244140625" hidden="0" customHeight="1">
       <x:c r="A22" s="40" t="n">
         <x:v>21</x:v>
       </x:c>
       <x:c r="B22" s="9" t="str">
-        <x:v>bmw-x3-transfer-case-actuator-2004</x:v>
+        <x:v>bmw-x5-coolant-pipe-leak-2007</x:v>
       </x:c>
       <x:c r="C22" s="9" t="str">
-        <x:v>2004-2023 | BMW | X3</x:v>
+        <x:v>2007-2010 | BMW | X5 | 4.8i, xDrive48i | N62, N62TU</x:v>
       </x:c>
       <x:c r="D22" s="9" t="str">
-        <x:v>Transfer Case Actuator Motor Failure (xDrive AWD System)</x:v>
+        <x:v>E70 N62 Coolant Transfer Pipe Leak (Pressure-Test First)</x:v>
       </x:c>
       <x:c r="E22" s="9" t="str">
-        <x:v>Replace the actuator motor assembly or rebuild using an aftermarket repair kit. DIY repair kits cost $100-150 and include replacement plastic gears, clips, and seals - straightforward installation saves $1,200+. Complete actuator motor replacement costs $540 for the assembly if DIY, or $1,500-2,200 at dealer. If transfer case itself is damaged from prolonged actuator failure, complete transfer case replacement costs $1,400-3,300. PREVENTIVE: If buying used X3 over 80k miles, budget for this repair - it's "when not if" on xDrive models. Check for clicking noise when shutting off ignition.</x:v>
+        <x:v>Pressure-test the cooling system cold and inspect the engine valley and all accessible connections to identify the exact leak before ordering parts. If inspection confirms the N62 transfer pipe and BMW ETK/AIR selects it for the VIN, replace pipe 11-14-1-439-975 with the required seals and one-time-use hardware from the VIN-specific repair diagram. Refill and bleed the cooling system with the specified coolant, repeat the pressure test, and verify stable temperature. Do not automatically replace an N63 pipe, thermostat, or unrelated hoses from this article.</x:v>
       </x:c>
       <x:c r="F22" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G22" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="396" hidden="0" customHeight="1">
+    <x:row r="23" ht="1082.4000244140625" hidden="0" customHeight="1">
       <x:c r="A23" s="40" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="B23" s="9" t="str">
-        <x:v>bmw-x3-transfer-case-actuator-2011</x:v>
+        <x:v>bmw-x5-n63-timing-chain-2008</x:v>
       </x:c>
       <x:c r="C23" s="9" t="str">
-        <x:v>2011-2026 | BMW | X3</x:v>
+        <x:v>2010-2013 | BMW | X5 | xDrive50i | N63</x:v>
       </x:c>
       <x:c r="D23" s="9" t="str">
-        <x:v>Transfer Case Actuator Motor Failure</x:v>
+        <x:v>Early N63 Timing-Chain Wear Check: ISTA Test Before Repair</x:v>
       </x:c>
       <x:c r="E23" s="9" t="str">
-        <x:v>Replace the transfer case actuator motor. Change the transfer case fluid at the same time. The actuator can be replaced without removing the entire transfer case. Rebuilt units are available at lower cost but OEM is recommended for reliability.</x:v>
+        <x:v>Check the VIN and service history with a BMW center, diagnose stored VANOS/camshaft faults first, and run BMW's ISTA timing-chain elongation test. If the result is 'Timing chain is OK,' do not replace parts on this claim. If it is 'not OK,' BMW SIB 11 16 14 directs replacement of both timing chains under the VIN-specific repair instruction, followed by the required oil/filter service, priming steps, programming, and shorter oil-service interval. A single tensioner 11-31-7-557-741 or a generic Cloyes kit is not the complete repair and must not be presented as what the owner needs. Tow the vehicle rather than driving it when severe mechanical noise, oil-pressure warnings, or loss of timing is present.</x:v>
       </x:c>
       <x:c r="F23" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G23" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="871.2000122070312" hidden="0" customHeight="1">
+    <x:row r="24" ht="1227.5999755859375" hidden="0" customHeight="1">
       <x:c r="A24" s="40" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="B24" s="9" t="str">
-        <x:v>bmw-x3-valve-cover-gasket-2004</x:v>
+        <x:v>bmw-x5-n63-wastegate-2008</x:v>
       </x:c>
       <x:c r="C24" s="9" t="str">
-        <x:v>2004-2017 | BMW | X3 | 2.5i, 3.0i, 3.0si | M54, N52</x:v>
+        <x:v>2010-2018 | BMW | X5 | xDrive50i | N63, N63TU</x:v>
       </x:c>
       <x:c r="D24" s="9" t="str">
-        <x:v>Valve Cover Gasket Oil Leaks (M54, N52 Engines)</x:v>
+        <x:v>N63/N63TU Low Boost or Turbo Rattle: Diagnose Vacuum Control First</x:v>
       </x:c>
       <x:c r="E24" s="9" t="str">
-        <x:v>Replace valve cover gasket and VANOS solenoid o-rings ($300-500 independent shop, $700-1,000 dealer, $80-150 DIY parts). On M54 engines, also replace ignition coil boots if contaminated by oil ($50 additional). Use OEM BMW gasket or Victor Reinz brand - aftermarket quality matters for long-term seal. Relatively straightforward DIY repair - saves $200-400 in labor. YouTube and Bimmerfest have detailed model-specific guides. Monitor oil level weekly and top off as needed (1 quart low is OK, 2+ quarts low risks engine damage).</x:v>
+        <x:v>Read all DME faults and compare requested versus actual boost under the BMW test plan. Pressure- or smoke-test the intake and charge-air path, verify vacuum supply from the pump and reservoir, inspect both banks' hoses and pressure converters, and test actuator movement before condemning a turbocharger. Identify the engine generation, failed bank, and exact hardware in BMW ETK/AIR. Check a 2010-2013 E70 VIN for the N63 Customer Care Package only as applicable; its published six-point scope includes air-mass sensors, injectors, vacuum pump, low-pressure fuel sensor/feed line, fresh-air turbo seals, and crankcase-ventilation lines, not an automatic wastegate replacement. No retail link is published until diagnosis selects a VIN-specific component.</x:v>
       </x:c>
       <x:c r="F24" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G24" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="409.20001220703125" hidden="0" customHeight="1">
+    <x:row r="25" ht="844.7999877929688" hidden="0" customHeight="1">
       <x:c r="A25" s="40" t="n">
         <x:v>24</x:v>
       </x:c>
       <x:c r="B25" s="9" t="str">
-        <x:v>bmw-x3-valve-cover-gasket-2011</x:v>
+        <x:v>bmw-x5-oil-leaks-2000</x:v>
       </x:c>
       <x:c r="C25" s="9" t="str">
-        <x:v>2011-2022 | BMW | X3 | N20, B48</x:v>
+        <x:v>2003-2006 | BMW | X5 | 3.0i | M54</x:v>
       </x:c>
       <x:c r="D25" s="9" t="str">
-        <x:v>Valve Cover Gasket Oil Leak</x:v>
+        <x:v>E53 3.0i M54 Valve-Cover Gasket Leak (Confirm the Source)</x:v>
       </x:c>
       <x:c r="E25" s="9" t="str">
-        <x:v>Replace the valve cover gasket. Inspect the valve cover for warping or cracks — if damaged, replace the entire cover assembly. Clean all oil residue from surrounding components. Use a torque wrench to prevent over-tightening which causes cover warping.</x:v>
+        <x:v>Clean the engine and trace the highest fresh-oil source before ordering a gasket. If the leak is at the M54 cylinder-head-cover perimeter or spark-plug-well seals, inspect the plastic cover for cracks, warpage, damaged fastener grommets, and crankcase-ventilation faults. Reuse the cover only if it passes inspection, then install VIN/production-confirmed gasket set 11-12-0-030-496 with the BMW-specified grommets and sealant locations and torque sequence. If the cover or another oil circuit is the source, select that separate repair instead.</x:v>
       </x:c>
       <x:c r="F25" s="9" t="n">
         <x:v>1</x:v>
@@ -15808,113 +17170,113 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="858" hidden="0" customHeight="1">
+    <x:row r="26" ht="1293.5999755859375" hidden="0" customHeight="1">
       <x:c r="A26" s="40" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="B26" s="9" t="str">
-        <x:v>bmw-x3-vanos-solenoid-2007</x:v>
+        <x:v>bmw-x5-transfer-case-actuator-2000</x:v>
       </x:c>
       <x:c r="C26" s="9" t="str">
-        <x:v>2007-2017 | BMW | X3 | M40i, M50, xDrive35i | N52, N55</x:v>
+        <x:v>2007-2013 | BMW | X5 | 3.0si, 4.8i, xDrive30i, xDrive35d, xDrive48i, X5 M | N52, N62, M57, S63</x:v>
       </x:c>
       <x:c r="D26" s="9" t="str">
-        <x:v>VANOS Solenoid Failure (N52, N55 Engines)</x:v>
+        <x:v>E70 ATC700 Transfer-Case Positioning Motor (Diagnosis Required)</x:v>
       </x:c>
       <x:c r="E26" s="9" t="str">
-        <x:v>Replace VANOS solenoids and seals ($250-400 European shops, $729-882 US average). Use high-quality oil (5W-30 or 0W-40 BMW LL-01 spec) and change every 5,000-7,000 miles to prevent future failures - cheap oil or extended intervals kill VANOS solenoids. Some cases may require complete VANOS unit rebuild ($1,500-2,500). PREVENTIVE: Replace VANOS solenoids and seals every 50k miles as maintenance - much cheaper than waiting for failure. On F25 X3 with N52/N55, check TSB SI B12 14 10 for VANOS gear assembly bolt issue.</x:v>
+        <x:v>Read BMW VTG/DSC faults and run the applicable ISTA transfer-case test plan before buying a motor. Confirm tire sizes and wear, battery voltage, wiring, transfer-case type, fluid condition, calibration, and—especially after differential or transfer-case replacement—the VIN-correct front and rear gear ratios. If testing confirms the ATC700 positioning motor and BMW ETK/AIR selects this application for the VIN, current BMW exchange servomotor 27-10-2-449-709 supersedes 27-10-7-568-267. Install the correct classification resistor/hardware supplied or specified for the VIN and perform the required VTG initialization/calibration. A generic gear-only kit is not a universal BMW repair and should not be ordered without opening and confirming the exact motor failure.</x:v>
       </x:c>
       <x:c r="F26" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G26" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="1016.4000244140625" hidden="0" customHeight="1">
+    <x:row r="27" ht="1042.800048828125" hidden="0" customHeight="1">
       <x:c r="A27" s="40" t="n">
         <x:v>26</x:v>
       </x:c>
       <x:c r="B27" s="9" t="str">
-        <x:v>bmw-x3-wastegate-rattle-2011</x:v>
+        <x:v>bmw-x5-transfer-case-actuator-2007</x:v>
       </x:c>
       <x:c r="C27" s="9" t="str">
-        <x:v>2011-2023 | BMW | X3 | M40i, M50, sDrive30i, xDrive28i, xDrive30i, xDrive35i</x:v>
+        <x:v>2019-2026 | BMW | X5</x:v>
       </x:c>
       <x:c r="D27" s="9" t="str">
-        <x:v>Turbocharger Wastegate Rattle (N55, N20, B58 Engines)</x:v>
+        <x:v>G05/F95 Transfer-Case Shudder: Tires and Fluid Diagnosis First</x:v>
       </x:c>
       <x:c r="E27" s="9" t="str">
-        <x:v>Replace wastegate actuator ($400-800) or use aftermarket wastegate repair kit with upgraded stainless steel bushings ($150-300). Some cases require complete turbocharger replacement ($2,000-$4,000). VTT (Vargas Turbo Technologies) repair kits popular on forums - upgraded materials prevent future rattle. MONITORING: Early wastegate rattle may be harmless (annoying but no performance loss). If car boosts normally and no underboost codes, can monitor rattle without urgent repair. However, if check engine light appears with code 30FF or boost pressure drops, repair immediately to prevent turbo damage.</x:v>
+        <x:v>Follow BMW SIB 27 02 20 in order: verify all four tires for VIN-correct size, brand/application, axle placement, and wear; diagnose any powertrain faults; then use ISTA to temporarily deactivate the transfer-case clutch and road-test the complaint. Only if the shudder disappears with the VTG deactivated does BMW direct an ATX13-X oil change with DTF-1, followed by VTG calibration. The clutch plates can require up to 125 miles after the service to become fully saturated and smooth out. If the symptom remains, continue diagnosis rather than buying an actuator or transfer case. Part numbers for any further repair must be selected by VIN in ETK/AIR.</x:v>
       </x:c>
       <x:c r="F27" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G27" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="778.7999877929688" hidden="0" customHeight="1">
+    <x:row r="28" ht="1214.4000244140625" hidden="0" customHeight="1">
       <x:c r="A28" s="40" t="n">
         <x:v>27</x:v>
       </x:c>
       <x:c r="B28" s="9" t="str">
-        <x:v>bmw-x3-water-pump-2007</x:v>
+        <x:v>bmw-x5-vanos-solenoid-2000</x:v>
       </x:c>
       <x:c r="C28" s="9" t="str">
-        <x:v>2007-2017 | BMW | X3 | sDrive30i, xDrive28i, xDrive30i | N52, N20</x:v>
+        <x:v>2010-2013 | BMW | X5 | xDrive30i, xDrive35i | N51, N52K, N52T, N55</x:v>
       </x:c>
       <x:c r="D28" s="9" t="str">
-        <x:v>Electric Water Pump Failure (N52, N20 Engines)</x:v>
+        <x:v>VANOS Adjustment-Unit Bolt Recall 23V-707 (E70 Inline-Six)</x:v>
       </x:c>
       <x:c r="E28" s="9" t="str">
-        <x:v>Replace electric water pump at first sign of failure ($800 parts + labor). Consider preventative replacement at 70-80k miles to avoid being stranded ($400 parts, DIY-able). CRITICAL: If you own 2013-2017 X3 28i, verify recall repair (protective shield installation) has been completed to prevent fire risk - check with BMW dealer using VIN. If engine overheats, PULL OVER IMMEDIATELY and shut off - driving with overheating warps cylinder heads ($4,000+ repair). Call tow truck.</x:v>
+        <x:v>Enter the VIN in BMW's official recall lookup and have an authorized BMW center complete recall 23V-707 if it is open. BMW's procedure is inspection-dependent: intact affected bolts are replaced; if bolts are loose or broken, the affected VANOS adjustment unit is replaced, and missing fragments must be recovered. The recall repair is free, so do not buy a solenoid or VANOS part first. If the VIN is outside the recall or a fault remains after the remedy, use BMW-capable diagnostics to test oil supply and pressure, wiring, sensors, control solenoids, adjustment units, and mechanical timing before selecting a part. If the engine runs roughly, makes unusual mechanical noise, loses power, or stalls, move out of traffic safely, stop driving, and contact BMW for transport guidance.</x:v>
       </x:c>
       <x:c r="F28" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G28" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="1240.800048828125" hidden="0" customHeight="1">
+    <x:row r="29" ht="1148.4000244140625" hidden="0" customHeight="1">
       <x:c r="A29" s="40" t="n">
         <x:v>28</x:v>
       </x:c>
       <x:c r="B29" s="9" t="str">
-        <x:v>bmw-x3m-brake-wear-2020</x:v>
+        <x:v>bmw-x5-water-pump-2007</x:v>
       </x:c>
       <x:c r="C29" s="9" t="str">
-        <x:v>2020-2023 | BMW | X3 M | S58</x:v>
+        <x:v>2011-2013 | BMW | X5 | xDrive35i | N55</x:v>
       </x:c>
       <x:c r="D29" s="9" t="str">
-        <x:v>Accelerated Brake Pad &amp; Rotor Wear from Vehicle Weight - F97 X3 M / F98 X4 M</x:v>
+        <x:v>E70 xDrive35i N55 Electric Coolant Pump (Fault-Confirmed)</x:v>
       </x:c>
       <x:c r="E29" s="9" t="str">
-        <x:v>Front brake replacement: OEM front rotor (34118054825 left, matching right) with OEM M compound pads. Complete OEM front brake kit available from BimmerWorld (34108064561K1, ~$800-$1,000). Rear brake kit similarly priced. For track use: Upgrade to Brembo GT brake pad set (BM8 compound) for improved heat resistance and longer pad life. EBC Yellowstuff or Hawk HPS 5.0 pads are popular street/track compromise choices ($150-$250 per axle). StopTech slotted rotors offer improved heat dissipation. For dedicated track cars: Brembo GT big brake kit with 412x38mm discs available ($4,000-$6,000 installed). Budget $2,000-$3,000 per year for brake maintenance if driving spiritedly. Use high-temperature brake fluid (Motul RBF 660 or ATE Typ 200) and flush every 12 months.</x:v>
+        <x:v>If the engine-temperature warning appears, stop safely, shut the engine off, and tow the vehicle if normal temperature cannot be confirmed. When cool, check coolant level and leaks, read BMW-specific faults, verify pump power/ground and communication, and run the ISTA coolant-pump activation/test plan. If those tests confirm the pump and BMW ETK/AIR selects 11-51-5-A05-704 for the VIN, replace it using the BMW procedure, select the thermostat separately only if testing or preventive planning justifies it, vacuum-fill or bleed the system as specified, and verify commanded pump operation and stable temperature. Do not use a fixed-mileage rule or this part number for an N52, N63, or F15 without VIN confirmation.</x:v>
       </x:c>
       <x:c r="F29" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G29" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="1188" hidden="0" customHeight="1">
+    <x:row r="30" ht="1056" hidden="0" customHeight="1">
       <x:c r="A30" s="40" t="n">
         <x:v>29</x:v>
       </x:c>
       <x:c r="B30" s="9" t="str">
-        <x:v>bmw-x3m-cooling-track-use-2020</x:v>
+        <x:v>bmw-x5m-brake-system-2010</x:v>
       </x:c>
       <x:c r="C30" s="9" t="str">
-        <x:v>2020-2023 | BMW | X3 M | S58</x:v>
+        <x:v>2010-2023 | BMW | X5 M</x:v>
       </x:c>
       <x:c r="D30" s="9" t="str">
-        <x:v>Cooling System Heat Soak During Track/Spirited Driving - F97 X3 M / F98 X4 M</x:v>
+        <x:v>Heavy-Duty Brake System Accelerated Wear - E70/F85/F95 X5 M</x:v>
       </x:c>
       <x:c r="E30" s="9" t="str">
-        <x:v>For track use: Upgrade intercooler to do88 front-mount intercooler ($1,200-$1,800) - the community standard for S58 heat management. Add CSF high-performance radiator ($600-$900) for sustained track work. Dinan or VRSF also offer intercooler upgrades in the $1,000-$1,500 range. For street/canyon driving: Stock cooling is adequate but ensure coolant flush every 2 years/30,000 miles and inspect expansion tank for cracks. Replace coolant expansion tank preemptively at 60,000 miles if car is driven hard. For all X3 M/X4 M: Use BMW coolant only (mixed 50/50 with distilled water), replace thermostat at 80,000 miles preventatively, inspect all coolant hoses for bulging or softening at every oil change.</x:v>
+        <x:v>E70 X5 M brakes: OEM front pads 34116799964 ($150-$250), rear pads 34216794879 ($120-$200). F85 X5 M front brake rotors: 34112284101/34112284102 with 6-pot caliper 34117845747/34117845748 and pads 34112284869. F85 rear: 385mm x 24mm perforated rotors 34212284903/34212284904 with 4-pot Brembo caliper and Textar pads. Budget $1,500-$2,500 per axle for complete brake service. For track use: EBC Yellowstuff or Hawk HPS 5.0 pads ($200-$350 per axle) with StopTech slotted rotors for improved heat management. Use Motul RBF 660 or ATE Typ 200 brake fluid - flush every 12 months. Budget $3,000-$5,000 per year for brake maintenance if driving spiritedly.</x:v>
       </x:c>
       <x:c r="F30" s="9" t="n">
         <x:v>0</x:v>
@@ -15923,21 +17285,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="1214.4000244140625" hidden="0" customHeight="1">
+    <x:row r="31" ht="1122" hidden="0" customHeight="1">
       <x:c r="A31" s="40" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="B31" s="9" t="str">
-        <x:v>bmw-x3m-differential-bolt-2020</x:v>
+        <x:v>bmw-x5m-rear-differential-2010</x:v>
       </x:c>
       <x:c r="C31" s="9" t="str">
-        <x:v>2020-2023 | BMW | X3 M | S58</x:v>
+        <x:v>2010-2023 | BMW | X5 M | S63</x:v>
       </x:c>
       <x:c r="D31" s="9" t="str">
-        <x:v>Rear Differential Mounting Bolt &amp; Bush Failure - F97 X3 M / F98 X4 M</x:v>
+        <x:v>Rear Differential Wear &amp; Fluid Degradation - E70/F85/F95 X5 M</x:v>
       </x:c>
       <x:c r="E31" s="9" t="str">
-        <x:v>Replace factory differential bolt, bush, and collar with FJ Motorwerkes uprated diff bolt and collar upgrade kit. The FJ kit uses premium CNC-machined stainless steel components that can handle 170,000 PSI (39% stronger than BMW's revised bolt). Kit price approximately $255 (GBP). Available from FJ Motorwerkes directly, BMG Performance, AM Tuning, and H4ck Performance. Installation is straightforward - rear differential does not need to be fully removed. Budget $400-$600 total including labor. This upgrade is considered MANDATORY by the X3 M/X4 M community for any car making stock or above power. JXB Performance also offers a driveshaft carrier bearing upgrade for cars experiencing propshaft vibration as a companion fix.</x:v>
+        <x:v>Change rear differential fluid every 30,000 miles (ignore BMW "lifetime fill" claim). E70 X5 M: No drain plug - fluid must be extracted through fill port with hand pump or suction device. Recommended fluid: Royal Purple 75W-140 GL5 synthetic or Red Line 75W-140 GL5 ($40-$60 per fill). Capacity approximately 1.2 liters. For limited-slip diff, ensure fluid is GL5 rated with limited-slip additive. If differential is making whining/howling noise: have a limited-slip differential specialist inspect internals (not generic BMW shop). Diff rebuild: $1,500-$3,000 at specialist. Complete differential replacement: $3,000-$5,500 + labor. Labor for fluid change: $150-$300 at independent shop.</x:v>
       </x:c>
       <x:c r="F31" s="9" t="n">
         <x:v>0</x:v>
@@ -15946,21 +17308,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="1293.5999755859375" hidden="0" customHeight="1">
+    <x:row r="32" ht="1386" hidden="0" customHeight="1">
       <x:c r="A32" s="40" t="n">
         <x:v>31</x:v>
       </x:c>
       <x:c r="B32" s="9" t="str">
-        <x:v>bmw-x3m-s58-bearing-recall-2020</x:v>
+        <x:v>bmw-x5m-s63-cooling-system-2010</x:v>
       </x:c>
       <x:c r="C32" s="9" t="str">
-        <x:v>2020-2021 | BMW | X3 M</x:v>
+        <x:v>2010-2023 | BMW | X5 M | 4.4i, 4.6is, 4.8is, M50i, M60i, xDrive48i, xDrive50e, xDrive50i | S63</x:v>
       </x:c>
       <x:c r="D32" s="9" t="str">
-        <x:v>S58 Engine Main Bearing Shell Recall / Stop Sale - F97 X3 M / F98 X4 M</x:v>
+        <x:v>S63 Cooling System Component Failures - E70/F85/F95 X5 M</x:v>
       </x:c>
       <x:c r="E32" s="9" t="str">
-        <x:v>Check VIN immediately against BMW recall database at bmwusa.com or contact your BMW dealer. If your vehicle is within the affected production date range, BMW will inspect and replace main bearing shells at no cost under the Tech Campaign. The repair requires removing the cylinder head and oil pan to access and replace all main bearing shells - this is a major repair (8-12 hours labor) but fully covered by BMW. Do NOT drive the vehicle if knocking is present. For S58 vehicles outside the recall range: Proactive rod bearing inspection is recommended at 60,000 miles for track-driven vehicles. ACL Race Series rod bearings 6B1510H-STD are the aftermarket upgrade choice on Bimmerpost for preventive replacement ($150-$250 for bearing set, $3,000-$5,000 total with labor).</x:v>
+        <x:v>PROACTIVE MAINTENANCE SCHEDULE: Replace electric water pump at 60,000 miles ($400-$700 + labor). Replace thermostat at same time ($150-$250). Replace expansion tank at 60,000-80,000 miles ($100-$200). Inspect all coolant hoses at every oil change - replace any that are soft, bulging, or showing surface cracks. E70 X5 M expansion tank vent hose: 17128627119 ($30-$50). Flush coolant system every 2 years or 30,000 miles (more frequent than BMW's 4-year recommendation). Use ONLY BMW coolant mixed 50/50 with distilled water. For E70 hot-V turbo coolant lines: GRYPHONTEK repair kit eliminates plastic T-fitting failure (see separate issue entry). Budget $1,500-$2,500 for complete cooling system refresh at 60,000 miles. This prevents catastrophic overheating that can destroy the S63 engine ($15,000-$34,000 engine replacement).</x:v>
       </x:c>
       <x:c r="F32" s="9" t="n">
         <x:v>0</x:v>
@@ -15969,21 +17331,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="1227.5999755859375" hidden="0" customHeight="1">
+    <x:row r="33" ht="1135.199951171875" hidden="0" customHeight="1">
       <x:c r="A33" s="40" t="n">
         <x:v>32</x:v>
       </x:c>
       <x:c r="B33" s="9" t="str">
-        <x:v>bmw-x3m-transfer-case-2020</x:v>
+        <x:v>bmw-x5m-s63-oil-leaks-2010</x:v>
       </x:c>
       <x:c r="C33" s="9" t="str">
-        <x:v>2020-2023 | BMW | X3 M | S58</x:v>
+        <x:v>2010-2023 | BMW | X5 M | 4.4i, 4.6is, 4.8is, M50i, M60i, xDrive48i, xDrive50e, xDrive50i | S63</x:v>
       </x:c>
       <x:c r="D33" s="9" t="str">
-        <x:v>xDrive Transfer Case Stress &amp; Fluid Degradation - F97 X3 M / F98 X4 M</x:v>
+        <x:v>S63 V8 Chronic Oil Leaks (Valve Cover, Oil Pan, Turbo Lines) - E70/F85/F95 X5 M</x:v>
       </x:c>
       <x:c r="E33" s="9" t="str">
-        <x:v>Change transfer case fluid every 30,000 miles (BMW says "lifetime fill" - this is NOT correct for M vehicles driven hard). Use BMW DTF-1 transfer case fluid or equivalent high-quality synthetic. Check tire tread depth at every service - all 4 tires must be within 2/32" of each other to prevent transfer case stress. Rotate tires every 5,000-7,000 miles. If transfer case actuator motor fails: FCP Euro guide for BMW transfer case actuator repair (part number varies by production date, ~$300-$600). For tuned cars: Consider transfer case brace/reinforcement and shortened fluid change intervals (every 15,000 miles). Complete transfer case replacement if internals are damaged: $3,000-$5,500 at independent specialist, $5,000-$8,000+ at dealer.</x:v>
+        <x:v>Valve cover gasket replacement (both sides): $1,200-$2,500 with labor. BMW plastic valve covers can crack and must be replaced entirely (not just gasket) - inspect during service. Oil filter housing gasket: $400-$800 with labor. Oil pan gasket: $2,000-$3,500 (requires engine/subframe drop). Turbo oil feed/return lines: replace with GRYPHONTEK or MAMBA upgraded silicone/braided lines during any turbo service ($200-$400). VANOS solenoid seals: $100-$200 (DIY-friendly). For comprehensive oil leak repair at 80,000+ miles: budget $3,000-$5,000 to address all common leak points simultaneously. Valve cover bolt torque is CRITICAL - too tight cracks the cover ($800-$1,200 per cover), too loose and it leaks.</x:v>
       </x:c>
       <x:c r="F33" s="9" t="n">
         <x:v>0</x:v>
@@ -15992,21 +17354,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="673.2000122070312" hidden="0" customHeight="1">
+    <x:row r="34" ht="1412.4000244140625" hidden="0" customHeight="1">
       <x:c r="A34" s="40" t="n">
         <x:v>33</x:v>
       </x:c>
       <x:c r="B34" s="9" t="str">
-        <x:v>bmw-x4-n20-timing-chain-2015</x:v>
+        <x:v>bmw-x5m-s63-rod-bearing-2010</x:v>
       </x:c>
       <x:c r="C34" s="9" t="str">
-        <x:v>2015-2016 | BMW | X4 | xDrive28i, xDrive30i</x:v>
+        <x:v>2010-2018 | BMW | X5 M | 4.4i, 4.6is, 4.8is, M50i, M60i, xDrive48i, xDrive50e, xDrive50i</x:v>
       </x:c>
       <x:c r="D34" s="9" t="str">
-        <x:v>N20 Timing Chain Premature Failure - F26 X4 xDrive28i</x:v>
+        <x:v>S63 V8 Rod Bearing Premature Wear &amp; Failure - E70/F85 X5 M</x:v>
       </x:c>
       <x:c r="E34" s="9" t="str">
-        <x:v>Complete timing chain kit replacement including chain, guides, tensioner, and sprockets. Must be performed by experienced BMW technician. Preventive replacement recommended at 60,000-80,000 miles. BMW extended warranty to 8 years/100,000 miles under class action settlement. Upgraded reinforced chain kit available from aftermarket. Labor is 10-14 hours for X4 due to AWD and tight engine bay.</x:v>
+        <x:v>PREVENTIVE: For track-driven X5 M, replace rod bearings proactively at 60,000-80,000 miles. ACL Race Series rod bearings (8B1578HX-STD for S63B44, +0.001" extra oil clearance) are the community gold standard ($200-$350 for bearing set). WPC surface-treated bearings from Lang Racing are the premium choice ($400-$600 set). Total cost for preventive rod bearing service: $4,500-$8,500 depending on shop. Oil analysis every 5,000 miles through Blackstone Labs ($30/test) to monitor bearing wear metals (lead and copper). Use only BMW 10W-60 synthetic oil with 5,000-7,500 mile oil change intervals. Never track the car on cold oil. Mporium BMW offers specialized S63 rod bearing service starting at $4,499. If catastrophic failure: rebuilt S63 engine from RK Autowerks (~$8,500 + installation), new BMW engine (~$34,000), or complete engine rebuild ($12,000-$18,000).</x:v>
       </x:c>
       <x:c r="F34" s="9" t="n">
         <x:v>0</x:v>
@@ -16015,21 +17377,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="686.4000244140625" hidden="0" customHeight="1">
+    <x:row r="35" ht="1214.4000244140625" hidden="0" customHeight="1">
       <x:c r="A35" s="40" t="n">
         <x:v>34</x:v>
       </x:c>
       <x:c r="B35" s="9" t="str">
-        <x:v>bmw-x4-n20-timing-chain-guide-2015</x:v>
+        <x:v>bmw-x5m-s63-turbo-coolant-line-2010</x:v>
       </x:c>
       <x:c r="C35" s="9" t="str">
-        <x:v>2015-2015 | BMW | X4 | N20</x:v>
+        <x:v>2010-2013 | BMW | X5 M</x:v>
       </x:c>
       <x:c r="D35" s="9" t="str">
-        <x:v>2015 X4 N20 Lower-Engine Whine Requires Timing-Chain Diagnosis</x:v>
+        <x:v>S63 Turbo Coolant Line Plastic T-Fitting Failure (Hot-V Design) - E70 X5 M</x:v>
       </x:c>
       <x:c r="E35" s="9" t="str">
-        <x:v>Confirm the exact xDrive28i variant, N20 engine, production date and VIN eligibility, then have a BMW-qualified technician reproduce the noise and follow current BMW diagnosis before replacing anything. The historical seven-year/70,000-mile coverage was a limited warranty extension, not a recall, and is not a current coverage promise. ShowMeTheParts established category-level fitment only, so no commerce link is approved.</x:v>
+        <x:v>Replace ALL factory plastic turbo coolant T-fittings and hoses with GRYPHONTEK S63 Turbo Coolant Line Repair Kit ($200-$400). Kit includes pre-shaped multi-layer reinforced silicone hoses, brass T-fittings (replacing factory plastic), and all necessary hose clamps. Direct bolt-on installation designed for the E70/E71 S63 engine bay. MAMBA Turbo also offers a reinforced turbo coolant line kit with brass and silicone components ($150-$350). This is a PROACTIVE replacement - do not wait for failure. Replace at first sign of coolant weeping or during any turbo service. Labor: $800-$1,500 due to tight access in hot-V engine valley. If turbo bearings are damaged from overheating: turbo replacement $3,000-$5,000 per unit.</x:v>
       </x:c>
       <x:c r="F35" s="9" t="n">
         <x:v>0</x:v>
@@ -16038,21 +17400,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="554.4000244140625" hidden="0" customHeight="1">
+    <x:row r="36" ht="1135.199951171875" hidden="0" customHeight="1">
       <x:c r="A36" s="40" t="n">
         <x:v>35</x:v>
       </x:c>
       <x:c r="B36" s="9" t="str">
-        <x:v>bmw-x4-oil-leak-2015</x:v>
+        <x:v>bmw-x5m-s63-vanos-solenoid-2010</x:v>
       </x:c>
       <x:c r="C36" s="9" t="str">
-        <x:v>2015-2023 | BMW | X4</x:v>
+        <x:v>2010-2023 | BMW | X5 M | 4.4i, 4.6is, 4.8is, M50i, M60i, xDrive48i, xDrive50e, xDrive50i | S63</x:v>
       </x:c>
       <x:c r="D36" s="9" t="str">
-        <x:v>Oil Leaks - Valve Cover &amp; Oil Filter Housing - All Models</x:v>
+        <x:v>S63 VANOS Solenoid Failure - E70/F85/F95 X5 M</x:v>
       </x:c>
       <x:c r="E36" s="9" t="str">
-        <x:v>Replace valve cover gasket and/or oil filter housing gasket. Valve cover replacement is 3-4 hours labor on X4. Oil filter housing gasket is 1-2 hours. Both are routine maintenance items on BMW turbo engines. Use OEM gaskets for best longevity. Clean oil residue from engine bay after repair. Monitor oil level regularly to catch leaks early.</x:v>
+        <x:v>Replace all 4 VANOS solenoids simultaneously - they are same age and if one has failed, others are close behind. Pierburg 11368605123 (OEM supplier) at $30-$50 each from Turner Motorsport or BimmerWorld. Genuine BMW 11368482268 for S63TU applications at $50-$70 each. Total parts cost: $120-$280 for all 4 solenoids. Also replace VANOS solenoid O-rings and filter screens during service. Labor: 1-2 hours professional ($150-$400 labor). This is one of the easier S63 repairs - accessible from top of engine without removing intake manifold. Natafox and Febi also offer quality aftermarket VANOS solenoids at lower cost ($20-$35 each). Clean VANOS system with fresh oil change immediately after solenoid replacement.</x:v>
       </x:c>
       <x:c r="F36" s="9" t="n">
         <x:v>0</x:v>
@@ -16061,21 +17423,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" ht="356.3999938964844" hidden="0" customHeight="1">
+    <x:row r="37" ht="1293.5999755859375" hidden="0" customHeight="1">
       <x:c r="A37" s="40" t="n">
         <x:v>36</x:v>
       </x:c>
       <x:c r="B37" s="9" t="str">
-        <x:v>bmw-x4-rear-differential-mount-2015</x:v>
+        <x:v>bmw-x5m-s63-wastegate-rattle-2010</x:v>
       </x:c>
       <x:c r="C37" s="9" t="str">
-        <x:v>2015-2023 | BMW | X4</x:v>
+        <x:v>2010-2018 | BMW | X5 M | S63</x:v>
       </x:c>
       <x:c r="D37" s="9" t="str">
-        <x:v>Rear Differential Mount Bushing Failure</x:v>
+        <x:v>S63 Twin Turbo Wastegate Rattle - E70/F85 X5 M</x:v>
       </x:c>
       <x:c r="E37" s="9" t="str">
-        <x:v>Replace rear differential mount bushings. Both front and rear differential bushings should be inspected and replaced as a set. Upgraded aftermarket bushings with stiffer rubber or polyurethane are available for longer service life.</x:v>
+        <x:v>Option 1 (Most cost-effective): MAMBA SUS316 stainless steel wastegate rattle flapper repair kit for S63 MGT2260 (part 077-0024, replaces 790463-2 / 790484-3), approximately $150-$300 per turbo. Requires turbo removal for installation. Option 2: Lskioer turbo wastegate rattle flapper repair kit for S63/S63TU MGT2260DSL ($80-$150 per kit on Amazon). Option 3: Replace turbo wastegate actuators with new OEM units ($300-$500 each). Option 4: Full turbocharger replacement with new or remanufactured units ($3,000-$5,000 per turbo + labor). Labor for turbo removal and reinstallation: $2,000-$3,500 for both turbos. While turbos are out: replace turbo oil feed/return lines, coolant lines, and all gaskets (GRYPHONTEK turbo coolant line repair kit for E70 X5M, ~$200-$400).</x:v>
       </x:c>
       <x:c r="F37" s="9" t="n">
         <x:v>0</x:v>
@@ -16084,21 +17446,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="620.4000244140625" hidden="0" customHeight="1">
+    <x:row r="38" ht="1069.199951171875" hidden="0" customHeight="1">
       <x:c r="A38" s="40" t="n">
         <x:v>37</x:v>
       </x:c>
       <x:c r="B38" s="9" t="str">
-        <x:v>bmw-x4-transfer-case-2015</x:v>
+        <x:v>bmw-x5m-transfer-case-actuator-2010</x:v>
       </x:c>
       <x:c r="C38" s="9" t="str">
-        <x:v>2015-2023 | BMW | X4</x:v>
+        <x:v>2010-2023 | BMW | X5 M</x:v>
       </x:c>
       <x:c r="D38" s="9" t="str">
-        <x:v>Transfer Case Actuator Motor Failure - All xDrive X4</x:v>
+        <x:v>xDrive Transfer Case Actuator Motor Failure - E70/F85/F95 X5 M</x:v>
       </x:c>
       <x:c r="E38" s="9" t="str">
-        <x:v>Diagnose specific failure. Transfer case actuator motor replacement ($800-1,200) is most common. Complete transfer case replacement required for internal failures ($2,500-4,000). Regular transfer case fluid changes every 50,000 miles may extend life. Some owners install aftermarket upgraded actuator motors. Common wear item on high-mileage xDrive BMW models.</x:v>
+        <x:v>Replace transfer case actuator motor. E70 X5 M: BMW 27107566296 or equivalent ($250-$450 for actuator motor). F85 X5 M: BMW 27608643153 or equivalent ($300-$500). F95 X5 M: check VIN-specific part number with dealer. FCP Euro has an excellent DIY guide for BMW transfer case actuator repair - the actuator can be replaced without removing the entire transfer case. Labor: 2-3 hours at specialist shop ($300-$600 labor). Change transfer case fluid at same time with BMW DTF-1 specification fluid. XeMODeX offers remanufactured transfer case actuator motors at reduced cost ($200-$350). For complete transfer case failure: $3,500-$6,000 for replacement unit + labor.</x:v>
       </x:c>
       <x:c r="F38" s="9" t="n">
         <x:v>0</x:v>
@@ -16107,21 +17469,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="1240.800048828125" hidden="0" customHeight="1">
+    <x:row r="39" ht="435.6000061035156" hidden="0" customHeight="1">
       <x:c r="A39" s="40" t="n">
         <x:v>38</x:v>
       </x:c>
       <x:c r="B39" s="9" t="str">
-        <x:v>bmw-x4m-brake-wear-2020</x:v>
+        <x:v>bmw-x6-adaptive-drive-malfunction-2008</x:v>
       </x:c>
       <x:c r="C39" s="9" t="str">
-        <x:v>2020-2023 | BMW | X4 M | S58</x:v>
+        <x:v>2008-2019 | BMW | X6</x:v>
       </x:c>
       <x:c r="D39" s="9" t="str">
-        <x:v>Accelerated Brake Pad &amp; Rotor Wear from Vehicle Weight - F98 X4 M / F98 X4 M</x:v>
+        <x:v>Adaptive Drive System Malfunction</x:v>
       </x:c>
       <x:c r="E39" s="9" t="str">
-        <x:v>Front brake replacement: OEM front rotor (34118054825 left, matching right) with OEM M compound pads. Complete OEM front brake kit available from BimmerWorld (34108064561K1, ~$800-$1,000). Rear brake kit similarly priced. For track use: Upgrade to Brembo GT brake pad set (BM8 compound) for improved heat resistance and longer pad life. EBC Yellowstuff or Hawk HPS 5.0 pads are popular street/track compromise choices ($150-$250 per axle). StopTech slotted rotors offer improved heat dissipation. For dedicated track cars: Brembo GT big brake kit with 412x38mm discs available ($4,000-$6,000 installed). Budget $2,000-$3,000 per year for brake maintenance if driving spiritedly. Use high-temperature brake fluid (Motul RBF 660 or ATE Typ 200) and flush every 12 months.</x:v>
+        <x:v>Diagnose specific Adaptive Drive component failure using BMW ISTA diagnostics. Replace the failed component — most commonly the hydraulic pump or valve block. If repair cost is prohibitive, some owners convert to conventional anti-roll bars as a permanent fix at lower cost.</x:v>
       </x:c>
       <x:c r="F39" s="9" t="n">
         <x:v>0</x:v>
@@ -16130,21 +17492,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="1188" hidden="0" customHeight="1">
+    <x:row r="40" ht="858" hidden="0" customHeight="1">
       <x:c r="A40" s="40" t="n">
         <x:v>39</x:v>
       </x:c>
       <x:c r="B40" s="9" t="str">
-        <x:v>bmw-x4m-cooling-track-use-2020</x:v>
+        <x:v>bmw-x6-air-suspension-2008</x:v>
       </x:c>
       <x:c r="C40" s="9" t="str">
-        <x:v>2020-2023 | BMW | X4 M</x:v>
+        <x:v>2008-2023 | BMW | X6</x:v>
       </x:c>
       <x:c r="D40" s="9" t="str">
-        <x:v>Cooling System Heat Soak During Track/Spirited Driving - F98 X4 M / F98 X4 M</x:v>
+        <x:v>Air Suspension Compressor &amp; Strut Failure</x:v>
       </x:c>
       <x:c r="E40" s="9" t="str">
-        <x:v>For track use: Upgrade intercooler to do88 front-mount intercooler ($1,200-$1,800) - the community standard for S58 heat management. Add CSF high-performance radiator ($600-$900) for sustained track work. Dinan or VRSF also offer intercooler upgrades in the $1,000-$1,500 range. For street/canyon driving: Stock cooling is adequate but ensure coolant flush every 2 years/30,000 miles and inspect expansion tank for cracks. Replace coolant expansion tank preemptively at 60,000 miles if car is driven hard. For all X3 M/X4 M: Use BMW coolant only (mixed 50/50 with distilled water), replace thermostat at 80,000 miles preventatively, inspect all coolant hoses for bulging or softening at every oil change.</x:v>
+        <x:v>Replace failed air springs or compressor. Arnott rear air spring A-2642 ($200-300 each). OEM F16 spring 37126795013 ($200). Arnott compressor P-2655 ($599). Or convert to coil springs: Strutmasters BB2RBM conversion kit ($1,200-1,800) permanently eliminates air suspension issues. Conversion is cheaper long-term than continued air suspension repairs. If keeping air suspension: inspect air springs at 60,000-80,000 miles for cracks/leaks before compressor damage occurs. Replace both air springs on same axle simultaneously.</x:v>
       </x:c>
       <x:c r="F40" s="9" t="n">
         <x:v>0</x:v>
@@ -16153,21 +17515,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="1214.4000244140625" hidden="0" customHeight="1">
+    <x:row r="41" ht="646.7999877929688" hidden="0" customHeight="1">
       <x:c r="A41" s="40" t="n">
         <x:v>40</x:v>
       </x:c>
       <x:c r="B41" s="9" t="str">
-        <x:v>bmw-x4m-differential-bolt-2020</x:v>
+        <x:v>bmw-x6-ibs-brake-recall-2023</x:v>
       </x:c>
       <x:c r="C41" s="9" t="str">
-        <x:v>2020-2023 | BMW | X4 M</x:v>
+        <x:v>2024-2024 | BMW | X6</x:v>
       </x:c>
       <x:c r="D41" s="9" t="str">
-        <x:v>Rear Differential Mounting Bolt &amp; Bush Failure - F98 X4 M / F98 X4 M</x:v>
+        <x:v>2024 X6 Integrated Brake System Recall 26V-422</x:v>
       </x:c>
       <x:c r="E41" s="9" t="str">
-        <x:v>Replace factory differential bolt, bush, and collar with FJ Motorwerkes uprated diff bolt and collar upgrade kit. The FJ kit uses premium CNC-machined stainless steel components that can handle 170,000 PSI (39% stronger than BMW's revised bolt). Kit price approximately $255 (GBP). Available from FJ Motorwerkes directly, BMG Performance, AM Tuning, and H4ck Performance. Installation is straightforward - rear differential does not need to be fully removed. Budget $400-$600 total including labor. This upgrade is considered MANDATORY by the X3 M/X4 M community for any car making stock or above power. JXB Performance also offers a driveshaft carrier bearing upgrade for cars experiencing propshaft vibration as a companion fix.</x:v>
+        <x:v>Check the VIN at NHTSA and with an authorized BMW dealer when campaign 26V-422 VINs become searchable, and arrange the free dealer inspection and module replacement if required. If a brake warning appears or pedal effort increases, avoid abrupt braking, allow extra stopping distance, stop safely and contact BMW roadside assistance; do not order brake electronics from this card.</x:v>
       </x:c>
       <x:c r="F41" s="9" t="n">
         <x:v>0</x:v>
@@ -16176,21 +17538,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="42" ht="1293.5999755859375" hidden="0" customHeight="1">
+    <x:row r="42" ht="924" hidden="0" customHeight="1">
       <x:c r="A42" s="40" t="n">
         <x:v>41</x:v>
       </x:c>
       <x:c r="B42" s="9" t="str">
-        <x:v>bmw-x4m-s58-bearing-recall-2020</x:v>
+        <x:v>bmw-x6-n63-timing-chain-2008</x:v>
       </x:c>
       <x:c r="C42" s="9" t="str">
-        <x:v>2020-2021 | BMW | X4 M | M40i, xDrive35i | S58</x:v>
+        <x:v>2008-2018 | BMW | X6 | M50i, xDrive50i</x:v>
       </x:c>
       <x:c r="D42" s="9" t="str">
-        <x:v>S58 Engine Main Bearing Shell Recall / Stop Sale - F98 X4 M / F98 X4 M</x:v>
+        <x:v>N63 Timing Chain Stretch &amp; Guide Failure (E71/F16 xDrive50i)</x:v>
       </x:c>
       <x:c r="E42" s="9" t="str">
-        <x:v>Check VIN immediately against BMW recall database at bmwusa.com or contact your BMW dealer. If your vehicle is within the affected production date range, BMW will inspect and replace main bearing shells at no cost under the Tech Campaign. The repair requires removing the cylinder head and oil pan to access and replace all main bearing shells - this is a major repair (8-12 hours labor) but fully covered by BMW. Do NOT drive the vehicle if knocking is present. For S58 vehicles outside the recall range: Proactive rod bearing inspection is recommended at 60,000 miles for track-driven vehicles. ACL Race Series rod bearings 6B1510H-STD are the aftermarket upgrade choice on Bimmerpost for preventive replacement ($150-$250 for bearing set, $3,000-$5,000 total with labor).</x:v>
+        <x:v>PREVENTIVE REPLACEMENT: If you own 2008-2014 E71 xDrive50i with N63, replace timing chain guides and tensioners IMMEDIATELY at 60,000-80,000 miles ($4,000-6,000) BEFORE failure. IWIS timing chain kit 90001521 ($800-1,200) or Turner kit 11317594899KT recommended. Replace lower chain guide 11147574373 at same time. If chain has already failed: complete engine replacement required ($15,000-25,000). Check VIN with BMW dealer for extended warranty eligibility. 2015+ N63TU engines have improved timing components but still require monitoring.</x:v>
       </x:c>
       <x:c r="F42" s="9" t="n">
         <x:v>0</x:v>
@@ -16199,21 +17561,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="43" ht="1227.5999755859375" hidden="0" customHeight="1">
+    <x:row r="43" ht="409.20001220703125" hidden="0" customHeight="1">
       <x:c r="A43" s="40" t="n">
         <x:v>42</x:v>
       </x:c>
       <x:c r="B43" s="9" t="str">
-        <x:v>bmw-x4m-transfer-case-2020</x:v>
+        <x:v>bmw-x6-n63-valve-stem-seal-wear-2008</x:v>
       </x:c>
       <x:c r="C43" s="9" t="str">
-        <x:v>2020-2023 | BMW | X4 M | S58</x:v>
+        <x:v>2008-2019 | BMW | X6 | N63</x:v>
       </x:c>
       <x:c r="D43" s="9" t="str">
-        <x:v>xDrive Transfer Case Stress &amp; Fluid Degradation - F98 X4 M / F98 X4 M</x:v>
+        <x:v>N63 Valve Stem Seal Degradation and Oil Burning</x:v>
       </x:c>
       <x:c r="E43" s="9" t="str">
-        <x:v>Change transfer case fluid every 30,000 miles (BMW says "lifetime fill" - this is NOT correct for M vehicles driven hard). Use BMW DTF-1 transfer case fluid or equivalent high-quality synthetic. Check tire tread depth at every service - all 4 tires must be within 2/32" of each other to prevent transfer case stress. Rotate tires every 5,000-7,000 miles. If transfer case actuator motor fails: FCP Euro guide for BMW transfer case actuator repair (part number varies by production date, ~$300-$600). For tuned cars: Consider transfer case brace/reinforcement and shortened fluid change intervals (every 15,000 miles). Complete transfer case replacement if internals are damaged: $3,000-$5,500 at independent specialist, $5,000-$8,000+ at dealer.</x:v>
+        <x:v>Replace all intake and exhaust valve stem seals. This is a major job requiring head work. Also replace turbo oil return lines and update engine software per BMW N63 Customer Care Package specifications. Ensure proper oil grade (BMW LL-01) is used.</x:v>
       </x:c>
       <x:c r="F43" s="9" t="n">
         <x:v>0</x:v>
@@ -16222,21 +17584,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="44" ht="1042.800048828125" hidden="0" customHeight="1">
+    <x:row r="44" ht="858" hidden="0" customHeight="1">
       <x:c r="A44" s="40" t="n">
         <x:v>43</x:v>
       </x:c>
       <x:c r="B44" s="9" t="str">
-        <x:v>bmw-x5-air-suspension-2007</x:v>
+        <x:v>bmw-x6-n63-valve-stem-seals-2008</x:v>
       </x:c>
       <x:c r="C44" s="9" t="str">
-        <x:v>2019-2026 | BMW | X5</x:v>
+        <x:v>2008-2023 | BMW | X6 | M50i, xDrive50i | N63</x:v>
       </x:c>
       <x:c r="D44" s="9" t="str">
-        <x:v>G05 Suspension Warning: Check Faults and Campaigns Before Parts</x:v>
+        <x:v>N63 Valve Stem Seal / Oil Consumption (xDrive50i)</x:v>
       </x:c>
       <x:c r="E44" s="9" t="str">
-        <x:v>Start with the VIN build/options, open-campaign status, exact warning, complete fault memory, and BMW ISTA test plan. If the VIN and production date match a BMW action, follow that bulletin: inspect the specified sensor-link holders, apply the specified software correction, or inspect the affected air line as directed. For other vehicles, test the particular system shown by the VIN and fault path before selecting any component. Do not buy a compressor, strut, spring, or conversion kit until the failed part and its VIN-specific number are established. This article intentionally has no retail link because no single part repairs all of these conditions.</x:v>
+        <x:v>Replace valve stem seals - extremely labor-intensive job requiring cylinder head work ($4,900-12,000 total). Elring seals 11340039494 ($80-120/set of 16, need 2 sets for V8). 5150 AutoSport Viton upgraded seals ($150-200) are recommended for better heat resistance in hot-vee configuration. AGA Tools kit AGA-N63-VSK-K ($500-800) includes specialized tools required. Reference TSB MC-10149960-9999 when visiting dealer. Some owners monitor oil levels and add as needed rather than repair. Use quality synthetic 0W-40 BMW LL-01 spec oil.</x:v>
       </x:c>
       <x:c r="F44" s="9" t="n">
         <x:v>0</x:v>
@@ -16245,44 +17607,44 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="45" ht="1148.4000244140625" hidden="0" customHeight="1">
+    <x:row r="45" ht="818.4000244140625" hidden="0" customHeight="1">
       <x:c r="A45" s="40" t="n">
         <x:v>44</x:v>
       </x:c>
       <x:c r="B45" s="9" t="str">
-        <x:v>bmw-x5-air-suspension-compressor-2007</x:v>
+        <x:v>bmw-x6-n63-wastegate-2008</x:v>
       </x:c>
       <x:c r="C45" s="9" t="str">
-        <x:v>2007-2013 | BMW | X5 | 3.0si, 4.8i, xDrive30i, xDrive35d, xDrive35i, xDrive48i, xDrive50i, X5 M | N52, N62, M57, N55, N63, S63</x:v>
+        <x:v>2008-2018 | BMW | X6 | M50i, xDrive50i</x:v>
       </x:c>
       <x:c r="D45" s="9" t="str">
-        <x:v>E70 Rear Air-Supply Unit: Diagnose the Self-Leveling System First</x:v>
+        <x:v>N63 Turbo Wastegate Rattle (xDrive50i)</x:v>
       </x:c>
       <x:c r="E45" s="9" t="str">
-        <x:v>Read the EHC fault memory and run the applicable BMW ISTA test plan before ordering a compressor. Confirm the vehicle is equipped with rear self-leveling suspension, compare left/right ride height, check system power and wiring, inspect the height-sensor links, and leak-test the air springs, lines, and valve system. Test the air supply only after those checks isolate it. If BMW ETK/AIR selects the E70 air-supply system for the VIN and diagnosis confirms that assembly, replace it with current part 37-20-6-859-714, follow the BMW repair procedure, clear faults, and perform the required ride-height calibration. Do not install a generic compressor or a coil-conversion kit from symptoms alone.</x:v>
+        <x:v>Repair options range from flapper repair kits ($50-100/turbo) to complete turbocharger replacement ($4,000-8,000 for both). Garrett MGT2256S flapper repair kit ($50-100 per turbo) is cheapest fix. MAMBA adjustable actuator kit ($150-300) provides more durable solution. OEM actuators 11657646093 available from BMW. Complete turbo replacement $2,000-4,000 per turbo. MONITORING: Wastegate rattle is early warning - address before complete turbo failure to avoid $8,000+ repair.</x:v>
       </x:c>
       <x:c r="F45" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G45" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" ht="1227.5999755859375" hidden="0" customHeight="1">
+    <x:row r="46" ht="409.20001220703125" hidden="0" customHeight="1">
       <x:c r="A46" s="40" t="n">
         <x:v>45</x:v>
       </x:c>
       <x:c r="B46" s="9" t="str">
-        <x:v>bmw-x5-carbon-buildup-2007</x:v>
+        <x:v>bmw-x6-rear-differential-bushing-2008</x:v>
       </x:c>
       <x:c r="C46" s="9" t="str">
-        <x:v>2011-2018 | BMW | X5 | xDrive35i, xDrive50i | N55, N63, N63TU1</x:v>
+        <x:v>2008-2026 | BMW | X6</x:v>
       </x:c>
       <x:c r="D46" s="9" t="str">
-        <x:v>Possible Intake-Valve Deposits on Direct-Injected Gasoline Engines</x:v>
+        <x:v>Rear Differential Bushing Deterioration</x:v>
       </x:c>
       <x:c r="E46" s="9" t="str">
-        <x:v>Diagnose the actual symptom before authorizing cleaning: read BMW-specific faults and misfire counters, check ignition and fueling, smoke-test the intake where indicated, verify crankcase ventilation operation, and inspect the intake valves with a borescope or by removing the intake manifold when the test plan supports it. If substantial deposits are confirmed and match the complaint, use an engine-specific professional mechanical-cleaning procedure that protects closed valves and removes all blasting media before reassembly. Do not present a universal catch can, chemical spray, fuel brand, short oil interval, or high-RPM driving as a proven repair. Any crankcase-ventilation modification also requires engine-specific fitment and emissions-law review.</x:v>
+        <x:v>Replace all rear differential mount bushings. Use OEM or equivalent quality bushings (Lemforder is the OEM supplier). Inspect the differential housing for any damage from excessive movement. Perform subframe alignment check after bushing replacement.</x:v>
       </x:c>
       <x:c r="F46" s="9" t="n">
         <x:v>0</x:v>
@@ -16291,67 +17653,67 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="47" ht="884.4000244140625" hidden="0" customHeight="1">
+    <x:row r="47" ht="765.5999755859375" hidden="0" customHeight="1">
       <x:c r="A47" s="40" t="n">
         <x:v>46</x:v>
       </x:c>
       <x:c r="B47" s="9" t="str">
-        <x:v>bmw-x5-coolant-pipe-leak-2007</x:v>
+        <x:v>bmw-x6-transfer-case-2008</x:v>
       </x:c>
       <x:c r="C47" s="9" t="str">
-        <x:v>2007-2010 | BMW | X5 | 4.8i, xDrive48i | N62, N62TU</x:v>
+        <x:v>2008-2023 | BMW | X6</x:v>
       </x:c>
       <x:c r="D47" s="9" t="str">
-        <x:v>E70 N62 Coolant Transfer Pipe Leak (Pressure-Test First)</x:v>
+        <x:v>Transfer Case Actuator Motor Failure (All xDrive Models)</x:v>
       </x:c>
       <x:c r="E47" s="9" t="str">
-        <x:v>Pressure-test the cooling system cold and inspect the engine valley and all accessible connections to identify the exact leak before ordering parts. If inspection confirms the N62 transfer pipe and BMW ETK/AIR selects it for the VIN, replace pipe 11-14-1-439-975 with the required seals and one-time-use hardware from the VIN-specific repair diagram. Refill and bleed the cooling system with the specified coolant, repeat the pressure test, and verify stable temperature. Do not automatically replace an N63 pipe, thermostat, or unrelated hoses from this article.</x:v>
+        <x:v>Replace the actuator motor assembly or rebuild using an aftermarket gear repair kit ($100-150). G06 actuator motor 27609469023 ($400-600) for complete replacement. DIY gear repair kits are straightforward and save $1,200+ over dealer replacement. Complete transfer case replacement if internal damage occurred: $1,400-3,300. PREVENTIVE: If buying used X6 over 80k miles, budget for this repair and listen for clicking noise when shutting off ignition.</x:v>
       </x:c>
       <x:c r="F47" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G47" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="48" ht="1082.4000244140625" hidden="0" customHeight="1">
+    <x:row r="48" ht="514.7999877929688" hidden="0" customHeight="1">
       <x:c r="A48" s="40" t="n">
         <x:v>47</x:v>
       </x:c>
       <x:c r="B48" s="9" t="str">
-        <x:v>bmw-x5-n63-timing-chain-2008</x:v>
+        <x:v>bmw-x6m-front-thrust-arm-bushing-2015</x:v>
       </x:c>
       <x:c r="C48" s="9" t="str">
-        <x:v>2010-2013 | BMW | X5 | xDrive50i | N63</x:v>
+        <x:v>2015-2025 | BMW | X6 M</x:v>
       </x:c>
       <x:c r="D48" s="9" t="str">
-        <x:v>Early N63 Timing-Chain Wear Check: ISTA Test Before Repair</x:v>
+        <x:v>Front Thrust Arm Bushing (Tension Strut) Premature Wear</x:v>
       </x:c>
       <x:c r="E48" s="9" t="str">
-        <x:v>Check the VIN and service history with a BMW center, diagnose stored VANOS/camshaft faults first, and run BMW's ISTA timing-chain elongation test. If the result is 'Timing chain is OK,' do not replace parts on this claim. If it is 'not OK,' BMW SIB 11 16 14 directs replacement of both timing chains under the VIN-specific repair instruction, followed by the required oil/filter service, priming steps, programming, and shorter oil-service interval. A single tensioner 11-31-7-557-741 or a generic Cloyes kit is not the complete repair and must not be presented as what the owner needs. Tow the vehicle rather than driving it when severe mechanical noise, oil-pressure warnings, or loss of timing is present.</x:v>
+        <x:v>Replace both front thrust arms as complete assemblies (the bushings are not serviceable separately). Use genuine BMW M-spec parts or Lemforder equivalents. Perform a 4-wheel alignment immediately after replacement. Upgrade to Powerflex polyurethane thrust arm bushings for extended lifespan, especially on tracked cars.</x:v>
       </x:c>
       <x:c r="F48" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G48" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="49" ht="1227.5999755859375" hidden="0" customHeight="1">
+    <x:row r="49" ht="897.5999755859375" hidden="0" customHeight="1">
       <x:c r="A49" s="40" t="n">
         <x:v>48</x:v>
       </x:c>
       <x:c r="B49" s="9" t="str">
-        <x:v>bmw-x5-n63-wastegate-2008</x:v>
+        <x:v>bmw-x6m-s63-rod-bearing-2010</x:v>
       </x:c>
       <x:c r="C49" s="9" t="str">
-        <x:v>2010-2018 | BMW | X5 | xDrive50i | N63, N63TU</x:v>
+        <x:v>2010-2023 | BMW | X6 M | M50i, xDrive50i | S63</x:v>
       </x:c>
       <x:c r="D49" s="9" t="str">
-        <x:v>N63/N63TU Low Boost or Turbo Rattle: Diagnose Vacuum Control First</x:v>
+        <x:v>S63 Rod Bearing Failure (X6 M)</x:v>
       </x:c>
       <x:c r="E49" s="9" t="str">
-        <x:v>Read all DME faults and compare requested versus actual boost under the BMW test plan. Pressure- or smoke-test the intake and charge-air path, verify vacuum supply from the pump and reservoir, inspect both banks' hoses and pressure converters, and test actuator movement before condemning a turbocharger. Identify the engine generation, failed bank, and exact hardware in BMW ETK/AIR. Check a 2010-2013 E70 VIN for the N63 Customer Care Package only as applicable; its published six-point scope includes air-mass sensors, injectors, vacuum pump, low-pressure fuel sensor/feed line, fresh-air turbo seals, and crankcase-ventilation lines, not an automatic wastegate replacement. No retail link is published until diagnosis selects a VIN-specific component.</x:v>
+        <x:v>PREVENTIVE: Replace rod bearings every 60,000-80,000 miles ($2,500-5,000 labor-intensive job). Use ACL Race 8B1578HX-STD ($150-250) or King CR8049SV ($120-200) upgraded bearings - these are stronger than OEM and provide better durability under high loads. Send oil samples for analysis (Blackstone Labs ~$30) every 5,000 miles to monitor bearing wear metals. If bearings have already failed: engine replacement required ($15,000-30,000). DO NOT buy used X6 M without documented bearing replacement history or fresh oil analysis.</x:v>
       </x:c>
       <x:c r="F49" s="9" t="n">
         <x:v>0</x:v>
@@ -16360,136 +17722,136 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="50" ht="844.7999877929688" hidden="0" customHeight="1">
+    <x:row r="50" ht="277.20001220703125" hidden="0" customHeight="1">
       <x:c r="A50" s="40" t="n">
         <x:v>49</x:v>
       </x:c>
       <x:c r="B50" s="9" t="str">
-        <x:v>bmw-x5-oil-leaks-2000</x:v>
+        <x:v>bmw-x6m-vanos-solenoid-2015</x:v>
       </x:c>
       <x:c r="C50" s="9" t="str">
-        <x:v>2003-2006 | BMW | X5 | 3.0i | M54</x:v>
+        <x:v>2015-2021 | BMW | X6 M | S63</x:v>
       </x:c>
       <x:c r="D50" s="9" t="str">
-        <x:v>E53 3.0i M54 Valve-Cover Gasket Leak (Confirm the Source)</x:v>
+        <x:v>VANOS Solenoid Oil Sludge Buildup</x:v>
       </x:c>
       <x:c r="E50" s="9" t="str">
-        <x:v>Clean the engine and trace the highest fresh-oil source before ordering a gasket. If the leak is at the M54 cylinder-head-cover perimeter or spark-plug-well seals, inspect the plastic cover for cracks, warpage, damaged fastener grommets, and crankcase-ventilation faults. Reuse the cover only if it passes inspection, then install VIN/production-confirmed gasket set 11-12-0-030-496 with the BMW-specified grommets and sealant locations and torque sequence. If the cover or another oil circuit is the source, select that separate repair instead.</x:v>
+        <x:v>Remove and clean or replace the VANOS solenoids. Perform an engine oil flush. Strictly follow 7,500-mile oil change intervals with BMW LL-01 rated 0W-40 synthetic oil.</x:v>
       </x:c>
       <x:c r="F50" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G50" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="51" ht="1293.5999755859375" hidden="0" customHeight="1">
+    <x:row r="51" ht="699.5999755859375" hidden="0" customHeight="1">
       <x:c r="A51" s="40" t="n">
         <x:v>50</x:v>
       </x:c>
       <x:c r="B51" s="9" t="str">
-        <x:v>bmw-x5-transfer-case-actuator-2000</x:v>
+        <x:v>bmw-x7-48v-battery-2020</x:v>
       </x:c>
       <x:c r="C51" s="9" t="str">
-        <x:v>2007-2013 | BMW | X5 | 3.0si, 4.8i, xDrive30i, xDrive35d, xDrive48i, X5 M | N52, N62, M57, S63</x:v>
+        <x:v>2020-2023 | BMW | X7</x:v>
       </x:c>
       <x:c r="D51" s="9" t="str">
-        <x:v>E70 ATC700 Transfer-Case Positioning Motor (Diagnosis Required)</x:v>
+        <x:v>48V Mild Hybrid Battery Issues</x:v>
       </x:c>
       <x:c r="E51" s="9" t="str">
-        <x:v>Read BMW VTG/DSC faults and run the applicable ISTA transfer-case test plan before buying a motor. Confirm tire sizes and wear, battery voltage, wiring, transfer-case type, fluid condition, calibration, and—especially after differential or transfer-case replacement—the VIN-correct front and rear gear ratios. If testing confirms the ATC700 positioning motor and BMW ETK/AIR selects this application for the VIN, current BMW exchange servomotor 27-10-2-449-709 supersedes 27-10-7-568-267. Install the correct classification resistor/hardware supplied or specified for the VIN and perform the required VTG initialization/calibration. A generic gear-only kit is not a universal BMW repair and should not be ordered without opening and confirming the exact motor failure.</x:v>
+        <x:v>Replace the 48V mild hybrid battery ($1,000-2,000 at dealer). Requires dealer-level diagnostic tools and coding after installation - this is NOT a DIY repair. The 48V battery is separate from the main 12V battery. No aftermarket alternatives currently available. Check if vehicle is still under BMW warranty or extended warranty coverage. Some owners choose to live with the failed auto start-stop rather than pay for replacement.</x:v>
       </x:c>
       <x:c r="F51" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G51" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="52" ht="1042.800048828125" hidden="0" customHeight="1">
+    <x:row r="52" ht="726" hidden="0" customHeight="1">
       <x:c r="A52" s="40" t="n">
         <x:v>51</x:v>
       </x:c>
       <x:c r="B52" s="9" t="str">
-        <x:v>bmw-x5-transfer-case-actuator-2007</x:v>
+        <x:v>bmw-x7-air-suspension-2019</x:v>
       </x:c>
       <x:c r="C52" s="9" t="str">
-        <x:v>2019-2026 | BMW | X5</x:v>
+        <x:v>2019-2023 | BMW | X7</x:v>
       </x:c>
       <x:c r="D52" s="9" t="str">
-        <x:v>G05/F95 Transfer-Case Shudder: Tires and Fluid Diagnosis First</x:v>
+        <x:v>Air Suspension Compressor &amp; Strut Failure (Standard Equipment)</x:v>
       </x:c>
       <x:c r="E52" s="9" t="str">
-        <x:v>Follow BMW SIB 27 02 20 in order: verify all four tires for VIN-correct size, brand/application, axle placement, and wear; diagnose any powertrain faults; then use ISTA to temporarily deactivate the transfer-case clutch and road-test the complaint. Only if the shudder disappears with the VTG deactivated does BMW direct an ATX13-X oil change with DTF-1, followed by VTG calibration. The clutch plates can require up to 125 miles after the service to become fully saturated and smooth out. If the symptom remains, continue diagnosis rather than buying an actuator or transfer case. Part numbers for any further repair must be selected by VIN in ETK/AIR.</x:v>
+        <x:v>Replace failed air struts and/or compressor. Front strut left 37106869035 ($1,500-2,000), right 37106869036 ($1,500-2,000), rear 37106869039 ($1,000-1,500). Compressor 37206861882 ($800-1,200). RebuildMasterTech rebuilt struts ($600-900 each) are a more affordable alternative. Total repair can reach $2,180-5,000+ depending on which components have failed. Replace both struts on same axle simultaneously. Inspect at 50,000 miles for early signs of leaking.</x:v>
       </x:c>
       <x:c r="F52" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G52" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="53" ht="1214.4000244140625" hidden="0" customHeight="1">
+    <x:row r="53" ht="435.6000061035156" hidden="0" customHeight="1">
       <x:c r="A53" s="40" t="n">
         <x:v>52</x:v>
       </x:c>
       <x:c r="B53" s="9" t="str">
-        <x:v>bmw-x5-vanos-solenoid-2000</x:v>
+        <x:v>bmw-x7-air-suspension-compressor-2019</x:v>
       </x:c>
       <x:c r="C53" s="9" t="str">
-        <x:v>2010-2013 | BMW | X5 | xDrive30i, xDrive35i | N51, N52K, N52T, N55</x:v>
+        <x:v>2019-2026 | BMW | X7</x:v>
       </x:c>
       <x:c r="D53" s="9" t="str">
-        <x:v>VANOS Adjustment-Unit Bolt Recall 23V-707 (E70 Inline-Six)</x:v>
+        <x:v>Air Suspension Compressor Failure</x:v>
       </x:c>
       <x:c r="E53" s="9" t="str">
-        <x:v>Enter the VIN in BMW's official recall lookup and have an authorized BMW center complete recall 23V-707 if it is open. BMW's procedure is inspection-dependent: intact affected bolts are replaced; if bolts are loose or broken, the affected VANOS adjustment unit is replaced, and missing fragments must be recovered. The recall repair is free, so do not buy a solenoid or VANOS part first. If the VIN is outside the recall or a fault remains after the remedy, use BMW-capable diagnostics to test oil supply and pressure, wiring, sensors, control solenoids, adjustment units, and mechanical timing before selecting a part. If the engine runs roughly, makes unusual mechanical noise, loses power, or stalls, move out of traffic safely, stop driving, and contact BMW for transport guidance.</x:v>
+        <x:v>Replace the air suspension compressor. Inspect all four air springs for leaks using soapy water solution. Replace any leaking air springs to prevent repeated compressor failure. Check the valve block for proper operation. The compressor is located under the rear of the vehicle.</x:v>
       </x:c>
       <x:c r="F53" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G53" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="54" ht="1148.4000244140625" hidden="0" customHeight="1">
+    <x:row r="54" ht="871.2000122070312" hidden="0" customHeight="1">
       <x:c r="A54" s="40" t="n">
         <x:v>53</x:v>
       </x:c>
       <x:c r="B54" s="9" t="str">
-        <x:v>bmw-x5-water-pump-2007</x:v>
+        <x:v>bmw-x7-b58-coolant-2019</x:v>
       </x:c>
       <x:c r="C54" s="9" t="str">
-        <x:v>2011-2013 | BMW | X5 | xDrive35i | N55</x:v>
+        <x:v>2019-2023 | BMW | X7 | xDrive40i | B58</x:v>
       </x:c>
       <x:c r="D54" s="9" t="str">
-        <x:v>E70 xDrive35i N55 Electric Coolant Pump (Fault-Confirmed)</x:v>
+        <x:v>B58 Coolant System Failures (xDrive40i)</x:v>
       </x:c>
       <x:c r="E54" s="9" t="str">
-        <x:v>If the engine-temperature warning appears, stop safely, shut the engine off, and tow the vehicle if normal temperature cannot be confirmed. When cool, check coolant level and leaks, read BMW-specific faults, verify pump power/ground and communication, and run the ISTA coolant-pump activation/test plan. If those tests confirm the pump and BMW ETK/AIR selects 11-51-5-A05-704 for the VIN, replace it using the BMW procedure, select the thermostat separately only if testing or preventive planning justifies it, vacuum-fill or bleed the system as specified, and verify commanded pump operation and stable temperature. Do not use a fixed-mileage rule or this part number for an N52, N63, or F15 without VIN confirmation.</x:v>
+        <x:v>Replace failed coolant system components. Water pump 11518482250 ($300-400). Thermostat 11537644811 ($150-250). Replace expansion tank and all plastic coolant connections when performing repair to prevent cascading failures. For 2023+ models, check VIN for recall 24V-608 coverage for coolant pump connector. Total repair $500-2,500 depending on extent of damage. PREVENTIVE: Replace thermostat and water pump at 60,000-70,000 miles before failure. Inspect coolant hoses and connections at every oil change after 50k miles.</x:v>
       </x:c>
       <x:c r="F54" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G54" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="55" ht="1056" hidden="0" customHeight="1">
+    <x:row r="55" ht="435.6000061035156" hidden="0" customHeight="1">
       <x:c r="A55" s="40" t="n">
         <x:v>54</x:v>
       </x:c>
       <x:c r="B55" s="9" t="str">
-        <x:v>bmw-x5m-brake-system-2010</x:v>
+        <x:v>bmw-x7-b58-coolant-expansion-tank-2019</x:v>
       </x:c>
       <x:c r="C55" s="9" t="str">
-        <x:v>2010-2023 | BMW | X5 M</x:v>
+        <x:v>2019-2026 | BMW | X7 | B58</x:v>
       </x:c>
       <x:c r="D55" s="9" t="str">
-        <x:v>Heavy-Duty Brake System Accelerated Wear - E70/F85/F95 X5 M</x:v>
+        <x:v>B58 Coolant Expansion Tank Crack</x:v>
       </x:c>
       <x:c r="E55" s="9" t="str">
-        <x:v>E70 X5 M brakes: OEM front pads 34116799964 ($150-$250), rear pads 34216794879 ($120-$200). F85 X5 M front brake rotors: 34112284101/34112284102 with 6-pot caliper 34117845747/34117845748 and pads 34112284869. F85 rear: 385mm x 24mm perforated rotors 34212284903/34212284904 with 4-pot Brembo caliper and Textar pads. Budget $1,500-$2,500 per axle for complete brake service. For track use: EBC Yellowstuff or Hawk HPS 5.0 pads ($200-$350 per axle) with StopTech slotted rotors for improved heat management. Use Motul RBF 660 or ATE Typ 200 brake fluid - flush every 12 months. Budget $3,000-$5,000 per year for brake maintenance if driving spiritedly.</x:v>
+        <x:v>Replace the coolant expansion tank with an updated BMW part that uses improved plastic composition. Also replace the cap and inspect all coolant hoses. Flush and refill the cooling system with BMW-approved coolant. Check for coolant contamination from the old tank.</x:v>
       </x:c>
       <x:c r="F55" s="9" t="n">
         <x:v>0</x:v>
@@ -16498,21 +17860,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="56" ht="1122" hidden="0" customHeight="1">
+    <x:row r="56" ht="646.7999877929688" hidden="0" customHeight="1">
       <x:c r="A56" s="40" t="n">
         <x:v>55</x:v>
       </x:c>
       <x:c r="B56" s="9" t="str">
-        <x:v>bmw-x5m-rear-differential-2010</x:v>
+        <x:v>bmw-x7-ibs-brake-recall-2023</x:v>
       </x:c>
       <x:c r="C56" s="9" t="str">
-        <x:v>2010-2023 | BMW | X5 M | S63</x:v>
+        <x:v>2023-2025 | BMW | X7</x:v>
       </x:c>
       <x:c r="D56" s="9" t="str">
-        <x:v>Rear Differential Wear &amp; Fluid Degradation - E70/F85/F95 X5 M</x:v>
+        <x:v>2023-2025 X7 Integrated Brake System Recall 26V-422</x:v>
       </x:c>
       <x:c r="E56" s="9" t="str">
-        <x:v>Change rear differential fluid every 30,000 miles (ignore BMW "lifetime fill" claim). E70 X5 M: No drain plug - fluid must be extracted through fill port with hand pump or suction device. Recommended fluid: Royal Purple 75W-140 GL5 synthetic or Red Line 75W-140 GL5 ($40-$60 per fill). Capacity approximately 1.2 liters. For limited-slip diff, ensure fluid is GL5 rated with limited-slip additive. If differential is making whining/howling noise: have a limited-slip differential specialist inspect internals (not generic BMW shop). Diff rebuild: $1,500-$3,000 at specialist. Complete differential replacement: $3,000-$5,500 + labor. Labor for fluid change: $150-$300 at independent shop.</x:v>
+        <x:v>Check the VIN at NHTSA and with an authorized BMW dealer when campaign 26V-422 VINs become searchable, and arrange the free dealer inspection and module replacement if required. If a brake warning appears or pedal effort increases, avoid abrupt braking, allow extra stopping distance, stop safely and contact BMW roadside assistance; do not order brake electronics from this card.</x:v>
       </x:c>
       <x:c r="F56" s="9" t="n">
         <x:v>0</x:v>
@@ -16521,21 +17883,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="57" ht="1386" hidden="0" customHeight="1">
+    <x:row r="57" ht="897.5999755859375" hidden="0" customHeight="1">
       <x:c r="A57" s="40" t="n">
         <x:v>56</x:v>
       </x:c>
       <x:c r="B57" s="9" t="str">
-        <x:v>bmw-x5m-s63-cooling-system-2010</x:v>
+        <x:v>bmw-x7-n63-oil-consumption-2019</x:v>
       </x:c>
       <x:c r="C57" s="9" t="str">
-        <x:v>2010-2023 | BMW | X5 M | 4.4i, 4.6is, 4.8is, M50i, M60i, xDrive48i, xDrive50e, xDrive50i | S63</x:v>
+        <x:v>2019-2023 | BMW | X7 | M50i, M60i, xDrive50i | N63TU3</x:v>
       </x:c>
       <x:c r="D57" s="9" t="str">
-        <x:v>S63 Cooling System Component Failures - E70/F85/F95 X5 M</x:v>
+        <x:v>N63TU3 Oil Consumption &amp; Valve Stem Seal Degradation (xDrive50i/M50i/M60i)</x:v>
       </x:c>
       <x:c r="E57" s="9" t="str">
-        <x:v>PROACTIVE MAINTENANCE SCHEDULE: Replace electric water pump at 60,000 miles ($400-$700 + labor). Replace thermostat at same time ($150-$250). Replace expansion tank at 60,000-80,000 miles ($100-$200). Inspect all coolant hoses at every oil change - replace any that are soft, bulging, or showing surface cracks. E70 X5 M expansion tank vent hose: 17128627119 ($30-$50). Flush coolant system every 2 years or 30,000 miles (more frequent than BMW's 4-year recommendation). Use ONLY BMW coolant mixed 50/50 with distilled water. For E70 hot-V turbo coolant lines: GRYPHONTEK repair kit eliminates plastic T-fitting failure (see separate issue entry). Budget $1,500-$2,500 for complete cooling system refresh at 60,000 miles. This prevents catastrophic overheating that can destroy the S63 engine ($15,000-$34,000 engine replacement).</x:v>
+        <x:v>Replace valve stem seals - extremely labor-intensive job requiring cylinder head work ($4,900-12,000 total). Elring seals 11340039494 for OEM spec. 5150 AutoSport Viton upgraded seals ($150-200) recommended for better heat resistance. AGA Tools kit includes specialized tools required. Reference TSB MC-10149960-9999 when visiting dealer. Check eligibility for class action settlement coverage. Some owners monitor oil levels and top off rather than repair. Use quality synthetic 0W-40 BMW LL-01 spec oil and check level every 500-1,000 miles.</x:v>
       </x:c>
       <x:c r="F57" s="9" t="n">
         <x:v>0</x:v>
@@ -16544,21 +17906,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="58" ht="1135.199951171875" hidden="0" customHeight="1">
+    <x:row r="58" ht="396" hidden="0" customHeight="1">
       <x:c r="A58" s="40" t="n">
         <x:v>57</x:v>
       </x:c>
       <x:c r="B58" s="9" t="str">
-        <x:v>bmw-x5m-s63-oil-leaks-2010</x:v>
+        <x:v>bmw-x7-panoramic-roof-rattle-2019</x:v>
       </x:c>
       <x:c r="C58" s="9" t="str">
-        <x:v>2010-2023 | BMW | X5 M | 4.4i, 4.6is, 4.8is, M50i, M60i, xDrive48i, xDrive50e, xDrive50i | S63</x:v>
+        <x:v>2019-2026 | BMW | X7</x:v>
       </x:c>
       <x:c r="D58" s="9" t="str">
-        <x:v>S63 V8 Chronic Oil Leaks (Valve Cover, Oil Pan, Turbo Lines) - E70/F85/F95 X5 M</x:v>
+        <x:v>Panoramic Sunroof Rattle and Creak</x:v>
       </x:c>
       <x:c r="E58" s="9" t="str">
-        <x:v>Valve cover gasket replacement (both sides): $1,200-$2,500 with labor. BMW plastic valve covers can crack and must be replaced entirely (not just gasket) - inspect during service. Oil filter housing gasket: $400-$800 with labor. Oil pan gasket: $2,000-$3,500 (requires engine/subframe drop). Turbo oil feed/return lines: replace with GRYPHONTEK or MAMBA upgraded silicone/braided lines during any turbo service ($200-$400). VANOS solenoid seals: $100-$200 (DIY-friendly). For comprehensive oil leak repair at 80,000+ miles: budget $3,000-$5,000 to address all common leak points simultaneously. Valve cover bolt torque is CRITICAL - too tight cracks the cover ($800-$1,200 per cover), too loose and it leaks.</x:v>
+        <x:v>Apply BMW-approved felt tape or lubricant to sunroof guide rails. Replace worn guide rail bushings. In severe cases, the sunroof cassette or seal may need replacement under warranty. BMW has issued updated guide rail components for early production vehicles.</x:v>
       </x:c>
       <x:c r="F58" s="9" t="n">
         <x:v>0</x:v>
@@ -16567,21 +17929,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="59" ht="1412.4000244140625" hidden="0" customHeight="1">
+    <x:row r="59" ht="778.7999877929688" hidden="0" customHeight="1">
       <x:c r="A59" s="40" t="n">
         <x:v>58</x:v>
       </x:c>
       <x:c r="B59" s="9" t="str">
-        <x:v>bmw-x5m-s63-rod-bearing-2010</x:v>
+        <x:v>bmw-x7-sunroof-leak-2019</x:v>
       </x:c>
       <x:c r="C59" s="9" t="str">
-        <x:v>2010-2018 | BMW | X5 M | 4.4i, 4.6is, 4.8is, M50i, M60i, xDrive48i, xDrive50e, xDrive50i</x:v>
+        <x:v>2019-2023 | BMW | X7</x:v>
       </x:c>
       <x:c r="D59" s="9" t="str">
-        <x:v>S63 V8 Rod Bearing Premature Wear &amp; Failure - E70/F85 X5 M</x:v>
+        <x:v>Panoramic Sunroof Water Leak</x:v>
       </x:c>
       <x:c r="E59" s="9" t="str">
-        <x:v>PREVENTIVE: For track-driven X5 M, replace rod bearings proactively at 60,000-80,000 miles. ACL Race Series rod bearings (8B1578HX-STD for S63B44, +0.001" extra oil clearance) are the community gold standard ($200-$350 for bearing set). WPC surface-treated bearings from Lang Racing are the premium choice ($400-$600 set). Total cost for preventive rod bearing service: $4,500-$8,500 depending on shop. Oil analysis every 5,000 miles through Blackstone Labs ($30/test) to monitor bearing wear metals (lead and copper). Use only BMW 10W-60 synthetic oil with 5,000-7,500 mile oil change intervals. Never track the car on cold oil. Mporium BMW offers specialized S63 rod bearing service starting at $4,499. If catastrophic failure: rebuilt S63 engine from RK Autowerks (~$8,500 + installation), new BMW engine (~$34,000), or complete engine rebuild ($12,000-$18,000).</x:v>
+        <x:v>Clear clogged sunroof drain tubes ($100-300 at shop). Reference TSB SIB 54 11 19 when visiting dealer. For persistent leaks, drain tube connections or sunroof seal may need replacement ($500-1,500). If water has damaged interior electronics, repair costs can reach $3,000. PREVENTIVE: Clear sunroof drains annually, especially in areas with heavy tree debris. Run compressed air or flexible drain snake through drain tubes during oil changes. Keep sunroof track clean of debris.</x:v>
       </x:c>
       <x:c r="F59" s="9" t="n">
         <x:v>0</x:v>
@@ -16590,21 +17952,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="60" ht="1214.4000244140625" hidden="0" customHeight="1">
+    <x:row r="60" ht="739.2000122070312" hidden="0" customHeight="1">
       <x:c r="A60" s="40" t="n">
         <x:v>59</x:v>
       </x:c>
       <x:c r="B60" s="9" t="str">
-        <x:v>bmw-x5m-s63-turbo-coolant-line-2010</x:v>
+        <x:v>bmw-x7-tire-wear-2019</x:v>
       </x:c>
       <x:c r="C60" s="9" t="str">
-        <x:v>2010-2013 | BMW | X5 M</x:v>
+        <x:v>2019-2023 | BMW | X7</x:v>
       </x:c>
       <x:c r="D60" s="9" t="str">
-        <x:v>S63 Turbo Coolant Line Plastic T-Fitting Failure (Hot-V Design) - E70 X5 M</x:v>
+        <x:v>Premature Tire Wear (Especially 21"/22" Wheels)</x:v>
       </x:c>
       <x:c r="E60" s="9" t="str">
-        <x:v>Replace ALL factory plastic turbo coolant T-fittings and hoses with GRYPHONTEK S63 Turbo Coolant Line Repair Kit ($200-$400). Kit includes pre-shaped multi-layer reinforced silicone hoses, brass T-fittings (replacing factory plastic), and all necessary hose clamps. Direct bolt-on installation designed for the E70/E71 S63 engine bay. MAMBA Turbo also offers a reinforced turbo coolant line kit with brass and silicone components ($150-$350). This is a PROACTIVE replacement - do not wait for failure. Replace at first sign of coolant weeping or during any turbo service. Labor: $800-$1,500 due to tight access in hot-V engine valley. If turbo bearings are damaged from overheating: turbo replacement $3,000-$5,000 per unit.</x:v>
+        <x:v>Have alignment adjusted to reduce aggressive camber settings ($200-400). Switch to quality tires designed for heavy SUVs: Michelin Pilot Sport 4S or Continental PremiumContact 6 are recommended. If possible, avoid 22" wheels and opt for 21" or smaller for better tire longevity and ride comfort. Alignment adjustment can extend tire life from 15,000 to 30,000+ miles. Total cost $200-2,000 depending on tire replacement needs. Check alignment every 10,000 miles.</x:v>
       </x:c>
       <x:c r="F60" s="9" t="n">
         <x:v>0</x:v>
@@ -16613,21 +17975,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="61" ht="1135.199951171875" hidden="0" customHeight="1">
+    <x:row r="61" ht="501.6000061035156" hidden="0" customHeight="1">
       <x:c r="A61" s="40" t="n">
         <x:v>60</x:v>
       </x:c>
       <x:c r="B61" s="9" t="str">
-        <x:v>bmw-x5m-s63-vanos-solenoid-2010</x:v>
+        <x:v>bmw-xm-airbag-passenger-knee-recall-2023</x:v>
       </x:c>
       <x:c r="C61" s="9" t="str">
-        <x:v>2010-2023 | BMW | X5 M | 4.4i, 4.6is, 4.8is, M50i, M60i, xDrive48i, xDrive50e, xDrive50i | S63</x:v>
+        <x:v>2023-2023 | BMW | XM</x:v>
       </x:c>
       <x:c r="D61" s="9" t="str">
-        <x:v>S63 VANOS Solenoid Failure - E70/F85/F95 X5 M</x:v>
+        <x:v>2023 XM Front-Passenger Knee-Airbag Recall 23V-622</x:v>
       </x:c>
       <x:c r="E61" s="9" t="str">
-        <x:v>Replace all 4 VANOS solenoids simultaneously - they are same age and if one has failed, others are close behind. Pierburg 11368605123 (OEM supplier) at $30-$50 each from Turner Motorsport or BimmerWorld. Genuine BMW 11368482268 for S63TU applications at $50-$70 each. Total parts cost: $120-$280 for all 4 solenoids. Also replace VANOS solenoid O-rings and filter screens during service. Labor: 1-2 hours professional ($150-$400 labor). This is one of the easier S63 repairs - accessible from top of engine without removing intake manifold. Natafox and Febi also offer quality aftermarket VANOS solenoids at lower cost ($20-$35 each). Clean VANOS system with fresh oil change immediately after solenoid replacement.</x:v>
+        <x:v>Check the VIN for an open 23V-622 campaign. If open, an authorized BMW dealer replaces the front-passenger knee airbag free of charge. Do not attempt airbag diagnosis or order a clock spring or airbag module from this card; supplemental-restraint work requires trained personnel and VIN-selected parts.</x:v>
       </x:c>
       <x:c r="F61" s="9" t="n">
         <x:v>0</x:v>
@@ -16636,21 +17998,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="62" ht="1293.5999755859375" hidden="0" customHeight="1">
+    <x:row r="62" ht="567.5999755859375" hidden="0" customHeight="1">
       <x:c r="A62" s="40" t="n">
         <x:v>61</x:v>
       </x:c>
       <x:c r="B62" s="9" t="str">
-        <x:v>bmw-x5m-s63-wastegate-rattle-2010</x:v>
+        <x:v>bmw-xm-hybrid-drivetrain-hesitation-2023</x:v>
       </x:c>
       <x:c r="C62" s="9" t="str">
-        <x:v>2010-2018 | BMW | X5 M | S63</x:v>
+        <x:v>2023-2024 | BMW | XM | S68 4.4L Twin-Turbo V8 Hybrid, S68</x:v>
       </x:c>
       <x:c r="D62" s="9" t="str">
-        <x:v>S63 Twin Turbo Wastegate Rattle - E70/F85 X5 M</x:v>
+        <x:v>Hybrid Drivetrain Hesitation and Power Delivery Lag</x:v>
       </x:c>
       <x:c r="E62" s="9" t="str">
-        <x:v>Option 1 (Most cost-effective): MAMBA SUS316 stainless steel wastegate rattle flapper repair kit for S63 MGT2260 (part 077-0024, replaces 790463-2 / 790484-3), approximately $150-$300 per turbo. Requires turbo removal for installation. Option 2: Lskioer turbo wastegate rattle flapper repair kit for S63/S63TU MGT2260DSL ($80-$150 per kit on Amazon). Option 3: Replace turbo wastegate actuators with new OEM units ($300-$500 each). Option 4: Full turbocharger replacement with new or remanufactured units ($3,000-$5,000 per turbo + labor). Labor for turbo removal and reinstallation: $2,000-$3,500 for both turbos. While turbos are out: replace turbo oil feed/return lines, coolant lines, and all gaskets (GRYPHONTEK turbo coolant line repair kit for E70 X5M, ~$200-$400).</x:v>
+        <x:v>Visit the dealer for the latest transmission and hybrid system software calibration updates. Select Sport or Sport Plus mode for more consistent power delivery. The latest software revisions significantly improve the electric-to-V8 handoff smoothness. If hesitation persists after updates, the dealer can reset the transmission adaptation values to relearn driving patterns.</x:v>
       </x:c>
       <x:c r="F62" s="9" t="n">
         <x:v>0</x:v>
@@ -16659,21 +18021,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="63" ht="1069.199951171875" hidden="0" customHeight="1">
+    <x:row r="63" ht="646.7999877929688" hidden="0" customHeight="1">
       <x:c r="A63" s="40" t="n">
         <x:v>62</x:v>
       </x:c>
       <x:c r="B63" s="9" t="str">
-        <x:v>bmw-x5m-transfer-case-actuator-2010</x:v>
+        <x:v>bmw-xm-integrated-brake-system-recall-2023</x:v>
       </x:c>
       <x:c r="C63" s="9" t="str">
-        <x:v>2010-2023 | BMW | X5 M</x:v>
+        <x:v>2023-2024 | BMW | XM</x:v>
       </x:c>
       <x:c r="D63" s="9" t="str">
-        <x:v>xDrive Transfer Case Actuator Motor Failure - E70/F85/F95 X5 M</x:v>
+        <x:v>2023-2024 XM Integrated Brake System Recall 26V-422</x:v>
       </x:c>
       <x:c r="E63" s="9" t="str">
-        <x:v>Replace transfer case actuator motor. E70 X5 M: BMW 27107566296 or equivalent ($250-$450 for actuator motor). F85 X5 M: BMW 27608643153 or equivalent ($300-$500). F95 X5 M: check VIN-specific part number with dealer. FCP Euro has an excellent DIY guide for BMW transfer case actuator repair - the actuator can be replaced without removing the entire transfer case. Labor: 2-3 hours at specialist shop ($300-$600 labor). Change transfer case fluid at same time with BMW DTF-1 specification fluid. XeMODeX offers remanufactured transfer case actuator motors at reduced cost ($200-$350). For complete transfer case failure: $3,500-$6,000 for replacement unit + labor.</x:v>
+        <x:v>Check the VIN at NHTSA and with an authorized BMW dealer when campaign 26V-422 VINs become searchable, and arrange the free dealer inspection and module replacement if required. If a brake warning appears or pedal effort increases, avoid abrupt braking, allow extra stopping distance, stop safely and contact BMW roadside assistance; wheel-speed sensors are not the recall remedy.</x:v>
       </x:c>
       <x:c r="F63" s="9" t="n">
         <x:v>0</x:v>
@@ -16682,21 +18044,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="64" ht="435.6000061035156" hidden="0" customHeight="1">
+    <x:row r="64" ht="646.7999877929688" hidden="0" customHeight="1">
       <x:c r="A64" s="40" t="n">
         <x:v>63</x:v>
       </x:c>
       <x:c r="B64" s="9" t="str">
-        <x:v>bmw-x6-adaptive-drive-malfunction-2008</x:v>
+        <x:v>bmw-xm-suspension-ride-quality-2023</x:v>
       </x:c>
       <x:c r="C64" s="9" t="str">
-        <x:v>2008-2019 | BMW | X6</x:v>
+        <x:v>2023-2024 | BMW | XM | S68 4.4L Twin-Turbo V8 Hybrid</x:v>
       </x:c>
       <x:c r="D64" s="9" t="str">
-        <x:v>Adaptive Drive System Malfunction</x:v>
+        <x:v>Harsh Ride Quality and Suspension Stiffness</x:v>
       </x:c>
       <x:c r="E64" s="9" t="str">
-        <x:v>Diagnose specific Adaptive Drive component failure using BMW ISTA diagnostics. Replace the failed component — most commonly the hydraulic pump or valve block. If repair cost is prohibitive, some owners convert to conventional anti-roll bars as a permanent fix at lower cost.</x:v>
+        <x:v>Check tire pressures regularly - overinflated tires significantly worsen the harsh ride. Some owners report improved comfort by switching to a tire with a taller sidewall profile (if available for the XM's wheel size). Use Comfort mode for daily driving. Unfortunately, no aftermarket spring or damper solution currently exists to significantly improve the ride without compromising the handling needed for the XM's weight.</x:v>
       </x:c>
       <x:c r="F64" s="9" t="n">
         <x:v>0</x:v>
@@ -16705,21 +18067,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="65" ht="858" hidden="0" customHeight="1">
+    <x:row r="65" ht="528" hidden="0" customHeight="1">
       <x:c r="A65" s="40" t="n">
         <x:v>64</x:v>
       </x:c>
       <x:c r="B65" s="9" t="str">
-        <x:v>bmw-x6-air-suspension-2008</x:v>
+        <x:v>bmw-z3-convertible-top-rear-window-cracking-clouding-bead-separatio</x:v>
       </x:c>
       <x:c r="C65" s="9" t="str">
-        <x:v>2008-2023 | BMW | X6</x:v>
+        <x:v>1996-2002 | BMW | Z3</x:v>
       </x:c>
       <x:c r="D65" s="9" t="str">
-        <x:v>Air Suspension Compressor &amp; Strut Failure</x:v>
+        <x:v>Convertible Top Rear Window Cracking, Clouding, and Bead Separation</x:v>
       </x:c>
       <x:c r="E65" s="9" t="str">
-        <x:v>Replace failed air springs or compressor. Arnott rear air spring A-2642 ($200-300 each). OEM F16 spring 37126795013 ($200). Arnott compressor P-2655 ($599). Or convert to coil springs: Strutmasters BB2RBM conversion kit ($1,200-1,800) permanently eliminates air suspension issues. Conversion is cheaper long-term than continued air suspension repairs. If keeping air suspension: inspect air springs at 60,000-80,000 miles for cracks/leaks before compressor damage occurs. Replace both air springs on same axle simultaneously.</x:v>
+        <x:v>Replace the rear window panel only — BMW used a zipper system so the clouded/cracked window unzips and a new window zips/tapes in without disturbing the fabric top. Re-gluing separated bead trim rarely holds, so window replacement is the durable fix. Job is a DIY-feasible 1-1.5 hours; replace the whole top only if the fabric is also degraded.</x:v>
       </x:c>
       <x:c r="F65" s="9" t="n">
         <x:v>0</x:v>
@@ -16728,22 +18090,20 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="66" ht="646.7999877929688" hidden="0" customHeight="1">
+    <x:row r="66" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A66" s="40" t="n">
         <x:v>65</x:v>
       </x:c>
       <x:c r="B66" s="9" t="str">
-        <x:v>bmw-x6-ibs-brake-recall-2023</x:v>
+        <x:v>bmw-z3-cooling-system-failure-1996</x:v>
       </x:c>
       <x:c r="C66" s="9" t="str">
-        <x:v>2024-2024 | BMW | X6</x:v>
+        <x:v>1996-2002 | BMW | Z3</x:v>
       </x:c>
       <x:c r="D66" s="9" t="str">
-        <x:v>2024 X6 Integrated Brake System Recall 26V-422</x:v>
-      </x:c>
-      <x:c r="E66" s="9" t="str">
-        <x:v>Check the VIN at NHTSA and with an authorized BMW dealer when campaign 26V-422 VINs become searchable, and arrange the free dealer inspection and module replacement if required. If a brake warning appears or pedal effort increases, avoid abrupt braking, allow extra stopping distance, stop safely and contact BMW roadside assistance; do not order brake electronics from this card.</x:v>
-      </x:c>
+        <x:v>Cooling System Component Failures</x:v>
+      </x:c>
+      <x:c r="E66" s="9" t="str"/>
       <x:c r="F66" s="9" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -16751,21 +18111,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="67" ht="924" hidden="0" customHeight="1">
+    <x:row r="67" ht="448.79998779296875" hidden="0" customHeight="1">
       <x:c r="A67" s="40" t="n">
         <x:v>66</x:v>
       </x:c>
       <x:c r="B67" s="9" t="str">
-        <x:v>bmw-x6-n63-timing-chain-2008</x:v>
+        <x:v>bmw-z3-cracked-exhaust-manifold-1-9l-4-cylinder</x:v>
       </x:c>
       <x:c r="C67" s="9" t="str">
-        <x:v>2008-2018 | BMW | X6 | M50i, xDrive50i</x:v>
+        <x:v>1996-2002 | BMW | Z3 | 1.9, 1.9i, Z3 1.9 | 1.9L M44 4-cylinder, 1.9L M43TU 4-cylinder</x:v>
       </x:c>
       <x:c r="D67" s="9" t="str">
-        <x:v>N63 Timing Chain Stretch &amp; Guide Failure (E71/F16 xDrive50i)</x:v>
+        <x:v>Cracked Exhaust Manifold on 1.9L 4-Cylinder (M44/M43)</x:v>
       </x:c>
       <x:c r="E67" s="9" t="str">
-        <x:v>PREVENTIVE REPLACEMENT: If you own 2008-2014 E71 xDrive50i with N63, replace timing chain guides and tensioners IMMEDIATELY at 60,000-80,000 miles ($4,000-6,000) BEFORE failure. IWIS timing chain kit 90001521 ($800-1,200) or Turner kit 11317594899KT recommended. Replace lower chain guide 11147574373 at same time. If chain has already failed: complete engine replacement required ($15,000-25,000). Check VIN with BMW dealer for extended warranty eligibility. 2015+ N63TU engines have improved timing components but still require monitoring.</x:v>
+        <x:v>Inspect the manifold for hairline cracks (a cold-engine listen or smoke test confirms the leak). Replace the cracked manifold with a used OE unit or an aftermarket stainless tubular header, and renew the manifold gasket and hardware. Allow roughly 3-4 hours labor.</x:v>
       </x:c>
       <x:c r="F67" s="9" t="n">
         <x:v>0</x:v>
@@ -16774,21 +18134,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="68" ht="409.20001220703125" hidden="0" customHeight="1">
+    <x:row r="68" ht="686.4000244140625" hidden="0" customHeight="1">
       <x:c r="A68" s="40" t="n">
         <x:v>67</x:v>
       </x:c>
       <x:c r="B68" s="9" t="str">
-        <x:v>bmw-x6-n63-valve-stem-seal-wear-2008</x:v>
+        <x:v>bmw-z3-differential-mount-ear-trunk-floor-pan-tearing</x:v>
       </x:c>
       <x:c r="C68" s="9" t="str">
-        <x:v>2008-2019 | BMW | X6 | N63</x:v>
+        <x:v>1996-2002 | BMW | Z3</x:v>
       </x:c>
       <x:c r="D68" s="9" t="str">
-        <x:v>N63 Valve Stem Seal Degradation and Oil Burning</x:v>
+        <x:v>Differential Mount Ear and Trunk Floor Pan Tearing</x:v>
       </x:c>
       <x:c r="E68" s="9" t="str">
-        <x:v>Replace all intake and exhaust valve stem seals. This is a major job requiring head work. Also replace turbo oil return lines and update engine software per BMW N63 Customer Care Package specifications. Ensure proper oil grade (BMW LL-01) is used.</x:v>
+        <x:v>Inspect the trunk floor around the differential mount and rear subframe pickup points for cracks, torn metal, and broken spot welds. Repair requires welding and a reinforcement/re-fabrication plate kit to tie the diff mount/subframe back into the floor. Switching the diff carrier bushings to polyurethane reduces carrier movement and the stress that causes the tearing. Catching it early greatly limits the repair scope.</x:v>
       </x:c>
       <x:c r="F68" s="9" t="n">
         <x:v>0</x:v>
@@ -16797,21 +18157,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="69" ht="858" hidden="0" customHeight="1">
+    <x:row r="69" ht="514.7999877929688" hidden="0" customHeight="1">
       <x:c r="A69" s="40" t="n">
         <x:v>68</x:v>
       </x:c>
       <x:c r="B69" s="9" t="str">
-        <x:v>bmw-x6-n63-valve-stem-seals-2008</x:v>
+        <x:v>bmw-z3-door-window-regulator-clip-mounting-tab-failure</x:v>
       </x:c>
       <x:c r="C69" s="9" t="str">
-        <x:v>2008-2023 | BMW | X6 | M50i, xDrive50i | N63</x:v>
+        <x:v>1996-2002 | BMW | Z3</x:v>
       </x:c>
       <x:c r="D69" s="9" t="str">
-        <x:v>N63 Valve Stem Seal / Oil Consumption (xDrive50i)</x:v>
+        <x:v>Door Window Regulator Clip / Mounting Tab Failure</x:v>
       </x:c>
       <x:c r="E69" s="9" t="str">
-        <x:v>Replace valve stem seals - extremely labor-intensive job requiring cylinder head work ($4,900-12,000 total). Elring seals 11340039494 ($80-120/set of 16, need 2 sets for V8). 5150 AutoSport Viton upgraded seals ($150-200) are recommended for better heat resistance in hot-vee configuration. AGA Tools kit AGA-N63-VSK-K ($500-800) includes specialized tools required. Reference TSB MC-10149960-9999 when visiting dealer. Some owners monitor oil levels and add as needed rather than repair. Use quality synthetic 0W-40 BMW LL-01 spec oil.</x:v>
+        <x:v>Replace the broken plastic regulator clips, or replace the regulator assembly if the cable or mechanism is also worn. If the welded mounting tab/anchor has torn from the door frame, it must be re-welded or reinforced before fitting a new regulator. Lubricate the window channels to reduce drag on the new parts.</x:v>
       </x:c>
       <x:c r="F69" s="9" t="n">
         <x:v>0</x:v>
@@ -16820,21 +18180,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="70" ht="818.4000244140625" hidden="0" customHeight="1">
+    <x:row r="70" ht="686.4000244140625" hidden="0" customHeight="1">
       <x:c r="A70" s="40" t="n">
         <x:v>69</x:v>
       </x:c>
       <x:c r="B70" s="9" t="str">
-        <x:v>bmw-x6-n63-wastegate-2008</x:v>
+        <x:v>bmw-z3-fuel-level-sender-failure-causing-erratic-dead-fuel-gauge</x:v>
       </x:c>
       <x:c r="C70" s="9" t="str">
-        <x:v>2008-2018 | BMW | X6 | M50i, xDrive50i</x:v>
+        <x:v>1996-2002 | BMW | Z3</x:v>
       </x:c>
       <x:c r="D70" s="9" t="str">
-        <x:v>N63 Turbo Wastegate Rattle (xDrive50i)</x:v>
+        <x:v>Fuel Level Sender Failure Causing Erratic or Dead Fuel Gauge</x:v>
       </x:c>
       <x:c r="E70" s="9" t="str">
-        <x:v>Repair options range from flapper repair kits ($50-100/turbo) to complete turbocharger replacement ($4,000-8,000 for both). Garrett MGT2256S flapper repair kit ($50-100 per turbo) is cheapest fix. MAMBA adjustable actuator kit ($150-300) provides more durable solution. OEM actuators 11657646093 available from BMW. Complete turbo replacement $2,000-4,000 per turbo. MONITORING: Wastegate rattle is early warning - address before complete turbo failure to avoid $8,000+ repair.</x:v>
+        <x:v>Remove the access panel behind the seats and inspect the sender. A dirty or lightly worn ceramic/resistor plate can sometimes be cleaned, but a cracked plate or worn brushes requires replacing the sender unit (or the complete fuel-pump/sender carrier assembly). Also check the tank vent valve, as tank vacuum can deform the float arm. Confirm wiring/ground integrity before condemning the sender.</x:v>
       </x:c>
       <x:c r="F70" s="9" t="n">
         <x:v>0</x:v>
@@ -16843,21 +18203,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="71" ht="409.20001220703125" hidden="0" customHeight="1">
+    <x:row r="71" ht="488.3999938964844" hidden="0" customHeight="1">
       <x:c r="A71" s="40" t="n">
         <x:v>70</x:v>
       </x:c>
       <x:c r="B71" s="9" t="str">
-        <x:v>bmw-x6-rear-differential-bushing-2008</x:v>
+        <x:v>bmw-z3-hvac-blower-final-stage-resistor-failure</x:v>
       </x:c>
       <x:c r="C71" s="9" t="str">
-        <x:v>2008-2026 | BMW | X6</x:v>
+        <x:v>1996-2002 | BMW | Z3</x:v>
       </x:c>
       <x:c r="D71" s="9" t="str">
-        <x:v>Rear Differential Bushing Deterioration</x:v>
+        <x:v>HVAC Blower Final Stage Resistor Failure (Fan Only Works on Max)</x:v>
       </x:c>
       <x:c r="E71" s="9" t="str">
-        <x:v>Replace all rear differential mount bushings. Use OEM or equivalent quality bushings (Lemforder is the OEM supplier). Inspect the differential housing for any damage from excessive movement. Perform subframe alignment check after bushing replacement.</x:v>
+        <x:v>Replace the blower final stage resistor (A/C cars: part under the scuttle/cowl; non-A/C cars: behind the passenger footwell panel). If a new resistor does not restore all speeds, test the blower motor itself, which may also be worn. Inspect for corrosion/water intrusion at the cowl on A/C cars.</x:v>
       </x:c>
       <x:c r="F71" s="9" t="n">
         <x:v>0</x:v>
@@ -16866,21 +18226,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="72" ht="765.5999755859375" hidden="0" customHeight="1">
+    <x:row r="72" ht="1584" hidden="0" customHeight="1">
       <x:c r="A72" s="40" t="n">
         <x:v>71</x:v>
       </x:c>
       <x:c r="B72" s="9" t="str">
-        <x:v>bmw-x6-transfer-case-2008</x:v>
+        <x:v>bmw-z3-rear-subframe-crack-1996</x:v>
       </x:c>
       <x:c r="C72" s="9" t="str">
-        <x:v>2008-2023 | BMW | X6</x:v>
+        <x:v>1996-2002 | BMW | Z3</x:v>
       </x:c>
       <x:c r="D72" s="9" t="str">
-        <x:v>Transfer Case Actuator Motor Failure (All xDrive Models)</x:v>
+        <x:v>Rear Subframe Mounting Point Cracking</x:v>
       </x:c>
       <x:c r="E72" s="9" t="str">
-        <x:v>Replace the actuator motor assembly or rebuild using an aftermarket gear repair kit ($100-150). G06 actuator motor 27609469023 ($400-600) for complete replacement. DIY gear repair kits are straightforward and save $1,200+ over dealer replacement. Complete transfer case replacement if internal damage occurred: $1,400-3,300. PREVENTIVE: If buying used X6 over 80k miles, budget for this repair and listen for clicking noise when shutting off ignition.</x:v>
+        <x:v>Inspect the trunk floor, differential mount area, and all rear subframe mounting points from above and below the car for spot-weld separation, torn sheet metal, and cracked seams; a dye penetrant test or removing trunk trim/seam sealer may be needed to reveal early damage. If cracking is present, the proper repair is to drop the rear axle carrier/subframe, weld and reinforce the damaged unibody mounting points and trunk floor with a reinforcement kit (commonly Randy Forbes-style dual-ear/differential mount reinforcement or equivalent), then reinstall with new subframe bushings, differential mount bushings, and perform a 4-wheel alignment. Minor early cracks may be repairable before major deformation, but advanced damage often requires fabrication and extensive welding by a chassis/body specialist; typical cost ranges from about $2,000-$3,500 for early reinforcement repairs and can exceed $4,000-$6,000 if the floor is torn or multiple mounting points are damaged.</x:v>
       </x:c>
       <x:c r="F72" s="9" t="n">
         <x:v>0</x:v>
@@ -16889,22 +18249,20 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="73" ht="514.7999877929688" hidden="0" customHeight="1">
+    <x:row r="73" ht="66" hidden="0" customHeight="1">
       <x:c r="A73" s="40" t="n">
         <x:v>72</x:v>
       </x:c>
       <x:c r="B73" s="9" t="str">
-        <x:v>bmw-x6m-front-thrust-arm-bushing-2015</x:v>
+        <x:v>bmw-z3-rear-subframe-cracking-1996</x:v>
       </x:c>
       <x:c r="C73" s="9" t="str">
-        <x:v>2015-2025 | BMW | X6 M</x:v>
+        <x:v>1996-2002 | BMW | Z3 | M52, M54</x:v>
       </x:c>
       <x:c r="D73" s="9" t="str">
-        <x:v>Front Thrust Arm Bushing (Tension Strut) Premature Wear</x:v>
-      </x:c>
-      <x:c r="E73" s="9" t="str">
-        <x:v>Replace both front thrust arms as complete assemblies (the bushings are not serviceable separately). Use genuine BMW M-spec parts or Lemforder equivalents. Perform a 4-wheel alignment immediately after replacement. Upgrade to Powerflex polyurethane thrust arm bushings for extended lifespan, especially on tracked cars.</x:v>
-      </x:c>
+        <x:v>Rear Subframe Mounting Point Cracks</x:v>
+      </x:c>
+      <x:c r="E73" s="9" t="str"/>
       <x:c r="F73" s="9" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -16912,21 +18270,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="74" ht="897.5999755859375" hidden="0" customHeight="1">
+    <x:row r="74" ht="475.20001220703125" hidden="0" customHeight="1">
       <x:c r="A74" s="40" t="n">
         <x:v>73</x:v>
       </x:c>
       <x:c r="B74" s="9" t="str">
-        <x:v>bmw-x6m-s63-rod-bearing-2010</x:v>
+        <x:v>bmw-z3-valve-cover-gasket-oil-leak</x:v>
       </x:c>
       <x:c r="C74" s="9" t="str">
-        <x:v>2010-2023 | BMW | X6 M | M50i, xDrive50i | S63</x:v>
+        <x:v>1997-2002 | BMW | Z3 | 2.3, 2.5i, 2.8, 3.0i | M52 2.8, M52TU 2.5/2.8, M54 2.5/3.0</x:v>
       </x:c>
       <x:c r="D74" s="9" t="str">
-        <x:v>S63 Rod Bearing Failure (X6 M)</x:v>
+        <x:v>Valve Cover Gasket Oil Leak (M52/M54 6-Cylinder)</x:v>
       </x:c>
       <x:c r="E74" s="9" t="str">
-        <x:v>PREVENTIVE: Replace rod bearings every 60,000-80,000 miles ($2,500-5,000 labor-intensive job). Use ACL Race 8B1578HX-STD ($150-250) or King CR8049SV ($120-200) upgraded bearings - these are stronger than OEM and provide better durability under high loads. Send oil samples for analysis (Blackstone Labs ~$30) every 5,000 miles to monitor bearing wear metals. If bearings have already failed: engine replacement required ($15,000-30,000). DO NOT buy used X6 M without documented bearing replacement history or fresh oil analysis.</x:v>
+        <x:v>Replace the valve cover gasket, the spark-plug-well/grommet seals, and the cover bolt seals. On M54 engines also clean oil from the plug wells and replace any oil-contaminated coil boots/coils. Use the correct torque sequence to avoid re-leaking. Inspect the cover for warping or cracks while it is off.</x:v>
       </x:c>
       <x:c r="F74" s="9" t="n">
         <x:v>0</x:v>
@@ -16935,21 +18293,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="75" ht="277.20001220703125" hidden="0" customHeight="1">
+    <x:row r="75" ht="1293.5999755859375" hidden="0" customHeight="1">
       <x:c r="A75" s="40" t="n">
         <x:v>74</x:v>
       </x:c>
       <x:c r="B75" s="9" t="str">
-        <x:v>bmw-x6m-vanos-solenoid-2015</x:v>
+        <x:v>bmw-z3-vanos-seals-1999</x:v>
       </x:c>
       <x:c r="C75" s="9" t="str">
-        <x:v>2015-2021 | BMW | X6 M | S63</x:v>
+        <x:v>1999-2002 | BMW | Z3 | M52, M54, S52</x:v>
       </x:c>
       <x:c r="D75" s="9" t="str">
-        <x:v>VANOS Solenoid Oil Sludge Buildup</x:v>
+        <x:v>VANOS Seal Failure (M52/M54/S52)</x:v>
       </x:c>
       <x:c r="E75" s="9" t="str">
-        <x:v>Remove and clean or replace the VANOS solenoids. Perform an engine oil flush. Strictly follow 7,500-mile oil change intervals with BMW LL-01 rated 0W-40 synthetic oil.</x:v>
+        <x:v>Confirm the fault by checking for cold-start VANOS rattle, rough idle, hesitation, and scanning for cam timing or mixture-related fault codes; on M52TU/M54/S52 engines, inspect VANOS operation and rule out vacuum leaks before disassembly. Repair typically involves removing the valve cover and VANOS unit, replacing the internal piston seals/O-rings with updated Viton/Teflon seals, renewing the valve cover gasket and VANOS oil line sealing washers, and then re-timing the cams to BMW specifications if required. If the unit still rattles after resealing, the VANOS bearing/anti-rattle components or the complete VANOS assembly may need replacement. Typical cost is about $60-$150 in seals/gaskets for DIY repair, $300-$700 for an independent shop reseal, or $800-$1,500+ if a rebuilt/replacement VANOS unit is installed.</x:v>
       </x:c>
       <x:c r="F75" s="9" t="n">
         <x:v>0</x:v>
@@ -16958,21 +18316,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="76" ht="699.5999755859375" hidden="0" customHeight="1">
+    <x:row r="76" ht="501.6000061035156" hidden="0" customHeight="1">
       <x:c r="A76" s="40" t="n">
         <x:v>75</x:v>
       </x:c>
       <x:c r="B76" s="9" t="str">
-        <x:v>bmw-x7-48v-battery-2020</x:v>
+        <x:v>bmw-z4-b58-coolant-tank-2019</x:v>
       </x:c>
       <x:c r="C76" s="9" t="str">
-        <x:v>2020-2023 | BMW | X7</x:v>
+        <x:v>2019-2026 | BMW | Z4 | B58</x:v>
       </x:c>
       <x:c r="D76" s="9" t="str">
-        <x:v>48V Mild Hybrid Battery Issues</x:v>
+        <x:v>B58 Coolant Expansion Tank Cracking</x:v>
       </x:c>
       <x:c r="E76" s="9" t="str">
-        <x:v>Replace the 48V mild hybrid battery ($1,000-2,000 at dealer). Requires dealer-level diagnostic tools and coding after installation - this is NOT a DIY repair. The 48V battery is separate from the main 12V battery. No aftermarket alternatives currently available. Check if vehicle is still under BMW warranty or extended warranty coverage. Some owners choose to live with the failed auto start-stop rather than pay for replacement.</x:v>
+        <x:v>Replace the coolant expansion tank with an updated BMW part or aftermarket aluminum tank. Inspect the tank and cap regularly for signs of cracking, discoloration, or seepage. When replacing, also replace the cap and check all coolant hoses for brittleness. Flush and refill with BMW-approved coolant.</x:v>
       </x:c>
       <x:c r="F76" s="9" t="n">
         <x:v>0</x:v>
@@ -16981,21 +18339,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="77" ht="726" hidden="0" customHeight="1">
+    <x:row r="77" ht="1306.800048828125" hidden="0" customHeight="1">
       <x:c r="A77" s="40" t="n">
         <x:v>76</x:v>
       </x:c>
       <x:c r="B77" s="9" t="str">
-        <x:v>bmw-x7-air-suspension-2019</x:v>
+        <x:v>bmw-z4-e85-convertible-top-hydraulic-2003</x:v>
       </x:c>
       <x:c r="C77" s="9" t="str">
-        <x:v>2019-2023 | BMW | X7</x:v>
+        <x:v>2003-2008 | BMW | Z4</x:v>
       </x:c>
       <x:c r="D77" s="9" t="str">
-        <x:v>Air Suspension Compressor &amp; Strut Failure (Standard Equipment)</x:v>
+        <x:v>Convertible Top Hydraulic Pump Motor Failure - E85 Z4</x:v>
       </x:c>
       <x:c r="E77" s="9" t="str">
-        <x:v>Replace failed air struts and/or compressor. Front strut left 37106869035 ($1,500-2,000), right 37106869036 ($1,500-2,000), rear 37106869039 ($1,000-1,500). Compressor 37206861882 ($800-1,200). RebuildMasterTech rebuilt struts ($600-900 each) are a more affordable alternative. Total repair can reach $2,180-5,000+ depending on which components have failed. Replace both struts on same axle simultaneously. Inspect at 50,000 miles for early signs of leaking.</x:v>
+        <x:v>Replace hydraulic pump motor assembly (BMW 54347193448 / supersedes 54347119633). OEM Genuine BMW pump: $800-$1,200. Aftermarket alternatives available on Amazon for $150-$300 but quality varies significantly. Dealer labor is $1,500-$2,500+ as BMW procedure requires full top removal. ZRoadster.org members have documented a motor relocation to the boot/trunk area which allows much easier future access. Hydraulic fluid: use Aral Vitamol ZHM or BMW 54340394395 hydraulic oil. PREVENTION: Clean drain holes annually, ensure rubber bungs are properly seated, and check for water intrusion in pump area at every service. Some owners have had success with pump motor rebuilds from roofmotors.co.uk ($300-$500) but quality of rebuilds varies.</x:v>
       </x:c>
       <x:c r="F77" s="9" t="n">
         <x:v>0</x:v>
@@ -17004,21 +18362,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="78" ht="435.6000061035156" hidden="0" customHeight="1">
+    <x:row r="78" ht="1135.199951171875" hidden="0" customHeight="1">
       <x:c r="A78" s="40" t="n">
         <x:v>77</x:v>
       </x:c>
       <x:c r="B78" s="9" t="str">
-        <x:v>bmw-x7-air-suspension-compressor-2019</x:v>
+        <x:v>bmw-z4-e85-window-regulator-2003</x:v>
       </x:c>
       <x:c r="C78" s="9" t="str">
-        <x:v>2019-2026 | BMW | X7</x:v>
+        <x:v>2003-2008 | BMW | Z4</x:v>
       </x:c>
       <x:c r="D78" s="9" t="str">
-        <x:v>Air Suspension Compressor Failure</x:v>
+        <x:v>Power Window Regulator Failure - E85 Z4</x:v>
       </x:c>
       <x:c r="E78" s="9" t="str">
-        <x:v>Replace the air suspension compressor. Inspect all four air springs for leaks using soapy water solution. Replace any leaking air springs to prevent repeated compressor failure. Check the valve block for proper operation. The compressor is located under the rear of the vehicle.</x:v>
+        <x:v>Option 1 (Budget): Window regulator repair kit - replacement cables and rollers for ~$18-$25 from eBay/Amazon (BWR974 for left/driver side). Requires removing door panel and threading new cables through existing regulator frame. DIY-friendly with Z4-forum.com guides. Option 2 (Recommended): Full window regulator replacement. Driver side: BMW 51337198909 ($180-$280 OEM, $80-$150 aftermarket). Passenger side: BMW 51337198910 ($180-$280 OEM, $80-$150 aftermarket). Labor: $200-$400 at independent shop, $500-$700+ at dealer. DIY: 2-3 hours with door panel removal guide from Pelican Parts. ZRoadster.org recommends full replacement over repair kit for long-term reliability.</x:v>
       </x:c>
       <x:c r="F78" s="9" t="n">
         <x:v>0</x:v>
@@ -17027,21 +18385,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="79" ht="871.2000122070312" hidden="0" customHeight="1">
+    <x:row r="79" ht="514.7999877929688" hidden="0" customHeight="1">
       <x:c r="A79" s="40" t="n">
         <x:v>78</x:v>
       </x:c>
       <x:c r="B79" s="9" t="str">
-        <x:v>bmw-x7-b58-coolant-2019</x:v>
+        <x:v>bmw-z4-electric-steering-rack-2003</x:v>
       </x:c>
       <x:c r="C79" s="9" t="str">
-        <x:v>2019-2023 | BMW | X7 | xDrive40i | B58</x:v>
+        <x:v>2012-2012 | BMW | Z4</x:v>
       </x:c>
       <x:c r="D79" s="9" t="str">
-        <x:v>B58 Coolant System Failures (xDrive40i)</x:v>
+        <x:v>2012 Z4 Electric Power-Steering Recall 12V-302</x:v>
       </x:c>
       <x:c r="E79" s="9" t="str">
-        <x:v>Replace failed coolant system components. Water pump 11518482250 ($300-400). Thermostat 11537644811 ($150-250). Replace expansion tank and all plastic coolant connections when performing repair to prevent cascading failures. For 2023+ models, check VIN for recall 24V-608 coverage for coolant pump connector. Total repair $500-2,500 depending on extent of damage. PREVENTIVE: Replace thermostat and water pump at 60,000-70,000 miles before failure. Inspect coolant hoses and connections at every oil change after 50k miles.</x:v>
+        <x:v>Check the VIN for an open 12V-302 campaign. If open, an authorized BMW dealer replaces the steering-assistance module free of charge. If the steering warning and audible alert occur, maintain control, reduce speed, stop safely and arrange dealer or roadside assistance; do not replace a steering rack from this card.</x:v>
       </x:c>
       <x:c r="F79" s="9" t="n">
         <x:v>0</x:v>
@@ -17050,21 +18408,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="80" ht="435.6000061035156" hidden="0" customHeight="1">
+    <x:row r="80" ht="633.5999755859375" hidden="0" customHeight="1">
       <x:c r="A80" s="40" t="n">
         <x:v>79</x:v>
       </x:c>
       <x:c r="B80" s="9" t="str">
-        <x:v>bmw-x7-b58-coolant-expansion-tank-2019</x:v>
+        <x:v>bmw-z4-electric-water-pump-2006</x:v>
       </x:c>
       <x:c r="C80" s="9" t="str">
-        <x:v>2019-2026 | BMW | X7 | B58</x:v>
+        <x:v>2012-2016 | BMW | Z4 | N20</x:v>
       </x:c>
       <x:c r="D80" s="9" t="str">
-        <x:v>B58 Coolant Expansion Tank Crack</x:v>
+        <x:v>2012-2016 Z4 sDrive28i Water-Pump Connector Recall 24V-608</x:v>
       </x:c>
       <x:c r="E80" s="9" t="str">
-        <x:v>Replace the coolant expansion tank with an updated BMW part that uses improved plastic composition. Also replace the cap and inspect all coolant hoses. Flush and refill the cooling system with BMW-approved coolant. Check for coolant contamination from the old tank.</x:v>
+        <x:v>Check the VIN for an open 24V-608 campaign. If open, an authorized BMW dealer inspects the water pump and connector, replaces them if necessary, and installs the protective shield free of charge. If smoke appears from the engine compartment, stop safely, switch off the vehicle, have occupants exit, move away from traffic and call emergency or roadside assistance; do not order a pump from this card.</x:v>
       </x:c>
       <x:c r="F80" s="9" t="n">
         <x:v>0</x:v>
@@ -17073,44 +18431,44 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="81" ht="646.7999877929688" hidden="0" customHeight="1">
+    <x:row r="81" ht="1359.5999755859375" hidden="0" customHeight="1">
       <x:c r="A81" s="40" t="n">
         <x:v>80</x:v>
       </x:c>
       <x:c r="B81" s="9" t="str">
-        <x:v>bmw-x7-ibs-brake-recall-2023</x:v>
+        <x:v>bmw-z4-g29-b58-water-pump-2019</x:v>
       </x:c>
       <x:c r="C81" s="9" t="str">
-        <x:v>2023-2025 | BMW | X7</x:v>
+        <x:v>2019-2025 | BMW | Z4 | M40i, sDrive35i, sDrive35is | B48, B58</x:v>
       </x:c>
       <x:c r="D81" s="9" t="str">
-        <x:v>2023-2025 X7 Integrated Brake System Recall 26V-422</x:v>
+        <x:v>B48/B58 Electric Water Pump &amp; Thermostat Failure - G29 Z4</x:v>
       </x:c>
       <x:c r="E81" s="9" t="str">
-        <x:v>Check the VIN at NHTSA and with an authorized BMW dealer when campaign 26V-422 VINs become searchable, and arrange the free dealer inspection and module replacement if required. If a brake warning appears or pedal effort increases, avoid abrupt braking, allow extra stopping distance, stop safely and contact BMW roadside assistance; do not order brake electronics from this card.</x:v>
+        <x:v>Preventative replacement recommended at 60,000 miles. Always replace water pump and thermostat together - they share labor overlap and frequently fail concurrently. B48 sDrive30i: Water pump BMW 11518632586 ($300-$450), Thermostat BMW 11538685978 ($100-$150). B58 M40i: Water pump BMW 11518650986 ($350-$500), Thermostat BMW 11538685978 ($100-$150). Mishimoto offers performance water pump alternatives for B58 with improved impeller design. Replace 3 O-rings between thermostat and pump housing, plus 2 O-rings on coolant tube to head. Must replace water pump mounting bolts (torque-to-yield). Labor: 3-4 hours. FCP Euro lifetime warranty kits available. Also inspect plastic cylinder head coolant outlet adapter - known to shear off causing massive coolant leak.</x:v>
       </x:c>
       <x:c r="F81" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G81" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="82" ht="897.5999755859375" hidden="0" customHeight="1">
+    <x:row r="82" ht="1122" hidden="0" customHeight="1">
       <x:c r="A82" s="40" t="n">
         <x:v>81</x:v>
       </x:c>
       <x:c r="B82" s="9" t="str">
-        <x:v>bmw-x7-n63-oil-consumption-2019</x:v>
+        <x:v>bmw-z4-n54-hpfp-2009</x:v>
       </x:c>
       <x:c r="C82" s="9" t="str">
-        <x:v>2019-2023 | BMW | X7 | M50i, M60i, xDrive50i | N63TU3</x:v>
+        <x:v>2009-2011 | BMW | Z4 | M40i, sDrive35i, sDrive35is | N54</x:v>
       </x:c>
       <x:c r="D82" s="9" t="str">
-        <x:v>N63TU3 Oil Consumption &amp; Valve Stem Seal Degradation (xDrive50i/M50i/M60i)</x:v>
+        <x:v>N54 High Pressure Fuel Pump (HPFP) Failure - E89 Z4 sDrive35i/35is</x:v>
       </x:c>
       <x:c r="E82" s="9" t="str">
-        <x:v>Replace valve stem seals - extremely labor-intensive job requiring cylinder head work ($4,900-12,000 total). Elring seals 11340039494 for OEM spec. 5150 AutoSport Viton upgraded seals ($150-200) recommended for better heat resistance. AGA Tools kit includes specialized tools required. Reference TSB MC-10149960-9999 when visiting dealer. Check eligibility for class action settlement coverage. Some owners monitor oil levels and top off rather than repair. Use quality synthetic 0W-40 BMW LL-01 spec oil and check level every 500-1,000 miles.</x:v>
+        <x:v>Replace HPFP with latest revision Genuine BMW unit. The pump went through multiple revisions - ONLY install the latest version. Part number evolution: Original -&gt; 13517592881 (Index 10, TSB fix) -&gt; 13517616170 (latest revision, most reliable). Genuine BMW 13517616170 is the definitive fix ($350-$550 for pump). Replacement is straightforward DIY (1-2 hours) with basic tools. Also available as complete kit from FCP Euro with lifetime warranty. BMW extended warranty coverage to 10 years/120,000 miles under customer care package for original owners - check VIN eligibility. Replace low-pressure fuel sensor at same time (13537537319) as it may have been damaged by pressure fluctuations ($35-$55).</x:v>
       </x:c>
       <x:c r="F82" s="9" t="n">
         <x:v>0</x:v>
@@ -17119,21 +18477,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="83" ht="396" hidden="0" customHeight="1">
+    <x:row r="83" ht="580.7999877929688" hidden="0" customHeight="1">
       <x:c r="A83" s="40" t="n">
         <x:v>82</x:v>
       </x:c>
       <x:c r="B83" s="9" t="str">
-        <x:v>bmw-x7-panoramic-roof-rattle-2019</x:v>
+        <x:v>bmw-z4-n54-wastegate-rattle-2009</x:v>
       </x:c>
       <x:c r="C83" s="9" t="str">
-        <x:v>2019-2026 | BMW | X7</x:v>
+        <x:v>2009-2010 | BMW | Z4 | N54</x:v>
       </x:c>
       <x:c r="D83" s="9" t="str">
-        <x:v>Panoramic Sunroof Rattle and Creak</x:v>
+        <x:v>2009-2010 Z4 sDrive35i N54 Wastegate Diagnosis</x:v>
       </x:c>
       <x:c r="E83" s="9" t="str">
-        <x:v>Apply BMW-approved felt tape or lubricant to sunroof guide rails. Replace worn guide rail bushings. In severe cases, the sunroof cassette or seal may need replacement under warranty. BMW has issued updated guide rail components for early production vehicles.</x:v>
+        <x:v>Confirm the VIN, engine, production date, DME faults, boost-control data and noise source using current BMW diagnostic information. Check VIN-specific coverage history with BMW, recognizing that the bulletin's time/mileage window may have expired. Do not replace a turbocharger, actuator or wastegate from this card without the required diagnosis.</x:v>
       </x:c>
       <x:c r="F83" s="9" t="n">
         <x:v>0</x:v>
@@ -17142,21 +18500,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="84" ht="778.7999877929688" hidden="0" customHeight="1">
+    <x:row r="84" ht="501.6000061035156" hidden="0" customHeight="1">
       <x:c r="A84" s="40" t="n">
         <x:v>83</x:v>
       </x:c>
       <x:c r="B84" s="9" t="str">
-        <x:v>bmw-x7-sunroof-leak-2019</x:v>
+        <x:v>bmw-z4-soft-top-hydraulic-2003</x:v>
       </x:c>
       <x:c r="C84" s="9" t="str">
-        <x:v>2019-2023 | BMW | X7</x:v>
+        <x:v>2009-2016 | BMW | Z4</x:v>
       </x:c>
       <x:c r="D84" s="9" t="str">
-        <x:v>Panoramic Sunroof Water Leak</x:v>
+        <x:v>Retractable Hard Top Hydraulic Mechanism Failure</x:v>
       </x:c>
       <x:c r="E84" s="9" t="str">
-        <x:v>Clear clogged sunroof drain tubes ($100-300 at shop). Reference TSB SIB 54 11 19 when visiting dealer. For persistent leaks, drain tube connections or sunroof seal may need replacement ($500-1,500). If water has damaged interior electronics, repair costs can reach $3,000. PREVENTIVE: Clear sunroof drains annually, especially in areas with heavy tree debris. Run compressed air or flexible drain snake through drain tubes during oil changes. Keep sunroof track clean of debris.</x:v>
+        <x:v>Diagnose the leak location and replace the failed component. Common failure points are the main hydraulic cylinders (left and right), the hydraulic pump motor, and the flexible hoses. The hydraulic fluid should be flushed and replaced with BMW-approved CHF 11S fluid. A full system bleed is required after any repair.</x:v>
       </x:c>
       <x:c r="F84" s="9" t="n">
         <x:v>0</x:v>
@@ -17165,21 +18523,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="85" ht="739.2000122070312" hidden="0" customHeight="1">
+    <x:row r="85" ht="1188" hidden="0" customHeight="1">
       <x:c r="A85" s="40" t="n">
         <x:v>84</x:v>
       </x:c>
       <x:c r="B85" s="9" t="str">
-        <x:v>bmw-x7-tire-wear-2019</x:v>
+        <x:v>bmw-z4-vanos-solenoid-2003</x:v>
       </x:c>
       <x:c r="C85" s="9" t="str">
-        <x:v>2019-2023 | BMW | X7</x:v>
+        <x:v>2003-2016 | BMW | Z4 | 2.5i, 3.0i, 3.0si, M40i, sDrive28i, sDrive30i, sDrive35i, sDrive35is | M54, N52, N54, N20</x:v>
       </x:c>
       <x:c r="D85" s="9" t="str">
-        <x:v>Premature Tire Wear (Especially 21"/22" Wheels)</x:v>
+        <x:v>VANOS Solenoid &amp; System Failure - E85/E89 Z4 (All Engines)</x:v>
       </x:c>
       <x:c r="E85" s="9" t="str">
-        <x:v>Have alignment adjusted to reduce aggressive camber settings ($200-400). Switch to quality tires designed for heavy SUVs: Michelin Pilot Sport 4S or Continental PremiumContact 6 are recommended. If possible, avoid 22" wheels and opt for 21" or smaller for better tire longevity and ride comfort. Alignment adjustment can extend tire life from 15,000 to 30,000+ miles. Total cost $200-2,000 depending on tire replacement needs. Check alignment every 10,000 miles.</x:v>
+        <x:v>Replace VANOS solenoids - inexpensive and straightforward repair. M54 (E85 2003-2005): 2 solenoids required, BMW 11361707323 ($35-$65 each). N52 (E85 2006-2008 / E89 2009-2011 28i): 2 solenoids, BMW 11367585425 ($40-$70 each). N54 (E89 35i/35is): 2 solenoids, BMW 11367585425 ($40-$70 each). N20 (E89 sDrive28i 2012-2016): 2 solenoids, BMW 11367585425 ($40-$70 each). Labor: under 1 hour for experienced mechanic, 2-3 hours DIY. Replace all solenoids at once even if only one has failed - the others are same age and will fail soon. Also replace VANOS solenoid O-rings and sealing plates during service. Clean VANOS system with Beisan Systems VANOS cleaning procedure for best results.</x:v>
       </x:c>
       <x:c r="F85" s="9" t="n">
         <x:v>0</x:v>
@@ -17188,597 +18546,26 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="86" ht="501.6000061035156" hidden="0" customHeight="1">
-      <x:c r="A86" s="40" t="n">
+    <x:row r="86" ht="554.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A86" s="42" t="n">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="B86" s="9" t="str">
-        <x:v>bmw-xm-airbag-passenger-knee-recall-2023</x:v>
-      </x:c>
-      <x:c r="C86" s="9" t="str">
-        <x:v>2023-2023 | BMW | XM</x:v>
-      </x:c>
-      <x:c r="D86" s="9" t="str">
-        <x:v>2023 XM Front-Passenger Knee-Airbag Recall 23V-622</x:v>
-      </x:c>
-      <x:c r="E86" s="9" t="str">
-        <x:v>Check the VIN for an open 23V-622 campaign. If open, an authorized BMW dealer replaces the front-passenger knee airbag free of charge. Do not attempt airbag diagnosis or order a clock spring or airbag module from this card; supplemental-restraint work requires trained personnel and VIN-selected parts.</x:v>
-      </x:c>
-      <x:c r="F86" s="9" t="n">
+      <x:c r="B86" s="43" t="str">
+        <x:v>bmw-z8-soft-top-mechanism-2000</x:v>
+      </x:c>
+      <x:c r="C86" s="43" t="str">
+        <x:v>2000-2003 | BMW | Z8</x:v>
+      </x:c>
+      <x:c r="D86" s="43" t="str">
+        <x:v>Power Soft Top Hydraulic System and Cable Failure</x:v>
+      </x:c>
+      <x:c r="E86" s="43" t="str">
+        <x:v>Rebuild the hydraulic cylinders with new seals rather than replacing ($200 vs $2,000+). Inspect and replace frayed cables. Adjust or replace the microswitch sensors at the windshield header latch. Lubricate the top mechanism pivot points with silicone grease annually. Store the car with the top up to reduce stress on the hydraulic system.</x:v>
+      </x:c>
+      <x:c r="F86" s="43" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G86" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="87" ht="567.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A87" s="40" t="n">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="B87" s="9" t="str">
-        <x:v>bmw-xm-hybrid-drivetrain-hesitation-2023</x:v>
-      </x:c>
-      <x:c r="C87" s="9" t="str">
-        <x:v>2023-2024 | BMW | XM | S68 4.4L Twin-Turbo V8 Hybrid, S68</x:v>
-      </x:c>
-      <x:c r="D87" s="9" t="str">
-        <x:v>Hybrid Drivetrain Hesitation and Power Delivery Lag</x:v>
-      </x:c>
-      <x:c r="E87" s="9" t="str">
-        <x:v>Visit the dealer for the latest transmission and hybrid system software calibration updates. Select Sport or Sport Plus mode for more consistent power delivery. The latest software revisions significantly improve the electric-to-V8 handoff smoothness. If hesitation persists after updates, the dealer can reset the transmission adaptation values to relearn driving patterns.</x:v>
-      </x:c>
-      <x:c r="F87" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G87" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="88" ht="646.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A88" s="40" t="n">
-        <x:v>87</x:v>
-      </x:c>
-      <x:c r="B88" s="9" t="str">
-        <x:v>bmw-xm-integrated-brake-system-recall-2023</x:v>
-      </x:c>
-      <x:c r="C88" s="9" t="str">
-        <x:v>2023-2024 | BMW | XM</x:v>
-      </x:c>
-      <x:c r="D88" s="9" t="str">
-        <x:v>2023-2024 XM Integrated Brake System Recall 26V-422</x:v>
-      </x:c>
-      <x:c r="E88" s="9" t="str">
-        <x:v>Check the VIN at NHTSA and with an authorized BMW dealer when campaign 26V-422 VINs become searchable, and arrange the free dealer inspection and module replacement if required. If a brake warning appears or pedal effort increases, avoid abrupt braking, allow extra stopping distance, stop safely and contact BMW roadside assistance; wheel-speed sensors are not the recall remedy.</x:v>
-      </x:c>
-      <x:c r="F88" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G88" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="89" ht="646.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A89" s="40" t="n">
-        <x:v>88</x:v>
-      </x:c>
-      <x:c r="B89" s="9" t="str">
-        <x:v>bmw-xm-suspension-ride-quality-2023</x:v>
-      </x:c>
-      <x:c r="C89" s="9" t="str">
-        <x:v>2023-2024 | BMW | XM | S68 4.4L Twin-Turbo V8 Hybrid</x:v>
-      </x:c>
-      <x:c r="D89" s="9" t="str">
-        <x:v>Harsh Ride Quality and Suspension Stiffness</x:v>
-      </x:c>
-      <x:c r="E89" s="9" t="str">
-        <x:v>Check tire pressures regularly - overinflated tires significantly worsen the harsh ride. Some owners report improved comfort by switching to a tire with a taller sidewall profile (if available for the XM's wheel size). Use Comfort mode for daily driving. Unfortunately, no aftermarket spring or damper solution currently exists to significantly improve the ride without compromising the handling needed for the XM's weight.</x:v>
-      </x:c>
-      <x:c r="F89" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G89" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="90" ht="528" hidden="0" customHeight="1">
-      <x:c r="A90" s="40" t="n">
-        <x:v>89</x:v>
-      </x:c>
-      <x:c r="B90" s="9" t="str">
-        <x:v>bmw-z3-convertible-top-rear-window-cracking-clouding-bead-separatio</x:v>
-      </x:c>
-      <x:c r="C90" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D90" s="9" t="str">
-        <x:v>Convertible Top Rear Window Cracking, Clouding, and Bead Separation</x:v>
-      </x:c>
-      <x:c r="E90" s="9" t="str">
-        <x:v>Replace the rear window panel only — BMW used a zipper system so the clouded/cracked window unzips and a new window zips/tapes in without disturbing the fabric top. Re-gluing separated bead trim rarely holds, so window replacement is the durable fix. Job is a DIY-feasible 1-1.5 hours; replace the whole top only if the fabric is also degraded.</x:v>
-      </x:c>
-      <x:c r="F90" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G90" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="91" ht="52.79999923706055" hidden="0" customHeight="1">
-      <x:c r="A91" s="40" t="n">
-        <x:v>90</x:v>
-      </x:c>
-      <x:c r="B91" s="9" t="str">
-        <x:v>bmw-z3-cooling-system-failure-1996</x:v>
-      </x:c>
-      <x:c r="C91" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D91" s="9" t="str">
-        <x:v>Cooling System Component Failures</x:v>
-      </x:c>
-      <x:c r="E91" s="9" t="str"/>
-      <x:c r="F91" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G91" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="92" ht="448.79998779296875" hidden="0" customHeight="1">
-      <x:c r="A92" s="40" t="n">
-        <x:v>91</x:v>
-      </x:c>
-      <x:c r="B92" s="9" t="str">
-        <x:v>bmw-z3-cracked-exhaust-manifold-1-9l-4-cylinder</x:v>
-      </x:c>
-      <x:c r="C92" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3 | 1.9, 1.9i, Z3 1.9 | 1.9L M44 4-cylinder, 1.9L M43TU 4-cylinder</x:v>
-      </x:c>
-      <x:c r="D92" s="9" t="str">
-        <x:v>Cracked Exhaust Manifold on 1.9L 4-Cylinder (M44/M43)</x:v>
-      </x:c>
-      <x:c r="E92" s="9" t="str">
-        <x:v>Inspect the manifold for hairline cracks (a cold-engine listen or smoke test confirms the leak). Replace the cracked manifold with a used OE unit or an aftermarket stainless tubular header, and renew the manifold gasket and hardware. Allow roughly 3-4 hours labor.</x:v>
-      </x:c>
-      <x:c r="F92" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G92" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="93" ht="686.4000244140625" hidden="0" customHeight="1">
-      <x:c r="A93" s="40" t="n">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="B93" s="9" t="str">
-        <x:v>bmw-z3-differential-mount-ear-trunk-floor-pan-tearing</x:v>
-      </x:c>
-      <x:c r="C93" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D93" s="9" t="str">
-        <x:v>Differential Mount Ear and Trunk Floor Pan Tearing</x:v>
-      </x:c>
-      <x:c r="E93" s="9" t="str">
-        <x:v>Inspect the trunk floor around the differential mount and rear subframe pickup points for cracks, torn metal, and broken spot welds. Repair requires welding and a reinforcement/re-fabrication plate kit to tie the diff mount/subframe back into the floor. Switching the diff carrier bushings to polyurethane reduces carrier movement and the stress that causes the tearing. Catching it early greatly limits the repair scope.</x:v>
-      </x:c>
-      <x:c r="F93" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G93" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="94" ht="514.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A94" s="40" t="n">
-        <x:v>93</x:v>
-      </x:c>
-      <x:c r="B94" s="9" t="str">
-        <x:v>bmw-z3-door-window-regulator-clip-mounting-tab-failure</x:v>
-      </x:c>
-      <x:c r="C94" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D94" s="9" t="str">
-        <x:v>Door Window Regulator Clip / Mounting Tab Failure</x:v>
-      </x:c>
-      <x:c r="E94" s="9" t="str">
-        <x:v>Replace the broken plastic regulator clips, or replace the regulator assembly if the cable or mechanism is also worn. If the welded mounting tab/anchor has torn from the door frame, it must be re-welded or reinforced before fitting a new regulator. Lubricate the window channels to reduce drag on the new parts.</x:v>
-      </x:c>
-      <x:c r="F94" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G94" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="95" ht="686.4000244140625" hidden="0" customHeight="1">
-      <x:c r="A95" s="40" t="n">
-        <x:v>94</x:v>
-      </x:c>
-      <x:c r="B95" s="9" t="str">
-        <x:v>bmw-z3-fuel-level-sender-failure-causing-erratic-dead-fuel-gauge</x:v>
-      </x:c>
-      <x:c r="C95" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D95" s="9" t="str">
-        <x:v>Fuel Level Sender Failure Causing Erratic or Dead Fuel Gauge</x:v>
-      </x:c>
-      <x:c r="E95" s="9" t="str">
-        <x:v>Remove the access panel behind the seats and inspect the sender. A dirty or lightly worn ceramic/resistor plate can sometimes be cleaned, but a cracked plate or worn brushes requires replacing the sender unit (or the complete fuel-pump/sender carrier assembly). Also check the tank vent valve, as tank vacuum can deform the float arm. Confirm wiring/ground integrity before condemning the sender.</x:v>
-      </x:c>
-      <x:c r="F95" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G95" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="96" ht="488.3999938964844" hidden="0" customHeight="1">
-      <x:c r="A96" s="40" t="n">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="B96" s="9" t="str">
-        <x:v>bmw-z3-hvac-blower-final-stage-resistor-failure</x:v>
-      </x:c>
-      <x:c r="C96" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D96" s="9" t="str">
-        <x:v>HVAC Blower Final Stage Resistor Failure (Fan Only Works on Max)</x:v>
-      </x:c>
-      <x:c r="E96" s="9" t="str">
-        <x:v>Replace the blower final stage resistor (A/C cars: part under the scuttle/cowl; non-A/C cars: behind the passenger footwell panel). If a new resistor does not restore all speeds, test the blower motor itself, which may also be worn. Inspect for corrosion/water intrusion at the cowl on A/C cars.</x:v>
-      </x:c>
-      <x:c r="F96" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G96" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="97" ht="1584" hidden="0" customHeight="1">
-      <x:c r="A97" s="40" t="n">
-        <x:v>96</x:v>
-      </x:c>
-      <x:c r="B97" s="9" t="str">
-        <x:v>bmw-z3-rear-subframe-crack-1996</x:v>
-      </x:c>
-      <x:c r="C97" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D97" s="9" t="str">
-        <x:v>Rear Subframe Mounting Point Cracking</x:v>
-      </x:c>
-      <x:c r="E97" s="9" t="str">
-        <x:v>Inspect the trunk floor, differential mount area, and all rear subframe mounting points from above and below the car for spot-weld separation, torn sheet metal, and cracked seams; a dye penetrant test or removing trunk trim/seam sealer may be needed to reveal early damage. If cracking is present, the proper repair is to drop the rear axle carrier/subframe, weld and reinforce the damaged unibody mounting points and trunk floor with a reinforcement kit (commonly Randy Forbes-style dual-ear/differential mount reinforcement or equivalent), then reinstall with new subframe bushings, differential mount bushings, and perform a 4-wheel alignment. Minor early cracks may be repairable before major deformation, but advanced damage often requires fabrication and extensive welding by a chassis/body specialist; typical cost ranges from about $2,000-$3,500 for early reinforcement repairs and can exceed $4,000-$6,000 if the floor is torn or multiple mounting points are damaged.</x:v>
-      </x:c>
-      <x:c r="F97" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G97" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="98" ht="66" hidden="0" customHeight="1">
-      <x:c r="A98" s="40" t="n">
-        <x:v>97</x:v>
-      </x:c>
-      <x:c r="B98" s="9" t="str">
-        <x:v>bmw-z3-rear-subframe-cracking-1996</x:v>
-      </x:c>
-      <x:c r="C98" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3 | M52, M54</x:v>
-      </x:c>
-      <x:c r="D98" s="9" t="str">
-        <x:v>Rear Subframe Mounting Point Cracks</x:v>
-      </x:c>
-      <x:c r="E98" s="9" t="str"/>
-      <x:c r="F98" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G98" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="99" ht="475.20001220703125" hidden="0" customHeight="1">
-      <x:c r="A99" s="40" t="n">
-        <x:v>98</x:v>
-      </x:c>
-      <x:c r="B99" s="9" t="str">
-        <x:v>bmw-z3-valve-cover-gasket-oil-leak</x:v>
-      </x:c>
-      <x:c r="C99" s="9" t="str">
-        <x:v>1997-2002 | BMW | Z3 | 2.3, 2.5i, 2.8, 3.0i | M52 2.8, M52TU 2.5/2.8, M54 2.5/3.0</x:v>
-      </x:c>
-      <x:c r="D99" s="9" t="str">
-        <x:v>Valve Cover Gasket Oil Leak (M52/M54 6-Cylinder)</x:v>
-      </x:c>
-      <x:c r="E99" s="9" t="str">
-        <x:v>Replace the valve cover gasket, the spark-plug-well/grommet seals, and the cover bolt seals. On M54 engines also clean oil from the plug wells and replace any oil-contaminated coil boots/coils. Use the correct torque sequence to avoid re-leaking. Inspect the cover for warping or cracks while it is off.</x:v>
-      </x:c>
-      <x:c r="F99" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G99" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="100" ht="1293.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A100" s="40" t="n">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="B100" s="9" t="str">
-        <x:v>bmw-z3-vanos-seals-1999</x:v>
-      </x:c>
-      <x:c r="C100" s="9" t="str">
-        <x:v>1999-2002 | BMW | Z3 | M52, M54, S52</x:v>
-      </x:c>
-      <x:c r="D100" s="9" t="str">
-        <x:v>VANOS Seal Failure (M52/M54/S52)</x:v>
-      </x:c>
-      <x:c r="E100" s="9" t="str">
-        <x:v>Confirm the fault by checking for cold-start VANOS rattle, rough idle, hesitation, and scanning for cam timing or mixture-related fault codes; on M52TU/M54/S52 engines, inspect VANOS operation and rule out vacuum leaks before disassembly. Repair typically involves removing the valve cover and VANOS unit, replacing the internal piston seals/O-rings with updated Viton/Teflon seals, renewing the valve cover gasket and VANOS oil line sealing washers, and then re-timing the cams to BMW specifications if required. If the unit still rattles after resealing, the VANOS bearing/anti-rattle components or the complete VANOS assembly may need replacement. Typical cost is about $60-$150 in seals/gaskets for DIY repair, $300-$700 for an independent shop reseal, or $800-$1,500+ if a rebuilt/replacement VANOS unit is installed.</x:v>
-      </x:c>
-      <x:c r="F100" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G100" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="101" ht="501.6000061035156" hidden="0" customHeight="1">
-      <x:c r="A101" s="40" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="B101" s="9" t="str">
-        <x:v>bmw-z4-b58-coolant-tank-2019</x:v>
-      </x:c>
-      <x:c r="C101" s="9" t="str">
-        <x:v>2019-2026 | BMW | Z4 | B58</x:v>
-      </x:c>
-      <x:c r="D101" s="9" t="str">
-        <x:v>B58 Coolant Expansion Tank Cracking</x:v>
-      </x:c>
-      <x:c r="E101" s="9" t="str">
-        <x:v>Replace the coolant expansion tank with an updated BMW part or aftermarket aluminum tank. Inspect the tank and cap regularly for signs of cracking, discoloration, or seepage. When replacing, also replace the cap and check all coolant hoses for brittleness. Flush and refill with BMW-approved coolant.</x:v>
-      </x:c>
-      <x:c r="F101" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G101" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="102" ht="1306.800048828125" hidden="0" customHeight="1">
-      <x:c r="A102" s="40" t="n">
-        <x:v>101</x:v>
-      </x:c>
-      <x:c r="B102" s="9" t="str">
-        <x:v>bmw-z4-e85-convertible-top-hydraulic-2003</x:v>
-      </x:c>
-      <x:c r="C102" s="9" t="str">
-        <x:v>2003-2008 | BMW | Z4</x:v>
-      </x:c>
-      <x:c r="D102" s="9" t="str">
-        <x:v>Convertible Top Hydraulic Pump Motor Failure - E85 Z4</x:v>
-      </x:c>
-      <x:c r="E102" s="9" t="str">
-        <x:v>Replace hydraulic pump motor assembly (BMW 54347193448 / supersedes 54347119633). OEM Genuine BMW pump: $800-$1,200. Aftermarket alternatives available on Amazon for $150-$300 but quality varies significantly. Dealer labor is $1,500-$2,500+ as BMW procedure requires full top removal. ZRoadster.org members have documented a motor relocation to the boot/trunk area which allows much easier future access. Hydraulic fluid: use Aral Vitamol ZHM or BMW 54340394395 hydraulic oil. PREVENTION: Clean drain holes annually, ensure rubber bungs are properly seated, and check for water intrusion in pump area at every service. Some owners have had success with pump motor rebuilds from roofmotors.co.uk ($300-$500) but quality of rebuilds varies.</x:v>
-      </x:c>
-      <x:c r="F102" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G102" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="103" ht="1135.199951171875" hidden="0" customHeight="1">
-      <x:c r="A103" s="40" t="n">
-        <x:v>102</x:v>
-      </x:c>
-      <x:c r="B103" s="9" t="str">
-        <x:v>bmw-z4-e85-window-regulator-2003</x:v>
-      </x:c>
-      <x:c r="C103" s="9" t="str">
-        <x:v>2003-2008 | BMW | Z4</x:v>
-      </x:c>
-      <x:c r="D103" s="9" t="str">
-        <x:v>Power Window Regulator Failure - E85 Z4</x:v>
-      </x:c>
-      <x:c r="E103" s="9" t="str">
-        <x:v>Option 1 (Budget): Window regulator repair kit - replacement cables and rollers for ~$18-$25 from eBay/Amazon (BWR974 for left/driver side). Requires removing door panel and threading new cables through existing regulator frame. DIY-friendly with Z4-forum.com guides. Option 2 (Recommended): Full window regulator replacement. Driver side: BMW 51337198909 ($180-$280 OEM, $80-$150 aftermarket). Passenger side: BMW 51337198910 ($180-$280 OEM, $80-$150 aftermarket). Labor: $200-$400 at independent shop, $500-$700+ at dealer. DIY: 2-3 hours with door panel removal guide from Pelican Parts. ZRoadster.org recommends full replacement over repair kit for long-term reliability.</x:v>
-      </x:c>
-      <x:c r="F103" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G103" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="104" ht="514.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A104" s="40" t="n">
-        <x:v>103</x:v>
-      </x:c>
-      <x:c r="B104" s="9" t="str">
-        <x:v>bmw-z4-electric-steering-rack-2003</x:v>
-      </x:c>
-      <x:c r="C104" s="9" t="str">
-        <x:v>2012-2012 | BMW | Z4</x:v>
-      </x:c>
-      <x:c r="D104" s="9" t="str">
-        <x:v>2012 Z4 Electric Power-Steering Recall 12V-302</x:v>
-      </x:c>
-      <x:c r="E104" s="9" t="str">
-        <x:v>Check the VIN for an open 12V-302 campaign. If open, an authorized BMW dealer replaces the steering-assistance module free of charge. If the steering warning and audible alert occur, maintain control, reduce speed, stop safely and arrange dealer or roadside assistance; do not replace a steering rack from this card.</x:v>
-      </x:c>
-      <x:c r="F104" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G104" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="105" ht="633.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A105" s="40" t="n">
-        <x:v>104</x:v>
-      </x:c>
-      <x:c r="B105" s="9" t="str">
-        <x:v>bmw-z4-electric-water-pump-2006</x:v>
-      </x:c>
-      <x:c r="C105" s="9" t="str">
-        <x:v>2012-2016 | BMW | Z4 | N20</x:v>
-      </x:c>
-      <x:c r="D105" s="9" t="str">
-        <x:v>2012-2016 Z4 sDrive28i Water-Pump Connector Recall 24V-608</x:v>
-      </x:c>
-      <x:c r="E105" s="9" t="str">
-        <x:v>Check the VIN for an open 24V-608 campaign. If open, an authorized BMW dealer inspects the water pump and connector, replaces them if necessary, and installs the protective shield free of charge. If smoke appears from the engine compartment, stop safely, switch off the vehicle, have occupants exit, move away from traffic and call emergency or roadside assistance; do not order a pump from this card.</x:v>
-      </x:c>
-      <x:c r="F105" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G105" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="106" ht="1359.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A106" s="40" t="n">
-        <x:v>105</x:v>
-      </x:c>
-      <x:c r="B106" s="9" t="str">
-        <x:v>bmw-z4-g29-b58-water-pump-2019</x:v>
-      </x:c>
-      <x:c r="C106" s="9" t="str">
-        <x:v>2019-2025 | BMW | Z4 | M40i, sDrive35i, sDrive35is | B48, B58</x:v>
-      </x:c>
-      <x:c r="D106" s="9" t="str">
-        <x:v>B48/B58 Electric Water Pump &amp; Thermostat Failure - G29 Z4</x:v>
-      </x:c>
-      <x:c r="E106" s="9" t="str">
-        <x:v>Preventative replacement recommended at 60,000 miles. Always replace water pump and thermostat together - they share labor overlap and frequently fail concurrently. B48 sDrive30i: Water pump BMW 11518632586 ($300-$450), Thermostat BMW 11538685978 ($100-$150). B58 M40i: Water pump BMW 11518650986 ($350-$500), Thermostat BMW 11538685978 ($100-$150). Mishimoto offers performance water pump alternatives for B58 with improved impeller design. Replace 3 O-rings between thermostat and pump housing, plus 2 O-rings on coolant tube to head. Must replace water pump mounting bolts (torque-to-yield). Labor: 3-4 hours. FCP Euro lifetime warranty kits available. Also inspect plastic cylinder head coolant outlet adapter - known to shear off causing massive coolant leak.</x:v>
-      </x:c>
-      <x:c r="F106" s="9" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G106" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="107" ht="1122" hidden="0" customHeight="1">
-      <x:c r="A107" s="40" t="n">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="B107" s="9" t="str">
-        <x:v>bmw-z4-n54-hpfp-2009</x:v>
-      </x:c>
-      <x:c r="C107" s="9" t="str">
-        <x:v>2009-2011 | BMW | Z4 | M40i, sDrive35i, sDrive35is | N54</x:v>
-      </x:c>
-      <x:c r="D107" s="9" t="str">
-        <x:v>N54 High Pressure Fuel Pump (HPFP) Failure - E89 Z4 sDrive35i/35is</x:v>
-      </x:c>
-      <x:c r="E107" s="9" t="str">
-        <x:v>Replace HPFP with latest revision Genuine BMW unit. The pump went through multiple revisions - ONLY install the latest version. Part number evolution: Original -&gt; 13517592881 (Index 10, TSB fix) -&gt; 13517616170 (latest revision, most reliable). Genuine BMW 13517616170 is the definitive fix ($350-$550 for pump). Replacement is straightforward DIY (1-2 hours) with basic tools. Also available as complete kit from FCP Euro with lifetime warranty. BMW extended warranty coverage to 10 years/120,000 miles under customer care package for original owners - check VIN eligibility. Replace low-pressure fuel sensor at same time (13537537319) as it may have been damaged by pressure fluctuations ($35-$55).</x:v>
-      </x:c>
-      <x:c r="F107" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G107" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="108" ht="580.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A108" s="40" t="n">
-        <x:v>107</x:v>
-      </x:c>
-      <x:c r="B108" s="9" t="str">
-        <x:v>bmw-z4-n54-wastegate-rattle-2009</x:v>
-      </x:c>
-      <x:c r="C108" s="9" t="str">
-        <x:v>2009-2010 | BMW | Z4 | N54</x:v>
-      </x:c>
-      <x:c r="D108" s="9" t="str">
-        <x:v>2009-2010 Z4 sDrive35i N54 Wastegate Diagnosis</x:v>
-      </x:c>
-      <x:c r="E108" s="9" t="str">
-        <x:v>Confirm the VIN, engine, production date, DME faults, boost-control data and noise source using current BMW diagnostic information. Check VIN-specific coverage history with BMW, recognizing that the bulletin's time/mileage window may have expired. Do not replace a turbocharger, actuator or wastegate from this card without the required diagnosis.</x:v>
-      </x:c>
-      <x:c r="F108" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G108" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="109" ht="501.6000061035156" hidden="0" customHeight="1">
-      <x:c r="A109" s="40" t="n">
-        <x:v>108</x:v>
-      </x:c>
-      <x:c r="B109" s="9" t="str">
-        <x:v>bmw-z4-soft-top-hydraulic-2003</x:v>
-      </x:c>
-      <x:c r="C109" s="9" t="str">
-        <x:v>2009-2016 | BMW | Z4</x:v>
-      </x:c>
-      <x:c r="D109" s="9" t="str">
-        <x:v>Retractable Hard Top Hydraulic Mechanism Failure</x:v>
-      </x:c>
-      <x:c r="E109" s="9" t="str">
-        <x:v>Diagnose the leak location and replace the failed component. Common failure points are the main hydraulic cylinders (left and right), the hydraulic pump motor, and the flexible hoses. The hydraulic fluid should be flushed and replaced with BMW-approved CHF 11S fluid. A full system bleed is required after any repair.</x:v>
-      </x:c>
-      <x:c r="F109" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G109" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="110" ht="1188" hidden="0" customHeight="1">
-      <x:c r="A110" s="40" t="n">
-        <x:v>109</x:v>
-      </x:c>
-      <x:c r="B110" s="9" t="str">
-        <x:v>bmw-z4-vanos-solenoid-2003</x:v>
-      </x:c>
-      <x:c r="C110" s="9" t="str">
-        <x:v>2003-2016 | BMW | Z4 | 2.5i, 3.0i, 3.0si, M40i, sDrive28i, sDrive30i, sDrive35i, sDrive35is | M54, N52, N54, N20</x:v>
-      </x:c>
-      <x:c r="D110" s="9" t="str">
-        <x:v>VANOS Solenoid &amp; System Failure - E85/E89 Z4 (All Engines)</x:v>
-      </x:c>
-      <x:c r="E110" s="9" t="str">
-        <x:v>Replace VANOS solenoids - inexpensive and straightforward repair. M54 (E85 2003-2005): 2 solenoids required, BMW 11361707323 ($35-$65 each). N52 (E85 2006-2008 / E89 2009-2011 28i): 2 solenoids, BMW 11367585425 ($40-$70 each). N54 (E89 35i/35is): 2 solenoids, BMW 11367585425 ($40-$70 each). N20 (E89 sDrive28i 2012-2016): 2 solenoids, BMW 11367585425 ($40-$70 each). Labor: under 1 hour for experienced mechanic, 2-3 hours DIY. Replace all solenoids at once even if only one has failed - the others are same age and will fail soon. Also replace VANOS solenoid O-rings and sealing plates during service. Clean VANOS system with Beisan Systems VANOS cleaning procedure for best results.</x:v>
-      </x:c>
-      <x:c r="F110" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G110" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="111" ht="554.4000244140625" hidden="0" customHeight="1">
-      <x:c r="A111" s="42" t="n">
-        <x:v>110</x:v>
-      </x:c>
-      <x:c r="B111" s="43" t="str">
-        <x:v>bmw-z8-soft-top-mechanism-2000</x:v>
-      </x:c>
-      <x:c r="C111" s="43" t="str">
-        <x:v>2000-2003 | BMW | Z8</x:v>
-      </x:c>
-      <x:c r="D111" s="43" t="str">
-        <x:v>Power Soft Top Hydraulic System and Cable Failure</x:v>
-      </x:c>
-      <x:c r="E111" s="43" t="str">
-        <x:v>Rebuild the hydraulic cylinders with new seals rather than replacing ($200 vs $2,000+). Inspect and replace frayed cables. Adjust or replace the microswitch sensors at the windshield header latch. Lubricate the top mechanism pivot points with silicone grease annually. Store the car with the top up to reduce stress on the hydraulic system.</x:v>
-      </x:c>
-      <x:c r="F111" s="43" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G111" s="44" t="str">
+      <x:c r="G86" s="44" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Extend BMW repair-first review to 325 issues
</commit_message>
<xml_diff>
--- a/outputs/bmw-repair-first-review/BMW-repair-first-fitment-review.xlsx
+++ b/outputs/bmw-repair-first-review/BMW-repair-first-fitment-review.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2a2783990d0d40c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BMW Review" sheetId="2" r:id="R14520d05eee340ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remaining Queue" sheetId="3" r:id="R5abd430bd65d4c88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="4" r:id="Rad630376318b466d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R6831979ca4fd4539"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BMW Review" sheetId="2" r:id="R61289c9b9a4243d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remaining Queue" sheetId="3" r:id="R4109b83f250a4aca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="4" r:id="R41d348202c3a4f50"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -484,7 +484,7 @@
         <x:v>Reviewed in this batch</x:v>
       </x:c>
       <x:c r="B5" s="13" t="n">
-        <x:v>300</x:v>
+        <x:v>325</x:v>
       </x:c>
       <x:c r="C5" s="11"/>
       <x:c r="D5" s="11"/>
@@ -498,7 +498,7 @@
         <x:v>Remaining queue</x:v>
       </x:c>
       <x:c r="B6" s="13" t="n">
-        <x:v>85</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C6" s="11"/>
       <x:c r="D6" s="11"/>
@@ -512,7 +512,7 @@
         <x:v>Issues with destinations</x:v>
       </x:c>
       <x:c r="B7" s="13" t="n">
-        <x:v>297</x:v>
+        <x:v>322</x:v>
       </x:c>
       <x:c r="C7" s="11"/>
       <x:c r="D7" s="11"/>
@@ -526,7 +526,7 @@
         <x:v>Destination entries</x:v>
       </x:c>
       <x:c r="B8" s="13" t="n">
-        <x:v>430</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C8" s="11"/>
       <x:c r="D8" s="11"/>
@@ -540,7 +540,7 @@
         <x:v>Distinct URLs</x:v>
       </x:c>
       <x:c r="B9" s="13" t="n">
-        <x:v>146</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="C9" s="11"/>
       <x:c r="D9" s="11"/>
@@ -16554,28 +16554,1390 @@
       </x:c>
     </x:row>
     <x:row r="434" ht="132" hidden="0" customHeight="1">
-      <x:c r="A434" s="42" t="str"/>
-      <x:c r="B434" s="43" t="str"/>
-      <x:c r="C434" s="43" t="str"/>
-      <x:c r="D434" s="43" t="str"/>
-      <x:c r="E434" s="43" t="str"/>
-      <x:c r="F434" s="43" t="str"/>
-      <x:c r="G434" s="43" t="str"/>
-      <x:c r="H434" s="43" t="str">
+      <x:c r="A434" s="40" t="str"/>
+      <x:c r="B434" s="9" t="str"/>
+      <x:c r="C434" s="9" t="str"/>
+      <x:c r="D434" s="9" t="str"/>
+      <x:c r="E434" s="9" t="str"/>
+      <x:c r="F434" s="9" t="str"/>
+      <x:c r="G434" s="9" t="str"/>
+      <x:c r="H434" s="9" t="str">
         <x:v>BMW X3 VANOS catalog</x:v>
       </x:c>
-      <x:c r="I434" s="43" t="str">
+      <x:c r="I434" s="9" t="str">
         <x:v>https://www.fcpeuro.com/BMW-parts/X3/VANOS-Solenoid/</x:v>
       </x:c>
-      <x:c r="J434" s="43" t="str">
+      <x:c r="J434" s="9" t="str">
         <x:v>2007-2017 X3; select N52/N55, intake/exhaust, VIN, and diagnosed component</x:v>
       </x:c>
-      <x:c r="K434" s="43" t="str">
+      <x:c r="K434" s="9" t="str">
         <x:v>engine-specific VANOS catalog</x:v>
       </x:c>
-      <x:c r="L434" s="43" t="str"/>
-      <x:c r="M434" s="43" t="str"/>
-      <x:c r="N434" s="44" t="str"/>
+      <x:c r="L434" s="9" t="str"/>
+      <x:c r="M434" s="9" t="str"/>
+      <x:c r="N434" s="41" t="str"/>
+    </x:row>
+    <x:row r="435" ht="1016.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A435" s="40" t="n">
+        <x:v>301</x:v>
+      </x:c>
+      <x:c r="B435" s="9" t="str">
+        <x:v>bmw-x3-wastegate-rattle-2011</x:v>
+      </x:c>
+      <x:c r="C435" s="9" t="str">
+        <x:v>2011-2023 | BMW | X3 | M40i, M50, sDrive30i, xDrive28i, xDrive30i, xDrive35i</x:v>
+      </x:c>
+      <x:c r="D435" s="9" t="str">
+        <x:v>Turbocharger Wastegate Rattle (N55, N20, B58 Engines)</x:v>
+      </x:c>
+      <x:c r="E435" s="9" t="str">
+        <x:v>Replace wastegate actuator ($400-800) or use aftermarket wastegate repair kit with upgraded stainless steel bushings ($150-300). Some cases require complete turbocharger replacement ($2,000-$4,000). VTT (Vargas Turbo Technologies) repair kits popular on forums - upgraded materials prevent future rattle. MONITORING: Early wastegate rattle may be harmless (annoying but no performance loss). If car boosts normally and no underboost codes, can monitor rattle without urgent repair. However, if check engine light appears with code 30FF or boost pressure drops, repair immediately to prevent turbo damage.</x:v>
+      </x:c>
+      <x:c r="F435" s="9" t="str">
+        <x:v>Boost/wastegate diagnosis; split N20/N55/B58 and vacuum/electronic actuation; actuator/repair kit only if serviceable; bank/VIN-specific turbo only for severe wear</x:v>
+      </x:c>
+      <x:c r="G435" s="9" t="str">
+        <x:v>ENGINE / ACTUATION-SYSTEM SPLIT</x:v>
+      </x:c>
+      <x:c r="H435" s="9" t="str">
+        <x:v>BMW X3 turbo-control catalog</x:v>
+      </x:c>
+      <x:c r="I435" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/X3/Turbocharger-Boost-Control-Valve/</x:v>
+      </x:c>
+      <x:c r="J435" s="9" t="str">
+        <x:v>2011-2023 X3; select engine, chassis, production date, and diagnosed control system</x:v>
+      </x:c>
+      <x:c r="K435" s="9" t="str">
+        <x:v>vehicle-specific boost-control catalog</x:v>
+      </x:c>
+      <x:c r="L435" s="9" t="str"/>
+      <x:c r="M435" s="9" t="str">
+        <x:v>The range combines three engine families and different actuator designs; rattle without boost loss can be monitored.</x:v>
+      </x:c>
+      <x:c r="N435" s="41" t="str">
+        <x:v>Do not attach one VTT kit or complete turbo across N20/N55/B58; confirm serviceability and exact fitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="436" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A436" s="40" t="str"/>
+      <x:c r="B436" s="9" t="str"/>
+      <x:c r="C436" s="9" t="str"/>
+      <x:c r="D436" s="9" t="str"/>
+      <x:c r="E436" s="9" t="str"/>
+      <x:c r="F436" s="9" t="str"/>
+      <x:c r="G436" s="9" t="str"/>
+      <x:c r="H436" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I436" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J436" s="9" t="str">
+        <x:v>wastegate play, boost leak, and turbo diagnosis</x:v>
+      </x:c>
+      <x:c r="K436" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L436" s="9" t="str"/>
+      <x:c r="M436" s="9" t="str"/>
+      <x:c r="N436" s="41" t="str"/>
+    </x:row>
+    <x:row r="437" ht="778.7999877929688" hidden="0" customHeight="1">
+      <x:c r="A437" s="40" t="n">
+        <x:v>302</x:v>
+      </x:c>
+      <x:c r="B437" s="9" t="str">
+        <x:v>bmw-x3-water-pump-2007</x:v>
+      </x:c>
+      <x:c r="C437" s="9" t="str">
+        <x:v>2007-2017 | BMW | X3 | sDrive30i, xDrive28i, xDrive30i | N52, N20</x:v>
+      </x:c>
+      <x:c r="D437" s="9" t="str">
+        <x:v>Electric Water Pump Failure (N52, N20 Engines)</x:v>
+      </x:c>
+      <x:c r="E437" s="9" t="str">
+        <x:v>Replace electric water pump at first sign of failure ($800 parts + labor). Consider preventative replacement at 70-80k miles to avoid being stranded ($400 parts, DIY-able). CRITICAL: If you own 2013-2017 X3 28i, verify recall repair (protective shield installation) has been completed to prevent fire risk - check with BMW dealer using VIN. If engine overheats, PULL OVER IMMEDIATELY and shut off - driving with overheating warps cylinder heads ($4,000+ repair). Call tow truck.</x:v>
+      </x:c>
+      <x:c r="F437" s="9" t="str">
+        <x:v>Stop/tow after overheat; split N52/N20 and pump variants; exact pump after fault test; thermostat by condition; VIN recall/campaign check where applicable</x:v>
+      </x:c>
+      <x:c r="G437" s="9" t="str">
+        <x:v>ENGINE / VIN / CAMPAIGN GATE</x:v>
+      </x:c>
+      <x:c r="H437" s="9" t="str">
+        <x:v>BMW recall lookup</x:v>
+      </x:c>
+      <x:c r="I437" s="9" t="str">
+        <x:v>https://www.bmwusa.com/safety-and-emission-recalls.html</x:v>
+      </x:c>
+      <x:c r="J437" s="9" t="str">
+        <x:v>VIN check for applicable X3 protective-shield campaign</x:v>
+      </x:c>
+      <x:c r="K437" s="9" t="str">
+        <x:v>manufacturer campaign route</x:v>
+      </x:c>
+      <x:c r="L437" s="9" t="str"/>
+      <x:c r="M437" s="9" t="str">
+        <x:v>N52 and N20 applications, recalls, and pump part numbers cannot be merged into one preventive replacement link.</x:v>
+      </x:c>
+      <x:c r="N437" s="41" t="str">
+        <x:v>Remove fixed 70-80k replacement and price claims; diagnose and verify VIN campaign status.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="438" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A438" s="40" t="str"/>
+      <x:c r="B438" s="9" t="str"/>
+      <x:c r="C438" s="9" t="str"/>
+      <x:c r="D438" s="9" t="str"/>
+      <x:c r="E438" s="9" t="str"/>
+      <x:c r="F438" s="9" t="str"/>
+      <x:c r="G438" s="9" t="str"/>
+      <x:c r="H438" s="9" t="str">
+        <x:v>BMW X3 water-pump catalog</x:v>
+      </x:c>
+      <x:c r="I438" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x3-water_pump.html</x:v>
+      </x:c>
+      <x:c r="J438" s="9" t="str">
+        <x:v>2007-2017 X3; exact engine, VIN, and pump circuit required</x:v>
+      </x:c>
+      <x:c r="K438" s="9" t="str">
+        <x:v>OEM pump catalog</x:v>
+      </x:c>
+      <x:c r="L438" s="9" t="str"/>
+      <x:c r="M438" s="9" t="str"/>
+      <x:c r="N438" s="41" t="str"/>
+    </x:row>
+    <x:row r="439" ht="1240.800048828125" hidden="0" customHeight="1">
+      <x:c r="A439" s="40" t="n">
+        <x:v>303</x:v>
+      </x:c>
+      <x:c r="B439" s="9" t="str">
+        <x:v>bmw-x3m-brake-wear-2020</x:v>
+      </x:c>
+      <x:c r="C439" s="9" t="str">
+        <x:v>2020-2023 | BMW | X3 M | S58</x:v>
+      </x:c>
+      <x:c r="D439" s="9" t="str">
+        <x:v>Accelerated Brake Pad &amp; Rotor Wear from Vehicle Weight - F97 X3 M / F98 X4 M</x:v>
+      </x:c>
+      <x:c r="E439" s="9" t="str">
+        <x:v>Front brake replacement: OEM front rotor (34118054825 left, matching right) with OEM M compound pads. Complete OEM front brake kit available from BimmerWorld (34108064561K1, ~$800-$1,000). Rear brake kit similarly priced. For track use: Upgrade to Brembo GT brake pad set (BM8 compound) for improved heat resistance and longer pad life. EBC Yellowstuff or Hawk HPS 5.0 pads are popular street/track compromise choices ($150-$250 per axle). StopTech slotted rotors offer improved heat dissipation. For dedicated track cars: Brembo GT big brake kit with 412x38mm discs available ($4,000-$6,000 installed). Budget $2,000-$3,000 per year for brake maintenance if driving spiritedly. Use high-temperature brake fluid (Motul RBF 660 or ATE Typ 200) and flush every 12 months.</x:v>
+      </x:c>
+      <x:c r="F439" s="9" t="str">
+        <x:v>Identify brake option and axle; measure pads/rotors; VIN/corner-specific OEM replacement; track pads/fluid only for actual use and temperature range</x:v>
+      </x:c>
+      <x:c r="G439" s="9" t="str">
+        <x:v>BRAKE-OPTION / AXLE GATE</x:v>
+      </x:c>
+      <x:c r="H439" s="9" t="str">
+        <x:v>BMW X3 M brake catalog</x:v>
+      </x:c>
+      <x:c r="I439" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/X3-M/Brakes/</x:v>
+      </x:c>
+      <x:c r="J439" s="9" t="str">
+        <x:v>2020-2023 F97 X3 M; select VIN, front/rear axle, rotor side, and brake option</x:v>
+      </x:c>
+      <x:c r="K439" s="9" t="str">
+        <x:v>vehicle-specific brake catalog</x:v>
+      </x:c>
+      <x:c r="L439" s="9" t="str"/>
+      <x:c r="M439" s="9" t="str">
+        <x:v>Rotors are side-specific and pad/fluid choices depend on street versus track use; the claimed BimmerWorld kit page was not verified.</x:v>
+      </x:c>
+      <x:c r="N439" s="41" t="str">
+        <x:v>Hold named aftermarket pads/rotors until exact F97 fitment, axle, and operating range are verified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="440" ht="66" hidden="0" customHeight="1">
+      <x:c r="A440" s="40" t="str"/>
+      <x:c r="B440" s="9" t="str"/>
+      <x:c r="C440" s="9" t="str"/>
+      <x:c r="D440" s="9" t="str"/>
+      <x:c r="E440" s="9" t="str"/>
+      <x:c r="F440" s="9" t="str"/>
+      <x:c r="G440" s="9" t="str"/>
+      <x:c r="H440" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I440" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J440" s="9" t="str">
+        <x:v>brake measurement and track-use setup</x:v>
+      </x:c>
+      <x:c r="K440" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L440" s="9" t="str"/>
+      <x:c r="M440" s="9" t="str"/>
+      <x:c r="N440" s="41" t="str"/>
+    </x:row>
+    <x:row r="441" ht="1188" hidden="0" customHeight="1">
+      <x:c r="A441" s="40" t="n">
+        <x:v>304</x:v>
+      </x:c>
+      <x:c r="B441" s="9" t="str">
+        <x:v>bmw-x3m-cooling-track-use-2020</x:v>
+      </x:c>
+      <x:c r="C441" s="9" t="str">
+        <x:v>2020-2023 | BMW | X3 M | S58</x:v>
+      </x:c>
+      <x:c r="D441" s="9" t="str">
+        <x:v>Cooling System Heat Soak During Track/Spirited Driving - F97 X3 M / F98 X4 M</x:v>
+      </x:c>
+      <x:c r="E441" s="9" t="str">
+        <x:v>For track use: Upgrade intercooler to do88 front-mount intercooler ($1,200-$1,800) - the community standard for S58 heat management. Add CSF high-performance radiator ($600-$900) for sustained track work. Dinan or VRSF also offer intercooler upgrades in the $1,000-$1,500 range. For street/canyon driving: Stock cooling is adequate but ensure coolant flush every 2 years/30,000 miles and inspect expansion tank for cracks. Replace coolant expansion tank preemptively at 60,000 miles if car is driven hard. For all X3 M/X4 M: Use BMW coolant only (mixed 50/50 with distilled water), replace thermostat at 80,000 miles preventatively, inspect all coolant hoses for bulging or softening at every oil change.</x:v>
+      </x:c>
+      <x:c r="F441" s="9" t="str">
+        <x:v>Log track temperatures; distinguish charge-cooler core, heat exchangers, engine radiator, oil cooling, and coolant maintenance; upgrade only the limiting circuit</x:v>
+      </x:c>
+      <x:c r="G441" s="9" t="str">
+        <x:v>TRACK CONFIGURATION / COOLING-CIRCUIT GATE</x:v>
+      </x:c>
+      <x:c r="H441" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I441" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J441" s="9" t="str">
+        <x:v>F97 X3 M S58 temperature diagnosis and track cooling plan</x:v>
+      </x:c>
+      <x:c r="K441" s="9" t="str">
+        <x:v>specialist service</x:v>
+      </x:c>
+      <x:c r="L441" s="9" t="str"/>
+      <x:c r="M441" s="9" t="str">
+        <x:v>The S58 uses water-to-air charge cooling; calling every front heat exchanger an intercooler obscures which circuit needs work.</x:v>
+      </x:c>
+      <x:c r="N441" s="41" t="str">
+        <x:v>Remove mandatory intervals and preemptive tank/thermostat replacements; log the actual limiting temperature/circuit first.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="442" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A442" s="40" t="str"/>
+      <x:c r="B442" s="9" t="str"/>
+      <x:c r="C442" s="9" t="str"/>
+      <x:c r="D442" s="9" t="str"/>
+      <x:c r="E442" s="9" t="str"/>
+      <x:c r="F442" s="9" t="str"/>
+      <x:c r="G442" s="9" t="str"/>
+      <x:c r="H442" s="9" t="str">
+        <x:v>Turner F97 X3 M cooling catalog</x:v>
+      </x:c>
+      <x:c r="I442" s="9" t="str">
+        <x:v>https://www.turnermotorsport.com/BMW-F97/c-163-bmw-cooling</x:v>
+      </x:c>
+      <x:c r="J442" s="9" t="str">
+        <x:v>F97 X3 M; select exact diagnosed circuit and verify live fitment</x:v>
+      </x:c>
+      <x:c r="K442" s="9" t="str">
+        <x:v>vehicle-specific cooling catalog</x:v>
+      </x:c>
+      <x:c r="L442" s="9" t="str"/>
+      <x:c r="M442" s="9" t="str"/>
+      <x:c r="N442" s="41" t="str"/>
+    </x:row>
+    <x:row r="443" ht="1214.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A443" s="40" t="n">
+        <x:v>305</x:v>
+      </x:c>
+      <x:c r="B443" s="9" t="str">
+        <x:v>bmw-x3m-differential-bolt-2020</x:v>
+      </x:c>
+      <x:c r="C443" s="9" t="str">
+        <x:v>2020-2023 | BMW | X3 M | S58</x:v>
+      </x:c>
+      <x:c r="D443" s="9" t="str">
+        <x:v>Rear Differential Mounting Bolt &amp; Bush Failure - F97 X3 M / F98 X4 M</x:v>
+      </x:c>
+      <x:c r="E443" s="9" t="str">
+        <x:v>Replace factory differential bolt, bush, and collar with FJ Motorwerkes uprated diff bolt and collar upgrade kit. The FJ kit uses premium CNC-machined stainless steel components that can handle 170,000 PSI (39% stronger than BMW's revised bolt). Kit price approximately $255 (GBP). Available from FJ Motorwerkes directly, BMG Performance, AM Tuning, and H4ck Performance. Installation is straightforward - rear differential does not need to be fully removed. Budget $400-$600 total including labor. This upgrade is considered MANDATORY by the X3 M/X4 M community for any car making stock or above power. JXB Performance also offers a driveshaft carrier bearing upgrade for cars experiencing propshaft vibration as a companion fix.</x:v>
+      </x:c>
+      <x:c r="F443" s="9" t="str">
+        <x:v>Inspect revised bolt/mount/bushing and driveline; F97/F98 FJ bolt/collar kit when owner accepts NVH/installation tradeoffs; torque verification</x:v>
+      </x:c>
+      <x:c r="G443" s="9" t="str">
+        <x:v>EXACT F97/F98 KIT; CLAIMS QUALIFIED</x:v>
+      </x:c>
+      <x:c r="H443" s="9" t="str">
+        <x:v>FJ X3M/X4M diff bolt and collar kit</x:v>
+      </x:c>
+      <x:c r="I443" s="9" t="str">
+        <x:v>https://bmgperformance.com/products/fj-motorwerkes-x3m-x4m-diff-bolt-and-collar-upgrade</x:v>
+      </x:c>
+      <x:c r="J443" s="9" t="str">
+        <x:v>F97 X3 M/F98 X4 M as explicitly listed; confirm stock, revision, and installer requirements</x:v>
+      </x:c>
+      <x:c r="K443" s="9" t="str">
+        <x:v>conditional differential-mount upgrade</x:v>
+      </x:c>
+      <x:c r="L443" s="9" t="str"/>
+      <x:c r="M443" s="9" t="str">
+        <x:v>The live page explicitly lists F97/F98 and discloses the complete bolt/bushing/collar contents.</x:v>
+      </x:c>
+      <x:c r="N443" s="41" t="str">
+        <x:v>Do not call the upgrade mandatory or repeat strength claims as independent proof; inspect the installed revision and discuss NVH.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="444" ht="1293.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A444" s="40" t="n">
+        <x:v>306</x:v>
+      </x:c>
+      <x:c r="B444" s="9" t="str">
+        <x:v>bmw-x3m-s58-bearing-recall-2020</x:v>
+      </x:c>
+      <x:c r="C444" s="9" t="str">
+        <x:v>2020-2021 | BMW | X3 M</x:v>
+      </x:c>
+      <x:c r="D444" s="9" t="str">
+        <x:v>S58 Engine Main Bearing Shell Recall / Stop Sale - F97 X3 M / F98 X4 M</x:v>
+      </x:c>
+      <x:c r="E444" s="9" t="str">
+        <x:v>Check VIN immediately against BMW recall database at bmwusa.com or contact your BMW dealer. If your vehicle is within the affected production date range, BMW will inspect and replace main bearing shells at no cost under the Tech Campaign. The repair requires removing the cylinder head and oil pan to access and replace all main bearing shells - this is a major repair (8-12 hours labor) but fully covered by BMW. Do NOT drive the vehicle if knocking is present. For S58 vehicles outside the recall range: Proactive rod bearing inspection is recommended at 60,000 miles for track-driven vehicles. ACL Race Series rod bearings 6B1510H-STD are the aftermarket upgrade choice on Bimmerpost for preventive replacement ($150-$250 for bearing set, $3,000-$5,000 total with labor).</x:v>
+      </x:c>
+      <x:c r="F444" s="9" t="str">
+        <x:v>VIN campaign check; stop/tow for knocking; free dealer main-bearing remedy if affected; no preventive rod-bearing product outside campaign without diagnosis</x:v>
+      </x:c>
+      <x:c r="G444" s="9" t="str">
+        <x:v>CAMPAIGN ROUTES ONLY; AFTERMARKET CLAIM REJECTED</x:v>
+      </x:c>
+      <x:c r="H444" s="9" t="str">
+        <x:v>BMW recall lookup</x:v>
+      </x:c>
+      <x:c r="I444" s="9" t="str">
+        <x:v>https://www.bmwusa.com/safety-and-emission-recalls.html</x:v>
+      </x:c>
+      <x:c r="J444" s="9" t="str">
+        <x:v>VIN check for S58 main-bearing technical campaign</x:v>
+      </x:c>
+      <x:c r="K444" s="9" t="str">
+        <x:v>manufacturer campaign route</x:v>
+      </x:c>
+      <x:c r="L444" s="9" t="str"/>
+      <x:c r="M444" s="9" t="str">
+        <x:v>Main-bearing campaign work is not equivalent to aftermarket rod-bearing prevention.</x:v>
+      </x:c>
+      <x:c r="N444" s="41" t="str">
+        <x:v>Remove the unrelated 60,000-mile ACL rod-bearing recommendation and verify whether the action is a recall or technical campaign before labeling it.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="445" ht="66" hidden="0" customHeight="1">
+      <x:c r="A445" s="40" t="str"/>
+      <x:c r="B445" s="9" t="str"/>
+      <x:c r="C445" s="9" t="str"/>
+      <x:c r="D445" s="9" t="str"/>
+      <x:c r="E445" s="9" t="str"/>
+      <x:c r="F445" s="9" t="str"/>
+      <x:c r="G445" s="9" t="str"/>
+      <x:c r="H445" s="9" t="str">
+        <x:v>BMW dealer locator</x:v>
+      </x:c>
+      <x:c r="I445" s="9" t="str">
+        <x:v>https://www.bmwusa.com/dealer-locator.html</x:v>
+      </x:c>
+      <x:c r="J445" s="9" t="str">
+        <x:v>campaign eligibility and covered repair</x:v>
+      </x:c>
+      <x:c r="K445" s="9" t="str">
+        <x:v>authorized repair</x:v>
+      </x:c>
+      <x:c r="L445" s="9" t="str"/>
+      <x:c r="M445" s="9" t="str"/>
+      <x:c r="N445" s="41" t="str"/>
+    </x:row>
+    <x:row r="446" ht="1227.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A446" s="40" t="n">
+        <x:v>307</x:v>
+      </x:c>
+      <x:c r="B446" s="9" t="str">
+        <x:v>bmw-x3m-transfer-case-2020</x:v>
+      </x:c>
+      <x:c r="C446" s="9" t="str">
+        <x:v>2020-2023 | BMW | X3 M | S58</x:v>
+      </x:c>
+      <x:c r="D446" s="9" t="str">
+        <x:v>xDrive Transfer Case Stress &amp; Fluid Degradation - F97 X3 M / F98 X4 M</x:v>
+      </x:c>
+      <x:c r="E446" s="9" t="str">
+        <x:v>Change transfer case fluid every 30,000 miles (BMW says "lifetime fill" - this is NOT correct for M vehicles driven hard). Use BMW DTF-1 transfer case fluid or equivalent high-quality synthetic. Check tire tread depth at every service - all 4 tires must be within 2/32" of each other to prevent transfer case stress. Rotate tires every 5,000-7,000 miles. If transfer case actuator motor fails: FCP Euro guide for BMW transfer case actuator repair (part number varies by production date, ~$300-$600). For tuned cars: Consider transfer case brace/reinforcement and shortened fluid change intervals (every 15,000 miles). Complete transfer case replacement if internals are damaged: $3,000-$5,500 at independent specialist, $5,000-$8,000+ at dealer.</x:v>
+      </x:c>
+      <x:c r="F446" s="9" t="str">
+        <x:v>Tire circumference/tread check; VTG faults and fluid condition; VIN-specific DTF-1 service if specified; actuator versus internal diagnosis; initialization</x:v>
+      </x:c>
+      <x:c r="G446" s="9" t="str">
+        <x:v>VIN / DIAGNOSIS / FLUID-SPEC GATE</x:v>
+      </x:c>
+      <x:c r="H446" s="9" t="str">
+        <x:v>BMW X3 M transfer-case catalog</x:v>
+      </x:c>
+      <x:c r="I446" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x3_m-transfer_case.html</x:v>
+      </x:c>
+      <x:c r="J446" s="9" t="str">
+        <x:v>2020-2023 F97 X3 M; VIN and production date required</x:v>
+      </x:c>
+      <x:c r="K446" s="9" t="str">
+        <x:v>OEM drivetrain catalog</x:v>
+      </x:c>
+      <x:c r="L446" s="9" t="str"/>
+      <x:c r="M446" s="9" t="str">
+        <x:v>Fluid interval, actuator, brace, and transfer-case replacement are distinct branches.</x:v>
+      </x:c>
+      <x:c r="N446" s="41" t="str">
+        <x:v>Remove mandatory 30k/15k intervals and generic tire-rotation advice; follow tire pattern/manual and exact unit specification.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="447" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A447" s="40" t="str"/>
+      <x:c r="B447" s="9" t="str"/>
+      <x:c r="C447" s="9" t="str"/>
+      <x:c r="D447" s="9" t="str"/>
+      <x:c r="E447" s="9" t="str"/>
+      <x:c r="F447" s="9" t="str"/>
+      <x:c r="G447" s="9" t="str"/>
+      <x:c r="H447" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I447" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J447" s="9" t="str">
+        <x:v>VTG diagnosis, fluid service, and initialization</x:v>
+      </x:c>
+      <x:c r="K447" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L447" s="9" t="str"/>
+      <x:c r="M447" s="9" t="str"/>
+      <x:c r="N447" s="41" t="str"/>
+    </x:row>
+    <x:row r="448" ht="673.2000122070312" hidden="0" customHeight="1">
+      <x:c r="A448" s="40" t="n">
+        <x:v>308</x:v>
+      </x:c>
+      <x:c r="B448" s="9" t="str">
+        <x:v>bmw-x4-n20-timing-chain-2015</x:v>
+      </x:c>
+      <x:c r="C448" s="9" t="str">
+        <x:v>2015-2016 | BMW | X4 | xDrive28i, xDrive30i</x:v>
+      </x:c>
+      <x:c r="D448" s="9" t="str">
+        <x:v>N20 Timing Chain Premature Failure - F26 X4 xDrive28i</x:v>
+      </x:c>
+      <x:c r="E448" s="9" t="str">
+        <x:v>Complete timing chain kit replacement including chain, guides, tensioner, and sprockets. Must be performed by experienced BMW technician. Preventive replacement recommended at 60,000-80,000 miles. BMW extended warranty to 8 years/100,000 miles under class action settlement. Upgraded reinforced chain kit available from aftermarket. Labor is 10-14 hours for X4 due to AWD and tight engine bay.</x:v>
+      </x:c>
+      <x:c r="F448" s="9" t="str">
+        <x:v>Confirm N20/production date and timing diagnosis; complete chain/guide/tensioner/oil-pump-chain service kit; specialist installation</x:v>
+      </x:c>
+      <x:c r="G448" s="9" t="str">
+        <x:v>EXACT N20 KIT AFTER DIAGNOSIS</x:v>
+      </x:c>
+      <x:c r="H448" s="9" t="str">
+        <x:v>FCP Euro N20/N26 timing kit 11318648732KT</x:v>
+      </x:c>
+      <x:c r="I448" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/products/bmw-n20-n26-timing-chain-kit-11318648732kt</x:v>
+      </x:c>
+      <x:c r="J448" s="9" t="str">
+        <x:v>2015-2016 F26 X4 xDrive28i N20 where cataloged; verify VIN and completeness</x:v>
+      </x:c>
+      <x:c r="K448" s="9" t="str">
+        <x:v>engine-specific timing kit</x:v>
+      </x:c>
+      <x:c r="L448" s="9" t="str"/>
+      <x:c r="M448" s="9" t="str">
+        <x:v>The live kit covers N20 applications including X4, subject to vehicle selection.</x:v>
+      </x:c>
+      <x:c r="N448" s="41" t="str">
+        <x:v>The cited warranty terms conflict with the adjacent corrected row; verify historical eligibility and remove universal preventive interval/labor claims.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="449" ht="686.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A449" s="40" t="n">
+        <x:v>309</x:v>
+      </x:c>
+      <x:c r="B449" s="9" t="str">
+        <x:v>bmw-x4-n20-timing-chain-guide-2015</x:v>
+      </x:c>
+      <x:c r="C449" s="9" t="str">
+        <x:v>2015-2015 | BMW | X4 | N20</x:v>
+      </x:c>
+      <x:c r="D449" s="9" t="str">
+        <x:v>2015 X4 N20 Lower-Engine Whine Requires Timing-Chain Diagnosis</x:v>
+      </x:c>
+      <x:c r="E449" s="9" t="str">
+        <x:v>Confirm the exact xDrive28i variant, N20 engine, production date and VIN eligibility, then have a BMW-qualified technician reproduce the noise and follow current BMW diagnosis before replacing anything. The historical seven-year/70,000-mile coverage was a limited warranty extension, not a recall, and is not a current coverage promise. ShowMeTheParts established category-level fitment only, so no commerce link is approved.</x:v>
+      </x:c>
+      <x:c r="F449" s="9" t="str">
+        <x:v>Variant/engine/production/VIN confirmation; noise reproduction and BMW diagnosis; expired historical coverage disclosed accurately</x:v>
+      </x:c>
+      <x:c r="G449" s="9" t="str">
+        <x:v>DIAGNOSIS / WARRANTY-HISTORY ROUTE</x:v>
+      </x:c>
+      <x:c r="H449" s="9" t="str">
+        <x:v>BMW dealer locator</x:v>
+      </x:c>
+      <x:c r="I449" s="9" t="str">
+        <x:v>https://www.bmwusa.com/dealer-locator.html</x:v>
+      </x:c>
+      <x:c r="J449" s="9" t="str">
+        <x:v>2015 F26 X4 N20 timing diagnosis and VIN history</x:v>
+      </x:c>
+      <x:c r="K449" s="9" t="str">
+        <x:v>BMW-qualified service</x:v>
+      </x:c>
+      <x:c r="L449" s="9" t="str"/>
+      <x:c r="M449" s="9" t="str">
+        <x:v>The corrected source explicitly rejects category fitment as proof of failure.</x:v>
+      </x:c>
+      <x:c r="N449" s="41" t="str">
+        <x:v>Consolidate with the prior timing row and preserve the expired-coverage warning.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="450" ht="554.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A450" s="40" t="n">
+        <x:v>310</x:v>
+      </x:c>
+      <x:c r="B450" s="9" t="str">
+        <x:v>bmw-x4-oil-leak-2015</x:v>
+      </x:c>
+      <x:c r="C450" s="9" t="str">
+        <x:v>2015-2023 | BMW | X4</x:v>
+      </x:c>
+      <x:c r="D450" s="9" t="str">
+        <x:v>Oil Leaks - Valve Cover &amp; Oil Filter Housing - All Models</x:v>
+      </x:c>
+      <x:c r="E450" s="9" t="str">
+        <x:v>Replace valve cover gasket and/or oil filter housing gasket. Valve cover replacement is 3-4 hours labor on X4. Oil filter housing gasket is 1-2 hours. Both are routine maintenance items on BMW turbo engines. Use OEM gaskets for best longevity. Clean oil residue from engine bay after repair. Monitor oil level regularly to catch leaks early.</x:v>
+      </x:c>
+      <x:c r="F450" s="9" t="str">
+        <x:v>Leak-source diagnosis; engine/VIN-specific valve-cover gasket/cover or oil-filter-housing gasket; cleanup and belt inspection</x:v>
+      </x:c>
+      <x:c r="G450" s="9" t="str">
+        <x:v>MULTI-ENGINE / LEAK-SOURCE SPLIT</x:v>
+      </x:c>
+      <x:c r="H450" s="9" t="str">
+        <x:v>BMW X4 engine-gasket catalog</x:v>
+      </x:c>
+      <x:c r="I450" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/X4/Engine-Gaskets-and-Seals/</x:v>
+      </x:c>
+      <x:c r="J450" s="9" t="str">
+        <x:v>2015-2023 F26/G02 X4; select engine, generation, VIN, and confirmed leak source</x:v>
+      </x:c>
+      <x:c r="K450" s="9" t="str">
+        <x:v>vehicle-specific gasket catalog</x:v>
+      </x:c>
+      <x:c r="L450" s="9" t="str"/>
+      <x:c r="M450" s="9" t="str">
+        <x:v>The row crosses two generations and several engines; the two leak locations require different parts.</x:v>
+      </x:c>
+      <x:c r="N450" s="41" t="str">
+        <x:v>Do not bundle both gaskets or repeat fixed labor times across all models.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="451" ht="356.3999938964844" hidden="0" customHeight="1">
+      <x:c r="A451" s="40" t="n">
+        <x:v>311</x:v>
+      </x:c>
+      <x:c r="B451" s="9" t="str">
+        <x:v>bmw-x4-rear-differential-mount-2015</x:v>
+      </x:c>
+      <x:c r="C451" s="9" t="str">
+        <x:v>2015-2023 | BMW | X4</x:v>
+      </x:c>
+      <x:c r="D451" s="9" t="str">
+        <x:v>Rear Differential Mount Bushing Failure</x:v>
+      </x:c>
+      <x:c r="E451" s="9" t="str">
+        <x:v>Replace rear differential mount bushings. Both front and rear differential bushings should be inspected and replaced as a set. Upgraded aftermarket bushings with stiffer rubber or polyurethane are available for longer service life.</x:v>
+      </x:c>
+      <x:c r="F451" s="9" t="str">
+        <x:v>Generation/VIN-specific mount inspection; exact front/rear bushing only if worn; aftermarket stiffness chosen with NVH tradeoff</x:v>
+      </x:c>
+      <x:c r="G451" s="9" t="str">
+        <x:v>GENERATION / POSITION GATE</x:v>
+      </x:c>
+      <x:c r="H451" s="9" t="str">
+        <x:v>BMW X4 differential-mount catalog</x:v>
+      </x:c>
+      <x:c r="I451" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x4-differential_mount.html</x:v>
+      </x:c>
+      <x:c r="J451" s="9" t="str">
+        <x:v>2015-2023 F26/G02 X4; VIN, axle, and bushing position required</x:v>
+      </x:c>
+      <x:c r="K451" s="9" t="str">
+        <x:v>OEM mount catalog</x:v>
+      </x:c>
+      <x:c r="L451" s="9" t="str"/>
+      <x:c r="M451" s="9" t="str">
+        <x:v>Front/rear mounts and two chassis generations are not one set, and stiffer bushings change NVH.</x:v>
+      </x:c>
+      <x:c r="N451" s="41" t="str">
+        <x:v>Inspect all mounts but replace only failed/strategically chosen components.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="452" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A452" s="40" t="str"/>
+      <x:c r="B452" s="9" t="str"/>
+      <x:c r="C452" s="9" t="str"/>
+      <x:c r="D452" s="9" t="str"/>
+      <x:c r="E452" s="9" t="str"/>
+      <x:c r="F452" s="9" t="str"/>
+      <x:c r="G452" s="9" t="str"/>
+      <x:c r="H452" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I452" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J452" s="9" t="str">
+        <x:v>driveline mount diagnosis</x:v>
+      </x:c>
+      <x:c r="K452" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L452" s="9" t="str"/>
+      <x:c r="M452" s="9" t="str"/>
+      <x:c r="N452" s="41" t="str"/>
+    </x:row>
+    <x:row r="453" ht="620.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A453" s="40" t="n">
+        <x:v>312</x:v>
+      </x:c>
+      <x:c r="B453" s="9" t="str">
+        <x:v>bmw-x4-transfer-case-2015</x:v>
+      </x:c>
+      <x:c r="C453" s="9" t="str">
+        <x:v>2015-2023 | BMW | X4</x:v>
+      </x:c>
+      <x:c r="D453" s="9" t="str">
+        <x:v>Transfer Case Actuator Motor Failure - All xDrive X4</x:v>
+      </x:c>
+      <x:c r="E453" s="9" t="str">
+        <x:v>Diagnose specific failure. Transfer case actuator motor replacement ($800-1,200) is most common. Complete transfer case replacement required for internal failures ($2,500-4,000). Regular transfer case fluid changes every 50,000 miles may extend life. Some owners install aftermarket upgraded actuator motors. Common wear item on high-mileage xDrive BMW models.</x:v>
+      </x:c>
+      <x:c r="F453" s="9" t="str">
+        <x:v>xDrive/VTG diagnosis; split F26/G02 transfer-case units; actuator versus internal failure; exact fluid and initialization</x:v>
+      </x:c>
+      <x:c r="G453" s="9" t="str">
+        <x:v>GENERATION / UNIT SPLIT</x:v>
+      </x:c>
+      <x:c r="H453" s="9" t="str">
+        <x:v>BMW X4 transfer-case catalog</x:v>
+      </x:c>
+      <x:c r="I453" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x4-transfer_case.html</x:v>
+      </x:c>
+      <x:c r="J453" s="9" t="str">
+        <x:v>2015-2023 F26/G02 xDrive; VIN and exact unit required</x:v>
+      </x:c>
+      <x:c r="K453" s="9" t="str">
+        <x:v>OEM transfer-case catalog</x:v>
+      </x:c>
+      <x:c r="L453" s="9" t="str"/>
+      <x:c r="M453" s="9" t="str">
+        <x:v>The row crosses incompatible transfer-case generations and multiple failure branches.</x:v>
+      </x:c>
+      <x:c r="N453" s="41" t="str">
+        <x:v>Do not attach a generic actuator or fixed 50,000-mile interval across all units.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="454" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A454" s="40" t="str"/>
+      <x:c r="B454" s="9" t="str"/>
+      <x:c r="C454" s="9" t="str"/>
+      <x:c r="D454" s="9" t="str"/>
+      <x:c r="E454" s="9" t="str"/>
+      <x:c r="F454" s="9" t="str"/>
+      <x:c r="G454" s="9" t="str"/>
+      <x:c r="H454" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I454" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J454" s="9" t="str">
+        <x:v>actuator/internal diagnosis and initialization</x:v>
+      </x:c>
+      <x:c r="K454" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L454" s="9" t="str"/>
+      <x:c r="M454" s="9" t="str"/>
+      <x:c r="N454" s="41" t="str"/>
+    </x:row>
+    <x:row r="455" ht="1240.800048828125" hidden="0" customHeight="1">
+      <x:c r="A455" s="40" t="n">
+        <x:v>313</x:v>
+      </x:c>
+      <x:c r="B455" s="9" t="str">
+        <x:v>bmw-x4m-brake-wear-2020</x:v>
+      </x:c>
+      <x:c r="C455" s="9" t="str">
+        <x:v>2020-2023 | BMW | X4 M | S58</x:v>
+      </x:c>
+      <x:c r="D455" s="9" t="str">
+        <x:v>Accelerated Brake Pad &amp; Rotor Wear from Vehicle Weight - F98 X4 M / F98 X4 M</x:v>
+      </x:c>
+      <x:c r="E455" s="9" t="str">
+        <x:v>Front brake replacement: OEM front rotor (34118054825 left, matching right) with OEM M compound pads. Complete OEM front brake kit available from BimmerWorld (34108064561K1, ~$800-$1,000). Rear brake kit similarly priced. For track use: Upgrade to Brembo GT brake pad set (BM8 compound) for improved heat resistance and longer pad life. EBC Yellowstuff or Hawk HPS 5.0 pads are popular street/track compromise choices ($150-$250 per axle). StopTech slotted rotors offer improved heat dissipation. For dedicated track cars: Brembo GT big brake kit with 412x38mm discs available ($4,000-$6,000 installed). Budget $2,000-$3,000 per year for brake maintenance if driving spiritedly. Use high-temperature brake fluid (Motul RBF 660 or ATE Typ 200) and flush every 12 months.</x:v>
+      </x:c>
+      <x:c r="F455" s="9" t="str">
+        <x:v>Identify brake option and axle; measure pads/rotors; side-specific OEM replacement; track compounds/fluid by use</x:v>
+      </x:c>
+      <x:c r="G455" s="9" t="str">
+        <x:v>DUPLICATE X3M/X4M BRAKE CONFIGURATION GATE</x:v>
+      </x:c>
+      <x:c r="H455" s="9" t="str">
+        <x:v>BMW X4 M brake catalog</x:v>
+      </x:c>
+      <x:c r="I455" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/X4-M/Brakes/</x:v>
+      </x:c>
+      <x:c r="J455" s="9" t="str">
+        <x:v>2020-2023 F98 X4 M; VIN, axle, side, and brake option required</x:v>
+      </x:c>
+      <x:c r="K455" s="9" t="str">
+        <x:v>vehicle-specific brake catalog</x:v>
+      </x:c>
+      <x:c r="L455" s="9" t="str"/>
+      <x:c r="M455" s="9" t="str">
+        <x:v>This duplicates the X3 M brake text and contains a repeated F98 model label; exact axle/option selection remains required.</x:v>
+      </x:c>
+      <x:c r="N455" s="41" t="str">
+        <x:v>Fix duplicated title text and hold named aftermarket compounds until exact F98 fitment/use is verified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="456" ht="1188" hidden="0" customHeight="1">
+      <x:c r="A456" s="40" t="n">
+        <x:v>314</x:v>
+      </x:c>
+      <x:c r="B456" s="9" t="str">
+        <x:v>bmw-x4m-cooling-track-use-2020</x:v>
+      </x:c>
+      <x:c r="C456" s="9" t="str">
+        <x:v>2020-2023 | BMW | X4 M</x:v>
+      </x:c>
+      <x:c r="D456" s="9" t="str">
+        <x:v>Cooling System Heat Soak During Track/Spirited Driving - F98 X4 M / F98 X4 M</x:v>
+      </x:c>
+      <x:c r="E456" s="9" t="str">
+        <x:v>For track use: Upgrade intercooler to do88 front-mount intercooler ($1,200-$1,800) - the community standard for S58 heat management. Add CSF high-performance radiator ($600-$900) for sustained track work. Dinan or VRSF also offer intercooler upgrades in the $1,000-$1,500 range. For street/canyon driving: Stock cooling is adequate but ensure coolant flush every 2 years/30,000 miles and inspect expansion tank for cracks. Replace coolant expansion tank preemptively at 60,000 miles if car is driven hard. For all X3 M/X4 M: Use BMW coolant only (mixed 50/50 with distilled water), replace thermostat at 80,000 miles preventatively, inspect all coolant hoses for bulging or softening at every oil change.</x:v>
+      </x:c>
+      <x:c r="F456" s="9" t="str">
+        <x:v>Log track temperatures; identify limiting S58 cooling circuit; targeted radiator/heat-exchanger/charge-cooler upgrade; maintenance by actual specification</x:v>
+      </x:c>
+      <x:c r="G456" s="9" t="str">
+        <x:v>DUPLICATE / COOLING-CIRCUIT GATE</x:v>
+      </x:c>
+      <x:c r="H456" s="9" t="str">
+        <x:v>Turner F98 X4 M cooling catalog</x:v>
+      </x:c>
+      <x:c r="I456" s="9" t="str">
+        <x:v>https://www.turnermotorsport.com/BMW-F98/c-163-bmw-cooling</x:v>
+      </x:c>
+      <x:c r="J456" s="9" t="str">
+        <x:v>F98 X4 M; select diagnosed circuit and verify live fitment</x:v>
+      </x:c>
+      <x:c r="K456" s="9" t="str">
+        <x:v>vehicle-specific cooling catalog</x:v>
+      </x:c>
+      <x:c r="L456" s="9" t="str"/>
+      <x:c r="M456" s="9" t="str">
+        <x:v>This duplicates X3 M text and conflates the water-to-air charge cooler with a generic front-mount intercooler.</x:v>
+      </x:c>
+      <x:c r="N456" s="41" t="str">
+        <x:v>Fix duplicated F98 title and remove blanket tank/thermostat replacement intervals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="457" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A457" s="40" t="str"/>
+      <x:c r="B457" s="9" t="str"/>
+      <x:c r="C457" s="9" t="str"/>
+      <x:c r="D457" s="9" t="str"/>
+      <x:c r="E457" s="9" t="str"/>
+      <x:c r="F457" s="9" t="str"/>
+      <x:c r="G457" s="9" t="str"/>
+      <x:c r="H457" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I457" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J457" s="9" t="str">
+        <x:v>S58 track temperature logging and setup</x:v>
+      </x:c>
+      <x:c r="K457" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L457" s="9" t="str"/>
+      <x:c r="M457" s="9" t="str"/>
+      <x:c r="N457" s="41" t="str"/>
+    </x:row>
+    <x:row r="458" ht="1214.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A458" s="40" t="n">
+        <x:v>315</x:v>
+      </x:c>
+      <x:c r="B458" s="9" t="str">
+        <x:v>bmw-x4m-differential-bolt-2020</x:v>
+      </x:c>
+      <x:c r="C458" s="9" t="str">
+        <x:v>2020-2023 | BMW | X4 M</x:v>
+      </x:c>
+      <x:c r="D458" s="9" t="str">
+        <x:v>Rear Differential Mounting Bolt &amp; Bush Failure - F98 X4 M / F98 X4 M</x:v>
+      </x:c>
+      <x:c r="E458" s="9" t="str">
+        <x:v>Replace factory differential bolt, bush, and collar with FJ Motorwerkes uprated diff bolt and collar upgrade kit. The FJ kit uses premium CNC-machined stainless steel components that can handle 170,000 PSI (39% stronger than BMW's revised bolt). Kit price approximately $255 (GBP). Available from FJ Motorwerkes directly, BMG Performance, AM Tuning, and H4ck Performance. Installation is straightforward - rear differential does not need to be fully removed. Budget $400-$600 total including labor. This upgrade is considered MANDATORY by the X3 M/X4 M community for any car making stock or above power. JXB Performance also offers a driveshaft carrier bearing upgrade for cars experiencing propshaft vibration as a companion fix.</x:v>
+      </x:c>
+      <x:c r="F458" s="9" t="str">
+        <x:v>Inspect bolt/mount revision; F97/F98 FJ bolt/collar kit when selected; installation/torque and NVH review</x:v>
+      </x:c>
+      <x:c r="G458" s="9" t="str">
+        <x:v>EXACT DUPLICATE F97/F98 KIT</x:v>
+      </x:c>
+      <x:c r="H458" s="9" t="str">
+        <x:v>FJ X3M/X4M diff bolt and collar kit</x:v>
+      </x:c>
+      <x:c r="I458" s="9" t="str">
+        <x:v>https://bmgperformance.com/products/fj-motorwerkes-x3m-x4m-diff-bolt-and-collar-upgrade</x:v>
+      </x:c>
+      <x:c r="J458" s="9" t="str">
+        <x:v>F98 X4 M explicitly listed; confirm stock/revision and installer requirements</x:v>
+      </x:c>
+      <x:c r="K458" s="9" t="str">
+        <x:v>conditional differential-mount upgrade</x:v>
+      </x:c>
+      <x:c r="L458" s="9" t="str"/>
+      <x:c r="M458" s="9" t="str">
+        <x:v>The live kit explicitly covers F98, but the row duplicates the X3 M content.</x:v>
+      </x:c>
+      <x:c r="N458" s="41" t="str">
+        <x:v>Do not call the kit mandatory or treat seller strength claims as independent validation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="459" ht="1293.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A459" s="40" t="n">
+        <x:v>316</x:v>
+      </x:c>
+      <x:c r="B459" s="9" t="str">
+        <x:v>bmw-x4m-s58-bearing-recall-2020</x:v>
+      </x:c>
+      <x:c r="C459" s="9" t="str">
+        <x:v>2020-2021 | BMW | X4 M | M40i, xDrive35i | S58</x:v>
+      </x:c>
+      <x:c r="D459" s="9" t="str">
+        <x:v>S58 Engine Main Bearing Shell Recall / Stop Sale - F98 X4 M / F98 X4 M</x:v>
+      </x:c>
+      <x:c r="E459" s="9" t="str">
+        <x:v>Check VIN immediately against BMW recall database at bmwusa.com or contact your BMW dealer. If your vehicle is within the affected production date range, BMW will inspect and replace main bearing shells at no cost under the Tech Campaign. The repair requires removing the cylinder head and oil pan to access and replace all main bearing shells - this is a major repair (8-12 hours labor) but fully covered by BMW. Do NOT drive the vehicle if knocking is present. For S58 vehicles outside the recall range: Proactive rod bearing inspection is recommended at 60,000 miles for track-driven vehicles. ACL Race Series rod bearings 6B1510H-STD are the aftermarket upgrade choice on Bimmerpost for preventive replacement ($150-$250 for bearing set, $3,000-$5,000 total with labor).</x:v>
+      </x:c>
+      <x:c r="F459" s="9" t="str">
+        <x:v>VIN campaign check; stop/tow for knocking; covered dealer main-bearing remedy if affected; no unrelated preventive rod-bearing sale</x:v>
+      </x:c>
+      <x:c r="G459" s="9" t="str">
+        <x:v>CAMPAIGN ROUTES ONLY</x:v>
+      </x:c>
+      <x:c r="H459" s="9" t="str">
+        <x:v>BMW recall lookup</x:v>
+      </x:c>
+      <x:c r="I459" s="9" t="str">
+        <x:v>https://www.bmwusa.com/safety-and-emission-recalls.html</x:v>
+      </x:c>
+      <x:c r="J459" s="9" t="str">
+        <x:v>VIN check for S58 main-bearing technical campaign</x:v>
+      </x:c>
+      <x:c r="K459" s="9" t="str">
+        <x:v>manufacturer campaign route</x:v>
+      </x:c>
+      <x:c r="L459" s="9" t="str"/>
+      <x:c r="M459" s="9" t="str">
+        <x:v>Main-bearing campaign work is distinct from aftermarket rod-bearing prevention.</x:v>
+      </x:c>
+      <x:c r="N459" s="41" t="str">
+        <x:v>Fix repeated F98 title, verify recall-versus-campaign terminology, and remove the unrelated ACL recommendation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="460" ht="66" hidden="0" customHeight="1">
+      <x:c r="A460" s="40" t="str"/>
+      <x:c r="B460" s="9" t="str"/>
+      <x:c r="C460" s="9" t="str"/>
+      <x:c r="D460" s="9" t="str"/>
+      <x:c r="E460" s="9" t="str"/>
+      <x:c r="F460" s="9" t="str"/>
+      <x:c r="G460" s="9" t="str"/>
+      <x:c r="H460" s="9" t="str">
+        <x:v>BMW dealer locator</x:v>
+      </x:c>
+      <x:c r="I460" s="9" t="str">
+        <x:v>https://www.bmwusa.com/dealer-locator.html</x:v>
+      </x:c>
+      <x:c r="J460" s="9" t="str">
+        <x:v>campaign eligibility/repair</x:v>
+      </x:c>
+      <x:c r="K460" s="9" t="str">
+        <x:v>authorized service</x:v>
+      </x:c>
+      <x:c r="L460" s="9" t="str"/>
+      <x:c r="M460" s="9" t="str"/>
+      <x:c r="N460" s="41" t="str"/>
+    </x:row>
+    <x:row r="461" ht="1227.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A461" s="40" t="n">
+        <x:v>317</x:v>
+      </x:c>
+      <x:c r="B461" s="9" t="str">
+        <x:v>bmw-x4m-transfer-case-2020</x:v>
+      </x:c>
+      <x:c r="C461" s="9" t="str">
+        <x:v>2020-2023 | BMW | X4 M | S58</x:v>
+      </x:c>
+      <x:c r="D461" s="9" t="str">
+        <x:v>xDrive Transfer Case Stress &amp; Fluid Degradation - F98 X4 M / F98 X4 M</x:v>
+      </x:c>
+      <x:c r="E461" s="9" t="str">
+        <x:v>Change transfer case fluid every 30,000 miles (BMW says "lifetime fill" - this is NOT correct for M vehicles driven hard). Use BMW DTF-1 transfer case fluid or equivalent high-quality synthetic. Check tire tread depth at every service - all 4 tires must be within 2/32" of each other to prevent transfer case stress. Rotate tires every 5,000-7,000 miles. If transfer case actuator motor fails: FCP Euro guide for BMW transfer case actuator repair (part number varies by production date, ~$300-$600). For tuned cars: Consider transfer case brace/reinforcement and shortened fluid change intervals (every 15,000 miles). Complete transfer case replacement if internals are damaged: $3,000-$5,500 at independent specialist, $5,000-$8,000+ at dealer.</x:v>
+      </x:c>
+      <x:c r="F461" s="9" t="str">
+        <x:v>Tire circumference/tread and VTG diagnosis; VIN-specific fluid/service; actuator versus internal failure; initialization</x:v>
+      </x:c>
+      <x:c r="G461" s="9" t="str">
+        <x:v>DUPLICATE / VIN-SPECIFIC DRIVETRAIN GATE</x:v>
+      </x:c>
+      <x:c r="H461" s="9" t="str">
+        <x:v>BMW X4 M transfer-case catalog</x:v>
+      </x:c>
+      <x:c r="I461" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x4_m-transfer_case.html</x:v>
+      </x:c>
+      <x:c r="J461" s="9" t="str">
+        <x:v>2020-2023 F98 X4 M; VIN and production date required</x:v>
+      </x:c>
+      <x:c r="K461" s="9" t="str">
+        <x:v>OEM drivetrain catalog</x:v>
+      </x:c>
+      <x:c r="L461" s="9" t="str"/>
+      <x:c r="M461" s="9" t="str">
+        <x:v>This duplicates the X3 M transfer-case text and contains multiple conditional branches.</x:v>
+      </x:c>
+      <x:c r="N461" s="41" t="str">
+        <x:v>Fix repeated F98 title and remove universal fluid/rotation/brace claims.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="462" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A462" s="40" t="str"/>
+      <x:c r="B462" s="9" t="str"/>
+      <x:c r="C462" s="9" t="str"/>
+      <x:c r="D462" s="9" t="str"/>
+      <x:c r="E462" s="9" t="str"/>
+      <x:c r="F462" s="9" t="str"/>
+      <x:c r="G462" s="9" t="str"/>
+      <x:c r="H462" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I462" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J462" s="9" t="str">
+        <x:v>VTG diagnosis/service/initialization</x:v>
+      </x:c>
+      <x:c r="K462" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L462" s="9" t="str"/>
+      <x:c r="M462" s="9" t="str"/>
+      <x:c r="N462" s="41" t="str"/>
+    </x:row>
+    <x:row r="463" ht="1042.800048828125" hidden="0" customHeight="1">
+      <x:c r="A463" s="40" t="n">
+        <x:v>318</x:v>
+      </x:c>
+      <x:c r="B463" s="9" t="str">
+        <x:v>bmw-x5-air-suspension-2007</x:v>
+      </x:c>
+      <x:c r="C463" s="9" t="str">
+        <x:v>2019-2026 | BMW | X5</x:v>
+      </x:c>
+      <x:c r="D463" s="9" t="str">
+        <x:v>G05 Suspension Warning: Check Faults and Campaigns Before Parts</x:v>
+      </x:c>
+      <x:c r="E463" s="9" t="str">
+        <x:v>Start with the VIN build/options, open-campaign status, exact warning, complete fault memory, and BMW ISTA test plan. If the VIN and production date match a BMW action, follow that bulletin: inspect the specified sensor-link holders, apply the specified software correction, or inspect the affected air line as directed. For other vehicles, test the particular system shown by the VIN and fault path before selecting any component. Do not buy a compressor, strut, spring, or conversion kit until the failed part and its VIN-specific number are established. This article intentionally has no retail link because no single part repairs all of these conditions.</x:v>
+      </x:c>
+      <x:c r="F463" s="9" t="str">
+        <x:v>G05 VIN/options/campaign check; exact warning and ISTA test plan; campaign-specific sensor holder/software/air-line remedy or diagnosed component</x:v>
+      </x:c>
+      <x:c r="G463" s="9" t="str">
+        <x:v>CAMPAIGN / DIAGNOSIS ROUTE; NO RETAIL PART</x:v>
+      </x:c>
+      <x:c r="H463" s="9" t="str">
+        <x:v>BMW recall lookup</x:v>
+      </x:c>
+      <x:c r="I463" s="9" t="str">
+        <x:v>https://www.bmwusa.com/safety-and-emission-recalls.html</x:v>
+      </x:c>
+      <x:c r="J463" s="9" t="str">
+        <x:v>G05 X5 VIN campaign check</x:v>
+      </x:c>
+      <x:c r="K463" s="9" t="str">
+        <x:v>manufacturer campaign route</x:v>
+      </x:c>
+      <x:c r="L463" s="9" t="str"/>
+      <x:c r="M463" s="9" t="str">
+        <x:v>The corrected article intentionally rejects a single compressor/strut/spring/conversion link.</x:v>
+      </x:c>
+      <x:c r="N463" s="41" t="str">
+        <x:v>Correct the issue ID's 2007 mismatch: the row is 2019-2026 G05.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="464" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A464" s="40" t="str"/>
+      <x:c r="B464" s="9" t="str"/>
+      <x:c r="C464" s="9" t="str"/>
+      <x:c r="D464" s="9" t="str"/>
+      <x:c r="E464" s="9" t="str"/>
+      <x:c r="F464" s="9" t="str"/>
+      <x:c r="G464" s="9" t="str"/>
+      <x:c r="H464" s="9" t="str">
+        <x:v>BMW dealer locator</x:v>
+      </x:c>
+      <x:c r="I464" s="9" t="str">
+        <x:v>https://www.bmwusa.com/dealer-locator.html</x:v>
+      </x:c>
+      <x:c r="J464" s="9" t="str">
+        <x:v>ISTA suspension diagnosis and VIN-selected remedy</x:v>
+      </x:c>
+      <x:c r="K464" s="9" t="str">
+        <x:v>authorized service</x:v>
+      </x:c>
+      <x:c r="L464" s="9" t="str"/>
+      <x:c r="M464" s="9" t="str"/>
+      <x:c r="N464" s="41" t="str"/>
+    </x:row>
+    <x:row r="465" ht="1148.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A465" s="40" t="n">
+        <x:v>319</x:v>
+      </x:c>
+      <x:c r="B465" s="9" t="str">
+        <x:v>bmw-x5-air-suspension-compressor-2007</x:v>
+      </x:c>
+      <x:c r="C465" s="9" t="str">
+        <x:v>2007-2013 | BMW | X5 | 3.0si, 4.8i, xDrive30i, xDrive35d, xDrive35i, xDrive48i, xDrive50i, X5 M | N52, N62, M57, N55, N63, S63</x:v>
+      </x:c>
+      <x:c r="D465" s="9" t="str">
+        <x:v>E70 Rear Air-Supply Unit: Diagnose the Self-Leveling System First</x:v>
+      </x:c>
+      <x:c r="E465" s="9" t="str">
+        <x:v>Read the EHC fault memory and run the applicable BMW ISTA test plan before ordering a compressor. Confirm the vehicle is equipped with rear self-leveling suspension, compare left/right ride height, check system power and wiring, inspect the height-sensor links, and leak-test the air springs, lines, and valve system. Test the air supply only after those checks isolate it. If BMW ETK/AIR selects the E70 air-supply system for the VIN and diagnosis confirms that assembly, replace it with current part 37-20-6-859-714, follow the BMW repair procedure, clear faults, and perform the required ride-height calibration. Do not install a generic compressor or a coil-conversion kit from symptoms alone.</x:v>
+      </x:c>
+      <x:c r="F465" s="9" t="str">
+        <x:v>EHC/ISTA diagnosis; confirm rear self-leveling option; leak-test springs/lines/valves; power/sensor checks; air-supply unit only after isolation; calibration</x:v>
+      </x:c>
+      <x:c r="G465" s="9" t="str">
+        <x:v>EXACT CONDITIONAL E70 AIR-SUPPLY UNIT</x:v>
+      </x:c>
+      <x:c r="H465" s="9" t="str">
+        <x:v>Genuine BMW air supply unit 37206859714</x:v>
+      </x:c>
+      <x:c r="I465" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/parts/bmw-rp_air_supply_system-37206859714.html</x:v>
+      </x:c>
+      <x:c r="J465" s="9" t="str">
+        <x:v>2007-2013 E70 X5 with applicable rear self-leveling system; VIN and diagnosis required</x:v>
+      </x:c>
+      <x:c r="K465" s="9" t="str">
+        <x:v>conditional air-supply/compressor assembly</x:v>
+      </x:c>
+      <x:c r="L465" s="9" t="str"/>
+      <x:c r="M465" s="9" t="str">
+        <x:v>The live OEM page explicitly lists E70 X5 fitment and superseded numbers.</x:v>
+      </x:c>
+      <x:c r="N465" s="41" t="str">
+        <x:v>Do not order from sagging alone; leak/sensor/power faults can mimic a failed compressor.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="466" ht="1227.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A466" s="40" t="n">
+        <x:v>320</x:v>
+      </x:c>
+      <x:c r="B466" s="9" t="str">
+        <x:v>bmw-x5-carbon-buildup-2007</x:v>
+      </x:c>
+      <x:c r="C466" s="9" t="str">
+        <x:v>2011-2018 | BMW | X5 | xDrive35i, xDrive50i | N55, N63, N63TU1</x:v>
+      </x:c>
+      <x:c r="D466" s="9" t="str">
+        <x:v>Possible Intake-Valve Deposits on Direct-Injected Gasoline Engines</x:v>
+      </x:c>
+      <x:c r="E466" s="9" t="str">
+        <x:v>Diagnose the actual symptom before authorizing cleaning: read BMW-specific faults and misfire counters, check ignition and fueling, smoke-test the intake where indicated, verify crankcase ventilation operation, and inspect the intake valves with a borescope or by removing the intake manifold when the test plan supports it. If substantial deposits are confirmed and match the complaint, use an engine-specific professional mechanical-cleaning procedure that protects closed valves and removes all blasting media before reassembly. Do not present a universal catch can, chemical spray, fuel brand, short oil interval, or high-RPM driving as a proven repair. Any crankcase-ventilation modification also requires engine-specific fitment and emissions-law review.</x:v>
+      </x:c>
+      <x:c r="F466" s="9" t="str">
+        <x:v>Engine-specific fault/misfire/ignition/fueling/PCV diagnosis; borescope/manifold inspection; professional mechanical cleaning only for confirmed deposits</x:v>
+      </x:c>
+      <x:c r="G466" s="9" t="str">
+        <x:v>SERVICE ROUTE; UNIVERSAL PRODUCTS REJECTED</x:v>
+      </x:c>
+      <x:c r="H466" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I466" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J466" s="9" t="str">
+        <x:v>2011-2018 direct-injected gasoline X5 engine-specific deposit diagnosis/cleaning</x:v>
+      </x:c>
+      <x:c r="K466" s="9" t="str">
+        <x:v>specialist service</x:v>
+      </x:c>
+      <x:c r="L466" s="9" t="str"/>
+      <x:c r="M466" s="9" t="str">
+        <x:v>The corrected source rejects universal catch cans, sprays, fuel, and intervals.</x:v>
+      </x:c>
+      <x:c r="N466" s="41" t="str">
+        <x:v>Correct the issue ID's 2007 mismatch and identify the exact engine before authorizing cleaning.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="467" ht="884.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A467" s="40" t="n">
+        <x:v>321</x:v>
+      </x:c>
+      <x:c r="B467" s="9" t="str">
+        <x:v>bmw-x5-coolant-pipe-leak-2007</x:v>
+      </x:c>
+      <x:c r="C467" s="9" t="str">
+        <x:v>2007-2010 | BMW | X5 | 4.8i, xDrive48i | N62, N62TU</x:v>
+      </x:c>
+      <x:c r="D467" s="9" t="str">
+        <x:v>E70 N62 Coolant Transfer Pipe Leak (Pressure-Test First)</x:v>
+      </x:c>
+      <x:c r="E467" s="9" t="str">
+        <x:v>Pressure-test the cooling system cold and inspect the engine valley and all accessible connections to identify the exact leak before ordering parts. If inspection confirms the N62 transfer pipe and BMW ETK/AIR selects it for the VIN, replace pipe 11-14-1-439-975 with the required seals and one-time-use hardware from the VIN-specific repair diagram. Refill and bleed the cooling system with the specified coolant, repeat the pressure test, and verify stable temperature. Do not automatically replace an N63 pipe, thermostat, or unrelated hoses from this article.</x:v>
+      </x:c>
+      <x:c r="F467" s="9" t="str">
+        <x:v>Cold pressure test; confirmed E70 N62 valley transfer pipe; BMW pipe 11141439975 with VIN-specific seals/hardware; correct coolant/bleed/retest</x:v>
+      </x:c>
+      <x:c r="G467" s="9" t="str">
+        <x:v>EXACT CONDITIONAL N62 PIPE</x:v>
+      </x:c>
+      <x:c r="H467" s="9" t="str">
+        <x:v>Genuine BMW coolant transfer pipe 11141439975</x:v>
+      </x:c>
+      <x:c r="I467" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/parts/bmw-coolant_pipe-11141439975.html</x:v>
+      </x:c>
+      <x:c r="J467" s="9" t="str">
+        <x:v>2007-2010 E70 X5 N62 where VIN-matched; seals/hardware from VIN diagram</x:v>
+      </x:c>
+      <x:c r="K467" s="9" t="str">
+        <x:v>conditional OEM transfer pipe</x:v>
+      </x:c>
+      <x:c r="L467" s="9" t="str"/>
+      <x:c r="M467" s="9" t="str">
+        <x:v>The corrected How to Fix provides the exact N62 pipe number and rejects unrelated N63/thermostat/hoses.</x:v>
+      </x:c>
+      <x:c r="N467" s="41" t="str">
+        <x:v>Approve only after the valley leak is pressure-test confirmed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="468" ht="1082.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A468" s="40" t="n">
+        <x:v>322</x:v>
+      </x:c>
+      <x:c r="B468" s="9" t="str">
+        <x:v>bmw-x5-n63-timing-chain-2008</x:v>
+      </x:c>
+      <x:c r="C468" s="9" t="str">
+        <x:v>2010-2013 | BMW | X5 | xDrive50i | N63</x:v>
+      </x:c>
+      <x:c r="D468" s="9" t="str">
+        <x:v>Early N63 Timing-Chain Wear Check: ISTA Test Before Repair</x:v>
+      </x:c>
+      <x:c r="E468" s="9" t="str">
+        <x:v>Check the VIN and service history with a BMW center, diagnose stored VANOS/camshaft faults first, and run BMW's ISTA timing-chain elongation test. If the result is 'Timing chain is OK,' do not replace parts on this claim. If it is 'not OK,' BMW SIB 11 16 14 directs replacement of both timing chains under the VIN-specific repair instruction, followed by the required oil/filter service, priming steps, programming, and shorter oil-service interval. A single tensioner 11-31-7-557-741 or a generic Cloyes kit is not the complete repair and must not be presented as what the owner needs. Tow the vehicle rather than driving it when severe mechanical noise, oil-pressure warnings, or loss of timing is present.</x:v>
+      </x:c>
+      <x:c r="F468" s="9" t="str">
+        <x:v>VIN/service history and DME diagnosis; ISTA elongation test; both timing chains only if test fails; complete SIB procedure including oil/filter/programming</x:v>
+      </x:c>
+      <x:c r="G468" s="9" t="str">
+        <x:v>BMW SIB / ISTA SERVICE ROUTE; NO GENERIC KIT</x:v>
+      </x:c>
+      <x:c r="H468" s="9" t="str">
+        <x:v>BMW dealer locator</x:v>
+      </x:c>
+      <x:c r="I468" s="9" t="str">
+        <x:v>https://www.bmwusa.com/dealer-locator.html</x:v>
+      </x:c>
+      <x:c r="J468" s="9" t="str">
+        <x:v>2010-2013 E70 X5 N63 SIB 11 16 14 timing test/repair</x:v>
+      </x:c>
+      <x:c r="K468" s="9" t="str">
+        <x:v>BMW test-plan and complete repair</x:v>
+      </x:c>
+      <x:c r="L468" s="9" t="str"/>
+      <x:c r="M468" s="9" t="str">
+        <x:v>The corrected source explicitly rejects a single tensioner and generic Cloyes kit as incomplete.</x:v>
+      </x:c>
+      <x:c r="N468" s="41" t="str">
+        <x:v>Correct the issue ID's 2008 mismatch; do not sell parts when ISTA says the chain is OK.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="469" ht="1227.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A469" s="40" t="n">
+        <x:v>323</x:v>
+      </x:c>
+      <x:c r="B469" s="9" t="str">
+        <x:v>bmw-x5-n63-wastegate-2008</x:v>
+      </x:c>
+      <x:c r="C469" s="9" t="str">
+        <x:v>2010-2018 | BMW | X5 | xDrive50i | N63, N63TU</x:v>
+      </x:c>
+      <x:c r="D469" s="9" t="str">
+        <x:v>N63/N63TU Low Boost or Turbo Rattle: Diagnose Vacuum Control First</x:v>
+      </x:c>
+      <x:c r="E469" s="9" t="str">
+        <x:v>Read all DME faults and compare requested versus actual boost under the BMW test plan. Pressure- or smoke-test the intake and charge-air path, verify vacuum supply from the pump and reservoir, inspect both banks' hoses and pressure converters, and test actuator movement before condemning a turbocharger. Identify the engine generation, failed bank, and exact hardware in BMW ETK/AIR. Check a 2010-2013 E70 VIN for the N63 Customer Care Package only as applicable; its published six-point scope includes air-mass sensors, injectors, vacuum pump, low-pressure fuel sensor/feed line, fresh-air turbo seals, and crankcase-ventilation lines, not an automatic wastegate replacement. No retail link is published until diagnosis selects a VIN-specific component.</x:v>
+      </x:c>
+      <x:c r="F469" s="9" t="str">
+        <x:v>DME boost data; charge-air smoke test; vacuum pump/reservoir/hoses/converters; actuator movement; engine generation/bank/VIN component only after diagnosis</x:v>
+      </x:c>
+      <x:c r="G469" s="9" t="str">
+        <x:v>DIAGNOSIS ROUTE; NO RETAIL PART</x:v>
+      </x:c>
+      <x:c r="H469" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I469" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J469" s="9" t="str">
+        <x:v>2010-2018 X5 N63/N63TU vacuum/boost/turbo diagnosis</x:v>
+      </x:c>
+      <x:c r="K469" s="9" t="str">
+        <x:v>specialist service</x:v>
+      </x:c>
+      <x:c r="L469" s="9" t="str"/>
+      <x:c r="M469" s="9" t="str">
+        <x:v>The corrected source requires vacuum and charge-air diagnosis and says the care package was not an automatic wastegate replacement.</x:v>
+      </x:c>
+      <x:c r="N469" s="41" t="str">
+        <x:v>Correct the issue ID's 2008 mismatch and hold all turbos/actuators until bank and root cause are identified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="470" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A470" s="40" t="str"/>
+      <x:c r="B470" s="9" t="str"/>
+      <x:c r="C470" s="9" t="str"/>
+      <x:c r="D470" s="9" t="str"/>
+      <x:c r="E470" s="9" t="str"/>
+      <x:c r="F470" s="9" t="str"/>
+      <x:c r="G470" s="9" t="str"/>
+      <x:c r="H470" s="9" t="str">
+        <x:v>BMW dealer locator</x:v>
+      </x:c>
+      <x:c r="I470" s="9" t="str">
+        <x:v>https://www.bmwusa.com/dealer-locator.html</x:v>
+      </x:c>
+      <x:c r="J470" s="9" t="str">
+        <x:v>2010-2013 E70 Customer Care Package history where applicable</x:v>
+      </x:c>
+      <x:c r="K470" s="9" t="str">
+        <x:v>VIN history/service</x:v>
+      </x:c>
+      <x:c r="L470" s="9" t="str"/>
+      <x:c r="M470" s="9" t="str"/>
+      <x:c r="N470" s="41" t="str"/>
+    </x:row>
+    <x:row r="471" ht="844.7999877929688" hidden="0" customHeight="1">
+      <x:c r="A471" s="40" t="n">
+        <x:v>324</x:v>
+      </x:c>
+      <x:c r="B471" s="9" t="str">
+        <x:v>bmw-x5-oil-leaks-2000</x:v>
+      </x:c>
+      <x:c r="C471" s="9" t="str">
+        <x:v>2003-2006 | BMW | X5 | 3.0i | M54</x:v>
+      </x:c>
+      <x:c r="D471" s="9" t="str">
+        <x:v>E53 3.0i M54 Valve-Cover Gasket Leak (Confirm the Source)</x:v>
+      </x:c>
+      <x:c r="E471" s="9" t="str">
+        <x:v>Clean the engine and trace the highest fresh-oil source before ordering a gasket. If the leak is at the M54 cylinder-head-cover perimeter or spark-plug-well seals, inspect the plastic cover for cracks, warpage, damaged fastener grommets, and crankcase-ventilation faults. Reuse the cover only if it passes inspection, then install VIN/production-confirmed gasket set 11-12-0-030-496 with the BMW-specified grommets and sealant locations and torque sequence. If the cover or another oil circuit is the source, select that separate repair instead.</x:v>
+      </x:c>
+      <x:c r="F471" s="9" t="str">
+        <x:v>Clean/trace highest leak source; M54 cover gasket set 11120030496 only for perimeter/wells; inspect cover, grommets, and CCV; separate other oil circuits</x:v>
+      </x:c>
+      <x:c r="G471" s="9" t="str">
+        <x:v>EXACT CONDITIONAL M54 GASKET SET</x:v>
+      </x:c>
+      <x:c r="H471" s="9" t="str">
+        <x:v>Genuine BMW valve-cover gasket set 11120030496</x:v>
+      </x:c>
+      <x:c r="I471" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/products/bmw-valve-cover-gasket-set-11120030496</x:v>
+      </x:c>
+      <x:c r="J471" s="9" t="str">
+        <x:v>2003-2006 E53 X5 3.0i M54 where cataloged; verify VIN and cover condition</x:v>
+      </x:c>
+      <x:c r="K471" s="9" t="str">
+        <x:v>conditional gasket set</x:v>
+      </x:c>
+      <x:c r="L471" s="9" t="str"/>
+      <x:c r="M471" s="9" t="str">
+        <x:v>The corrected source narrows the issue to E53 M54 and supplies the exact gasket-set number.</x:v>
+      </x:c>
+      <x:c r="N471" s="41" t="str">
+        <x:v>Correct the issue ID's 2000 mismatch; reuse the cover only if it passes inspection.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="472" ht="1293.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A472" s="42" t="n">
+        <x:v>325</x:v>
+      </x:c>
+      <x:c r="B472" s="43" t="str">
+        <x:v>bmw-x5-transfer-case-actuator-2000</x:v>
+      </x:c>
+      <x:c r="C472" s="43" t="str">
+        <x:v>2007-2013 | BMW | X5 | 3.0si, 4.8i, xDrive30i, xDrive35d, xDrive48i, X5 M | N52, N62, M57, S63</x:v>
+      </x:c>
+      <x:c r="D472" s="43" t="str">
+        <x:v>E70 ATC700 Transfer-Case Positioning Motor (Diagnosis Required)</x:v>
+      </x:c>
+      <x:c r="E472" s="43" t="str">
+        <x:v>Read BMW VTG/DSC faults and run the applicable ISTA transfer-case test plan before buying a motor. Confirm tire sizes and wear, battery voltage, wiring, transfer-case type, fluid condition, calibration, and—especially after differential or transfer-case replacement—the VIN-correct front and rear gear ratios. If testing confirms the ATC700 positioning motor and BMW ETK/AIR selects this application for the VIN, current BMW exchange servomotor 27-10-2-449-709 supersedes 27-10-7-568-267. Install the correct classification resistor/hardware supplied or specified for the VIN and perform the required VTG initialization/calibration. A generic gear-only kit is not a universal BMW repair and should not be ordered without opening and confirming the exact motor failure.</x:v>
+      </x:c>
+      <x:c r="F472" s="43" t="str">
+        <x:v>VTG/DSC ISTA diagnosis; tires/voltage/wiring/unit/fluid/ratios; confirmed ATC700 exchange servomotor 27102449709; resistor/hardware; initialization</x:v>
+      </x:c>
+      <x:c r="G472" s="43" t="str">
+        <x:v>EXACT CONDITIONAL ATC700 SERVOMOTOR</x:v>
+      </x:c>
+      <x:c r="H472" s="43" t="str">
+        <x:v>Genuine BMW exchange servomotor 27102449709</x:v>
+      </x:c>
+      <x:c r="I472" s="43" t="str">
+        <x:v>https://www.bmwpartsdeal.com/parts/bmw-rp_actuator-27102449709.html</x:v>
+      </x:c>
+      <x:c r="J472" s="43" t="str">
+        <x:v>2007-2013 E70 X5 ATC700 where VIN/ETK selects it; verify classification resistor/hardware</x:v>
+      </x:c>
+      <x:c r="K472" s="43" t="str">
+        <x:v>conditional transfer-case positioning motor</x:v>
+      </x:c>
+      <x:c r="L472" s="43" t="str"/>
+      <x:c r="M472" s="43" t="str">
+        <x:v>The corrected source supplies the current superseding motor and requires ATC700/VIN confirmation.</x:v>
+      </x:c>
+      <x:c r="N472" s="44" t="str">
+        <x:v>Correct the issue ID's 2000 mismatch and reject generic gear-only kits without opening/confirming the motor fault.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -16618,90 +17980,90 @@
         <x:v>Queue status</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="1016.4000244140625" hidden="0" customHeight="1">
+    <x:row r="2" ht="1042.800048828125" hidden="0" customHeight="1">
       <x:c r="A2" s="40" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>bmw-x3-wastegate-rattle-2011</x:v>
+        <x:v>bmw-x5-transfer-case-actuator-2007</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>2011-2023 | BMW | X3 | M40i, M50, sDrive30i, xDrive28i, xDrive30i, xDrive35i</x:v>
+        <x:v>2019-2026 | BMW | X5</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
-        <x:v>Turbocharger Wastegate Rattle (N55, N20, B58 Engines)</x:v>
+        <x:v>G05/F95 Transfer-Case Shudder: Tires and Fluid Diagnosis First</x:v>
       </x:c>
       <x:c r="E2" s="9" t="str">
-        <x:v>Replace wastegate actuator ($400-800) or use aftermarket wastegate repair kit with upgraded stainless steel bushings ($150-300). Some cases require complete turbocharger replacement ($2,000-$4,000). VTT (Vargas Turbo Technologies) repair kits popular on forums - upgraded materials prevent future rattle. MONITORING: Early wastegate rattle may be harmless (annoying but no performance loss). If car boosts normally and no underboost codes, can monitor rattle without urgent repair. However, if check engine light appears with code 30FF or boost pressure drops, repair immediately to prevent turbo damage.</x:v>
+        <x:v>Follow BMW SIB 27 02 20 in order: verify all four tires for VIN-correct size, brand/application, axle placement, and wear; diagnose any powertrain faults; then use ISTA to temporarily deactivate the transfer-case clutch and road-test the complaint. Only if the shudder disappears with the VTG deactivated does BMW direct an ATX13-X oil change with DTF-1, followed by VTG calibration. The clutch plates can require up to 125 miles after the service to become fully saturated and smooth out. If the symptom remains, continue diagnosis rather than buying an actuator or transfer case. Part numbers for any further repair must be selected by VIN in ETK/AIR.</x:v>
       </x:c>
       <x:c r="F2" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G2" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="778.7999877929688" hidden="0" customHeight="1">
+    <x:row r="3" ht="1214.4000244140625" hidden="0" customHeight="1">
       <x:c r="A3" s="40" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>bmw-x3-water-pump-2007</x:v>
+        <x:v>bmw-x5-vanos-solenoid-2000</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
-        <x:v>2007-2017 | BMW | X3 | sDrive30i, xDrive28i, xDrive30i | N52, N20</x:v>
+        <x:v>2010-2013 | BMW | X5 | xDrive30i, xDrive35i | N51, N52K, N52T, N55</x:v>
       </x:c>
       <x:c r="D3" s="9" t="str">
-        <x:v>Electric Water Pump Failure (N52, N20 Engines)</x:v>
+        <x:v>VANOS Adjustment-Unit Bolt Recall 23V-707 (E70 Inline-Six)</x:v>
       </x:c>
       <x:c r="E3" s="9" t="str">
-        <x:v>Replace electric water pump at first sign of failure ($800 parts + labor). Consider preventative replacement at 70-80k miles to avoid being stranded ($400 parts, DIY-able). CRITICAL: If you own 2013-2017 X3 28i, verify recall repair (protective shield installation) has been completed to prevent fire risk - check with BMW dealer using VIN. If engine overheats, PULL OVER IMMEDIATELY and shut off - driving with overheating warps cylinder heads ($4,000+ repair). Call tow truck.</x:v>
+        <x:v>Enter the VIN in BMW's official recall lookup and have an authorized BMW center complete recall 23V-707 if it is open. BMW's procedure is inspection-dependent: intact affected bolts are replaced; if bolts are loose or broken, the affected VANOS adjustment unit is replaced, and missing fragments must be recovered. The recall repair is free, so do not buy a solenoid or VANOS part first. If the VIN is outside the recall or a fault remains after the remedy, use BMW-capable diagnostics to test oil supply and pressure, wiring, sensors, control solenoids, adjustment units, and mechanical timing before selecting a part. If the engine runs roughly, makes unusual mechanical noise, loses power, or stalls, move out of traffic safely, stop driving, and contact BMW for transport guidance.</x:v>
       </x:c>
       <x:c r="F3" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G3" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="1240.800048828125" hidden="0" customHeight="1">
+    <x:row r="4" ht="1148.4000244140625" hidden="0" customHeight="1">
       <x:c r="A4" s="40" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>bmw-x3m-brake-wear-2020</x:v>
+        <x:v>bmw-x5-water-pump-2007</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>2020-2023 | BMW | X3 M | S58</x:v>
+        <x:v>2011-2013 | BMW | X5 | xDrive35i | N55</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
-        <x:v>Accelerated Brake Pad &amp; Rotor Wear from Vehicle Weight - F97 X3 M / F98 X4 M</x:v>
+        <x:v>E70 xDrive35i N55 Electric Coolant Pump (Fault-Confirmed)</x:v>
       </x:c>
       <x:c r="E4" s="9" t="str">
-        <x:v>Front brake replacement: OEM front rotor (34118054825 left, matching right) with OEM M compound pads. Complete OEM front brake kit available from BimmerWorld (34108064561K1, ~$800-$1,000). Rear brake kit similarly priced. For track use: Upgrade to Brembo GT brake pad set (BM8 compound) for improved heat resistance and longer pad life. EBC Yellowstuff or Hawk HPS 5.0 pads are popular street/track compromise choices ($150-$250 per axle). StopTech slotted rotors offer improved heat dissipation. For dedicated track cars: Brembo GT big brake kit with 412x38mm discs available ($4,000-$6,000 installed). Budget $2,000-$3,000 per year for brake maintenance if driving spiritedly. Use high-temperature brake fluid (Motul RBF 660 or ATE Typ 200) and flush every 12 months.</x:v>
+        <x:v>If the engine-temperature warning appears, stop safely, shut the engine off, and tow the vehicle if normal temperature cannot be confirmed. When cool, check coolant level and leaks, read BMW-specific faults, verify pump power/ground and communication, and run the ISTA coolant-pump activation/test plan. If those tests confirm the pump and BMW ETK/AIR selects 11-51-5-A05-704 for the VIN, replace it using the BMW procedure, select the thermostat separately only if testing or preventive planning justifies it, vacuum-fill or bleed the system as specified, and verify commanded pump operation and stable temperature. Do not use a fixed-mileage rule or this part number for an N52, N63, or F15 without VIN confirmation.</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G4" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="1188" hidden="0" customHeight="1">
+    <x:row r="5" ht="1056" hidden="0" customHeight="1">
       <x:c r="A5" s="40" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>bmw-x3m-cooling-track-use-2020</x:v>
+        <x:v>bmw-x5m-brake-system-2010</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>2020-2023 | BMW | X3 M | S58</x:v>
+        <x:v>2010-2023 | BMW | X5 M</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Cooling System Heat Soak During Track/Spirited Driving - F97 X3 M / F98 X4 M</x:v>
+        <x:v>Heavy-Duty Brake System Accelerated Wear - E70/F85/F95 X5 M</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>For track use: Upgrade intercooler to do88 front-mount intercooler ($1,200-$1,800) - the community standard for S58 heat management. Add CSF high-performance radiator ($600-$900) for sustained track work. Dinan or VRSF also offer intercooler upgrades in the $1,000-$1,500 range. For street/canyon driving: Stock cooling is adequate but ensure coolant flush every 2 years/30,000 miles and inspect expansion tank for cracks. Replace coolant expansion tank preemptively at 60,000 miles if car is driven hard. For all X3 M/X4 M: Use BMW coolant only (mixed 50/50 with distilled water), replace thermostat at 80,000 miles preventatively, inspect all coolant hoses for bulging or softening at every oil change.</x:v>
+        <x:v>E70 X5 M brakes: OEM front pads 34116799964 ($150-$250), rear pads 34216794879 ($120-$200). F85 X5 M front brake rotors: 34112284101/34112284102 with 6-pot caliper 34117845747/34117845748 and pads 34112284869. F85 rear: 385mm x 24mm perforated rotors 34212284903/34212284904 with 4-pot Brembo caliper and Textar pads. Budget $1,500-$2,500 per axle for complete brake service. For track use: EBC Yellowstuff or Hawk HPS 5.0 pads ($200-$350 per axle) with StopTech slotted rotors for improved heat management. Use Motul RBF 660 or ATE Typ 200 brake fluid - flush every 12 months. Budget $3,000-$5,000 per year for brake maintenance if driving spiritedly.</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
         <x:v>0</x:v>
@@ -16710,21 +18072,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="1214.4000244140625" hidden="0" customHeight="1">
+    <x:row r="6" ht="1122" hidden="0" customHeight="1">
       <x:c r="A6" s="40" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>bmw-x3m-differential-bolt-2020</x:v>
+        <x:v>bmw-x5m-rear-differential-2010</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
-        <x:v>2020-2023 | BMW | X3 M | S58</x:v>
+        <x:v>2010-2023 | BMW | X5 M | S63</x:v>
       </x:c>
       <x:c r="D6" s="9" t="str">
-        <x:v>Rear Differential Mounting Bolt &amp; Bush Failure - F97 X3 M / F98 X4 M</x:v>
+        <x:v>Rear Differential Wear &amp; Fluid Degradation - E70/F85/F95 X5 M</x:v>
       </x:c>
       <x:c r="E6" s="9" t="str">
-        <x:v>Replace factory differential bolt, bush, and collar with FJ Motorwerkes uprated diff bolt and collar upgrade kit. The FJ kit uses premium CNC-machined stainless steel components that can handle 170,000 PSI (39% stronger than BMW's revised bolt). Kit price approximately $255 (GBP). Available from FJ Motorwerkes directly, BMG Performance, AM Tuning, and H4ck Performance. Installation is straightforward - rear differential does not need to be fully removed. Budget $400-$600 total including labor. This upgrade is considered MANDATORY by the X3 M/X4 M community for any car making stock or above power. JXB Performance also offers a driveshaft carrier bearing upgrade for cars experiencing propshaft vibration as a companion fix.</x:v>
+        <x:v>Change rear differential fluid every 30,000 miles (ignore BMW "lifetime fill" claim). E70 X5 M: No drain plug - fluid must be extracted through fill port with hand pump or suction device. Recommended fluid: Royal Purple 75W-140 GL5 synthetic or Red Line 75W-140 GL5 ($40-$60 per fill). Capacity approximately 1.2 liters. For limited-slip diff, ensure fluid is GL5 rated with limited-slip additive. If differential is making whining/howling noise: have a limited-slip differential specialist inspect internals (not generic BMW shop). Diff rebuild: $1,500-$3,000 at specialist. Complete differential replacement: $3,000-$5,500 + labor. Labor for fluid change: $150-$300 at independent shop.</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
         <x:v>0</x:v>
@@ -16733,21 +18095,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="1293.5999755859375" hidden="0" customHeight="1">
+    <x:row r="7" ht="1386" hidden="0" customHeight="1">
       <x:c r="A7" s="40" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>bmw-x3m-s58-bearing-recall-2020</x:v>
+        <x:v>bmw-x5m-s63-cooling-system-2010</x:v>
       </x:c>
       <x:c r="C7" s="9" t="str">
-        <x:v>2020-2021 | BMW | X3 M</x:v>
+        <x:v>2010-2023 | BMW | X5 M | 4.4i, 4.6is, 4.8is, M50i, M60i, xDrive48i, xDrive50e, xDrive50i | S63</x:v>
       </x:c>
       <x:c r="D7" s="9" t="str">
-        <x:v>S58 Engine Main Bearing Shell Recall / Stop Sale - F97 X3 M / F98 X4 M</x:v>
+        <x:v>S63 Cooling System Component Failures - E70/F85/F95 X5 M</x:v>
       </x:c>
       <x:c r="E7" s="9" t="str">
-        <x:v>Check VIN immediately against BMW recall database at bmwusa.com or contact your BMW dealer. If your vehicle is within the affected production date range, BMW will inspect and replace main bearing shells at no cost under the Tech Campaign. The repair requires removing the cylinder head and oil pan to access and replace all main bearing shells - this is a major repair (8-12 hours labor) but fully covered by BMW. Do NOT drive the vehicle if knocking is present. For S58 vehicles outside the recall range: Proactive rod bearing inspection is recommended at 60,000 miles for track-driven vehicles. ACL Race Series rod bearings 6B1510H-STD are the aftermarket upgrade choice on Bimmerpost for preventive replacement ($150-$250 for bearing set, $3,000-$5,000 total with labor).</x:v>
+        <x:v>PROACTIVE MAINTENANCE SCHEDULE: Replace electric water pump at 60,000 miles ($400-$700 + labor). Replace thermostat at same time ($150-$250). Replace expansion tank at 60,000-80,000 miles ($100-$200). Inspect all coolant hoses at every oil change - replace any that are soft, bulging, or showing surface cracks. E70 X5 M expansion tank vent hose: 17128627119 ($30-$50). Flush coolant system every 2 years or 30,000 miles (more frequent than BMW's 4-year recommendation). Use ONLY BMW coolant mixed 50/50 with distilled water. For E70 hot-V turbo coolant lines: GRYPHONTEK repair kit eliminates plastic T-fitting failure (see separate issue entry). Budget $1,500-$2,500 for complete cooling system refresh at 60,000 miles. This prevents catastrophic overheating that can destroy the S63 engine ($15,000-$34,000 engine replacement).</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
         <x:v>0</x:v>
@@ -16756,21 +18118,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="1227.5999755859375" hidden="0" customHeight="1">
+    <x:row r="8" ht="1135.199951171875" hidden="0" customHeight="1">
       <x:c r="A8" s="40" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>bmw-x3m-transfer-case-2020</x:v>
+        <x:v>bmw-x5m-s63-oil-leaks-2010</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
-        <x:v>2020-2023 | BMW | X3 M | S58</x:v>
+        <x:v>2010-2023 | BMW | X5 M | 4.4i, 4.6is, 4.8is, M50i, M60i, xDrive48i, xDrive50e, xDrive50i | S63</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
-        <x:v>xDrive Transfer Case Stress &amp; Fluid Degradation - F97 X3 M / F98 X4 M</x:v>
+        <x:v>S63 V8 Chronic Oil Leaks (Valve Cover, Oil Pan, Turbo Lines) - E70/F85/F95 X5 M</x:v>
       </x:c>
       <x:c r="E8" s="9" t="str">
-        <x:v>Change transfer case fluid every 30,000 miles (BMW says "lifetime fill" - this is NOT correct for M vehicles driven hard). Use BMW DTF-1 transfer case fluid or equivalent high-quality synthetic. Check tire tread depth at every service - all 4 tires must be within 2/32" of each other to prevent transfer case stress. Rotate tires every 5,000-7,000 miles. If transfer case actuator motor fails: FCP Euro guide for BMW transfer case actuator repair (part number varies by production date, ~$300-$600). For tuned cars: Consider transfer case brace/reinforcement and shortened fluid change intervals (every 15,000 miles). Complete transfer case replacement if internals are damaged: $3,000-$5,500 at independent specialist, $5,000-$8,000+ at dealer.</x:v>
+        <x:v>Valve cover gasket replacement (both sides): $1,200-$2,500 with labor. BMW plastic valve covers can crack and must be replaced entirely (not just gasket) - inspect during service. Oil filter housing gasket: $400-$800 with labor. Oil pan gasket: $2,000-$3,500 (requires engine/subframe drop). Turbo oil feed/return lines: replace with GRYPHONTEK or MAMBA upgraded silicone/braided lines during any turbo service ($200-$400). VANOS solenoid seals: $100-$200 (DIY-friendly). For comprehensive oil leak repair at 80,000+ miles: budget $3,000-$5,000 to address all common leak points simultaneously. Valve cover bolt torque is CRITICAL - too tight cracks the cover ($800-$1,200 per cover), too loose and it leaks.</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
         <x:v>0</x:v>
@@ -16779,21 +18141,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="673.2000122070312" hidden="0" customHeight="1">
+    <x:row r="9" ht="1412.4000244140625" hidden="0" customHeight="1">
       <x:c r="A9" s="40" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>bmw-x4-n20-timing-chain-2015</x:v>
+        <x:v>bmw-x5m-s63-rod-bearing-2010</x:v>
       </x:c>
       <x:c r="C9" s="9" t="str">
-        <x:v>2015-2016 | BMW | X4 | xDrive28i, xDrive30i</x:v>
+        <x:v>2010-2018 | BMW | X5 M | 4.4i, 4.6is, 4.8is, M50i, M60i, xDrive48i, xDrive50e, xDrive50i</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str">
-        <x:v>N20 Timing Chain Premature Failure - F26 X4 xDrive28i</x:v>
+        <x:v>S63 V8 Rod Bearing Premature Wear &amp; Failure - E70/F85 X5 M</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
-        <x:v>Complete timing chain kit replacement including chain, guides, tensioner, and sprockets. Must be performed by experienced BMW technician. Preventive replacement recommended at 60,000-80,000 miles. BMW extended warranty to 8 years/100,000 miles under class action settlement. Upgraded reinforced chain kit available from aftermarket. Labor is 10-14 hours for X4 due to AWD and tight engine bay.</x:v>
+        <x:v>PREVENTIVE: For track-driven X5 M, replace rod bearings proactively at 60,000-80,000 miles. ACL Race Series rod bearings (8B1578HX-STD for S63B44, +0.001" extra oil clearance) are the community gold standard ($200-$350 for bearing set). WPC surface-treated bearings from Lang Racing are the premium choice ($400-$600 set). Total cost for preventive rod bearing service: $4,500-$8,500 depending on shop. Oil analysis every 5,000 miles through Blackstone Labs ($30/test) to monitor bearing wear metals (lead and copper). Use only BMW 10W-60 synthetic oil with 5,000-7,500 mile oil change intervals. Never track the car on cold oil. Mporium BMW offers specialized S63 rod bearing service starting at $4,499. If catastrophic failure: rebuilt S63 engine from RK Autowerks (~$8,500 + installation), new BMW engine (~$34,000), or complete engine rebuild ($12,000-$18,000).</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
         <x:v>0</x:v>
@@ -16802,21 +18164,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="686.4000244140625" hidden="0" customHeight="1">
+    <x:row r="10" ht="1214.4000244140625" hidden="0" customHeight="1">
       <x:c r="A10" s="40" t="n">
         <x:v>9</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>bmw-x4-n20-timing-chain-guide-2015</x:v>
+        <x:v>bmw-x5m-s63-turbo-coolant-line-2010</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
-        <x:v>2015-2015 | BMW | X4 | N20</x:v>
+        <x:v>2010-2013 | BMW | X5 M</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
-        <x:v>2015 X4 N20 Lower-Engine Whine Requires Timing-Chain Diagnosis</x:v>
+        <x:v>S63 Turbo Coolant Line Plastic T-Fitting Failure (Hot-V Design) - E70 X5 M</x:v>
       </x:c>
       <x:c r="E10" s="9" t="str">
-        <x:v>Confirm the exact xDrive28i variant, N20 engine, production date and VIN eligibility, then have a BMW-qualified technician reproduce the noise and follow current BMW diagnosis before replacing anything. The historical seven-year/70,000-mile coverage was a limited warranty extension, not a recall, and is not a current coverage promise. ShowMeTheParts established category-level fitment only, so no commerce link is approved.</x:v>
+        <x:v>Replace ALL factory plastic turbo coolant T-fittings and hoses with GRYPHONTEK S63 Turbo Coolant Line Repair Kit ($200-$400). Kit includes pre-shaped multi-layer reinforced silicone hoses, brass T-fittings (replacing factory plastic), and all necessary hose clamps. Direct bolt-on installation designed for the E70/E71 S63 engine bay. MAMBA Turbo also offers a reinforced turbo coolant line kit with brass and silicone components ($150-$350). This is a PROACTIVE replacement - do not wait for failure. Replace at first sign of coolant weeping or during any turbo service. Labor: $800-$1,500 due to tight access in hot-V engine valley. If turbo bearings are damaged from overheating: turbo replacement $3,000-$5,000 per unit.</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
         <x:v>0</x:v>
@@ -16825,21 +18187,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="554.4000244140625" hidden="0" customHeight="1">
+    <x:row r="11" ht="1135.199951171875" hidden="0" customHeight="1">
       <x:c r="A11" s="40" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>bmw-x4-oil-leak-2015</x:v>
+        <x:v>bmw-x5m-s63-vanos-solenoid-2010</x:v>
       </x:c>
       <x:c r="C11" s="9" t="str">
-        <x:v>2015-2023 | BMW | X4</x:v>
+        <x:v>2010-2023 | BMW | X5 M | 4.4i, 4.6is, 4.8is, M50i, M60i, xDrive48i, xDrive50e, xDrive50i | S63</x:v>
       </x:c>
       <x:c r="D11" s="9" t="str">
-        <x:v>Oil Leaks - Valve Cover &amp; Oil Filter Housing - All Models</x:v>
+        <x:v>S63 VANOS Solenoid Failure - E70/F85/F95 X5 M</x:v>
       </x:c>
       <x:c r="E11" s="9" t="str">
-        <x:v>Replace valve cover gasket and/or oil filter housing gasket. Valve cover replacement is 3-4 hours labor on X4. Oil filter housing gasket is 1-2 hours. Both are routine maintenance items on BMW turbo engines. Use OEM gaskets for best longevity. Clean oil residue from engine bay after repair. Monitor oil level regularly to catch leaks early.</x:v>
+        <x:v>Replace all 4 VANOS solenoids simultaneously - they are same age and if one has failed, others are close behind. Pierburg 11368605123 (OEM supplier) at $30-$50 each from Turner Motorsport or BimmerWorld. Genuine BMW 11368482268 for S63TU applications at $50-$70 each. Total parts cost: $120-$280 for all 4 solenoids. Also replace VANOS solenoid O-rings and filter screens during service. Labor: 1-2 hours professional ($150-$400 labor). This is one of the easier S63 repairs - accessible from top of engine without removing intake manifold. Natafox and Febi also offer quality aftermarket VANOS solenoids at lower cost ($20-$35 each). Clean VANOS system with fresh oil change immediately after solenoid replacement.</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
         <x:v>0</x:v>
@@ -16848,21 +18210,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="356.3999938964844" hidden="0" customHeight="1">
+    <x:row r="12" ht="1293.5999755859375" hidden="0" customHeight="1">
       <x:c r="A12" s="40" t="n">
         <x:v>11</x:v>
       </x:c>
       <x:c r="B12" s="9" t="str">
-        <x:v>bmw-x4-rear-differential-mount-2015</x:v>
+        <x:v>bmw-x5m-s63-wastegate-rattle-2010</x:v>
       </x:c>
       <x:c r="C12" s="9" t="str">
-        <x:v>2015-2023 | BMW | X4</x:v>
+        <x:v>2010-2018 | BMW | X5 M | S63</x:v>
       </x:c>
       <x:c r="D12" s="9" t="str">
-        <x:v>Rear Differential Mount Bushing Failure</x:v>
+        <x:v>S63 Twin Turbo Wastegate Rattle - E70/F85 X5 M</x:v>
       </x:c>
       <x:c r="E12" s="9" t="str">
-        <x:v>Replace rear differential mount bushings. Both front and rear differential bushings should be inspected and replaced as a set. Upgraded aftermarket bushings with stiffer rubber or polyurethane are available for longer service life.</x:v>
+        <x:v>Option 1 (Most cost-effective): MAMBA SUS316 stainless steel wastegate rattle flapper repair kit for S63 MGT2260 (part 077-0024, replaces 790463-2 / 790484-3), approximately $150-$300 per turbo. Requires turbo removal for installation. Option 2: Lskioer turbo wastegate rattle flapper repair kit for S63/S63TU MGT2260DSL ($80-$150 per kit on Amazon). Option 3: Replace turbo wastegate actuators with new OEM units ($300-$500 each). Option 4: Full turbocharger replacement with new or remanufactured units ($3,000-$5,000 per turbo + labor). Labor for turbo removal and reinstallation: $2,000-$3,500 for both turbos. While turbos are out: replace turbo oil feed/return lines, coolant lines, and all gaskets (GRYPHONTEK turbo coolant line repair kit for E70 X5M, ~$200-$400).</x:v>
       </x:c>
       <x:c r="F12" s="9" t="n">
         <x:v>0</x:v>
@@ -16871,21 +18233,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="620.4000244140625" hidden="0" customHeight="1">
+    <x:row r="13" ht="1069.199951171875" hidden="0" customHeight="1">
       <x:c r="A13" s="40" t="n">
         <x:v>12</x:v>
       </x:c>
       <x:c r="B13" s="9" t="str">
-        <x:v>bmw-x4-transfer-case-2015</x:v>
+        <x:v>bmw-x5m-transfer-case-actuator-2010</x:v>
       </x:c>
       <x:c r="C13" s="9" t="str">
-        <x:v>2015-2023 | BMW | X4</x:v>
+        <x:v>2010-2023 | BMW | X5 M</x:v>
       </x:c>
       <x:c r="D13" s="9" t="str">
-        <x:v>Transfer Case Actuator Motor Failure - All xDrive X4</x:v>
+        <x:v>xDrive Transfer Case Actuator Motor Failure - E70/F85/F95 X5 M</x:v>
       </x:c>
       <x:c r="E13" s="9" t="str">
-        <x:v>Diagnose specific failure. Transfer case actuator motor replacement ($800-1,200) is most common. Complete transfer case replacement required for internal failures ($2,500-4,000). Regular transfer case fluid changes every 50,000 miles may extend life. Some owners install aftermarket upgraded actuator motors. Common wear item on high-mileage xDrive BMW models.</x:v>
+        <x:v>Replace transfer case actuator motor. E70 X5 M: BMW 27107566296 or equivalent ($250-$450 for actuator motor). F85 X5 M: BMW 27608643153 or equivalent ($300-$500). F95 X5 M: check VIN-specific part number with dealer. FCP Euro has an excellent DIY guide for BMW transfer case actuator repair - the actuator can be replaced without removing the entire transfer case. Labor: 2-3 hours at specialist shop ($300-$600 labor). Change transfer case fluid at same time with BMW DTF-1 specification fluid. XeMODeX offers remanufactured transfer case actuator motors at reduced cost ($200-$350). For complete transfer case failure: $3,500-$6,000 for replacement unit + labor.</x:v>
       </x:c>
       <x:c r="F13" s="9" t="n">
         <x:v>0</x:v>
@@ -16894,21 +18256,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="1240.800048828125" hidden="0" customHeight="1">
+    <x:row r="14" ht="435.6000061035156" hidden="0" customHeight="1">
       <x:c r="A14" s="40" t="n">
         <x:v>13</x:v>
       </x:c>
       <x:c r="B14" s="9" t="str">
-        <x:v>bmw-x4m-brake-wear-2020</x:v>
+        <x:v>bmw-x6-adaptive-drive-malfunction-2008</x:v>
       </x:c>
       <x:c r="C14" s="9" t="str">
-        <x:v>2020-2023 | BMW | X4 M | S58</x:v>
+        <x:v>2008-2019 | BMW | X6</x:v>
       </x:c>
       <x:c r="D14" s="9" t="str">
-        <x:v>Accelerated Brake Pad &amp; Rotor Wear from Vehicle Weight - F98 X4 M / F98 X4 M</x:v>
+        <x:v>Adaptive Drive System Malfunction</x:v>
       </x:c>
       <x:c r="E14" s="9" t="str">
-        <x:v>Front brake replacement: OEM front rotor (34118054825 left, matching right) with OEM M compound pads. Complete OEM front brake kit available from BimmerWorld (34108064561K1, ~$800-$1,000). Rear brake kit similarly priced. For track use: Upgrade to Brembo GT brake pad set (BM8 compound) for improved heat resistance and longer pad life. EBC Yellowstuff or Hawk HPS 5.0 pads are popular street/track compromise choices ($150-$250 per axle). StopTech slotted rotors offer improved heat dissipation. For dedicated track cars: Brembo GT big brake kit with 412x38mm discs available ($4,000-$6,000 installed). Budget $2,000-$3,000 per year for brake maintenance if driving spiritedly. Use high-temperature brake fluid (Motul RBF 660 or ATE Typ 200) and flush every 12 months.</x:v>
+        <x:v>Diagnose specific Adaptive Drive component failure using BMW ISTA diagnostics. Replace the failed component — most commonly the hydraulic pump or valve block. If repair cost is prohibitive, some owners convert to conventional anti-roll bars as a permanent fix at lower cost.</x:v>
       </x:c>
       <x:c r="F14" s="9" t="n">
         <x:v>0</x:v>
@@ -16917,21 +18279,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="1188" hidden="0" customHeight="1">
+    <x:row r="15" ht="858" hidden="0" customHeight="1">
       <x:c r="A15" s="40" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="B15" s="9" t="str">
-        <x:v>bmw-x4m-cooling-track-use-2020</x:v>
+        <x:v>bmw-x6-air-suspension-2008</x:v>
       </x:c>
       <x:c r="C15" s="9" t="str">
-        <x:v>2020-2023 | BMW | X4 M</x:v>
+        <x:v>2008-2023 | BMW | X6</x:v>
       </x:c>
       <x:c r="D15" s="9" t="str">
-        <x:v>Cooling System Heat Soak During Track/Spirited Driving - F98 X4 M / F98 X4 M</x:v>
+        <x:v>Air Suspension Compressor &amp; Strut Failure</x:v>
       </x:c>
       <x:c r="E15" s="9" t="str">
-        <x:v>For track use: Upgrade intercooler to do88 front-mount intercooler ($1,200-$1,800) - the community standard for S58 heat management. Add CSF high-performance radiator ($600-$900) for sustained track work. Dinan or VRSF also offer intercooler upgrades in the $1,000-$1,500 range. For street/canyon driving: Stock cooling is adequate but ensure coolant flush every 2 years/30,000 miles and inspect expansion tank for cracks. Replace coolant expansion tank preemptively at 60,000 miles if car is driven hard. For all X3 M/X4 M: Use BMW coolant only (mixed 50/50 with distilled water), replace thermostat at 80,000 miles preventatively, inspect all coolant hoses for bulging or softening at every oil change.</x:v>
+        <x:v>Replace failed air springs or compressor. Arnott rear air spring A-2642 ($200-300 each). OEM F16 spring 37126795013 ($200). Arnott compressor P-2655 ($599). Or convert to coil springs: Strutmasters BB2RBM conversion kit ($1,200-1,800) permanently eliminates air suspension issues. Conversion is cheaper long-term than continued air suspension repairs. If keeping air suspension: inspect air springs at 60,000-80,000 miles for cracks/leaks before compressor damage occurs. Replace both air springs on same axle simultaneously.</x:v>
       </x:c>
       <x:c r="F15" s="9" t="n">
         <x:v>0</x:v>
@@ -16940,21 +18302,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="1214.4000244140625" hidden="0" customHeight="1">
+    <x:row r="16" ht="646.7999877929688" hidden="0" customHeight="1">
       <x:c r="A16" s="40" t="n">
         <x:v>15</x:v>
       </x:c>
       <x:c r="B16" s="9" t="str">
-        <x:v>bmw-x4m-differential-bolt-2020</x:v>
+        <x:v>bmw-x6-ibs-brake-recall-2023</x:v>
       </x:c>
       <x:c r="C16" s="9" t="str">
-        <x:v>2020-2023 | BMW | X4 M</x:v>
+        <x:v>2024-2024 | BMW | X6</x:v>
       </x:c>
       <x:c r="D16" s="9" t="str">
-        <x:v>Rear Differential Mounting Bolt &amp; Bush Failure - F98 X4 M / F98 X4 M</x:v>
+        <x:v>2024 X6 Integrated Brake System Recall 26V-422</x:v>
       </x:c>
       <x:c r="E16" s="9" t="str">
-        <x:v>Replace factory differential bolt, bush, and collar with FJ Motorwerkes uprated diff bolt and collar upgrade kit. The FJ kit uses premium CNC-machined stainless steel components that can handle 170,000 PSI (39% stronger than BMW's revised bolt). Kit price approximately $255 (GBP). Available from FJ Motorwerkes directly, BMG Performance, AM Tuning, and H4ck Performance. Installation is straightforward - rear differential does not need to be fully removed. Budget $400-$600 total including labor. This upgrade is considered MANDATORY by the X3 M/X4 M community for any car making stock or above power. JXB Performance also offers a driveshaft carrier bearing upgrade for cars experiencing propshaft vibration as a companion fix.</x:v>
+        <x:v>Check the VIN at NHTSA and with an authorized BMW dealer when campaign 26V-422 VINs become searchable, and arrange the free dealer inspection and module replacement if required. If a brake warning appears or pedal effort increases, avoid abrupt braking, allow extra stopping distance, stop safely and contact BMW roadside assistance; do not order brake electronics from this card.</x:v>
       </x:c>
       <x:c r="F16" s="9" t="n">
         <x:v>0</x:v>
@@ -16963,21 +18325,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="1293.5999755859375" hidden="0" customHeight="1">
+    <x:row r="17" ht="924" hidden="0" customHeight="1">
       <x:c r="A17" s="40" t="n">
         <x:v>16</x:v>
       </x:c>
       <x:c r="B17" s="9" t="str">
-        <x:v>bmw-x4m-s58-bearing-recall-2020</x:v>
+        <x:v>bmw-x6-n63-timing-chain-2008</x:v>
       </x:c>
       <x:c r="C17" s="9" t="str">
-        <x:v>2020-2021 | BMW | X4 M | M40i, xDrive35i | S58</x:v>
+        <x:v>2008-2018 | BMW | X6 | M50i, xDrive50i</x:v>
       </x:c>
       <x:c r="D17" s="9" t="str">
-        <x:v>S58 Engine Main Bearing Shell Recall / Stop Sale - F98 X4 M / F98 X4 M</x:v>
+        <x:v>N63 Timing Chain Stretch &amp; Guide Failure (E71/F16 xDrive50i)</x:v>
       </x:c>
       <x:c r="E17" s="9" t="str">
-        <x:v>Check VIN immediately against BMW recall database at bmwusa.com or contact your BMW dealer. If your vehicle is within the affected production date range, BMW will inspect and replace main bearing shells at no cost under the Tech Campaign. The repair requires removing the cylinder head and oil pan to access and replace all main bearing shells - this is a major repair (8-12 hours labor) but fully covered by BMW. Do NOT drive the vehicle if knocking is present. For S58 vehicles outside the recall range: Proactive rod bearing inspection is recommended at 60,000 miles for track-driven vehicles. ACL Race Series rod bearings 6B1510H-STD are the aftermarket upgrade choice on Bimmerpost for preventive replacement ($150-$250 for bearing set, $3,000-$5,000 total with labor).</x:v>
+        <x:v>PREVENTIVE REPLACEMENT: If you own 2008-2014 E71 xDrive50i with N63, replace timing chain guides and tensioners IMMEDIATELY at 60,000-80,000 miles ($4,000-6,000) BEFORE failure. IWIS timing chain kit 90001521 ($800-1,200) or Turner kit 11317594899KT recommended. Replace lower chain guide 11147574373 at same time. If chain has already failed: complete engine replacement required ($15,000-25,000). Check VIN with BMW dealer for extended warranty eligibility. 2015+ N63TU engines have improved timing components but still require monitoring.</x:v>
       </x:c>
       <x:c r="F17" s="9" t="n">
         <x:v>0</x:v>
@@ -16986,21 +18348,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="1227.5999755859375" hidden="0" customHeight="1">
+    <x:row r="18" ht="409.20001220703125" hidden="0" customHeight="1">
       <x:c r="A18" s="40" t="n">
         <x:v>17</x:v>
       </x:c>
       <x:c r="B18" s="9" t="str">
-        <x:v>bmw-x4m-transfer-case-2020</x:v>
+        <x:v>bmw-x6-n63-valve-stem-seal-wear-2008</x:v>
       </x:c>
       <x:c r="C18" s="9" t="str">
-        <x:v>2020-2023 | BMW | X4 M | S58</x:v>
+        <x:v>2008-2019 | BMW | X6 | N63</x:v>
       </x:c>
       <x:c r="D18" s="9" t="str">
-        <x:v>xDrive Transfer Case Stress &amp; Fluid Degradation - F98 X4 M / F98 X4 M</x:v>
+        <x:v>N63 Valve Stem Seal Degradation and Oil Burning</x:v>
       </x:c>
       <x:c r="E18" s="9" t="str">
-        <x:v>Change transfer case fluid every 30,000 miles (BMW says "lifetime fill" - this is NOT correct for M vehicles driven hard). Use BMW DTF-1 transfer case fluid or equivalent high-quality synthetic. Check tire tread depth at every service - all 4 tires must be within 2/32" of each other to prevent transfer case stress. Rotate tires every 5,000-7,000 miles. If transfer case actuator motor fails: FCP Euro guide for BMW transfer case actuator repair (part number varies by production date, ~$300-$600). For tuned cars: Consider transfer case brace/reinforcement and shortened fluid change intervals (every 15,000 miles). Complete transfer case replacement if internals are damaged: $3,000-$5,500 at independent specialist, $5,000-$8,000+ at dealer.</x:v>
+        <x:v>Replace all intake and exhaust valve stem seals. This is a major job requiring head work. Also replace turbo oil return lines and update engine software per BMW N63 Customer Care Package specifications. Ensure proper oil grade (BMW LL-01) is used.</x:v>
       </x:c>
       <x:c r="F18" s="9" t="n">
         <x:v>0</x:v>
@@ -17009,21 +18371,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="1042.800048828125" hidden="0" customHeight="1">
+    <x:row r="19" ht="858" hidden="0" customHeight="1">
       <x:c r="A19" s="40" t="n">
         <x:v>18</x:v>
       </x:c>
       <x:c r="B19" s="9" t="str">
-        <x:v>bmw-x5-air-suspension-2007</x:v>
+        <x:v>bmw-x6-n63-valve-stem-seals-2008</x:v>
       </x:c>
       <x:c r="C19" s="9" t="str">
-        <x:v>2019-2026 | BMW | X5</x:v>
+        <x:v>2008-2023 | BMW | X6 | M50i, xDrive50i | N63</x:v>
       </x:c>
       <x:c r="D19" s="9" t="str">
-        <x:v>G05 Suspension Warning: Check Faults and Campaigns Before Parts</x:v>
+        <x:v>N63 Valve Stem Seal / Oil Consumption (xDrive50i)</x:v>
       </x:c>
       <x:c r="E19" s="9" t="str">
-        <x:v>Start with the VIN build/options, open-campaign status, exact warning, complete fault memory, and BMW ISTA test plan. If the VIN and production date match a BMW action, follow that bulletin: inspect the specified sensor-link holders, apply the specified software correction, or inspect the affected air line as directed. For other vehicles, test the particular system shown by the VIN and fault path before selecting any component. Do not buy a compressor, strut, spring, or conversion kit until the failed part and its VIN-specific number are established. This article intentionally has no retail link because no single part repairs all of these conditions.</x:v>
+        <x:v>Replace valve stem seals - extremely labor-intensive job requiring cylinder head work ($4,900-12,000 total). Elring seals 11340039494 ($80-120/set of 16, need 2 sets for V8). 5150 AutoSport Viton upgraded seals ($150-200) are recommended for better heat resistance in hot-vee configuration. AGA Tools kit AGA-N63-VSK-K ($500-800) includes specialized tools required. Reference TSB MC-10149960-9999 when visiting dealer. Some owners monitor oil levels and add as needed rather than repair. Use quality synthetic 0W-40 BMW LL-01 spec oil.</x:v>
       </x:c>
       <x:c r="F19" s="9" t="n">
         <x:v>0</x:v>
@@ -17032,44 +18394,44 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="1148.4000244140625" hidden="0" customHeight="1">
+    <x:row r="20" ht="818.4000244140625" hidden="0" customHeight="1">
       <x:c r="A20" s="40" t="n">
         <x:v>19</x:v>
       </x:c>
       <x:c r="B20" s="9" t="str">
-        <x:v>bmw-x5-air-suspension-compressor-2007</x:v>
+        <x:v>bmw-x6-n63-wastegate-2008</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>2007-2013 | BMW | X5 | 3.0si, 4.8i, xDrive30i, xDrive35d, xDrive35i, xDrive48i, xDrive50i, X5 M | N52, N62, M57, N55, N63, S63</x:v>
+        <x:v>2008-2018 | BMW | X6 | M50i, xDrive50i</x:v>
       </x:c>
       <x:c r="D20" s="9" t="str">
-        <x:v>E70 Rear Air-Supply Unit: Diagnose the Self-Leveling System First</x:v>
+        <x:v>N63 Turbo Wastegate Rattle (xDrive50i)</x:v>
       </x:c>
       <x:c r="E20" s="9" t="str">
-        <x:v>Read the EHC fault memory and run the applicable BMW ISTA test plan before ordering a compressor. Confirm the vehicle is equipped with rear self-leveling suspension, compare left/right ride height, check system power and wiring, inspect the height-sensor links, and leak-test the air springs, lines, and valve system. Test the air supply only after those checks isolate it. If BMW ETK/AIR selects the E70 air-supply system for the VIN and diagnosis confirms that assembly, replace it with current part 37-20-6-859-714, follow the BMW repair procedure, clear faults, and perform the required ride-height calibration. Do not install a generic compressor or a coil-conversion kit from symptoms alone.</x:v>
+        <x:v>Repair options range from flapper repair kits ($50-100/turbo) to complete turbocharger replacement ($4,000-8,000 for both). Garrett MGT2256S flapper repair kit ($50-100 per turbo) is cheapest fix. MAMBA adjustable actuator kit ($150-300) provides more durable solution. OEM actuators 11657646093 available from BMW. Complete turbo replacement $2,000-4,000 per turbo. MONITORING: Wastegate rattle is early warning - address before complete turbo failure to avoid $8,000+ repair.</x:v>
       </x:c>
       <x:c r="F20" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G20" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="1227.5999755859375" hidden="0" customHeight="1">
+    <x:row r="21" ht="409.20001220703125" hidden="0" customHeight="1">
       <x:c r="A21" s="40" t="n">
         <x:v>20</x:v>
       </x:c>
       <x:c r="B21" s="9" t="str">
-        <x:v>bmw-x5-carbon-buildup-2007</x:v>
+        <x:v>bmw-x6-rear-differential-bushing-2008</x:v>
       </x:c>
       <x:c r="C21" s="9" t="str">
-        <x:v>2011-2018 | BMW | X5 | xDrive35i, xDrive50i | N55, N63, N63TU1</x:v>
+        <x:v>2008-2026 | BMW | X6</x:v>
       </x:c>
       <x:c r="D21" s="9" t="str">
-        <x:v>Possible Intake-Valve Deposits on Direct-Injected Gasoline Engines</x:v>
+        <x:v>Rear Differential Bushing Deterioration</x:v>
       </x:c>
       <x:c r="E21" s="9" t="str">
-        <x:v>Diagnose the actual symptom before authorizing cleaning: read BMW-specific faults and misfire counters, check ignition and fueling, smoke-test the intake where indicated, verify crankcase ventilation operation, and inspect the intake valves with a borescope or by removing the intake manifold when the test plan supports it. If substantial deposits are confirmed and match the complaint, use an engine-specific professional mechanical-cleaning procedure that protects closed valves and removes all blasting media before reassembly. Do not present a universal catch can, chemical spray, fuel brand, short oil interval, or high-RPM driving as a proven repair. Any crankcase-ventilation modification also requires engine-specific fitment and emissions-law review.</x:v>
+        <x:v>Replace all rear differential mount bushings. Use OEM or equivalent quality bushings (Lemforder is the OEM supplier). Inspect the differential housing for any damage from excessive movement. Perform subframe alignment check after bushing replacement.</x:v>
       </x:c>
       <x:c r="F21" s="9" t="n">
         <x:v>0</x:v>
@@ -17078,67 +18440,67 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="884.4000244140625" hidden="0" customHeight="1">
+    <x:row r="22" ht="765.5999755859375" hidden="0" customHeight="1">
       <x:c r="A22" s="40" t="n">
         <x:v>21</x:v>
       </x:c>
       <x:c r="B22" s="9" t="str">
-        <x:v>bmw-x5-coolant-pipe-leak-2007</x:v>
+        <x:v>bmw-x6-transfer-case-2008</x:v>
       </x:c>
       <x:c r="C22" s="9" t="str">
-        <x:v>2007-2010 | BMW | X5 | 4.8i, xDrive48i | N62, N62TU</x:v>
+        <x:v>2008-2023 | BMW | X6</x:v>
       </x:c>
       <x:c r="D22" s="9" t="str">
-        <x:v>E70 N62 Coolant Transfer Pipe Leak (Pressure-Test First)</x:v>
+        <x:v>Transfer Case Actuator Motor Failure (All xDrive Models)</x:v>
       </x:c>
       <x:c r="E22" s="9" t="str">
-        <x:v>Pressure-test the cooling system cold and inspect the engine valley and all accessible connections to identify the exact leak before ordering parts. If inspection confirms the N62 transfer pipe and BMW ETK/AIR selects it for the VIN, replace pipe 11-14-1-439-975 with the required seals and one-time-use hardware from the VIN-specific repair diagram. Refill and bleed the cooling system with the specified coolant, repeat the pressure test, and verify stable temperature. Do not automatically replace an N63 pipe, thermostat, or unrelated hoses from this article.</x:v>
+        <x:v>Replace the actuator motor assembly or rebuild using an aftermarket gear repair kit ($100-150). G06 actuator motor 27609469023 ($400-600) for complete replacement. DIY gear repair kits are straightforward and save $1,200+ over dealer replacement. Complete transfer case replacement if internal damage occurred: $1,400-3,300. PREVENTIVE: If buying used X6 over 80k miles, budget for this repair and listen for clicking noise when shutting off ignition.</x:v>
       </x:c>
       <x:c r="F22" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G22" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="1082.4000244140625" hidden="0" customHeight="1">
+    <x:row r="23" ht="514.7999877929688" hidden="0" customHeight="1">
       <x:c r="A23" s="40" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="B23" s="9" t="str">
-        <x:v>bmw-x5-n63-timing-chain-2008</x:v>
+        <x:v>bmw-x6m-front-thrust-arm-bushing-2015</x:v>
       </x:c>
       <x:c r="C23" s="9" t="str">
-        <x:v>2010-2013 | BMW | X5 | xDrive50i | N63</x:v>
+        <x:v>2015-2025 | BMW | X6 M</x:v>
       </x:c>
       <x:c r="D23" s="9" t="str">
-        <x:v>Early N63 Timing-Chain Wear Check: ISTA Test Before Repair</x:v>
+        <x:v>Front Thrust Arm Bushing (Tension Strut) Premature Wear</x:v>
       </x:c>
       <x:c r="E23" s="9" t="str">
-        <x:v>Check the VIN and service history with a BMW center, diagnose stored VANOS/camshaft faults first, and run BMW's ISTA timing-chain elongation test. If the result is 'Timing chain is OK,' do not replace parts on this claim. If it is 'not OK,' BMW SIB 11 16 14 directs replacement of both timing chains under the VIN-specific repair instruction, followed by the required oil/filter service, priming steps, programming, and shorter oil-service interval. A single tensioner 11-31-7-557-741 or a generic Cloyes kit is not the complete repair and must not be presented as what the owner needs. Tow the vehicle rather than driving it when severe mechanical noise, oil-pressure warnings, or loss of timing is present.</x:v>
+        <x:v>Replace both front thrust arms as complete assemblies (the bushings are not serviceable separately). Use genuine BMW M-spec parts or Lemforder equivalents. Perform a 4-wheel alignment immediately after replacement. Upgrade to Powerflex polyurethane thrust arm bushings for extended lifespan, especially on tracked cars.</x:v>
       </x:c>
       <x:c r="F23" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G23" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="1227.5999755859375" hidden="0" customHeight="1">
+    <x:row r="24" ht="897.5999755859375" hidden="0" customHeight="1">
       <x:c r="A24" s="40" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="B24" s="9" t="str">
-        <x:v>bmw-x5-n63-wastegate-2008</x:v>
+        <x:v>bmw-x6m-s63-rod-bearing-2010</x:v>
       </x:c>
       <x:c r="C24" s="9" t="str">
-        <x:v>2010-2018 | BMW | X5 | xDrive50i | N63, N63TU</x:v>
+        <x:v>2010-2023 | BMW | X6 M | M50i, xDrive50i | S63</x:v>
       </x:c>
       <x:c r="D24" s="9" t="str">
-        <x:v>N63/N63TU Low Boost or Turbo Rattle: Diagnose Vacuum Control First</x:v>
+        <x:v>S63 Rod Bearing Failure (X6 M)</x:v>
       </x:c>
       <x:c r="E24" s="9" t="str">
-        <x:v>Read all DME faults and compare requested versus actual boost under the BMW test plan. Pressure- or smoke-test the intake and charge-air path, verify vacuum supply from the pump and reservoir, inspect both banks' hoses and pressure converters, and test actuator movement before condemning a turbocharger. Identify the engine generation, failed bank, and exact hardware in BMW ETK/AIR. Check a 2010-2013 E70 VIN for the N63 Customer Care Package only as applicable; its published six-point scope includes air-mass sensors, injectors, vacuum pump, low-pressure fuel sensor/feed line, fresh-air turbo seals, and crankcase-ventilation lines, not an automatic wastegate replacement. No retail link is published until diagnosis selects a VIN-specific component.</x:v>
+        <x:v>PREVENTIVE: Replace rod bearings every 60,000-80,000 miles ($2,500-5,000 labor-intensive job). Use ACL Race 8B1578HX-STD ($150-250) or King CR8049SV ($120-200) upgraded bearings - these are stronger than OEM and provide better durability under high loads. Send oil samples for analysis (Blackstone Labs ~$30) every 5,000 miles to monitor bearing wear metals. If bearings have already failed: engine replacement required ($15,000-30,000). DO NOT buy used X6 M without documented bearing replacement history or fresh oil analysis.</x:v>
       </x:c>
       <x:c r="F24" s="9" t="n">
         <x:v>0</x:v>
@@ -17147,136 +18509,136 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="844.7999877929688" hidden="0" customHeight="1">
+    <x:row r="25" ht="277.20001220703125" hidden="0" customHeight="1">
       <x:c r="A25" s="40" t="n">
         <x:v>24</x:v>
       </x:c>
       <x:c r="B25" s="9" t="str">
-        <x:v>bmw-x5-oil-leaks-2000</x:v>
+        <x:v>bmw-x6m-vanos-solenoid-2015</x:v>
       </x:c>
       <x:c r="C25" s="9" t="str">
-        <x:v>2003-2006 | BMW | X5 | 3.0i | M54</x:v>
+        <x:v>2015-2021 | BMW | X6 M | S63</x:v>
       </x:c>
       <x:c r="D25" s="9" t="str">
-        <x:v>E53 3.0i M54 Valve-Cover Gasket Leak (Confirm the Source)</x:v>
+        <x:v>VANOS Solenoid Oil Sludge Buildup</x:v>
       </x:c>
       <x:c r="E25" s="9" t="str">
-        <x:v>Clean the engine and trace the highest fresh-oil source before ordering a gasket. If the leak is at the M54 cylinder-head-cover perimeter or spark-plug-well seals, inspect the plastic cover for cracks, warpage, damaged fastener grommets, and crankcase-ventilation faults. Reuse the cover only if it passes inspection, then install VIN/production-confirmed gasket set 11-12-0-030-496 with the BMW-specified grommets and sealant locations and torque sequence. If the cover or another oil circuit is the source, select that separate repair instead.</x:v>
+        <x:v>Remove and clean or replace the VANOS solenoids. Perform an engine oil flush. Strictly follow 7,500-mile oil change intervals with BMW LL-01 rated 0W-40 synthetic oil.</x:v>
       </x:c>
       <x:c r="F25" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G25" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="1293.5999755859375" hidden="0" customHeight="1">
+    <x:row r="26" ht="699.5999755859375" hidden="0" customHeight="1">
       <x:c r="A26" s="40" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="B26" s="9" t="str">
-        <x:v>bmw-x5-transfer-case-actuator-2000</x:v>
+        <x:v>bmw-x7-48v-battery-2020</x:v>
       </x:c>
       <x:c r="C26" s="9" t="str">
-        <x:v>2007-2013 | BMW | X5 | 3.0si, 4.8i, xDrive30i, xDrive35d, xDrive48i, X5 M | N52, N62, M57, S63</x:v>
+        <x:v>2020-2023 | BMW | X7</x:v>
       </x:c>
       <x:c r="D26" s="9" t="str">
-        <x:v>E70 ATC700 Transfer-Case Positioning Motor (Diagnosis Required)</x:v>
+        <x:v>48V Mild Hybrid Battery Issues</x:v>
       </x:c>
       <x:c r="E26" s="9" t="str">
-        <x:v>Read BMW VTG/DSC faults and run the applicable ISTA transfer-case test plan before buying a motor. Confirm tire sizes and wear, battery voltage, wiring, transfer-case type, fluid condition, calibration, and—especially after differential or transfer-case replacement—the VIN-correct front and rear gear ratios. If testing confirms the ATC700 positioning motor and BMW ETK/AIR selects this application for the VIN, current BMW exchange servomotor 27-10-2-449-709 supersedes 27-10-7-568-267. Install the correct classification resistor/hardware supplied or specified for the VIN and perform the required VTG initialization/calibration. A generic gear-only kit is not a universal BMW repair and should not be ordered without opening and confirming the exact motor failure.</x:v>
+        <x:v>Replace the 48V mild hybrid battery ($1,000-2,000 at dealer). Requires dealer-level diagnostic tools and coding after installation - this is NOT a DIY repair. The 48V battery is separate from the main 12V battery. No aftermarket alternatives currently available. Check if vehicle is still under BMW warranty or extended warranty coverage. Some owners choose to live with the failed auto start-stop rather than pay for replacement.</x:v>
       </x:c>
       <x:c r="F26" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G26" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="1042.800048828125" hidden="0" customHeight="1">
+    <x:row r="27" ht="726" hidden="0" customHeight="1">
       <x:c r="A27" s="40" t="n">
         <x:v>26</x:v>
       </x:c>
       <x:c r="B27" s="9" t="str">
-        <x:v>bmw-x5-transfer-case-actuator-2007</x:v>
+        <x:v>bmw-x7-air-suspension-2019</x:v>
       </x:c>
       <x:c r="C27" s="9" t="str">
-        <x:v>2019-2026 | BMW | X5</x:v>
+        <x:v>2019-2023 | BMW | X7</x:v>
       </x:c>
       <x:c r="D27" s="9" t="str">
-        <x:v>G05/F95 Transfer-Case Shudder: Tires and Fluid Diagnosis First</x:v>
+        <x:v>Air Suspension Compressor &amp; Strut Failure (Standard Equipment)</x:v>
       </x:c>
       <x:c r="E27" s="9" t="str">
-        <x:v>Follow BMW SIB 27 02 20 in order: verify all four tires for VIN-correct size, brand/application, axle placement, and wear; diagnose any powertrain faults; then use ISTA to temporarily deactivate the transfer-case clutch and road-test the complaint. Only if the shudder disappears with the VTG deactivated does BMW direct an ATX13-X oil change with DTF-1, followed by VTG calibration. The clutch plates can require up to 125 miles after the service to become fully saturated and smooth out. If the symptom remains, continue diagnosis rather than buying an actuator or transfer case. Part numbers for any further repair must be selected by VIN in ETK/AIR.</x:v>
+        <x:v>Replace failed air struts and/or compressor. Front strut left 37106869035 ($1,500-2,000), right 37106869036 ($1,500-2,000), rear 37106869039 ($1,000-1,500). Compressor 37206861882 ($800-1,200). RebuildMasterTech rebuilt struts ($600-900 each) are a more affordable alternative. Total repair can reach $2,180-5,000+ depending on which components have failed. Replace both struts on same axle simultaneously. Inspect at 50,000 miles for early signs of leaking.</x:v>
       </x:c>
       <x:c r="F27" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G27" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="1214.4000244140625" hidden="0" customHeight="1">
+    <x:row r="28" ht="435.6000061035156" hidden="0" customHeight="1">
       <x:c r="A28" s="40" t="n">
         <x:v>27</x:v>
       </x:c>
       <x:c r="B28" s="9" t="str">
-        <x:v>bmw-x5-vanos-solenoid-2000</x:v>
+        <x:v>bmw-x7-air-suspension-compressor-2019</x:v>
       </x:c>
       <x:c r="C28" s="9" t="str">
-        <x:v>2010-2013 | BMW | X5 | xDrive30i, xDrive35i | N51, N52K, N52T, N55</x:v>
+        <x:v>2019-2026 | BMW | X7</x:v>
       </x:c>
       <x:c r="D28" s="9" t="str">
-        <x:v>VANOS Adjustment-Unit Bolt Recall 23V-707 (E70 Inline-Six)</x:v>
+        <x:v>Air Suspension Compressor Failure</x:v>
       </x:c>
       <x:c r="E28" s="9" t="str">
-        <x:v>Enter the VIN in BMW's official recall lookup and have an authorized BMW center complete recall 23V-707 if it is open. BMW's procedure is inspection-dependent: intact affected bolts are replaced; if bolts are loose or broken, the affected VANOS adjustment unit is replaced, and missing fragments must be recovered. The recall repair is free, so do not buy a solenoid or VANOS part first. If the VIN is outside the recall or a fault remains after the remedy, use BMW-capable diagnostics to test oil supply and pressure, wiring, sensors, control solenoids, adjustment units, and mechanical timing before selecting a part. If the engine runs roughly, makes unusual mechanical noise, loses power, or stalls, move out of traffic safely, stop driving, and contact BMW for transport guidance.</x:v>
+        <x:v>Replace the air suspension compressor. Inspect all four air springs for leaks using soapy water solution. Replace any leaking air springs to prevent repeated compressor failure. Check the valve block for proper operation. The compressor is located under the rear of the vehicle.</x:v>
       </x:c>
       <x:c r="F28" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G28" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="1148.4000244140625" hidden="0" customHeight="1">
+    <x:row r="29" ht="871.2000122070312" hidden="0" customHeight="1">
       <x:c r="A29" s="40" t="n">
         <x:v>28</x:v>
       </x:c>
       <x:c r="B29" s="9" t="str">
-        <x:v>bmw-x5-water-pump-2007</x:v>
+        <x:v>bmw-x7-b58-coolant-2019</x:v>
       </x:c>
       <x:c r="C29" s="9" t="str">
-        <x:v>2011-2013 | BMW | X5 | xDrive35i | N55</x:v>
+        <x:v>2019-2023 | BMW | X7 | xDrive40i | B58</x:v>
       </x:c>
       <x:c r="D29" s="9" t="str">
-        <x:v>E70 xDrive35i N55 Electric Coolant Pump (Fault-Confirmed)</x:v>
+        <x:v>B58 Coolant System Failures (xDrive40i)</x:v>
       </x:c>
       <x:c r="E29" s="9" t="str">
-        <x:v>If the engine-temperature warning appears, stop safely, shut the engine off, and tow the vehicle if normal temperature cannot be confirmed. When cool, check coolant level and leaks, read BMW-specific faults, verify pump power/ground and communication, and run the ISTA coolant-pump activation/test plan. If those tests confirm the pump and BMW ETK/AIR selects 11-51-5-A05-704 for the VIN, replace it using the BMW procedure, select the thermostat separately only if testing or preventive planning justifies it, vacuum-fill or bleed the system as specified, and verify commanded pump operation and stable temperature. Do not use a fixed-mileage rule or this part number for an N52, N63, or F15 without VIN confirmation.</x:v>
+        <x:v>Replace failed coolant system components. Water pump 11518482250 ($300-400). Thermostat 11537644811 ($150-250). Replace expansion tank and all plastic coolant connections when performing repair to prevent cascading failures. For 2023+ models, check VIN for recall 24V-608 coverage for coolant pump connector. Total repair $500-2,500 depending on extent of damage. PREVENTIVE: Replace thermostat and water pump at 60,000-70,000 miles before failure. Inspect coolant hoses and connections at every oil change after 50k miles.</x:v>
       </x:c>
       <x:c r="F29" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G29" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="1056" hidden="0" customHeight="1">
+    <x:row r="30" ht="435.6000061035156" hidden="0" customHeight="1">
       <x:c r="A30" s="40" t="n">
         <x:v>29</x:v>
       </x:c>
       <x:c r="B30" s="9" t="str">
-        <x:v>bmw-x5m-brake-system-2010</x:v>
+        <x:v>bmw-x7-b58-coolant-expansion-tank-2019</x:v>
       </x:c>
       <x:c r="C30" s="9" t="str">
-        <x:v>2010-2023 | BMW | X5 M</x:v>
+        <x:v>2019-2026 | BMW | X7 | B58</x:v>
       </x:c>
       <x:c r="D30" s="9" t="str">
-        <x:v>Heavy-Duty Brake System Accelerated Wear - E70/F85/F95 X5 M</x:v>
+        <x:v>B58 Coolant Expansion Tank Crack</x:v>
       </x:c>
       <x:c r="E30" s="9" t="str">
-        <x:v>E70 X5 M brakes: OEM front pads 34116799964 ($150-$250), rear pads 34216794879 ($120-$200). F85 X5 M front brake rotors: 34112284101/34112284102 with 6-pot caliper 34117845747/34117845748 and pads 34112284869. F85 rear: 385mm x 24mm perforated rotors 34212284903/34212284904 with 4-pot Brembo caliper and Textar pads. Budget $1,500-$2,500 per axle for complete brake service. For track use: EBC Yellowstuff or Hawk HPS 5.0 pads ($200-$350 per axle) with StopTech slotted rotors for improved heat management. Use Motul RBF 660 or ATE Typ 200 brake fluid - flush every 12 months. Budget $3,000-$5,000 per year for brake maintenance if driving spiritedly.</x:v>
+        <x:v>Replace the coolant expansion tank with an updated BMW part that uses improved plastic composition. Also replace the cap and inspect all coolant hoses. Flush and refill the cooling system with BMW-approved coolant. Check for coolant contamination from the old tank.</x:v>
       </x:c>
       <x:c r="F30" s="9" t="n">
         <x:v>0</x:v>
@@ -17285,21 +18647,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="1122" hidden="0" customHeight="1">
+    <x:row r="31" ht="646.7999877929688" hidden="0" customHeight="1">
       <x:c r="A31" s="40" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="B31" s="9" t="str">
-        <x:v>bmw-x5m-rear-differential-2010</x:v>
+        <x:v>bmw-x7-ibs-brake-recall-2023</x:v>
       </x:c>
       <x:c r="C31" s="9" t="str">
-        <x:v>2010-2023 | BMW | X5 M | S63</x:v>
+        <x:v>2023-2025 | BMW | X7</x:v>
       </x:c>
       <x:c r="D31" s="9" t="str">
-        <x:v>Rear Differential Wear &amp; Fluid Degradation - E70/F85/F95 X5 M</x:v>
+        <x:v>2023-2025 X7 Integrated Brake System Recall 26V-422</x:v>
       </x:c>
       <x:c r="E31" s="9" t="str">
-        <x:v>Change rear differential fluid every 30,000 miles (ignore BMW "lifetime fill" claim). E70 X5 M: No drain plug - fluid must be extracted through fill port with hand pump or suction device. Recommended fluid: Royal Purple 75W-140 GL5 synthetic or Red Line 75W-140 GL5 ($40-$60 per fill). Capacity approximately 1.2 liters. For limited-slip diff, ensure fluid is GL5 rated with limited-slip additive. If differential is making whining/howling noise: have a limited-slip differential specialist inspect internals (not generic BMW shop). Diff rebuild: $1,500-$3,000 at specialist. Complete differential replacement: $3,000-$5,500 + labor. Labor for fluid change: $150-$300 at independent shop.</x:v>
+        <x:v>Check the VIN at NHTSA and with an authorized BMW dealer when campaign 26V-422 VINs become searchable, and arrange the free dealer inspection and module replacement if required. If a brake warning appears or pedal effort increases, avoid abrupt braking, allow extra stopping distance, stop safely and contact BMW roadside assistance; do not order brake electronics from this card.</x:v>
       </x:c>
       <x:c r="F31" s="9" t="n">
         <x:v>0</x:v>
@@ -17308,21 +18670,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="1386" hidden="0" customHeight="1">
+    <x:row r="32" ht="897.5999755859375" hidden="0" customHeight="1">
       <x:c r="A32" s="40" t="n">
         <x:v>31</x:v>
       </x:c>
       <x:c r="B32" s="9" t="str">
-        <x:v>bmw-x5m-s63-cooling-system-2010</x:v>
+        <x:v>bmw-x7-n63-oil-consumption-2019</x:v>
       </x:c>
       <x:c r="C32" s="9" t="str">
-        <x:v>2010-2023 | BMW | X5 M | 4.4i, 4.6is, 4.8is, M50i, M60i, xDrive48i, xDrive50e, xDrive50i | S63</x:v>
+        <x:v>2019-2023 | BMW | X7 | M50i, M60i, xDrive50i | N63TU3</x:v>
       </x:c>
       <x:c r="D32" s="9" t="str">
-        <x:v>S63 Cooling System Component Failures - E70/F85/F95 X5 M</x:v>
+        <x:v>N63TU3 Oil Consumption &amp; Valve Stem Seal Degradation (xDrive50i/M50i/M60i)</x:v>
       </x:c>
       <x:c r="E32" s="9" t="str">
-        <x:v>PROACTIVE MAINTENANCE SCHEDULE: Replace electric water pump at 60,000 miles ($400-$700 + labor). Replace thermostat at same time ($150-$250). Replace expansion tank at 60,000-80,000 miles ($100-$200). Inspect all coolant hoses at every oil change - replace any that are soft, bulging, or showing surface cracks. E70 X5 M expansion tank vent hose: 17128627119 ($30-$50). Flush coolant system every 2 years or 30,000 miles (more frequent than BMW's 4-year recommendation). Use ONLY BMW coolant mixed 50/50 with distilled water. For E70 hot-V turbo coolant lines: GRYPHONTEK repair kit eliminates plastic T-fitting failure (see separate issue entry). Budget $1,500-$2,500 for complete cooling system refresh at 60,000 miles. This prevents catastrophic overheating that can destroy the S63 engine ($15,000-$34,000 engine replacement).</x:v>
+        <x:v>Replace valve stem seals - extremely labor-intensive job requiring cylinder head work ($4,900-12,000 total). Elring seals 11340039494 for OEM spec. 5150 AutoSport Viton upgraded seals ($150-200) recommended for better heat resistance. AGA Tools kit includes specialized tools required. Reference TSB MC-10149960-9999 when visiting dealer. Check eligibility for class action settlement coverage. Some owners monitor oil levels and top off rather than repair. Use quality synthetic 0W-40 BMW LL-01 spec oil and check level every 500-1,000 miles.</x:v>
       </x:c>
       <x:c r="F32" s="9" t="n">
         <x:v>0</x:v>
@@ -17331,21 +18693,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="1135.199951171875" hidden="0" customHeight="1">
+    <x:row r="33" ht="396" hidden="0" customHeight="1">
       <x:c r="A33" s="40" t="n">
         <x:v>32</x:v>
       </x:c>
       <x:c r="B33" s="9" t="str">
-        <x:v>bmw-x5m-s63-oil-leaks-2010</x:v>
+        <x:v>bmw-x7-panoramic-roof-rattle-2019</x:v>
       </x:c>
       <x:c r="C33" s="9" t="str">
-        <x:v>2010-2023 | BMW | X5 M | 4.4i, 4.6is, 4.8is, M50i, M60i, xDrive48i, xDrive50e, xDrive50i | S63</x:v>
+        <x:v>2019-2026 | BMW | X7</x:v>
       </x:c>
       <x:c r="D33" s="9" t="str">
-        <x:v>S63 V8 Chronic Oil Leaks (Valve Cover, Oil Pan, Turbo Lines) - E70/F85/F95 X5 M</x:v>
+        <x:v>Panoramic Sunroof Rattle and Creak</x:v>
       </x:c>
       <x:c r="E33" s="9" t="str">
-        <x:v>Valve cover gasket replacement (both sides): $1,200-$2,500 with labor. BMW plastic valve covers can crack and must be replaced entirely (not just gasket) - inspect during service. Oil filter housing gasket: $400-$800 with labor. Oil pan gasket: $2,000-$3,500 (requires engine/subframe drop). Turbo oil feed/return lines: replace with GRYPHONTEK or MAMBA upgraded silicone/braided lines during any turbo service ($200-$400). VANOS solenoid seals: $100-$200 (DIY-friendly). For comprehensive oil leak repair at 80,000+ miles: budget $3,000-$5,000 to address all common leak points simultaneously. Valve cover bolt torque is CRITICAL - too tight cracks the cover ($800-$1,200 per cover), too loose and it leaks.</x:v>
+        <x:v>Apply BMW-approved felt tape or lubricant to sunroof guide rails. Replace worn guide rail bushings. In severe cases, the sunroof cassette or seal may need replacement under warranty. BMW has issued updated guide rail components for early production vehicles.</x:v>
       </x:c>
       <x:c r="F33" s="9" t="n">
         <x:v>0</x:v>
@@ -17354,21 +18716,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="1412.4000244140625" hidden="0" customHeight="1">
+    <x:row r="34" ht="778.7999877929688" hidden="0" customHeight="1">
       <x:c r="A34" s="40" t="n">
         <x:v>33</x:v>
       </x:c>
       <x:c r="B34" s="9" t="str">
-        <x:v>bmw-x5m-s63-rod-bearing-2010</x:v>
+        <x:v>bmw-x7-sunroof-leak-2019</x:v>
       </x:c>
       <x:c r="C34" s="9" t="str">
-        <x:v>2010-2018 | BMW | X5 M | 4.4i, 4.6is, 4.8is, M50i, M60i, xDrive48i, xDrive50e, xDrive50i</x:v>
+        <x:v>2019-2023 | BMW | X7</x:v>
       </x:c>
       <x:c r="D34" s="9" t="str">
-        <x:v>S63 V8 Rod Bearing Premature Wear &amp; Failure - E70/F85 X5 M</x:v>
+        <x:v>Panoramic Sunroof Water Leak</x:v>
       </x:c>
       <x:c r="E34" s="9" t="str">
-        <x:v>PREVENTIVE: For track-driven X5 M, replace rod bearings proactively at 60,000-80,000 miles. ACL Race Series rod bearings (8B1578HX-STD for S63B44, +0.001" extra oil clearance) are the community gold standard ($200-$350 for bearing set). WPC surface-treated bearings from Lang Racing are the premium choice ($400-$600 set). Total cost for preventive rod bearing service: $4,500-$8,500 depending on shop. Oil analysis every 5,000 miles through Blackstone Labs ($30/test) to monitor bearing wear metals (lead and copper). Use only BMW 10W-60 synthetic oil with 5,000-7,500 mile oil change intervals. Never track the car on cold oil. Mporium BMW offers specialized S63 rod bearing service starting at $4,499. If catastrophic failure: rebuilt S63 engine from RK Autowerks (~$8,500 + installation), new BMW engine (~$34,000), or complete engine rebuild ($12,000-$18,000).</x:v>
+        <x:v>Clear clogged sunroof drain tubes ($100-300 at shop). Reference TSB SIB 54 11 19 when visiting dealer. For persistent leaks, drain tube connections or sunroof seal may need replacement ($500-1,500). If water has damaged interior electronics, repair costs can reach $3,000. PREVENTIVE: Clear sunroof drains annually, especially in areas with heavy tree debris. Run compressed air or flexible drain snake through drain tubes during oil changes. Keep sunroof track clean of debris.</x:v>
       </x:c>
       <x:c r="F34" s="9" t="n">
         <x:v>0</x:v>
@@ -17377,21 +18739,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="1214.4000244140625" hidden="0" customHeight="1">
+    <x:row r="35" ht="739.2000122070312" hidden="0" customHeight="1">
       <x:c r="A35" s="40" t="n">
         <x:v>34</x:v>
       </x:c>
       <x:c r="B35" s="9" t="str">
-        <x:v>bmw-x5m-s63-turbo-coolant-line-2010</x:v>
+        <x:v>bmw-x7-tire-wear-2019</x:v>
       </x:c>
       <x:c r="C35" s="9" t="str">
-        <x:v>2010-2013 | BMW | X5 M</x:v>
+        <x:v>2019-2023 | BMW | X7</x:v>
       </x:c>
       <x:c r="D35" s="9" t="str">
-        <x:v>S63 Turbo Coolant Line Plastic T-Fitting Failure (Hot-V Design) - E70 X5 M</x:v>
+        <x:v>Premature Tire Wear (Especially 21"/22" Wheels)</x:v>
       </x:c>
       <x:c r="E35" s="9" t="str">
-        <x:v>Replace ALL factory plastic turbo coolant T-fittings and hoses with GRYPHONTEK S63 Turbo Coolant Line Repair Kit ($200-$400). Kit includes pre-shaped multi-layer reinforced silicone hoses, brass T-fittings (replacing factory plastic), and all necessary hose clamps. Direct bolt-on installation designed for the E70/E71 S63 engine bay. MAMBA Turbo also offers a reinforced turbo coolant line kit with brass and silicone components ($150-$350). This is a PROACTIVE replacement - do not wait for failure. Replace at first sign of coolant weeping or during any turbo service. Labor: $800-$1,500 due to tight access in hot-V engine valley. If turbo bearings are damaged from overheating: turbo replacement $3,000-$5,000 per unit.</x:v>
+        <x:v>Have alignment adjusted to reduce aggressive camber settings ($200-400). Switch to quality tires designed for heavy SUVs: Michelin Pilot Sport 4S or Continental PremiumContact 6 are recommended. If possible, avoid 22" wheels and opt for 21" or smaller for better tire longevity and ride comfort. Alignment adjustment can extend tire life from 15,000 to 30,000+ miles. Total cost $200-2,000 depending on tire replacement needs. Check alignment every 10,000 miles.</x:v>
       </x:c>
       <x:c r="F35" s="9" t="n">
         <x:v>0</x:v>
@@ -17400,21 +18762,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="1135.199951171875" hidden="0" customHeight="1">
+    <x:row r="36" ht="501.6000061035156" hidden="0" customHeight="1">
       <x:c r="A36" s="40" t="n">
         <x:v>35</x:v>
       </x:c>
       <x:c r="B36" s="9" t="str">
-        <x:v>bmw-x5m-s63-vanos-solenoid-2010</x:v>
+        <x:v>bmw-xm-airbag-passenger-knee-recall-2023</x:v>
       </x:c>
       <x:c r="C36" s="9" t="str">
-        <x:v>2010-2023 | BMW | X5 M | 4.4i, 4.6is, 4.8is, M50i, M60i, xDrive48i, xDrive50e, xDrive50i | S63</x:v>
+        <x:v>2023-2023 | BMW | XM</x:v>
       </x:c>
       <x:c r="D36" s="9" t="str">
-        <x:v>S63 VANOS Solenoid Failure - E70/F85/F95 X5 M</x:v>
+        <x:v>2023 XM Front-Passenger Knee-Airbag Recall 23V-622</x:v>
       </x:c>
       <x:c r="E36" s="9" t="str">
-        <x:v>Replace all 4 VANOS solenoids simultaneously - they are same age and if one has failed, others are close behind. Pierburg 11368605123 (OEM supplier) at $30-$50 each from Turner Motorsport or BimmerWorld. Genuine BMW 11368482268 for S63TU applications at $50-$70 each. Total parts cost: $120-$280 for all 4 solenoids. Also replace VANOS solenoid O-rings and filter screens during service. Labor: 1-2 hours professional ($150-$400 labor). This is one of the easier S63 repairs - accessible from top of engine without removing intake manifold. Natafox and Febi also offer quality aftermarket VANOS solenoids at lower cost ($20-$35 each). Clean VANOS system with fresh oil change immediately after solenoid replacement.</x:v>
+        <x:v>Check the VIN for an open 23V-622 campaign. If open, an authorized BMW dealer replaces the front-passenger knee airbag free of charge. Do not attempt airbag diagnosis or order a clock spring or airbag module from this card; supplemental-restraint work requires trained personnel and VIN-selected parts.</x:v>
       </x:c>
       <x:c r="F36" s="9" t="n">
         <x:v>0</x:v>
@@ -17423,21 +18785,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" ht="1293.5999755859375" hidden="0" customHeight="1">
+    <x:row r="37" ht="567.5999755859375" hidden="0" customHeight="1">
       <x:c r="A37" s="40" t="n">
         <x:v>36</x:v>
       </x:c>
       <x:c r="B37" s="9" t="str">
-        <x:v>bmw-x5m-s63-wastegate-rattle-2010</x:v>
+        <x:v>bmw-xm-hybrid-drivetrain-hesitation-2023</x:v>
       </x:c>
       <x:c r="C37" s="9" t="str">
-        <x:v>2010-2018 | BMW | X5 M | S63</x:v>
+        <x:v>2023-2024 | BMW | XM | S68 4.4L Twin-Turbo V8 Hybrid, S68</x:v>
       </x:c>
       <x:c r="D37" s="9" t="str">
-        <x:v>S63 Twin Turbo Wastegate Rattle - E70/F85 X5 M</x:v>
+        <x:v>Hybrid Drivetrain Hesitation and Power Delivery Lag</x:v>
       </x:c>
       <x:c r="E37" s="9" t="str">
-        <x:v>Option 1 (Most cost-effective): MAMBA SUS316 stainless steel wastegate rattle flapper repair kit for S63 MGT2260 (part 077-0024, replaces 790463-2 / 790484-3), approximately $150-$300 per turbo. Requires turbo removal for installation. Option 2: Lskioer turbo wastegate rattle flapper repair kit for S63/S63TU MGT2260DSL ($80-$150 per kit on Amazon). Option 3: Replace turbo wastegate actuators with new OEM units ($300-$500 each). Option 4: Full turbocharger replacement with new or remanufactured units ($3,000-$5,000 per turbo + labor). Labor for turbo removal and reinstallation: $2,000-$3,500 for both turbos. While turbos are out: replace turbo oil feed/return lines, coolant lines, and all gaskets (GRYPHONTEK turbo coolant line repair kit for E70 X5M, ~$200-$400).</x:v>
+        <x:v>Visit the dealer for the latest transmission and hybrid system software calibration updates. Select Sport or Sport Plus mode for more consistent power delivery. The latest software revisions significantly improve the electric-to-V8 handoff smoothness. If hesitation persists after updates, the dealer can reset the transmission adaptation values to relearn driving patterns.</x:v>
       </x:c>
       <x:c r="F37" s="9" t="n">
         <x:v>0</x:v>
@@ -17446,21 +18808,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="1069.199951171875" hidden="0" customHeight="1">
+    <x:row r="38" ht="646.7999877929688" hidden="0" customHeight="1">
       <x:c r="A38" s="40" t="n">
         <x:v>37</x:v>
       </x:c>
       <x:c r="B38" s="9" t="str">
-        <x:v>bmw-x5m-transfer-case-actuator-2010</x:v>
+        <x:v>bmw-xm-integrated-brake-system-recall-2023</x:v>
       </x:c>
       <x:c r="C38" s="9" t="str">
-        <x:v>2010-2023 | BMW | X5 M</x:v>
+        <x:v>2023-2024 | BMW | XM</x:v>
       </x:c>
       <x:c r="D38" s="9" t="str">
-        <x:v>xDrive Transfer Case Actuator Motor Failure - E70/F85/F95 X5 M</x:v>
+        <x:v>2023-2024 XM Integrated Brake System Recall 26V-422</x:v>
       </x:c>
       <x:c r="E38" s="9" t="str">
-        <x:v>Replace transfer case actuator motor. E70 X5 M: BMW 27107566296 or equivalent ($250-$450 for actuator motor). F85 X5 M: BMW 27608643153 or equivalent ($300-$500). F95 X5 M: check VIN-specific part number with dealer. FCP Euro has an excellent DIY guide for BMW transfer case actuator repair - the actuator can be replaced without removing the entire transfer case. Labor: 2-3 hours at specialist shop ($300-$600 labor). Change transfer case fluid at same time with BMW DTF-1 specification fluid. XeMODeX offers remanufactured transfer case actuator motors at reduced cost ($200-$350). For complete transfer case failure: $3,500-$6,000 for replacement unit + labor.</x:v>
+        <x:v>Check the VIN at NHTSA and with an authorized BMW dealer when campaign 26V-422 VINs become searchable, and arrange the free dealer inspection and module replacement if required. If a brake warning appears or pedal effort increases, avoid abrupt braking, allow extra stopping distance, stop safely and contact BMW roadside assistance; wheel-speed sensors are not the recall remedy.</x:v>
       </x:c>
       <x:c r="F38" s="9" t="n">
         <x:v>0</x:v>
@@ -17469,21 +18831,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="435.6000061035156" hidden="0" customHeight="1">
+    <x:row r="39" ht="646.7999877929688" hidden="0" customHeight="1">
       <x:c r="A39" s="40" t="n">
         <x:v>38</x:v>
       </x:c>
       <x:c r="B39" s="9" t="str">
-        <x:v>bmw-x6-adaptive-drive-malfunction-2008</x:v>
+        <x:v>bmw-xm-suspension-ride-quality-2023</x:v>
       </x:c>
       <x:c r="C39" s="9" t="str">
-        <x:v>2008-2019 | BMW | X6</x:v>
+        <x:v>2023-2024 | BMW | XM | S68 4.4L Twin-Turbo V8 Hybrid</x:v>
       </x:c>
       <x:c r="D39" s="9" t="str">
-        <x:v>Adaptive Drive System Malfunction</x:v>
+        <x:v>Harsh Ride Quality and Suspension Stiffness</x:v>
       </x:c>
       <x:c r="E39" s="9" t="str">
-        <x:v>Diagnose specific Adaptive Drive component failure using BMW ISTA diagnostics. Replace the failed component — most commonly the hydraulic pump or valve block. If repair cost is prohibitive, some owners convert to conventional anti-roll bars as a permanent fix at lower cost.</x:v>
+        <x:v>Check tire pressures regularly - overinflated tires significantly worsen the harsh ride. Some owners report improved comfort by switching to a tire with a taller sidewall profile (if available for the XM's wheel size). Use Comfort mode for daily driving. Unfortunately, no aftermarket spring or damper solution currently exists to significantly improve the ride without compromising the handling needed for the XM's weight.</x:v>
       </x:c>
       <x:c r="F39" s="9" t="n">
         <x:v>0</x:v>
@@ -17492,21 +18854,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="858" hidden="0" customHeight="1">
+    <x:row r="40" ht="528" hidden="0" customHeight="1">
       <x:c r="A40" s="40" t="n">
         <x:v>39</x:v>
       </x:c>
       <x:c r="B40" s="9" t="str">
-        <x:v>bmw-x6-air-suspension-2008</x:v>
+        <x:v>bmw-z3-convertible-top-rear-window-cracking-clouding-bead-separatio</x:v>
       </x:c>
       <x:c r="C40" s="9" t="str">
-        <x:v>2008-2023 | BMW | X6</x:v>
+        <x:v>1996-2002 | BMW | Z3</x:v>
       </x:c>
       <x:c r="D40" s="9" t="str">
-        <x:v>Air Suspension Compressor &amp; Strut Failure</x:v>
+        <x:v>Convertible Top Rear Window Cracking, Clouding, and Bead Separation</x:v>
       </x:c>
       <x:c r="E40" s="9" t="str">
-        <x:v>Replace failed air springs or compressor. Arnott rear air spring A-2642 ($200-300 each). OEM F16 spring 37126795013 ($200). Arnott compressor P-2655 ($599). Or convert to coil springs: Strutmasters BB2RBM conversion kit ($1,200-1,800) permanently eliminates air suspension issues. Conversion is cheaper long-term than continued air suspension repairs. If keeping air suspension: inspect air springs at 60,000-80,000 miles for cracks/leaks before compressor damage occurs. Replace both air springs on same axle simultaneously.</x:v>
+        <x:v>Replace the rear window panel only — BMW used a zipper system so the clouded/cracked window unzips and a new window zips/tapes in without disturbing the fabric top. Re-gluing separated bead trim rarely holds, so window replacement is the durable fix. Job is a DIY-feasible 1-1.5 hours; replace the whole top only if the fabric is also degraded.</x:v>
       </x:c>
       <x:c r="F40" s="9" t="n">
         <x:v>0</x:v>
@@ -17515,22 +18877,20 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="646.7999877929688" hidden="0" customHeight="1">
+    <x:row r="41" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A41" s="40" t="n">
         <x:v>40</x:v>
       </x:c>
       <x:c r="B41" s="9" t="str">
-        <x:v>bmw-x6-ibs-brake-recall-2023</x:v>
+        <x:v>bmw-z3-cooling-system-failure-1996</x:v>
       </x:c>
       <x:c r="C41" s="9" t="str">
-        <x:v>2024-2024 | BMW | X6</x:v>
+        <x:v>1996-2002 | BMW | Z3</x:v>
       </x:c>
       <x:c r="D41" s="9" t="str">
-        <x:v>2024 X6 Integrated Brake System Recall 26V-422</x:v>
-      </x:c>
-      <x:c r="E41" s="9" t="str">
-        <x:v>Check the VIN at NHTSA and with an authorized BMW dealer when campaign 26V-422 VINs become searchable, and arrange the free dealer inspection and module replacement if required. If a brake warning appears or pedal effort increases, avoid abrupt braking, allow extra stopping distance, stop safely and contact BMW roadside assistance; do not order brake electronics from this card.</x:v>
-      </x:c>
+        <x:v>Cooling System Component Failures</x:v>
+      </x:c>
+      <x:c r="E41" s="9" t="str"/>
       <x:c r="F41" s="9" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -17538,21 +18898,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="42" ht="924" hidden="0" customHeight="1">
+    <x:row r="42" ht="448.79998779296875" hidden="0" customHeight="1">
       <x:c r="A42" s="40" t="n">
         <x:v>41</x:v>
       </x:c>
       <x:c r="B42" s="9" t="str">
-        <x:v>bmw-x6-n63-timing-chain-2008</x:v>
+        <x:v>bmw-z3-cracked-exhaust-manifold-1-9l-4-cylinder</x:v>
       </x:c>
       <x:c r="C42" s="9" t="str">
-        <x:v>2008-2018 | BMW | X6 | M50i, xDrive50i</x:v>
+        <x:v>1996-2002 | BMW | Z3 | 1.9, 1.9i, Z3 1.9 | 1.9L M44 4-cylinder, 1.9L M43TU 4-cylinder</x:v>
       </x:c>
       <x:c r="D42" s="9" t="str">
-        <x:v>N63 Timing Chain Stretch &amp; Guide Failure (E71/F16 xDrive50i)</x:v>
+        <x:v>Cracked Exhaust Manifold on 1.9L 4-Cylinder (M44/M43)</x:v>
       </x:c>
       <x:c r="E42" s="9" t="str">
-        <x:v>PREVENTIVE REPLACEMENT: If you own 2008-2014 E71 xDrive50i with N63, replace timing chain guides and tensioners IMMEDIATELY at 60,000-80,000 miles ($4,000-6,000) BEFORE failure. IWIS timing chain kit 90001521 ($800-1,200) or Turner kit 11317594899KT recommended. Replace lower chain guide 11147574373 at same time. If chain has already failed: complete engine replacement required ($15,000-25,000). Check VIN with BMW dealer for extended warranty eligibility. 2015+ N63TU engines have improved timing components but still require monitoring.</x:v>
+        <x:v>Inspect the manifold for hairline cracks (a cold-engine listen or smoke test confirms the leak). Replace the cracked manifold with a used OE unit or an aftermarket stainless tubular header, and renew the manifold gasket and hardware. Allow roughly 3-4 hours labor.</x:v>
       </x:c>
       <x:c r="F42" s="9" t="n">
         <x:v>0</x:v>
@@ -17561,21 +18921,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="43" ht="409.20001220703125" hidden="0" customHeight="1">
+    <x:row r="43" ht="686.4000244140625" hidden="0" customHeight="1">
       <x:c r="A43" s="40" t="n">
         <x:v>42</x:v>
       </x:c>
       <x:c r="B43" s="9" t="str">
-        <x:v>bmw-x6-n63-valve-stem-seal-wear-2008</x:v>
+        <x:v>bmw-z3-differential-mount-ear-trunk-floor-pan-tearing</x:v>
       </x:c>
       <x:c r="C43" s="9" t="str">
-        <x:v>2008-2019 | BMW | X6 | N63</x:v>
+        <x:v>1996-2002 | BMW | Z3</x:v>
       </x:c>
       <x:c r="D43" s="9" t="str">
-        <x:v>N63 Valve Stem Seal Degradation and Oil Burning</x:v>
+        <x:v>Differential Mount Ear and Trunk Floor Pan Tearing</x:v>
       </x:c>
       <x:c r="E43" s="9" t="str">
-        <x:v>Replace all intake and exhaust valve stem seals. This is a major job requiring head work. Also replace turbo oil return lines and update engine software per BMW N63 Customer Care Package specifications. Ensure proper oil grade (BMW LL-01) is used.</x:v>
+        <x:v>Inspect the trunk floor around the differential mount and rear subframe pickup points for cracks, torn metal, and broken spot welds. Repair requires welding and a reinforcement/re-fabrication plate kit to tie the diff mount/subframe back into the floor. Switching the diff carrier bushings to polyurethane reduces carrier movement and the stress that causes the tearing. Catching it early greatly limits the repair scope.</x:v>
       </x:c>
       <x:c r="F43" s="9" t="n">
         <x:v>0</x:v>
@@ -17584,21 +18944,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="44" ht="858" hidden="0" customHeight="1">
+    <x:row r="44" ht="514.7999877929688" hidden="0" customHeight="1">
       <x:c r="A44" s="40" t="n">
         <x:v>43</x:v>
       </x:c>
       <x:c r="B44" s="9" t="str">
-        <x:v>bmw-x6-n63-valve-stem-seals-2008</x:v>
+        <x:v>bmw-z3-door-window-regulator-clip-mounting-tab-failure</x:v>
       </x:c>
       <x:c r="C44" s="9" t="str">
-        <x:v>2008-2023 | BMW | X6 | M50i, xDrive50i | N63</x:v>
+        <x:v>1996-2002 | BMW | Z3</x:v>
       </x:c>
       <x:c r="D44" s="9" t="str">
-        <x:v>N63 Valve Stem Seal / Oil Consumption (xDrive50i)</x:v>
+        <x:v>Door Window Regulator Clip / Mounting Tab Failure</x:v>
       </x:c>
       <x:c r="E44" s="9" t="str">
-        <x:v>Replace valve stem seals - extremely labor-intensive job requiring cylinder head work ($4,900-12,000 total). Elring seals 11340039494 ($80-120/set of 16, need 2 sets for V8). 5150 AutoSport Viton upgraded seals ($150-200) are recommended for better heat resistance in hot-vee configuration. AGA Tools kit AGA-N63-VSK-K ($500-800) includes specialized tools required. Reference TSB MC-10149960-9999 when visiting dealer. Some owners monitor oil levels and add as needed rather than repair. Use quality synthetic 0W-40 BMW LL-01 spec oil.</x:v>
+        <x:v>Replace the broken plastic regulator clips, or replace the regulator assembly if the cable or mechanism is also worn. If the welded mounting tab/anchor has torn from the door frame, it must be re-welded or reinforced before fitting a new regulator. Lubricate the window channels to reduce drag on the new parts.</x:v>
       </x:c>
       <x:c r="F44" s="9" t="n">
         <x:v>0</x:v>
@@ -17607,21 +18967,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="45" ht="818.4000244140625" hidden="0" customHeight="1">
+    <x:row r="45" ht="686.4000244140625" hidden="0" customHeight="1">
       <x:c r="A45" s="40" t="n">
         <x:v>44</x:v>
       </x:c>
       <x:c r="B45" s="9" t="str">
-        <x:v>bmw-x6-n63-wastegate-2008</x:v>
+        <x:v>bmw-z3-fuel-level-sender-failure-causing-erratic-dead-fuel-gauge</x:v>
       </x:c>
       <x:c r="C45" s="9" t="str">
-        <x:v>2008-2018 | BMW | X6 | M50i, xDrive50i</x:v>
+        <x:v>1996-2002 | BMW | Z3</x:v>
       </x:c>
       <x:c r="D45" s="9" t="str">
-        <x:v>N63 Turbo Wastegate Rattle (xDrive50i)</x:v>
+        <x:v>Fuel Level Sender Failure Causing Erratic or Dead Fuel Gauge</x:v>
       </x:c>
       <x:c r="E45" s="9" t="str">
-        <x:v>Repair options range from flapper repair kits ($50-100/turbo) to complete turbocharger replacement ($4,000-8,000 for both). Garrett MGT2256S flapper repair kit ($50-100 per turbo) is cheapest fix. MAMBA adjustable actuator kit ($150-300) provides more durable solution. OEM actuators 11657646093 available from BMW. Complete turbo replacement $2,000-4,000 per turbo. MONITORING: Wastegate rattle is early warning - address before complete turbo failure to avoid $8,000+ repair.</x:v>
+        <x:v>Remove the access panel behind the seats and inspect the sender. A dirty or lightly worn ceramic/resistor plate can sometimes be cleaned, but a cracked plate or worn brushes requires replacing the sender unit (or the complete fuel-pump/sender carrier assembly). Also check the tank vent valve, as tank vacuum can deform the float arm. Confirm wiring/ground integrity before condemning the sender.</x:v>
       </x:c>
       <x:c r="F45" s="9" t="n">
         <x:v>0</x:v>
@@ -17630,21 +18990,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" ht="409.20001220703125" hidden="0" customHeight="1">
+    <x:row r="46" ht="488.3999938964844" hidden="0" customHeight="1">
       <x:c r="A46" s="40" t="n">
         <x:v>45</x:v>
       </x:c>
       <x:c r="B46" s="9" t="str">
-        <x:v>bmw-x6-rear-differential-bushing-2008</x:v>
+        <x:v>bmw-z3-hvac-blower-final-stage-resistor-failure</x:v>
       </x:c>
       <x:c r="C46" s="9" t="str">
-        <x:v>2008-2026 | BMW | X6</x:v>
+        <x:v>1996-2002 | BMW | Z3</x:v>
       </x:c>
       <x:c r="D46" s="9" t="str">
-        <x:v>Rear Differential Bushing Deterioration</x:v>
+        <x:v>HVAC Blower Final Stage Resistor Failure (Fan Only Works on Max)</x:v>
       </x:c>
       <x:c r="E46" s="9" t="str">
-        <x:v>Replace all rear differential mount bushings. Use OEM or equivalent quality bushings (Lemforder is the OEM supplier). Inspect the differential housing for any damage from excessive movement. Perform subframe alignment check after bushing replacement.</x:v>
+        <x:v>Replace the blower final stage resistor (A/C cars: part under the scuttle/cowl; non-A/C cars: behind the passenger footwell panel). If a new resistor does not restore all speeds, test the blower motor itself, which may also be worn. Inspect for corrosion/water intrusion at the cowl on A/C cars.</x:v>
       </x:c>
       <x:c r="F46" s="9" t="n">
         <x:v>0</x:v>
@@ -17653,21 +19013,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="47" ht="765.5999755859375" hidden="0" customHeight="1">
+    <x:row r="47" ht="1584" hidden="0" customHeight="1">
       <x:c r="A47" s="40" t="n">
         <x:v>46</x:v>
       </x:c>
       <x:c r="B47" s="9" t="str">
-        <x:v>bmw-x6-transfer-case-2008</x:v>
+        <x:v>bmw-z3-rear-subframe-crack-1996</x:v>
       </x:c>
       <x:c r="C47" s="9" t="str">
-        <x:v>2008-2023 | BMW | X6</x:v>
+        <x:v>1996-2002 | BMW | Z3</x:v>
       </x:c>
       <x:c r="D47" s="9" t="str">
-        <x:v>Transfer Case Actuator Motor Failure (All xDrive Models)</x:v>
+        <x:v>Rear Subframe Mounting Point Cracking</x:v>
       </x:c>
       <x:c r="E47" s="9" t="str">
-        <x:v>Replace the actuator motor assembly or rebuild using an aftermarket gear repair kit ($100-150). G06 actuator motor 27609469023 ($400-600) for complete replacement. DIY gear repair kits are straightforward and save $1,200+ over dealer replacement. Complete transfer case replacement if internal damage occurred: $1,400-3,300. PREVENTIVE: If buying used X6 over 80k miles, budget for this repair and listen for clicking noise when shutting off ignition.</x:v>
+        <x:v>Inspect the trunk floor, differential mount area, and all rear subframe mounting points from above and below the car for spot-weld separation, torn sheet metal, and cracked seams; a dye penetrant test or removing trunk trim/seam sealer may be needed to reveal early damage. If cracking is present, the proper repair is to drop the rear axle carrier/subframe, weld and reinforce the damaged unibody mounting points and trunk floor with a reinforcement kit (commonly Randy Forbes-style dual-ear/differential mount reinforcement or equivalent), then reinstall with new subframe bushings, differential mount bushings, and perform a 4-wheel alignment. Minor early cracks may be repairable before major deformation, but advanced damage often requires fabrication and extensive welding by a chassis/body specialist; typical cost ranges from about $2,000-$3,500 for early reinforcement repairs and can exceed $4,000-$6,000 if the floor is torn or multiple mounting points are damaged.</x:v>
       </x:c>
       <x:c r="F47" s="9" t="n">
         <x:v>0</x:v>
@@ -17676,22 +19036,20 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="48" ht="514.7999877929688" hidden="0" customHeight="1">
+    <x:row r="48" ht="66" hidden="0" customHeight="1">
       <x:c r="A48" s="40" t="n">
         <x:v>47</x:v>
       </x:c>
       <x:c r="B48" s="9" t="str">
-        <x:v>bmw-x6m-front-thrust-arm-bushing-2015</x:v>
+        <x:v>bmw-z3-rear-subframe-cracking-1996</x:v>
       </x:c>
       <x:c r="C48" s="9" t="str">
-        <x:v>2015-2025 | BMW | X6 M</x:v>
+        <x:v>1996-2002 | BMW | Z3 | M52, M54</x:v>
       </x:c>
       <x:c r="D48" s="9" t="str">
-        <x:v>Front Thrust Arm Bushing (Tension Strut) Premature Wear</x:v>
-      </x:c>
-      <x:c r="E48" s="9" t="str">
-        <x:v>Replace both front thrust arms as complete assemblies (the bushings are not serviceable separately). Use genuine BMW M-spec parts or Lemforder equivalents. Perform a 4-wheel alignment immediately after replacement. Upgrade to Powerflex polyurethane thrust arm bushings for extended lifespan, especially on tracked cars.</x:v>
-      </x:c>
+        <x:v>Rear Subframe Mounting Point Cracks</x:v>
+      </x:c>
+      <x:c r="E48" s="9" t="str"/>
       <x:c r="F48" s="9" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -17699,21 +19057,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="49" ht="897.5999755859375" hidden="0" customHeight="1">
+    <x:row r="49" ht="475.20001220703125" hidden="0" customHeight="1">
       <x:c r="A49" s="40" t="n">
         <x:v>48</x:v>
       </x:c>
       <x:c r="B49" s="9" t="str">
-        <x:v>bmw-x6m-s63-rod-bearing-2010</x:v>
+        <x:v>bmw-z3-valve-cover-gasket-oil-leak</x:v>
       </x:c>
       <x:c r="C49" s="9" t="str">
-        <x:v>2010-2023 | BMW | X6 M | M50i, xDrive50i | S63</x:v>
+        <x:v>1997-2002 | BMW | Z3 | 2.3, 2.5i, 2.8, 3.0i | M52 2.8, M52TU 2.5/2.8, M54 2.5/3.0</x:v>
       </x:c>
       <x:c r="D49" s="9" t="str">
-        <x:v>S63 Rod Bearing Failure (X6 M)</x:v>
+        <x:v>Valve Cover Gasket Oil Leak (M52/M54 6-Cylinder)</x:v>
       </x:c>
       <x:c r="E49" s="9" t="str">
-        <x:v>PREVENTIVE: Replace rod bearings every 60,000-80,000 miles ($2,500-5,000 labor-intensive job). Use ACL Race 8B1578HX-STD ($150-250) or King CR8049SV ($120-200) upgraded bearings - these are stronger than OEM and provide better durability under high loads. Send oil samples for analysis (Blackstone Labs ~$30) every 5,000 miles to monitor bearing wear metals. If bearings have already failed: engine replacement required ($15,000-30,000). DO NOT buy used X6 M without documented bearing replacement history or fresh oil analysis.</x:v>
+        <x:v>Replace the valve cover gasket, the spark-plug-well/grommet seals, and the cover bolt seals. On M54 engines also clean oil from the plug wells and replace any oil-contaminated coil boots/coils. Use the correct torque sequence to avoid re-leaking. Inspect the cover for warping or cracks while it is off.</x:v>
       </x:c>
       <x:c r="F49" s="9" t="n">
         <x:v>0</x:v>
@@ -17722,21 +19080,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="50" ht="277.20001220703125" hidden="0" customHeight="1">
+    <x:row r="50" ht="1293.5999755859375" hidden="0" customHeight="1">
       <x:c r="A50" s="40" t="n">
         <x:v>49</x:v>
       </x:c>
       <x:c r="B50" s="9" t="str">
-        <x:v>bmw-x6m-vanos-solenoid-2015</x:v>
+        <x:v>bmw-z3-vanos-seals-1999</x:v>
       </x:c>
       <x:c r="C50" s="9" t="str">
-        <x:v>2015-2021 | BMW | X6 M | S63</x:v>
+        <x:v>1999-2002 | BMW | Z3 | M52, M54, S52</x:v>
       </x:c>
       <x:c r="D50" s="9" t="str">
-        <x:v>VANOS Solenoid Oil Sludge Buildup</x:v>
+        <x:v>VANOS Seal Failure (M52/M54/S52)</x:v>
       </x:c>
       <x:c r="E50" s="9" t="str">
-        <x:v>Remove and clean or replace the VANOS solenoids. Perform an engine oil flush. Strictly follow 7,500-mile oil change intervals with BMW LL-01 rated 0W-40 synthetic oil.</x:v>
+        <x:v>Confirm the fault by checking for cold-start VANOS rattle, rough idle, hesitation, and scanning for cam timing or mixture-related fault codes; on M52TU/M54/S52 engines, inspect VANOS operation and rule out vacuum leaks before disassembly. Repair typically involves removing the valve cover and VANOS unit, replacing the internal piston seals/O-rings with updated Viton/Teflon seals, renewing the valve cover gasket and VANOS oil line sealing washers, and then re-timing the cams to BMW specifications if required. If the unit still rattles after resealing, the VANOS bearing/anti-rattle components or the complete VANOS assembly may need replacement. Typical cost is about $60-$150 in seals/gaskets for DIY repair, $300-$700 for an independent shop reseal, or $800-$1,500+ if a rebuilt/replacement VANOS unit is installed.</x:v>
       </x:c>
       <x:c r="F50" s="9" t="n">
         <x:v>0</x:v>
@@ -17745,21 +19103,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="51" ht="699.5999755859375" hidden="0" customHeight="1">
+    <x:row r="51" ht="501.6000061035156" hidden="0" customHeight="1">
       <x:c r="A51" s="40" t="n">
         <x:v>50</x:v>
       </x:c>
       <x:c r="B51" s="9" t="str">
-        <x:v>bmw-x7-48v-battery-2020</x:v>
+        <x:v>bmw-z4-b58-coolant-tank-2019</x:v>
       </x:c>
       <x:c r="C51" s="9" t="str">
-        <x:v>2020-2023 | BMW | X7</x:v>
+        <x:v>2019-2026 | BMW | Z4 | B58</x:v>
       </x:c>
       <x:c r="D51" s="9" t="str">
-        <x:v>48V Mild Hybrid Battery Issues</x:v>
+        <x:v>B58 Coolant Expansion Tank Cracking</x:v>
       </x:c>
       <x:c r="E51" s="9" t="str">
-        <x:v>Replace the 48V mild hybrid battery ($1,000-2,000 at dealer). Requires dealer-level diagnostic tools and coding after installation - this is NOT a DIY repair. The 48V battery is separate from the main 12V battery. No aftermarket alternatives currently available. Check if vehicle is still under BMW warranty or extended warranty coverage. Some owners choose to live with the failed auto start-stop rather than pay for replacement.</x:v>
+        <x:v>Replace the coolant expansion tank with an updated BMW part or aftermarket aluminum tank. Inspect the tank and cap regularly for signs of cracking, discoloration, or seepage. When replacing, also replace the cap and check all coolant hoses for brittleness. Flush and refill with BMW-approved coolant.</x:v>
       </x:c>
       <x:c r="F51" s="9" t="n">
         <x:v>0</x:v>
@@ -17768,21 +19126,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="52" ht="726" hidden="0" customHeight="1">
+    <x:row r="52" ht="1306.800048828125" hidden="0" customHeight="1">
       <x:c r="A52" s="40" t="n">
         <x:v>51</x:v>
       </x:c>
       <x:c r="B52" s="9" t="str">
-        <x:v>bmw-x7-air-suspension-2019</x:v>
+        <x:v>bmw-z4-e85-convertible-top-hydraulic-2003</x:v>
       </x:c>
       <x:c r="C52" s="9" t="str">
-        <x:v>2019-2023 | BMW | X7</x:v>
+        <x:v>2003-2008 | BMW | Z4</x:v>
       </x:c>
       <x:c r="D52" s="9" t="str">
-        <x:v>Air Suspension Compressor &amp; Strut Failure (Standard Equipment)</x:v>
+        <x:v>Convertible Top Hydraulic Pump Motor Failure - E85 Z4</x:v>
       </x:c>
       <x:c r="E52" s="9" t="str">
-        <x:v>Replace failed air struts and/or compressor. Front strut left 37106869035 ($1,500-2,000), right 37106869036 ($1,500-2,000), rear 37106869039 ($1,000-1,500). Compressor 37206861882 ($800-1,200). RebuildMasterTech rebuilt struts ($600-900 each) are a more affordable alternative. Total repair can reach $2,180-5,000+ depending on which components have failed. Replace both struts on same axle simultaneously. Inspect at 50,000 miles for early signs of leaking.</x:v>
+        <x:v>Replace hydraulic pump motor assembly (BMW 54347193448 / supersedes 54347119633). OEM Genuine BMW pump: $800-$1,200. Aftermarket alternatives available on Amazon for $150-$300 but quality varies significantly. Dealer labor is $1,500-$2,500+ as BMW procedure requires full top removal. ZRoadster.org members have documented a motor relocation to the boot/trunk area which allows much easier future access. Hydraulic fluid: use Aral Vitamol ZHM or BMW 54340394395 hydraulic oil. PREVENTION: Clean drain holes annually, ensure rubber bungs are properly seated, and check for water intrusion in pump area at every service. Some owners have had success with pump motor rebuilds from roofmotors.co.uk ($300-$500) but quality of rebuilds varies.</x:v>
       </x:c>
       <x:c r="F52" s="9" t="n">
         <x:v>0</x:v>
@@ -17791,21 +19149,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="53" ht="435.6000061035156" hidden="0" customHeight="1">
+    <x:row r="53" ht="1135.199951171875" hidden="0" customHeight="1">
       <x:c r="A53" s="40" t="n">
         <x:v>52</x:v>
       </x:c>
       <x:c r="B53" s="9" t="str">
-        <x:v>bmw-x7-air-suspension-compressor-2019</x:v>
+        <x:v>bmw-z4-e85-window-regulator-2003</x:v>
       </x:c>
       <x:c r="C53" s="9" t="str">
-        <x:v>2019-2026 | BMW | X7</x:v>
+        <x:v>2003-2008 | BMW | Z4</x:v>
       </x:c>
       <x:c r="D53" s="9" t="str">
-        <x:v>Air Suspension Compressor Failure</x:v>
+        <x:v>Power Window Regulator Failure - E85 Z4</x:v>
       </x:c>
       <x:c r="E53" s="9" t="str">
-        <x:v>Replace the air suspension compressor. Inspect all four air springs for leaks using soapy water solution. Replace any leaking air springs to prevent repeated compressor failure. Check the valve block for proper operation. The compressor is located under the rear of the vehicle.</x:v>
+        <x:v>Option 1 (Budget): Window regulator repair kit - replacement cables and rollers for ~$18-$25 from eBay/Amazon (BWR974 for left/driver side). Requires removing door panel and threading new cables through existing regulator frame. DIY-friendly with Z4-forum.com guides. Option 2 (Recommended): Full window regulator replacement. Driver side: BMW 51337198909 ($180-$280 OEM, $80-$150 aftermarket). Passenger side: BMW 51337198910 ($180-$280 OEM, $80-$150 aftermarket). Labor: $200-$400 at independent shop, $500-$700+ at dealer. DIY: 2-3 hours with door panel removal guide from Pelican Parts. ZRoadster.org recommends full replacement over repair kit for long-term reliability.</x:v>
       </x:c>
       <x:c r="F53" s="9" t="n">
         <x:v>0</x:v>
@@ -17814,21 +19172,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="54" ht="871.2000122070312" hidden="0" customHeight="1">
+    <x:row r="54" ht="514.7999877929688" hidden="0" customHeight="1">
       <x:c r="A54" s="40" t="n">
         <x:v>53</x:v>
       </x:c>
       <x:c r="B54" s="9" t="str">
-        <x:v>bmw-x7-b58-coolant-2019</x:v>
+        <x:v>bmw-z4-electric-steering-rack-2003</x:v>
       </x:c>
       <x:c r="C54" s="9" t="str">
-        <x:v>2019-2023 | BMW | X7 | xDrive40i | B58</x:v>
+        <x:v>2012-2012 | BMW | Z4</x:v>
       </x:c>
       <x:c r="D54" s="9" t="str">
-        <x:v>B58 Coolant System Failures (xDrive40i)</x:v>
+        <x:v>2012 Z4 Electric Power-Steering Recall 12V-302</x:v>
       </x:c>
       <x:c r="E54" s="9" t="str">
-        <x:v>Replace failed coolant system components. Water pump 11518482250 ($300-400). Thermostat 11537644811 ($150-250). Replace expansion tank and all plastic coolant connections when performing repair to prevent cascading failures. For 2023+ models, check VIN for recall 24V-608 coverage for coolant pump connector. Total repair $500-2,500 depending on extent of damage. PREVENTIVE: Replace thermostat and water pump at 60,000-70,000 miles before failure. Inspect coolant hoses and connections at every oil change after 50k miles.</x:v>
+        <x:v>Check the VIN for an open 12V-302 campaign. If open, an authorized BMW dealer replaces the steering-assistance module free of charge. If the steering warning and audible alert occur, maintain control, reduce speed, stop safely and arrange dealer or roadside assistance; do not replace a steering rack from this card.</x:v>
       </x:c>
       <x:c r="F54" s="9" t="n">
         <x:v>0</x:v>
@@ -17837,21 +19195,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="55" ht="435.6000061035156" hidden="0" customHeight="1">
+    <x:row r="55" ht="633.5999755859375" hidden="0" customHeight="1">
       <x:c r="A55" s="40" t="n">
         <x:v>54</x:v>
       </x:c>
       <x:c r="B55" s="9" t="str">
-        <x:v>bmw-x7-b58-coolant-expansion-tank-2019</x:v>
+        <x:v>bmw-z4-electric-water-pump-2006</x:v>
       </x:c>
       <x:c r="C55" s="9" t="str">
-        <x:v>2019-2026 | BMW | X7 | B58</x:v>
+        <x:v>2012-2016 | BMW | Z4 | N20</x:v>
       </x:c>
       <x:c r="D55" s="9" t="str">
-        <x:v>B58 Coolant Expansion Tank Crack</x:v>
+        <x:v>2012-2016 Z4 sDrive28i Water-Pump Connector Recall 24V-608</x:v>
       </x:c>
       <x:c r="E55" s="9" t="str">
-        <x:v>Replace the coolant expansion tank with an updated BMW part that uses improved plastic composition. Also replace the cap and inspect all coolant hoses. Flush and refill the cooling system with BMW-approved coolant. Check for coolant contamination from the old tank.</x:v>
+        <x:v>Check the VIN for an open 24V-608 campaign. If open, an authorized BMW dealer inspects the water pump and connector, replaces them if necessary, and installs the protective shield free of charge. If smoke appears from the engine compartment, stop safely, switch off the vehicle, have occupants exit, move away from traffic and call emergency or roadside assistance; do not order a pump from this card.</x:v>
       </x:c>
       <x:c r="F55" s="9" t="n">
         <x:v>0</x:v>
@@ -17860,44 +19218,44 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="56" ht="646.7999877929688" hidden="0" customHeight="1">
+    <x:row r="56" ht="1359.5999755859375" hidden="0" customHeight="1">
       <x:c r="A56" s="40" t="n">
         <x:v>55</x:v>
       </x:c>
       <x:c r="B56" s="9" t="str">
-        <x:v>bmw-x7-ibs-brake-recall-2023</x:v>
+        <x:v>bmw-z4-g29-b58-water-pump-2019</x:v>
       </x:c>
       <x:c r="C56" s="9" t="str">
-        <x:v>2023-2025 | BMW | X7</x:v>
+        <x:v>2019-2025 | BMW | Z4 | M40i, sDrive35i, sDrive35is | B48, B58</x:v>
       </x:c>
       <x:c r="D56" s="9" t="str">
-        <x:v>2023-2025 X7 Integrated Brake System Recall 26V-422</x:v>
+        <x:v>B48/B58 Electric Water Pump &amp; Thermostat Failure - G29 Z4</x:v>
       </x:c>
       <x:c r="E56" s="9" t="str">
-        <x:v>Check the VIN at NHTSA and with an authorized BMW dealer when campaign 26V-422 VINs become searchable, and arrange the free dealer inspection and module replacement if required. If a brake warning appears or pedal effort increases, avoid abrupt braking, allow extra stopping distance, stop safely and contact BMW roadside assistance; do not order brake electronics from this card.</x:v>
+        <x:v>Preventative replacement recommended at 60,000 miles. Always replace water pump and thermostat together - they share labor overlap and frequently fail concurrently. B48 sDrive30i: Water pump BMW 11518632586 ($300-$450), Thermostat BMW 11538685978 ($100-$150). B58 M40i: Water pump BMW 11518650986 ($350-$500), Thermostat BMW 11538685978 ($100-$150). Mishimoto offers performance water pump alternatives for B58 with improved impeller design. Replace 3 O-rings between thermostat and pump housing, plus 2 O-rings on coolant tube to head. Must replace water pump mounting bolts (torque-to-yield). Labor: 3-4 hours. FCP Euro lifetime warranty kits available. Also inspect plastic cylinder head coolant outlet adapter - known to shear off causing massive coolant leak.</x:v>
       </x:c>
       <x:c r="F56" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G56" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="57" ht="897.5999755859375" hidden="0" customHeight="1">
+    <x:row r="57" ht="1122" hidden="0" customHeight="1">
       <x:c r="A57" s="40" t="n">
         <x:v>56</x:v>
       </x:c>
       <x:c r="B57" s="9" t="str">
-        <x:v>bmw-x7-n63-oil-consumption-2019</x:v>
+        <x:v>bmw-z4-n54-hpfp-2009</x:v>
       </x:c>
       <x:c r="C57" s="9" t="str">
-        <x:v>2019-2023 | BMW | X7 | M50i, M60i, xDrive50i | N63TU3</x:v>
+        <x:v>2009-2011 | BMW | Z4 | M40i, sDrive35i, sDrive35is | N54</x:v>
       </x:c>
       <x:c r="D57" s="9" t="str">
-        <x:v>N63TU3 Oil Consumption &amp; Valve Stem Seal Degradation (xDrive50i/M50i/M60i)</x:v>
+        <x:v>N54 High Pressure Fuel Pump (HPFP) Failure - E89 Z4 sDrive35i/35is</x:v>
       </x:c>
       <x:c r="E57" s="9" t="str">
-        <x:v>Replace valve stem seals - extremely labor-intensive job requiring cylinder head work ($4,900-12,000 total). Elring seals 11340039494 for OEM spec. 5150 AutoSport Viton upgraded seals ($150-200) recommended for better heat resistance. AGA Tools kit includes specialized tools required. Reference TSB MC-10149960-9999 when visiting dealer. Check eligibility for class action settlement coverage. Some owners monitor oil levels and top off rather than repair. Use quality synthetic 0W-40 BMW LL-01 spec oil and check level every 500-1,000 miles.</x:v>
+        <x:v>Replace HPFP with latest revision Genuine BMW unit. The pump went through multiple revisions - ONLY install the latest version. Part number evolution: Original -&gt; 13517592881 (Index 10, TSB fix) -&gt; 13517616170 (latest revision, most reliable). Genuine BMW 13517616170 is the definitive fix ($350-$550 for pump). Replacement is straightforward DIY (1-2 hours) with basic tools. Also available as complete kit from FCP Euro with lifetime warranty. BMW extended warranty coverage to 10 years/120,000 miles under customer care package for original owners - check VIN eligibility. Replace low-pressure fuel sensor at same time (13537537319) as it may have been damaged by pressure fluctuations ($35-$55).</x:v>
       </x:c>
       <x:c r="F57" s="9" t="n">
         <x:v>0</x:v>
@@ -17906,21 +19264,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="58" ht="396" hidden="0" customHeight="1">
+    <x:row r="58" ht="580.7999877929688" hidden="0" customHeight="1">
       <x:c r="A58" s="40" t="n">
         <x:v>57</x:v>
       </x:c>
       <x:c r="B58" s="9" t="str">
-        <x:v>bmw-x7-panoramic-roof-rattle-2019</x:v>
+        <x:v>bmw-z4-n54-wastegate-rattle-2009</x:v>
       </x:c>
       <x:c r="C58" s="9" t="str">
-        <x:v>2019-2026 | BMW | X7</x:v>
+        <x:v>2009-2010 | BMW | Z4 | N54</x:v>
       </x:c>
       <x:c r="D58" s="9" t="str">
-        <x:v>Panoramic Sunroof Rattle and Creak</x:v>
+        <x:v>2009-2010 Z4 sDrive35i N54 Wastegate Diagnosis</x:v>
       </x:c>
       <x:c r="E58" s="9" t="str">
-        <x:v>Apply BMW-approved felt tape or lubricant to sunroof guide rails. Replace worn guide rail bushings. In severe cases, the sunroof cassette or seal may need replacement under warranty. BMW has issued updated guide rail components for early production vehicles.</x:v>
+        <x:v>Confirm the VIN, engine, production date, DME faults, boost-control data and noise source using current BMW diagnostic information. Check VIN-specific coverage history with BMW, recognizing that the bulletin's time/mileage window may have expired. Do not replace a turbocharger, actuator or wastegate from this card without the required diagnosis.</x:v>
       </x:c>
       <x:c r="F58" s="9" t="n">
         <x:v>0</x:v>
@@ -17929,21 +19287,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="59" ht="778.7999877929688" hidden="0" customHeight="1">
+    <x:row r="59" ht="501.6000061035156" hidden="0" customHeight="1">
       <x:c r="A59" s="40" t="n">
         <x:v>58</x:v>
       </x:c>
       <x:c r="B59" s="9" t="str">
-        <x:v>bmw-x7-sunroof-leak-2019</x:v>
+        <x:v>bmw-z4-soft-top-hydraulic-2003</x:v>
       </x:c>
       <x:c r="C59" s="9" t="str">
-        <x:v>2019-2023 | BMW | X7</x:v>
+        <x:v>2009-2016 | BMW | Z4</x:v>
       </x:c>
       <x:c r="D59" s="9" t="str">
-        <x:v>Panoramic Sunroof Water Leak</x:v>
+        <x:v>Retractable Hard Top Hydraulic Mechanism Failure</x:v>
       </x:c>
       <x:c r="E59" s="9" t="str">
-        <x:v>Clear clogged sunroof drain tubes ($100-300 at shop). Reference TSB SIB 54 11 19 when visiting dealer. For persistent leaks, drain tube connections or sunroof seal may need replacement ($500-1,500). If water has damaged interior electronics, repair costs can reach $3,000. PREVENTIVE: Clear sunroof drains annually, especially in areas with heavy tree debris. Run compressed air or flexible drain snake through drain tubes during oil changes. Keep sunroof track clean of debris.</x:v>
+        <x:v>Diagnose the leak location and replace the failed component. Common failure points are the main hydraulic cylinders (left and right), the hydraulic pump motor, and the flexible hoses. The hydraulic fluid should be flushed and replaced with BMW-approved CHF 11S fluid. A full system bleed is required after any repair.</x:v>
       </x:c>
       <x:c r="F59" s="9" t="n">
         <x:v>0</x:v>
@@ -17952,21 +19310,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="60" ht="739.2000122070312" hidden="0" customHeight="1">
+    <x:row r="60" ht="1188" hidden="0" customHeight="1">
       <x:c r="A60" s="40" t="n">
         <x:v>59</x:v>
       </x:c>
       <x:c r="B60" s="9" t="str">
-        <x:v>bmw-x7-tire-wear-2019</x:v>
+        <x:v>bmw-z4-vanos-solenoid-2003</x:v>
       </x:c>
       <x:c r="C60" s="9" t="str">
-        <x:v>2019-2023 | BMW | X7</x:v>
+        <x:v>2003-2016 | BMW | Z4 | 2.5i, 3.0i, 3.0si, M40i, sDrive28i, sDrive30i, sDrive35i, sDrive35is | M54, N52, N54, N20</x:v>
       </x:c>
       <x:c r="D60" s="9" t="str">
-        <x:v>Premature Tire Wear (Especially 21"/22" Wheels)</x:v>
+        <x:v>VANOS Solenoid &amp; System Failure - E85/E89 Z4 (All Engines)</x:v>
       </x:c>
       <x:c r="E60" s="9" t="str">
-        <x:v>Have alignment adjusted to reduce aggressive camber settings ($200-400). Switch to quality tires designed for heavy SUVs: Michelin Pilot Sport 4S or Continental PremiumContact 6 are recommended. If possible, avoid 22" wheels and opt for 21" or smaller for better tire longevity and ride comfort. Alignment adjustment can extend tire life from 15,000 to 30,000+ miles. Total cost $200-2,000 depending on tire replacement needs. Check alignment every 10,000 miles.</x:v>
+        <x:v>Replace VANOS solenoids - inexpensive and straightforward repair. M54 (E85 2003-2005): 2 solenoids required, BMW 11361707323 ($35-$65 each). N52 (E85 2006-2008 / E89 2009-2011 28i): 2 solenoids, BMW 11367585425 ($40-$70 each). N54 (E89 35i/35is): 2 solenoids, BMW 11367585425 ($40-$70 each). N20 (E89 sDrive28i 2012-2016): 2 solenoids, BMW 11367585425 ($40-$70 each). Labor: under 1 hour for experienced mechanic, 2-3 hours DIY. Replace all solenoids at once even if only one has failed - the others are same age and will fail soon. Also replace VANOS solenoid O-rings and sealing plates during service. Clean VANOS system with Beisan Systems VANOS cleaning procedure for best results.</x:v>
       </x:c>
       <x:c r="F60" s="9" t="n">
         <x:v>0</x:v>
@@ -17975,597 +19333,26 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="61" ht="501.6000061035156" hidden="0" customHeight="1">
-      <x:c r="A61" s="40" t="n">
+    <x:row r="61" ht="554.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A61" s="42" t="n">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="B61" s="9" t="str">
-        <x:v>bmw-xm-airbag-passenger-knee-recall-2023</x:v>
-      </x:c>
-      <x:c r="C61" s="9" t="str">
-        <x:v>2023-2023 | BMW | XM</x:v>
-      </x:c>
-      <x:c r="D61" s="9" t="str">
-        <x:v>2023 XM Front-Passenger Knee-Airbag Recall 23V-622</x:v>
-      </x:c>
-      <x:c r="E61" s="9" t="str">
-        <x:v>Check the VIN for an open 23V-622 campaign. If open, an authorized BMW dealer replaces the front-passenger knee airbag free of charge. Do not attempt airbag diagnosis or order a clock spring or airbag module from this card; supplemental-restraint work requires trained personnel and VIN-selected parts.</x:v>
-      </x:c>
-      <x:c r="F61" s="9" t="n">
+      <x:c r="B61" s="43" t="str">
+        <x:v>bmw-z8-soft-top-mechanism-2000</x:v>
+      </x:c>
+      <x:c r="C61" s="43" t="str">
+        <x:v>2000-2003 | BMW | Z8</x:v>
+      </x:c>
+      <x:c r="D61" s="43" t="str">
+        <x:v>Power Soft Top Hydraulic System and Cable Failure</x:v>
+      </x:c>
+      <x:c r="E61" s="43" t="str">
+        <x:v>Rebuild the hydraulic cylinders with new seals rather than replacing ($200 vs $2,000+). Inspect and replace frayed cables. Adjust or replace the microswitch sensors at the windshield header latch. Lubricate the top mechanism pivot points with silicone grease annually. Store the car with the top up to reduce stress on the hydraulic system.</x:v>
+      </x:c>
+      <x:c r="F61" s="43" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G61" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="62" ht="567.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A62" s="40" t="n">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="B62" s="9" t="str">
-        <x:v>bmw-xm-hybrid-drivetrain-hesitation-2023</x:v>
-      </x:c>
-      <x:c r="C62" s="9" t="str">
-        <x:v>2023-2024 | BMW | XM | S68 4.4L Twin-Turbo V8 Hybrid, S68</x:v>
-      </x:c>
-      <x:c r="D62" s="9" t="str">
-        <x:v>Hybrid Drivetrain Hesitation and Power Delivery Lag</x:v>
-      </x:c>
-      <x:c r="E62" s="9" t="str">
-        <x:v>Visit the dealer for the latest transmission and hybrid system software calibration updates. Select Sport or Sport Plus mode for more consistent power delivery. The latest software revisions significantly improve the electric-to-V8 handoff smoothness. If hesitation persists after updates, the dealer can reset the transmission adaptation values to relearn driving patterns.</x:v>
-      </x:c>
-      <x:c r="F62" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G62" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="63" ht="646.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A63" s="40" t="n">
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="B63" s="9" t="str">
-        <x:v>bmw-xm-integrated-brake-system-recall-2023</x:v>
-      </x:c>
-      <x:c r="C63" s="9" t="str">
-        <x:v>2023-2024 | BMW | XM</x:v>
-      </x:c>
-      <x:c r="D63" s="9" t="str">
-        <x:v>2023-2024 XM Integrated Brake System Recall 26V-422</x:v>
-      </x:c>
-      <x:c r="E63" s="9" t="str">
-        <x:v>Check the VIN at NHTSA and with an authorized BMW dealer when campaign 26V-422 VINs become searchable, and arrange the free dealer inspection and module replacement if required. If a brake warning appears or pedal effort increases, avoid abrupt braking, allow extra stopping distance, stop safely and contact BMW roadside assistance; wheel-speed sensors are not the recall remedy.</x:v>
-      </x:c>
-      <x:c r="F63" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G63" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="64" ht="646.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A64" s="40" t="n">
-        <x:v>63</x:v>
-      </x:c>
-      <x:c r="B64" s="9" t="str">
-        <x:v>bmw-xm-suspension-ride-quality-2023</x:v>
-      </x:c>
-      <x:c r="C64" s="9" t="str">
-        <x:v>2023-2024 | BMW | XM | S68 4.4L Twin-Turbo V8 Hybrid</x:v>
-      </x:c>
-      <x:c r="D64" s="9" t="str">
-        <x:v>Harsh Ride Quality and Suspension Stiffness</x:v>
-      </x:c>
-      <x:c r="E64" s="9" t="str">
-        <x:v>Check tire pressures regularly - overinflated tires significantly worsen the harsh ride. Some owners report improved comfort by switching to a tire with a taller sidewall profile (if available for the XM's wheel size). Use Comfort mode for daily driving. Unfortunately, no aftermarket spring or damper solution currently exists to significantly improve the ride without compromising the handling needed for the XM's weight.</x:v>
-      </x:c>
-      <x:c r="F64" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G64" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="65" ht="528" hidden="0" customHeight="1">
-      <x:c r="A65" s="40" t="n">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="B65" s="9" t="str">
-        <x:v>bmw-z3-convertible-top-rear-window-cracking-clouding-bead-separatio</x:v>
-      </x:c>
-      <x:c r="C65" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D65" s="9" t="str">
-        <x:v>Convertible Top Rear Window Cracking, Clouding, and Bead Separation</x:v>
-      </x:c>
-      <x:c r="E65" s="9" t="str">
-        <x:v>Replace the rear window panel only — BMW used a zipper system so the clouded/cracked window unzips and a new window zips/tapes in without disturbing the fabric top. Re-gluing separated bead trim rarely holds, so window replacement is the durable fix. Job is a DIY-feasible 1-1.5 hours; replace the whole top only if the fabric is also degraded.</x:v>
-      </x:c>
-      <x:c r="F65" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G65" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="66" ht="52.79999923706055" hidden="0" customHeight="1">
-      <x:c r="A66" s="40" t="n">
-        <x:v>65</x:v>
-      </x:c>
-      <x:c r="B66" s="9" t="str">
-        <x:v>bmw-z3-cooling-system-failure-1996</x:v>
-      </x:c>
-      <x:c r="C66" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D66" s="9" t="str">
-        <x:v>Cooling System Component Failures</x:v>
-      </x:c>
-      <x:c r="E66" s="9" t="str"/>
-      <x:c r="F66" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G66" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="67" ht="448.79998779296875" hidden="0" customHeight="1">
-      <x:c r="A67" s="40" t="n">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="B67" s="9" t="str">
-        <x:v>bmw-z3-cracked-exhaust-manifold-1-9l-4-cylinder</x:v>
-      </x:c>
-      <x:c r="C67" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3 | 1.9, 1.9i, Z3 1.9 | 1.9L M44 4-cylinder, 1.9L M43TU 4-cylinder</x:v>
-      </x:c>
-      <x:c r="D67" s="9" t="str">
-        <x:v>Cracked Exhaust Manifold on 1.9L 4-Cylinder (M44/M43)</x:v>
-      </x:c>
-      <x:c r="E67" s="9" t="str">
-        <x:v>Inspect the manifold for hairline cracks (a cold-engine listen or smoke test confirms the leak). Replace the cracked manifold with a used OE unit or an aftermarket stainless tubular header, and renew the manifold gasket and hardware. Allow roughly 3-4 hours labor.</x:v>
-      </x:c>
-      <x:c r="F67" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G67" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="68" ht="686.4000244140625" hidden="0" customHeight="1">
-      <x:c r="A68" s="40" t="n">
-        <x:v>67</x:v>
-      </x:c>
-      <x:c r="B68" s="9" t="str">
-        <x:v>bmw-z3-differential-mount-ear-trunk-floor-pan-tearing</x:v>
-      </x:c>
-      <x:c r="C68" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D68" s="9" t="str">
-        <x:v>Differential Mount Ear and Trunk Floor Pan Tearing</x:v>
-      </x:c>
-      <x:c r="E68" s="9" t="str">
-        <x:v>Inspect the trunk floor around the differential mount and rear subframe pickup points for cracks, torn metal, and broken spot welds. Repair requires welding and a reinforcement/re-fabrication plate kit to tie the diff mount/subframe back into the floor. Switching the diff carrier bushings to polyurethane reduces carrier movement and the stress that causes the tearing. Catching it early greatly limits the repair scope.</x:v>
-      </x:c>
-      <x:c r="F68" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G68" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="69" ht="514.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A69" s="40" t="n">
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="B69" s="9" t="str">
-        <x:v>bmw-z3-door-window-regulator-clip-mounting-tab-failure</x:v>
-      </x:c>
-      <x:c r="C69" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D69" s="9" t="str">
-        <x:v>Door Window Regulator Clip / Mounting Tab Failure</x:v>
-      </x:c>
-      <x:c r="E69" s="9" t="str">
-        <x:v>Replace the broken plastic regulator clips, or replace the regulator assembly if the cable or mechanism is also worn. If the welded mounting tab/anchor has torn from the door frame, it must be re-welded or reinforced before fitting a new regulator. Lubricate the window channels to reduce drag on the new parts.</x:v>
-      </x:c>
-      <x:c r="F69" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G69" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="70" ht="686.4000244140625" hidden="0" customHeight="1">
-      <x:c r="A70" s="40" t="n">
-        <x:v>69</x:v>
-      </x:c>
-      <x:c r="B70" s="9" t="str">
-        <x:v>bmw-z3-fuel-level-sender-failure-causing-erratic-dead-fuel-gauge</x:v>
-      </x:c>
-      <x:c r="C70" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D70" s="9" t="str">
-        <x:v>Fuel Level Sender Failure Causing Erratic or Dead Fuel Gauge</x:v>
-      </x:c>
-      <x:c r="E70" s="9" t="str">
-        <x:v>Remove the access panel behind the seats and inspect the sender. A dirty or lightly worn ceramic/resistor plate can sometimes be cleaned, but a cracked plate or worn brushes requires replacing the sender unit (or the complete fuel-pump/sender carrier assembly). Also check the tank vent valve, as tank vacuum can deform the float arm. Confirm wiring/ground integrity before condemning the sender.</x:v>
-      </x:c>
-      <x:c r="F70" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G70" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="71" ht="488.3999938964844" hidden="0" customHeight="1">
-      <x:c r="A71" s="40" t="n">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="B71" s="9" t="str">
-        <x:v>bmw-z3-hvac-blower-final-stage-resistor-failure</x:v>
-      </x:c>
-      <x:c r="C71" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D71" s="9" t="str">
-        <x:v>HVAC Blower Final Stage Resistor Failure (Fan Only Works on Max)</x:v>
-      </x:c>
-      <x:c r="E71" s="9" t="str">
-        <x:v>Replace the blower final stage resistor (A/C cars: part under the scuttle/cowl; non-A/C cars: behind the passenger footwell panel). If a new resistor does not restore all speeds, test the blower motor itself, which may also be worn. Inspect for corrosion/water intrusion at the cowl on A/C cars.</x:v>
-      </x:c>
-      <x:c r="F71" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G71" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="72" ht="1584" hidden="0" customHeight="1">
-      <x:c r="A72" s="40" t="n">
-        <x:v>71</x:v>
-      </x:c>
-      <x:c r="B72" s="9" t="str">
-        <x:v>bmw-z3-rear-subframe-crack-1996</x:v>
-      </x:c>
-      <x:c r="C72" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D72" s="9" t="str">
-        <x:v>Rear Subframe Mounting Point Cracking</x:v>
-      </x:c>
-      <x:c r="E72" s="9" t="str">
-        <x:v>Inspect the trunk floor, differential mount area, and all rear subframe mounting points from above and below the car for spot-weld separation, torn sheet metal, and cracked seams; a dye penetrant test or removing trunk trim/seam sealer may be needed to reveal early damage. If cracking is present, the proper repair is to drop the rear axle carrier/subframe, weld and reinforce the damaged unibody mounting points and trunk floor with a reinforcement kit (commonly Randy Forbes-style dual-ear/differential mount reinforcement or equivalent), then reinstall with new subframe bushings, differential mount bushings, and perform a 4-wheel alignment. Minor early cracks may be repairable before major deformation, but advanced damage often requires fabrication and extensive welding by a chassis/body specialist; typical cost ranges from about $2,000-$3,500 for early reinforcement repairs and can exceed $4,000-$6,000 if the floor is torn or multiple mounting points are damaged.</x:v>
-      </x:c>
-      <x:c r="F72" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G72" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="73" ht="66" hidden="0" customHeight="1">
-      <x:c r="A73" s="40" t="n">
-        <x:v>72</x:v>
-      </x:c>
-      <x:c r="B73" s="9" t="str">
-        <x:v>bmw-z3-rear-subframe-cracking-1996</x:v>
-      </x:c>
-      <x:c r="C73" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3 | M52, M54</x:v>
-      </x:c>
-      <x:c r="D73" s="9" t="str">
-        <x:v>Rear Subframe Mounting Point Cracks</x:v>
-      </x:c>
-      <x:c r="E73" s="9" t="str"/>
-      <x:c r="F73" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G73" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="74" ht="475.20001220703125" hidden="0" customHeight="1">
-      <x:c r="A74" s="40" t="n">
-        <x:v>73</x:v>
-      </x:c>
-      <x:c r="B74" s="9" t="str">
-        <x:v>bmw-z3-valve-cover-gasket-oil-leak</x:v>
-      </x:c>
-      <x:c r="C74" s="9" t="str">
-        <x:v>1997-2002 | BMW | Z3 | 2.3, 2.5i, 2.8, 3.0i | M52 2.8, M52TU 2.5/2.8, M54 2.5/3.0</x:v>
-      </x:c>
-      <x:c r="D74" s="9" t="str">
-        <x:v>Valve Cover Gasket Oil Leak (M52/M54 6-Cylinder)</x:v>
-      </x:c>
-      <x:c r="E74" s="9" t="str">
-        <x:v>Replace the valve cover gasket, the spark-plug-well/grommet seals, and the cover bolt seals. On M54 engines also clean oil from the plug wells and replace any oil-contaminated coil boots/coils. Use the correct torque sequence to avoid re-leaking. Inspect the cover for warping or cracks while it is off.</x:v>
-      </x:c>
-      <x:c r="F74" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G74" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="75" ht="1293.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A75" s="40" t="n">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="B75" s="9" t="str">
-        <x:v>bmw-z3-vanos-seals-1999</x:v>
-      </x:c>
-      <x:c r="C75" s="9" t="str">
-        <x:v>1999-2002 | BMW | Z3 | M52, M54, S52</x:v>
-      </x:c>
-      <x:c r="D75" s="9" t="str">
-        <x:v>VANOS Seal Failure (M52/M54/S52)</x:v>
-      </x:c>
-      <x:c r="E75" s="9" t="str">
-        <x:v>Confirm the fault by checking for cold-start VANOS rattle, rough idle, hesitation, and scanning for cam timing or mixture-related fault codes; on M52TU/M54/S52 engines, inspect VANOS operation and rule out vacuum leaks before disassembly. Repair typically involves removing the valve cover and VANOS unit, replacing the internal piston seals/O-rings with updated Viton/Teflon seals, renewing the valve cover gasket and VANOS oil line sealing washers, and then re-timing the cams to BMW specifications if required. If the unit still rattles after resealing, the VANOS bearing/anti-rattle components or the complete VANOS assembly may need replacement. Typical cost is about $60-$150 in seals/gaskets for DIY repair, $300-$700 for an independent shop reseal, or $800-$1,500+ if a rebuilt/replacement VANOS unit is installed.</x:v>
-      </x:c>
-      <x:c r="F75" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G75" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="76" ht="501.6000061035156" hidden="0" customHeight="1">
-      <x:c r="A76" s="40" t="n">
-        <x:v>75</x:v>
-      </x:c>
-      <x:c r="B76" s="9" t="str">
-        <x:v>bmw-z4-b58-coolant-tank-2019</x:v>
-      </x:c>
-      <x:c r="C76" s="9" t="str">
-        <x:v>2019-2026 | BMW | Z4 | B58</x:v>
-      </x:c>
-      <x:c r="D76" s="9" t="str">
-        <x:v>B58 Coolant Expansion Tank Cracking</x:v>
-      </x:c>
-      <x:c r="E76" s="9" t="str">
-        <x:v>Replace the coolant expansion tank with an updated BMW part or aftermarket aluminum tank. Inspect the tank and cap regularly for signs of cracking, discoloration, or seepage. When replacing, also replace the cap and check all coolant hoses for brittleness. Flush and refill with BMW-approved coolant.</x:v>
-      </x:c>
-      <x:c r="F76" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G76" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="77" ht="1306.800048828125" hidden="0" customHeight="1">
-      <x:c r="A77" s="40" t="n">
-        <x:v>76</x:v>
-      </x:c>
-      <x:c r="B77" s="9" t="str">
-        <x:v>bmw-z4-e85-convertible-top-hydraulic-2003</x:v>
-      </x:c>
-      <x:c r="C77" s="9" t="str">
-        <x:v>2003-2008 | BMW | Z4</x:v>
-      </x:c>
-      <x:c r="D77" s="9" t="str">
-        <x:v>Convertible Top Hydraulic Pump Motor Failure - E85 Z4</x:v>
-      </x:c>
-      <x:c r="E77" s="9" t="str">
-        <x:v>Replace hydraulic pump motor assembly (BMW 54347193448 / supersedes 54347119633). OEM Genuine BMW pump: $800-$1,200. Aftermarket alternatives available on Amazon for $150-$300 but quality varies significantly. Dealer labor is $1,500-$2,500+ as BMW procedure requires full top removal. ZRoadster.org members have documented a motor relocation to the boot/trunk area which allows much easier future access. Hydraulic fluid: use Aral Vitamol ZHM or BMW 54340394395 hydraulic oil. PREVENTION: Clean drain holes annually, ensure rubber bungs are properly seated, and check for water intrusion in pump area at every service. Some owners have had success with pump motor rebuilds from roofmotors.co.uk ($300-$500) but quality of rebuilds varies.</x:v>
-      </x:c>
-      <x:c r="F77" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G77" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="78" ht="1135.199951171875" hidden="0" customHeight="1">
-      <x:c r="A78" s="40" t="n">
-        <x:v>77</x:v>
-      </x:c>
-      <x:c r="B78" s="9" t="str">
-        <x:v>bmw-z4-e85-window-regulator-2003</x:v>
-      </x:c>
-      <x:c r="C78" s="9" t="str">
-        <x:v>2003-2008 | BMW | Z4</x:v>
-      </x:c>
-      <x:c r="D78" s="9" t="str">
-        <x:v>Power Window Regulator Failure - E85 Z4</x:v>
-      </x:c>
-      <x:c r="E78" s="9" t="str">
-        <x:v>Option 1 (Budget): Window regulator repair kit - replacement cables and rollers for ~$18-$25 from eBay/Amazon (BWR974 for left/driver side). Requires removing door panel and threading new cables through existing regulator frame. DIY-friendly with Z4-forum.com guides. Option 2 (Recommended): Full window regulator replacement. Driver side: BMW 51337198909 ($180-$280 OEM, $80-$150 aftermarket). Passenger side: BMW 51337198910 ($180-$280 OEM, $80-$150 aftermarket). Labor: $200-$400 at independent shop, $500-$700+ at dealer. DIY: 2-3 hours with door panel removal guide from Pelican Parts. ZRoadster.org recommends full replacement over repair kit for long-term reliability.</x:v>
-      </x:c>
-      <x:c r="F78" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G78" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="79" ht="514.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A79" s="40" t="n">
-        <x:v>78</x:v>
-      </x:c>
-      <x:c r="B79" s="9" t="str">
-        <x:v>bmw-z4-electric-steering-rack-2003</x:v>
-      </x:c>
-      <x:c r="C79" s="9" t="str">
-        <x:v>2012-2012 | BMW | Z4</x:v>
-      </x:c>
-      <x:c r="D79" s="9" t="str">
-        <x:v>2012 Z4 Electric Power-Steering Recall 12V-302</x:v>
-      </x:c>
-      <x:c r="E79" s="9" t="str">
-        <x:v>Check the VIN for an open 12V-302 campaign. If open, an authorized BMW dealer replaces the steering-assistance module free of charge. If the steering warning and audible alert occur, maintain control, reduce speed, stop safely and arrange dealer or roadside assistance; do not replace a steering rack from this card.</x:v>
-      </x:c>
-      <x:c r="F79" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G79" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="80" ht="633.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A80" s="40" t="n">
-        <x:v>79</x:v>
-      </x:c>
-      <x:c r="B80" s="9" t="str">
-        <x:v>bmw-z4-electric-water-pump-2006</x:v>
-      </x:c>
-      <x:c r="C80" s="9" t="str">
-        <x:v>2012-2016 | BMW | Z4 | N20</x:v>
-      </x:c>
-      <x:c r="D80" s="9" t="str">
-        <x:v>2012-2016 Z4 sDrive28i Water-Pump Connector Recall 24V-608</x:v>
-      </x:c>
-      <x:c r="E80" s="9" t="str">
-        <x:v>Check the VIN for an open 24V-608 campaign. If open, an authorized BMW dealer inspects the water pump and connector, replaces them if necessary, and installs the protective shield free of charge. If smoke appears from the engine compartment, stop safely, switch off the vehicle, have occupants exit, move away from traffic and call emergency or roadside assistance; do not order a pump from this card.</x:v>
-      </x:c>
-      <x:c r="F80" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G80" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="81" ht="1359.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A81" s="40" t="n">
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="B81" s="9" t="str">
-        <x:v>bmw-z4-g29-b58-water-pump-2019</x:v>
-      </x:c>
-      <x:c r="C81" s="9" t="str">
-        <x:v>2019-2025 | BMW | Z4 | M40i, sDrive35i, sDrive35is | B48, B58</x:v>
-      </x:c>
-      <x:c r="D81" s="9" t="str">
-        <x:v>B48/B58 Electric Water Pump &amp; Thermostat Failure - G29 Z4</x:v>
-      </x:c>
-      <x:c r="E81" s="9" t="str">
-        <x:v>Preventative replacement recommended at 60,000 miles. Always replace water pump and thermostat together - they share labor overlap and frequently fail concurrently. B48 sDrive30i: Water pump BMW 11518632586 ($300-$450), Thermostat BMW 11538685978 ($100-$150). B58 M40i: Water pump BMW 11518650986 ($350-$500), Thermostat BMW 11538685978 ($100-$150). Mishimoto offers performance water pump alternatives for B58 with improved impeller design. Replace 3 O-rings between thermostat and pump housing, plus 2 O-rings on coolant tube to head. Must replace water pump mounting bolts (torque-to-yield). Labor: 3-4 hours. FCP Euro lifetime warranty kits available. Also inspect plastic cylinder head coolant outlet adapter - known to shear off causing massive coolant leak.</x:v>
-      </x:c>
-      <x:c r="F81" s="9" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G81" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="82" ht="1122" hidden="0" customHeight="1">
-      <x:c r="A82" s="40" t="n">
-        <x:v>81</x:v>
-      </x:c>
-      <x:c r="B82" s="9" t="str">
-        <x:v>bmw-z4-n54-hpfp-2009</x:v>
-      </x:c>
-      <x:c r="C82" s="9" t="str">
-        <x:v>2009-2011 | BMW | Z4 | M40i, sDrive35i, sDrive35is | N54</x:v>
-      </x:c>
-      <x:c r="D82" s="9" t="str">
-        <x:v>N54 High Pressure Fuel Pump (HPFP) Failure - E89 Z4 sDrive35i/35is</x:v>
-      </x:c>
-      <x:c r="E82" s="9" t="str">
-        <x:v>Replace HPFP with latest revision Genuine BMW unit. The pump went through multiple revisions - ONLY install the latest version. Part number evolution: Original -&gt; 13517592881 (Index 10, TSB fix) -&gt; 13517616170 (latest revision, most reliable). Genuine BMW 13517616170 is the definitive fix ($350-$550 for pump). Replacement is straightforward DIY (1-2 hours) with basic tools. Also available as complete kit from FCP Euro with lifetime warranty. BMW extended warranty coverage to 10 years/120,000 miles under customer care package for original owners - check VIN eligibility. Replace low-pressure fuel sensor at same time (13537537319) as it may have been damaged by pressure fluctuations ($35-$55).</x:v>
-      </x:c>
-      <x:c r="F82" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G82" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="83" ht="580.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A83" s="40" t="n">
-        <x:v>82</x:v>
-      </x:c>
-      <x:c r="B83" s="9" t="str">
-        <x:v>bmw-z4-n54-wastegate-rattle-2009</x:v>
-      </x:c>
-      <x:c r="C83" s="9" t="str">
-        <x:v>2009-2010 | BMW | Z4 | N54</x:v>
-      </x:c>
-      <x:c r="D83" s="9" t="str">
-        <x:v>2009-2010 Z4 sDrive35i N54 Wastegate Diagnosis</x:v>
-      </x:c>
-      <x:c r="E83" s="9" t="str">
-        <x:v>Confirm the VIN, engine, production date, DME faults, boost-control data and noise source using current BMW diagnostic information. Check VIN-specific coverage history with BMW, recognizing that the bulletin's time/mileage window may have expired. Do not replace a turbocharger, actuator or wastegate from this card without the required diagnosis.</x:v>
-      </x:c>
-      <x:c r="F83" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G83" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="84" ht="501.6000061035156" hidden="0" customHeight="1">
-      <x:c r="A84" s="40" t="n">
-        <x:v>83</x:v>
-      </x:c>
-      <x:c r="B84" s="9" t="str">
-        <x:v>bmw-z4-soft-top-hydraulic-2003</x:v>
-      </x:c>
-      <x:c r="C84" s="9" t="str">
-        <x:v>2009-2016 | BMW | Z4</x:v>
-      </x:c>
-      <x:c r="D84" s="9" t="str">
-        <x:v>Retractable Hard Top Hydraulic Mechanism Failure</x:v>
-      </x:c>
-      <x:c r="E84" s="9" t="str">
-        <x:v>Diagnose the leak location and replace the failed component. Common failure points are the main hydraulic cylinders (left and right), the hydraulic pump motor, and the flexible hoses. The hydraulic fluid should be flushed and replaced with BMW-approved CHF 11S fluid. A full system bleed is required after any repair.</x:v>
-      </x:c>
-      <x:c r="F84" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G84" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="85" ht="1188" hidden="0" customHeight="1">
-      <x:c r="A85" s="40" t="n">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="B85" s="9" t="str">
-        <x:v>bmw-z4-vanos-solenoid-2003</x:v>
-      </x:c>
-      <x:c r="C85" s="9" t="str">
-        <x:v>2003-2016 | BMW | Z4 | 2.5i, 3.0i, 3.0si, M40i, sDrive28i, sDrive30i, sDrive35i, sDrive35is | M54, N52, N54, N20</x:v>
-      </x:c>
-      <x:c r="D85" s="9" t="str">
-        <x:v>VANOS Solenoid &amp; System Failure - E85/E89 Z4 (All Engines)</x:v>
-      </x:c>
-      <x:c r="E85" s="9" t="str">
-        <x:v>Replace VANOS solenoids - inexpensive and straightforward repair. M54 (E85 2003-2005): 2 solenoids required, BMW 11361707323 ($35-$65 each). N52 (E85 2006-2008 / E89 2009-2011 28i): 2 solenoids, BMW 11367585425 ($40-$70 each). N54 (E89 35i/35is): 2 solenoids, BMW 11367585425 ($40-$70 each). N20 (E89 sDrive28i 2012-2016): 2 solenoids, BMW 11367585425 ($40-$70 each). Labor: under 1 hour for experienced mechanic, 2-3 hours DIY. Replace all solenoids at once even if only one has failed - the others are same age and will fail soon. Also replace VANOS solenoid O-rings and sealing plates during service. Clean VANOS system with Beisan Systems VANOS cleaning procedure for best results.</x:v>
-      </x:c>
-      <x:c r="F85" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G85" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="86" ht="554.4000244140625" hidden="0" customHeight="1">
-      <x:c r="A86" s="42" t="n">
-        <x:v>85</x:v>
-      </x:c>
-      <x:c r="B86" s="43" t="str">
-        <x:v>bmw-z8-soft-top-mechanism-2000</x:v>
-      </x:c>
-      <x:c r="C86" s="43" t="str">
-        <x:v>2000-2003 | BMW | Z8</x:v>
-      </x:c>
-      <x:c r="D86" s="43" t="str">
-        <x:v>Power Soft Top Hydraulic System and Cable Failure</x:v>
-      </x:c>
-      <x:c r="E86" s="43" t="str">
-        <x:v>Rebuild the hydraulic cylinders with new seals rather than replacing ($200 vs $2,000+). Inspect and replace frayed cables. Adjust or replace the microswitch sensors at the windshield header latch. Lubricate the top mechanism pivot points with silicone grease annually. Store the car with the top up to reduce stress on the hydraulic system.</x:v>
-      </x:c>
-      <x:c r="F86" s="43" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G86" s="44" t="str">
+      <x:c r="G61" s="44" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Extend BMW repair-first review to 355 issues
</commit_message>
<xml_diff>
--- a/outputs/bmw-repair-first-review/BMW-repair-first-fitment-review.xlsx
+++ b/outputs/bmw-repair-first-review/BMW-repair-first-fitment-review.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R6831979ca4fd4539"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BMW Review" sheetId="2" r:id="R61289c9b9a4243d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remaining Queue" sheetId="3" r:id="R4109b83f250a4aca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="4" r:id="R41d348202c3a4f50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R1107562feb5945bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BMW Review" sheetId="2" r:id="R3e212442ffa8471c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remaining Queue" sheetId="3" r:id="Rb4c1333bdb694861"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="4" r:id="Rac92b2d12a0042ac"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -484,7 +484,7 @@
         <x:v>Reviewed in this batch</x:v>
       </x:c>
       <x:c r="B5" s="13" t="n">
-        <x:v>325</x:v>
+        <x:v>355</x:v>
       </x:c>
       <x:c r="C5" s="11"/>
       <x:c r="D5" s="11"/>
@@ -498,7 +498,7 @@
         <x:v>Remaining queue</x:v>
       </x:c>
       <x:c r="B6" s="13" t="n">
-        <x:v>60</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C6" s="11"/>
       <x:c r="D6" s="11"/>
@@ -512,7 +512,7 @@
         <x:v>Issues with destinations</x:v>
       </x:c>
       <x:c r="B7" s="13" t="n">
-        <x:v>322</x:v>
+        <x:v>352</x:v>
       </x:c>
       <x:c r="C7" s="11"/>
       <x:c r="D7" s="11"/>
@@ -526,7 +526,7 @@
         <x:v>Destination entries</x:v>
       </x:c>
       <x:c r="B8" s="13" t="n">
-        <x:v>468</x:v>
+        <x:v>521</x:v>
       </x:c>
       <x:c r="C8" s="11"/>
       <x:c r="D8" s="11"/>
@@ -540,7 +540,7 @@
         <x:v>Distinct URLs</x:v>
       </x:c>
       <x:c r="B9" s="13" t="n">
-        <x:v>161</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="C9" s="11"/>
       <x:c r="D9" s="11"/>
@@ -17898,46 +17898,1858 @@
       </x:c>
     </x:row>
     <x:row r="472" ht="1293.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A472" s="42" t="n">
+      <x:c r="A472" s="40" t="n">
         <x:v>325</x:v>
       </x:c>
-      <x:c r="B472" s="43" t="str">
+      <x:c r="B472" s="9" t="str">
         <x:v>bmw-x5-transfer-case-actuator-2000</x:v>
       </x:c>
-      <x:c r="C472" s="43" t="str">
+      <x:c r="C472" s="9" t="str">
         <x:v>2007-2013 | BMW | X5 | 3.0si, 4.8i, xDrive30i, xDrive35d, xDrive48i, X5 M | N52, N62, M57, S63</x:v>
       </x:c>
-      <x:c r="D472" s="43" t="str">
+      <x:c r="D472" s="9" t="str">
         <x:v>E70 ATC700 Transfer-Case Positioning Motor (Diagnosis Required)</x:v>
       </x:c>
-      <x:c r="E472" s="43" t="str">
+      <x:c r="E472" s="9" t="str">
         <x:v>Read BMW VTG/DSC faults and run the applicable ISTA transfer-case test plan before buying a motor. Confirm tire sizes and wear, battery voltage, wiring, transfer-case type, fluid condition, calibration, and—especially after differential or transfer-case replacement—the VIN-correct front and rear gear ratios. If testing confirms the ATC700 positioning motor and BMW ETK/AIR selects this application for the VIN, current BMW exchange servomotor 27-10-2-449-709 supersedes 27-10-7-568-267. Install the correct classification resistor/hardware supplied or specified for the VIN and perform the required VTG initialization/calibration. A generic gear-only kit is not a universal BMW repair and should not be ordered without opening and confirming the exact motor failure.</x:v>
       </x:c>
-      <x:c r="F472" s="43" t="str">
+      <x:c r="F472" s="9" t="str">
         <x:v>VTG/DSC ISTA diagnosis; tires/voltage/wiring/unit/fluid/ratios; confirmed ATC700 exchange servomotor 27102449709; resistor/hardware; initialization</x:v>
       </x:c>
-      <x:c r="G472" s="43" t="str">
+      <x:c r="G472" s="9" t="str">
         <x:v>EXACT CONDITIONAL ATC700 SERVOMOTOR</x:v>
       </x:c>
-      <x:c r="H472" s="43" t="str">
+      <x:c r="H472" s="9" t="str">
         <x:v>Genuine BMW exchange servomotor 27102449709</x:v>
       </x:c>
-      <x:c r="I472" s="43" t="str">
+      <x:c r="I472" s="9" t="str">
         <x:v>https://www.bmwpartsdeal.com/parts/bmw-rp_actuator-27102449709.html</x:v>
       </x:c>
-      <x:c r="J472" s="43" t="str">
+      <x:c r="J472" s="9" t="str">
         <x:v>2007-2013 E70 X5 ATC700 where VIN/ETK selects it; verify classification resistor/hardware</x:v>
       </x:c>
-      <x:c r="K472" s="43" t="str">
+      <x:c r="K472" s="9" t="str">
         <x:v>conditional transfer-case positioning motor</x:v>
       </x:c>
-      <x:c r="L472" s="43" t="str"/>
-      <x:c r="M472" s="43" t="str">
+      <x:c r="L472" s="9" t="str"/>
+      <x:c r="M472" s="9" t="str">
         <x:v>The corrected source supplies the current superseding motor and requires ATC700/VIN confirmation.</x:v>
       </x:c>
-      <x:c r="N472" s="44" t="str">
+      <x:c r="N472" s="41" t="str">
         <x:v>Correct the issue ID's 2000 mismatch and reject generic gear-only kits without opening/confirming the motor fault.</x:v>
       </x:c>
+    </x:row>
+    <x:row r="473" ht="1042.800048828125" hidden="0" customHeight="1">
+      <x:c r="A473" s="40" t="n">
+        <x:v>326</x:v>
+      </x:c>
+      <x:c r="B473" s="9" t="str">
+        <x:v>bmw-x5-transfer-case-actuator-2007</x:v>
+      </x:c>
+      <x:c r="C473" s="9" t="str">
+        <x:v>2019-2026 | BMW | X5</x:v>
+      </x:c>
+      <x:c r="D473" s="9" t="str">
+        <x:v>G05/F95 Transfer-Case Shudder: Tires and Fluid Diagnosis First</x:v>
+      </x:c>
+      <x:c r="E473" s="9" t="str">
+        <x:v>Follow BMW SIB 27 02 20 in order: verify all four tires for VIN-correct size, brand/application, axle placement, and wear; diagnose any powertrain faults; then use ISTA to temporarily deactivate the transfer-case clutch and road-test the complaint. Only if the shudder disappears with the VTG deactivated does BMW direct an ATX13-X oil change with DTF-1, followed by VTG calibration. The clutch plates can require up to 125 miles after the service to become fully saturated and smooth out. If the symptom remains, continue diagnosis rather than buying an actuator or transfer case. Part numbers for any further repair must be selected by VIN in ETK/AIR.</x:v>
+      </x:c>
+      <x:c r="F473" s="9" t="str">
+        <x:v>SIB 27 02 20 sequence: tire/application/wear check, powertrain faults, ISTA VTG deactivation road test, ATX13-X DTF-1 service only if shudder disappears, calibration and saturation period</x:v>
+      </x:c>
+      <x:c r="G473" s="9" t="str">
+        <x:v>BMW SIB SERVICE ROUTE; NO ACTUATOR LINK</x:v>
+      </x:c>
+      <x:c r="H473" s="9" t="str">
+        <x:v>BMW dealer locator</x:v>
+      </x:c>
+      <x:c r="I473" s="9" t="str">
+        <x:v>https://www.bmwusa.com/dealer-locator.html</x:v>
+      </x:c>
+      <x:c r="J473" s="9" t="str">
+        <x:v>2019-2026 G05/F95 X5 SIB 27 02 20 diagnosis and VTG service</x:v>
+      </x:c>
+      <x:c r="K473" s="9" t="str">
+        <x:v>BMW test-plan service</x:v>
+      </x:c>
+      <x:c r="L473" s="9" t="str"/>
+      <x:c r="M473" s="9" t="str">
+        <x:v>The corrected source explicitly requires tires and a clutch-deactivation test before fluid and rejects actuator/transfer-case purchase.</x:v>
+      </x:c>
+      <x:c r="N473" s="41" t="str">
+        <x:v>Correct the issue ID's 2007 mismatch and continue diagnosis if VTG deactivation does not remove shudder.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="474" ht="1214.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A474" s="40" t="n">
+        <x:v>327</x:v>
+      </x:c>
+      <x:c r="B474" s="9" t="str">
+        <x:v>bmw-x5-vanos-solenoid-2000</x:v>
+      </x:c>
+      <x:c r="C474" s="9" t="str">
+        <x:v>2010-2013 | BMW | X5 | xDrive30i, xDrive35i | N51, N52K, N52T, N55</x:v>
+      </x:c>
+      <x:c r="D474" s="9" t="str">
+        <x:v>VANOS Adjustment-Unit Bolt Recall 23V-707 (E70 Inline-Six)</x:v>
+      </x:c>
+      <x:c r="E474" s="9" t="str">
+        <x:v>Enter the VIN in BMW's official recall lookup and have an authorized BMW center complete recall 23V-707 if it is open. BMW's procedure is inspection-dependent: intact affected bolts are replaced; if bolts are loose or broken, the affected VANOS adjustment unit is replaced, and missing fragments must be recovered. The recall repair is free, so do not buy a solenoid or VANOS part first. If the VIN is outside the recall or a fault remains after the remedy, use BMW-capable diagnostics to test oil supply and pressure, wiring, sensors, control solenoids, adjustment units, and mechanical timing before selecting a part. If the engine runs roughly, makes unusual mechanical noise, loses power, or stalls, move out of traffic safely, stop driving, and contact BMW for transport guidance.</x:v>
+      </x:c>
+      <x:c r="F474" s="9" t="str">
+        <x:v>VIN recall 23V-707 check; free inspection-dependent bolt or adjustment-unit repair; fragment recovery; BMW diagnosis only if outside/after recall</x:v>
+      </x:c>
+      <x:c r="G474" s="9" t="str">
+        <x:v>RECALL ROUTES ONLY</x:v>
+      </x:c>
+      <x:c r="H474" s="9" t="str">
+        <x:v>BMW recall lookup</x:v>
+      </x:c>
+      <x:c r="I474" s="9" t="str">
+        <x:v>https://www.bmwusa.com/safety-and-emission-recalls.html</x:v>
+      </x:c>
+      <x:c r="J474" s="9" t="str">
+        <x:v>VIN check for 23V-707</x:v>
+      </x:c>
+      <x:c r="K474" s="9" t="str">
+        <x:v>manufacturer recall remedy</x:v>
+      </x:c>
+      <x:c r="L474" s="9" t="str"/>
+      <x:c r="M474" s="9" t="str">
+        <x:v>The repair is an inspection-dependent recall and specifically says not to buy a solenoid or VANOS part first.</x:v>
+      </x:c>
+      <x:c r="N474" s="41" t="str">
+        <x:v>Correct the issue ID's 2000 mismatch; stop driving for roughness, mechanical noise, loss of power, or stalling.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="475" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A475" s="40" t="str"/>
+      <x:c r="B475" s="9" t="str"/>
+      <x:c r="C475" s="9" t="str"/>
+      <x:c r="D475" s="9" t="str"/>
+      <x:c r="E475" s="9" t="str"/>
+      <x:c r="F475" s="9" t="str"/>
+      <x:c r="G475" s="9" t="str"/>
+      <x:c r="H475" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I475" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J475" s="9" t="str">
+        <x:v>independent VIN recall-status check</x:v>
+      </x:c>
+      <x:c r="K475" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L475" s="9" t="str"/>
+      <x:c r="M475" s="9" t="str"/>
+      <x:c r="N475" s="41" t="str"/>
+    </x:row>
+    <x:row r="476" ht="1148.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A476" s="40" t="n">
+        <x:v>328</x:v>
+      </x:c>
+      <x:c r="B476" s="9" t="str">
+        <x:v>bmw-x5-water-pump-2007</x:v>
+      </x:c>
+      <x:c r="C476" s="9" t="str">
+        <x:v>2011-2013 | BMW | X5 | xDrive35i | N55</x:v>
+      </x:c>
+      <x:c r="D476" s="9" t="str">
+        <x:v>E70 xDrive35i N55 Electric Coolant Pump (Fault-Confirmed)</x:v>
+      </x:c>
+      <x:c r="E476" s="9" t="str">
+        <x:v>If the engine-temperature warning appears, stop safely, shut the engine off, and tow the vehicle if normal temperature cannot be confirmed. When cool, check coolant level and leaks, read BMW-specific faults, verify pump power/ground and communication, and run the ISTA coolant-pump activation/test plan. If those tests confirm the pump and BMW ETK/AIR selects 11-51-5-A05-704 for the VIN, replace it using the BMW procedure, select the thermostat separately only if testing or preventive planning justifies it, vacuum-fill or bleed the system as specified, and verify commanded pump operation and stable temperature. Do not use a fixed-mileage rule or this part number for an N52, N63, or F15 without VIN confirmation.</x:v>
+      </x:c>
+      <x:c r="F476" s="9" t="str">
+        <x:v>Stop/tow after temperature warning; leak/level/fault/power/communication/ISTA test; pump 11515A05704 only when VIN/test confirm; thermostat separately; bleed/verify</x:v>
+      </x:c>
+      <x:c r="G476" s="9" t="str">
+        <x:v>EXACT CONDITIONAL E70 N55 PUMP</x:v>
+      </x:c>
+      <x:c r="H476" s="9" t="str">
+        <x:v>Genuine BMW electric coolant pump 11515A05704</x:v>
+      </x:c>
+      <x:c r="I476" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/parts/bmw-coolant_pump_electric-11515a05704.html</x:v>
+      </x:c>
+      <x:c r="J476" s="9" t="str">
+        <x:v>2011-2013 E70 X5 xDrive35i N55 where VIN/ETK selects it</x:v>
+      </x:c>
+      <x:c r="K476" s="9" t="str">
+        <x:v>conditional electric coolant pump</x:v>
+      </x:c>
+      <x:c r="L476" s="9" t="str"/>
+      <x:c r="M476" s="9" t="str">
+        <x:v>The corrected source narrows the pump to E70 N55 and makes thermostat replacement conditional.</x:v>
+      </x:c>
+      <x:c r="N476" s="41" t="str">
+        <x:v>Correct the issue ID's 2007 mismatch; do not use this pump for N52/N63/F15.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="477" ht="1056" hidden="0" customHeight="1">
+      <x:c r="A477" s="40" t="n">
+        <x:v>329</x:v>
+      </x:c>
+      <x:c r="B477" s="9" t="str">
+        <x:v>bmw-x5m-brake-system-2010</x:v>
+      </x:c>
+      <x:c r="C477" s="9" t="str">
+        <x:v>2010-2023 | BMW | X5 M</x:v>
+      </x:c>
+      <x:c r="D477" s="9" t="str">
+        <x:v>Heavy-Duty Brake System Accelerated Wear - E70/F85/F95 X5 M</x:v>
+      </x:c>
+      <x:c r="E477" s="9" t="str">
+        <x:v>E70 X5 M brakes: OEM front pads 34116799964 ($150-$250), rear pads 34216794879 ($120-$200). F85 X5 M front brake rotors: 34112284101/34112284102 with 6-pot caliper 34117845747/34117845748 and pads 34112284869. F85 rear: 385mm x 24mm perforated rotors 34212284903/34212284904 with 4-pot Brembo caliper and Textar pads. Budget $1,500-$2,500 per axle for complete brake service. For track use: EBC Yellowstuff or Hawk HPS 5.0 pads ($200-$350 per axle) with StopTech slotted rotors for improved heat management. Use Motul RBF 660 or ATE Typ 200 brake fluid - flush every 12 months. Budget $3,000-$5,000 per year for brake maintenance if driving spiritedly.</x:v>
+      </x:c>
+      <x:c r="F477" s="9" t="str">
+        <x:v>Split E70/F85/F95; identify brake option and axle; measure pads/rotors; side-specific OEM replacement; track compounds/fluid only by actual use</x:v>
+      </x:c>
+      <x:c r="G477" s="9" t="str">
+        <x:v>THREE-GENERATION BRAKE SPLIT</x:v>
+      </x:c>
+      <x:c r="H477" s="9" t="str">
+        <x:v>BMW X5 M brake catalog</x:v>
+      </x:c>
+      <x:c r="I477" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/X5-M/Brakes/</x:v>
+      </x:c>
+      <x:c r="J477" s="9" t="str">
+        <x:v>2010-2023 E70/F85/F95 X5 M; select generation, VIN, axle, side, and brake option</x:v>
+      </x:c>
+      <x:c r="K477" s="9" t="str">
+        <x:v>vehicle-specific brake catalog</x:v>
+      </x:c>
+      <x:c r="L477" s="9" t="str"/>
+      <x:c r="M477" s="9" t="str">
+        <x:v>Three generations use different pads, rotors, calipers, and options; named aftermarket products cannot be applied across the row.</x:v>
+      </x:c>
+      <x:c r="N477" s="41" t="str">
+        <x:v>Split generations and verify each part number; remove blanket annual cost and fluid-interval claims.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="478" ht="66" hidden="0" customHeight="1">
+      <x:c r="A478" s="40" t="str"/>
+      <x:c r="B478" s="9" t="str"/>
+      <x:c r="C478" s="9" t="str"/>
+      <x:c r="D478" s="9" t="str"/>
+      <x:c r="E478" s="9" t="str"/>
+      <x:c r="F478" s="9" t="str"/>
+      <x:c r="G478" s="9" t="str"/>
+      <x:c r="H478" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I478" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J478" s="9" t="str">
+        <x:v>brake measurement and track-use setup</x:v>
+      </x:c>
+      <x:c r="K478" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L478" s="9" t="str"/>
+      <x:c r="M478" s="9" t="str"/>
+      <x:c r="N478" s="41" t="str"/>
+    </x:row>
+    <x:row r="479" ht="1122" hidden="0" customHeight="1">
+      <x:c r="A479" s="40" t="n">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="B479" s="9" t="str">
+        <x:v>bmw-x5m-rear-differential-2010</x:v>
+      </x:c>
+      <x:c r="C479" s="9" t="str">
+        <x:v>2010-2023 | BMW | X5 M | S63</x:v>
+      </x:c>
+      <x:c r="D479" s="9" t="str">
+        <x:v>Rear Differential Wear &amp; Fluid Degradation - E70/F85/F95 X5 M</x:v>
+      </x:c>
+      <x:c r="E479" s="9" t="str">
+        <x:v>Change rear differential fluid every 30,000 miles (ignore BMW "lifetime fill" claim). E70 X5 M: No drain plug - fluid must be extracted through fill port with hand pump or suction device. Recommended fluid: Royal Purple 75W-140 GL5 synthetic or Red Line 75W-140 GL5 ($40-$60 per fill). Capacity approximately 1.2 liters. For limited-slip diff, ensure fluid is GL5 rated with limited-slip additive. If differential is making whining/howling noise: have a limited-slip differential specialist inspect internals (not generic BMW shop). Diff rebuild: $1,500-$3,000 at specialist. Complete differential replacement: $3,000-$5,500 + labor. Labor for fluid change: $150-$300 at independent shop.</x:v>
+      </x:c>
+      <x:c r="F479" s="9" t="str">
+        <x:v>Generation/VIN-specific differential diagnosis; correct BMW fluid/specification and fill method; leak/noise/internal inspection; specialist rebuild only if confirmed</x:v>
+      </x:c>
+      <x:c r="G479" s="9" t="str">
+        <x:v>DIFFERENTIAL / FLUID-SPEC SPLIT</x:v>
+      </x:c>
+      <x:c r="H479" s="9" t="str">
+        <x:v>Genuine BMW X5 M differential catalog</x:v>
+      </x:c>
+      <x:c r="I479" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x5_m-differential.html</x:v>
+      </x:c>
+      <x:c r="J479" s="9" t="str">
+        <x:v>2010-2023 E70/F85/F95; VIN, axle unit, and fluid specification required</x:v>
+      </x:c>
+      <x:c r="K479" s="9" t="str">
+        <x:v>OEM differential catalog</x:v>
+      </x:c>
+      <x:c r="L479" s="9" t="str"/>
+      <x:c r="M479" s="9" t="str">
+        <x:v>The row combines different differential designs and recommends generic GL-5 fluids without proving BMW specification compatibility.</x:v>
+      </x:c>
+      <x:c r="N479" s="41" t="str">
+        <x:v>Do not use Royal Purple/Red Line by viscosity alone or assume a universal 1.2-liter capacity/30k interval.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="480" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A480" s="40" t="str"/>
+      <x:c r="B480" s="9" t="str"/>
+      <x:c r="C480" s="9" t="str"/>
+      <x:c r="D480" s="9" t="str"/>
+      <x:c r="E480" s="9" t="str"/>
+      <x:c r="F480" s="9" t="str"/>
+      <x:c r="G480" s="9" t="str"/>
+      <x:c r="H480" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I480" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J480" s="9" t="str">
+        <x:v>limited-slip/active differential diagnosis and service</x:v>
+      </x:c>
+      <x:c r="K480" s="9" t="str">
+        <x:v>specialist service</x:v>
+      </x:c>
+      <x:c r="L480" s="9" t="str"/>
+      <x:c r="M480" s="9" t="str"/>
+      <x:c r="N480" s="41" t="str"/>
+    </x:row>
+    <x:row r="481" ht="1386" hidden="0" customHeight="1">
+      <x:c r="A481" s="40" t="n">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="B481" s="9" t="str">
+        <x:v>bmw-x5m-s63-cooling-system-2010</x:v>
+      </x:c>
+      <x:c r="C481" s="9" t="str">
+        <x:v>2010-2023 | BMW | X5 M | 4.4i, 4.6is, 4.8is, M50i, M60i, xDrive48i, xDrive50e, xDrive50i | S63</x:v>
+      </x:c>
+      <x:c r="D481" s="9" t="str">
+        <x:v>S63 Cooling System Component Failures - E70/F85/F95 X5 M</x:v>
+      </x:c>
+      <x:c r="E481" s="9" t="str">
+        <x:v>PROACTIVE MAINTENANCE SCHEDULE: Replace electric water pump at 60,000 miles ($400-$700 + labor). Replace thermostat at same time ($150-$250). Replace expansion tank at 60,000-80,000 miles ($100-$200). Inspect all coolant hoses at every oil change - replace any that are soft, bulging, or showing surface cracks. E70 X5 M expansion tank vent hose: 17128627119 ($30-$50). Flush coolant system every 2 years or 30,000 miles (more frequent than BMW's 4-year recommendation). Use ONLY BMW coolant mixed 50/50 with distilled water. For E70 hot-V turbo coolant lines: GRYPHONTEK repair kit eliminates plastic T-fitting failure (see separate issue entry). Budget $1,500-$2,500 for complete cooling system refresh at 60,000 miles. This prevents catastrophic overheating that can destroy the S63 engine ($15,000-$34,000 engine replacement).</x:v>
+      </x:c>
+      <x:c r="F481" s="9" t="str">
+        <x:v>Split S63 generations and cooling circuits; pressure/fault diagnosis; pump/thermostat/tank/hoses only by exact failure and VIN; correct coolant/service schedule</x:v>
+      </x:c>
+      <x:c r="G481" s="9" t="str">
+        <x:v>THREE-GENERATION COOLING SPLIT</x:v>
+      </x:c>
+      <x:c r="H481" s="9" t="str">
+        <x:v>BMW X5 M cooling catalog</x:v>
+      </x:c>
+      <x:c r="I481" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/X5-M/Cooling-System/</x:v>
+      </x:c>
+      <x:c r="J481" s="9" t="str">
+        <x:v>E70/F85/F95 X5 M; select generation, engine revision, circuit, and VIN</x:v>
+      </x:c>
+      <x:c r="K481" s="9" t="str">
+        <x:v>vehicle-specific cooling catalog</x:v>
+      </x:c>
+      <x:c r="L481" s="9" t="str"/>
+      <x:c r="M481" s="9" t="str">
+        <x:v>The source imposes one proactive schedule across three S63 revisions and multiple main/auxiliary cooling circuits.</x:v>
+      </x:c>
+      <x:c r="N481" s="41" t="str">
+        <x:v>Remove blanket 60k pump/thermostat/tank replacement and 2-year coolant interval; diagnose and follow exact BMW specification.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="482" ht="1135.199951171875" hidden="0" customHeight="1">
+      <x:c r="A482" s="40" t="n">
+        <x:v>332</x:v>
+      </x:c>
+      <x:c r="B482" s="9" t="str">
+        <x:v>bmw-x5m-s63-oil-leaks-2010</x:v>
+      </x:c>
+      <x:c r="C482" s="9" t="str">
+        <x:v>2010-2023 | BMW | X5 M | 4.4i, 4.6is, 4.8is, M50i, M60i, xDrive48i, xDrive50e, xDrive50i | S63</x:v>
+      </x:c>
+      <x:c r="D482" s="9" t="str">
+        <x:v>S63 V8 Chronic Oil Leaks (Valve Cover, Oil Pan, Turbo Lines) - E70/F85/F95 X5 M</x:v>
+      </x:c>
+      <x:c r="E482" s="9" t="str">
+        <x:v>Valve cover gasket replacement (both sides): $1,200-$2,500 with labor. BMW plastic valve covers can crack and must be replaced entirely (not just gasket) - inspect during service. Oil filter housing gasket: $400-$800 with labor. Oil pan gasket: $2,000-$3,500 (requires engine/subframe drop). Turbo oil feed/return lines: replace with GRYPHONTEK or MAMBA upgraded silicone/braided lines during any turbo service ($200-$400). VANOS solenoid seals: $100-$200 (DIY-friendly). For comprehensive oil leak repair at 80,000+ miles: budget $3,000-$5,000 to address all common leak points simultaneously. Valve cover bolt torque is CRITICAL - too tight cracks the cover ($800-$1,200 per cover), too loose and it leaks.</x:v>
+      </x:c>
+      <x:c r="F482" s="9" t="str">
+        <x:v>Trace highest fresh leak; split valve covers, filter housing, oil pan, turbo feed/return, and VANOS seals by generation/bank/source; complete cover only if cracked/warped</x:v>
+      </x:c>
+      <x:c r="G482" s="9" t="str">
+        <x:v>LEAK-SOURCE / GENERATION SPLIT</x:v>
+      </x:c>
+      <x:c r="H482" s="9" t="str">
+        <x:v>BMW X5 M engine-gasket catalog</x:v>
+      </x:c>
+      <x:c r="I482" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/X5-M/Engine-Gaskets-and-Seals/</x:v>
+      </x:c>
+      <x:c r="J482" s="9" t="str">
+        <x:v>2010-2023 E70/F85/F95; select exact engine revision, VIN, bank, and confirmed leak source</x:v>
+      </x:c>
+      <x:c r="K482" s="9" t="str">
+        <x:v>vehicle-specific seal catalog</x:v>
+      </x:c>
+      <x:c r="L482" s="9" t="str"/>
+      <x:c r="M482" s="9" t="str">
+        <x:v>The article lists many independent leak sources and unverified aftermarket line brands; no all-in-one repair is valid.</x:v>
+      </x:c>
+      <x:c r="N482" s="41" t="str">
+        <x:v>Do not bundle all leak points or claim engine/subframe removal universally; verify generation and repair procedure.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="483" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A483" s="40" t="str"/>
+      <x:c r="B483" s="9" t="str"/>
+      <x:c r="C483" s="9" t="str"/>
+      <x:c r="D483" s="9" t="str"/>
+      <x:c r="E483" s="9" t="str"/>
+      <x:c r="F483" s="9" t="str"/>
+      <x:c r="G483" s="9" t="str"/>
+      <x:c r="H483" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I483" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J483" s="9" t="str">
+        <x:v>S63 leak tracing and repair planning</x:v>
+      </x:c>
+      <x:c r="K483" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L483" s="9" t="str"/>
+      <x:c r="M483" s="9" t="str"/>
+      <x:c r="N483" s="41" t="str"/>
+    </x:row>
+    <x:row r="484" ht="1412.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A484" s="40" t="n">
+        <x:v>333</x:v>
+      </x:c>
+      <x:c r="B484" s="9" t="str">
+        <x:v>bmw-x5m-s63-rod-bearing-2010</x:v>
+      </x:c>
+      <x:c r="C484" s="9" t="str">
+        <x:v>2010-2018 | BMW | X5 M | 4.4i, 4.6is, 4.8is, M50i, M60i, xDrive48i, xDrive50e, xDrive50i</x:v>
+      </x:c>
+      <x:c r="D484" s="9" t="str">
+        <x:v>S63 V8 Rod Bearing Premature Wear &amp; Failure - E70/F85 X5 M</x:v>
+      </x:c>
+      <x:c r="E484" s="9" t="str">
+        <x:v>PREVENTIVE: For track-driven X5 M, replace rod bearings proactively at 60,000-80,000 miles. ACL Race Series rod bearings (8B1578HX-STD for S63B44, +0.001" extra oil clearance) are the community gold standard ($200-$350 for bearing set). WPC surface-treated bearings from Lang Racing are the premium choice ($400-$600 set). Total cost for preventive rod bearing service: $4,500-$8,500 depending on shop. Oil analysis every 5,000 miles through Blackstone Labs ($30/test) to monitor bearing wear metals (lead and copper). Use only BMW 10W-60 synthetic oil with 5,000-7,500 mile oil change intervals. Never track the car on cold oil. Mporium BMW offers specialized S63 rod bearing service starting at $4,499. If catastrophic failure: rebuilt S63 engine from RK Autowerks (~$8,500 + installation), new BMW engine (~$34,000), or complete engine rebuild ($12,000-$18,000).</x:v>
+      </x:c>
+      <x:c r="F484" s="9" t="str">
+        <x:v>Engine-revision-specific oil-pressure/noise diagnosis; measured bearing clearances; engine-builder-selected bearings/fasteners; optional oil trending</x:v>
+      </x:c>
+      <x:c r="G484" s="9" t="str">
+        <x:v>SPECULATIVE PREVENTIVE CLAIM CORRECTED</x:v>
+      </x:c>
+      <x:c r="H484" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I484" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J484" s="9" t="str">
+        <x:v>2010-2018 E70/F85 X5 M S63 bottom-end assessment</x:v>
+      </x:c>
+      <x:c r="K484" s="9" t="str">
+        <x:v>engine-builder service</x:v>
+      </x:c>
+      <x:c r="L484" s="9" t="str"/>
+      <x:c r="M484" s="9" t="str">
+        <x:v>The source prescribes ACL/WPC, intervals, and oil without engine-revision/clearance evidence; 10W-60 is not a universal S63 specification.</x:v>
+      </x:c>
+      <x:c r="N484" s="41" t="str">
+        <x:v>Remove fixed preventive interval, 'gold standard,' and universal 10W-60 advice.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="485" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A485" s="40" t="str"/>
+      <x:c r="B485" s="9" t="str"/>
+      <x:c r="C485" s="9" t="str"/>
+      <x:c r="D485" s="9" t="str"/>
+      <x:c r="E485" s="9" t="str"/>
+      <x:c r="F485" s="9" t="str"/>
+      <x:c r="G485" s="9" t="str"/>
+      <x:c r="H485" s="9" t="str">
+        <x:v>Blackstone oil-analysis kit</x:v>
+      </x:c>
+      <x:c r="I485" s="9" t="str">
+        <x:v>https://www.blackstone-labs.com/products/free-test-kits/</x:v>
+      </x:c>
+      <x:c r="J485" s="9" t="str">
+        <x:v>optional trending only; not conclusive bearing diagnosis</x:v>
+      </x:c>
+      <x:c r="K485" s="9" t="str">
+        <x:v>oil-analysis service</x:v>
+      </x:c>
+      <x:c r="L485" s="9" t="str"/>
+      <x:c r="M485" s="9" t="str"/>
+      <x:c r="N485" s="41" t="str"/>
+    </x:row>
+    <x:row r="486" ht="1214.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A486" s="40" t="n">
+        <x:v>334</x:v>
+      </x:c>
+      <x:c r="B486" s="9" t="str">
+        <x:v>bmw-x5m-s63-turbo-coolant-line-2010</x:v>
+      </x:c>
+      <x:c r="C486" s="9" t="str">
+        <x:v>2010-2013 | BMW | X5 M</x:v>
+      </x:c>
+      <x:c r="D486" s="9" t="str">
+        <x:v>S63 Turbo Coolant Line Plastic T-Fitting Failure (Hot-V Design) - E70 X5 M</x:v>
+      </x:c>
+      <x:c r="E486" s="9" t="str">
+        <x:v>Replace ALL factory plastic turbo coolant T-fittings and hoses with GRYPHONTEK S63 Turbo Coolant Line Repair Kit ($200-$400). Kit includes pre-shaped multi-layer reinforced silicone hoses, brass T-fittings (replacing factory plastic), and all necessary hose clamps. Direct bolt-on installation designed for the E70/E71 S63 engine bay. MAMBA Turbo also offers a reinforced turbo coolant line kit with brass and silicone components ($150-$350). This is a PROACTIVE replacement - do not wait for failure. Replace at first sign of coolant weeping or during any turbo service. Labor: $800-$1,500 due to tight access in hot-V engine valley. If turbo bearings are damaged from overheating: turbo replacement $3,000-$5,000 per unit.</x:v>
+      </x:c>
+      <x:c r="F486" s="9" t="str">
+        <x:v>Pressure-test and confirm E70 S63 turbo-coolant line/T-fitting leak; exact reinforced line/fitting kit or VIN-specific OEM components; coolant refill/bleed; turbo inspection after overheat</x:v>
+      </x:c>
+      <x:c r="G486" s="9" t="str">
+        <x:v>E70-SPECIFIC DIAGNOSIS; AFTERMARKET KIT HELD</x:v>
+      </x:c>
+      <x:c r="H486" s="9" t="str">
+        <x:v>BMW X5 M turbo-cooling catalog</x:v>
+      </x:c>
+      <x:c r="I486" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x5_m-turbocharger_cooling.html</x:v>
+      </x:c>
+      <x:c r="J486" s="9" t="str">
+        <x:v>2010-2013 E70 X5 M S63; VIN and failed line/fitting required</x:v>
+      </x:c>
+      <x:c r="K486" s="9" t="str">
+        <x:v>OEM cooling-line catalog</x:v>
+      </x:c>
+      <x:c r="L486" s="9" t="str"/>
+      <x:c r="M486" s="9" t="str">
+        <x:v>No exact live GRYPHONTEK/MAMBA page with complete E70 kit contents was verified in this pass.</x:v>
+      </x:c>
+      <x:c r="N486" s="41" t="str">
+        <x:v>Do not call proactive replacement mandatory; approve an aftermarket kit only after opening and verifying exact E70 fitment/contents.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="487" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A487" s="40" t="str"/>
+      <x:c r="B487" s="9" t="str"/>
+      <x:c r="C487" s="9" t="str"/>
+      <x:c r="D487" s="9" t="str"/>
+      <x:c r="E487" s="9" t="str"/>
+      <x:c r="F487" s="9" t="str"/>
+      <x:c r="G487" s="9" t="str"/>
+      <x:c r="H487" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I487" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J487" s="9" t="str">
+        <x:v>hot-V leak diagnosis and repair</x:v>
+      </x:c>
+      <x:c r="K487" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L487" s="9" t="str"/>
+      <x:c r="M487" s="9" t="str"/>
+      <x:c r="N487" s="41" t="str"/>
+    </x:row>
+    <x:row r="488" ht="1135.199951171875" hidden="0" customHeight="1">
+      <x:c r="A488" s="40" t="n">
+        <x:v>335</x:v>
+      </x:c>
+      <x:c r="B488" s="9" t="str">
+        <x:v>bmw-x5m-s63-vanos-solenoid-2010</x:v>
+      </x:c>
+      <x:c r="C488" s="9" t="str">
+        <x:v>2010-2023 | BMW | X5 M | 4.4i, 4.6is, 4.8is, M50i, M60i, xDrive48i, xDrive50e, xDrive50i | S63</x:v>
+      </x:c>
+      <x:c r="D488" s="9" t="str">
+        <x:v>S63 VANOS Solenoid Failure - E70/F85/F95 X5 M</x:v>
+      </x:c>
+      <x:c r="E488" s="9" t="str">
+        <x:v>Replace all 4 VANOS solenoids simultaneously - they are same age and if one has failed, others are close behind. Pierburg 11368605123 (OEM supplier) at $30-$50 each from Turner Motorsport or BimmerWorld. Genuine BMW 11368482268 for S63TU applications at $50-$70 each. Total parts cost: $120-$280 for all 4 solenoids. Also replace VANOS solenoid O-rings and filter screens during service. Labor: 1-2 hours professional ($150-$400 labor). This is one of the easier S63 repairs - accessible from top of engine without removing intake manifold. Natafox and Febi also offer quality aftermarket VANOS solenoids at lower cost ($20-$35 each). Clean VANOS system with fresh oil change immediately after solenoid replacement.</x:v>
+      </x:c>
+      <x:c r="F488" s="9" t="str">
+        <x:v>Engine-revision and intake/exhaust/bank diagnosis; exact solenoid and seals; screens/oil condition by service procedure; quantity based on confirmed failures</x:v>
+      </x:c>
+      <x:c r="G488" s="9" t="str">
+        <x:v>PART-NUMBER / POSITION / GENERATION GATE</x:v>
+      </x:c>
+      <x:c r="H488" s="9" t="str">
+        <x:v>BMW X5 M VANOS-solenoid catalog</x:v>
+      </x:c>
+      <x:c r="I488" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/X5-M/VANOS-Solenoid/</x:v>
+      </x:c>
+      <x:c r="J488" s="9" t="str">
+        <x:v>E70/F85/F95 X5 M; select S63 revision, VIN, position, and exact number</x:v>
+      </x:c>
+      <x:c r="K488" s="9" t="str">
+        <x:v>vehicle-specific VANOS catalog</x:v>
+      </x:c>
+      <x:c r="L488" s="9" t="str"/>
+      <x:c r="M488" s="9" t="str">
+        <x:v>The source names two part numbers across three generations and requires all four without evidence.</x:v>
+      </x:c>
+      <x:c r="N488" s="41" t="str">
+        <x:v>Do not replace all four automatically or recommend an engine flush; diagnose position and follow current oil specification.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="489" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A489" s="40" t="str"/>
+      <x:c r="B489" s="9" t="str"/>
+      <x:c r="C489" s="9" t="str"/>
+      <x:c r="D489" s="9" t="str"/>
+      <x:c r="E489" s="9" t="str"/>
+      <x:c r="F489" s="9" t="str"/>
+      <x:c r="G489" s="9" t="str"/>
+      <x:c r="H489" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I489" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J489" s="9" t="str">
+        <x:v>BMW-capable VANOS diagnosis</x:v>
+      </x:c>
+      <x:c r="K489" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L489" s="9" t="str"/>
+      <x:c r="M489" s="9" t="str"/>
+      <x:c r="N489" s="41" t="str"/>
+    </x:row>
+    <x:row r="490" ht="1293.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A490" s="40" t="n">
+        <x:v>336</x:v>
+      </x:c>
+      <x:c r="B490" s="9" t="str">
+        <x:v>bmw-x5m-s63-wastegate-rattle-2010</x:v>
+      </x:c>
+      <x:c r="C490" s="9" t="str">
+        <x:v>2010-2018 | BMW | X5 M | S63</x:v>
+      </x:c>
+      <x:c r="D490" s="9" t="str">
+        <x:v>S63 Twin Turbo Wastegate Rattle - E70/F85 X5 M</x:v>
+      </x:c>
+      <x:c r="E490" s="9" t="str">
+        <x:v>Option 1 (Most cost-effective): MAMBA SUS316 stainless steel wastegate rattle flapper repair kit for S63 MGT2260 (part 077-0024, replaces 790463-2 / 790484-3), approximately $150-$300 per turbo. Requires turbo removal for installation. Option 2: Lskioer turbo wastegate rattle flapper repair kit for S63/S63TU MGT2260DSL ($80-$150 per kit on Amazon). Option 3: Replace turbo wastegate actuators with new OEM units ($300-$500 each). Option 4: Full turbocharger replacement with new or remanufactured units ($3,000-$5,000 per turbo + labor). Labor for turbo removal and reinstallation: $2,000-$3,500 for both turbos. While turbos are out: replace turbo oil feed/return lines, coolant lines, and all gaskets (GRYPHONTEK turbo coolant line repair kit for E70 X5M, ~$200-$400).</x:v>
+      </x:c>
+      <x:c r="F490" s="9" t="str">
+        <x:v>Boost/vacuum/wastegate diagnosis; identify S63 generation, turbo model, bank, and flapper/actuator serviceability; turbo only for confirmed severe wear; access lines/gaskets by condition</x:v>
+      </x:c>
+      <x:c r="G490" s="9" t="str">
+        <x:v>TURBO-MODEL / BANK GATE; KITS HELD</x:v>
+      </x:c>
+      <x:c r="H490" s="9" t="str">
+        <x:v>BMW X5 M turbo catalog</x:v>
+      </x:c>
+      <x:c r="I490" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x5_m-turbocharger.html</x:v>
+      </x:c>
+      <x:c r="J490" s="9" t="str">
+        <x:v>2010-2018 E70/F85 X5 M; VIN, engine revision, bank, and turbo number required</x:v>
+      </x:c>
+      <x:c r="K490" s="9" t="str">
+        <x:v>OEM turbo catalog</x:v>
+      </x:c>
+      <x:c r="L490" s="9" t="str"/>
+      <x:c r="M490" s="9" t="str">
+        <x:v>The named repair kits were not verified against every turbo number and generation in the row.</x:v>
+      </x:c>
+      <x:c r="N490" s="41" t="str">
+        <x:v>Do not approve flapper/actuator kits by engine name alone; turbo removal and machine work require exact compatibility.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="491" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A491" s="40" t="str"/>
+      <x:c r="B491" s="9" t="str"/>
+      <x:c r="C491" s="9" t="str"/>
+      <x:c r="D491" s="9" t="str"/>
+      <x:c r="E491" s="9" t="str"/>
+      <x:c r="F491" s="9" t="str"/>
+      <x:c r="G491" s="9" t="str"/>
+      <x:c r="H491" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I491" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J491" s="9" t="str">
+        <x:v>wastegate/boost/turbo diagnosis</x:v>
+      </x:c>
+      <x:c r="K491" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L491" s="9" t="str"/>
+      <x:c r="M491" s="9" t="str"/>
+      <x:c r="N491" s="41" t="str"/>
+    </x:row>
+    <x:row r="492" ht="1069.199951171875" hidden="0" customHeight="1">
+      <x:c r="A492" s="40" t="n">
+        <x:v>337</x:v>
+      </x:c>
+      <x:c r="B492" s="9" t="str">
+        <x:v>bmw-x5m-transfer-case-actuator-2010</x:v>
+      </x:c>
+      <x:c r="C492" s="9" t="str">
+        <x:v>2010-2023 | BMW | X5 M</x:v>
+      </x:c>
+      <x:c r="D492" s="9" t="str">
+        <x:v>xDrive Transfer Case Actuator Motor Failure - E70/F85/F95 X5 M</x:v>
+      </x:c>
+      <x:c r="E492" s="9" t="str">
+        <x:v>Replace transfer case actuator motor. E70 X5 M: BMW 27107566296 or equivalent ($250-$450 for actuator motor). F85 X5 M: BMW 27608643153 or equivalent ($300-$500). F95 X5 M: check VIN-specific part number with dealer. FCP Euro has an excellent DIY guide for BMW transfer case actuator repair - the actuator can be replaced without removing the entire transfer case. Labor: 2-3 hours at specialist shop ($300-$600 labor). Change transfer case fluid at same time with BMW DTF-1 specification fluid. XeMODeX offers remanufactured transfer case actuator motors at reduced cost ($200-$350). For complete transfer case failure: $3,500-$6,000 for replacement unit + labor.</x:v>
+      </x:c>
+      <x:c r="F492" s="9" t="str">
+        <x:v>VTG/DSC diagnosis; split E70/F85/F95 units; exact motor only if test confirms; fluid to exact unit; initialization/calibration; internal transfer-case branch</x:v>
+      </x:c>
+      <x:c r="G492" s="9" t="str">
+        <x:v>THREE-GENERATION UNIT SPLIT</x:v>
+      </x:c>
+      <x:c r="H492" s="9" t="str">
+        <x:v>BMW X5 M transfer-case catalog</x:v>
+      </x:c>
+      <x:c r="I492" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x5_m-transfer_case.html</x:v>
+      </x:c>
+      <x:c r="J492" s="9" t="str">
+        <x:v>2010-2023 E70/F85/F95; VIN and exact transfer-case unit required</x:v>
+      </x:c>
+      <x:c r="K492" s="9" t="str">
+        <x:v>OEM drivetrain catalog</x:v>
+      </x:c>
+      <x:c r="L492" s="9" t="str"/>
+      <x:c r="M492" s="9" t="str">
+        <x:v>The three generations have different actuator numbers and diagnostic paths.</x:v>
+      </x:c>
+      <x:c r="N492" s="41" t="str">
+        <x:v>Do not attach 27107566296 or 27608643153 beyond verified VIN fitment, and do not claim removal procedure universally.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="493" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A493" s="40" t="str"/>
+      <x:c r="B493" s="9" t="str"/>
+      <x:c r="C493" s="9" t="str"/>
+      <x:c r="D493" s="9" t="str"/>
+      <x:c r="E493" s="9" t="str"/>
+      <x:c r="F493" s="9" t="str"/>
+      <x:c r="G493" s="9" t="str"/>
+      <x:c r="H493" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I493" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J493" s="9" t="str">
+        <x:v>VTG test plan and initialization</x:v>
+      </x:c>
+      <x:c r="K493" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L493" s="9" t="str"/>
+      <x:c r="M493" s="9" t="str"/>
+      <x:c r="N493" s="41" t="str"/>
+    </x:row>
+    <x:row r="494" ht="435.6000061035156" hidden="0" customHeight="1">
+      <x:c r="A494" s="40" t="n">
+        <x:v>338</x:v>
+      </x:c>
+      <x:c r="B494" s="9" t="str">
+        <x:v>bmw-x6-adaptive-drive-malfunction-2008</x:v>
+      </x:c>
+      <x:c r="C494" s="9" t="str">
+        <x:v>2008-2019 | BMW | X6</x:v>
+      </x:c>
+      <x:c r="D494" s="9" t="str">
+        <x:v>Adaptive Drive System Malfunction</x:v>
+      </x:c>
+      <x:c r="E494" s="9" t="str">
+        <x:v>Diagnose specific Adaptive Drive component failure using BMW ISTA diagnostics. Replace the failed component — most commonly the hydraulic pump or valve block. If repair cost is prohibitive, some owners convert to conventional anti-roll bars as a permanent fix at lower cost.</x:v>
+      </x:c>
+      <x:c r="F494" s="9" t="str">
+        <x:v>VIN/options and ISTA diagnosis; distinguish hydraulic pump, valve block, sensors, lines, active anti-roll bars, and wiring; exact component only after test; conversion as separate modification</x:v>
+      </x:c>
+      <x:c r="G494" s="9" t="str">
+        <x:v>OPTION / COMPONENT DIAGNOSIS ROUTE</x:v>
+      </x:c>
+      <x:c r="H494" s="9" t="str">
+        <x:v>BMW X6 Adaptive Drive catalog</x:v>
+      </x:c>
+      <x:c r="I494" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x6-active_suspension.html</x:v>
+      </x:c>
+      <x:c r="J494" s="9" t="str">
+        <x:v>2008-2019 E71/F16 X6; VIN, option codes, and diagnosed component required</x:v>
+      </x:c>
+      <x:c r="K494" s="9" t="str">
+        <x:v>OEM active-suspension catalog</x:v>
+      </x:c>
+      <x:c r="L494" s="9" t="str"/>
+      <x:c r="M494" s="9" t="str">
+        <x:v>The symptom can originate in several hydraulic/electronic components and spans two generations.</x:v>
+      </x:c>
+      <x:c r="N494" s="41" t="str">
+        <x:v>Do not default to pump/valve block or present conventional-bar conversion as the normal repair.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="495" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A495" s="40" t="str"/>
+      <x:c r="B495" s="9" t="str"/>
+      <x:c r="C495" s="9" t="str"/>
+      <x:c r="D495" s="9" t="str"/>
+      <x:c r="E495" s="9" t="str"/>
+      <x:c r="F495" s="9" t="str"/>
+      <x:c r="G495" s="9" t="str"/>
+      <x:c r="H495" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I495" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J495" s="9" t="str">
+        <x:v>ISTA Adaptive Drive diagnosis</x:v>
+      </x:c>
+      <x:c r="K495" s="9" t="str">
+        <x:v>specialist service</x:v>
+      </x:c>
+      <x:c r="L495" s="9" t="str"/>
+      <x:c r="M495" s="9" t="str"/>
+      <x:c r="N495" s="41" t="str"/>
+    </x:row>
+    <x:row r="496" ht="858" hidden="0" customHeight="1">
+      <x:c r="A496" s="40" t="n">
+        <x:v>339</x:v>
+      </x:c>
+      <x:c r="B496" s="9" t="str">
+        <x:v>bmw-x6-air-suspension-2008</x:v>
+      </x:c>
+      <x:c r="C496" s="9" t="str">
+        <x:v>2008-2023 | BMW | X6</x:v>
+      </x:c>
+      <x:c r="D496" s="9" t="str">
+        <x:v>Air Suspension Compressor &amp; Strut Failure</x:v>
+      </x:c>
+      <x:c r="E496" s="9" t="str">
+        <x:v>Replace failed air springs or compressor. Arnott rear air spring A-2642 ($200-300 each). OEM F16 spring 37126795013 ($200). Arnott compressor P-2655 ($599). Or convert to coil springs: Strutmasters BB2RBM conversion kit ($1,200-1,800) permanently eliminates air suspension issues. Conversion is cheaper long-term than continued air suspension repairs. If keeping air suspension: inspect air springs at 60,000-80,000 miles for cracks/leaks before compressor damage occurs. Replace both air springs on same axle simultaneously.</x:v>
+      </x:c>
+      <x:c r="F496" s="9" t="str">
+        <x:v>Generation/options/fault diagnosis; leak-test springs/struts/lines/valve block; compressor power/output; exact failed component; coil conversion only as separately engineered/legal choice</x:v>
+      </x:c>
+      <x:c r="G496" s="9" t="str">
+        <x:v>MULTI-GENERATION AIR-SUSPENSION SPLIT</x:v>
+      </x:c>
+      <x:c r="H496" s="9" t="str">
+        <x:v>BMW X6 air-suspension catalog</x:v>
+      </x:c>
+      <x:c r="I496" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/X6/Air-Suspension/</x:v>
+      </x:c>
+      <x:c r="J496" s="9" t="str">
+        <x:v>2008-2023 E71/F16/G06; select generation, VIN, axle/corner, and diagnosed component</x:v>
+      </x:c>
+      <x:c r="K496" s="9" t="str">
+        <x:v>vehicle-specific air-suspension catalog</x:v>
+      </x:c>
+      <x:c r="L496" s="9" t="str"/>
+      <x:c r="M496" s="9" t="str">
+        <x:v>Named Arnott/OEM/conversion products do not span three generations and configurations.</x:v>
+      </x:c>
+      <x:c r="N496" s="41" t="str">
+        <x:v>Do not replace axle pairs or convert to coils automatically; repair the diagnosed source and preserve chassis-control compatibility.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="497" ht="66" hidden="0" customHeight="1">
+      <x:c r="A497" s="40" t="str"/>
+      <x:c r="B497" s="9" t="str"/>
+      <x:c r="C497" s="9" t="str"/>
+      <x:c r="D497" s="9" t="str"/>
+      <x:c r="E497" s="9" t="str"/>
+      <x:c r="F497" s="9" t="str"/>
+      <x:c r="G497" s="9" t="str"/>
+      <x:c r="H497" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I497" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J497" s="9" t="str">
+        <x:v>leak and compressor diagnosis/calibration</x:v>
+      </x:c>
+      <x:c r="K497" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L497" s="9" t="str"/>
+      <x:c r="M497" s="9" t="str"/>
+      <x:c r="N497" s="41" t="str"/>
+    </x:row>
+    <x:row r="498" ht="646.7999877929688" hidden="0" customHeight="1">
+      <x:c r="A498" s="40" t="n">
+        <x:v>340</x:v>
+      </x:c>
+      <x:c r="B498" s="9" t="str">
+        <x:v>bmw-x6-ibs-brake-recall-2023</x:v>
+      </x:c>
+      <x:c r="C498" s="9" t="str">
+        <x:v>2024-2024 | BMW | X6</x:v>
+      </x:c>
+      <x:c r="D498" s="9" t="str">
+        <x:v>2024 X6 Integrated Brake System Recall 26V-422</x:v>
+      </x:c>
+      <x:c r="E498" s="9" t="str">
+        <x:v>Check the VIN at NHTSA and with an authorized BMW dealer when campaign 26V-422 VINs become searchable, and arrange the free dealer inspection and module replacement if required. If a brake warning appears or pedal effort increases, avoid abrupt braking, allow extra stopping distance, stop safely and contact BMW roadside assistance; do not order brake electronics from this card.</x:v>
+      </x:c>
+      <x:c r="F498" s="9" t="str">
+        <x:v>VIN recall 26V-422 check; free dealer inspection/module replacement if required; increased-distance/roadside safety response for warnings</x:v>
+      </x:c>
+      <x:c r="G498" s="9" t="str">
+        <x:v>RECALL ROUTES ONLY</x:v>
+      </x:c>
+      <x:c r="H498" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I498" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J498" s="9" t="str">
+        <x:v>VIN check for 26V-422</x:v>
+      </x:c>
+      <x:c r="K498" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L498" s="9" t="str"/>
+      <x:c r="M498" s="9" t="str">
+        <x:v>The remedy is an authorized safety recall, not retail brake electronics.</x:v>
+      </x:c>
+      <x:c r="N498" s="41" t="str">
+        <x:v>Correct the issue ID's 2023 mismatch: the row is 2024 X6.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="499" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A499" s="40" t="str"/>
+      <x:c r="B499" s="9" t="str"/>
+      <x:c r="C499" s="9" t="str"/>
+      <x:c r="D499" s="9" t="str"/>
+      <x:c r="E499" s="9" t="str"/>
+      <x:c r="F499" s="9" t="str"/>
+      <x:c r="G499" s="9" t="str"/>
+      <x:c r="H499" s="9" t="str">
+        <x:v>BMW recall lookup</x:v>
+      </x:c>
+      <x:c r="I499" s="9" t="str">
+        <x:v>https://www.bmwusa.com/safety-and-emission-recalls.html</x:v>
+      </x:c>
+      <x:c r="J499" s="9" t="str">
+        <x:v>manufacturer VIN/campaign status</x:v>
+      </x:c>
+      <x:c r="K499" s="9" t="str">
+        <x:v>manufacturer recall remedy</x:v>
+      </x:c>
+      <x:c r="L499" s="9" t="str"/>
+      <x:c r="M499" s="9" t="str"/>
+      <x:c r="N499" s="41" t="str"/>
+    </x:row>
+    <x:row r="500" ht="924" hidden="0" customHeight="1">
+      <x:c r="A500" s="40" t="n">
+        <x:v>341</x:v>
+      </x:c>
+      <x:c r="B500" s="9" t="str">
+        <x:v>bmw-x6-n63-timing-chain-2008</x:v>
+      </x:c>
+      <x:c r="C500" s="9" t="str">
+        <x:v>2008-2018 | BMW | X6 | M50i, xDrive50i</x:v>
+      </x:c>
+      <x:c r="D500" s="9" t="str">
+        <x:v>N63 Timing Chain Stretch &amp; Guide Failure (E71/F16 xDrive50i)</x:v>
+      </x:c>
+      <x:c r="E500" s="9" t="str">
+        <x:v>PREVENTIVE REPLACEMENT: If you own 2008-2014 E71 xDrive50i with N63, replace timing chain guides and tensioners IMMEDIATELY at 60,000-80,000 miles ($4,000-6,000) BEFORE failure. IWIS timing chain kit 90001521 ($800-1,200) or Turner kit 11317594899KT recommended. Replace lower chain guide 11147574373 at same time. If chain has already failed: complete engine replacement required ($15,000-25,000). Check VIN with BMW dealer for extended warranty eligibility. 2015+ N63TU engines have improved timing components but still require monitoring.</x:v>
+      </x:c>
+      <x:c r="F500" s="9" t="str">
+        <x:v>Split N63/N63TU and production/VIN; DME/VANOS faults and ISTA elongation test; complete chain repair only if failed; historical warranty check</x:v>
+      </x:c>
+      <x:c r="G500" s="9" t="str">
+        <x:v>ENGINE-GENERATION / ISTA GATE</x:v>
+      </x:c>
+      <x:c r="H500" s="9" t="str">
+        <x:v>BMW dealer locator</x:v>
+      </x:c>
+      <x:c r="I500" s="9" t="str">
+        <x:v>https://www.bmwusa.com/dealer-locator.html</x:v>
+      </x:c>
+      <x:c r="J500" s="9" t="str">
+        <x:v>E71/F16 X6 N63 timing test, VIN history, and complete repair</x:v>
+      </x:c>
+      <x:c r="K500" s="9" t="str">
+        <x:v>BMW-qualified service</x:v>
+      </x:c>
+      <x:c r="L500" s="9" t="str"/>
+      <x:c r="M500" s="9" t="str">
+        <x:v>The source prescribes immediate 60-80k replacement and named kits without an elongation test or complete-generation fitment.</x:v>
+      </x:c>
+      <x:c r="N500" s="41" t="str">
+        <x:v>Remove 'immediately,' fixed interval, and engine-replacement certainty; split N63/N63TU and verify complete SIB procedure.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="501" ht="409.20001220703125" hidden="0" customHeight="1">
+      <x:c r="A501" s="40" t="n">
+        <x:v>342</x:v>
+      </x:c>
+      <x:c r="B501" s="9" t="str">
+        <x:v>bmw-x6-n63-valve-stem-seal-wear-2008</x:v>
+      </x:c>
+      <x:c r="C501" s="9" t="str">
+        <x:v>2008-2019 | BMW | X6 | N63</x:v>
+      </x:c>
+      <x:c r="D501" s="9" t="str">
+        <x:v>N63 Valve Stem Seal Degradation and Oil Burning</x:v>
+      </x:c>
+      <x:c r="E501" s="9" t="str">
+        <x:v>Replace all intake and exhaust valve stem seals. This is a major job requiring head work. Also replace turbo oil return lines and update engine software per BMW N63 Customer Care Package specifications. Ensure proper oil grade (BMW LL-01) is used.</x:v>
+      </x:c>
+      <x:c r="F501" s="9" t="str">
+        <x:v>Oil-consumption/smoke/leak/turbo/PCV diagnosis; engine-revision-specific valve seals only after confirmation; turbo-return lines/software only if separately indicated</x:v>
+      </x:c>
+      <x:c r="G501" s="9" t="str">
+        <x:v>DUPLICATE / GENERATION-SPECIFIC SERVICE ROUTE</x:v>
+      </x:c>
+      <x:c r="H501" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I501" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J501" s="9" t="str">
+        <x:v>2008-2019 X6 N63/N63TU oil-consumption and valve-seal diagnosis</x:v>
+      </x:c>
+      <x:c r="K501" s="9" t="str">
+        <x:v>equipped specialist service</x:v>
+      </x:c>
+      <x:c r="L501" s="9" t="str"/>
+      <x:c r="M501" s="9" t="str">
+        <x:v>This overlaps the next valve-seal row and bundles unrelated turbo lines/software.</x:v>
+      </x:c>
+      <x:c r="N501" s="41" t="str">
+        <x:v>Consolidate duplicate rows and diagnose oil source before authorizing head/valve-seal work.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="502" ht="858" hidden="0" customHeight="1">
+      <x:c r="A502" s="40" t="n">
+        <x:v>343</x:v>
+      </x:c>
+      <x:c r="B502" s="9" t="str">
+        <x:v>bmw-x6-n63-valve-stem-seals-2008</x:v>
+      </x:c>
+      <x:c r="C502" s="9" t="str">
+        <x:v>2008-2023 | BMW | X6 | M50i, xDrive50i | N63</x:v>
+      </x:c>
+      <x:c r="D502" s="9" t="str">
+        <x:v>N63 Valve Stem Seal / Oil Consumption (xDrive50i)</x:v>
+      </x:c>
+      <x:c r="E502" s="9" t="str">
+        <x:v>Replace valve stem seals - extremely labor-intensive job requiring cylinder head work ($4,900-12,000 total). Elring seals 11340039494 ($80-120/set of 16, need 2 sets for V8). 5150 AutoSport Viton upgraded seals ($150-200) are recommended for better heat resistance in hot-vee configuration. AGA Tools kit AGA-N63-VSK-K ($500-800) includes specialized tools required. Reference TSB MC-10149960-9999 when visiting dealer. Some owners monitor oil levels and add as needed rather than repair. Use quality synthetic 0W-40 BMW LL-01 spec oil.</x:v>
+      </x:c>
+      <x:c r="F502" s="9" t="str">
+        <x:v>Split N63 revisions/generations; oil-consumption and smoke diagnosis; exact valve-stem seals; head-on/head-off method by equipped specialist; tooling not sold as repair part</x:v>
+      </x:c>
+      <x:c r="G502" s="9" t="str">
+        <x:v>GENERATION / SERVICE-METHOD GATE</x:v>
+      </x:c>
+      <x:c r="H502" s="9" t="str">
+        <x:v>Genuine BMW X6 valve-seal catalog</x:v>
+      </x:c>
+      <x:c r="I502" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x6-valve_stem_seal.html</x:v>
+      </x:c>
+      <x:c r="J502" s="9" t="str">
+        <x:v>2008-2023 X6; VIN, N63 revision, and quantity required</x:v>
+      </x:c>
+      <x:c r="K502" s="9" t="str">
+        <x:v>OEM seal catalog</x:v>
+      </x:c>
+      <x:c r="L502" s="9" t="str"/>
+      <x:c r="M502" s="9" t="str">
+        <x:v>The row crosses multiple N63 revisions and the AGA item is a professional tool, not a replacement part.</x:v>
+      </x:c>
+      <x:c r="N502" s="41" t="str">
+        <x:v>Do not recommend generic Viton seals or monitoring without checking catalyst/oil-consumption risk and exact engine.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="503" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A503" s="40" t="str"/>
+      <x:c r="B503" s="9" t="str"/>
+      <x:c r="C503" s="9" t="str"/>
+      <x:c r="D503" s="9" t="str"/>
+      <x:c r="E503" s="9" t="str"/>
+      <x:c r="F503" s="9" t="str"/>
+      <x:c r="G503" s="9" t="str"/>
+      <x:c r="H503" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I503" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J503" s="9" t="str">
+        <x:v>N63 valve-seal diagnosis and equipped repair</x:v>
+      </x:c>
+      <x:c r="K503" s="9" t="str">
+        <x:v>specialist service</x:v>
+      </x:c>
+      <x:c r="L503" s="9" t="str"/>
+      <x:c r="M503" s="9" t="str"/>
+      <x:c r="N503" s="41" t="str"/>
+    </x:row>
+    <x:row r="504" ht="818.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A504" s="40" t="n">
+        <x:v>344</x:v>
+      </x:c>
+      <x:c r="B504" s="9" t="str">
+        <x:v>bmw-x6-n63-wastegate-2008</x:v>
+      </x:c>
+      <x:c r="C504" s="9" t="str">
+        <x:v>2008-2018 | BMW | X6 | M50i, xDrive50i</x:v>
+      </x:c>
+      <x:c r="D504" s="9" t="str">
+        <x:v>N63 Turbo Wastegate Rattle (xDrive50i)</x:v>
+      </x:c>
+      <x:c r="E504" s="9" t="str">
+        <x:v>Repair options range from flapper repair kits ($50-100/turbo) to complete turbocharger replacement ($4,000-8,000 for both). Garrett MGT2256S flapper repair kit ($50-100 per turbo) is cheapest fix. MAMBA adjustable actuator kit ($150-300) provides more durable solution. OEM actuators 11657646093 available from BMW. Complete turbo replacement $2,000-4,000 per turbo. MONITORING: Wastegate rattle is early warning - address before complete turbo failure to avoid $8,000+ repair.</x:v>
+      </x:c>
+      <x:c r="F504" s="9" t="str">
+        <x:v>Boost/vacuum/charge-air diagnosis; identify N63 generation, turbo number, bank, actuator/flapper serviceability; complete turbo only for confirmed severe wear</x:v>
+      </x:c>
+      <x:c r="G504" s="9" t="str">
+        <x:v>TURBO-NUMBER / GENERATION GATE</x:v>
+      </x:c>
+      <x:c r="H504" s="9" t="str">
+        <x:v>BMW X6 turbocharger catalog</x:v>
+      </x:c>
+      <x:c r="I504" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x6-turbocharger.html</x:v>
+      </x:c>
+      <x:c r="J504" s="9" t="str">
+        <x:v>2008-2018 E71/F16 xDrive50i; VIN, engine revision, bank, and turbo number required</x:v>
+      </x:c>
+      <x:c r="K504" s="9" t="str">
+        <x:v>OEM turbo catalog</x:v>
+      </x:c>
+      <x:c r="L504" s="9" t="str"/>
+      <x:c r="M504" s="9" t="str">
+        <x:v>Garrett/MAMBA/OEM part claims were not verified across every turbo and engine revision.</x:v>
+      </x:c>
+      <x:c r="N504" s="41" t="str">
+        <x:v>Rattle alone is not proof of imminent turbo failure; approve repair hardware only by exact turbo number.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="505" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A505" s="40" t="str"/>
+      <x:c r="B505" s="9" t="str"/>
+      <x:c r="C505" s="9" t="str"/>
+      <x:c r="D505" s="9" t="str"/>
+      <x:c r="E505" s="9" t="str"/>
+      <x:c r="F505" s="9" t="str"/>
+      <x:c r="G505" s="9" t="str"/>
+      <x:c r="H505" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I505" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J505" s="9" t="str">
+        <x:v>boost/wastegate diagnosis</x:v>
+      </x:c>
+      <x:c r="K505" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L505" s="9" t="str"/>
+      <x:c r="M505" s="9" t="str"/>
+      <x:c r="N505" s="41" t="str"/>
+    </x:row>
+    <x:row r="506" ht="409.20001220703125" hidden="0" customHeight="1">
+      <x:c r="A506" s="40" t="n">
+        <x:v>345</x:v>
+      </x:c>
+      <x:c r="B506" s="9" t="str">
+        <x:v>bmw-x6-rear-differential-bushing-2008</x:v>
+      </x:c>
+      <x:c r="C506" s="9" t="str">
+        <x:v>2008-2026 | BMW | X6</x:v>
+      </x:c>
+      <x:c r="D506" s="9" t="str">
+        <x:v>Rear Differential Bushing Deterioration</x:v>
+      </x:c>
+      <x:c r="E506" s="9" t="str">
+        <x:v>Replace all rear differential mount bushings. Use OEM or equivalent quality bushings (Lemforder is the OEM supplier). Inspect the differential housing for any damage from excessive movement. Perform subframe alignment check after bushing replacement.</x:v>
+      </x:c>
+      <x:c r="F506" s="9" t="str">
+        <x:v>Generation/VIN/position-specific mount inspection; exact failed bushing/mount; housing/subframe check; alignment only if repair procedure disturbs geometry</x:v>
+      </x:c>
+      <x:c r="G506" s="9" t="str">
+        <x:v>THREE-GENERATION / POSITION SPLIT</x:v>
+      </x:c>
+      <x:c r="H506" s="9" t="str">
+        <x:v>BMW X6 differential-mount catalog</x:v>
+      </x:c>
+      <x:c r="I506" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x6-differential_mount.html</x:v>
+      </x:c>
+      <x:c r="J506" s="9" t="str">
+        <x:v>2008-2026 E71/F16/G06 X6; VIN, axle unit, and mount position required</x:v>
+      </x:c>
+      <x:c r="K506" s="9" t="str">
+        <x:v>OEM mount catalog</x:v>
+      </x:c>
+      <x:c r="L506" s="9" t="str"/>
+      <x:c r="M506" s="9" t="str">
+        <x:v>The row spans three generations; no single Lemforder/OEM bushing or 'all bushings' set applies.</x:v>
+      </x:c>
+      <x:c r="N506" s="41" t="str">
+        <x:v>Replace diagnosed mounts, verify supplier/fitment per part, and do not require alignment universally.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="507" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A507" s="40" t="str"/>
+      <x:c r="B507" s="9" t="str"/>
+      <x:c r="C507" s="9" t="str"/>
+      <x:c r="D507" s="9" t="str"/>
+      <x:c r="E507" s="9" t="str"/>
+      <x:c r="F507" s="9" t="str"/>
+      <x:c r="G507" s="9" t="str"/>
+      <x:c r="H507" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I507" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J507" s="9" t="str">
+        <x:v>driveline mount diagnosis</x:v>
+      </x:c>
+      <x:c r="K507" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L507" s="9" t="str"/>
+      <x:c r="M507" s="9" t="str"/>
+      <x:c r="N507" s="41" t="str"/>
+    </x:row>
+    <x:row r="508" ht="765.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A508" s="40" t="n">
+        <x:v>346</x:v>
+      </x:c>
+      <x:c r="B508" s="9" t="str">
+        <x:v>bmw-x6-transfer-case-2008</x:v>
+      </x:c>
+      <x:c r="C508" s="9" t="str">
+        <x:v>2008-2023 | BMW | X6</x:v>
+      </x:c>
+      <x:c r="D508" s="9" t="str">
+        <x:v>Transfer Case Actuator Motor Failure (All xDrive Models)</x:v>
+      </x:c>
+      <x:c r="E508" s="9" t="str">
+        <x:v>Replace the actuator motor assembly or rebuild using an aftermarket gear repair kit ($100-150). G06 actuator motor 27609469023 ($400-600) for complete replacement. DIY gear repair kits are straightforward and save $1,200+ over dealer replacement. Complete transfer case replacement if internal damage occurred: $1,400-3,300. PREVENTIVE: If buying used X6 over 80k miles, budget for this repair and listen for clicking noise when shutting off ignition.</x:v>
+      </x:c>
+      <x:c r="F508" s="9" t="str">
+        <x:v>VTG/DSC diagnosis; split E71/F16/G06 units; tire/voltage/wiring/fluid/calibration checks; exact actuator or internal repair only after confirmation</x:v>
+      </x:c>
+      <x:c r="G508" s="9" t="str">
+        <x:v>THREE-GENERATION TRANSFER-CASE SPLIT</x:v>
+      </x:c>
+      <x:c r="H508" s="9" t="str">
+        <x:v>BMW X6 transfer-case catalog</x:v>
+      </x:c>
+      <x:c r="I508" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x6-transfer_case.html</x:v>
+      </x:c>
+      <x:c r="J508" s="9" t="str">
+        <x:v>2008-2023 xDrive X6; VIN and exact unit required</x:v>
+      </x:c>
+      <x:c r="K508" s="9" t="str">
+        <x:v>OEM drivetrain catalog</x:v>
+      </x:c>
+      <x:c r="L508" s="9" t="str"/>
+      <x:c r="M508" s="9" t="str">
+        <x:v>One G06 actuator number and generic gear kit cannot cover E71/F16/G06.</x:v>
+      </x:c>
+      <x:c r="N508" s="41" t="str">
+        <x:v>Remove 'straightforward,' fixed savings, clicking-only diagnosis, and blanket used-car prediction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="509" ht="66" hidden="0" customHeight="1">
+      <x:c r="A509" s="40" t="str"/>
+      <x:c r="B509" s="9" t="str"/>
+      <x:c r="C509" s="9" t="str"/>
+      <x:c r="D509" s="9" t="str"/>
+      <x:c r="E509" s="9" t="str"/>
+      <x:c r="F509" s="9" t="str"/>
+      <x:c r="G509" s="9" t="str"/>
+      <x:c r="H509" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I509" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J509" s="9" t="str">
+        <x:v>VTG diagnosis and initialization</x:v>
+      </x:c>
+      <x:c r="K509" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L509" s="9" t="str"/>
+      <x:c r="M509" s="9" t="str"/>
+      <x:c r="N509" s="41" t="str"/>
+    </x:row>
+    <x:row r="510" ht="514.7999877929688" hidden="0" customHeight="1">
+      <x:c r="A510" s="40" t="n">
+        <x:v>347</x:v>
+      </x:c>
+      <x:c r="B510" s="9" t="str">
+        <x:v>bmw-x6m-front-thrust-arm-bushing-2015</x:v>
+      </x:c>
+      <x:c r="C510" s="9" t="str">
+        <x:v>2015-2025 | BMW | X6 M</x:v>
+      </x:c>
+      <x:c r="D510" s="9" t="str">
+        <x:v>Front Thrust Arm Bushing (Tension Strut) Premature Wear</x:v>
+      </x:c>
+      <x:c r="E510" s="9" t="str">
+        <x:v>Replace both front thrust arms as complete assemblies (the bushings are not serviceable separately). Use genuine BMW M-spec parts or Lemforder equivalents. Perform a 4-wheel alignment immediately after replacement. Upgrade to Powerflex polyurethane thrust arm bushings for extended lifespan, especially on tracked cars.</x:v>
+      </x:c>
+      <x:c r="F510" s="9" t="str">
+        <x:v>Split F86/F96; side-specific thrust-arm/bushing/ball-joint inspection; complete arm or serviceable bushing per design; alignment; polyurethane only by NVH/use choice</x:v>
+      </x:c>
+      <x:c r="G510" s="9" t="str">
+        <x:v>GENERATION / SIDE-SPECIFIC SUSPENSION GATE</x:v>
+      </x:c>
+      <x:c r="H510" s="9" t="str">
+        <x:v>BMW X6 M control-arm catalog</x:v>
+      </x:c>
+      <x:c r="I510" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/X6-M/Control-Arm/</x:v>
+      </x:c>
+      <x:c r="J510" s="9" t="str">
+        <x:v>2015-2025 F86/F96 X6 M; select generation, side, position, and VIN</x:v>
+      </x:c>
+      <x:c r="K510" s="9" t="str">
+        <x:v>vehicle-specific arm catalog</x:v>
+      </x:c>
+      <x:c r="L510" s="9" t="str"/>
+      <x:c r="M510" s="9" t="str">
+        <x:v>The row crosses generations and the claim that bushings are never separately serviceable was not verified across both.</x:v>
+      </x:c>
+      <x:c r="N510" s="41" t="str">
+        <x:v>Do not require both complete arms or polyurethane without inspection and NVH discussion.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="511" ht="66" hidden="0" customHeight="1">
+      <x:c r="A511" s="40" t="str"/>
+      <x:c r="B511" s="9" t="str"/>
+      <x:c r="C511" s="9" t="str"/>
+      <x:c r="D511" s="9" t="str"/>
+      <x:c r="E511" s="9" t="str"/>
+      <x:c r="F511" s="9" t="str"/>
+      <x:c r="G511" s="9" t="str"/>
+      <x:c r="H511" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I511" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J511" s="9" t="str">
+        <x:v>suspension inspection and alignment</x:v>
+      </x:c>
+      <x:c r="K511" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L511" s="9" t="str"/>
+      <x:c r="M511" s="9" t="str"/>
+      <x:c r="N511" s="41" t="str"/>
+    </x:row>
+    <x:row r="512" ht="897.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A512" s="40" t="n">
+        <x:v>348</x:v>
+      </x:c>
+      <x:c r="B512" s="9" t="str">
+        <x:v>bmw-x6m-s63-rod-bearing-2010</x:v>
+      </x:c>
+      <x:c r="C512" s="9" t="str">
+        <x:v>2010-2023 | BMW | X6 M | M50i, xDrive50i | S63</x:v>
+      </x:c>
+      <x:c r="D512" s="9" t="str">
+        <x:v>S63 Rod Bearing Failure (X6 M)</x:v>
+      </x:c>
+      <x:c r="E512" s="9" t="str">
+        <x:v>PREVENTIVE: Replace rod bearings every 60,000-80,000 miles ($2,500-5,000 labor-intensive job). Use ACL Race 8B1578HX-STD ($150-250) or King CR8049SV ($120-200) upgraded bearings - these are stronger than OEM and provide better durability under high loads. Send oil samples for analysis (Blackstone Labs ~$30) every 5,000 miles to monitor bearing wear metals. If bearings have already failed: engine replacement required ($15,000-30,000). DO NOT buy used X6 M without documented bearing replacement history or fresh oil analysis.</x:v>
+      </x:c>
+      <x:c r="F512" s="9" t="str">
+        <x:v>S63-revision-specific diagnosis; oil pressure/noise and measured clearance; engine-builder-selected bearings/fasteners; optional oil trending</x:v>
+      </x:c>
+      <x:c r="G512" s="9" t="str">
+        <x:v>SPECULATIVE PREVENTIVE CLAIM CORRECTED</x:v>
+      </x:c>
+      <x:c r="H512" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I512" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J512" s="9" t="str">
+        <x:v>2010-2023 X6 M S63 bottom-end assessment</x:v>
+      </x:c>
+      <x:c r="K512" s="9" t="str">
+        <x:v>engine-builder service</x:v>
+      </x:c>
+      <x:c r="L512" s="9" t="str"/>
+      <x:c r="M512" s="9" t="str">
+        <x:v>The row spans several S63 revisions and prescribes aftermarket parts/intervals without clearance evidence.</x:v>
+      </x:c>
+      <x:c r="N512" s="41" t="str">
+        <x:v>Remove fixed preventive interval, universal bearing numbers, and the claim oil analysis/documentation guarantees condition.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="513" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A513" s="40" t="str"/>
+      <x:c r="B513" s="9" t="str"/>
+      <x:c r="C513" s="9" t="str"/>
+      <x:c r="D513" s="9" t="str"/>
+      <x:c r="E513" s="9" t="str"/>
+      <x:c r="F513" s="9" t="str"/>
+      <x:c r="G513" s="9" t="str"/>
+      <x:c r="H513" s="9" t="str">
+        <x:v>Blackstone oil-analysis kit</x:v>
+      </x:c>
+      <x:c r="I513" s="9" t="str">
+        <x:v>https://www.blackstone-labs.com/products/free-test-kits/</x:v>
+      </x:c>
+      <x:c r="J513" s="9" t="str">
+        <x:v>optional trending only; not conclusive bearing diagnosis</x:v>
+      </x:c>
+      <x:c r="K513" s="9" t="str">
+        <x:v>oil-analysis service</x:v>
+      </x:c>
+      <x:c r="L513" s="9" t="str"/>
+      <x:c r="M513" s="9" t="str"/>
+      <x:c r="N513" s="41" t="str"/>
+    </x:row>
+    <x:row r="514" ht="290.3999938964844" hidden="0" customHeight="1">
+      <x:c r="A514" s="40" t="n">
+        <x:v>349</x:v>
+      </x:c>
+      <x:c r="B514" s="9" t="str">
+        <x:v>bmw-x6m-vanos-solenoid-2015</x:v>
+      </x:c>
+      <x:c r="C514" s="9" t="str">
+        <x:v>2015-2021 | BMW | X6 M | S63</x:v>
+      </x:c>
+      <x:c r="D514" s="9" t="str">
+        <x:v>VANOS Solenoid Oil Sludge Buildup</x:v>
+      </x:c>
+      <x:c r="E514" s="9" t="str">
+        <x:v>Remove and clean or replace the VANOS solenoids. Perform an engine oil flush. Strictly follow 7,500-mile oil change intervals with BMW LL-01 rated 0W-40 synthetic oil.</x:v>
+      </x:c>
+      <x:c r="F514" s="9" t="str">
+        <x:v>BMW-capable diagnosis; engine-revision/intake/exhaust/bank identification; clean only when service procedure supports and electronics test good; exact solenoid/seals; correct oil service</x:v>
+      </x:c>
+      <x:c r="G514" s="9" t="str">
+        <x:v>GENERATION / POSITION / DIAGNOSIS GATE</x:v>
+      </x:c>
+      <x:c r="H514" s="9" t="str">
+        <x:v>BMW X6 M VANOS-solenoid catalog</x:v>
+      </x:c>
+      <x:c r="I514" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/X6-M/VANOS-Solenoid/</x:v>
+      </x:c>
+      <x:c r="J514" s="9" t="str">
+        <x:v>2015-2021 F86/F96 X6 M; select VIN, S63 revision, and position</x:v>
+      </x:c>
+      <x:c r="K514" s="9" t="str">
+        <x:v>vehicle-specific VANOS catalog</x:v>
+      </x:c>
+      <x:c r="L514" s="9" t="str"/>
+      <x:c r="M514" s="9" t="str">
+        <x:v>Sludge is not automatically cured by solenoid cleaning, and an engine flush can create risk.</x:v>
+      </x:c>
+      <x:c r="N514" s="41" t="str">
+        <x:v>Remove engine-flush instruction and fixed oil interval; diagnose oil supply, wiring, and mechanism before parts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="515" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A515" s="40" t="str"/>
+      <x:c r="B515" s="9" t="str"/>
+      <x:c r="C515" s="9" t="str"/>
+      <x:c r="D515" s="9" t="str"/>
+      <x:c r="E515" s="9" t="str"/>
+      <x:c r="F515" s="9" t="str"/>
+      <x:c r="G515" s="9" t="str"/>
+      <x:c r="H515" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I515" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J515" s="9" t="str">
+        <x:v>VANOS/oil-pressure diagnosis</x:v>
+      </x:c>
+      <x:c r="K515" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L515" s="9" t="str"/>
+      <x:c r="M515" s="9" t="str"/>
+      <x:c r="N515" s="41" t="str"/>
+    </x:row>
+    <x:row r="516" ht="699.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A516" s="40" t="n">
+        <x:v>350</x:v>
+      </x:c>
+      <x:c r="B516" s="9" t="str">
+        <x:v>bmw-x7-48v-battery-2020</x:v>
+      </x:c>
+      <x:c r="C516" s="9" t="str">
+        <x:v>2020-2023 | BMW | X7</x:v>
+      </x:c>
+      <x:c r="D516" s="9" t="str">
+        <x:v>48V Mild Hybrid Battery Issues</x:v>
+      </x:c>
+      <x:c r="E516" s="9" t="str">
+        <x:v>Replace the 48V mild hybrid battery ($1,000-2,000 at dealer). Requires dealer-level diagnostic tools and coding after installation - this is NOT a DIY repair. The 48V battery is separate from the main 12V battery. No aftermarket alternatives currently available. Check if vehicle is still under BMW warranty or extended warranty coverage. Some owners choose to live with the failed auto start-stop rather than pay for replacement.</x:v>
+      </x:c>
+      <x:c r="F516" s="9" t="str">
+        <x:v>Confirm vehicle actually has 48V system; BMW-capable energy diagnosis; warranty/VIN check; exact 48V battery only if failed; coding/commissioning</x:v>
+      </x:c>
+      <x:c r="G516" s="9" t="str">
+        <x:v>EQUIPMENT / CODING / WARRANTY GATE</x:v>
+      </x:c>
+      <x:c r="H516" s="9" t="str">
+        <x:v>BMW dealer locator</x:v>
+      </x:c>
+      <x:c r="I516" s="9" t="str">
+        <x:v>https://www.bmwusa.com/dealer-locator.html</x:v>
+      </x:c>
+      <x:c r="J516" s="9" t="str">
+        <x:v>2020-2023 X7 48V equipment confirmation, diagnosis, warranty, and coding</x:v>
+      </x:c>
+      <x:c r="K516" s="9" t="str">
+        <x:v>high-voltage-capable service</x:v>
+      </x:c>
+      <x:c r="L516" s="9" t="str"/>
+      <x:c r="M516" s="9" t="str">
+        <x:v>Not every X7 in the range has the same mild-hybrid system, and replacement requires energy diagnosis/coding.</x:v>
+      </x:c>
+      <x:c r="N516" s="41" t="str">
+        <x:v>Do not infer a failed 48V battery from start-stop behavior or advise living with an active electrical fault.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="517" ht="726" hidden="0" customHeight="1">
+      <x:c r="A517" s="40" t="n">
+        <x:v>351</x:v>
+      </x:c>
+      <x:c r="B517" s="9" t="str">
+        <x:v>bmw-x7-air-suspension-2019</x:v>
+      </x:c>
+      <x:c r="C517" s="9" t="str">
+        <x:v>2019-2023 | BMW | X7</x:v>
+      </x:c>
+      <x:c r="D517" s="9" t="str">
+        <x:v>Air Suspension Compressor &amp; Strut Failure (Standard Equipment)</x:v>
+      </x:c>
+      <x:c r="E517" s="9" t="str">
+        <x:v>Replace failed air struts and/or compressor. Front strut left 37106869035 ($1,500-2,000), right 37106869036 ($1,500-2,000), rear 37106869039 ($1,000-1,500). Compressor 37206861882 ($800-1,200). RebuildMasterTech rebuilt struts ($600-900 each) are a more affordable alternative. Total repair can reach $2,180-5,000+ depending on which components have failed. Replace both struts on same axle simultaneously. Inspect at 50,000 miles for early signs of leaking.</x:v>
+      </x:c>
+      <x:c r="F517" s="9" t="str">
+        <x:v>VIN/options/corner-specific leak and fault diagnosis; exact strut/spring/compressor/valve block; axle mate only by condition/strategy; calibration</x:v>
+      </x:c>
+      <x:c r="G517" s="9" t="str">
+        <x:v>VIN / CORNER / COMPONENT GATE</x:v>
+      </x:c>
+      <x:c r="H517" s="9" t="str">
+        <x:v>BMW X7 air-suspension catalog</x:v>
+      </x:c>
+      <x:c r="I517" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/X7/Air-Suspension/</x:v>
+      </x:c>
+      <x:c r="J517" s="9" t="str">
+        <x:v>2019-2023 G07 X7; VIN, axle, side, option, and diagnosed component required</x:v>
+      </x:c>
+      <x:c r="K517" s="9" t="str">
+        <x:v>vehicle-specific air-suspension catalog</x:v>
+      </x:c>
+      <x:c r="L517" s="9" t="str"/>
+      <x:c r="M517" s="9" t="str">
+        <x:v>The listed part numbers and rebuilt struts were not proven across all X7 builds/options.</x:v>
+      </x:c>
+      <x:c r="N517" s="41" t="str">
+        <x:v>Do not automatically replace axle pairs or use fixed 50k inspection/replacement claims.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="518" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A518" s="40" t="str"/>
+      <x:c r="B518" s="9" t="str"/>
+      <x:c r="C518" s="9" t="str"/>
+      <x:c r="D518" s="9" t="str"/>
+      <x:c r="E518" s="9" t="str"/>
+      <x:c r="F518" s="9" t="str"/>
+      <x:c r="G518" s="9" t="str"/>
+      <x:c r="H518" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I518" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J518" s="9" t="str">
+        <x:v>leak diagnosis and ride-height calibration</x:v>
+      </x:c>
+      <x:c r="K518" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L518" s="9" t="str"/>
+      <x:c r="M518" s="9" t="str"/>
+      <x:c r="N518" s="41" t="str"/>
+    </x:row>
+    <x:row r="519" ht="435.6000061035156" hidden="0" customHeight="1">
+      <x:c r="A519" s="40" t="n">
+        <x:v>352</x:v>
+      </x:c>
+      <x:c r="B519" s="9" t="str">
+        <x:v>bmw-x7-air-suspension-compressor-2019</x:v>
+      </x:c>
+      <x:c r="C519" s="9" t="str">
+        <x:v>2019-2026 | BMW | X7</x:v>
+      </x:c>
+      <x:c r="D519" s="9" t="str">
+        <x:v>Air Suspension Compressor Failure</x:v>
+      </x:c>
+      <x:c r="E519" s="9" t="str">
+        <x:v>Replace the air suspension compressor. Inspect all four air springs for leaks using soapy water solution. Replace any leaking air springs to prevent repeated compressor failure. Check the valve block for proper operation. The compressor is located under the rear of the vehicle.</x:v>
+      </x:c>
+      <x:c r="F519" s="9" t="str">
+        <x:v>Fault/power/output diagnosis; leak-test all air springs/lines/valve block; exact VIN compressor only if failed; repair leaks first; calibration</x:v>
+      </x:c>
+      <x:c r="G519" s="9" t="str">
+        <x:v>DIAGNOSIS / VIN-SPECIFIC COMPRESSOR</x:v>
+      </x:c>
+      <x:c r="H519" s="9" t="str">
+        <x:v>Genuine BMW X7 air-supply catalog</x:v>
+      </x:c>
+      <x:c r="I519" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x7-air_suspension_compressor.html</x:v>
+      </x:c>
+      <x:c r="J519" s="9" t="str">
+        <x:v>2019-2026 G07 X7; VIN and diagnosed air-supply unit required</x:v>
+      </x:c>
+      <x:c r="K519" s="9" t="str">
+        <x:v>OEM compressor catalog</x:v>
+      </x:c>
+      <x:c r="L519" s="9" t="str"/>
+      <x:c r="M519" s="9" t="str">
+        <x:v>A compressor can be damaged by leaks, but soapy-water checks alone may not isolate every valve/line/control fault.</x:v>
+      </x:c>
+      <x:c r="N519" s="41" t="str">
+        <x:v>Repair the leak/root cause before a compressor and verify exact location/procedure by VIN.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="520" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A520" s="40" t="str"/>
+      <x:c r="B520" s="9" t="str"/>
+      <x:c r="C520" s="9" t="str"/>
+      <x:c r="D520" s="9" t="str"/>
+      <x:c r="E520" s="9" t="str"/>
+      <x:c r="F520" s="9" t="str"/>
+      <x:c r="G520" s="9" t="str"/>
+      <x:c r="H520" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I520" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J520" s="9" t="str">
+        <x:v>air-leak and compressor diagnosis/calibration</x:v>
+      </x:c>
+      <x:c r="K520" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L520" s="9" t="str"/>
+      <x:c r="M520" s="9" t="str"/>
+      <x:c r="N520" s="41" t="str"/>
+    </x:row>
+    <x:row r="521" ht="871.2000122070312" hidden="0" customHeight="1">
+      <x:c r="A521" s="40" t="n">
+        <x:v>353</x:v>
+      </x:c>
+      <x:c r="B521" s="9" t="str">
+        <x:v>bmw-x7-b58-coolant-2019</x:v>
+      </x:c>
+      <x:c r="C521" s="9" t="str">
+        <x:v>2019-2023 | BMW | X7 | xDrive40i | B58</x:v>
+      </x:c>
+      <x:c r="D521" s="9" t="str">
+        <x:v>B58 Coolant System Failures (xDrive40i)</x:v>
+      </x:c>
+      <x:c r="E521" s="9" t="str">
+        <x:v>Replace failed coolant system components. Water pump 11518482250 ($300-400). Thermostat 11537644811 ($150-250). Replace expansion tank and all plastic coolant connections when performing repair to prevent cascading failures. For 2023+ models, check VIN for recall 24V-608 coverage for coolant pump connector. Total repair $500-2,500 depending on extent of damage. PREVENTIVE: Replace thermostat and water pump at 60,000-70,000 miles before failure. Inspect coolant hoses and connections at every oil change after 50k miles.</x:v>
+      </x:c>
+      <x:c r="F521" s="9" t="str">
+        <x:v>Pressure/fault diagnosis; exact B58 generation and coolant circuit; pump/thermostat/tank/connections only if failed; VIN recall 24V-608 check where applicable</x:v>
+      </x:c>
+      <x:c r="G521" s="9" t="str">
+        <x:v>RECALL / ENGINE-REVISION / CIRCUIT GATE</x:v>
+      </x:c>
+      <x:c r="H521" s="9" t="str">
+        <x:v>BMW recall lookup</x:v>
+      </x:c>
+      <x:c r="I521" s="9" t="str">
+        <x:v>https://www.bmwusa.com/safety-and-emission-recalls.html</x:v>
+      </x:c>
+      <x:c r="J521" s="9" t="str">
+        <x:v>VIN check for 24V-608 or related coolant-pump action</x:v>
+      </x:c>
+      <x:c r="K521" s="9" t="str">
+        <x:v>manufacturer recall route</x:v>
+      </x:c>
+      <x:c r="L521" s="9" t="str"/>
+      <x:c r="M521" s="9" t="str">
+        <x:v>The source bundles several components and part numbers across revisions while making preventive claims.</x:v>
+      </x:c>
+      <x:c r="N521" s="41" t="str">
+        <x:v>Do not replace all plastic connections/pump/thermostat/tank from one fault or use fixed 60-70k intervals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="522" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A522" s="40" t="str"/>
+      <x:c r="B522" s="9" t="str"/>
+      <x:c r="C522" s="9" t="str"/>
+      <x:c r="D522" s="9" t="str"/>
+      <x:c r="E522" s="9" t="str"/>
+      <x:c r="F522" s="9" t="str"/>
+      <x:c r="G522" s="9" t="str"/>
+      <x:c r="H522" s="9" t="str">
+        <x:v>BMW X7 cooling catalog</x:v>
+      </x:c>
+      <x:c r="I522" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/X7/Cooling-System/</x:v>
+      </x:c>
+      <x:c r="J522" s="9" t="str">
+        <x:v>2019-2023 xDrive40i; VIN, B58 revision, and failed circuit/component required</x:v>
+      </x:c>
+      <x:c r="K522" s="9" t="str">
+        <x:v>vehicle-specific cooling catalog</x:v>
+      </x:c>
+      <x:c r="L522" s="9" t="str"/>
+      <x:c r="M522" s="9" t="str"/>
+      <x:c r="N522" s="41" t="str"/>
+    </x:row>
+    <x:row r="523" ht="435.6000061035156" hidden="0" customHeight="1">
+      <x:c r="A523" s="40" t="n">
+        <x:v>354</x:v>
+      </x:c>
+      <x:c r="B523" s="9" t="str">
+        <x:v>bmw-x7-b58-coolant-expansion-tank-2019</x:v>
+      </x:c>
+      <x:c r="C523" s="9" t="str">
+        <x:v>2019-2026 | BMW | X7 | B58</x:v>
+      </x:c>
+      <x:c r="D523" s="9" t="str">
+        <x:v>B58 Coolant Expansion Tank Crack</x:v>
+      </x:c>
+      <x:c r="E523" s="9" t="str">
+        <x:v>Replace the coolant expansion tank with an updated BMW part that uses improved plastic composition. Also replace the cap and inspect all coolant hoses. Flush and refill the cooling system with BMW-approved coolant. Check for coolant contamination from the old tank.</x:v>
+      </x:c>
+      <x:c r="F523" s="9" t="str">
+        <x:v>Pressure-test/confirm tank crack; VIN/circuit-specific expansion tank and cap by condition; hose inspection; correct coolant/bleed/retest</x:v>
+      </x:c>
+      <x:c r="G523" s="9" t="str">
+        <x:v>VIN / COOLING-CIRCUIT GATE</x:v>
+      </x:c>
+      <x:c r="H523" s="9" t="str">
+        <x:v>BMW X7 expansion-tank catalog</x:v>
+      </x:c>
+      <x:c r="I523" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/X7/Expansion-Tank/</x:v>
+      </x:c>
+      <x:c r="J523" s="9" t="str">
+        <x:v>2019-2026 G07 X7; VIN, engine, and coolant circuit required</x:v>
+      </x:c>
+      <x:c r="K523" s="9" t="str">
+        <x:v>vehicle-specific tank catalog</x:v>
+      </x:c>
+      <x:c r="L523" s="9" t="str"/>
+      <x:c r="M523" s="9" t="str">
+        <x:v>An exact updated part/supersession and 'improved plastic' claim were not verified for every build/circuit.</x:v>
+      </x:c>
+      <x:c r="N523" s="41" t="str">
+        <x:v>Do not promise an updated material; replace cap/hoses only if required by condition/procedure.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="524" ht="646.7999877929688" hidden="0" customHeight="1">
+      <x:c r="A524" s="40" t="n">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="B524" s="9" t="str">
+        <x:v>bmw-x7-ibs-brake-recall-2023</x:v>
+      </x:c>
+      <x:c r="C524" s="9" t="str">
+        <x:v>2023-2025 | BMW | X7</x:v>
+      </x:c>
+      <x:c r="D524" s="9" t="str">
+        <x:v>2023-2025 X7 Integrated Brake System Recall 26V-422</x:v>
+      </x:c>
+      <x:c r="E524" s="9" t="str">
+        <x:v>Check the VIN at NHTSA and with an authorized BMW dealer when campaign 26V-422 VINs become searchable, and arrange the free dealer inspection and module replacement if required. If a brake warning appears or pedal effort increases, avoid abrupt braking, allow extra stopping distance, stop safely and contact BMW roadside assistance; do not order brake electronics from this card.</x:v>
+      </x:c>
+      <x:c r="F524" s="9" t="str">
+        <x:v>VIN recall 26V-422 check; free dealer inspection/module replacement if required; safety response for warning/increased pedal effort</x:v>
+      </x:c>
+      <x:c r="G524" s="9" t="str">
+        <x:v>RECALL ROUTES ONLY</x:v>
+      </x:c>
+      <x:c r="H524" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I524" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J524" s="9" t="str">
+        <x:v>VIN check for 26V-422</x:v>
+      </x:c>
+      <x:c r="K524" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L524" s="9" t="str"/>
+      <x:c r="M524" s="9" t="str">
+        <x:v>The repair is an authorized safety recall and the article correctly rejects retail brake electronics.</x:v>
+      </x:c>
+      <x:c r="N524" s="41" t="str">
+        <x:v>Keep the safety instructions and VIN gate primary.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="525" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A525" s="42" t="str"/>
+      <x:c r="B525" s="43" t="str"/>
+      <x:c r="C525" s="43" t="str"/>
+      <x:c r="D525" s="43" t="str"/>
+      <x:c r="E525" s="43" t="str"/>
+      <x:c r="F525" s="43" t="str"/>
+      <x:c r="G525" s="43" t="str"/>
+      <x:c r="H525" s="43" t="str">
+        <x:v>BMW recall lookup</x:v>
+      </x:c>
+      <x:c r="I525" s="43" t="str">
+        <x:v>https://www.bmwusa.com/safety-and-emission-recalls.html</x:v>
+      </x:c>
+      <x:c r="J525" s="43" t="str">
+        <x:v>manufacturer VIN/campaign status</x:v>
+      </x:c>
+      <x:c r="K525" s="43" t="str">
+        <x:v>manufacturer recall remedy</x:v>
+      </x:c>
+      <x:c r="L525" s="43" t="str"/>
+      <x:c r="M525" s="43" t="str"/>
+      <x:c r="N525" s="44" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -17980,90 +19792,90 @@
         <x:v>Queue status</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="1042.800048828125" hidden="0" customHeight="1">
+    <x:row r="2" ht="897.5999755859375" hidden="0" customHeight="1">
       <x:c r="A2" s="40" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>bmw-x5-transfer-case-actuator-2007</x:v>
+        <x:v>bmw-x7-n63-oil-consumption-2019</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>2019-2026 | BMW | X5</x:v>
+        <x:v>2019-2023 | BMW | X7 | M50i, M60i, xDrive50i | N63TU3</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
-        <x:v>G05/F95 Transfer-Case Shudder: Tires and Fluid Diagnosis First</x:v>
+        <x:v>N63TU3 Oil Consumption &amp; Valve Stem Seal Degradation (xDrive50i/M50i/M60i)</x:v>
       </x:c>
       <x:c r="E2" s="9" t="str">
-        <x:v>Follow BMW SIB 27 02 20 in order: verify all four tires for VIN-correct size, brand/application, axle placement, and wear; diagnose any powertrain faults; then use ISTA to temporarily deactivate the transfer-case clutch and road-test the complaint. Only if the shudder disappears with the VTG deactivated does BMW direct an ATX13-X oil change with DTF-1, followed by VTG calibration. The clutch plates can require up to 125 miles after the service to become fully saturated and smooth out. If the symptom remains, continue diagnosis rather than buying an actuator or transfer case. Part numbers for any further repair must be selected by VIN in ETK/AIR.</x:v>
+        <x:v>Replace valve stem seals - extremely labor-intensive job requiring cylinder head work ($4,900-12,000 total). Elring seals 11340039494 for OEM spec. 5150 AutoSport Viton upgraded seals ($150-200) recommended for better heat resistance. AGA Tools kit includes specialized tools required. Reference TSB MC-10149960-9999 when visiting dealer. Check eligibility for class action settlement coverage. Some owners monitor oil levels and top off rather than repair. Use quality synthetic 0W-40 BMW LL-01 spec oil and check level every 500-1,000 miles.</x:v>
       </x:c>
       <x:c r="F2" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G2" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="1214.4000244140625" hidden="0" customHeight="1">
+    <x:row r="3" ht="396" hidden="0" customHeight="1">
       <x:c r="A3" s="40" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>bmw-x5-vanos-solenoid-2000</x:v>
+        <x:v>bmw-x7-panoramic-roof-rattle-2019</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
-        <x:v>2010-2013 | BMW | X5 | xDrive30i, xDrive35i | N51, N52K, N52T, N55</x:v>
+        <x:v>2019-2026 | BMW | X7</x:v>
       </x:c>
       <x:c r="D3" s="9" t="str">
-        <x:v>VANOS Adjustment-Unit Bolt Recall 23V-707 (E70 Inline-Six)</x:v>
+        <x:v>Panoramic Sunroof Rattle and Creak</x:v>
       </x:c>
       <x:c r="E3" s="9" t="str">
-        <x:v>Enter the VIN in BMW's official recall lookup and have an authorized BMW center complete recall 23V-707 if it is open. BMW's procedure is inspection-dependent: intact affected bolts are replaced; if bolts are loose or broken, the affected VANOS adjustment unit is replaced, and missing fragments must be recovered. The recall repair is free, so do not buy a solenoid or VANOS part first. If the VIN is outside the recall or a fault remains after the remedy, use BMW-capable diagnostics to test oil supply and pressure, wiring, sensors, control solenoids, adjustment units, and mechanical timing before selecting a part. If the engine runs roughly, makes unusual mechanical noise, loses power, or stalls, move out of traffic safely, stop driving, and contact BMW for transport guidance.</x:v>
+        <x:v>Apply BMW-approved felt tape or lubricant to sunroof guide rails. Replace worn guide rail bushings. In severe cases, the sunroof cassette or seal may need replacement under warranty. BMW has issued updated guide rail components for early production vehicles.</x:v>
       </x:c>
       <x:c r="F3" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G3" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="1148.4000244140625" hidden="0" customHeight="1">
+    <x:row r="4" ht="778.7999877929688" hidden="0" customHeight="1">
       <x:c r="A4" s="40" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>bmw-x5-water-pump-2007</x:v>
+        <x:v>bmw-x7-sunroof-leak-2019</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>2011-2013 | BMW | X5 | xDrive35i | N55</x:v>
+        <x:v>2019-2023 | BMW | X7</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
-        <x:v>E70 xDrive35i N55 Electric Coolant Pump (Fault-Confirmed)</x:v>
+        <x:v>Panoramic Sunroof Water Leak</x:v>
       </x:c>
       <x:c r="E4" s="9" t="str">
-        <x:v>If the engine-temperature warning appears, stop safely, shut the engine off, and tow the vehicle if normal temperature cannot be confirmed. When cool, check coolant level and leaks, read BMW-specific faults, verify pump power/ground and communication, and run the ISTA coolant-pump activation/test plan. If those tests confirm the pump and BMW ETK/AIR selects 11-51-5-A05-704 for the VIN, replace it using the BMW procedure, select the thermostat separately only if testing or preventive planning justifies it, vacuum-fill or bleed the system as specified, and verify commanded pump operation and stable temperature. Do not use a fixed-mileage rule or this part number for an N52, N63, or F15 without VIN confirmation.</x:v>
+        <x:v>Clear clogged sunroof drain tubes ($100-300 at shop). Reference TSB SIB 54 11 19 when visiting dealer. For persistent leaks, drain tube connections or sunroof seal may need replacement ($500-1,500). If water has damaged interior electronics, repair costs can reach $3,000. PREVENTIVE: Clear sunroof drains annually, especially in areas with heavy tree debris. Run compressed air or flexible drain snake through drain tubes during oil changes. Keep sunroof track clean of debris.</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G4" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="1056" hidden="0" customHeight="1">
+    <x:row r="5" ht="739.2000122070312" hidden="0" customHeight="1">
       <x:c r="A5" s="40" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>bmw-x5m-brake-system-2010</x:v>
+        <x:v>bmw-x7-tire-wear-2019</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>2010-2023 | BMW | X5 M</x:v>
+        <x:v>2019-2023 | BMW | X7</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Heavy-Duty Brake System Accelerated Wear - E70/F85/F95 X5 M</x:v>
+        <x:v>Premature Tire Wear (Especially 21"/22" Wheels)</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>E70 X5 M brakes: OEM front pads 34116799964 ($150-$250), rear pads 34216794879 ($120-$200). F85 X5 M front brake rotors: 34112284101/34112284102 with 6-pot caliper 34117845747/34117845748 and pads 34112284869. F85 rear: 385mm x 24mm perforated rotors 34212284903/34212284904 with 4-pot Brembo caliper and Textar pads. Budget $1,500-$2,500 per axle for complete brake service. For track use: EBC Yellowstuff or Hawk HPS 5.0 pads ($200-$350 per axle) with StopTech slotted rotors for improved heat management. Use Motul RBF 660 or ATE Typ 200 brake fluid - flush every 12 months. Budget $3,000-$5,000 per year for brake maintenance if driving spiritedly.</x:v>
+        <x:v>Have alignment adjusted to reduce aggressive camber settings ($200-400). Switch to quality tires designed for heavy SUVs: Michelin Pilot Sport 4S or Continental PremiumContact 6 are recommended. If possible, avoid 22" wheels and opt for 21" or smaller for better tire longevity and ride comfort. Alignment adjustment can extend tire life from 15,000 to 30,000+ miles. Total cost $200-2,000 depending on tire replacement needs. Check alignment every 10,000 miles.</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
         <x:v>0</x:v>
@@ -18072,21 +19884,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="1122" hidden="0" customHeight="1">
+    <x:row r="6" ht="501.6000061035156" hidden="0" customHeight="1">
       <x:c r="A6" s="40" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>bmw-x5m-rear-differential-2010</x:v>
+        <x:v>bmw-xm-airbag-passenger-knee-recall-2023</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
-        <x:v>2010-2023 | BMW | X5 M | S63</x:v>
+        <x:v>2023-2023 | BMW | XM</x:v>
       </x:c>
       <x:c r="D6" s="9" t="str">
-        <x:v>Rear Differential Wear &amp; Fluid Degradation - E70/F85/F95 X5 M</x:v>
+        <x:v>2023 XM Front-Passenger Knee-Airbag Recall 23V-622</x:v>
       </x:c>
       <x:c r="E6" s="9" t="str">
-        <x:v>Change rear differential fluid every 30,000 miles (ignore BMW "lifetime fill" claim). E70 X5 M: No drain plug - fluid must be extracted through fill port with hand pump or suction device. Recommended fluid: Royal Purple 75W-140 GL5 synthetic or Red Line 75W-140 GL5 ($40-$60 per fill). Capacity approximately 1.2 liters. For limited-slip diff, ensure fluid is GL5 rated with limited-slip additive. If differential is making whining/howling noise: have a limited-slip differential specialist inspect internals (not generic BMW shop). Diff rebuild: $1,500-$3,000 at specialist. Complete differential replacement: $3,000-$5,500 + labor. Labor for fluid change: $150-$300 at independent shop.</x:v>
+        <x:v>Check the VIN for an open 23V-622 campaign. If open, an authorized BMW dealer replaces the front-passenger knee airbag free of charge. Do not attempt airbag diagnosis or order a clock spring or airbag module from this card; supplemental-restraint work requires trained personnel and VIN-selected parts.</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
         <x:v>0</x:v>
@@ -18095,21 +19907,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="1386" hidden="0" customHeight="1">
+    <x:row r="7" ht="567.5999755859375" hidden="0" customHeight="1">
       <x:c r="A7" s="40" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>bmw-x5m-s63-cooling-system-2010</x:v>
+        <x:v>bmw-xm-hybrid-drivetrain-hesitation-2023</x:v>
       </x:c>
       <x:c r="C7" s="9" t="str">
-        <x:v>2010-2023 | BMW | X5 M | 4.4i, 4.6is, 4.8is, M50i, M60i, xDrive48i, xDrive50e, xDrive50i | S63</x:v>
+        <x:v>2023-2024 | BMW | XM | S68 4.4L Twin-Turbo V8 Hybrid, S68</x:v>
       </x:c>
       <x:c r="D7" s="9" t="str">
-        <x:v>S63 Cooling System Component Failures - E70/F85/F95 X5 M</x:v>
+        <x:v>Hybrid Drivetrain Hesitation and Power Delivery Lag</x:v>
       </x:c>
       <x:c r="E7" s="9" t="str">
-        <x:v>PROACTIVE MAINTENANCE SCHEDULE: Replace electric water pump at 60,000 miles ($400-$700 + labor). Replace thermostat at same time ($150-$250). Replace expansion tank at 60,000-80,000 miles ($100-$200). Inspect all coolant hoses at every oil change - replace any that are soft, bulging, or showing surface cracks. E70 X5 M expansion tank vent hose: 17128627119 ($30-$50). Flush coolant system every 2 years or 30,000 miles (more frequent than BMW's 4-year recommendation). Use ONLY BMW coolant mixed 50/50 with distilled water. For E70 hot-V turbo coolant lines: GRYPHONTEK repair kit eliminates plastic T-fitting failure (see separate issue entry). Budget $1,500-$2,500 for complete cooling system refresh at 60,000 miles. This prevents catastrophic overheating that can destroy the S63 engine ($15,000-$34,000 engine replacement).</x:v>
+        <x:v>Visit the dealer for the latest transmission and hybrid system software calibration updates. Select Sport or Sport Plus mode for more consistent power delivery. The latest software revisions significantly improve the electric-to-V8 handoff smoothness. If hesitation persists after updates, the dealer can reset the transmission adaptation values to relearn driving patterns.</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
         <x:v>0</x:v>
@@ -18118,21 +19930,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="1135.199951171875" hidden="0" customHeight="1">
+    <x:row r="8" ht="646.7999877929688" hidden="0" customHeight="1">
       <x:c r="A8" s="40" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>bmw-x5m-s63-oil-leaks-2010</x:v>
+        <x:v>bmw-xm-integrated-brake-system-recall-2023</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
-        <x:v>2010-2023 | BMW | X5 M | 4.4i, 4.6is, 4.8is, M50i, M60i, xDrive48i, xDrive50e, xDrive50i | S63</x:v>
+        <x:v>2023-2024 | BMW | XM</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
-        <x:v>S63 V8 Chronic Oil Leaks (Valve Cover, Oil Pan, Turbo Lines) - E70/F85/F95 X5 M</x:v>
+        <x:v>2023-2024 XM Integrated Brake System Recall 26V-422</x:v>
       </x:c>
       <x:c r="E8" s="9" t="str">
-        <x:v>Valve cover gasket replacement (both sides): $1,200-$2,500 with labor. BMW plastic valve covers can crack and must be replaced entirely (not just gasket) - inspect during service. Oil filter housing gasket: $400-$800 with labor. Oil pan gasket: $2,000-$3,500 (requires engine/subframe drop). Turbo oil feed/return lines: replace with GRYPHONTEK or MAMBA upgraded silicone/braided lines during any turbo service ($200-$400). VANOS solenoid seals: $100-$200 (DIY-friendly). For comprehensive oil leak repair at 80,000+ miles: budget $3,000-$5,000 to address all common leak points simultaneously. Valve cover bolt torque is CRITICAL - too tight cracks the cover ($800-$1,200 per cover), too loose and it leaks.</x:v>
+        <x:v>Check the VIN at NHTSA and with an authorized BMW dealer when campaign 26V-422 VINs become searchable, and arrange the free dealer inspection and module replacement if required. If a brake warning appears or pedal effort increases, avoid abrupt braking, allow extra stopping distance, stop safely and contact BMW roadside assistance; wheel-speed sensors are not the recall remedy.</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
         <x:v>0</x:v>
@@ -18141,21 +19953,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="1412.4000244140625" hidden="0" customHeight="1">
+    <x:row r="9" ht="646.7999877929688" hidden="0" customHeight="1">
       <x:c r="A9" s="40" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>bmw-x5m-s63-rod-bearing-2010</x:v>
+        <x:v>bmw-xm-suspension-ride-quality-2023</x:v>
       </x:c>
       <x:c r="C9" s="9" t="str">
-        <x:v>2010-2018 | BMW | X5 M | 4.4i, 4.6is, 4.8is, M50i, M60i, xDrive48i, xDrive50e, xDrive50i</x:v>
+        <x:v>2023-2024 | BMW | XM | S68 4.4L Twin-Turbo V8 Hybrid</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str">
-        <x:v>S63 V8 Rod Bearing Premature Wear &amp; Failure - E70/F85 X5 M</x:v>
+        <x:v>Harsh Ride Quality and Suspension Stiffness</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
-        <x:v>PREVENTIVE: For track-driven X5 M, replace rod bearings proactively at 60,000-80,000 miles. ACL Race Series rod bearings (8B1578HX-STD for S63B44, +0.001" extra oil clearance) are the community gold standard ($200-$350 for bearing set). WPC surface-treated bearings from Lang Racing are the premium choice ($400-$600 set). Total cost for preventive rod bearing service: $4,500-$8,500 depending on shop. Oil analysis every 5,000 miles through Blackstone Labs ($30/test) to monitor bearing wear metals (lead and copper). Use only BMW 10W-60 synthetic oil with 5,000-7,500 mile oil change intervals. Never track the car on cold oil. Mporium BMW offers specialized S63 rod bearing service starting at $4,499. If catastrophic failure: rebuilt S63 engine from RK Autowerks (~$8,500 + installation), new BMW engine (~$34,000), or complete engine rebuild ($12,000-$18,000).</x:v>
+        <x:v>Check tire pressures regularly - overinflated tires significantly worsen the harsh ride. Some owners report improved comfort by switching to a tire with a taller sidewall profile (if available for the XM's wheel size). Use Comfort mode for daily driving. Unfortunately, no aftermarket spring or damper solution currently exists to significantly improve the ride without compromising the handling needed for the XM's weight.</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
         <x:v>0</x:v>
@@ -18164,21 +19976,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="1214.4000244140625" hidden="0" customHeight="1">
+    <x:row r="10" ht="528" hidden="0" customHeight="1">
       <x:c r="A10" s="40" t="n">
         <x:v>9</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>bmw-x5m-s63-turbo-coolant-line-2010</x:v>
+        <x:v>bmw-z3-convertible-top-rear-window-cracking-clouding-bead-separatio</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
-        <x:v>2010-2013 | BMW | X5 M</x:v>
+        <x:v>1996-2002 | BMW | Z3</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
-        <x:v>S63 Turbo Coolant Line Plastic T-Fitting Failure (Hot-V Design) - E70 X5 M</x:v>
+        <x:v>Convertible Top Rear Window Cracking, Clouding, and Bead Separation</x:v>
       </x:c>
       <x:c r="E10" s="9" t="str">
-        <x:v>Replace ALL factory plastic turbo coolant T-fittings and hoses with GRYPHONTEK S63 Turbo Coolant Line Repair Kit ($200-$400). Kit includes pre-shaped multi-layer reinforced silicone hoses, brass T-fittings (replacing factory plastic), and all necessary hose clamps. Direct bolt-on installation designed for the E70/E71 S63 engine bay. MAMBA Turbo also offers a reinforced turbo coolant line kit with brass and silicone components ($150-$350). This is a PROACTIVE replacement - do not wait for failure. Replace at first sign of coolant weeping or during any turbo service. Labor: $800-$1,500 due to tight access in hot-V engine valley. If turbo bearings are damaged from overheating: turbo replacement $3,000-$5,000 per unit.</x:v>
+        <x:v>Replace the rear window panel only — BMW used a zipper system so the clouded/cracked window unzips and a new window zips/tapes in without disturbing the fabric top. Re-gluing separated bead trim rarely holds, so window replacement is the durable fix. Job is a DIY-feasible 1-1.5 hours; replace the whole top only if the fabric is also degraded.</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
         <x:v>0</x:v>
@@ -18187,22 +19999,20 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="1135.199951171875" hidden="0" customHeight="1">
+    <x:row r="11" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A11" s="40" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>bmw-x5m-s63-vanos-solenoid-2010</x:v>
+        <x:v>bmw-z3-cooling-system-failure-1996</x:v>
       </x:c>
       <x:c r="C11" s="9" t="str">
-        <x:v>2010-2023 | BMW | X5 M | 4.4i, 4.6is, 4.8is, M50i, M60i, xDrive48i, xDrive50e, xDrive50i | S63</x:v>
+        <x:v>1996-2002 | BMW | Z3</x:v>
       </x:c>
       <x:c r="D11" s="9" t="str">
-        <x:v>S63 VANOS Solenoid Failure - E70/F85/F95 X5 M</x:v>
-      </x:c>
-      <x:c r="E11" s="9" t="str">
-        <x:v>Replace all 4 VANOS solenoids simultaneously - they are same age and if one has failed, others are close behind. Pierburg 11368605123 (OEM supplier) at $30-$50 each from Turner Motorsport or BimmerWorld. Genuine BMW 11368482268 for S63TU applications at $50-$70 each. Total parts cost: $120-$280 for all 4 solenoids. Also replace VANOS solenoid O-rings and filter screens during service. Labor: 1-2 hours professional ($150-$400 labor). This is one of the easier S63 repairs - accessible from top of engine without removing intake manifold. Natafox and Febi also offer quality aftermarket VANOS solenoids at lower cost ($20-$35 each). Clean VANOS system with fresh oil change immediately after solenoid replacement.</x:v>
-      </x:c>
+        <x:v>Cooling System Component Failures</x:v>
+      </x:c>
+      <x:c r="E11" s="9" t="str"/>
       <x:c r="F11" s="9" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -18210,21 +20020,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="1293.5999755859375" hidden="0" customHeight="1">
+    <x:row r="12" ht="448.79998779296875" hidden="0" customHeight="1">
       <x:c r="A12" s="40" t="n">
         <x:v>11</x:v>
       </x:c>
       <x:c r="B12" s="9" t="str">
-        <x:v>bmw-x5m-s63-wastegate-rattle-2010</x:v>
+        <x:v>bmw-z3-cracked-exhaust-manifold-1-9l-4-cylinder</x:v>
       </x:c>
       <x:c r="C12" s="9" t="str">
-        <x:v>2010-2018 | BMW | X5 M | S63</x:v>
+        <x:v>1996-2002 | BMW | Z3 | 1.9, 1.9i, Z3 1.9 | 1.9L M44 4-cylinder, 1.9L M43TU 4-cylinder</x:v>
       </x:c>
       <x:c r="D12" s="9" t="str">
-        <x:v>S63 Twin Turbo Wastegate Rattle - E70/F85 X5 M</x:v>
+        <x:v>Cracked Exhaust Manifold on 1.9L 4-Cylinder (M44/M43)</x:v>
       </x:c>
       <x:c r="E12" s="9" t="str">
-        <x:v>Option 1 (Most cost-effective): MAMBA SUS316 stainless steel wastegate rattle flapper repair kit for S63 MGT2260 (part 077-0024, replaces 790463-2 / 790484-3), approximately $150-$300 per turbo. Requires turbo removal for installation. Option 2: Lskioer turbo wastegate rattle flapper repair kit for S63/S63TU MGT2260DSL ($80-$150 per kit on Amazon). Option 3: Replace turbo wastegate actuators with new OEM units ($300-$500 each). Option 4: Full turbocharger replacement with new or remanufactured units ($3,000-$5,000 per turbo + labor). Labor for turbo removal and reinstallation: $2,000-$3,500 for both turbos. While turbos are out: replace turbo oil feed/return lines, coolant lines, and all gaskets (GRYPHONTEK turbo coolant line repair kit for E70 X5M, ~$200-$400).</x:v>
+        <x:v>Inspect the manifold for hairline cracks (a cold-engine listen or smoke test confirms the leak). Replace the cracked manifold with a used OE unit or an aftermarket stainless tubular header, and renew the manifold gasket and hardware. Allow roughly 3-4 hours labor.</x:v>
       </x:c>
       <x:c r="F12" s="9" t="n">
         <x:v>0</x:v>
@@ -18233,21 +20043,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="1069.199951171875" hidden="0" customHeight="1">
+    <x:row r="13" ht="686.4000244140625" hidden="0" customHeight="1">
       <x:c r="A13" s="40" t="n">
         <x:v>12</x:v>
       </x:c>
       <x:c r="B13" s="9" t="str">
-        <x:v>bmw-x5m-transfer-case-actuator-2010</x:v>
+        <x:v>bmw-z3-differential-mount-ear-trunk-floor-pan-tearing</x:v>
       </x:c>
       <x:c r="C13" s="9" t="str">
-        <x:v>2010-2023 | BMW | X5 M</x:v>
+        <x:v>1996-2002 | BMW | Z3</x:v>
       </x:c>
       <x:c r="D13" s="9" t="str">
-        <x:v>xDrive Transfer Case Actuator Motor Failure - E70/F85/F95 X5 M</x:v>
+        <x:v>Differential Mount Ear and Trunk Floor Pan Tearing</x:v>
       </x:c>
       <x:c r="E13" s="9" t="str">
-        <x:v>Replace transfer case actuator motor. E70 X5 M: BMW 27107566296 or equivalent ($250-$450 for actuator motor). F85 X5 M: BMW 27608643153 or equivalent ($300-$500). F95 X5 M: check VIN-specific part number with dealer. FCP Euro has an excellent DIY guide for BMW transfer case actuator repair - the actuator can be replaced without removing the entire transfer case. Labor: 2-3 hours at specialist shop ($300-$600 labor). Change transfer case fluid at same time with BMW DTF-1 specification fluid. XeMODeX offers remanufactured transfer case actuator motors at reduced cost ($200-$350). For complete transfer case failure: $3,500-$6,000 for replacement unit + labor.</x:v>
+        <x:v>Inspect the trunk floor around the differential mount and rear subframe pickup points for cracks, torn metal, and broken spot welds. Repair requires welding and a reinforcement/re-fabrication plate kit to tie the diff mount/subframe back into the floor. Switching the diff carrier bushings to polyurethane reduces carrier movement and the stress that causes the tearing. Catching it early greatly limits the repair scope.</x:v>
       </x:c>
       <x:c r="F13" s="9" t="n">
         <x:v>0</x:v>
@@ -18256,21 +20066,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="435.6000061035156" hidden="0" customHeight="1">
+    <x:row r="14" ht="514.7999877929688" hidden="0" customHeight="1">
       <x:c r="A14" s="40" t="n">
         <x:v>13</x:v>
       </x:c>
       <x:c r="B14" s="9" t="str">
-        <x:v>bmw-x6-adaptive-drive-malfunction-2008</x:v>
+        <x:v>bmw-z3-door-window-regulator-clip-mounting-tab-failure</x:v>
       </x:c>
       <x:c r="C14" s="9" t="str">
-        <x:v>2008-2019 | BMW | X6</x:v>
+        <x:v>1996-2002 | BMW | Z3</x:v>
       </x:c>
       <x:c r="D14" s="9" t="str">
-        <x:v>Adaptive Drive System Malfunction</x:v>
+        <x:v>Door Window Regulator Clip / Mounting Tab Failure</x:v>
       </x:c>
       <x:c r="E14" s="9" t="str">
-        <x:v>Diagnose specific Adaptive Drive component failure using BMW ISTA diagnostics. Replace the failed component — most commonly the hydraulic pump or valve block. If repair cost is prohibitive, some owners convert to conventional anti-roll bars as a permanent fix at lower cost.</x:v>
+        <x:v>Replace the broken plastic regulator clips, or replace the regulator assembly if the cable or mechanism is also worn. If the welded mounting tab/anchor has torn from the door frame, it must be re-welded or reinforced before fitting a new regulator. Lubricate the window channels to reduce drag on the new parts.</x:v>
       </x:c>
       <x:c r="F14" s="9" t="n">
         <x:v>0</x:v>
@@ -18279,21 +20089,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="858" hidden="0" customHeight="1">
+    <x:row r="15" ht="686.4000244140625" hidden="0" customHeight="1">
       <x:c r="A15" s="40" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="B15" s="9" t="str">
-        <x:v>bmw-x6-air-suspension-2008</x:v>
+        <x:v>bmw-z3-fuel-level-sender-failure-causing-erratic-dead-fuel-gauge</x:v>
       </x:c>
       <x:c r="C15" s="9" t="str">
-        <x:v>2008-2023 | BMW | X6</x:v>
+        <x:v>1996-2002 | BMW | Z3</x:v>
       </x:c>
       <x:c r="D15" s="9" t="str">
-        <x:v>Air Suspension Compressor &amp; Strut Failure</x:v>
+        <x:v>Fuel Level Sender Failure Causing Erratic or Dead Fuel Gauge</x:v>
       </x:c>
       <x:c r="E15" s="9" t="str">
-        <x:v>Replace failed air springs or compressor. Arnott rear air spring A-2642 ($200-300 each). OEM F16 spring 37126795013 ($200). Arnott compressor P-2655 ($599). Or convert to coil springs: Strutmasters BB2RBM conversion kit ($1,200-1,800) permanently eliminates air suspension issues. Conversion is cheaper long-term than continued air suspension repairs. If keeping air suspension: inspect air springs at 60,000-80,000 miles for cracks/leaks before compressor damage occurs. Replace both air springs on same axle simultaneously.</x:v>
+        <x:v>Remove the access panel behind the seats and inspect the sender. A dirty or lightly worn ceramic/resistor plate can sometimes be cleaned, but a cracked plate or worn brushes requires replacing the sender unit (or the complete fuel-pump/sender carrier assembly). Also check the tank vent valve, as tank vacuum can deform the float arm. Confirm wiring/ground integrity before condemning the sender.</x:v>
       </x:c>
       <x:c r="F15" s="9" t="n">
         <x:v>0</x:v>
@@ -18302,21 +20112,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="646.7999877929688" hidden="0" customHeight="1">
+    <x:row r="16" ht="488.3999938964844" hidden="0" customHeight="1">
       <x:c r="A16" s="40" t="n">
         <x:v>15</x:v>
       </x:c>
       <x:c r="B16" s="9" t="str">
-        <x:v>bmw-x6-ibs-brake-recall-2023</x:v>
+        <x:v>bmw-z3-hvac-blower-final-stage-resistor-failure</x:v>
       </x:c>
       <x:c r="C16" s="9" t="str">
-        <x:v>2024-2024 | BMW | X6</x:v>
+        <x:v>1996-2002 | BMW | Z3</x:v>
       </x:c>
       <x:c r="D16" s="9" t="str">
-        <x:v>2024 X6 Integrated Brake System Recall 26V-422</x:v>
+        <x:v>HVAC Blower Final Stage Resistor Failure (Fan Only Works on Max)</x:v>
       </x:c>
       <x:c r="E16" s="9" t="str">
-        <x:v>Check the VIN at NHTSA and with an authorized BMW dealer when campaign 26V-422 VINs become searchable, and arrange the free dealer inspection and module replacement if required. If a brake warning appears or pedal effort increases, avoid abrupt braking, allow extra stopping distance, stop safely and contact BMW roadside assistance; do not order brake electronics from this card.</x:v>
+        <x:v>Replace the blower final stage resistor (A/C cars: part under the scuttle/cowl; non-A/C cars: behind the passenger footwell panel). If a new resistor does not restore all speeds, test the blower motor itself, which may also be worn. Inspect for corrosion/water intrusion at the cowl on A/C cars.</x:v>
       </x:c>
       <x:c r="F16" s="9" t="n">
         <x:v>0</x:v>
@@ -18325,21 +20135,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="924" hidden="0" customHeight="1">
+    <x:row r="17" ht="1584" hidden="0" customHeight="1">
       <x:c r="A17" s="40" t="n">
         <x:v>16</x:v>
       </x:c>
       <x:c r="B17" s="9" t="str">
-        <x:v>bmw-x6-n63-timing-chain-2008</x:v>
+        <x:v>bmw-z3-rear-subframe-crack-1996</x:v>
       </x:c>
       <x:c r="C17" s="9" t="str">
-        <x:v>2008-2018 | BMW | X6 | M50i, xDrive50i</x:v>
+        <x:v>1996-2002 | BMW | Z3</x:v>
       </x:c>
       <x:c r="D17" s="9" t="str">
-        <x:v>N63 Timing Chain Stretch &amp; Guide Failure (E71/F16 xDrive50i)</x:v>
+        <x:v>Rear Subframe Mounting Point Cracking</x:v>
       </x:c>
       <x:c r="E17" s="9" t="str">
-        <x:v>PREVENTIVE REPLACEMENT: If you own 2008-2014 E71 xDrive50i with N63, replace timing chain guides and tensioners IMMEDIATELY at 60,000-80,000 miles ($4,000-6,000) BEFORE failure. IWIS timing chain kit 90001521 ($800-1,200) or Turner kit 11317594899KT recommended. Replace lower chain guide 11147574373 at same time. If chain has already failed: complete engine replacement required ($15,000-25,000). Check VIN with BMW dealer for extended warranty eligibility. 2015+ N63TU engines have improved timing components but still require monitoring.</x:v>
+        <x:v>Inspect the trunk floor, differential mount area, and all rear subframe mounting points from above and below the car for spot-weld separation, torn sheet metal, and cracked seams; a dye penetrant test or removing trunk trim/seam sealer may be needed to reveal early damage. If cracking is present, the proper repair is to drop the rear axle carrier/subframe, weld and reinforce the damaged unibody mounting points and trunk floor with a reinforcement kit (commonly Randy Forbes-style dual-ear/differential mount reinforcement or equivalent), then reinstall with new subframe bushings, differential mount bushings, and perform a 4-wheel alignment. Minor early cracks may be repairable before major deformation, but advanced damage often requires fabrication and extensive welding by a chassis/body specialist; typical cost ranges from about $2,000-$3,500 for early reinforcement repairs and can exceed $4,000-$6,000 if the floor is torn or multiple mounting points are damaged.</x:v>
       </x:c>
       <x:c r="F17" s="9" t="n">
         <x:v>0</x:v>
@@ -18348,22 +20158,20 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="409.20001220703125" hidden="0" customHeight="1">
+    <x:row r="18" ht="66" hidden="0" customHeight="1">
       <x:c r="A18" s="40" t="n">
         <x:v>17</x:v>
       </x:c>
       <x:c r="B18" s="9" t="str">
-        <x:v>bmw-x6-n63-valve-stem-seal-wear-2008</x:v>
+        <x:v>bmw-z3-rear-subframe-cracking-1996</x:v>
       </x:c>
       <x:c r="C18" s="9" t="str">
-        <x:v>2008-2019 | BMW | X6 | N63</x:v>
+        <x:v>1996-2002 | BMW | Z3 | M52, M54</x:v>
       </x:c>
       <x:c r="D18" s="9" t="str">
-        <x:v>N63 Valve Stem Seal Degradation and Oil Burning</x:v>
-      </x:c>
-      <x:c r="E18" s="9" t="str">
-        <x:v>Replace all intake and exhaust valve stem seals. This is a major job requiring head work. Also replace turbo oil return lines and update engine software per BMW N63 Customer Care Package specifications. Ensure proper oil grade (BMW LL-01) is used.</x:v>
-      </x:c>
+        <x:v>Rear Subframe Mounting Point Cracks</x:v>
+      </x:c>
+      <x:c r="E18" s="9" t="str"/>
       <x:c r="F18" s="9" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -18371,21 +20179,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="858" hidden="0" customHeight="1">
+    <x:row r="19" ht="475.20001220703125" hidden="0" customHeight="1">
       <x:c r="A19" s="40" t="n">
         <x:v>18</x:v>
       </x:c>
       <x:c r="B19" s="9" t="str">
-        <x:v>bmw-x6-n63-valve-stem-seals-2008</x:v>
+        <x:v>bmw-z3-valve-cover-gasket-oil-leak</x:v>
       </x:c>
       <x:c r="C19" s="9" t="str">
-        <x:v>2008-2023 | BMW | X6 | M50i, xDrive50i | N63</x:v>
+        <x:v>1997-2002 | BMW | Z3 | 2.3, 2.5i, 2.8, 3.0i | M52 2.8, M52TU 2.5/2.8, M54 2.5/3.0</x:v>
       </x:c>
       <x:c r="D19" s="9" t="str">
-        <x:v>N63 Valve Stem Seal / Oil Consumption (xDrive50i)</x:v>
+        <x:v>Valve Cover Gasket Oil Leak (M52/M54 6-Cylinder)</x:v>
       </x:c>
       <x:c r="E19" s="9" t="str">
-        <x:v>Replace valve stem seals - extremely labor-intensive job requiring cylinder head work ($4,900-12,000 total). Elring seals 11340039494 ($80-120/set of 16, need 2 sets for V8). 5150 AutoSport Viton upgraded seals ($150-200) are recommended for better heat resistance in hot-vee configuration. AGA Tools kit AGA-N63-VSK-K ($500-800) includes specialized tools required. Reference TSB MC-10149960-9999 when visiting dealer. Some owners monitor oil levels and add as needed rather than repair. Use quality synthetic 0W-40 BMW LL-01 spec oil.</x:v>
+        <x:v>Replace the valve cover gasket, the spark-plug-well/grommet seals, and the cover bolt seals. On M54 engines also clean oil from the plug wells and replace any oil-contaminated coil boots/coils. Use the correct torque sequence to avoid re-leaking. Inspect the cover for warping or cracks while it is off.</x:v>
       </x:c>
       <x:c r="F19" s="9" t="n">
         <x:v>0</x:v>
@@ -18394,21 +20202,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="818.4000244140625" hidden="0" customHeight="1">
+    <x:row r="20" ht="1293.5999755859375" hidden="0" customHeight="1">
       <x:c r="A20" s="40" t="n">
         <x:v>19</x:v>
       </x:c>
       <x:c r="B20" s="9" t="str">
-        <x:v>bmw-x6-n63-wastegate-2008</x:v>
+        <x:v>bmw-z3-vanos-seals-1999</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>2008-2018 | BMW | X6 | M50i, xDrive50i</x:v>
+        <x:v>1999-2002 | BMW | Z3 | M52, M54, S52</x:v>
       </x:c>
       <x:c r="D20" s="9" t="str">
-        <x:v>N63 Turbo Wastegate Rattle (xDrive50i)</x:v>
+        <x:v>VANOS Seal Failure (M52/M54/S52)</x:v>
       </x:c>
       <x:c r="E20" s="9" t="str">
-        <x:v>Repair options range from flapper repair kits ($50-100/turbo) to complete turbocharger replacement ($4,000-8,000 for both). Garrett MGT2256S flapper repair kit ($50-100 per turbo) is cheapest fix. MAMBA adjustable actuator kit ($150-300) provides more durable solution. OEM actuators 11657646093 available from BMW. Complete turbo replacement $2,000-4,000 per turbo. MONITORING: Wastegate rattle is early warning - address before complete turbo failure to avoid $8,000+ repair.</x:v>
+        <x:v>Confirm the fault by checking for cold-start VANOS rattle, rough idle, hesitation, and scanning for cam timing or mixture-related fault codes; on M52TU/M54/S52 engines, inspect VANOS operation and rule out vacuum leaks before disassembly. Repair typically involves removing the valve cover and VANOS unit, replacing the internal piston seals/O-rings with updated Viton/Teflon seals, renewing the valve cover gasket and VANOS oil line sealing washers, and then re-timing the cams to BMW specifications if required. If the unit still rattles after resealing, the VANOS bearing/anti-rattle components or the complete VANOS assembly may need replacement. Typical cost is about $60-$150 in seals/gaskets for DIY repair, $300-$700 for an independent shop reseal, or $800-$1,500+ if a rebuilt/replacement VANOS unit is installed.</x:v>
       </x:c>
       <x:c r="F20" s="9" t="n">
         <x:v>0</x:v>
@@ -18417,21 +20225,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="409.20001220703125" hidden="0" customHeight="1">
+    <x:row r="21" ht="501.6000061035156" hidden="0" customHeight="1">
       <x:c r="A21" s="40" t="n">
         <x:v>20</x:v>
       </x:c>
       <x:c r="B21" s="9" t="str">
-        <x:v>bmw-x6-rear-differential-bushing-2008</x:v>
+        <x:v>bmw-z4-b58-coolant-tank-2019</x:v>
       </x:c>
       <x:c r="C21" s="9" t="str">
-        <x:v>2008-2026 | BMW | X6</x:v>
+        <x:v>2019-2026 | BMW | Z4 | B58</x:v>
       </x:c>
       <x:c r="D21" s="9" t="str">
-        <x:v>Rear Differential Bushing Deterioration</x:v>
+        <x:v>B58 Coolant Expansion Tank Cracking</x:v>
       </x:c>
       <x:c r="E21" s="9" t="str">
-        <x:v>Replace all rear differential mount bushings. Use OEM or equivalent quality bushings (Lemforder is the OEM supplier). Inspect the differential housing for any damage from excessive movement. Perform subframe alignment check after bushing replacement.</x:v>
+        <x:v>Replace the coolant expansion tank with an updated BMW part or aftermarket aluminum tank. Inspect the tank and cap regularly for signs of cracking, discoloration, or seepage. When replacing, also replace the cap and check all coolant hoses for brittleness. Flush and refill with BMW-approved coolant.</x:v>
       </x:c>
       <x:c r="F21" s="9" t="n">
         <x:v>0</x:v>
@@ -18440,21 +20248,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="765.5999755859375" hidden="0" customHeight="1">
+    <x:row r="22" ht="1306.800048828125" hidden="0" customHeight="1">
       <x:c r="A22" s="40" t="n">
         <x:v>21</x:v>
       </x:c>
       <x:c r="B22" s="9" t="str">
-        <x:v>bmw-x6-transfer-case-2008</x:v>
+        <x:v>bmw-z4-e85-convertible-top-hydraulic-2003</x:v>
       </x:c>
       <x:c r="C22" s="9" t="str">
-        <x:v>2008-2023 | BMW | X6</x:v>
+        <x:v>2003-2008 | BMW | Z4</x:v>
       </x:c>
       <x:c r="D22" s="9" t="str">
-        <x:v>Transfer Case Actuator Motor Failure (All xDrive Models)</x:v>
+        <x:v>Convertible Top Hydraulic Pump Motor Failure - E85 Z4</x:v>
       </x:c>
       <x:c r="E22" s="9" t="str">
-        <x:v>Replace the actuator motor assembly or rebuild using an aftermarket gear repair kit ($100-150). G06 actuator motor 27609469023 ($400-600) for complete replacement. DIY gear repair kits are straightforward and save $1,200+ over dealer replacement. Complete transfer case replacement if internal damage occurred: $1,400-3,300. PREVENTIVE: If buying used X6 over 80k miles, budget for this repair and listen for clicking noise when shutting off ignition.</x:v>
+        <x:v>Replace hydraulic pump motor assembly (BMW 54347193448 / supersedes 54347119633). OEM Genuine BMW pump: $800-$1,200. Aftermarket alternatives available on Amazon for $150-$300 but quality varies significantly. Dealer labor is $1,500-$2,500+ as BMW procedure requires full top removal. ZRoadster.org members have documented a motor relocation to the boot/trunk area which allows much easier future access. Hydraulic fluid: use Aral Vitamol ZHM or BMW 54340394395 hydraulic oil. PREVENTION: Clean drain holes annually, ensure rubber bungs are properly seated, and check for water intrusion in pump area at every service. Some owners have had success with pump motor rebuilds from roofmotors.co.uk ($300-$500) but quality of rebuilds varies.</x:v>
       </x:c>
       <x:c r="F22" s="9" t="n">
         <x:v>0</x:v>
@@ -18463,21 +20271,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="514.7999877929688" hidden="0" customHeight="1">
+    <x:row r="23" ht="1135.199951171875" hidden="0" customHeight="1">
       <x:c r="A23" s="40" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="B23" s="9" t="str">
-        <x:v>bmw-x6m-front-thrust-arm-bushing-2015</x:v>
+        <x:v>bmw-z4-e85-window-regulator-2003</x:v>
       </x:c>
       <x:c r="C23" s="9" t="str">
-        <x:v>2015-2025 | BMW | X6 M</x:v>
+        <x:v>2003-2008 | BMW | Z4</x:v>
       </x:c>
       <x:c r="D23" s="9" t="str">
-        <x:v>Front Thrust Arm Bushing (Tension Strut) Premature Wear</x:v>
+        <x:v>Power Window Regulator Failure - E85 Z4</x:v>
       </x:c>
       <x:c r="E23" s="9" t="str">
-        <x:v>Replace both front thrust arms as complete assemblies (the bushings are not serviceable separately). Use genuine BMW M-spec parts or Lemforder equivalents. Perform a 4-wheel alignment immediately after replacement. Upgrade to Powerflex polyurethane thrust arm bushings for extended lifespan, especially on tracked cars.</x:v>
+        <x:v>Option 1 (Budget): Window regulator repair kit - replacement cables and rollers for ~$18-$25 from eBay/Amazon (BWR974 for left/driver side). Requires removing door panel and threading new cables through existing regulator frame. DIY-friendly with Z4-forum.com guides. Option 2 (Recommended): Full window regulator replacement. Driver side: BMW 51337198909 ($180-$280 OEM, $80-$150 aftermarket). Passenger side: BMW 51337198910 ($180-$280 OEM, $80-$150 aftermarket). Labor: $200-$400 at independent shop, $500-$700+ at dealer. DIY: 2-3 hours with door panel removal guide from Pelican Parts. ZRoadster.org recommends full replacement over repair kit for long-term reliability.</x:v>
       </x:c>
       <x:c r="F23" s="9" t="n">
         <x:v>0</x:v>
@@ -18486,21 +20294,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="897.5999755859375" hidden="0" customHeight="1">
+    <x:row r="24" ht="514.7999877929688" hidden="0" customHeight="1">
       <x:c r="A24" s="40" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="B24" s="9" t="str">
-        <x:v>bmw-x6m-s63-rod-bearing-2010</x:v>
+        <x:v>bmw-z4-electric-steering-rack-2003</x:v>
       </x:c>
       <x:c r="C24" s="9" t="str">
-        <x:v>2010-2023 | BMW | X6 M | M50i, xDrive50i | S63</x:v>
+        <x:v>2012-2012 | BMW | Z4</x:v>
       </x:c>
       <x:c r="D24" s="9" t="str">
-        <x:v>S63 Rod Bearing Failure (X6 M)</x:v>
+        <x:v>2012 Z4 Electric Power-Steering Recall 12V-302</x:v>
       </x:c>
       <x:c r="E24" s="9" t="str">
-        <x:v>PREVENTIVE: Replace rod bearings every 60,000-80,000 miles ($2,500-5,000 labor-intensive job). Use ACL Race 8B1578HX-STD ($150-250) or King CR8049SV ($120-200) upgraded bearings - these are stronger than OEM and provide better durability under high loads. Send oil samples for analysis (Blackstone Labs ~$30) every 5,000 miles to monitor bearing wear metals. If bearings have already failed: engine replacement required ($15,000-30,000). DO NOT buy used X6 M without documented bearing replacement history or fresh oil analysis.</x:v>
+        <x:v>Check the VIN for an open 12V-302 campaign. If open, an authorized BMW dealer replaces the steering-assistance module free of charge. If the steering warning and audible alert occur, maintain control, reduce speed, stop safely and arrange dealer or roadside assistance; do not replace a steering rack from this card.</x:v>
       </x:c>
       <x:c r="F24" s="9" t="n">
         <x:v>0</x:v>
@@ -18509,21 +20317,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="277.20001220703125" hidden="0" customHeight="1">
+    <x:row r="25" ht="633.5999755859375" hidden="0" customHeight="1">
       <x:c r="A25" s="40" t="n">
         <x:v>24</x:v>
       </x:c>
       <x:c r="B25" s="9" t="str">
-        <x:v>bmw-x6m-vanos-solenoid-2015</x:v>
+        <x:v>bmw-z4-electric-water-pump-2006</x:v>
       </x:c>
       <x:c r="C25" s="9" t="str">
-        <x:v>2015-2021 | BMW | X6 M | S63</x:v>
+        <x:v>2012-2016 | BMW | Z4 | N20</x:v>
       </x:c>
       <x:c r="D25" s="9" t="str">
-        <x:v>VANOS Solenoid Oil Sludge Buildup</x:v>
+        <x:v>2012-2016 Z4 sDrive28i Water-Pump Connector Recall 24V-608</x:v>
       </x:c>
       <x:c r="E25" s="9" t="str">
-        <x:v>Remove and clean or replace the VANOS solenoids. Perform an engine oil flush. Strictly follow 7,500-mile oil change intervals with BMW LL-01 rated 0W-40 synthetic oil.</x:v>
+        <x:v>Check the VIN for an open 24V-608 campaign. If open, an authorized BMW dealer inspects the water pump and connector, replaces them if necessary, and installs the protective shield free of charge. If smoke appears from the engine compartment, stop safely, switch off the vehicle, have occupants exit, move away from traffic and call emergency or roadside assistance; do not order a pump from this card.</x:v>
       </x:c>
       <x:c r="F25" s="9" t="n">
         <x:v>0</x:v>
@@ -18532,44 +20340,44 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="699.5999755859375" hidden="0" customHeight="1">
+    <x:row r="26" ht="1359.5999755859375" hidden="0" customHeight="1">
       <x:c r="A26" s="40" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="B26" s="9" t="str">
-        <x:v>bmw-x7-48v-battery-2020</x:v>
+        <x:v>bmw-z4-g29-b58-water-pump-2019</x:v>
       </x:c>
       <x:c r="C26" s="9" t="str">
-        <x:v>2020-2023 | BMW | X7</x:v>
+        <x:v>2019-2025 | BMW | Z4 | M40i, sDrive35i, sDrive35is | B48, B58</x:v>
       </x:c>
       <x:c r="D26" s="9" t="str">
-        <x:v>48V Mild Hybrid Battery Issues</x:v>
+        <x:v>B48/B58 Electric Water Pump &amp; Thermostat Failure - G29 Z4</x:v>
       </x:c>
       <x:c r="E26" s="9" t="str">
-        <x:v>Replace the 48V mild hybrid battery ($1,000-2,000 at dealer). Requires dealer-level diagnostic tools and coding after installation - this is NOT a DIY repair. The 48V battery is separate from the main 12V battery. No aftermarket alternatives currently available. Check if vehicle is still under BMW warranty or extended warranty coverage. Some owners choose to live with the failed auto start-stop rather than pay for replacement.</x:v>
+        <x:v>Preventative replacement recommended at 60,000 miles. Always replace water pump and thermostat together - they share labor overlap and frequently fail concurrently. B48 sDrive30i: Water pump BMW 11518632586 ($300-$450), Thermostat BMW 11538685978 ($100-$150). B58 M40i: Water pump BMW 11518650986 ($350-$500), Thermostat BMW 11538685978 ($100-$150). Mishimoto offers performance water pump alternatives for B58 with improved impeller design. Replace 3 O-rings between thermostat and pump housing, plus 2 O-rings on coolant tube to head. Must replace water pump mounting bolts (torque-to-yield). Labor: 3-4 hours. FCP Euro lifetime warranty kits available. Also inspect plastic cylinder head coolant outlet adapter - known to shear off causing massive coolant leak.</x:v>
       </x:c>
       <x:c r="F26" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G26" s="41" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="726" hidden="0" customHeight="1">
+    <x:row r="27" ht="1122" hidden="0" customHeight="1">
       <x:c r="A27" s="40" t="n">
         <x:v>26</x:v>
       </x:c>
       <x:c r="B27" s="9" t="str">
-        <x:v>bmw-x7-air-suspension-2019</x:v>
+        <x:v>bmw-z4-n54-hpfp-2009</x:v>
       </x:c>
       <x:c r="C27" s="9" t="str">
-        <x:v>2019-2023 | BMW | X7</x:v>
+        <x:v>2009-2011 | BMW | Z4 | M40i, sDrive35i, sDrive35is | N54</x:v>
       </x:c>
       <x:c r="D27" s="9" t="str">
-        <x:v>Air Suspension Compressor &amp; Strut Failure (Standard Equipment)</x:v>
+        <x:v>N54 High Pressure Fuel Pump (HPFP) Failure - E89 Z4 sDrive35i/35is</x:v>
       </x:c>
       <x:c r="E27" s="9" t="str">
-        <x:v>Replace failed air struts and/or compressor. Front strut left 37106869035 ($1,500-2,000), right 37106869036 ($1,500-2,000), rear 37106869039 ($1,000-1,500). Compressor 37206861882 ($800-1,200). RebuildMasterTech rebuilt struts ($600-900 each) are a more affordable alternative. Total repair can reach $2,180-5,000+ depending on which components have failed. Replace both struts on same axle simultaneously. Inspect at 50,000 miles for early signs of leaking.</x:v>
+        <x:v>Replace HPFP with latest revision Genuine BMW unit. The pump went through multiple revisions - ONLY install the latest version. Part number evolution: Original -&gt; 13517592881 (Index 10, TSB fix) -&gt; 13517616170 (latest revision, most reliable). Genuine BMW 13517616170 is the definitive fix ($350-$550 for pump). Replacement is straightforward DIY (1-2 hours) with basic tools. Also available as complete kit from FCP Euro with lifetime warranty. BMW extended warranty coverage to 10 years/120,000 miles under customer care package for original owners - check VIN eligibility. Replace low-pressure fuel sensor at same time (13537537319) as it may have been damaged by pressure fluctuations ($35-$55).</x:v>
       </x:c>
       <x:c r="F27" s="9" t="n">
         <x:v>0</x:v>
@@ -18578,21 +20386,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="435.6000061035156" hidden="0" customHeight="1">
+    <x:row r="28" ht="580.7999877929688" hidden="0" customHeight="1">
       <x:c r="A28" s="40" t="n">
         <x:v>27</x:v>
       </x:c>
       <x:c r="B28" s="9" t="str">
-        <x:v>bmw-x7-air-suspension-compressor-2019</x:v>
+        <x:v>bmw-z4-n54-wastegate-rattle-2009</x:v>
       </x:c>
       <x:c r="C28" s="9" t="str">
-        <x:v>2019-2026 | BMW | X7</x:v>
+        <x:v>2009-2010 | BMW | Z4 | N54</x:v>
       </x:c>
       <x:c r="D28" s="9" t="str">
-        <x:v>Air Suspension Compressor Failure</x:v>
+        <x:v>2009-2010 Z4 sDrive35i N54 Wastegate Diagnosis</x:v>
       </x:c>
       <x:c r="E28" s="9" t="str">
-        <x:v>Replace the air suspension compressor. Inspect all four air springs for leaks using soapy water solution. Replace any leaking air springs to prevent repeated compressor failure. Check the valve block for proper operation. The compressor is located under the rear of the vehicle.</x:v>
+        <x:v>Confirm the VIN, engine, production date, DME faults, boost-control data and noise source using current BMW diagnostic information. Check VIN-specific coverage history with BMW, recognizing that the bulletin's time/mileage window may have expired. Do not replace a turbocharger, actuator or wastegate from this card without the required diagnosis.</x:v>
       </x:c>
       <x:c r="F28" s="9" t="n">
         <x:v>0</x:v>
@@ -18601,21 +20409,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="871.2000122070312" hidden="0" customHeight="1">
+    <x:row r="29" ht="501.6000061035156" hidden="0" customHeight="1">
       <x:c r="A29" s="40" t="n">
         <x:v>28</x:v>
       </x:c>
       <x:c r="B29" s="9" t="str">
-        <x:v>bmw-x7-b58-coolant-2019</x:v>
+        <x:v>bmw-z4-soft-top-hydraulic-2003</x:v>
       </x:c>
       <x:c r="C29" s="9" t="str">
-        <x:v>2019-2023 | BMW | X7 | xDrive40i | B58</x:v>
+        <x:v>2009-2016 | BMW | Z4</x:v>
       </x:c>
       <x:c r="D29" s="9" t="str">
-        <x:v>B58 Coolant System Failures (xDrive40i)</x:v>
+        <x:v>Retractable Hard Top Hydraulic Mechanism Failure</x:v>
       </x:c>
       <x:c r="E29" s="9" t="str">
-        <x:v>Replace failed coolant system components. Water pump 11518482250 ($300-400). Thermostat 11537644811 ($150-250). Replace expansion tank and all plastic coolant connections when performing repair to prevent cascading failures. For 2023+ models, check VIN for recall 24V-608 coverage for coolant pump connector. Total repair $500-2,500 depending on extent of damage. PREVENTIVE: Replace thermostat and water pump at 60,000-70,000 miles before failure. Inspect coolant hoses and connections at every oil change after 50k miles.</x:v>
+        <x:v>Diagnose the leak location and replace the failed component. Common failure points are the main hydraulic cylinders (left and right), the hydraulic pump motor, and the flexible hoses. The hydraulic fluid should be flushed and replaced with BMW-approved CHF 11S fluid. A full system bleed is required after any repair.</x:v>
       </x:c>
       <x:c r="F29" s="9" t="n">
         <x:v>0</x:v>
@@ -18624,21 +20432,21 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="435.6000061035156" hidden="0" customHeight="1">
+    <x:row r="30" ht="1188" hidden="0" customHeight="1">
       <x:c r="A30" s="40" t="n">
         <x:v>29</x:v>
       </x:c>
       <x:c r="B30" s="9" t="str">
-        <x:v>bmw-x7-b58-coolant-expansion-tank-2019</x:v>
+        <x:v>bmw-z4-vanos-solenoid-2003</x:v>
       </x:c>
       <x:c r="C30" s="9" t="str">
-        <x:v>2019-2026 | BMW | X7 | B58</x:v>
+        <x:v>2003-2016 | BMW | Z4 | 2.5i, 3.0i, 3.0si, M40i, sDrive28i, sDrive30i, sDrive35i, sDrive35is | M54, N52, N54, N20</x:v>
       </x:c>
       <x:c r="D30" s="9" t="str">
-        <x:v>B58 Coolant Expansion Tank Crack</x:v>
+        <x:v>VANOS Solenoid &amp; System Failure - E85/E89 Z4 (All Engines)</x:v>
       </x:c>
       <x:c r="E30" s="9" t="str">
-        <x:v>Replace the coolant expansion tank with an updated BMW part that uses improved plastic composition. Also replace the cap and inspect all coolant hoses. Flush and refill the cooling system with BMW-approved coolant. Check for coolant contamination from the old tank.</x:v>
+        <x:v>Replace VANOS solenoids - inexpensive and straightforward repair. M54 (E85 2003-2005): 2 solenoids required, BMW 11361707323 ($35-$65 each). N52 (E85 2006-2008 / E89 2009-2011 28i): 2 solenoids, BMW 11367585425 ($40-$70 each). N54 (E89 35i/35is): 2 solenoids, BMW 11367585425 ($40-$70 each). N20 (E89 sDrive28i 2012-2016): 2 solenoids, BMW 11367585425 ($40-$70 each). Labor: under 1 hour for experienced mechanic, 2-3 hours DIY. Replace all solenoids at once even if only one has failed - the others are same age and will fail soon. Also replace VANOS solenoid O-rings and sealing plates during service. Clean VANOS system with Beisan Systems VANOS cleaning procedure for best results.</x:v>
       </x:c>
       <x:c r="F30" s="9" t="n">
         <x:v>0</x:v>
@@ -18647,712 +20455,26 @@
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="646.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A31" s="40" t="n">
+    <x:row r="31" ht="554.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A31" s="42" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="B31" s="9" t="str">
-        <x:v>bmw-x7-ibs-brake-recall-2023</x:v>
-      </x:c>
-      <x:c r="C31" s="9" t="str">
-        <x:v>2023-2025 | BMW | X7</x:v>
-      </x:c>
-      <x:c r="D31" s="9" t="str">
-        <x:v>2023-2025 X7 Integrated Brake System Recall 26V-422</x:v>
-      </x:c>
-      <x:c r="E31" s="9" t="str">
-        <x:v>Check the VIN at NHTSA and with an authorized BMW dealer when campaign 26V-422 VINs become searchable, and arrange the free dealer inspection and module replacement if required. If a brake warning appears or pedal effort increases, avoid abrupt braking, allow extra stopping distance, stop safely and contact BMW roadside assistance; do not order brake electronics from this card.</x:v>
-      </x:c>
-      <x:c r="F31" s="9" t="n">
+      <x:c r="B31" s="43" t="str">
+        <x:v>bmw-z8-soft-top-mechanism-2000</x:v>
+      </x:c>
+      <x:c r="C31" s="43" t="str">
+        <x:v>2000-2003 | BMW | Z8</x:v>
+      </x:c>
+      <x:c r="D31" s="43" t="str">
+        <x:v>Power Soft Top Hydraulic System and Cable Failure</x:v>
+      </x:c>
+      <x:c r="E31" s="43" t="str">
+        <x:v>Rebuild the hydraulic cylinders with new seals rather than replacing ($200 vs $2,000+). Inspect and replace frayed cables. Adjust or replace the microswitch sensors at the windshield header latch. Lubricate the top mechanism pivot points with silicone grease annually. Store the car with the top up to reduce stress on the hydraulic system.</x:v>
+      </x:c>
+      <x:c r="F31" s="43" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G31" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="897.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A32" s="40" t="n">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="B32" s="9" t="str">
-        <x:v>bmw-x7-n63-oil-consumption-2019</x:v>
-      </x:c>
-      <x:c r="C32" s="9" t="str">
-        <x:v>2019-2023 | BMW | X7 | M50i, M60i, xDrive50i | N63TU3</x:v>
-      </x:c>
-      <x:c r="D32" s="9" t="str">
-        <x:v>N63TU3 Oil Consumption &amp; Valve Stem Seal Degradation (xDrive50i/M50i/M60i)</x:v>
-      </x:c>
-      <x:c r="E32" s="9" t="str">
-        <x:v>Replace valve stem seals - extremely labor-intensive job requiring cylinder head work ($4,900-12,000 total). Elring seals 11340039494 for OEM spec. 5150 AutoSport Viton upgraded seals ($150-200) recommended for better heat resistance. AGA Tools kit includes specialized tools required. Reference TSB MC-10149960-9999 when visiting dealer. Check eligibility for class action settlement coverage. Some owners monitor oil levels and top off rather than repair. Use quality synthetic 0W-40 BMW LL-01 spec oil and check level every 500-1,000 miles.</x:v>
-      </x:c>
-      <x:c r="F32" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G32" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="396" hidden="0" customHeight="1">
-      <x:c r="A33" s="40" t="n">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="B33" s="9" t="str">
-        <x:v>bmw-x7-panoramic-roof-rattle-2019</x:v>
-      </x:c>
-      <x:c r="C33" s="9" t="str">
-        <x:v>2019-2026 | BMW | X7</x:v>
-      </x:c>
-      <x:c r="D33" s="9" t="str">
-        <x:v>Panoramic Sunroof Rattle and Creak</x:v>
-      </x:c>
-      <x:c r="E33" s="9" t="str">
-        <x:v>Apply BMW-approved felt tape or lubricant to sunroof guide rails. Replace worn guide rail bushings. In severe cases, the sunroof cassette or seal may need replacement under warranty. BMW has issued updated guide rail components for early production vehicles.</x:v>
-      </x:c>
-      <x:c r="F33" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G33" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="778.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A34" s="40" t="n">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="B34" s="9" t="str">
-        <x:v>bmw-x7-sunroof-leak-2019</x:v>
-      </x:c>
-      <x:c r="C34" s="9" t="str">
-        <x:v>2019-2023 | BMW | X7</x:v>
-      </x:c>
-      <x:c r="D34" s="9" t="str">
-        <x:v>Panoramic Sunroof Water Leak</x:v>
-      </x:c>
-      <x:c r="E34" s="9" t="str">
-        <x:v>Clear clogged sunroof drain tubes ($100-300 at shop). Reference TSB SIB 54 11 19 when visiting dealer. For persistent leaks, drain tube connections or sunroof seal may need replacement ($500-1,500). If water has damaged interior electronics, repair costs can reach $3,000. PREVENTIVE: Clear sunroof drains annually, especially in areas with heavy tree debris. Run compressed air or flexible drain snake through drain tubes during oil changes. Keep sunroof track clean of debris.</x:v>
-      </x:c>
-      <x:c r="F34" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G34" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="739.2000122070312" hidden="0" customHeight="1">
-      <x:c r="A35" s="40" t="n">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="B35" s="9" t="str">
-        <x:v>bmw-x7-tire-wear-2019</x:v>
-      </x:c>
-      <x:c r="C35" s="9" t="str">
-        <x:v>2019-2023 | BMW | X7</x:v>
-      </x:c>
-      <x:c r="D35" s="9" t="str">
-        <x:v>Premature Tire Wear (Especially 21"/22" Wheels)</x:v>
-      </x:c>
-      <x:c r="E35" s="9" t="str">
-        <x:v>Have alignment adjusted to reduce aggressive camber settings ($200-400). Switch to quality tires designed for heavy SUVs: Michelin Pilot Sport 4S or Continental PremiumContact 6 are recommended. If possible, avoid 22" wheels and opt for 21" or smaller for better tire longevity and ride comfort. Alignment adjustment can extend tire life from 15,000 to 30,000+ miles. Total cost $200-2,000 depending on tire replacement needs. Check alignment every 10,000 miles.</x:v>
-      </x:c>
-      <x:c r="F35" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G35" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="501.6000061035156" hidden="0" customHeight="1">
-      <x:c r="A36" s="40" t="n">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="B36" s="9" t="str">
-        <x:v>bmw-xm-airbag-passenger-knee-recall-2023</x:v>
-      </x:c>
-      <x:c r="C36" s="9" t="str">
-        <x:v>2023-2023 | BMW | XM</x:v>
-      </x:c>
-      <x:c r="D36" s="9" t="str">
-        <x:v>2023 XM Front-Passenger Knee-Airbag Recall 23V-622</x:v>
-      </x:c>
-      <x:c r="E36" s="9" t="str">
-        <x:v>Check the VIN for an open 23V-622 campaign. If open, an authorized BMW dealer replaces the front-passenger knee airbag free of charge. Do not attempt airbag diagnosis or order a clock spring or airbag module from this card; supplemental-restraint work requires trained personnel and VIN-selected parts.</x:v>
-      </x:c>
-      <x:c r="F36" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G36" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="567.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A37" s="40" t="n">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="B37" s="9" t="str">
-        <x:v>bmw-xm-hybrid-drivetrain-hesitation-2023</x:v>
-      </x:c>
-      <x:c r="C37" s="9" t="str">
-        <x:v>2023-2024 | BMW | XM | S68 4.4L Twin-Turbo V8 Hybrid, S68</x:v>
-      </x:c>
-      <x:c r="D37" s="9" t="str">
-        <x:v>Hybrid Drivetrain Hesitation and Power Delivery Lag</x:v>
-      </x:c>
-      <x:c r="E37" s="9" t="str">
-        <x:v>Visit the dealer for the latest transmission and hybrid system software calibration updates. Select Sport or Sport Plus mode for more consistent power delivery. The latest software revisions significantly improve the electric-to-V8 handoff smoothness. If hesitation persists after updates, the dealer can reset the transmission adaptation values to relearn driving patterns.</x:v>
-      </x:c>
-      <x:c r="F37" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G37" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="646.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A38" s="40" t="n">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="B38" s="9" t="str">
-        <x:v>bmw-xm-integrated-brake-system-recall-2023</x:v>
-      </x:c>
-      <x:c r="C38" s="9" t="str">
-        <x:v>2023-2024 | BMW | XM</x:v>
-      </x:c>
-      <x:c r="D38" s="9" t="str">
-        <x:v>2023-2024 XM Integrated Brake System Recall 26V-422</x:v>
-      </x:c>
-      <x:c r="E38" s="9" t="str">
-        <x:v>Check the VIN at NHTSA and with an authorized BMW dealer when campaign 26V-422 VINs become searchable, and arrange the free dealer inspection and module replacement if required. If a brake warning appears or pedal effort increases, avoid abrupt braking, allow extra stopping distance, stop safely and contact BMW roadside assistance; wheel-speed sensors are not the recall remedy.</x:v>
-      </x:c>
-      <x:c r="F38" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G38" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="646.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A39" s="40" t="n">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="B39" s="9" t="str">
-        <x:v>bmw-xm-suspension-ride-quality-2023</x:v>
-      </x:c>
-      <x:c r="C39" s="9" t="str">
-        <x:v>2023-2024 | BMW | XM | S68 4.4L Twin-Turbo V8 Hybrid</x:v>
-      </x:c>
-      <x:c r="D39" s="9" t="str">
-        <x:v>Harsh Ride Quality and Suspension Stiffness</x:v>
-      </x:c>
-      <x:c r="E39" s="9" t="str">
-        <x:v>Check tire pressures regularly - overinflated tires significantly worsen the harsh ride. Some owners report improved comfort by switching to a tire with a taller sidewall profile (if available for the XM's wheel size). Use Comfort mode for daily driving. Unfortunately, no aftermarket spring or damper solution currently exists to significantly improve the ride without compromising the handling needed for the XM's weight.</x:v>
-      </x:c>
-      <x:c r="F39" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G39" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="528" hidden="0" customHeight="1">
-      <x:c r="A40" s="40" t="n">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="B40" s="9" t="str">
-        <x:v>bmw-z3-convertible-top-rear-window-cracking-clouding-bead-separatio</x:v>
-      </x:c>
-      <x:c r="C40" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D40" s="9" t="str">
-        <x:v>Convertible Top Rear Window Cracking, Clouding, and Bead Separation</x:v>
-      </x:c>
-      <x:c r="E40" s="9" t="str">
-        <x:v>Replace the rear window panel only — BMW used a zipper system so the clouded/cracked window unzips and a new window zips/tapes in without disturbing the fabric top. Re-gluing separated bead trim rarely holds, so window replacement is the durable fix. Job is a DIY-feasible 1-1.5 hours; replace the whole top only if the fabric is also degraded.</x:v>
-      </x:c>
-      <x:c r="F40" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G40" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41" ht="52.79999923706055" hidden="0" customHeight="1">
-      <x:c r="A41" s="40" t="n">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="B41" s="9" t="str">
-        <x:v>bmw-z3-cooling-system-failure-1996</x:v>
-      </x:c>
-      <x:c r="C41" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D41" s="9" t="str">
-        <x:v>Cooling System Component Failures</x:v>
-      </x:c>
-      <x:c r="E41" s="9" t="str"/>
-      <x:c r="F41" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G41" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42" ht="448.79998779296875" hidden="0" customHeight="1">
-      <x:c r="A42" s="40" t="n">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="B42" s="9" t="str">
-        <x:v>bmw-z3-cracked-exhaust-manifold-1-9l-4-cylinder</x:v>
-      </x:c>
-      <x:c r="C42" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3 | 1.9, 1.9i, Z3 1.9 | 1.9L M44 4-cylinder, 1.9L M43TU 4-cylinder</x:v>
-      </x:c>
-      <x:c r="D42" s="9" t="str">
-        <x:v>Cracked Exhaust Manifold on 1.9L 4-Cylinder (M44/M43)</x:v>
-      </x:c>
-      <x:c r="E42" s="9" t="str">
-        <x:v>Inspect the manifold for hairline cracks (a cold-engine listen or smoke test confirms the leak). Replace the cracked manifold with a used OE unit or an aftermarket stainless tubular header, and renew the manifold gasket and hardware. Allow roughly 3-4 hours labor.</x:v>
-      </x:c>
-      <x:c r="F42" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G42" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43" ht="686.4000244140625" hidden="0" customHeight="1">
-      <x:c r="A43" s="40" t="n">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="B43" s="9" t="str">
-        <x:v>bmw-z3-differential-mount-ear-trunk-floor-pan-tearing</x:v>
-      </x:c>
-      <x:c r="C43" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D43" s="9" t="str">
-        <x:v>Differential Mount Ear and Trunk Floor Pan Tearing</x:v>
-      </x:c>
-      <x:c r="E43" s="9" t="str">
-        <x:v>Inspect the trunk floor around the differential mount and rear subframe pickup points for cracks, torn metal, and broken spot welds. Repair requires welding and a reinforcement/re-fabrication plate kit to tie the diff mount/subframe back into the floor. Switching the diff carrier bushings to polyurethane reduces carrier movement and the stress that causes the tearing. Catching it early greatly limits the repair scope.</x:v>
-      </x:c>
-      <x:c r="F43" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G43" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44" ht="514.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A44" s="40" t="n">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="B44" s="9" t="str">
-        <x:v>bmw-z3-door-window-regulator-clip-mounting-tab-failure</x:v>
-      </x:c>
-      <x:c r="C44" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D44" s="9" t="str">
-        <x:v>Door Window Regulator Clip / Mounting Tab Failure</x:v>
-      </x:c>
-      <x:c r="E44" s="9" t="str">
-        <x:v>Replace the broken plastic regulator clips, or replace the regulator assembly if the cable or mechanism is also worn. If the welded mounting tab/anchor has torn from the door frame, it must be re-welded or reinforced before fitting a new regulator. Lubricate the window channels to reduce drag on the new parts.</x:v>
-      </x:c>
-      <x:c r="F44" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G44" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45" ht="686.4000244140625" hidden="0" customHeight="1">
-      <x:c r="A45" s="40" t="n">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="B45" s="9" t="str">
-        <x:v>bmw-z3-fuel-level-sender-failure-causing-erratic-dead-fuel-gauge</x:v>
-      </x:c>
-      <x:c r="C45" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D45" s="9" t="str">
-        <x:v>Fuel Level Sender Failure Causing Erratic or Dead Fuel Gauge</x:v>
-      </x:c>
-      <x:c r="E45" s="9" t="str">
-        <x:v>Remove the access panel behind the seats and inspect the sender. A dirty or lightly worn ceramic/resistor plate can sometimes be cleaned, but a cracked plate or worn brushes requires replacing the sender unit (or the complete fuel-pump/sender carrier assembly). Also check the tank vent valve, as tank vacuum can deform the float arm. Confirm wiring/ground integrity before condemning the sender.</x:v>
-      </x:c>
-      <x:c r="F45" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G45" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46" ht="488.3999938964844" hidden="0" customHeight="1">
-      <x:c r="A46" s="40" t="n">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="B46" s="9" t="str">
-        <x:v>bmw-z3-hvac-blower-final-stage-resistor-failure</x:v>
-      </x:c>
-      <x:c r="C46" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D46" s="9" t="str">
-        <x:v>HVAC Blower Final Stage Resistor Failure (Fan Only Works on Max)</x:v>
-      </x:c>
-      <x:c r="E46" s="9" t="str">
-        <x:v>Replace the blower final stage resistor (A/C cars: part under the scuttle/cowl; non-A/C cars: behind the passenger footwell panel). If a new resistor does not restore all speeds, test the blower motor itself, which may also be worn. Inspect for corrosion/water intrusion at the cowl on A/C cars.</x:v>
-      </x:c>
-      <x:c r="F46" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G46" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47" ht="1584" hidden="0" customHeight="1">
-      <x:c r="A47" s="40" t="n">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="B47" s="9" t="str">
-        <x:v>bmw-z3-rear-subframe-crack-1996</x:v>
-      </x:c>
-      <x:c r="C47" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D47" s="9" t="str">
-        <x:v>Rear Subframe Mounting Point Cracking</x:v>
-      </x:c>
-      <x:c r="E47" s="9" t="str">
-        <x:v>Inspect the trunk floor, differential mount area, and all rear subframe mounting points from above and below the car for spot-weld separation, torn sheet metal, and cracked seams; a dye penetrant test or removing trunk trim/seam sealer may be needed to reveal early damage. If cracking is present, the proper repair is to drop the rear axle carrier/subframe, weld and reinforce the damaged unibody mounting points and trunk floor with a reinforcement kit (commonly Randy Forbes-style dual-ear/differential mount reinforcement or equivalent), then reinstall with new subframe bushings, differential mount bushings, and perform a 4-wheel alignment. Minor early cracks may be repairable before major deformation, but advanced damage often requires fabrication and extensive welding by a chassis/body specialist; typical cost ranges from about $2,000-$3,500 for early reinforcement repairs and can exceed $4,000-$6,000 if the floor is torn or multiple mounting points are damaged.</x:v>
-      </x:c>
-      <x:c r="F47" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G47" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48" ht="66" hidden="0" customHeight="1">
-      <x:c r="A48" s="40" t="n">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="B48" s="9" t="str">
-        <x:v>bmw-z3-rear-subframe-cracking-1996</x:v>
-      </x:c>
-      <x:c r="C48" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3 | M52, M54</x:v>
-      </x:c>
-      <x:c r="D48" s="9" t="str">
-        <x:v>Rear Subframe Mounting Point Cracks</x:v>
-      </x:c>
-      <x:c r="E48" s="9" t="str"/>
-      <x:c r="F48" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G48" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49" ht="475.20001220703125" hidden="0" customHeight="1">
-      <x:c r="A49" s="40" t="n">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="B49" s="9" t="str">
-        <x:v>bmw-z3-valve-cover-gasket-oil-leak</x:v>
-      </x:c>
-      <x:c r="C49" s="9" t="str">
-        <x:v>1997-2002 | BMW | Z3 | 2.3, 2.5i, 2.8, 3.0i | M52 2.8, M52TU 2.5/2.8, M54 2.5/3.0</x:v>
-      </x:c>
-      <x:c r="D49" s="9" t="str">
-        <x:v>Valve Cover Gasket Oil Leak (M52/M54 6-Cylinder)</x:v>
-      </x:c>
-      <x:c r="E49" s="9" t="str">
-        <x:v>Replace the valve cover gasket, the spark-plug-well/grommet seals, and the cover bolt seals. On M54 engines also clean oil from the plug wells and replace any oil-contaminated coil boots/coils. Use the correct torque sequence to avoid re-leaking. Inspect the cover for warping or cracks while it is off.</x:v>
-      </x:c>
-      <x:c r="F49" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G49" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="50" ht="1293.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A50" s="40" t="n">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="B50" s="9" t="str">
-        <x:v>bmw-z3-vanos-seals-1999</x:v>
-      </x:c>
-      <x:c r="C50" s="9" t="str">
-        <x:v>1999-2002 | BMW | Z3 | M52, M54, S52</x:v>
-      </x:c>
-      <x:c r="D50" s="9" t="str">
-        <x:v>VANOS Seal Failure (M52/M54/S52)</x:v>
-      </x:c>
-      <x:c r="E50" s="9" t="str">
-        <x:v>Confirm the fault by checking for cold-start VANOS rattle, rough idle, hesitation, and scanning for cam timing or mixture-related fault codes; on M52TU/M54/S52 engines, inspect VANOS operation and rule out vacuum leaks before disassembly. Repair typically involves removing the valve cover and VANOS unit, replacing the internal piston seals/O-rings with updated Viton/Teflon seals, renewing the valve cover gasket and VANOS oil line sealing washers, and then re-timing the cams to BMW specifications if required. If the unit still rattles after resealing, the VANOS bearing/anti-rattle components or the complete VANOS assembly may need replacement. Typical cost is about $60-$150 in seals/gaskets for DIY repair, $300-$700 for an independent shop reseal, or $800-$1,500+ if a rebuilt/replacement VANOS unit is installed.</x:v>
-      </x:c>
-      <x:c r="F50" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G50" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="51" ht="501.6000061035156" hidden="0" customHeight="1">
-      <x:c r="A51" s="40" t="n">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="B51" s="9" t="str">
-        <x:v>bmw-z4-b58-coolant-tank-2019</x:v>
-      </x:c>
-      <x:c r="C51" s="9" t="str">
-        <x:v>2019-2026 | BMW | Z4 | B58</x:v>
-      </x:c>
-      <x:c r="D51" s="9" t="str">
-        <x:v>B58 Coolant Expansion Tank Cracking</x:v>
-      </x:c>
-      <x:c r="E51" s="9" t="str">
-        <x:v>Replace the coolant expansion tank with an updated BMW part or aftermarket aluminum tank. Inspect the tank and cap regularly for signs of cracking, discoloration, or seepage. When replacing, also replace the cap and check all coolant hoses for brittleness. Flush and refill with BMW-approved coolant.</x:v>
-      </x:c>
-      <x:c r="F51" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G51" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="52" ht="1306.800048828125" hidden="0" customHeight="1">
-      <x:c r="A52" s="40" t="n">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="B52" s="9" t="str">
-        <x:v>bmw-z4-e85-convertible-top-hydraulic-2003</x:v>
-      </x:c>
-      <x:c r="C52" s="9" t="str">
-        <x:v>2003-2008 | BMW | Z4</x:v>
-      </x:c>
-      <x:c r="D52" s="9" t="str">
-        <x:v>Convertible Top Hydraulic Pump Motor Failure - E85 Z4</x:v>
-      </x:c>
-      <x:c r="E52" s="9" t="str">
-        <x:v>Replace hydraulic pump motor assembly (BMW 54347193448 / supersedes 54347119633). OEM Genuine BMW pump: $800-$1,200. Aftermarket alternatives available on Amazon for $150-$300 but quality varies significantly. Dealer labor is $1,500-$2,500+ as BMW procedure requires full top removal. ZRoadster.org members have documented a motor relocation to the boot/trunk area which allows much easier future access. Hydraulic fluid: use Aral Vitamol ZHM or BMW 54340394395 hydraulic oil. PREVENTION: Clean drain holes annually, ensure rubber bungs are properly seated, and check for water intrusion in pump area at every service. Some owners have had success with pump motor rebuilds from roofmotors.co.uk ($300-$500) but quality of rebuilds varies.</x:v>
-      </x:c>
-      <x:c r="F52" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G52" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="53" ht="1135.199951171875" hidden="0" customHeight="1">
-      <x:c r="A53" s="40" t="n">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="B53" s="9" t="str">
-        <x:v>bmw-z4-e85-window-regulator-2003</x:v>
-      </x:c>
-      <x:c r="C53" s="9" t="str">
-        <x:v>2003-2008 | BMW | Z4</x:v>
-      </x:c>
-      <x:c r="D53" s="9" t="str">
-        <x:v>Power Window Regulator Failure - E85 Z4</x:v>
-      </x:c>
-      <x:c r="E53" s="9" t="str">
-        <x:v>Option 1 (Budget): Window regulator repair kit - replacement cables and rollers for ~$18-$25 from eBay/Amazon (BWR974 for left/driver side). Requires removing door panel and threading new cables through existing regulator frame. DIY-friendly with Z4-forum.com guides. Option 2 (Recommended): Full window regulator replacement. Driver side: BMW 51337198909 ($180-$280 OEM, $80-$150 aftermarket). Passenger side: BMW 51337198910 ($180-$280 OEM, $80-$150 aftermarket). Labor: $200-$400 at independent shop, $500-$700+ at dealer. DIY: 2-3 hours with door panel removal guide from Pelican Parts. ZRoadster.org recommends full replacement over repair kit for long-term reliability.</x:v>
-      </x:c>
-      <x:c r="F53" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G53" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="54" ht="514.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A54" s="40" t="n">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="B54" s="9" t="str">
-        <x:v>bmw-z4-electric-steering-rack-2003</x:v>
-      </x:c>
-      <x:c r="C54" s="9" t="str">
-        <x:v>2012-2012 | BMW | Z4</x:v>
-      </x:c>
-      <x:c r="D54" s="9" t="str">
-        <x:v>2012 Z4 Electric Power-Steering Recall 12V-302</x:v>
-      </x:c>
-      <x:c r="E54" s="9" t="str">
-        <x:v>Check the VIN for an open 12V-302 campaign. If open, an authorized BMW dealer replaces the steering-assistance module free of charge. If the steering warning and audible alert occur, maintain control, reduce speed, stop safely and arrange dealer or roadside assistance; do not replace a steering rack from this card.</x:v>
-      </x:c>
-      <x:c r="F54" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G54" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="55" ht="633.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A55" s="40" t="n">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="B55" s="9" t="str">
-        <x:v>bmw-z4-electric-water-pump-2006</x:v>
-      </x:c>
-      <x:c r="C55" s="9" t="str">
-        <x:v>2012-2016 | BMW | Z4 | N20</x:v>
-      </x:c>
-      <x:c r="D55" s="9" t="str">
-        <x:v>2012-2016 Z4 sDrive28i Water-Pump Connector Recall 24V-608</x:v>
-      </x:c>
-      <x:c r="E55" s="9" t="str">
-        <x:v>Check the VIN for an open 24V-608 campaign. If open, an authorized BMW dealer inspects the water pump and connector, replaces them if necessary, and installs the protective shield free of charge. If smoke appears from the engine compartment, stop safely, switch off the vehicle, have occupants exit, move away from traffic and call emergency or roadside assistance; do not order a pump from this card.</x:v>
-      </x:c>
-      <x:c r="F55" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G55" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="56" ht="1359.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A56" s="40" t="n">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="B56" s="9" t="str">
-        <x:v>bmw-z4-g29-b58-water-pump-2019</x:v>
-      </x:c>
-      <x:c r="C56" s="9" t="str">
-        <x:v>2019-2025 | BMW | Z4 | M40i, sDrive35i, sDrive35is | B48, B58</x:v>
-      </x:c>
-      <x:c r="D56" s="9" t="str">
-        <x:v>B48/B58 Electric Water Pump &amp; Thermostat Failure - G29 Z4</x:v>
-      </x:c>
-      <x:c r="E56" s="9" t="str">
-        <x:v>Preventative replacement recommended at 60,000 miles. Always replace water pump and thermostat together - they share labor overlap and frequently fail concurrently. B48 sDrive30i: Water pump BMW 11518632586 ($300-$450), Thermostat BMW 11538685978 ($100-$150). B58 M40i: Water pump BMW 11518650986 ($350-$500), Thermostat BMW 11538685978 ($100-$150). Mishimoto offers performance water pump alternatives for B58 with improved impeller design. Replace 3 O-rings between thermostat and pump housing, plus 2 O-rings on coolant tube to head. Must replace water pump mounting bolts (torque-to-yield). Labor: 3-4 hours. FCP Euro lifetime warranty kits available. Also inspect plastic cylinder head coolant outlet adapter - known to shear off causing massive coolant leak.</x:v>
-      </x:c>
-      <x:c r="F56" s="9" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G56" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="57" ht="1122" hidden="0" customHeight="1">
-      <x:c r="A57" s="40" t="n">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="B57" s="9" t="str">
-        <x:v>bmw-z4-n54-hpfp-2009</x:v>
-      </x:c>
-      <x:c r="C57" s="9" t="str">
-        <x:v>2009-2011 | BMW | Z4 | M40i, sDrive35i, sDrive35is | N54</x:v>
-      </x:c>
-      <x:c r="D57" s="9" t="str">
-        <x:v>N54 High Pressure Fuel Pump (HPFP) Failure - E89 Z4 sDrive35i/35is</x:v>
-      </x:c>
-      <x:c r="E57" s="9" t="str">
-        <x:v>Replace HPFP with latest revision Genuine BMW unit. The pump went through multiple revisions - ONLY install the latest version. Part number evolution: Original -&gt; 13517592881 (Index 10, TSB fix) -&gt; 13517616170 (latest revision, most reliable). Genuine BMW 13517616170 is the definitive fix ($350-$550 for pump). Replacement is straightforward DIY (1-2 hours) with basic tools. Also available as complete kit from FCP Euro with lifetime warranty. BMW extended warranty coverage to 10 years/120,000 miles under customer care package for original owners - check VIN eligibility. Replace low-pressure fuel sensor at same time (13537537319) as it may have been damaged by pressure fluctuations ($35-$55).</x:v>
-      </x:c>
-      <x:c r="F57" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G57" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="58" ht="580.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A58" s="40" t="n">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="B58" s="9" t="str">
-        <x:v>bmw-z4-n54-wastegate-rattle-2009</x:v>
-      </x:c>
-      <x:c r="C58" s="9" t="str">
-        <x:v>2009-2010 | BMW | Z4 | N54</x:v>
-      </x:c>
-      <x:c r="D58" s="9" t="str">
-        <x:v>2009-2010 Z4 sDrive35i N54 Wastegate Diagnosis</x:v>
-      </x:c>
-      <x:c r="E58" s="9" t="str">
-        <x:v>Confirm the VIN, engine, production date, DME faults, boost-control data and noise source using current BMW diagnostic information. Check VIN-specific coverage history with BMW, recognizing that the bulletin's time/mileage window may have expired. Do not replace a turbocharger, actuator or wastegate from this card without the required diagnosis.</x:v>
-      </x:c>
-      <x:c r="F58" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G58" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="59" ht="501.6000061035156" hidden="0" customHeight="1">
-      <x:c r="A59" s="40" t="n">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="B59" s="9" t="str">
-        <x:v>bmw-z4-soft-top-hydraulic-2003</x:v>
-      </x:c>
-      <x:c r="C59" s="9" t="str">
-        <x:v>2009-2016 | BMW | Z4</x:v>
-      </x:c>
-      <x:c r="D59" s="9" t="str">
-        <x:v>Retractable Hard Top Hydraulic Mechanism Failure</x:v>
-      </x:c>
-      <x:c r="E59" s="9" t="str">
-        <x:v>Diagnose the leak location and replace the failed component. Common failure points are the main hydraulic cylinders (left and right), the hydraulic pump motor, and the flexible hoses. The hydraulic fluid should be flushed and replaced with BMW-approved CHF 11S fluid. A full system bleed is required after any repair.</x:v>
-      </x:c>
-      <x:c r="F59" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G59" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="60" ht="1188" hidden="0" customHeight="1">
-      <x:c r="A60" s="40" t="n">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="B60" s="9" t="str">
-        <x:v>bmw-z4-vanos-solenoid-2003</x:v>
-      </x:c>
-      <x:c r="C60" s="9" t="str">
-        <x:v>2003-2016 | BMW | Z4 | 2.5i, 3.0i, 3.0si, M40i, sDrive28i, sDrive30i, sDrive35i, sDrive35is | M54, N52, N54, N20</x:v>
-      </x:c>
-      <x:c r="D60" s="9" t="str">
-        <x:v>VANOS Solenoid &amp; System Failure - E85/E89 Z4 (All Engines)</x:v>
-      </x:c>
-      <x:c r="E60" s="9" t="str">
-        <x:v>Replace VANOS solenoids - inexpensive and straightforward repair. M54 (E85 2003-2005): 2 solenoids required, BMW 11361707323 ($35-$65 each). N52 (E85 2006-2008 / E89 2009-2011 28i): 2 solenoids, BMW 11367585425 ($40-$70 each). N54 (E89 35i/35is): 2 solenoids, BMW 11367585425 ($40-$70 each). N20 (E89 sDrive28i 2012-2016): 2 solenoids, BMW 11367585425 ($40-$70 each). Labor: under 1 hour for experienced mechanic, 2-3 hours DIY. Replace all solenoids at once even if only one has failed - the others are same age and will fail soon. Also replace VANOS solenoid O-rings and sealing plates during service. Clean VANOS system with Beisan Systems VANOS cleaning procedure for best results.</x:v>
-      </x:c>
-      <x:c r="F60" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G60" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="61" ht="554.4000244140625" hidden="0" customHeight="1">
-      <x:c r="A61" s="42" t="n">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="B61" s="43" t="str">
-        <x:v>bmw-z8-soft-top-mechanism-2000</x:v>
-      </x:c>
-      <x:c r="C61" s="43" t="str">
-        <x:v>2000-2003 | BMW | Z8</x:v>
-      </x:c>
-      <x:c r="D61" s="43" t="str">
-        <x:v>Power Soft Top Hydraulic System and Cable Failure</x:v>
-      </x:c>
-      <x:c r="E61" s="43" t="str">
-        <x:v>Rebuild the hydraulic cylinders with new seals rather than replacing ($200 vs $2,000+). Inspect and replace frayed cables. Adjust or replace the microswitch sensors at the windshield header latch. Lubricate the top mechanism pivot points with silicone grease annually. Store the car with the top up to reduce stress on the hydraulic system.</x:v>
-      </x:c>
-      <x:c r="F61" s="43" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G61" s="44" t="str">
+      <x:c r="G31" s="44" t="str">
         <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Complete BMW repair-first fitment review
</commit_message>
<xml_diff>
--- a/outputs/bmw-repair-first-review/BMW-repair-first-fitment-review.xlsx
+++ b/outputs/bmw-repair-first-review/BMW-repair-first-fitment-review.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R1107562feb5945bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BMW Review" sheetId="2" r:id="R3e212442ffa8471c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remaining Queue" sheetId="3" r:id="Rb4c1333bdb694861"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="4" r:id="Rac92b2d12a0042ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R126ed53da6774142"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BMW Review" sheetId="2" r:id="R9a7f8857fbf64a4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remaining Queue" sheetId="3" r:id="Rfbc97d9a80de4b67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="4" r:id="R6629f3c1e440402d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -90,7 +90,7 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="9">
+  <x:borders count="12">
     <x:border/>
     <x:border>
       <x:left/>
@@ -120,11 +120,25 @@
       <x:right/>
       <x:bottom/>
     </x:border>
+    <x:border>
+      <x:left/>
+      <x:top/>
+      <x:bottom/>
+    </x:border>
+    <x:border>
+      <x:top/>
+      <x:bottom/>
+    </x:border>
+    <x:border>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="50">
+  <x:cellXfs count="53">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -215,6 +229,15 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
@@ -484,7 +507,7 @@
         <x:v>Reviewed in this batch</x:v>
       </x:c>
       <x:c r="B5" s="13" t="n">
-        <x:v>355</x:v>
+        <x:v>385</x:v>
       </x:c>
       <x:c r="C5" s="11"/>
       <x:c r="D5" s="11"/>
@@ -498,7 +521,7 @@
         <x:v>Remaining queue</x:v>
       </x:c>
       <x:c r="B6" s="13" t="n">
-        <x:v>30</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C6" s="11"/>
       <x:c r="D6" s="11"/>
@@ -512,7 +535,7 @@
         <x:v>Issues with destinations</x:v>
       </x:c>
       <x:c r="B7" s="13" t="n">
-        <x:v>352</x:v>
+        <x:v>380</x:v>
       </x:c>
       <x:c r="C7" s="11"/>
       <x:c r="D7" s="11"/>
@@ -526,7 +549,7 @@
         <x:v>Destination entries</x:v>
       </x:c>
       <x:c r="B8" s="13" t="n">
-        <x:v>521</x:v>
+        <x:v>575</x:v>
       </x:c>
       <x:c r="C8" s="11"/>
       <x:c r="D8" s="11"/>
@@ -540,7 +563,7 @@
         <x:v>Distinct URLs</x:v>
       </x:c>
       <x:c r="B9" s="13" t="n">
-        <x:v>182</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="C9" s="11"/>
       <x:c r="D9" s="11"/>
@@ -568,7 +591,7 @@
         <x:v>Missing How to Fix</x:v>
       </x:c>
       <x:c r="B11" s="13" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C11" s="11"/>
       <x:c r="D11" s="11"/>
@@ -19728,28 +19751,1888 @@
       </x:c>
     </x:row>
     <x:row r="525" ht="79.19999694824219" hidden="0" customHeight="1">
-      <x:c r="A525" s="42" t="str"/>
-      <x:c r="B525" s="43" t="str"/>
-      <x:c r="C525" s="43" t="str"/>
-      <x:c r="D525" s="43" t="str"/>
-      <x:c r="E525" s="43" t="str"/>
-      <x:c r="F525" s="43" t="str"/>
-      <x:c r="G525" s="43" t="str"/>
-      <x:c r="H525" s="43" t="str">
+      <x:c r="A525" s="40" t="str"/>
+      <x:c r="B525" s="9" t="str"/>
+      <x:c r="C525" s="9" t="str"/>
+      <x:c r="D525" s="9" t="str"/>
+      <x:c r="E525" s="9" t="str"/>
+      <x:c r="F525" s="9" t="str"/>
+      <x:c r="G525" s="9" t="str"/>
+      <x:c r="H525" s="9" t="str">
         <x:v>BMW recall lookup</x:v>
       </x:c>
-      <x:c r="I525" s="43" t="str">
+      <x:c r="I525" s="9" t="str">
         <x:v>https://www.bmwusa.com/safety-and-emission-recalls.html</x:v>
       </x:c>
-      <x:c r="J525" s="43" t="str">
+      <x:c r="J525" s="9" t="str">
         <x:v>manufacturer VIN/campaign status</x:v>
       </x:c>
-      <x:c r="K525" s="43" t="str">
+      <x:c r="K525" s="9" t="str">
         <x:v>manufacturer recall remedy</x:v>
       </x:c>
-      <x:c r="L525" s="43" t="str"/>
-      <x:c r="M525" s="43" t="str"/>
-      <x:c r="N525" s="44" t="str"/>
+      <x:c r="L525" s="9" t="str"/>
+      <x:c r="M525" s="9" t="str"/>
+      <x:c r="N525" s="41" t="str"/>
+    </x:row>
+    <x:row r="526" ht="897.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A526" s="40" t="n">
+        <x:v>356</x:v>
+      </x:c>
+      <x:c r="B526" s="9" t="str">
+        <x:v>bmw-x7-n63-oil-consumption-2019</x:v>
+      </x:c>
+      <x:c r="C526" s="9" t="str">
+        <x:v>2019-2023 | BMW | X7 | M50i, M60i, xDrive50i | N63TU3</x:v>
+      </x:c>
+      <x:c r="D526" s="9" t="str">
+        <x:v>N63TU3 Oil Consumption &amp; Valve Stem Seal Degradation (xDrive50i/M50i/M60i)</x:v>
+      </x:c>
+      <x:c r="E526" s="9" t="str">
+        <x:v>Replace valve stem seals - extremely labor-intensive job requiring cylinder head work ($4,900-12,000 total). Elring seals 11340039494 for OEM spec. 5150 AutoSport Viton upgraded seals ($150-200) recommended for better heat resistance. AGA Tools kit includes specialized tools required. Reference TSB MC-10149960-9999 when visiting dealer. Check eligibility for class action settlement coverage. Some owners monitor oil levels and top off rather than repair. Use quality synthetic 0W-40 BMW LL-01 spec oil and check level every 500-1,000 miles.</x:v>
+      </x:c>
+      <x:c r="F526" s="9" t="str">
+        <x:v>Split xDrive50i/M50i N63TU3 from M60i S68; documented consumption/leak/PCV/turbo/combustion diagnosis; valve seals only after confirmation; warranty/settlement check</x:v>
+      </x:c>
+      <x:c r="G526" s="9" t="str">
+        <x:v>MAJOR ENGINE / MODEL SPLIT</x:v>
+      </x:c>
+      <x:c r="H526" s="9" t="str">
+        <x:v>BMW dealer locator</x:v>
+      </x:c>
+      <x:c r="I526" s="9" t="str">
+        <x:v>https://www.bmwusa.com/dealer-locator.html</x:v>
+      </x:c>
+      <x:c r="J526" s="9" t="str">
+        <x:v>2019-2023 X7 oil-consumption test, engine identification, warranty/TSB history</x:v>
+      </x:c>
+      <x:c r="K526" s="9" t="str">
+        <x:v>manufacturer-capable diagnosis</x:v>
+      </x:c>
+      <x:c r="L526" s="9" t="str"/>
+      <x:c r="M526" s="9" t="str">
+        <x:v>The source incorrectly groups the M60i's S68 with N63TU3 models and prescribes seals/oil before diagnosis.</x:v>
+      </x:c>
+      <x:c r="N526" s="41" t="str">
+        <x:v>Split M60i/S68, verify current oil specification by VIN, and do not advise monitoring/top-off as a substitute for diagnosing excessive consumption.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="527" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A527" s="40" t="str"/>
+      <x:c r="B527" s="9" t="str"/>
+      <x:c r="C527" s="9" t="str"/>
+      <x:c r="D527" s="9" t="str"/>
+      <x:c r="E527" s="9" t="str"/>
+      <x:c r="F527" s="9" t="str"/>
+      <x:c r="G527" s="9" t="str"/>
+      <x:c r="H527" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I527" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J527" s="9" t="str">
+        <x:v>N63TU3/S68 oil-source and valve-seal diagnosis</x:v>
+      </x:c>
+      <x:c r="K527" s="9" t="str">
+        <x:v>specialist service</x:v>
+      </x:c>
+      <x:c r="L527" s="9" t="str"/>
+      <x:c r="M527" s="9" t="str"/>
+      <x:c r="N527" s="41" t="str"/>
+    </x:row>
+    <x:row r="528" ht="396" hidden="0" customHeight="1">
+      <x:c r="A528" s="40" t="n">
+        <x:v>357</x:v>
+      </x:c>
+      <x:c r="B528" s="9" t="str">
+        <x:v>bmw-x7-panoramic-roof-rattle-2019</x:v>
+      </x:c>
+      <x:c r="C528" s="9" t="str">
+        <x:v>2019-2026 | BMW | X7</x:v>
+      </x:c>
+      <x:c r="D528" s="9" t="str">
+        <x:v>Panoramic Sunroof Rattle and Creak</x:v>
+      </x:c>
+      <x:c r="E528" s="9" t="str">
+        <x:v>Apply BMW-approved felt tape or lubricant to sunroof guide rails. Replace worn guide rail bushings. In severe cases, the sunroof cassette or seal may need replacement under warranty. BMW has issued updated guide rail components for early production vehicles.</x:v>
+      </x:c>
+      <x:c r="F528" s="9" t="str">
+        <x:v>Reproduce/localize rattle; inspect guides, seals, cassette, fasteners, and body flex; BMW-approved lubricant/felt only where procedure specifies; warranty/updated-parts check</x:v>
+      </x:c>
+      <x:c r="G528" s="9" t="str">
+        <x:v>SERVICE / VIN / BULLETIN GATE</x:v>
+      </x:c>
+      <x:c r="H528" s="9" t="str">
+        <x:v>BMW dealer locator</x:v>
+      </x:c>
+      <x:c r="I528" s="9" t="str">
+        <x:v>https://www.bmwusa.com/dealer-locator.html</x:v>
+      </x:c>
+      <x:c r="J528" s="9" t="str">
+        <x:v>2019-2026 G07 X7 panoramic-roof diagnosis, bulletin and warranty check</x:v>
+      </x:c>
+      <x:c r="K528" s="9" t="str">
+        <x:v>manufacturer-capable service</x:v>
+      </x:c>
+      <x:c r="L528" s="9" t="str"/>
+      <x:c r="M528" s="9" t="str">
+        <x:v>Felt, lubricant, guide parts, seals, and cassette replacement are different branches; updated components were not identified by exact bulletin/part.</x:v>
+      </x:c>
+      <x:c r="N528" s="41" t="str">
+        <x:v>Do not apply generic lubricant or sell a cassette from a creak alone.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="529" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A529" s="40" t="str"/>
+      <x:c r="B529" s="9" t="str"/>
+      <x:c r="C529" s="9" t="str"/>
+      <x:c r="D529" s="9" t="str"/>
+      <x:c r="E529" s="9" t="str"/>
+      <x:c r="F529" s="9" t="str"/>
+      <x:c r="G529" s="9" t="str"/>
+      <x:c r="H529" s="9" t="str">
+        <x:v>Genuine BMW X7 sunroof catalog</x:v>
+      </x:c>
+      <x:c r="I529" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x7-sunroof.html</x:v>
+      </x:c>
+      <x:c r="J529" s="9" t="str">
+        <x:v>VIN-specific guides/seals/cassette only after diagnosis</x:v>
+      </x:c>
+      <x:c r="K529" s="9" t="str">
+        <x:v>OEM roof catalog</x:v>
+      </x:c>
+      <x:c r="L529" s="9" t="str"/>
+      <x:c r="M529" s="9" t="str"/>
+      <x:c r="N529" s="41" t="str"/>
+    </x:row>
+    <x:row r="530" ht="778.7999877929688" hidden="0" customHeight="1">
+      <x:c r="A530" s="40" t="n">
+        <x:v>358</x:v>
+      </x:c>
+      <x:c r="B530" s="9" t="str">
+        <x:v>bmw-x7-sunroof-leak-2019</x:v>
+      </x:c>
+      <x:c r="C530" s="9" t="str">
+        <x:v>2019-2023 | BMW | X7</x:v>
+      </x:c>
+      <x:c r="D530" s="9" t="str">
+        <x:v>Panoramic Sunroof Water Leak</x:v>
+      </x:c>
+      <x:c r="E530" s="9" t="str">
+        <x:v>Clear clogged sunroof drain tubes ($100-300 at shop). Reference TSB SIB 54 11 19 when visiting dealer. For persistent leaks, drain tube connections or sunroof seal may need replacement ($500-1,500). If water has damaged interior electronics, repair costs can reach $3,000. PREVENTIVE: Clear sunroof drains annually, especially in areas with heavy tree debris. Run compressed air or flexible drain snake through drain tubes during oil changes. Keep sunroof track clean of debris.</x:v>
+      </x:c>
+      <x:c r="F530" s="9" t="str">
+        <x:v>Controlled water test; SIB 54 11 19 applicability; inspect drains/connections/seals/cassette; clear drains without disconnecting/damaging tubes; electronics/moisture assessment</x:v>
+      </x:c>
+      <x:c r="G530" s="9" t="str">
+        <x:v>SIB / LEAK-SOURCE SERVICE ROUTE</x:v>
+      </x:c>
+      <x:c r="H530" s="9" t="str">
+        <x:v>BMW dealer locator</x:v>
+      </x:c>
+      <x:c r="I530" s="9" t="str">
+        <x:v>https://www.bmwusa.com/dealer-locator.html</x:v>
+      </x:c>
+      <x:c r="J530" s="9" t="str">
+        <x:v>2019-2023 G07 X7 SIB 54 11 19 and water-leak diagnosis</x:v>
+      </x:c>
+      <x:c r="K530" s="9" t="str">
+        <x:v>manufacturer-capable service</x:v>
+      </x:c>
+      <x:c r="L530" s="9" t="str"/>
+      <x:c r="M530" s="9" t="str">
+        <x:v>Drain blockage, disconnected tube, seal, and cassette leak require different repairs.</x:v>
+      </x:c>
+      <x:c r="N530" s="41" t="str">
+        <x:v>Do not use unregulated compressed air, which can detach drain tubes; use the BMW procedure and controlled pressure/manual clearing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="531" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A531" s="40" t="str"/>
+      <x:c r="B531" s="9" t="str"/>
+      <x:c r="C531" s="9" t="str"/>
+      <x:c r="D531" s="9" t="str"/>
+      <x:c r="E531" s="9" t="str"/>
+      <x:c r="F531" s="9" t="str"/>
+      <x:c r="G531" s="9" t="str"/>
+      <x:c r="H531" s="9" t="str">
+        <x:v>BMW X7 sunroof catalog</x:v>
+      </x:c>
+      <x:c r="I531" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-x7-sunroof.html</x:v>
+      </x:c>
+      <x:c r="J531" s="9" t="str">
+        <x:v>VIN-specific drain/seal/cassette component only after leak test</x:v>
+      </x:c>
+      <x:c r="K531" s="9" t="str">
+        <x:v>OEM roof catalog</x:v>
+      </x:c>
+      <x:c r="L531" s="9" t="str"/>
+      <x:c r="M531" s="9" t="str"/>
+      <x:c r="N531" s="41" t="str"/>
+    </x:row>
+    <x:row r="532" ht="739.2000122070312" hidden="0" customHeight="1">
+      <x:c r="A532" s="40" t="n">
+        <x:v>359</x:v>
+      </x:c>
+      <x:c r="B532" s="9" t="str">
+        <x:v>bmw-x7-tire-wear-2019</x:v>
+      </x:c>
+      <x:c r="C532" s="9" t="str">
+        <x:v>2019-2023 | BMW | X7</x:v>
+      </x:c>
+      <x:c r="D532" s="9" t="str">
+        <x:v>Premature Tire Wear (Especially 21"/22" Wheels)</x:v>
+      </x:c>
+      <x:c r="E532" s="9" t="str">
+        <x:v>Have alignment adjusted to reduce aggressive camber settings ($200-400). Switch to quality tires designed for heavy SUVs: Michelin Pilot Sport 4S or Continental PremiumContact 6 are recommended. If possible, avoid 22" wheels and opt for 21" or smaller for better tire longevity and ride comfort. Alignment adjustment can extend tire life from 15,000 to 30,000+ miles. Total cost $200-2,000 depending on tire replacement needs. Check alignment every 10,000 miles.</x:v>
+      </x:c>
+      <x:c r="F532" s="9" t="str">
+        <x:v>Tire size/load/speed/run-flat/staggered setup and tread pattern; suspension/play and alignment diagnosis; VIN-approved alignment target; exact replacement tires by configuration</x:v>
+      </x:c>
+      <x:c r="G532" s="9" t="str">
+        <x:v>TIRE-CONFIGURATION / ALIGNMENT GATE</x:v>
+      </x:c>
+      <x:c r="H532" s="9" t="str">
+        <x:v>Tire Rack BMW X7 tire selector</x:v>
+      </x:c>
+      <x:c r="I532" s="9" t="str">
+        <x:v>https://www.tirerack.com/tires/SelectTireSize.jsp?autoMake=BMW&amp;autoModel=X7</x:v>
+      </x:c>
+      <x:c r="J532" s="9" t="str">
+        <x:v>select exact year/trim/wheel size/load and axle before tire choice</x:v>
+      </x:c>
+      <x:c r="K532" s="9" t="str">
+        <x:v>vehicle-configured tire catalog</x:v>
+      </x:c>
+      <x:c r="L532" s="9" t="str"/>
+      <x:c r="M532" s="9" t="str">
+        <x:v>The row names tires without proving every X7 size/load/staggered application and suggests reducing camber outside specification.</x:v>
+      </x:c>
+      <x:c r="N532" s="41" t="str">
+        <x:v>Use VIN-approved alignment tolerances and exact load/speed rating; do not promise doubled tire life.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="533" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A533" s="40" t="str"/>
+      <x:c r="B533" s="9" t="str"/>
+      <x:c r="C533" s="9" t="str"/>
+      <x:c r="D533" s="9" t="str"/>
+      <x:c r="E533" s="9" t="str"/>
+      <x:c r="F533" s="9" t="str"/>
+      <x:c r="G533" s="9" t="str"/>
+      <x:c r="H533" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I533" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J533" s="9" t="str">
+        <x:v>suspension inspection and four-wheel alignment</x:v>
+      </x:c>
+      <x:c r="K533" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L533" s="9" t="str"/>
+      <x:c r="M533" s="9" t="str"/>
+      <x:c r="N533" s="41" t="str"/>
+    </x:row>
+    <x:row r="534" ht="501.6000061035156" hidden="0" customHeight="1">
+      <x:c r="A534" s="40" t="n">
+        <x:v>360</x:v>
+      </x:c>
+      <x:c r="B534" s="9" t="str">
+        <x:v>bmw-xm-airbag-passenger-knee-recall-2023</x:v>
+      </x:c>
+      <x:c r="C534" s="9" t="str">
+        <x:v>2023-2023 | BMW | XM</x:v>
+      </x:c>
+      <x:c r="D534" s="9" t="str">
+        <x:v>2023 XM Front-Passenger Knee-Airbag Recall 23V-622</x:v>
+      </x:c>
+      <x:c r="E534" s="9" t="str">
+        <x:v>Check the VIN for an open 23V-622 campaign. If open, an authorized BMW dealer replaces the front-passenger knee airbag free of charge. Do not attempt airbag diagnosis or order a clock spring or airbag module from this card; supplemental-restraint work requires trained personnel and VIN-selected parts.</x:v>
+      </x:c>
+      <x:c r="F534" s="9" t="str">
+        <x:v>VIN recall 23V-622 check; free authorized passenger knee-airbag replacement; no DIY restraint-system work</x:v>
+      </x:c>
+      <x:c r="G534" s="9" t="str">
+        <x:v>RECALL ROUTES ONLY</x:v>
+      </x:c>
+      <x:c r="H534" s="9" t="str">
+        <x:v>BMW recall lookup</x:v>
+      </x:c>
+      <x:c r="I534" s="9" t="str">
+        <x:v>https://www.bmwusa.com/safety-and-emission-recalls.html</x:v>
+      </x:c>
+      <x:c r="J534" s="9" t="str">
+        <x:v>VIN check for 23V-622</x:v>
+      </x:c>
+      <x:c r="K534" s="9" t="str">
+        <x:v>manufacturer recall remedy</x:v>
+      </x:c>
+      <x:c r="L534" s="9" t="str"/>
+      <x:c r="M534" s="9" t="str">
+        <x:v>Airbag work requires VIN-selected campaign parts and trained personnel.</x:v>
+      </x:c>
+      <x:c r="N534" s="41" t="str">
+        <x:v>Do not link a clock spring, module, or airbag product.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="535" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A535" s="40" t="str"/>
+      <x:c r="B535" s="9" t="str"/>
+      <x:c r="C535" s="9" t="str"/>
+      <x:c r="D535" s="9" t="str"/>
+      <x:c r="E535" s="9" t="str"/>
+      <x:c r="F535" s="9" t="str"/>
+      <x:c r="G535" s="9" t="str"/>
+      <x:c r="H535" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I535" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J535" s="9" t="str">
+        <x:v>independent VIN recall-status check</x:v>
+      </x:c>
+      <x:c r="K535" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L535" s="9" t="str"/>
+      <x:c r="M535" s="9" t="str"/>
+      <x:c r="N535" s="41" t="str"/>
+    </x:row>
+    <x:row r="536" ht="567.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A536" s="40" t="n">
+        <x:v>361</x:v>
+      </x:c>
+      <x:c r="B536" s="9" t="str">
+        <x:v>bmw-xm-hybrid-drivetrain-hesitation-2023</x:v>
+      </x:c>
+      <x:c r="C536" s="9" t="str">
+        <x:v>2023-2024 | BMW | XM | S68 4.4L Twin-Turbo V8 Hybrid, S68</x:v>
+      </x:c>
+      <x:c r="D536" s="9" t="str">
+        <x:v>Hybrid Drivetrain Hesitation and Power Delivery Lag</x:v>
+      </x:c>
+      <x:c r="E536" s="9" t="str">
+        <x:v>Visit the dealer for the latest transmission and hybrid system software calibration updates. Select Sport or Sport Plus mode for more consistent power delivery. The latest software revisions significantly improve the electric-to-V8 handoff smoothness. If hesitation persists after updates, the dealer can reset the transmission adaptation values to relearn driving patterns.</x:v>
+      </x:c>
+      <x:c r="F536" s="9" t="str">
+        <x:v>Fault memory and current integration/software level; official transmission/hybrid update; adaptation reset only per test plan; mechanical/high-voltage diagnosis if persistent</x:v>
+      </x:c>
+      <x:c r="G536" s="9" t="str">
+        <x:v>HYBRID SOFTWARE / DEALER SERVICE ROUTE</x:v>
+      </x:c>
+      <x:c r="H536" s="9" t="str">
+        <x:v>BMW dealer locator</x:v>
+      </x:c>
+      <x:c r="I536" s="9" t="str">
+        <x:v>https://www.bmwusa.com/dealer-locator.html</x:v>
+      </x:c>
+      <x:c r="J536" s="9" t="str">
+        <x:v>2023-2024 XM hybrid drivetrain software and high-voltage diagnosis</x:v>
+      </x:c>
+      <x:c r="K536" s="9" t="str">
+        <x:v>authorized hybrid service</x:v>
+      </x:c>
+      <x:c r="L536" s="9" t="str"/>
+      <x:c r="M536" s="9" t="str">
+        <x:v>This is software/high-voltage diagnosis, not a retail part; drive mode is a preference, not a repair.</x:v>
+      </x:c>
+      <x:c r="N536" s="41" t="str">
+        <x:v>Do not promise an update or adaptation reset will fix every hesitation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="537" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A537" s="40" t="str"/>
+      <x:c r="B537" s="9" t="str"/>
+      <x:c r="C537" s="9" t="str"/>
+      <x:c r="D537" s="9" t="str"/>
+      <x:c r="E537" s="9" t="str"/>
+      <x:c r="F537" s="9" t="str"/>
+      <x:c r="G537" s="9" t="str"/>
+      <x:c r="H537" s="9" t="str">
+        <x:v>BMW Remote Software Upgrade</x:v>
+      </x:c>
+      <x:c r="I537" s="9" t="str">
+        <x:v>https://www.bmwusa.com/explore/connecteddrive/remote-software-upgrade.html</x:v>
+      </x:c>
+      <x:c r="J537" s="9" t="str">
+        <x:v>only when an official update is offered to the VIN</x:v>
+      </x:c>
+      <x:c r="K537" s="9" t="str">
+        <x:v>official update information</x:v>
+      </x:c>
+      <x:c r="L537" s="9" t="str"/>
+      <x:c r="M537" s="9" t="str"/>
+      <x:c r="N537" s="41" t="str"/>
+    </x:row>
+    <x:row r="538" ht="646.7999877929688" hidden="0" customHeight="1">
+      <x:c r="A538" s="40" t="n">
+        <x:v>362</x:v>
+      </x:c>
+      <x:c r="B538" s="9" t="str">
+        <x:v>bmw-xm-integrated-brake-system-recall-2023</x:v>
+      </x:c>
+      <x:c r="C538" s="9" t="str">
+        <x:v>2023-2024 | BMW | XM</x:v>
+      </x:c>
+      <x:c r="D538" s="9" t="str">
+        <x:v>2023-2024 XM Integrated Brake System Recall 26V-422</x:v>
+      </x:c>
+      <x:c r="E538" s="9" t="str">
+        <x:v>Check the VIN at NHTSA and with an authorized BMW dealer when campaign 26V-422 VINs become searchable, and arrange the free dealer inspection and module replacement if required. If a brake warning appears or pedal effort increases, avoid abrupt braking, allow extra stopping distance, stop safely and contact BMW roadside assistance; wheel-speed sensors are not the recall remedy.</x:v>
+      </x:c>
+      <x:c r="F538" s="9" t="str">
+        <x:v>VIN recall 26V-422 check; free dealer inspection/module replacement if required; safety response for warning/increased pedal effort</x:v>
+      </x:c>
+      <x:c r="G538" s="9" t="str">
+        <x:v>RECALL ROUTES ONLY</x:v>
+      </x:c>
+      <x:c r="H538" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I538" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J538" s="9" t="str">
+        <x:v>VIN check for 26V-422</x:v>
+      </x:c>
+      <x:c r="K538" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L538" s="9" t="str"/>
+      <x:c r="M538" s="9" t="str">
+        <x:v>Wheel-speed sensors are not the stated recall remedy and retail electronics are inappropriate.</x:v>
+      </x:c>
+      <x:c r="N538" s="41" t="str">
+        <x:v>Keep VIN and brake-warning safety instructions primary.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="539" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A539" s="40" t="str"/>
+      <x:c r="B539" s="9" t="str"/>
+      <x:c r="C539" s="9" t="str"/>
+      <x:c r="D539" s="9" t="str"/>
+      <x:c r="E539" s="9" t="str"/>
+      <x:c r="F539" s="9" t="str"/>
+      <x:c r="G539" s="9" t="str"/>
+      <x:c r="H539" s="9" t="str">
+        <x:v>BMW recall lookup</x:v>
+      </x:c>
+      <x:c r="I539" s="9" t="str">
+        <x:v>https://www.bmwusa.com/safety-and-emission-recalls.html</x:v>
+      </x:c>
+      <x:c r="J539" s="9" t="str">
+        <x:v>manufacturer VIN/campaign status</x:v>
+      </x:c>
+      <x:c r="K539" s="9" t="str">
+        <x:v>manufacturer recall remedy</x:v>
+      </x:c>
+      <x:c r="L539" s="9" t="str"/>
+      <x:c r="M539" s="9" t="str"/>
+      <x:c r="N539" s="41" t="str"/>
+    </x:row>
+    <x:row r="540" ht="646.7999877929688" hidden="0" customHeight="1">
+      <x:c r="A540" s="40" t="n">
+        <x:v>363</x:v>
+      </x:c>
+      <x:c r="B540" s="9" t="str">
+        <x:v>bmw-xm-suspension-ride-quality-2023</x:v>
+      </x:c>
+      <x:c r="C540" s="9" t="str">
+        <x:v>2023-2024 | BMW | XM | S68 4.4L Twin-Turbo V8 Hybrid</x:v>
+      </x:c>
+      <x:c r="D540" s="9" t="str">
+        <x:v>Harsh Ride Quality and Suspension Stiffness</x:v>
+      </x:c>
+      <x:c r="E540" s="9" t="str">
+        <x:v>Check tire pressures regularly - overinflated tires significantly worsen the harsh ride. Some owners report improved comfort by switching to a tire with a taller sidewall profile (if available for the XM's wheel size). Use Comfort mode for daily driving. Unfortunately, no aftermarket spring or damper solution currently exists to significantly improve the ride without compromising the handling needed for the XM's weight.</x:v>
+      </x:c>
+      <x:c r="F540" s="9" t="str">
+        <x:v>Cold tire-pressure/load check; verify wheel/tire size and damage; alignment/suspension fault diagnosis; Comfort mode; alternate tire only with exact approved size/load/speed rating</x:v>
+      </x:c>
+      <x:c r="G540" s="9" t="str">
+        <x:v>CONDITION / CONFIGURATION GUIDANCE; NO SUSPENSION PART</x:v>
+      </x:c>
+      <x:c r="H540" s="9" t="str">
+        <x:v>BMW dealer locator</x:v>
+      </x:c>
+      <x:c r="I540" s="9" t="str">
+        <x:v>https://www.bmwusa.com/dealer-locator.html</x:v>
+      </x:c>
+      <x:c r="J540" s="9" t="str">
+        <x:v>2023-2024 XM suspension fault, software, alignment, and approved tire configuration</x:v>
+      </x:c>
+      <x:c r="K540" s="9" t="str">
+        <x:v>manufacturer-capable service</x:v>
+      </x:c>
+      <x:c r="L540" s="9" t="str"/>
+      <x:c r="M540" s="9" t="str">
+        <x:v>Harshness may be normal tuning, pressure, tire, alignment, or a fault; no universal spring/damper product was identified.</x:v>
+      </x:c>
+      <x:c r="N540" s="41" t="str">
+        <x:v>Do not alter tire diameter/load rating or claim no aftermarket solution exists indefinitely.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="541" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A541" s="40" t="str"/>
+      <x:c r="B541" s="9" t="str"/>
+      <x:c r="C541" s="9" t="str"/>
+      <x:c r="D541" s="9" t="str"/>
+      <x:c r="E541" s="9" t="str"/>
+      <x:c r="F541" s="9" t="str"/>
+      <x:c r="G541" s="9" t="str"/>
+      <x:c r="H541" s="9" t="str">
+        <x:v>Tire Rack BMW XM tire selector</x:v>
+      </x:c>
+      <x:c r="I541" s="9" t="str">
+        <x:v>https://www.tirerack.com/tires/SelectTireSize.jsp?autoMake=BMW&amp;autoModel=XM</x:v>
+      </x:c>
+      <x:c r="J541" s="9" t="str">
+        <x:v>exact year/wheel/load configuration only</x:v>
+      </x:c>
+      <x:c r="K541" s="9" t="str">
+        <x:v>configured tire catalog</x:v>
+      </x:c>
+      <x:c r="L541" s="9" t="str"/>
+      <x:c r="M541" s="9" t="str"/>
+      <x:c r="N541" s="41" t="str"/>
+    </x:row>
+    <x:row r="542" ht="528" hidden="0" customHeight="1">
+      <x:c r="A542" s="40" t="n">
+        <x:v>364</x:v>
+      </x:c>
+      <x:c r="B542" s="9" t="str">
+        <x:v>bmw-z3-convertible-top-rear-window-cracking-clouding-bead-separatio</x:v>
+      </x:c>
+      <x:c r="C542" s="9" t="str">
+        <x:v>1996-2002 | BMW | Z3</x:v>
+      </x:c>
+      <x:c r="D542" s="9" t="str">
+        <x:v>Convertible Top Rear Window Cracking, Clouding, and Bead Separation</x:v>
+      </x:c>
+      <x:c r="E542" s="9" t="str">
+        <x:v>Replace the rear window panel only — BMW used a zipper system so the clouded/cracked window unzips and a new window zips/tapes in without disturbing the fabric top. Re-gluing separated bead trim rarely holds, so window replacement is the durable fix. Job is a DIY-feasible 1-1.5 hours; replace the whole top only if the fabric is also degraded.</x:v>
+      </x:c>
+      <x:c r="F542" s="9" t="str">
+        <x:v>Confirm zipper-style original/replacement top; exact rear-window panel and zipper/seal kit; fabric/top replacement only if fabric/zipper/cassette condition requires</x:v>
+      </x:c>
+      <x:c r="G542" s="9" t="str">
+        <x:v>TOP / ZIPPER CONFIGURATION GATE</x:v>
+      </x:c>
+      <x:c r="H542" s="9" t="str">
+        <x:v>Genuine BMW Z3 convertible-top catalog</x:v>
+      </x:c>
+      <x:c r="I542" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-z3-convertible_top.html</x:v>
+      </x:c>
+      <x:c r="J542" s="9" t="str">
+        <x:v>1996-2002 Z3; VIN and installed top/window configuration required</x:v>
+      </x:c>
+      <x:c r="K542" s="9" t="str">
+        <x:v>OEM roof/window catalog</x:v>
+      </x:c>
+      <x:c r="L542" s="9" t="str"/>
+      <x:c r="M542" s="9" t="str">
+        <x:v>A zipper replacement is viable only if the installed top/zipper is compatible and sound.</x:v>
+      </x:c>
+      <x:c r="N542" s="41" t="str">
+        <x:v>Do not promise a 1-1.5-hour DIY or panel-only repair for aftermarket tops or damaged zipper tracks.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="543" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A543" s="40" t="str"/>
+      <x:c r="B543" s="9" t="str"/>
+      <x:c r="C543" s="9" t="str"/>
+      <x:c r="D543" s="9" t="str"/>
+      <x:c r="E543" s="9" t="str"/>
+      <x:c r="F543" s="9" t="str"/>
+      <x:c r="G543" s="9" t="str"/>
+      <x:c r="H543" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I543" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J543" s="9" t="str">
+        <x:v>top/window condition and installation assessment</x:v>
+      </x:c>
+      <x:c r="K543" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L543" s="9" t="str"/>
+      <x:c r="M543" s="9" t="str"/>
+      <x:c r="N543" s="41" t="str"/>
+    </x:row>
+    <x:row r="544" ht="158.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A544" s="40" t="n">
+        <x:v>365</x:v>
+      </x:c>
+      <x:c r="B544" s="9" t="str">
+        <x:v>bmw-z3-cooling-system-failure-1996</x:v>
+      </x:c>
+      <x:c r="C544" s="9" t="str">
+        <x:v>1996-2002 | BMW | Z3</x:v>
+      </x:c>
+      <x:c r="D544" s="9" t="str">
+        <x:v>Cooling System Component Failures</x:v>
+      </x:c>
+      <x:c r="E544" s="9" t="str"/>
+      <x:c r="F544" s="9" t="str"/>
+      <x:c r="G544" s="9" t="str">
+        <x:v>SOURCE HOW-TO-FIX REQUIRED / NO LINK</x:v>
+      </x:c>
+      <x:c r="H544" s="9" t="str"/>
+      <x:c r="I544" s="9" t="str"/>
+      <x:c r="J544" s="9" t="str"/>
+      <x:c r="K544" s="9" t="str"/>
+      <x:c r="L544" s="9" t="str"/>
+      <x:c r="M544" s="9" t="str">
+        <x:v>The source has no How to Fix instructions, so there is no repair item to map responsibly.</x:v>
+      </x:c>
+      <x:c r="N544" s="41" t="str">
+        <x:v>Write and approve an engine-specific diagnostic/repair procedure before commerce research.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="545" ht="448.79998779296875" hidden="0" customHeight="1">
+      <x:c r="A545" s="40" t="n">
+        <x:v>366</x:v>
+      </x:c>
+      <x:c r="B545" s="9" t="str">
+        <x:v>bmw-z3-cracked-exhaust-manifold-1-9l-4-cylinder</x:v>
+      </x:c>
+      <x:c r="C545" s="9" t="str">
+        <x:v>1996-2002 | BMW | Z3 | 1.9, 1.9i, Z3 1.9 | 1.9L M44 4-cylinder, 1.9L M43TU 4-cylinder</x:v>
+      </x:c>
+      <x:c r="D545" s="9" t="str">
+        <x:v>Cracked Exhaust Manifold on 1.9L 4-Cylinder (M44/M43)</x:v>
+      </x:c>
+      <x:c r="E545" s="9" t="str">
+        <x:v>Inspect the manifold for hairline cracks (a cold-engine listen or smoke test confirms the leak). Replace the cracked manifold with a used OE unit or an aftermarket stainless tubular header, and renew the manifold gasket and hardware. Allow roughly 3-4 hours labor.</x:v>
+      </x:c>
+      <x:c r="F545" s="9" t="str">
+        <x:v>Confirm M44 versus non-US M43 and crack location; smoke/cold test; exact manifold/header with emissions legality; gasket and one-time hardware</x:v>
+      </x:c>
+      <x:c r="G545" s="9" t="str">
+        <x:v>ENGINE / MARKET / EMISSIONS GATE</x:v>
+      </x:c>
+      <x:c r="H545" s="9" t="str">
+        <x:v>Genuine BMW Z3 exhaust-manifold catalog</x:v>
+      </x:c>
+      <x:c r="I545" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-z3-exhaust_manifold.html</x:v>
+      </x:c>
+      <x:c r="J545" s="9" t="str">
+        <x:v>1996-1999 US Z3 1.9L M44 where VIN-matched; M43 is non-US/different</x:v>
+      </x:c>
+      <x:c r="K545" s="9" t="str">
+        <x:v>OEM manifold catalog</x:v>
+      </x:c>
+      <x:c r="L545" s="9" t="str"/>
+      <x:c r="M545" s="9" t="str">
+        <x:v>M44/M43 markets and emissions equipment differ, and a used manifold or tubular header needs exact fitment/legal review.</x:v>
+      </x:c>
+      <x:c r="N545" s="41" t="str">
+        <x:v>Narrow US fitment to M44 years and do not approve a header without catalyst/emissions compatibility.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="546" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A546" s="40" t="str"/>
+      <x:c r="B546" s="9" t="str"/>
+      <x:c r="C546" s="9" t="str"/>
+      <x:c r="D546" s="9" t="str"/>
+      <x:c r="E546" s="9" t="str"/>
+      <x:c r="F546" s="9" t="str"/>
+      <x:c r="G546" s="9" t="str"/>
+      <x:c r="H546" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I546" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J546" s="9" t="str">
+        <x:v>crack diagnosis and emissions-compliant repair</x:v>
+      </x:c>
+      <x:c r="K546" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L546" s="9" t="str"/>
+      <x:c r="M546" s="9" t="str"/>
+      <x:c r="N546" s="41" t="str"/>
+    </x:row>
+    <x:row r="547" ht="686.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A547" s="40" t="n">
+        <x:v>367</x:v>
+      </x:c>
+      <x:c r="B547" s="9" t="str">
+        <x:v>bmw-z3-differential-mount-ear-trunk-floor-pan-tearing</x:v>
+      </x:c>
+      <x:c r="C547" s="9" t="str">
+        <x:v>1996-2002 | BMW | Z3</x:v>
+      </x:c>
+      <x:c r="D547" s="9" t="str">
+        <x:v>Differential Mount Ear and Trunk Floor Pan Tearing</x:v>
+      </x:c>
+      <x:c r="E547" s="9" t="str">
+        <x:v>Inspect the trunk floor around the differential mount and rear subframe pickup points for cracks, torn metal, and broken spot welds. Repair requires welding and a reinforcement/re-fabrication plate kit to tie the diff mount/subframe back into the floor. Switching the diff carrier bushings to polyurethane reduces carrier movement and the stress that causes the tearing. Catching it early greatly limits the repair scope.</x:v>
+      </x:c>
+      <x:c r="F547" s="9" t="str">
+        <x:v>Full top/bottom structural inspection; crack/spot-weld assessment; chassis-specialist weld/reinforcement design; subframe/diff bushings only as part of engineered repair; alignment</x:v>
+      </x:c>
+      <x:c r="G547" s="9" t="str">
+        <x:v>STRUCTURAL SPECIALIST ROUTE; KIT HELD</x:v>
+      </x:c>
+      <x:c r="H547" s="9" t="str">
+        <x:v>Randy Forbes Z3 reinforcement information</x:v>
+      </x:c>
+      <x:c r="I547" s="9" t="str">
+        <x:v>https://www.spcarsplus.com/</x:v>
+      </x:c>
+      <x:c r="J547" s="9" t="str">
+        <x:v>Z3 structural reinforcement reference; confirm current kit/service availability and exact chassis</x:v>
+      </x:c>
+      <x:c r="K547" s="9" t="str">
+        <x:v>specialist reinforcement source</x:v>
+      </x:c>
+      <x:c r="L547" s="9" t="str"/>
+      <x:c r="M547" s="9" t="str">
+        <x:v>Repair scope depends on structural damage; polyurethane alone does not repair or necessarily reduce every stress mode.</x:v>
+      </x:c>
+      <x:c r="N547" s="41" t="str">
+        <x:v>Do not install bushings as a substitute for welding/reinforcement or approve a plate kit without current exact contents.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="548" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A548" s="40" t="str"/>
+      <x:c r="B548" s="9" t="str"/>
+      <x:c r="C548" s="9" t="str"/>
+      <x:c r="D548" s="9" t="str"/>
+      <x:c r="E548" s="9" t="str"/>
+      <x:c r="F548" s="9" t="str"/>
+      <x:c r="G548" s="9" t="str"/>
+      <x:c r="H548" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I548" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J548" s="9" t="str">
+        <x:v>Z3 chassis/body structural inspection and welding referral</x:v>
+      </x:c>
+      <x:c r="K548" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L548" s="9" t="str"/>
+      <x:c r="M548" s="9" t="str"/>
+      <x:c r="N548" s="41" t="str"/>
+    </x:row>
+    <x:row r="549" ht="514.7999877929688" hidden="0" customHeight="1">
+      <x:c r="A549" s="40" t="n">
+        <x:v>368</x:v>
+      </x:c>
+      <x:c r="B549" s="9" t="str">
+        <x:v>bmw-z3-door-window-regulator-clip-mounting-tab-failure</x:v>
+      </x:c>
+      <x:c r="C549" s="9" t="str">
+        <x:v>1996-2002 | BMW | Z3</x:v>
+      </x:c>
+      <x:c r="D549" s="9" t="str">
+        <x:v>Door Window Regulator Clip / Mounting Tab Failure</x:v>
+      </x:c>
+      <x:c r="E549" s="9" t="str">
+        <x:v>Replace the broken plastic regulator clips, or replace the regulator assembly if the cable or mechanism is also worn. If the welded mounting tab/anchor has torn from the door frame, it must be re-welded or reinforced before fitting a new regulator. Lubricate the window channels to reduce drag on the new parts.</x:v>
+      </x:c>
+      <x:c r="F549" s="9" t="str">
+        <x:v>Door/side diagnosis; exact plastic clips if mechanism healthy; side-specific regulator if cable/mechanism worn; weld/reinforce torn door anchor; channel lubrication</x:v>
+      </x:c>
+      <x:c r="G549" s="9" t="str">
+        <x:v>SIDE / FAILURE-BRANCH CATALOG</x:v>
+      </x:c>
+      <x:c r="H549" s="9" t="str">
+        <x:v>BMW Z3 window-regulator catalog</x:v>
+      </x:c>
+      <x:c r="I549" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/Z3/Window-Regulator/</x:v>
+      </x:c>
+      <x:c r="J549" s="9" t="str">
+        <x:v>1996-2002 Z3; select left/right and clip-versus-regulator branch</x:v>
+      </x:c>
+      <x:c r="K549" s="9" t="str">
+        <x:v>vehicle-specific regulator catalog</x:v>
+      </x:c>
+      <x:c r="L549" s="9" t="str"/>
+      <x:c r="M549" s="9" t="str">
+        <x:v>Clips, regulator, and torn door anchor are three different repairs.</x:v>
+      </x:c>
+      <x:c r="N549" s="41" t="str">
+        <x:v>Do not sell a regulator when only a clip failed or fit new parts to an unrepaired torn anchor.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="550" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A550" s="40" t="str"/>
+      <x:c r="B550" s="9" t="str"/>
+      <x:c r="C550" s="9" t="str"/>
+      <x:c r="D550" s="9" t="str"/>
+      <x:c r="E550" s="9" t="str"/>
+      <x:c r="F550" s="9" t="str"/>
+      <x:c r="G550" s="9" t="str"/>
+      <x:c r="H550" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I550" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J550" s="9" t="str">
+        <x:v>torn mounting-tab welding and window adjustment</x:v>
+      </x:c>
+      <x:c r="K550" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L550" s="9" t="str"/>
+      <x:c r="M550" s="9" t="str"/>
+      <x:c r="N550" s="41" t="str"/>
+    </x:row>
+    <x:row r="551" ht="686.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A551" s="40" t="n">
+        <x:v>369</x:v>
+      </x:c>
+      <x:c r="B551" s="9" t="str">
+        <x:v>bmw-z3-fuel-level-sender-failure-causing-erratic-dead-fuel-gauge</x:v>
+      </x:c>
+      <x:c r="C551" s="9" t="str">
+        <x:v>1996-2002 | BMW | Z3</x:v>
+      </x:c>
+      <x:c r="D551" s="9" t="str">
+        <x:v>Fuel Level Sender Failure Causing Erratic or Dead Fuel Gauge</x:v>
+      </x:c>
+      <x:c r="E551" s="9" t="str">
+        <x:v>Remove the access panel behind the seats and inspect the sender. A dirty or lightly worn ceramic/resistor plate can sometimes be cleaned, but a cracked plate or worn brushes requires replacing the sender unit (or the complete fuel-pump/sender carrier assembly). Also check the tank vent valve, as tank vacuum can deform the float arm. Confirm wiring/ground integrity before condemning the sender.</x:v>
+      </x:c>
+      <x:c r="F551" s="9" t="str">
+        <x:v>Wiring/ground and tank-vent diagnosis; sender plate/brush inspection; clean only if serviceable; VIN/tank-side-specific sender or complete carrier if required</x:v>
+      </x:c>
+      <x:c r="G551" s="9" t="str">
+        <x:v>DIAGNOSIS / TANK-CONFIGURATION GATE</x:v>
+      </x:c>
+      <x:c r="H551" s="9" t="str">
+        <x:v>BMW Z3 fuel-sender catalog</x:v>
+      </x:c>
+      <x:c r="I551" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-z3-fuel_level_sensor.html</x:v>
+      </x:c>
+      <x:c r="J551" s="9" t="str">
+        <x:v>1996-2002 Z3; VIN, tank configuration, and sender/carrier branch required</x:v>
+      </x:c>
+      <x:c r="K551" s="9" t="str">
+        <x:v>OEM sender catalog</x:v>
+      </x:c>
+      <x:c r="L551" s="9" t="str"/>
+      <x:c r="M551" s="9" t="str">
+        <x:v>Gauge faults can be electrical, sender wear, carrier, or tank-vacuum deformation.</x:v>
+      </x:c>
+      <x:c r="N551" s="41" t="str">
+        <x:v>Do not condemn the sender before wiring/ground/vent checks or clean a cracked/worn resistor plate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="552" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A552" s="40" t="str"/>
+      <x:c r="B552" s="9" t="str"/>
+      <x:c r="C552" s="9" t="str"/>
+      <x:c r="D552" s="9" t="str"/>
+      <x:c r="E552" s="9" t="str"/>
+      <x:c r="F552" s="9" t="str"/>
+      <x:c r="G552" s="9" t="str"/>
+      <x:c r="H552" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I552" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J552" s="9" t="str">
+        <x:v>fuel-level circuit and tank-vent diagnosis</x:v>
+      </x:c>
+      <x:c r="K552" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L552" s="9" t="str"/>
+      <x:c r="M552" s="9" t="str"/>
+      <x:c r="N552" s="41" t="str"/>
+    </x:row>
+    <x:row r="553" ht="488.3999938964844" hidden="0" customHeight="1">
+      <x:c r="A553" s="40" t="n">
+        <x:v>370</x:v>
+      </x:c>
+      <x:c r="B553" s="9" t="str">
+        <x:v>bmw-z3-hvac-blower-final-stage-resistor-failure</x:v>
+      </x:c>
+      <x:c r="C553" s="9" t="str">
+        <x:v>1996-2002 | BMW | Z3</x:v>
+      </x:c>
+      <x:c r="D553" s="9" t="str">
+        <x:v>HVAC Blower Final Stage Resistor Failure (Fan Only Works on Max)</x:v>
+      </x:c>
+      <x:c r="E553" s="9" t="str">
+        <x:v>Replace the blower final stage resistor (A/C cars: part under the scuttle/cowl; non-A/C cars: behind the passenger footwell panel). If a new resistor does not restore all speeds, test the blower motor itself, which may also be worn. Inspect for corrosion/water intrusion at the cowl on A/C cars.</x:v>
+      </x:c>
+      <x:c r="F553" s="9" t="str">
+        <x:v>A/C versus non-A/C configuration; blower-speed/resistor circuit diagnosis; exact resistor; blower motor and water/cowl inspection if unresolved</x:v>
+      </x:c>
+      <x:c r="G553" s="9" t="str">
+        <x:v>HVAC-CONFIGURATION GATE</x:v>
+      </x:c>
+      <x:c r="H553" s="9" t="str">
+        <x:v>BMW Z3 blower-resistor catalog</x:v>
+      </x:c>
+      <x:c r="I553" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/Z3/Blower-Motor-Resistor/</x:v>
+      </x:c>
+      <x:c r="J553" s="9" t="str">
+        <x:v>1996-2002 Z3; confirm A/C equipment, VIN, and resistor location/part</x:v>
+      </x:c>
+      <x:c r="K553" s="9" t="str">
+        <x:v>vehicle-specific resistor catalog</x:v>
+      </x:c>
+      <x:c r="L553" s="9" t="str"/>
+      <x:c r="M553" s="9" t="str">
+        <x:v>The source identifies different locations/configurations and a blower-motor fallback.</x:v>
+      </x:c>
+      <x:c r="N553" s="41" t="str">
+        <x:v>Do not assume max-only operation proves the resistor without circuit testing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="554" ht="66" hidden="0" customHeight="1">
+      <x:c r="A554" s="40" t="str"/>
+      <x:c r="B554" s="9" t="str"/>
+      <x:c r="C554" s="9" t="str"/>
+      <x:c r="D554" s="9" t="str"/>
+      <x:c r="E554" s="9" t="str"/>
+      <x:c r="F554" s="9" t="str"/>
+      <x:c r="G554" s="9" t="str"/>
+      <x:c r="H554" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I554" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J554" s="9" t="str">
+        <x:v>blower circuit/water-intrusion diagnosis</x:v>
+      </x:c>
+      <x:c r="K554" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L554" s="9" t="str"/>
+      <x:c r="M554" s="9" t="str"/>
+      <x:c r="N554" s="41" t="str"/>
+    </x:row>
+    <x:row r="555" ht="1584" hidden="0" customHeight="1">
+      <x:c r="A555" s="40" t="n">
+        <x:v>371</x:v>
+      </x:c>
+      <x:c r="B555" s="9" t="str">
+        <x:v>bmw-z3-rear-subframe-crack-1996</x:v>
+      </x:c>
+      <x:c r="C555" s="9" t="str">
+        <x:v>1996-2002 | BMW | Z3</x:v>
+      </x:c>
+      <x:c r="D555" s="9" t="str">
+        <x:v>Rear Subframe Mounting Point Cracking</x:v>
+      </x:c>
+      <x:c r="E555" s="9" t="str">
+        <x:v>Inspect the trunk floor, differential mount area, and all rear subframe mounting points from above and below the car for spot-weld separation, torn sheet metal, and cracked seams; a dye penetrant test or removing trunk trim/seam sealer may be needed to reveal early damage. If cracking is present, the proper repair is to drop the rear axle carrier/subframe, weld and reinforce the damaged unibody mounting points and trunk floor with a reinforcement kit (commonly Randy Forbes-style dual-ear/differential mount reinforcement or equivalent), then reinstall with new subframe bushings, differential mount bushings, and perform a 4-wheel alignment. Minor early cracks may be repairable before major deformation, but advanced damage often requires fabrication and extensive welding by a chassis/body specialist; typical cost ranges from about $2,000-$3,500 for early reinforcement repairs and can exceed $4,000-$6,000 if the floor is torn or multiple mounting points are damaged.</x:v>
+      </x:c>
+      <x:c r="F555" s="9" t="str">
+        <x:v>Top/bottom structural inspection including hidden seams; chassis-specialist fabrication/welding; exact reinforcement strategy; bushings/fasteners by condition; alignment</x:v>
+      </x:c>
+      <x:c r="G555" s="9" t="str">
+        <x:v>STRUCTURAL SPECIALIST ROUTE</x:v>
+      </x:c>
+      <x:c r="H555" s="9" t="str">
+        <x:v>Randy Forbes Z3 reinforcement information</x:v>
+      </x:c>
+      <x:c r="I555" s="9" t="str">
+        <x:v>https://www.spcarsplus.com/</x:v>
+      </x:c>
+      <x:c r="J555" s="9" t="str">
+        <x:v>Z3 dual-ear/trunk-floor reinforcement reference; verify current kit/service and exact damage</x:v>
+      </x:c>
+      <x:c r="K555" s="9" t="str">
+        <x:v>specialist reinforcement source</x:v>
+      </x:c>
+      <x:c r="L555" s="9" t="str"/>
+      <x:c r="M555" s="9" t="str">
+        <x:v>Advanced unibody damage requires individualized fabrication; a catalog kit alone is not the repair.</x:v>
+      </x:c>
+      <x:c r="N555" s="41" t="str">
+        <x:v>Consolidate with the differential-mount/trunk-floor duplicate and avoid fixed cost promises.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="556" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A556" s="40" t="str"/>
+      <x:c r="B556" s="9" t="str"/>
+      <x:c r="C556" s="9" t="str"/>
+      <x:c r="D556" s="9" t="str"/>
+      <x:c r="E556" s="9" t="str"/>
+      <x:c r="F556" s="9" t="str"/>
+      <x:c r="G556" s="9" t="str"/>
+      <x:c r="H556" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I556" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J556" s="9" t="str">
+        <x:v>structural inspection and qualified body/chassis referral</x:v>
+      </x:c>
+      <x:c r="K556" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L556" s="9" t="str"/>
+      <x:c r="M556" s="9" t="str"/>
+      <x:c r="N556" s="41" t="str"/>
+    </x:row>
+    <x:row r="557" ht="198" hidden="0" customHeight="1">
+      <x:c r="A557" s="40" t="n">
+        <x:v>372</x:v>
+      </x:c>
+      <x:c r="B557" s="9" t="str">
+        <x:v>bmw-z3-rear-subframe-cracking-1996</x:v>
+      </x:c>
+      <x:c r="C557" s="9" t="str">
+        <x:v>1996-2002 | BMW | Z3 | M52, M54</x:v>
+      </x:c>
+      <x:c r="D557" s="9" t="str">
+        <x:v>Rear Subframe Mounting Point Cracks</x:v>
+      </x:c>
+      <x:c r="E557" s="9" t="str"/>
+      <x:c r="F557" s="9" t="str"/>
+      <x:c r="G557" s="9" t="str">
+        <x:v>SOURCE HOW-TO-FIX REQUIRED / NO LINK</x:v>
+      </x:c>
+      <x:c r="H557" s="9" t="str"/>
+      <x:c r="I557" s="9" t="str"/>
+      <x:c r="J557" s="9" t="str"/>
+      <x:c r="K557" s="9" t="str"/>
+      <x:c r="L557" s="9" t="str"/>
+      <x:c r="M557" s="9" t="str">
+        <x:v>This duplicate source row has no How to Fix instructions.</x:v>
+      </x:c>
+      <x:c r="N557" s="41" t="str">
+        <x:v>Merge with the fully described Z3 trunk-floor/subframe issue or add an approved structural repair procedure before links.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="558" ht="475.20001220703125" hidden="0" customHeight="1">
+      <x:c r="A558" s="40" t="n">
+        <x:v>373</x:v>
+      </x:c>
+      <x:c r="B558" s="9" t="str">
+        <x:v>bmw-z3-valve-cover-gasket-oil-leak</x:v>
+      </x:c>
+      <x:c r="C558" s="9" t="str">
+        <x:v>1997-2002 | BMW | Z3 | 2.3, 2.5i, 2.8, 3.0i | M52 2.8, M52TU 2.5/2.8, M54 2.5/3.0</x:v>
+      </x:c>
+      <x:c r="D558" s="9" t="str">
+        <x:v>Valve Cover Gasket Oil Leak (M52/M54 6-Cylinder)</x:v>
+      </x:c>
+      <x:c r="E558" s="9" t="str">
+        <x:v>Replace the valve cover gasket, the spark-plug-well/grommet seals, and the cover bolt seals. On M54 engines also clean oil from the plug wells and replace any oil-contaminated coil boots/coils. Use the correct torque sequence to avoid re-leaking. Inspect the cover for warping or cracks while it is off.</x:v>
+      </x:c>
+      <x:c r="F558" s="9" t="str">
+        <x:v>Confirm M52/S52/M52TU/M54 and leak source; engine-specific cover gasket, plug-well seals/grommets/bolt seals; cover inspection; oil-damaged boots/coils by condition; torque procedure</x:v>
+      </x:c>
+      <x:c r="G558" s="9" t="str">
+        <x:v>ENGINE / COVER-CONFIGURATION GATE</x:v>
+      </x:c>
+      <x:c r="H558" s="9" t="str">
+        <x:v>BMW Z3 valve-cover gasket catalog</x:v>
+      </x:c>
+      <x:c r="I558" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/Z3/Valve-Cover-Gasket/</x:v>
+      </x:c>
+      <x:c r="J558" s="9" t="str">
+        <x:v>1997-2002 six-cylinder Z3; select exact engine/VIN and kit contents</x:v>
+      </x:c>
+      <x:c r="K558" s="9" t="str">
+        <x:v>engine-specific gasket catalog</x:v>
+      </x:c>
+      <x:c r="L558" s="9" t="str"/>
+      <x:c r="M558" s="9" t="str">
+        <x:v>The years include multiple six-cylinder engines and gasket/cover details.</x:v>
+      </x:c>
+      <x:c r="N558" s="41" t="str">
+        <x:v>Do not attach one M54 kit to M52/S52/M52TU; replace boots/coils only if oil-damaged/test-failed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="559" ht="1293.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A559" s="40" t="n">
+        <x:v>374</x:v>
+      </x:c>
+      <x:c r="B559" s="9" t="str">
+        <x:v>bmw-z3-vanos-seals-1999</x:v>
+      </x:c>
+      <x:c r="C559" s="9" t="str">
+        <x:v>1999-2002 | BMW | Z3 | M52, M54, S52</x:v>
+      </x:c>
+      <x:c r="D559" s="9" t="str">
+        <x:v>VANOS Seal Failure (M52/M54/S52)</x:v>
+      </x:c>
+      <x:c r="E559" s="9" t="str">
+        <x:v>Confirm the fault by checking for cold-start VANOS rattle, rough idle, hesitation, and scanning for cam timing or mixture-related fault codes; on M52TU/M54/S52 engines, inspect VANOS operation and rule out vacuum leaks before disassembly. Repair typically involves removing the valve cover and VANOS unit, replacing the internal piston seals/O-rings with updated Viton/Teflon seals, renewing the valve cover gasket and VANOS oil line sealing washers, and then re-timing the cams to BMW specifications if required. If the unit still rattles after resealing, the VANOS bearing/anti-rattle components or the complete VANOS assembly may need replacement. Typical cost is about $60-$150 in seals/gaskets for DIY repair, $300-$700 for an independent shop reseal, or $800-$1,500+ if a rebuilt/replacement VANOS unit is installed.</x:v>
+      </x:c>
+      <x:c r="F559" s="9" t="str">
+        <x:v>Split S52 single VANOS from M52TU/M54 double VANOS; vacuum/oil/timing diagnosis; engine-specific seals/anti-rattle components; gasket/washers by access; timing only when procedure requires</x:v>
+      </x:c>
+      <x:c r="G559" s="9" t="str">
+        <x:v>ENGINE / VANOS-TYPE SPLIT</x:v>
+      </x:c>
+      <x:c r="H559" s="9" t="str">
+        <x:v>Beisan VANOS product catalog</x:v>
+      </x:c>
+      <x:c r="I559" s="9" t="str">
+        <x:v>https://beisansystems.com/shop/</x:v>
+      </x:c>
+      <x:c r="J559" s="9" t="str">
+        <x:v>select M50tu/M52 single or M52tu/M54 double VANOS product by exact Z3 engine</x:v>
+      </x:c>
+      <x:c r="K559" s="9" t="str">
+        <x:v>engine-specific seal catalog</x:v>
+      </x:c>
+      <x:c r="L559" s="9" t="str"/>
+      <x:c r="M559" s="9" t="str">
+        <x:v>S52 and M52TU/M54 use different VANOS types and seal kits; the source incorrectly treats them as one repair.</x:v>
+      </x:c>
+      <x:c r="N559" s="41" t="str">
+        <x:v>Split single/double VANOS, do not infer a scanner product from DTCs, and verify whether cam re-timing is actually disturbed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="560" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A560" s="40" t="str"/>
+      <x:c r="B560" s="9" t="str"/>
+      <x:c r="C560" s="9" t="str"/>
+      <x:c r="D560" s="9" t="str"/>
+      <x:c r="E560" s="9" t="str"/>
+      <x:c r="F560" s="9" t="str"/>
+      <x:c r="G560" s="9" t="str"/>
+      <x:c r="H560" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I560" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J560" s="9" t="str">
+        <x:v>VANOS/vacuum/timing diagnosis and installation</x:v>
+      </x:c>
+      <x:c r="K560" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L560" s="9" t="str"/>
+      <x:c r="M560" s="9" t="str"/>
+      <x:c r="N560" s="41" t="str"/>
+    </x:row>
+    <x:row r="561" ht="501.6000061035156" hidden="0" customHeight="1">
+      <x:c r="A561" s="40" t="n">
+        <x:v>375</x:v>
+      </x:c>
+      <x:c r="B561" s="9" t="str">
+        <x:v>bmw-z4-b58-coolant-tank-2019</x:v>
+      </x:c>
+      <x:c r="C561" s="9" t="str">
+        <x:v>2019-2026 | BMW | Z4 | B58</x:v>
+      </x:c>
+      <x:c r="D561" s="9" t="str">
+        <x:v>B58 Coolant Expansion Tank Cracking</x:v>
+      </x:c>
+      <x:c r="E561" s="9" t="str">
+        <x:v>Replace the coolant expansion tank with an updated BMW part or aftermarket aluminum tank. Inspect the tank and cap regularly for signs of cracking, discoloration, or seepage. When replacing, also replace the cap and check all coolant hoses for brittleness. Flush and refill with BMW-approved coolant.</x:v>
+      </x:c>
+      <x:c r="F561" s="9" t="str">
+        <x:v>Pressure-test and identify coolant circuit; VIN-specific tank; updated/superseded OEM part only if cataloged; aluminum tank only with proven G29 fitment/interfaces; cap/hoses by condition; correct coolant/bleed</x:v>
+      </x:c>
+      <x:c r="G561" s="9" t="str">
+        <x:v>VIN / CIRCUIT GATE; ALUMINUM CLAIM HELD</x:v>
+      </x:c>
+      <x:c r="H561" s="9" t="str">
+        <x:v>BMW Z4 expansion-tank catalog</x:v>
+      </x:c>
+      <x:c r="I561" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/Z4/Expansion-Tank/</x:v>
+      </x:c>
+      <x:c r="J561" s="9" t="str">
+        <x:v>2019-2026 G29 Z4; select B48/B58, VIN, and coolant circuit</x:v>
+      </x:c>
+      <x:c r="K561" s="9" t="str">
+        <x:v>vehicle-specific tank catalog</x:v>
+      </x:c>
+      <x:c r="L561" s="9" t="str"/>
+      <x:c r="M561" s="9" t="str">
+        <x:v>The source does not identify an exact updated or aluminum tank and G29 has multiple cooling circuits.</x:v>
+      </x:c>
+      <x:c r="N561" s="41" t="str">
+        <x:v>Do not promise updated plastic or approve aluminum without exact cap/sensor/hose/pressure fitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="562" ht="1306.800048828125" hidden="0" customHeight="1">
+      <x:c r="A562" s="40" t="n">
+        <x:v>376</x:v>
+      </x:c>
+      <x:c r="B562" s="9" t="str">
+        <x:v>bmw-z4-e85-convertible-top-hydraulic-2003</x:v>
+      </x:c>
+      <x:c r="C562" s="9" t="str">
+        <x:v>2003-2008 | BMW | Z4</x:v>
+      </x:c>
+      <x:c r="D562" s="9" t="str">
+        <x:v>Convertible Top Hydraulic Pump Motor Failure - E85 Z4</x:v>
+      </x:c>
+      <x:c r="E562" s="9" t="str">
+        <x:v>Replace hydraulic pump motor assembly (BMW 54347193448 / supersedes 54347119633). OEM Genuine BMW pump: $800-$1,200. Aftermarket alternatives available on Amazon for $150-$300 but quality varies significantly. Dealer labor is $1,500-$2,500+ as BMW procedure requires full top removal. ZRoadster.org members have documented a motor relocation to the boot/trunk area which allows much easier future access. Hydraulic fluid: use Aral Vitamol ZHM or BMW 54340394395 hydraulic oil. PREVENTION: Clean drain holes annually, ensure rubber bungs are properly seated, and check for water intrusion in pump area at every service. Some owners have had success with pump motor rebuilds from roofmotors.co.uk ($300-$500) but quality of rebuilds varies.</x:v>
+      </x:c>
+      <x:c r="F562" s="9" t="str">
+        <x:v>Roof fault/leak/water-intrusion diagnosis; pump motor 54347193448 only if confirmed; correct top fluid 54340394395; drains and mounting inspection; relocation/rebuild as specialist modification</x:v>
+      </x:c>
+      <x:c r="G562" s="9" t="str">
+        <x:v>EXACT CONDITIONAL E85 PUMP / FLUID</x:v>
+      </x:c>
+      <x:c r="H562" s="9" t="str">
+        <x:v>Genuine BMW E85 roof pump 54347193448</x:v>
+      </x:c>
+      <x:c r="I562" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/parts/bmw-hydraulic_unit-54347193448.html</x:v>
+      </x:c>
+      <x:c r="J562" s="9" t="str">
+        <x:v>2003-2008 E85 Z4 where VIN-matched; supersedes 54347119633</x:v>
+      </x:c>
+      <x:c r="K562" s="9" t="str">
+        <x:v>conditional hydraulic unit/pump</x:v>
+      </x:c>
+      <x:c r="L562" s="9" t="str"/>
+      <x:c r="M562" s="9" t="str">
+        <x:v>The OEM number/supersession is exact, but water, motor, pump, cylinders, and microswitches must be distinguished.</x:v>
+      </x:c>
+      <x:c r="N562" s="41" t="str">
+        <x:v>Do not recommend unverified Amazon motors or a relocation/rebuild without specialist quality and water-management review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="563" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A563" s="40" t="str"/>
+      <x:c r="B563" s="9" t="str"/>
+      <x:c r="C563" s="9" t="str"/>
+      <x:c r="D563" s="9" t="str"/>
+      <x:c r="E563" s="9" t="str"/>
+      <x:c r="F563" s="9" t="str"/>
+      <x:c r="G563" s="9" t="str"/>
+      <x:c r="H563" s="9" t="str">
+        <x:v>BMW roof hydraulic fluid 54340394395</x:v>
+      </x:c>
+      <x:c r="I563" s="9" t="str">
+        <x:v>https://www.rmeuropean.com/Products/54340394395-MFG36-V11915.aspx</x:v>
+      </x:c>
+      <x:c r="J563" s="9" t="str">
+        <x:v>verify E85 roof-system application and service procedure</x:v>
+      </x:c>
+      <x:c r="K563" s="9" t="str">
+        <x:v>specified hydraulic fluid</x:v>
+      </x:c>
+      <x:c r="L563" s="9" t="str"/>
+      <x:c r="M563" s="9" t="str"/>
+      <x:c r="N563" s="41" t="str"/>
+    </x:row>
+    <x:row r="564" ht="1135.199951171875" hidden="0" customHeight="1">
+      <x:c r="A564" s="40" t="n">
+        <x:v>377</x:v>
+      </x:c>
+      <x:c r="B564" s="9" t="str">
+        <x:v>bmw-z4-e85-window-regulator-2003</x:v>
+      </x:c>
+      <x:c r="C564" s="9" t="str">
+        <x:v>2003-2008 | BMW | Z4</x:v>
+      </x:c>
+      <x:c r="D564" s="9" t="str">
+        <x:v>Power Window Regulator Failure - E85 Z4</x:v>
+      </x:c>
+      <x:c r="E564" s="9" t="str">
+        <x:v>Option 1 (Budget): Window regulator repair kit - replacement cables and rollers for ~$18-$25 from eBay/Amazon (BWR974 for left/driver side). Requires removing door panel and threading new cables through existing regulator frame. DIY-friendly with Z4-forum.com guides. Option 2 (Recommended): Full window regulator replacement. Driver side: BMW 51337198909 ($180-$280 OEM, $80-$150 aftermarket). Passenger side: BMW 51337198910 ($180-$280 OEM, $80-$150 aftermarket). Labor: $200-$400 at independent shop, $500-$700+ at dealer. DIY: 2-3 hours with door panel removal guide from Pelican Parts. ZRoadster.org recommends full replacement over repair kit for long-term reliability.</x:v>
+      </x:c>
+      <x:c r="F564" s="9" t="str">
+        <x:v>Left/right diagnosis; repair cables/rollers only if frame/gears sound; complete regulator 51337198909 left or 51337198910 right; window adjustment</x:v>
+      </x:c>
+      <x:c r="G564" s="9" t="str">
+        <x:v>EXACT SIDE-SPECIFIC OEM REGULATORS</x:v>
+      </x:c>
+      <x:c r="H564" s="9" t="str">
+        <x:v>Genuine BMW left regulator 51337198909</x:v>
+      </x:c>
+      <x:c r="I564" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/parts/bmw-window_lifter_without_motor_left-51337198909.html</x:v>
+      </x:c>
+      <x:c r="J564" s="9" t="str">
+        <x:v>2003-2008 E85 Z4 left/driver side where VIN-matched</x:v>
+      </x:c>
+      <x:c r="K564" s="9" t="str">
+        <x:v>left regulator</x:v>
+      </x:c>
+      <x:c r="L564" s="9" t="str"/>
+      <x:c r="M564" s="9" t="str">
+        <x:v>The source provides distinct left/right OEM numbers and separates repair-kit from complete-regulator branches.</x:v>
+      </x:c>
+      <x:c r="N564" s="41" t="str">
+        <x:v>Do not approve BWR974 by marketplace title alone or call cable rethreading universally DIY-friendly.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="565" ht="145.1999969482422" hidden="0" customHeight="1">
+      <x:c r="A565" s="40" t="str"/>
+      <x:c r="B565" s="9" t="str"/>
+      <x:c r="C565" s="9" t="str"/>
+      <x:c r="D565" s="9" t="str"/>
+      <x:c r="E565" s="9" t="str"/>
+      <x:c r="F565" s="9" t="str"/>
+      <x:c r="G565" s="9" t="str"/>
+      <x:c r="H565" s="9" t="str">
+        <x:v>Genuine BMW right regulator 51337198910</x:v>
+      </x:c>
+      <x:c r="I565" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/parts/bmw-window_lifter_without_motor_right-51337198910.html</x:v>
+      </x:c>
+      <x:c r="J565" s="9" t="str">
+        <x:v>2003-2008 E85 Z4 right/passenger side where VIN-matched</x:v>
+      </x:c>
+      <x:c r="K565" s="9" t="str">
+        <x:v>right regulator</x:v>
+      </x:c>
+      <x:c r="L565" s="9" t="str"/>
+      <x:c r="M565" s="9" t="str"/>
+      <x:c r="N565" s="41" t="str"/>
+    </x:row>
+    <x:row r="566" ht="514.7999877929688" hidden="0" customHeight="1">
+      <x:c r="A566" s="40" t="n">
+        <x:v>378</x:v>
+      </x:c>
+      <x:c r="B566" s="9" t="str">
+        <x:v>bmw-z4-electric-steering-rack-2003</x:v>
+      </x:c>
+      <x:c r="C566" s="9" t="str">
+        <x:v>2012-2012 | BMW | Z4</x:v>
+      </x:c>
+      <x:c r="D566" s="9" t="str">
+        <x:v>2012 Z4 Electric Power-Steering Recall 12V-302</x:v>
+      </x:c>
+      <x:c r="E566" s="9" t="str">
+        <x:v>Check the VIN for an open 12V-302 campaign. If open, an authorized BMW dealer replaces the steering-assistance module free of charge. If the steering warning and audible alert occur, maintain control, reduce speed, stop safely and arrange dealer or roadside assistance; do not replace a steering rack from this card.</x:v>
+      </x:c>
+      <x:c r="F566" s="9" t="str">
+        <x:v>VIN recall 12V-302 check; free steering-assistance module replacement; roadside safety response for warning/assist loss</x:v>
+      </x:c>
+      <x:c r="G566" s="9" t="str">
+        <x:v>RECALL ROUTES ONLY</x:v>
+      </x:c>
+      <x:c r="H566" s="9" t="str">
+        <x:v>BMW recall lookup</x:v>
+      </x:c>
+      <x:c r="I566" s="9" t="str">
+        <x:v>https://www.bmwusa.com/safety-and-emission-recalls.html</x:v>
+      </x:c>
+      <x:c r="J566" s="9" t="str">
+        <x:v>VIN check for 12V-302</x:v>
+      </x:c>
+      <x:c r="K566" s="9" t="str">
+        <x:v>manufacturer recall remedy</x:v>
+      </x:c>
+      <x:c r="L566" s="9" t="str"/>
+      <x:c r="M566" s="9" t="str">
+        <x:v>The recall remedy is a steering-assistance module, not a steering rack.</x:v>
+      </x:c>
+      <x:c r="N566" s="41" t="str">
+        <x:v>Correct the issue ID's 2003 mismatch: the row is 2012 Z4.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="567" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A567" s="40" t="str"/>
+      <x:c r="B567" s="9" t="str"/>
+      <x:c r="C567" s="9" t="str"/>
+      <x:c r="D567" s="9" t="str"/>
+      <x:c r="E567" s="9" t="str"/>
+      <x:c r="F567" s="9" t="str"/>
+      <x:c r="G567" s="9" t="str"/>
+      <x:c r="H567" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I567" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J567" s="9" t="str">
+        <x:v>independent VIN recall-status check</x:v>
+      </x:c>
+      <x:c r="K567" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L567" s="9" t="str"/>
+      <x:c r="M567" s="9" t="str"/>
+      <x:c r="N567" s="41" t="str"/>
+    </x:row>
+    <x:row r="568" ht="633.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A568" s="40" t="n">
+        <x:v>379</x:v>
+      </x:c>
+      <x:c r="B568" s="9" t="str">
+        <x:v>bmw-z4-electric-water-pump-2006</x:v>
+      </x:c>
+      <x:c r="C568" s="9" t="str">
+        <x:v>2012-2016 | BMW | Z4 | N20</x:v>
+      </x:c>
+      <x:c r="D568" s="9" t="str">
+        <x:v>2012-2016 Z4 sDrive28i Water-Pump Connector Recall 24V-608</x:v>
+      </x:c>
+      <x:c r="E568" s="9" t="str">
+        <x:v>Check the VIN for an open 24V-608 campaign. If open, an authorized BMW dealer inspects the water pump and connector, replaces them if necessary, and installs the protective shield free of charge. If smoke appears from the engine compartment, stop safely, switch off the vehicle, have occupants exit, move away from traffic and call emergency or roadside assistance; do not order a pump from this card.</x:v>
+      </x:c>
+      <x:c r="F568" s="9" t="str">
+        <x:v>VIN recall 24V-608 check; free pump/connector inspection, conditional replacement and protective shield; fire-safety response for smoke</x:v>
+      </x:c>
+      <x:c r="G568" s="9" t="str">
+        <x:v>RECALL ROUTES ONLY</x:v>
+      </x:c>
+      <x:c r="H568" s="9" t="str">
+        <x:v>BMW recall lookup</x:v>
+      </x:c>
+      <x:c r="I568" s="9" t="str">
+        <x:v>https://www.bmwusa.com/safety-and-emission-recalls.html</x:v>
+      </x:c>
+      <x:c r="J568" s="9" t="str">
+        <x:v>VIN check for 24V-608</x:v>
+      </x:c>
+      <x:c r="K568" s="9" t="str">
+        <x:v>manufacturer recall remedy</x:v>
+      </x:c>
+      <x:c r="L568" s="9" t="str"/>
+      <x:c r="M568" s="9" t="str">
+        <x:v>The campaign decides whether pump/connector replacement is required and supplies the shield free.</x:v>
+      </x:c>
+      <x:c r="N568" s="41" t="str">
+        <x:v>Correct the issue ID's 2006 mismatch and do not order a pump from this recall card.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="569" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A569" s="40" t="str"/>
+      <x:c r="B569" s="9" t="str"/>
+      <x:c r="C569" s="9" t="str"/>
+      <x:c r="D569" s="9" t="str"/>
+      <x:c r="E569" s="9" t="str"/>
+      <x:c r="F569" s="9" t="str"/>
+      <x:c r="G569" s="9" t="str"/>
+      <x:c r="H569" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I569" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J569" s="9" t="str">
+        <x:v>independent VIN recall-status check</x:v>
+      </x:c>
+      <x:c r="K569" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L569" s="9" t="str"/>
+      <x:c r="M569" s="9" t="str"/>
+      <x:c r="N569" s="41" t="str"/>
+    </x:row>
+    <x:row r="570" ht="1359.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A570" s="40" t="n">
+        <x:v>380</x:v>
+      </x:c>
+      <x:c r="B570" s="9" t="str">
+        <x:v>bmw-z4-g29-b58-water-pump-2019</x:v>
+      </x:c>
+      <x:c r="C570" s="9" t="str">
+        <x:v>2019-2025 | BMW | Z4 | M40i, sDrive35i, sDrive35is | B48, B58</x:v>
+      </x:c>
+      <x:c r="D570" s="9" t="str">
+        <x:v>B48/B58 Electric Water Pump &amp; Thermostat Failure - G29 Z4</x:v>
+      </x:c>
+      <x:c r="E570" s="9" t="str">
+        <x:v>Preventative replacement recommended at 60,000 miles. Always replace water pump and thermostat together - they share labor overlap and frequently fail concurrently. B48 sDrive30i: Water pump BMW 11518632586 ($300-$450), Thermostat BMW 11538685978 ($100-$150). B58 M40i: Water pump BMW 11518650986 ($350-$500), Thermostat BMW 11538685978 ($100-$150). Mishimoto offers performance water pump alternatives for B58 with improved impeller design. Replace 3 O-rings between thermostat and pump housing, plus 2 O-rings on coolant tube to head. Must replace water pump mounting bolts (torque-to-yield). Labor: 3-4 hours. FCP Euro lifetime warranty kits available. Also inspect plastic cylinder head coolant outlet adapter - known to shear off causing massive coolant leak.</x:v>
+      </x:c>
+      <x:c r="F570" s="9" t="str">
+        <x:v>Split B48/B58 and main/auxiliary cooling circuits; fault/pressure diagnosis; identify mechanical versus electric pump; thermostat and seals/bolts only by exact procedure; outlet adapter inspection</x:v>
+      </x:c>
+      <x:c r="G570" s="9" t="str">
+        <x:v>MAJOR PUMP-TYPE / ENGINE CORRECTION</x:v>
+      </x:c>
+      <x:c r="H570" s="9" t="str">
+        <x:v>Genuine BMW G29 Z4 water-pump catalog</x:v>
+      </x:c>
+      <x:c r="I570" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-z4-water_pump.html</x:v>
+      </x:c>
+      <x:c r="J570" s="9" t="str">
+        <x:v>2019-2025 G29; VIN, B48/B58 engine, and coolant circuit required</x:v>
+      </x:c>
+      <x:c r="K570" s="9" t="str">
+        <x:v>OEM pump/thermostat catalog</x:v>
+      </x:c>
+      <x:c r="L570" s="9" t="str"/>
+      <x:c r="M570" s="9" t="str">
+        <x:v>B48/B58 modular engines have multiple pumps/circuits and the source's universal 'electric pump and thermostat together' statement is not reliable.</x:v>
+      </x:c>
+      <x:c r="N570" s="41" t="str">
+        <x:v>Remove fixed 60k replacement, unverified part numbers/Mishimoto claim, and mandatory paired replacement until exact VIN diagram/procedure is established.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="571" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A571" s="40" t="str"/>
+      <x:c r="B571" s="9" t="str"/>
+      <x:c r="C571" s="9" t="str"/>
+      <x:c r="D571" s="9" t="str"/>
+      <x:c r="E571" s="9" t="str"/>
+      <x:c r="F571" s="9" t="str"/>
+      <x:c r="G571" s="9" t="str"/>
+      <x:c r="H571" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I571" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J571" s="9" t="str">
+        <x:v>cooling-system diagnosis and bleed</x:v>
+      </x:c>
+      <x:c r="K571" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L571" s="9" t="str"/>
+      <x:c r="M571" s="9" t="str"/>
+      <x:c r="N571" s="41" t="str"/>
+    </x:row>
+    <x:row r="572" ht="1122" hidden="0" customHeight="1">
+      <x:c r="A572" s="40" t="n">
+        <x:v>381</x:v>
+      </x:c>
+      <x:c r="B572" s="9" t="str">
+        <x:v>bmw-z4-n54-hpfp-2009</x:v>
+      </x:c>
+      <x:c r="C572" s="9" t="str">
+        <x:v>2009-2011 | BMW | Z4 | M40i, sDrive35i, sDrive35is | N54</x:v>
+      </x:c>
+      <x:c r="D572" s="9" t="str">
+        <x:v>N54 High Pressure Fuel Pump (HPFP) Failure - E89 Z4 sDrive35i/35is</x:v>
+      </x:c>
+      <x:c r="E572" s="9" t="str">
+        <x:v>Replace HPFP with latest revision Genuine BMW unit. The pump went through multiple revisions - ONLY install the latest version. Part number evolution: Original -&gt; 13517592881 (Index 10, TSB fix) -&gt; 13517616170 (latest revision, most reliable). Genuine BMW 13517616170 is the definitive fix ($350-$550 for pump). Replacement is straightforward DIY (1-2 hours) with basic tools. Also available as complete kit from FCP Euro with lifetime warranty. BMW extended warranty coverage to 10 years/120,000 miles under customer care package for original owners - check VIN eligibility. Replace low-pressure fuel sensor at same time (13537537319) as it may have been damaged by pressure fluctuations ($35-$55).</x:v>
+      </x:c>
+      <x:c r="F572" s="9" t="str">
+        <x:v>BMW fuel-pressure and low-side diagnosis; VIN/current supersession check; latest compatible HPFP only after confirmed failure; low-pressure sensor only if test-failed; expired historical coverage disclosed</x:v>
+      </x:c>
+      <x:c r="G572" s="9" t="str">
+        <x:v>DIAGNOSIS / CURRENT-SUPERSESSION GATE</x:v>
+      </x:c>
+      <x:c r="H572" s="9" t="str">
+        <x:v>Genuine BMW Z4 high-pressure pump catalog</x:v>
+      </x:c>
+      <x:c r="I572" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-z4-fuel_pump.html</x:v>
+      </x:c>
+      <x:c r="J572" s="9" t="str">
+        <x:v>2009-2011 E89 sDrive35i/35is N54; VIN and current supersession required</x:v>
+      </x:c>
+      <x:c r="K572" s="9" t="str">
+        <x:v>OEM HPFP catalog</x:v>
+      </x:c>
+      <x:c r="L572" s="9" t="str"/>
+      <x:c r="M572" s="9" t="str">
+        <x:v>The claimed 'latest' number and customer-care coverage may have been superseded/expired, and the low-pressure sensor is not automatic.</x:v>
+      </x:c>
+      <x:c r="N572" s="41" t="str">
+        <x:v>Do not call HPFP replacement straightforward or definitive without pressure diagnosis/current ETK.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="573" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A573" s="40" t="str"/>
+      <x:c r="B573" s="9" t="str"/>
+      <x:c r="C573" s="9" t="str"/>
+      <x:c r="D573" s="9" t="str"/>
+      <x:c r="E573" s="9" t="str"/>
+      <x:c r="F573" s="9" t="str"/>
+      <x:c r="G573" s="9" t="str"/>
+      <x:c r="H573" s="9" t="str">
+        <x:v>BMW dealer locator</x:v>
+      </x:c>
+      <x:c r="I573" s="9" t="str">
+        <x:v>https://www.bmwusa.com/dealer-locator.html</x:v>
+      </x:c>
+      <x:c r="J573" s="9" t="str">
+        <x:v>fuel-pressure diagnosis and historical coverage/VIN review</x:v>
+      </x:c>
+      <x:c r="K573" s="9" t="str">
+        <x:v>BMW-qualified service</x:v>
+      </x:c>
+      <x:c r="L573" s="9" t="str"/>
+      <x:c r="M573" s="9" t="str"/>
+      <x:c r="N573" s="41" t="str"/>
+    </x:row>
+    <x:row r="574" ht="580.7999877929688" hidden="0" customHeight="1">
+      <x:c r="A574" s="40" t="n">
+        <x:v>382</x:v>
+      </x:c>
+      <x:c r="B574" s="9" t="str">
+        <x:v>bmw-z4-n54-wastegate-rattle-2009</x:v>
+      </x:c>
+      <x:c r="C574" s="9" t="str">
+        <x:v>2009-2010 | BMW | Z4 | N54</x:v>
+      </x:c>
+      <x:c r="D574" s="9" t="str">
+        <x:v>2009-2010 Z4 sDrive35i N54 Wastegate Diagnosis</x:v>
+      </x:c>
+      <x:c r="E574" s="9" t="str">
+        <x:v>Confirm the VIN, engine, production date, DME faults, boost-control data and noise source using current BMW diagnostic information. Check VIN-specific coverage history with BMW, recognizing that the bulletin's time/mileage window may have expired. Do not replace a turbocharger, actuator or wastegate from this card without the required diagnosis.</x:v>
+      </x:c>
+      <x:c r="F574" s="9" t="str">
+        <x:v>VIN/engine/production/DME/boost-control/noise-source diagnosis; historical coverage check; exact turbo/actuator/wastegate only after confirmation</x:v>
+      </x:c>
+      <x:c r="G574" s="9" t="str">
+        <x:v>DIAGNOSIS ROUTE; NO RETAIL PART</x:v>
+      </x:c>
+      <x:c r="H574" s="9" t="str">
+        <x:v>BMW dealer locator</x:v>
+      </x:c>
+      <x:c r="I574" s="9" t="str">
+        <x:v>https://www.bmwusa.com/dealer-locator.html</x:v>
+      </x:c>
+      <x:c r="J574" s="9" t="str">
+        <x:v>2009-2010 E89 sDrive35i N54 diagnostic and coverage-history check</x:v>
+      </x:c>
+      <x:c r="K574" s="9" t="str">
+        <x:v>BMW-qualified service</x:v>
+      </x:c>
+      <x:c r="L574" s="9" t="str"/>
+      <x:c r="M574" s="9" t="str">
+        <x:v>The corrected source explicitly rejects turbo/actuator/wastegate purchase without diagnosis.</x:v>
+      </x:c>
+      <x:c r="N574" s="41" t="str">
+        <x:v>Preserve the expired-coverage caveat and do not attach marketplace repair kits.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="575" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A575" s="40" t="str"/>
+      <x:c r="B575" s="9" t="str"/>
+      <x:c r="C575" s="9" t="str"/>
+      <x:c r="D575" s="9" t="str"/>
+      <x:c r="E575" s="9" t="str"/>
+      <x:c r="F575" s="9" t="str"/>
+      <x:c r="G575" s="9" t="str"/>
+      <x:c r="H575" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I575" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J575" s="9" t="str">
+        <x:v>N54 boost/wastegate diagnosis</x:v>
+      </x:c>
+      <x:c r="K575" s="9" t="str">
+        <x:v>specialist service</x:v>
+      </x:c>
+      <x:c r="L575" s="9" t="str"/>
+      <x:c r="M575" s="9" t="str"/>
+      <x:c r="N575" s="41" t="str"/>
+    </x:row>
+    <x:row r="576" ht="501.6000061035156" hidden="0" customHeight="1">
+      <x:c r="A576" s="40" t="n">
+        <x:v>383</x:v>
+      </x:c>
+      <x:c r="B576" s="9" t="str">
+        <x:v>bmw-z4-soft-top-hydraulic-2003</x:v>
+      </x:c>
+      <x:c r="C576" s="9" t="str">
+        <x:v>2009-2016 | BMW | Z4</x:v>
+      </x:c>
+      <x:c r="D576" s="9" t="str">
+        <x:v>Retractable Hard Top Hydraulic Mechanism Failure</x:v>
+      </x:c>
+      <x:c r="E576" s="9" t="str">
+        <x:v>Diagnose the leak location and replace the failed component. Common failure points are the main hydraulic cylinders (left and right), the hydraulic pump motor, and the flexible hoses. The hydraulic fluid should be flushed and replaced with BMW-approved CHF 11S fluid. A full system bleed is required after any repair.</x:v>
+      </x:c>
+      <x:c r="F576" s="9" t="str">
+        <x:v>E89 retractable-hardtop fault and leak-location diagnosis; exact left/right cylinder, hose, pump, microswitch or sensor; BMW-specified hydraulic fluid and full bleed</x:v>
+      </x:c>
+      <x:c r="G576" s="9" t="str">
+        <x:v>COMPONENT / SIDE / FLUID-SPEC GATE</x:v>
+      </x:c>
+      <x:c r="H576" s="9" t="str">
+        <x:v>Genuine BMW E89 folding-top hydraulics catalog</x:v>
+      </x:c>
+      <x:c r="I576" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-z4-convertible_top_motor.html</x:v>
+      </x:c>
+      <x:c r="J576" s="9" t="str">
+        <x:v>2009-2016 E89 Z4; VIN and diagnosed pump/cylinder/hose/sensor required</x:v>
+      </x:c>
+      <x:c r="K576" s="9" t="str">
+        <x:v>OEM roof-system catalog</x:v>
+      </x:c>
+      <x:c r="L576" s="9" t="str"/>
+      <x:c r="M576" s="9" t="str">
+        <x:v>The mechanism has many hydraulic/control branches, and CHF 11S was not verified as the correct roof fluid for every E89 procedure.</x:v>
+      </x:c>
+      <x:c r="N576" s="41" t="str">
+        <x:v>Correct the issue ID's 2003 mismatch and verify BMW fluid part/specification rather than assuming power-steering hydraulic fluid.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="577" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A577" s="40" t="str"/>
+      <x:c r="B577" s="9" t="str"/>
+      <x:c r="C577" s="9" t="str"/>
+      <x:c r="D577" s="9" t="str"/>
+      <x:c r="E577" s="9" t="str"/>
+      <x:c r="F577" s="9" t="str"/>
+      <x:c r="G577" s="9" t="str"/>
+      <x:c r="H577" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I577" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J577" s="9" t="str">
+        <x:v>retractable-hardtop hydraulic/control diagnosis and bleed</x:v>
+      </x:c>
+      <x:c r="K577" s="9" t="str">
+        <x:v>specialist service</x:v>
+      </x:c>
+      <x:c r="L577" s="9" t="str"/>
+      <x:c r="M577" s="9" t="str"/>
+      <x:c r="N577" s="41" t="str"/>
+    </x:row>
+    <x:row r="578" ht="1188" hidden="0" customHeight="1">
+      <x:c r="A578" s="40" t="n">
+        <x:v>384</x:v>
+      </x:c>
+      <x:c r="B578" s="9" t="str">
+        <x:v>bmw-z4-vanos-solenoid-2003</x:v>
+      </x:c>
+      <x:c r="C578" s="9" t="str">
+        <x:v>2003-2016 | BMW | Z4 | 2.5i, 3.0i, 3.0si, M40i, sDrive28i, sDrive30i, sDrive35i, sDrive35is | M54, N52, N54, N20</x:v>
+      </x:c>
+      <x:c r="D578" s="9" t="str">
+        <x:v>VANOS Solenoid &amp; System Failure - E85/E89 Z4 (All Engines)</x:v>
+      </x:c>
+      <x:c r="E578" s="9" t="str">
+        <x:v>Replace VANOS solenoids - inexpensive and straightforward repair. M54 (E85 2003-2005): 2 solenoids required, BMW 11361707323 ($35-$65 each). N52 (E85 2006-2008 / E89 2009-2011 28i): 2 solenoids, BMW 11367585425 ($40-$70 each). N54 (E89 35i/35is): 2 solenoids, BMW 11367585425 ($40-$70 each). N20 (E89 sDrive28i 2012-2016): 2 solenoids, BMW 11367585425 ($40-$70 each). Labor: under 1 hour for experienced mechanic, 2-3 hours DIY. Replace all solenoids at once even if only one has failed - the others are same age and will fail soon. Also replace VANOS solenoid O-rings and sealing plates during service. Clean VANOS system with Beisan Systems VANOS cleaning procedure for best results.</x:v>
+      </x:c>
+      <x:c r="F578" s="9" t="str">
+        <x:v>Split M54/N52/N54/N20 and VANOS architecture; BMW-capable oil-pressure/wiring/timing diagnosis; exact intake/exhaust/engine solenoid or complete VANOS component; seals by procedure</x:v>
+      </x:c>
+      <x:c r="G578" s="9" t="str">
+        <x:v>MAJOR ENGINE / VANOS-ARCHITECTURE SPLIT</x:v>
+      </x:c>
+      <x:c r="H578" s="9" t="str">
+        <x:v>BMW Z4 VANOS-solenoid catalog</x:v>
+      </x:c>
+      <x:c r="I578" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/BMW-parts/Z4/VANOS-Solenoid/</x:v>
+      </x:c>
+      <x:c r="J578" s="9" t="str">
+        <x:v>2003-2016 E85/E89; select exact engine, VIN, position, and diagnosed component</x:v>
+      </x:c>
+      <x:c r="K578" s="9" t="str">
+        <x:v>engine-specific VANOS catalog</x:v>
+      </x:c>
+      <x:c r="L578" s="9" t="str"/>
+      <x:c r="M578" s="9" t="str">
+        <x:v>The source assigns two solenoids/part numbers across engines with different VANOS designs and automatically replaces all units.</x:v>
+      </x:c>
+      <x:c r="N578" s="41" t="str">
+        <x:v>M54 is not accurately represented by two external solenoids; split every engine, remove all-at-once and cleaning/flush claims, and verify exact position/number.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="579" ht="66" hidden="0" customHeight="1">
+      <x:c r="A579" s="40" t="str"/>
+      <x:c r="B579" s="9" t="str"/>
+      <x:c r="C579" s="9" t="str"/>
+      <x:c r="D579" s="9" t="str"/>
+      <x:c r="E579" s="9" t="str"/>
+      <x:c r="F579" s="9" t="str"/>
+      <x:c r="G579" s="9" t="str"/>
+      <x:c r="H579" s="9" t="str">
+        <x:v>BMW specialist locator</x:v>
+      </x:c>
+      <x:c r="I579" s="9" t="str">
+        <x:v>https://www.bimmershops.com/</x:v>
+      </x:c>
+      <x:c r="J579" s="9" t="str">
+        <x:v>BMW-capable VANOS/oil/timing diagnosis</x:v>
+      </x:c>
+      <x:c r="K579" s="9" t="str">
+        <x:v>service route</x:v>
+      </x:c>
+      <x:c r="L579" s="9" t="str"/>
+      <x:c r="M579" s="9" t="str"/>
+      <x:c r="N579" s="41" t="str"/>
+    </x:row>
+    <x:row r="580" ht="554.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A580" s="40" t="n">
+        <x:v>385</x:v>
+      </x:c>
+      <x:c r="B580" s="9" t="str">
+        <x:v>bmw-z8-soft-top-mechanism-2000</x:v>
+      </x:c>
+      <x:c r="C580" s="9" t="str">
+        <x:v>2000-2003 | BMW | Z8</x:v>
+      </x:c>
+      <x:c r="D580" s="9" t="str">
+        <x:v>Power Soft Top Hydraulic System and Cable Failure</x:v>
+      </x:c>
+      <x:c r="E580" s="9" t="str">
+        <x:v>Rebuild the hydraulic cylinders with new seals rather than replacing ($200 vs $2,000+). Inspect and replace frayed cables. Adjust or replace the microswitch sensors at the windshield header latch. Lubricate the top mechanism pivot points with silicone grease annually. Store the car with the top up to reduce stress on the hydraulic system.</x:v>
+      </x:c>
+      <x:c r="F580" s="9" t="str">
+        <x:v>Leak/pressure/cable/latch/microswitch diagnosis; exact cylinder rebuild by specialist if rebuildable; frayed cable or sensor by VIN/position; correct lubricant/storage guidance</x:v>
+      </x:c>
+      <x:c r="G580" s="9" t="str">
+        <x:v>SPECIALIST REBUILD / COMPONENT GATE</x:v>
+      </x:c>
+      <x:c r="H580" s="9" t="str">
+        <x:v>BMW Z8 soft-top catalog</x:v>
+      </x:c>
+      <x:c r="I580" s="9" t="str">
+        <x:v>https://www.bmwpartsdeal.com/oem-bmw-z8-convertible_top.html</x:v>
+      </x:c>
+      <x:c r="J580" s="9" t="str">
+        <x:v>2000-2003 E52 Z8; VIN and exact hydraulic/cable/sensor component required</x:v>
+      </x:c>
+      <x:c r="K580" s="9" t="str">
+        <x:v>OEM roof-system catalog</x:v>
+      </x:c>
+      <x:c r="L580" s="9" t="str"/>
+      <x:c r="M580" s="9" t="str">
+        <x:v>Cylinder rebuild, cable replacement, microswitch adjustment, and mechanism lubrication are separate branches.</x:v>
+      </x:c>
+      <x:c r="N580" s="41" t="str">
+        <x:v>Do not quote rebuild/replacement prices or annual silicone-grease/storage rules without the current specialist/BMW procedure.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="581" ht="158.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A581" s="42" t="str"/>
+      <x:c r="B581" s="43" t="str"/>
+      <x:c r="C581" s="43" t="str"/>
+      <x:c r="D581" s="43" t="str"/>
+      <x:c r="E581" s="43" t="str"/>
+      <x:c r="F581" s="43" t="str"/>
+      <x:c r="G581" s="43" t="str"/>
+      <x:c r="H581" s="43" t="str">
+        <x:v>Top Hydraulics BMW services</x:v>
+      </x:c>
+      <x:c r="I581" s="43" t="str">
+        <x:v>https://www.tophydraulics.com/bmw/</x:v>
+      </x:c>
+      <x:c r="J581" s="43" t="str">
+        <x:v>verify current Z8/E52 cylinder rebuild offering, core terms, and exact cylinder before shipment</x:v>
+      </x:c>
+      <x:c r="K581" s="43" t="str">
+        <x:v>conditional hydraulic rebuild service</x:v>
+      </x:c>
+      <x:c r="L581" s="43" t="str"/>
+      <x:c r="M581" s="43" t="str"/>
+      <x:c r="N581" s="44" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -19770,712 +21653,26 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A1" s="37" t="str">
+      <x:c r="A1" s="45" t="str">
         <x:v>#</x:v>
       </x:c>
-      <x:c r="B1" s="38" t="str">
+      <x:c r="B1" s="46" t="str">
         <x:v>Issue ID</x:v>
       </x:c>
-      <x:c r="C1" s="38" t="str">
+      <x:c r="C1" s="46" t="str">
         <x:v>YMMT</x:v>
       </x:c>
-      <x:c r="D1" s="38" t="str">
+      <x:c r="D1" s="46" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="E1" s="38" t="str">
+      <x:c r="E1" s="46" t="str">
         <x:v>Full How to Fix</x:v>
       </x:c>
-      <x:c r="F1" s="38" t="str">
+      <x:c r="F1" s="46" t="str">
         <x:v>Existing claim count</x:v>
       </x:c>
-      <x:c r="G1" s="39" t="str">
+      <x:c r="G1" s="47" t="str">
         <x:v>Queue status</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="897.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A2" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B2" s="9" t="str">
-        <x:v>bmw-x7-n63-oil-consumption-2019</x:v>
-      </x:c>
-      <x:c r="C2" s="9" t="str">
-        <x:v>2019-2023 | BMW | X7 | M50i, M60i, xDrive50i | N63TU3</x:v>
-      </x:c>
-      <x:c r="D2" s="9" t="str">
-        <x:v>N63TU3 Oil Consumption &amp; Valve Stem Seal Degradation (xDrive50i/M50i/M60i)</x:v>
-      </x:c>
-      <x:c r="E2" s="9" t="str">
-        <x:v>Replace valve stem seals - extremely labor-intensive job requiring cylinder head work ($4,900-12,000 total). Elring seals 11340039494 for OEM spec. 5150 AutoSport Viton upgraded seals ($150-200) recommended for better heat resistance. AGA Tools kit includes specialized tools required. Reference TSB MC-10149960-9999 when visiting dealer. Check eligibility for class action settlement coverage. Some owners monitor oil levels and top off rather than repair. Use quality synthetic 0W-40 BMW LL-01 spec oil and check level every 500-1,000 miles.</x:v>
-      </x:c>
-      <x:c r="F2" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G2" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="396" hidden="0" customHeight="1">
-      <x:c r="A3" s="40" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B3" s="9" t="str">
-        <x:v>bmw-x7-panoramic-roof-rattle-2019</x:v>
-      </x:c>
-      <x:c r="C3" s="9" t="str">
-        <x:v>2019-2026 | BMW | X7</x:v>
-      </x:c>
-      <x:c r="D3" s="9" t="str">
-        <x:v>Panoramic Sunroof Rattle and Creak</x:v>
-      </x:c>
-      <x:c r="E3" s="9" t="str">
-        <x:v>Apply BMW-approved felt tape or lubricant to sunroof guide rails. Replace worn guide rail bushings. In severe cases, the sunroof cassette or seal may need replacement under warranty. BMW has issued updated guide rail components for early production vehicles.</x:v>
-      </x:c>
-      <x:c r="F3" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G3" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="778.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A4" s="40" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B4" s="9" t="str">
-        <x:v>bmw-x7-sunroof-leak-2019</x:v>
-      </x:c>
-      <x:c r="C4" s="9" t="str">
-        <x:v>2019-2023 | BMW | X7</x:v>
-      </x:c>
-      <x:c r="D4" s="9" t="str">
-        <x:v>Panoramic Sunroof Water Leak</x:v>
-      </x:c>
-      <x:c r="E4" s="9" t="str">
-        <x:v>Clear clogged sunroof drain tubes ($100-300 at shop). Reference TSB SIB 54 11 19 when visiting dealer. For persistent leaks, drain tube connections or sunroof seal may need replacement ($500-1,500). If water has damaged interior electronics, repair costs can reach $3,000. PREVENTIVE: Clear sunroof drains annually, especially in areas with heavy tree debris. Run compressed air or flexible drain snake through drain tubes during oil changes. Keep sunroof track clean of debris.</x:v>
-      </x:c>
-      <x:c r="F4" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G4" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="739.2000122070312" hidden="0" customHeight="1">
-      <x:c r="A5" s="40" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B5" s="9" t="str">
-        <x:v>bmw-x7-tire-wear-2019</x:v>
-      </x:c>
-      <x:c r="C5" s="9" t="str">
-        <x:v>2019-2023 | BMW | X7</x:v>
-      </x:c>
-      <x:c r="D5" s="9" t="str">
-        <x:v>Premature Tire Wear (Especially 21"/22" Wheels)</x:v>
-      </x:c>
-      <x:c r="E5" s="9" t="str">
-        <x:v>Have alignment adjusted to reduce aggressive camber settings ($200-400). Switch to quality tires designed for heavy SUVs: Michelin Pilot Sport 4S or Continental PremiumContact 6 are recommended. If possible, avoid 22" wheels and opt for 21" or smaller for better tire longevity and ride comfort. Alignment adjustment can extend tire life from 15,000 to 30,000+ miles. Total cost $200-2,000 depending on tire replacement needs. Check alignment every 10,000 miles.</x:v>
-      </x:c>
-      <x:c r="F5" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G5" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="501.6000061035156" hidden="0" customHeight="1">
-      <x:c r="A6" s="40" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B6" s="9" t="str">
-        <x:v>bmw-xm-airbag-passenger-knee-recall-2023</x:v>
-      </x:c>
-      <x:c r="C6" s="9" t="str">
-        <x:v>2023-2023 | BMW | XM</x:v>
-      </x:c>
-      <x:c r="D6" s="9" t="str">
-        <x:v>2023 XM Front-Passenger Knee-Airbag Recall 23V-622</x:v>
-      </x:c>
-      <x:c r="E6" s="9" t="str">
-        <x:v>Check the VIN for an open 23V-622 campaign. If open, an authorized BMW dealer replaces the front-passenger knee airbag free of charge. Do not attempt airbag diagnosis or order a clock spring or airbag module from this card; supplemental-restraint work requires trained personnel and VIN-selected parts.</x:v>
-      </x:c>
-      <x:c r="F6" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G6" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="567.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A7" s="40" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B7" s="9" t="str">
-        <x:v>bmw-xm-hybrid-drivetrain-hesitation-2023</x:v>
-      </x:c>
-      <x:c r="C7" s="9" t="str">
-        <x:v>2023-2024 | BMW | XM | S68 4.4L Twin-Turbo V8 Hybrid, S68</x:v>
-      </x:c>
-      <x:c r="D7" s="9" t="str">
-        <x:v>Hybrid Drivetrain Hesitation and Power Delivery Lag</x:v>
-      </x:c>
-      <x:c r="E7" s="9" t="str">
-        <x:v>Visit the dealer for the latest transmission and hybrid system software calibration updates. Select Sport or Sport Plus mode for more consistent power delivery. The latest software revisions significantly improve the electric-to-V8 handoff smoothness. If hesitation persists after updates, the dealer can reset the transmission adaptation values to relearn driving patterns.</x:v>
-      </x:c>
-      <x:c r="F7" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G7" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="646.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A8" s="40" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="B8" s="9" t="str">
-        <x:v>bmw-xm-integrated-brake-system-recall-2023</x:v>
-      </x:c>
-      <x:c r="C8" s="9" t="str">
-        <x:v>2023-2024 | BMW | XM</x:v>
-      </x:c>
-      <x:c r="D8" s="9" t="str">
-        <x:v>2023-2024 XM Integrated Brake System Recall 26V-422</x:v>
-      </x:c>
-      <x:c r="E8" s="9" t="str">
-        <x:v>Check the VIN at NHTSA and with an authorized BMW dealer when campaign 26V-422 VINs become searchable, and arrange the free dealer inspection and module replacement if required. If a brake warning appears or pedal effort increases, avoid abrupt braking, allow extra stopping distance, stop safely and contact BMW roadside assistance; wheel-speed sensors are not the recall remedy.</x:v>
-      </x:c>
-      <x:c r="F8" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G8" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="646.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A9" s="40" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="B9" s="9" t="str">
-        <x:v>bmw-xm-suspension-ride-quality-2023</x:v>
-      </x:c>
-      <x:c r="C9" s="9" t="str">
-        <x:v>2023-2024 | BMW | XM | S68 4.4L Twin-Turbo V8 Hybrid</x:v>
-      </x:c>
-      <x:c r="D9" s="9" t="str">
-        <x:v>Harsh Ride Quality and Suspension Stiffness</x:v>
-      </x:c>
-      <x:c r="E9" s="9" t="str">
-        <x:v>Check tire pressures regularly - overinflated tires significantly worsen the harsh ride. Some owners report improved comfort by switching to a tire with a taller sidewall profile (if available for the XM's wheel size). Use Comfort mode for daily driving. Unfortunately, no aftermarket spring or damper solution currently exists to significantly improve the ride without compromising the handling needed for the XM's weight.</x:v>
-      </x:c>
-      <x:c r="F9" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G9" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="528" hidden="0" customHeight="1">
-      <x:c r="A10" s="40" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B10" s="9" t="str">
-        <x:v>bmw-z3-convertible-top-rear-window-cracking-clouding-bead-separatio</x:v>
-      </x:c>
-      <x:c r="C10" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D10" s="9" t="str">
-        <x:v>Convertible Top Rear Window Cracking, Clouding, and Bead Separation</x:v>
-      </x:c>
-      <x:c r="E10" s="9" t="str">
-        <x:v>Replace the rear window panel only — BMW used a zipper system so the clouded/cracked window unzips and a new window zips/tapes in without disturbing the fabric top. Re-gluing separated bead trim rarely holds, so window replacement is the durable fix. Job is a DIY-feasible 1-1.5 hours; replace the whole top only if the fabric is also degraded.</x:v>
-      </x:c>
-      <x:c r="F10" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G10" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="52.79999923706055" hidden="0" customHeight="1">
-      <x:c r="A11" s="40" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B11" s="9" t="str">
-        <x:v>bmw-z3-cooling-system-failure-1996</x:v>
-      </x:c>
-      <x:c r="C11" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D11" s="9" t="str">
-        <x:v>Cooling System Component Failures</x:v>
-      </x:c>
-      <x:c r="E11" s="9" t="str"/>
-      <x:c r="F11" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G11" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="448.79998779296875" hidden="0" customHeight="1">
-      <x:c r="A12" s="40" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B12" s="9" t="str">
-        <x:v>bmw-z3-cracked-exhaust-manifold-1-9l-4-cylinder</x:v>
-      </x:c>
-      <x:c r="C12" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3 | 1.9, 1.9i, Z3 1.9 | 1.9L M44 4-cylinder, 1.9L M43TU 4-cylinder</x:v>
-      </x:c>
-      <x:c r="D12" s="9" t="str">
-        <x:v>Cracked Exhaust Manifold on 1.9L 4-Cylinder (M44/M43)</x:v>
-      </x:c>
-      <x:c r="E12" s="9" t="str">
-        <x:v>Inspect the manifold for hairline cracks (a cold-engine listen or smoke test confirms the leak). Replace the cracked manifold with a used OE unit or an aftermarket stainless tubular header, and renew the manifold gasket and hardware. Allow roughly 3-4 hours labor.</x:v>
-      </x:c>
-      <x:c r="F12" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G12" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="686.4000244140625" hidden="0" customHeight="1">
-      <x:c r="A13" s="40" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B13" s="9" t="str">
-        <x:v>bmw-z3-differential-mount-ear-trunk-floor-pan-tearing</x:v>
-      </x:c>
-      <x:c r="C13" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D13" s="9" t="str">
-        <x:v>Differential Mount Ear and Trunk Floor Pan Tearing</x:v>
-      </x:c>
-      <x:c r="E13" s="9" t="str">
-        <x:v>Inspect the trunk floor around the differential mount and rear subframe pickup points for cracks, torn metal, and broken spot welds. Repair requires welding and a reinforcement/re-fabrication plate kit to tie the diff mount/subframe back into the floor. Switching the diff carrier bushings to polyurethane reduces carrier movement and the stress that causes the tearing. Catching it early greatly limits the repair scope.</x:v>
-      </x:c>
-      <x:c r="F13" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G13" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="514.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A14" s="40" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B14" s="9" t="str">
-        <x:v>bmw-z3-door-window-regulator-clip-mounting-tab-failure</x:v>
-      </x:c>
-      <x:c r="C14" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D14" s="9" t="str">
-        <x:v>Door Window Regulator Clip / Mounting Tab Failure</x:v>
-      </x:c>
-      <x:c r="E14" s="9" t="str">
-        <x:v>Replace the broken plastic regulator clips, or replace the regulator assembly if the cable or mechanism is also worn. If the welded mounting tab/anchor has torn from the door frame, it must be re-welded or reinforced before fitting a new regulator. Lubricate the window channels to reduce drag on the new parts.</x:v>
-      </x:c>
-      <x:c r="F14" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G14" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="686.4000244140625" hidden="0" customHeight="1">
-      <x:c r="A15" s="40" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B15" s="9" t="str">
-        <x:v>bmw-z3-fuel-level-sender-failure-causing-erratic-dead-fuel-gauge</x:v>
-      </x:c>
-      <x:c r="C15" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D15" s="9" t="str">
-        <x:v>Fuel Level Sender Failure Causing Erratic or Dead Fuel Gauge</x:v>
-      </x:c>
-      <x:c r="E15" s="9" t="str">
-        <x:v>Remove the access panel behind the seats and inspect the sender. A dirty or lightly worn ceramic/resistor plate can sometimes be cleaned, but a cracked plate or worn brushes requires replacing the sender unit (or the complete fuel-pump/sender carrier assembly). Also check the tank vent valve, as tank vacuum can deform the float arm. Confirm wiring/ground integrity before condemning the sender.</x:v>
-      </x:c>
-      <x:c r="F15" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G15" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="488.3999938964844" hidden="0" customHeight="1">
-      <x:c r="A16" s="40" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="B16" s="9" t="str">
-        <x:v>bmw-z3-hvac-blower-final-stage-resistor-failure</x:v>
-      </x:c>
-      <x:c r="C16" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D16" s="9" t="str">
-        <x:v>HVAC Blower Final Stage Resistor Failure (Fan Only Works on Max)</x:v>
-      </x:c>
-      <x:c r="E16" s="9" t="str">
-        <x:v>Replace the blower final stage resistor (A/C cars: part under the scuttle/cowl; non-A/C cars: behind the passenger footwell panel). If a new resistor does not restore all speeds, test the blower motor itself, which may also be worn. Inspect for corrosion/water intrusion at the cowl on A/C cars.</x:v>
-      </x:c>
-      <x:c r="F16" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G16" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="1584" hidden="0" customHeight="1">
-      <x:c r="A17" s="40" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B17" s="9" t="str">
-        <x:v>bmw-z3-rear-subframe-crack-1996</x:v>
-      </x:c>
-      <x:c r="C17" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3</x:v>
-      </x:c>
-      <x:c r="D17" s="9" t="str">
-        <x:v>Rear Subframe Mounting Point Cracking</x:v>
-      </x:c>
-      <x:c r="E17" s="9" t="str">
-        <x:v>Inspect the trunk floor, differential mount area, and all rear subframe mounting points from above and below the car for spot-weld separation, torn sheet metal, and cracked seams; a dye penetrant test or removing trunk trim/seam sealer may be needed to reveal early damage. If cracking is present, the proper repair is to drop the rear axle carrier/subframe, weld and reinforce the damaged unibody mounting points and trunk floor with a reinforcement kit (commonly Randy Forbes-style dual-ear/differential mount reinforcement or equivalent), then reinstall with new subframe bushings, differential mount bushings, and perform a 4-wheel alignment. Minor early cracks may be repairable before major deformation, but advanced damage often requires fabrication and extensive welding by a chassis/body specialist; typical cost ranges from about $2,000-$3,500 for early reinforcement repairs and can exceed $4,000-$6,000 if the floor is torn or multiple mounting points are damaged.</x:v>
-      </x:c>
-      <x:c r="F17" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G17" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="66" hidden="0" customHeight="1">
-      <x:c r="A18" s="40" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B18" s="9" t="str">
-        <x:v>bmw-z3-rear-subframe-cracking-1996</x:v>
-      </x:c>
-      <x:c r="C18" s="9" t="str">
-        <x:v>1996-2002 | BMW | Z3 | M52, M54</x:v>
-      </x:c>
-      <x:c r="D18" s="9" t="str">
-        <x:v>Rear Subframe Mounting Point Cracks</x:v>
-      </x:c>
-      <x:c r="E18" s="9" t="str"/>
-      <x:c r="F18" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G18" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="475.20001220703125" hidden="0" customHeight="1">
-      <x:c r="A19" s="40" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="B19" s="9" t="str">
-        <x:v>bmw-z3-valve-cover-gasket-oil-leak</x:v>
-      </x:c>
-      <x:c r="C19" s="9" t="str">
-        <x:v>1997-2002 | BMW | Z3 | 2.3, 2.5i, 2.8, 3.0i | M52 2.8, M52TU 2.5/2.8, M54 2.5/3.0</x:v>
-      </x:c>
-      <x:c r="D19" s="9" t="str">
-        <x:v>Valve Cover Gasket Oil Leak (M52/M54 6-Cylinder)</x:v>
-      </x:c>
-      <x:c r="E19" s="9" t="str">
-        <x:v>Replace the valve cover gasket, the spark-plug-well/grommet seals, and the cover bolt seals. On M54 engines also clean oil from the plug wells and replace any oil-contaminated coil boots/coils. Use the correct torque sequence to avoid re-leaking. Inspect the cover for warping or cracks while it is off.</x:v>
-      </x:c>
-      <x:c r="F19" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G19" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="1293.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A20" s="40" t="n">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="B20" s="9" t="str">
-        <x:v>bmw-z3-vanos-seals-1999</x:v>
-      </x:c>
-      <x:c r="C20" s="9" t="str">
-        <x:v>1999-2002 | BMW | Z3 | M52, M54, S52</x:v>
-      </x:c>
-      <x:c r="D20" s="9" t="str">
-        <x:v>VANOS Seal Failure (M52/M54/S52)</x:v>
-      </x:c>
-      <x:c r="E20" s="9" t="str">
-        <x:v>Confirm the fault by checking for cold-start VANOS rattle, rough idle, hesitation, and scanning for cam timing or mixture-related fault codes; on M52TU/M54/S52 engines, inspect VANOS operation and rule out vacuum leaks before disassembly. Repair typically involves removing the valve cover and VANOS unit, replacing the internal piston seals/O-rings with updated Viton/Teflon seals, renewing the valve cover gasket and VANOS oil line sealing washers, and then re-timing the cams to BMW specifications if required. If the unit still rattles after resealing, the VANOS bearing/anti-rattle components or the complete VANOS assembly may need replacement. Typical cost is about $60-$150 in seals/gaskets for DIY repair, $300-$700 for an independent shop reseal, or $800-$1,500+ if a rebuilt/replacement VANOS unit is installed.</x:v>
-      </x:c>
-      <x:c r="F20" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G20" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="501.6000061035156" hidden="0" customHeight="1">
-      <x:c r="A21" s="40" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B21" s="9" t="str">
-        <x:v>bmw-z4-b58-coolant-tank-2019</x:v>
-      </x:c>
-      <x:c r="C21" s="9" t="str">
-        <x:v>2019-2026 | BMW | Z4 | B58</x:v>
-      </x:c>
-      <x:c r="D21" s="9" t="str">
-        <x:v>B58 Coolant Expansion Tank Cracking</x:v>
-      </x:c>
-      <x:c r="E21" s="9" t="str">
-        <x:v>Replace the coolant expansion tank with an updated BMW part or aftermarket aluminum tank. Inspect the tank and cap regularly for signs of cracking, discoloration, or seepage. When replacing, also replace the cap and check all coolant hoses for brittleness. Flush and refill with BMW-approved coolant.</x:v>
-      </x:c>
-      <x:c r="F21" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G21" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="1306.800048828125" hidden="0" customHeight="1">
-      <x:c r="A22" s="40" t="n">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="B22" s="9" t="str">
-        <x:v>bmw-z4-e85-convertible-top-hydraulic-2003</x:v>
-      </x:c>
-      <x:c r="C22" s="9" t="str">
-        <x:v>2003-2008 | BMW | Z4</x:v>
-      </x:c>
-      <x:c r="D22" s="9" t="str">
-        <x:v>Convertible Top Hydraulic Pump Motor Failure - E85 Z4</x:v>
-      </x:c>
-      <x:c r="E22" s="9" t="str">
-        <x:v>Replace hydraulic pump motor assembly (BMW 54347193448 / supersedes 54347119633). OEM Genuine BMW pump: $800-$1,200. Aftermarket alternatives available on Amazon for $150-$300 but quality varies significantly. Dealer labor is $1,500-$2,500+ as BMW procedure requires full top removal. ZRoadster.org members have documented a motor relocation to the boot/trunk area which allows much easier future access. Hydraulic fluid: use Aral Vitamol ZHM or BMW 54340394395 hydraulic oil. PREVENTION: Clean drain holes annually, ensure rubber bungs are properly seated, and check for water intrusion in pump area at every service. Some owners have had success with pump motor rebuilds from roofmotors.co.uk ($300-$500) but quality of rebuilds varies.</x:v>
-      </x:c>
-      <x:c r="F22" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G22" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="1135.199951171875" hidden="0" customHeight="1">
-      <x:c r="A23" s="40" t="n">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B23" s="9" t="str">
-        <x:v>bmw-z4-e85-window-regulator-2003</x:v>
-      </x:c>
-      <x:c r="C23" s="9" t="str">
-        <x:v>2003-2008 | BMW | Z4</x:v>
-      </x:c>
-      <x:c r="D23" s="9" t="str">
-        <x:v>Power Window Regulator Failure - E85 Z4</x:v>
-      </x:c>
-      <x:c r="E23" s="9" t="str">
-        <x:v>Option 1 (Budget): Window regulator repair kit - replacement cables and rollers for ~$18-$25 from eBay/Amazon (BWR974 for left/driver side). Requires removing door panel and threading new cables through existing regulator frame. DIY-friendly with Z4-forum.com guides. Option 2 (Recommended): Full window regulator replacement. Driver side: BMW 51337198909 ($180-$280 OEM, $80-$150 aftermarket). Passenger side: BMW 51337198910 ($180-$280 OEM, $80-$150 aftermarket). Labor: $200-$400 at independent shop, $500-$700+ at dealer. DIY: 2-3 hours with door panel removal guide from Pelican Parts. ZRoadster.org recommends full replacement over repair kit for long-term reliability.</x:v>
-      </x:c>
-      <x:c r="F23" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G23" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="514.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A24" s="40" t="n">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="B24" s="9" t="str">
-        <x:v>bmw-z4-electric-steering-rack-2003</x:v>
-      </x:c>
-      <x:c r="C24" s="9" t="str">
-        <x:v>2012-2012 | BMW | Z4</x:v>
-      </x:c>
-      <x:c r="D24" s="9" t="str">
-        <x:v>2012 Z4 Electric Power-Steering Recall 12V-302</x:v>
-      </x:c>
-      <x:c r="E24" s="9" t="str">
-        <x:v>Check the VIN for an open 12V-302 campaign. If open, an authorized BMW dealer replaces the steering-assistance module free of charge. If the steering warning and audible alert occur, maintain control, reduce speed, stop safely and arrange dealer or roadside assistance; do not replace a steering rack from this card.</x:v>
-      </x:c>
-      <x:c r="F24" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G24" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="633.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A25" s="40" t="n">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="B25" s="9" t="str">
-        <x:v>bmw-z4-electric-water-pump-2006</x:v>
-      </x:c>
-      <x:c r="C25" s="9" t="str">
-        <x:v>2012-2016 | BMW | Z4 | N20</x:v>
-      </x:c>
-      <x:c r="D25" s="9" t="str">
-        <x:v>2012-2016 Z4 sDrive28i Water-Pump Connector Recall 24V-608</x:v>
-      </x:c>
-      <x:c r="E25" s="9" t="str">
-        <x:v>Check the VIN for an open 24V-608 campaign. If open, an authorized BMW dealer inspects the water pump and connector, replaces them if necessary, and installs the protective shield free of charge. If smoke appears from the engine compartment, stop safely, switch off the vehicle, have occupants exit, move away from traffic and call emergency or roadside assistance; do not order a pump from this card.</x:v>
-      </x:c>
-      <x:c r="F25" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G25" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="1359.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A26" s="40" t="n">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="B26" s="9" t="str">
-        <x:v>bmw-z4-g29-b58-water-pump-2019</x:v>
-      </x:c>
-      <x:c r="C26" s="9" t="str">
-        <x:v>2019-2025 | BMW | Z4 | M40i, sDrive35i, sDrive35is | B48, B58</x:v>
-      </x:c>
-      <x:c r="D26" s="9" t="str">
-        <x:v>B48/B58 Electric Water Pump &amp; Thermostat Failure - G29 Z4</x:v>
-      </x:c>
-      <x:c r="E26" s="9" t="str">
-        <x:v>Preventative replacement recommended at 60,000 miles. Always replace water pump and thermostat together - they share labor overlap and frequently fail concurrently. B48 sDrive30i: Water pump BMW 11518632586 ($300-$450), Thermostat BMW 11538685978 ($100-$150). B58 M40i: Water pump BMW 11518650986 ($350-$500), Thermostat BMW 11538685978 ($100-$150). Mishimoto offers performance water pump alternatives for B58 with improved impeller design. Replace 3 O-rings between thermostat and pump housing, plus 2 O-rings on coolant tube to head. Must replace water pump mounting bolts (torque-to-yield). Labor: 3-4 hours. FCP Euro lifetime warranty kits available. Also inspect plastic cylinder head coolant outlet adapter - known to shear off causing massive coolant leak.</x:v>
-      </x:c>
-      <x:c r="F26" s="9" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G26" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="1122" hidden="0" customHeight="1">
-      <x:c r="A27" s="40" t="n">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="B27" s="9" t="str">
-        <x:v>bmw-z4-n54-hpfp-2009</x:v>
-      </x:c>
-      <x:c r="C27" s="9" t="str">
-        <x:v>2009-2011 | BMW | Z4 | M40i, sDrive35i, sDrive35is | N54</x:v>
-      </x:c>
-      <x:c r="D27" s="9" t="str">
-        <x:v>N54 High Pressure Fuel Pump (HPFP) Failure - E89 Z4 sDrive35i/35is</x:v>
-      </x:c>
-      <x:c r="E27" s="9" t="str">
-        <x:v>Replace HPFP with latest revision Genuine BMW unit. The pump went through multiple revisions - ONLY install the latest version. Part number evolution: Original -&gt; 13517592881 (Index 10, TSB fix) -&gt; 13517616170 (latest revision, most reliable). Genuine BMW 13517616170 is the definitive fix ($350-$550 for pump). Replacement is straightforward DIY (1-2 hours) with basic tools. Also available as complete kit from FCP Euro with lifetime warranty. BMW extended warranty coverage to 10 years/120,000 miles under customer care package for original owners - check VIN eligibility. Replace low-pressure fuel sensor at same time (13537537319) as it may have been damaged by pressure fluctuations ($35-$55).</x:v>
-      </x:c>
-      <x:c r="F27" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G27" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="580.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A28" s="40" t="n">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="B28" s="9" t="str">
-        <x:v>bmw-z4-n54-wastegate-rattle-2009</x:v>
-      </x:c>
-      <x:c r="C28" s="9" t="str">
-        <x:v>2009-2010 | BMW | Z4 | N54</x:v>
-      </x:c>
-      <x:c r="D28" s="9" t="str">
-        <x:v>2009-2010 Z4 sDrive35i N54 Wastegate Diagnosis</x:v>
-      </x:c>
-      <x:c r="E28" s="9" t="str">
-        <x:v>Confirm the VIN, engine, production date, DME faults, boost-control data and noise source using current BMW diagnostic information. Check VIN-specific coverage history with BMW, recognizing that the bulletin's time/mileage window may have expired. Do not replace a turbocharger, actuator or wastegate from this card without the required diagnosis.</x:v>
-      </x:c>
-      <x:c r="F28" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G28" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="501.6000061035156" hidden="0" customHeight="1">
-      <x:c r="A29" s="40" t="n">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="B29" s="9" t="str">
-        <x:v>bmw-z4-soft-top-hydraulic-2003</x:v>
-      </x:c>
-      <x:c r="C29" s="9" t="str">
-        <x:v>2009-2016 | BMW | Z4</x:v>
-      </x:c>
-      <x:c r="D29" s="9" t="str">
-        <x:v>Retractable Hard Top Hydraulic Mechanism Failure</x:v>
-      </x:c>
-      <x:c r="E29" s="9" t="str">
-        <x:v>Diagnose the leak location and replace the failed component. Common failure points are the main hydraulic cylinders (left and right), the hydraulic pump motor, and the flexible hoses. The hydraulic fluid should be flushed and replaced with BMW-approved CHF 11S fluid. A full system bleed is required after any repair.</x:v>
-      </x:c>
-      <x:c r="F29" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G29" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="1188" hidden="0" customHeight="1">
-      <x:c r="A30" s="40" t="n">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="B30" s="9" t="str">
-        <x:v>bmw-z4-vanos-solenoid-2003</x:v>
-      </x:c>
-      <x:c r="C30" s="9" t="str">
-        <x:v>2003-2016 | BMW | Z4 | 2.5i, 3.0i, 3.0si, M40i, sDrive28i, sDrive30i, sDrive35i, sDrive35is | M54, N52, N54, N20</x:v>
-      </x:c>
-      <x:c r="D30" s="9" t="str">
-        <x:v>VANOS Solenoid &amp; System Failure - E85/E89 Z4 (All Engines)</x:v>
-      </x:c>
-      <x:c r="E30" s="9" t="str">
-        <x:v>Replace VANOS solenoids - inexpensive and straightforward repair. M54 (E85 2003-2005): 2 solenoids required, BMW 11361707323 ($35-$65 each). N52 (E85 2006-2008 / E89 2009-2011 28i): 2 solenoids, BMW 11367585425 ($40-$70 each). N54 (E89 35i/35is): 2 solenoids, BMW 11367585425 ($40-$70 each). N20 (E89 sDrive28i 2012-2016): 2 solenoids, BMW 11367585425 ($40-$70 each). Labor: under 1 hour for experienced mechanic, 2-3 hours DIY. Replace all solenoids at once even if only one has failed - the others are same age and will fail soon. Also replace VANOS solenoid O-rings and sealing plates during service. Clean VANOS system with Beisan Systems VANOS cleaning procedure for best results.</x:v>
-      </x:c>
-      <x:c r="F30" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G30" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="554.4000244140625" hidden="0" customHeight="1">
-      <x:c r="A31" s="42" t="n">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="B31" s="43" t="str">
-        <x:v>bmw-z8-soft-top-mechanism-2000</x:v>
-      </x:c>
-      <x:c r="C31" s="43" t="str">
-        <x:v>2000-2003 | BMW | Z8</x:v>
-      </x:c>
-      <x:c r="D31" s="43" t="str">
-        <x:v>Power Soft Top Hydraulic System and Cable Failure</x:v>
-      </x:c>
-      <x:c r="E31" s="43" t="str">
-        <x:v>Rebuild the hydraulic cylinders with new seals rather than replacing ($200 vs $2,000+). Inspect and replace frayed cables. Adjust or replace the microswitch sensors at the windshield header latch. Lubricate the top mechanism pivot points with silicone grease annually. Store the car with the top up to reduce stress on the hydraulic system.</x:v>
-      </x:c>
-      <x:c r="F31" s="43" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G31" s="44" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -20510,7 +21707,7 @@
       <x:c r="F2" s="28"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="45" t="str">
+      <x:c r="A3" s="48" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="B3" s="15" t="str">
@@ -20522,7 +21719,7 @@
       <x:c r="F3" s="28"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="45" t="str">
+      <x:c r="A4" s="48" t="str">
         <x:v>2</x:v>
       </x:c>
       <x:c r="B4" s="15" t="str">
@@ -20534,7 +21731,7 @@
       <x:c r="F4" s="28"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="45" t="str">
+      <x:c r="A5" s="48" t="str">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B5" s="15" t="str">
@@ -20546,7 +21743,7 @@
       <x:c r="F5" s="28"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="45" t="str">
+      <x:c r="A6" s="48" t="str">
         <x:v>4</x:v>
       </x:c>
       <x:c r="B6" s="15" t="str">
@@ -20558,7 +21755,7 @@
       <x:c r="F6" s="28"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="45" t="str">
+      <x:c r="A7" s="48" t="str">
         <x:v>5</x:v>
       </x:c>
       <x:c r="B7" s="15" t="str">
@@ -20570,7 +21767,7 @@
       <x:c r="F7" s="28"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="45" t="str">
+      <x:c r="A8" s="48" t="str">
         <x:v>6</x:v>
       </x:c>
       <x:c r="B8" s="15" t="str">
@@ -20582,7 +21779,7 @@
       <x:c r="F8" s="28"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="45" t="str">
+      <x:c r="A9" s="48" t="str">
         <x:v>7</x:v>
       </x:c>
       <x:c r="B9" s="15" t="str">
@@ -20594,7 +21791,7 @@
       <x:c r="F9" s="28"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="45" t="str">
+      <x:c r="A10" s="48" t="str">
         <x:v>8</x:v>
       </x:c>
       <x:c r="B10" s="15" t="str">
@@ -20614,7 +21811,7 @@
       <x:c r="F11" s="28"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="46" t="str">
+      <x:c r="A12" s="49" t="str">
         <x:v>Artifact state</x:v>
       </x:c>
       <x:c r="B12" s="11" t="str">
@@ -20626,7 +21823,7 @@
       <x:c r="F12" s="28"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="46" t="str">
+      <x:c r="A13" s="49" t="str">
         <x:v>Source</x:v>
       </x:c>
       <x:c r="B13" s="11" t="str">
@@ -20638,7 +21835,7 @@
       <x:c r="F13" s="28"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="46" t="str">
+      <x:c r="A14" s="49" t="str">
         <x:v>Review input</x:v>
       </x:c>
       <x:c r="B14" s="11" t="str">
@@ -20650,16 +21847,16 @@
       <x:c r="F14" s="28"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="47" t="str">
+      <x:c r="A15" s="50" t="str">
         <x:v>Generated ledger</x:v>
       </x:c>
-      <x:c r="B15" s="48" t="str">
+      <x:c r="B15" s="51" t="str">
         <x:v>data\bmw-repair-first-review\review-ledger.json</x:v>
       </x:c>
-      <x:c r="C15" s="48"/>
-      <x:c r="D15" s="48"/>
-      <x:c r="E15" s="48"/>
-      <x:c r="F15" s="49"/>
+      <x:c r="C15" s="51"/>
+      <x:c r="D15" s="51"/>
+      <x:c r="E15" s="51"/>
+      <x:c r="F15" s="52"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>